<commit_message>
Refresh dashboard Mon 09/07/2026 17:03
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 04 Sep 2026 16:48</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 07 Sep 2026 17:03</t>
         </is>
       </c>
     </row>
@@ -805,14 +805,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 04 Sep 2026</t>
+          <t>MTD as of 07 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 04 Sep 2026</t>
+          <t>YTD as of 07 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
@@ -1220,22 +1220,22 @@
         <v>914323824.5555556</v>
       </c>
       <c r="AD7" s="11" t="n">
-        <v>75379454</v>
+        <v>3860720333</v>
       </c>
       <c r="AE7" s="11" t="n">
-        <v>4434.085529411765</v>
+        <v>227101.1960588235</v>
       </c>
       <c r="AF7" s="11" t="n">
-        <v>398833.08994709</v>
+        <v>20427091.70899471</v>
       </c>
       <c r="AG7" s="11" t="n">
-        <v>172882582295</v>
+        <v>176667923174</v>
       </c>
       <c r="AH7" s="11" t="n">
-        <v>10169563.66441176</v>
+        <v>10392230.77494118</v>
       </c>
       <c r="AI7" s="11" t="n">
-        <v>914722657.6455027</v>
+        <v>934750916.2645503</v>
       </c>
     </row>
     <row r="8">
@@ -1401,17 +1401,23 @@
       <c r="AC9" s="11" t="n">
         <v>198819750.8201058</v>
       </c>
-      <c r="AD9" s="11" t="n"/>
-      <c r="AE9" s="11" t="n"/>
-      <c r="AF9" s="11" t="n"/>
+      <c r="AD9" s="11" t="n">
+        <v>3785340879</v>
+      </c>
+      <c r="AE9" s="11" t="n">
+        <v>222667.1105294118</v>
+      </c>
+      <c r="AF9" s="11" t="n">
+        <v>20028258.61904762</v>
+      </c>
       <c r="AG9" s="11" t="n">
-        <v>37576932905</v>
+        <v>41362273784</v>
       </c>
       <c r="AH9" s="11" t="n">
-        <v>2210407.817941176</v>
+        <v>2433074.928470588</v>
       </c>
       <c r="AI9" s="11" t="n">
-        <v>198819750.8201058</v>
+        <v>218848009.4391534</v>
       </c>
     </row>
     <row r="10">
@@ -2184,22 +2190,22 @@
         <v>2321849.073439153</v>
       </c>
       <c r="AD20" s="13" t="n">
-        <v>4158000</v>
+        <v>5934000</v>
       </c>
       <c r="AE20" s="13" t="n">
-        <v>244.5882352941177</v>
+        <v>349.0588235294118</v>
       </c>
       <c r="AF20" s="13" t="n">
-        <v>22000</v>
+        <v>31396.8253968254</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>442987474.88</v>
+        <v>444763474.88</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>26058.08675764706</v>
+        <v>26162.55734588236</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>2343849.073439153</v>
+        <v>2353245.898835979</v>
       </c>
     </row>
     <row r="21">
@@ -2436,22 +2442,22 @@
         <v>332547.6190476191</v>
       </c>
       <c r="AD23" s="11" t="n">
-        <v>4158000</v>
+        <v>5561500</v>
       </c>
       <c r="AE23" s="11" t="n">
-        <v>244.5882352941177</v>
+        <v>327.1470588235294</v>
       </c>
       <c r="AF23" s="11" t="n">
-        <v>22000</v>
+        <v>29425.92592592593</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>67009500</v>
+        <v>68413000</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>3941.735294117646</v>
+        <v>4024.294117647058</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>354547.6190476191</v>
+        <v>361973.544973545</v>
       </c>
     </row>
     <row r="24">
@@ -2767,17 +2773,23 @@
       <c r="AC28" s="13" t="n">
         <v>62858.95238095238</v>
       </c>
-      <c r="AD28" s="13" t="n"/>
-      <c r="AE28" s="13" t="n"/>
-      <c r="AF28" s="13" t="n"/>
+      <c r="AD28" s="13" t="n">
+        <v>372500</v>
+      </c>
+      <c r="AE28" s="13" t="n">
+        <v>21.91176470588235</v>
+      </c>
+      <c r="AF28" s="13" t="n">
+        <v>1970.899470899471</v>
+      </c>
       <c r="AG28" s="13" t="n">
-        <v>11880342</v>
+        <v>12252842</v>
       </c>
       <c r="AH28" s="13" t="n">
-        <v>698.8436470588234</v>
+        <v>720.7554117647057</v>
       </c>
       <c r="AI28" s="13" t="n">
-        <v>62858.95238095238</v>
+        <v>64829.85185185185</v>
       </c>
     </row>
     <row r="29">
@@ -3822,22 +3834,22 @@
         <v>1180222393.205714</v>
       </c>
       <c r="AD44" s="15" t="n">
-        <v>79537454</v>
+        <v>3866654333</v>
       </c>
       <c r="AE44" s="15" t="n">
-        <v>4678.673764705883</v>
+        <v>227450.254882353</v>
       </c>
       <c r="AF44" s="15" t="n">
-        <v>420833.08994709</v>
+        <v>20458488.53439153</v>
       </c>
       <c r="AG44" s="15" t="n">
-        <v>223141569769.88</v>
+        <v>226928686648.88</v>
       </c>
       <c r="AH44" s="15" t="n">
-        <v>13125974.69234588</v>
+        <v>13348746.27346353</v>
       </c>
       <c r="AI44" s="15" t="n">
-        <v>1180643226.295661</v>
+        <v>1200680881.740106</v>
       </c>
     </row>
     <row r="45">
@@ -10065,17 +10077,23 @@
       <c r="AC126" s="11" t="n">
         <v>-1736052.91005291</v>
       </c>
-      <c r="AD126" s="11" t="n"/>
-      <c r="AE126" s="11" t="n"/>
-      <c r="AF126" s="11" t="n"/>
+      <c r="AD126" s="11" t="n">
+        <v>-7000000</v>
+      </c>
+      <c r="AE126" s="11" t="n">
+        <v>-411.7647058823529</v>
+      </c>
+      <c r="AF126" s="11" t="n">
+        <v>-37037.03703703704</v>
+      </c>
       <c r="AG126" s="11" t="n">
-        <v>-328114000</v>
+        <v>-335114000</v>
       </c>
       <c r="AH126" s="11" t="n">
-        <v>-19300.82352941177</v>
+        <v>-19712.58823529412</v>
       </c>
       <c r="AI126" s="11" t="n">
-        <v>-1736052.91005291</v>
+        <v>-1773089.947089947</v>
       </c>
     </row>
     <row r="127">
@@ -10372,22 +10390,22 @@
         <v>-132568430.7276719</v>
       </c>
       <c r="AD129" s="15" t="n">
-        <v>-8362300</v>
+        <v>-15362300</v>
       </c>
       <c r="AE129" s="15" t="n">
-        <v>-491.9</v>
+        <v>-903.6647058823529</v>
       </c>
       <c r="AF129" s="15" t="n">
-        <v>-44244.97354497355</v>
+        <v>-81282.01058201058</v>
       </c>
       <c r="AG129" s="15" t="n">
-        <v>-25063795707.53</v>
+        <v>-25070795707.53</v>
       </c>
       <c r="AH129" s="15" t="n">
-        <v>-1474340.923972353</v>
+        <v>-1474752.688678235</v>
       </c>
       <c r="AI129" s="15" t="n">
-        <v>-132612675.7012169</v>
+        <v>-132649712.738254</v>
       </c>
     </row>
     <row r="130">
@@ -11140,22 +11158,22 @@
         <v>-230400464.7853439</v>
       </c>
       <c r="AD138" s="15" t="n">
-        <v>-11312300</v>
+        <v>-18312300</v>
       </c>
       <c r="AE138" s="15" t="n">
-        <v>-665.4294117647058</v>
+        <v>-1077.194117647059</v>
       </c>
       <c r="AF138" s="15" t="n">
-        <v>-59853.43915343915</v>
+        <v>-96890.47619047618</v>
       </c>
       <c r="AG138" s="15" t="n">
-        <v>-43557000144.43001</v>
+        <v>-43564000144.43001</v>
       </c>
       <c r="AH138" s="15" t="n">
-        <v>-2562176.479084118</v>
+        <v>-2562588.24379</v>
       </c>
       <c r="AI138" s="15" t="n">
-        <v>-230460318.2244973</v>
+        <v>-230497355.2615344</v>
       </c>
     </row>
     <row r="139">
@@ -12334,22 +12352,22 @@
         <v>-1529478500.653757</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-358870498</v>
+        <v>-365870498</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-21110.02929411765</v>
+        <v>-21521.794</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-1898785.703703704</v>
+        <v>-1935822.740740741</v>
       </c>
       <c r="AG153" s="19" t="n">
-        <v>-289430307121.5599</v>
+        <v>-289437307121.5599</v>
       </c>
       <c r="AH153" s="19" t="n">
-        <v>-17025312.18362118</v>
+        <v>-17025723.94832706</v>
       </c>
       <c r="AI153" s="19" t="n">
-        <v>-1531377286.35746</v>
+        <v>-1531414323.394497</v>
       </c>
     </row>
     <row r="154">
@@ -12440,22 +12458,22 @@
         <v>-349256107.4480425</v>
       </c>
       <c r="AD154" s="19" t="n">
-        <v>-279333044</v>
+        <v>3500783835</v>
       </c>
       <c r="AE154" s="19" t="n">
-        <v>-16431.35552941177</v>
+        <v>205928.4608823529</v>
       </c>
       <c r="AF154" s="19" t="n">
-        <v>-1477952.613756614</v>
+        <v>18522665.79365079</v>
       </c>
       <c r="AG154" s="19" t="n">
-        <v>-66288737351.68</v>
+        <v>-62508620472.68</v>
       </c>
       <c r="AH154" s="19" t="n">
-        <v>-3899337.491275295</v>
+        <v>-3676977.67486353</v>
       </c>
       <c r="AI154" s="19" t="n">
-        <v>-350734060.061799</v>
+        <v>-330733441.6543916</v>
       </c>
     </row>
     <row r="155">
@@ -12546,22 +12564,22 @@
         <v>7747388.987724859</v>
       </c>
       <c r="AD155" s="7" t="n">
-        <v>1184923474.679998</v>
+        <v>4965040353.679998</v>
       </c>
       <c r="AE155" s="7" t="n">
-        <v>69701.38086352932</v>
+        <v>292061.197275294</v>
       </c>
       <c r="AF155" s="7" t="n">
-        <v>6269436.373968245</v>
+        <v>26270054.78137565</v>
       </c>
       <c r="AG155" s="7" t="n">
-        <v>1184923474.679998</v>
+        <v>4965040353.679998</v>
       </c>
       <c r="AH155" s="7" t="n">
-        <v>69701.38086352932</v>
+        <v>292061.197275294</v>
       </c>
       <c r="AI155" s="7" t="n">
-        <v>6269436.373968245</v>
+        <v>26270054.78137565</v>
       </c>
     </row>
   </sheetData>
@@ -13026,16 +13044,16 @@
         <v>1136676704</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>-271176244</v>
+        <v>3514164635</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>865500460</v>
+        <v>4650841339</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>50911.79176470589</v>
+        <v>273578.9022941177</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>4579367.513227513</v>
+        <v>24607626.13227513</v>
       </c>
     </row>
     <row r="7">
@@ -13122,16 +13140,16 @@
         <v>172976399.24</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>-8181800</v>
+        <v>-13405800</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>164794599.24</v>
+        <v>159570599.24</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>9693.799955294118</v>
+        <v>9386.505837647059</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>871929.0965079366</v>
+        <v>844288.884867725</v>
       </c>
     </row>
     <row r="10">
@@ -13241,13 +13259,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>1184923476.68</v>
+        <v>4965040355.679999</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>69701.38098117648</v>
+        <v>292061.1973929412</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>6269436.384550265</v>
+        <v>26270054.79195767</v>
       </c>
     </row>
   </sheetData>
@@ -13317,7 +13335,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 04 Sep 2026 16:48 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 07 Sep 2026 17:03 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -13392,14 +13410,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 04 Sep 2026</t>
+          <t>MTD as of 07 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 04 Sep 2026</t>
+          <t>YTD as of 07 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
@@ -13807,22 +13825,22 @@
         <v>914.3238245555556</v>
       </c>
       <c r="AD7" s="11" t="n">
-        <v>75.379454</v>
+        <v>3860.720333</v>
       </c>
       <c r="AE7" s="11" t="n">
-        <v>0.004434085529411764</v>
+        <v>0.2271011960588235</v>
       </c>
       <c r="AF7" s="11" t="n">
-        <v>0.3988330899470899</v>
+        <v>20.42709170899471</v>
       </c>
       <c r="AG7" s="11" t="n">
-        <v>172882.582295</v>
+        <v>176667.923174</v>
       </c>
       <c r="AH7" s="11" t="n">
-        <v>10.16956366441176</v>
+        <v>10.39223077494118</v>
       </c>
       <c r="AI7" s="11" t="n">
-        <v>914.7226576455026</v>
+        <v>934.7509162645503</v>
       </c>
     </row>
     <row r="8">
@@ -13988,17 +14006,23 @@
       <c r="AC9" s="11" t="n">
         <v>198.8197508201058</v>
       </c>
-      <c r="AD9" s="11" t="n"/>
-      <c r="AE9" s="11" t="n"/>
-      <c r="AF9" s="11" t="n"/>
+      <c r="AD9" s="11" t="n">
+        <v>3785.340879</v>
+      </c>
+      <c r="AE9" s="11" t="n">
+        <v>0.2226671105294118</v>
+      </c>
+      <c r="AF9" s="11" t="n">
+        <v>20.02825861904762</v>
+      </c>
       <c r="AG9" s="11" t="n">
-        <v>37576.932905</v>
+        <v>41362.273784</v>
       </c>
       <c r="AH9" s="11" t="n">
-        <v>2.210407817941176</v>
+        <v>2.433074928470588</v>
       </c>
       <c r="AI9" s="11" t="n">
-        <v>198.8197508201058</v>
+        <v>218.8480094391534</v>
       </c>
     </row>
     <row r="10">
@@ -14771,22 +14795,22 @@
         <v>2.321849073439154</v>
       </c>
       <c r="AD20" s="13" t="n">
-        <v>4.158</v>
+        <v>5.934</v>
       </c>
       <c r="AE20" s="13" t="n">
-        <v>0.0002445882352941176</v>
+        <v>0.0003490588235294118</v>
       </c>
       <c r="AF20" s="13" t="n">
-        <v>0.022</v>
+        <v>0.0313968253968254</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>442.98747488</v>
+        <v>444.76347488</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>0.02605808675764706</v>
+        <v>0.02616255734588235</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>2.343849073439153</v>
+        <v>2.353245898835979</v>
       </c>
     </row>
     <row r="21">
@@ -15023,22 +15047,22 @@
         <v>0.332547619047619</v>
       </c>
       <c r="AD23" s="11" t="n">
-        <v>4.158</v>
+        <v>5.5615</v>
       </c>
       <c r="AE23" s="11" t="n">
-        <v>0.0002445882352941176</v>
+        <v>0.0003271470588235294</v>
       </c>
       <c r="AF23" s="11" t="n">
-        <v>0.022</v>
+        <v>0.02942592592592592</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>67.0095</v>
+        <v>68.413</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>0.003941735294117648</v>
+        <v>0.004024294117647059</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>0.3545476190476191</v>
+        <v>0.3619735449735449</v>
       </c>
     </row>
     <row r="24">
@@ -15354,17 +15378,23 @@
       <c r="AC28" s="13" t="n">
         <v>0.06285895238095238</v>
       </c>
-      <c r="AD28" s="13" t="n"/>
-      <c r="AE28" s="13" t="n"/>
-      <c r="AF28" s="13" t="n"/>
+      <c r="AD28" s="13" t="n">
+        <v>0.3725</v>
+      </c>
+      <c r="AE28" s="13" t="n">
+        <v>2.191176470588235e-05</v>
+      </c>
+      <c r="AF28" s="13" t="n">
+        <v>0.001970899470899471</v>
+      </c>
       <c r="AG28" s="13" t="n">
-        <v>11.880342</v>
+        <v>12.252842</v>
       </c>
       <c r="AH28" s="13" t="n">
-        <v>0.0006988436470588235</v>
+        <v>0.0007207554117647059</v>
       </c>
       <c r="AI28" s="13" t="n">
-        <v>0.06285895238095238</v>
+        <v>0.06482985185185185</v>
       </c>
     </row>
     <row r="29">
@@ -16409,22 +16439,22 @@
         <v>1180.222393205714</v>
       </c>
       <c r="AD44" s="15" t="n">
-        <v>79.537454</v>
+        <v>3866.654333</v>
       </c>
       <c r="AE44" s="15" t="n">
-        <v>0.004678673764705882</v>
+        <v>0.2274502548823529</v>
       </c>
       <c r="AF44" s="15" t="n">
-        <v>0.42083308994709</v>
+        <v>20.45848853439153</v>
       </c>
       <c r="AG44" s="15" t="n">
-        <v>223141.56976988</v>
+        <v>226928.68664888</v>
       </c>
       <c r="AH44" s="15" t="n">
-        <v>13.12597469234588</v>
+        <v>13.34874627346353</v>
       </c>
       <c r="AI44" s="15" t="n">
-        <v>1180.643226295661</v>
+        <v>1200.680881740106</v>
       </c>
     </row>
     <row r="45">
@@ -22652,17 +22682,23 @@
       <c r="AC126" s="11" t="n">
         <v>-1.73605291005291</v>
       </c>
-      <c r="AD126" s="11" t="n"/>
-      <c r="AE126" s="11" t="n"/>
-      <c r="AF126" s="11" t="n"/>
+      <c r="AD126" s="11" t="n">
+        <v>-7</v>
+      </c>
+      <c r="AE126" s="11" t="n">
+        <v>-0.000411764705882353</v>
+      </c>
+      <c r="AF126" s="11" t="n">
+        <v>-0.03703703703703703</v>
+      </c>
       <c r="AG126" s="11" t="n">
-        <v>-328.114</v>
+        <v>-335.114</v>
       </c>
       <c r="AH126" s="11" t="n">
-        <v>-0.01930082352941177</v>
+        <v>-0.01971258823529412</v>
       </c>
       <c r="AI126" s="11" t="n">
-        <v>-1.73605291005291</v>
+        <v>-1.773089947089947</v>
       </c>
     </row>
     <row r="127">
@@ -22959,22 +22995,22 @@
         <v>-132.568430727672</v>
       </c>
       <c r="AD129" s="15" t="n">
-        <v>-8.362299999999999</v>
+        <v>-15.3623</v>
       </c>
       <c r="AE129" s="15" t="n">
-        <v>-0.0004919</v>
+        <v>-0.0009036647058823529</v>
       </c>
       <c r="AF129" s="15" t="n">
-        <v>-0.04424497354497354</v>
+        <v>-0.08128201058201058</v>
       </c>
       <c r="AG129" s="15" t="n">
-        <v>-25063.79570753</v>
+        <v>-25070.79570753</v>
       </c>
       <c r="AH129" s="15" t="n">
-        <v>-1.474340923972353</v>
+        <v>-1.474752688678236</v>
       </c>
       <c r="AI129" s="15" t="n">
-        <v>-132.6126757012169</v>
+        <v>-132.649712738254</v>
       </c>
     </row>
     <row r="130">
@@ -23727,22 +23763,22 @@
         <v>-230.4004647853439</v>
       </c>
       <c r="AD138" s="15" t="n">
-        <v>-11.3123</v>
+        <v>-18.3123</v>
       </c>
       <c r="AE138" s="15" t="n">
-        <v>-0.0006654294117647059</v>
+        <v>-0.001077194117647059</v>
       </c>
       <c r="AF138" s="15" t="n">
-        <v>-0.05985343915343916</v>
+        <v>-0.09689047619047619</v>
       </c>
       <c r="AG138" s="15" t="n">
-        <v>-43557.00014443</v>
+        <v>-43564.00014443</v>
       </c>
       <c r="AH138" s="15" t="n">
-        <v>-2.562176479084117</v>
+        <v>-2.56258824379</v>
       </c>
       <c r="AI138" s="15" t="n">
-        <v>-230.4603182244973</v>
+        <v>-230.4973552615344</v>
       </c>
     </row>
     <row r="139">
@@ -24921,22 +24957,22 @@
         <v>-1529.478500653756</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-358.870498</v>
+        <v>-365.870498</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-0.02111002929411765</v>
+        <v>-0.021521794</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-1.898785703703704</v>
+        <v>-1.935822740740741</v>
       </c>
       <c r="AG153" s="19" t="n">
-        <v>-289430.3071215599</v>
+        <v>-289437.3071215599</v>
       </c>
       <c r="AH153" s="19" t="n">
-        <v>-17.02531218362118</v>
+        <v>-17.02572394832706</v>
       </c>
       <c r="AI153" s="19" t="n">
-        <v>-1531.37728635746</v>
+        <v>-1531.414323394497</v>
       </c>
     </row>
     <row r="154">
@@ -25027,22 +25063,22 @@
         <v>-349.2561074480424</v>
       </c>
       <c r="AD154" s="19" t="n">
-        <v>-279.333044</v>
+        <v>3500.783835</v>
       </c>
       <c r="AE154" s="19" t="n">
-        <v>-0.01643135552941176</v>
+        <v>0.2059284608823529</v>
       </c>
       <c r="AF154" s="19" t="n">
-        <v>-1.477952613756614</v>
+        <v>18.52266579365079</v>
       </c>
       <c r="AG154" s="19" t="n">
-        <v>-66288.73735168001</v>
+        <v>-62508.62047268001</v>
       </c>
       <c r="AH154" s="19" t="n">
-        <v>-3.899337491275295</v>
+        <v>-3.67697767486353</v>
       </c>
       <c r="AI154" s="19" t="n">
-        <v>-350.734060061799</v>
+        <v>-330.7334416543916</v>
       </c>
     </row>
     <row r="155">
@@ -25133,22 +25169,22 @@
         <v>7.747388987724859</v>
       </c>
       <c r="AD155" s="7" t="n">
-        <v>1184.923474679998</v>
+        <v>4965.040353679999</v>
       </c>
       <c r="AE155" s="7" t="n">
-        <v>0.06970138086352932</v>
+        <v>0.2920611972752941</v>
       </c>
       <c r="AF155" s="7" t="n">
-        <v>6.269436373968245</v>
+        <v>26.27005478137565</v>
       </c>
       <c r="AG155" s="7" t="n">
-        <v>1184.923474679998</v>
+        <v>4965.040353679999</v>
       </c>
       <c r="AH155" s="7" t="n">
-        <v>0.06970138086352932</v>
+        <v>0.2920611972752941</v>
       </c>
       <c r="AI155" s="7" t="n">
-        <v>6.269436373968245</v>
+        <v>26.27005478137565</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Wed 09/09/2026 11:37
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 07 Sep 2026 17:03</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 09 Sep 2026 11:37</t>
         </is>
       </c>
     </row>
@@ -805,14 +805,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 07 Sep 2026</t>
+          <t>MTD as of 09 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 07 Sep 2026</t>
+          <t>YTD as of 09 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
@@ -13335,7 +13335,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 07 Sep 2026 17:03 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 09 Sep 2026 11:37 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -13410,14 +13410,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 07 Sep 2026</t>
+          <t>MTD as of 09 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 07 Sep 2026</t>
+          <t>YTD as of 09 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>

</xml_diff>

<commit_message>
Refresh dashboard Wed 09/09/2026 11:45
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 09 Sep 2026 11:37</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 09 Sep 2026 11:45</t>
         </is>
       </c>
     </row>
@@ -13335,7 +13335,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 09 Sep 2026 11:37 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 09 Sep 2026 11:45 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Wed 09/09/2026 16:19
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 09 Sep 2026 11:45</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 09 Sep 2026 16:19</t>
         </is>
       </c>
     </row>
@@ -2190,22 +2190,22 @@
         <v>2321849.073439153</v>
       </c>
       <c r="AD20" s="13" t="n">
-        <v>5934000</v>
+        <v>13875500</v>
       </c>
       <c r="AE20" s="13" t="n">
-        <v>349.0588235294118</v>
+        <v>816.2058823529412</v>
       </c>
       <c r="AF20" s="13" t="n">
-        <v>31396.8253968254</v>
+        <v>73415.34391534391</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>444763474.88</v>
+        <v>452704974.88</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>26162.55734588236</v>
+        <v>26629.70440470588</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>2353245.898835979</v>
+        <v>2395264.417354497</v>
       </c>
     </row>
     <row r="21">
@@ -2442,22 +2442,22 @@
         <v>332547.6190476191</v>
       </c>
       <c r="AD23" s="11" t="n">
-        <v>5561500</v>
+        <v>13503000</v>
       </c>
       <c r="AE23" s="11" t="n">
-        <v>327.1470588235294</v>
+        <v>794.2941176470588</v>
       </c>
       <c r="AF23" s="11" t="n">
-        <v>29425.92592592593</v>
+        <v>71444.44444444444</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>68413000</v>
+        <v>76354500</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>4024.294117647058</v>
+        <v>4491.441176470587</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>361973.544973545</v>
+        <v>403992.0634920635</v>
       </c>
     </row>
     <row r="24">
@@ -3834,22 +3834,22 @@
         <v>1180222393.205714</v>
       </c>
       <c r="AD44" s="15" t="n">
-        <v>3866654333</v>
+        <v>3874595833</v>
       </c>
       <c r="AE44" s="15" t="n">
-        <v>227450.254882353</v>
+        <v>227917.4019411765</v>
       </c>
       <c r="AF44" s="15" t="n">
-        <v>20458488.53439153</v>
+        <v>20500507.05291005</v>
       </c>
       <c r="AG44" s="15" t="n">
-        <v>226928686648.88</v>
+        <v>226936628148.88</v>
       </c>
       <c r="AH44" s="15" t="n">
-        <v>13348746.27346353</v>
+        <v>13349213.42052235</v>
       </c>
       <c r="AI44" s="15" t="n">
-        <v>1200680881.740106</v>
+        <v>1200722900.258625</v>
       </c>
     </row>
     <row r="45">
@@ -4498,34 +4498,34 @@
         <v>-1644358.121693122</v>
       </c>
       <c r="X54" s="13" t="n">
-        <v>-351295896</v>
+        <v>-374832396</v>
       </c>
       <c r="Y54" s="13" t="n">
-        <v>-20664.46447058823</v>
+        <v>-22048.96447058823</v>
       </c>
       <c r="Z54" s="13" t="n">
-        <v>-1858708.444444444</v>
+        <v>-1983240.190476191</v>
       </c>
       <c r="AA54" s="13" t="n">
-        <v>-1356464410</v>
+        <v>-1380000910</v>
       </c>
       <c r="AB54" s="13" t="n">
-        <v>-79792.02411764706</v>
+        <v>-81176.52411764706</v>
       </c>
       <c r="AC54" s="13" t="n">
-        <v>-7177060.370370369</v>
+        <v>-7301592.116402116</v>
       </c>
       <c r="AD54" s="13" t="n"/>
       <c r="AE54" s="13" t="n"/>
       <c r="AF54" s="13" t="n"/>
       <c r="AG54" s="13" t="n">
-        <v>-1356464410</v>
+        <v>-1380000910</v>
       </c>
       <c r="AH54" s="13" t="n">
-        <v>-79792.02411764706</v>
+        <v>-81176.52411764706</v>
       </c>
       <c r="AI54" s="13" t="n">
-        <v>-7177060.370370369</v>
+        <v>-7301592.116402116</v>
       </c>
     </row>
     <row r="55">
@@ -5148,34 +5148,34 @@
         <v>-4972000.248677249</v>
       </c>
       <c r="X62" s="15" t="n">
-        <v>-1669450550</v>
+        <v>-1692987050</v>
       </c>
       <c r="Y62" s="15" t="n">
-        <v>-98202.97352941177</v>
+        <v>-99587.47352941177</v>
       </c>
       <c r="Z62" s="15" t="n">
-        <v>-8833071.693121694</v>
+        <v>-8957603.439153438</v>
       </c>
       <c r="AA62" s="15" t="n">
-        <v>-15962224681.88</v>
+        <v>-15985761181.88</v>
       </c>
       <c r="AB62" s="15" t="n">
-        <v>-938954.3930517647</v>
+        <v>-940338.8930517647</v>
       </c>
       <c r="AC62" s="15" t="n">
-        <v>-84456215.24804235</v>
+        <v>-84580746.99407408</v>
       </c>
       <c r="AD62" s="15" t="n"/>
       <c r="AE62" s="15" t="n"/>
       <c r="AF62" s="15" t="n"/>
       <c r="AG62" s="15" t="n">
-        <v>-15962224681.88</v>
+        <v>-15985761181.88</v>
       </c>
       <c r="AH62" s="15" t="n">
-        <v>-938954.3930517647</v>
+        <v>-940338.8930517647</v>
       </c>
       <c r="AI62" s="15" t="n">
-        <v>-84456215.24804235</v>
+        <v>-84580746.99407408</v>
       </c>
     </row>
     <row r="63">
@@ -6333,17 +6333,23 @@
       <c r="AC81" s="13" t="n">
         <v>-48834989.68539683</v>
       </c>
-      <c r="AD81" s="13" t="n"/>
-      <c r="AE81" s="13" t="n"/>
-      <c r="AF81" s="13" t="n"/>
+      <c r="AD81" s="13" t="n">
+        <v>-14626100</v>
+      </c>
+      <c r="AE81" s="13" t="n">
+        <v>-860.3588235294118</v>
+      </c>
+      <c r="AF81" s="13" t="n">
+        <v>-77386.77248677249</v>
+      </c>
       <c r="AG81" s="13" t="n">
-        <v>-9229813050.540001</v>
+        <v>-9244439150.540001</v>
       </c>
       <c r="AH81" s="13" t="n">
-        <v>-542930.1794435293</v>
+        <v>-543790.5382670588</v>
       </c>
       <c r="AI81" s="13" t="n">
-        <v>-48834989.68539683</v>
+        <v>-48912376.4578836</v>
       </c>
     </row>
     <row r="82">
@@ -6634,22 +6640,22 @@
         <v>-126334224.2039154</v>
       </c>
       <c r="AD84" s="15" t="n">
-        <v>-286804298</v>
+        <v>-301430398</v>
       </c>
       <c r="AE84" s="15" t="n">
-        <v>-16870.84105882353</v>
+        <v>-17731.19988235294</v>
       </c>
       <c r="AF84" s="15" t="n">
-        <v>-1517483.058201058</v>
+        <v>-1594869.830687831</v>
       </c>
       <c r="AG84" s="15" t="n">
-        <v>-24163972672.54</v>
+        <v>-24178598772.54</v>
       </c>
       <c r="AH84" s="15" t="n">
-        <v>-1421410.157208235</v>
+        <v>-1422270.516031765</v>
       </c>
       <c r="AI84" s="15" t="n">
-        <v>-127851707.2621164</v>
+        <v>-127929094.0346032</v>
       </c>
     </row>
     <row r="85">
@@ -9480,22 +9486,22 @@
         <v>-3587797.08994709</v>
       </c>
       <c r="X119" s="11" t="n">
-        <v>-1090252254</v>
+        <v>-1066715754</v>
       </c>
       <c r="Y119" s="11" t="n">
-        <v>-64132.48552941177</v>
+        <v>-62747.98552941177</v>
       </c>
       <c r="Z119" s="11" t="n">
-        <v>-5768530.444444444</v>
+        <v>-5643998.698412699</v>
       </c>
       <c r="AA119" s="11" t="n">
-        <v>-5648971481</v>
+        <v>-5625434981</v>
       </c>
       <c r="AB119" s="11" t="n">
-        <v>-332292.4400588235</v>
+        <v>-330907.9400588235</v>
       </c>
       <c r="AC119" s="11" t="n">
-        <v>-29888737.994709</v>
+        <v>-29764206.24867725</v>
       </c>
       <c r="AD119" s="11" t="n">
         <v>-2950000</v>
@@ -9507,13 +9513,13 @@
         <v>-15608.46560846561</v>
       </c>
       <c r="AG119" s="11" t="n">
-        <v>-5651921481</v>
+        <v>-5628384981</v>
       </c>
       <c r="AH119" s="11" t="n">
-        <v>-332465.9694705882</v>
+        <v>-331081.4694705882</v>
       </c>
       <c r="AI119" s="11" t="n">
-        <v>-29904346.46031746</v>
+        <v>-29779814.71428572</v>
       </c>
     </row>
     <row r="120">
@@ -9586,22 +9592,22 @@
         <v>-3587797.08994709</v>
       </c>
       <c r="X120" s="15" t="n">
-        <v>-1090252254</v>
+        <v>-1066715754</v>
       </c>
       <c r="Y120" s="15" t="n">
-        <v>-64132.48552941177</v>
+        <v>-62747.98552941177</v>
       </c>
       <c r="Z120" s="15" t="n">
-        <v>-5768530.444444444</v>
+        <v>-5643998.698412699</v>
       </c>
       <c r="AA120" s="15" t="n">
-        <v>-5648971481</v>
+        <v>-5625434981</v>
       </c>
       <c r="AB120" s="15" t="n">
-        <v>-332292.4400588235</v>
+        <v>-330907.9400588235</v>
       </c>
       <c r="AC120" s="15" t="n">
-        <v>-29888737.994709</v>
+        <v>-29764206.24867725</v>
       </c>
       <c r="AD120" s="15" t="n">
         <v>-2950000</v>
@@ -9613,13 +9619,13 @@
         <v>-15608.46560846561</v>
       </c>
       <c r="AG120" s="15" t="n">
-        <v>-5651921481</v>
+        <v>-5628384981</v>
       </c>
       <c r="AH120" s="15" t="n">
-        <v>-332465.9694705882</v>
+        <v>-331081.4694705882</v>
       </c>
       <c r="AI120" s="15" t="n">
-        <v>-29904346.46031746</v>
+        <v>-29779814.71428572</v>
       </c>
     </row>
     <row r="121">
@@ -10289,17 +10295,23 @@
       <c r="AC128" s="11" t="n">
         <v>-5875121.76190476</v>
       </c>
-      <c r="AD128" s="11" t="n"/>
-      <c r="AE128" s="11" t="n"/>
-      <c r="AF128" s="11" t="n"/>
+      <c r="AD128" s="11" t="n">
+        <v>-52098966</v>
+      </c>
+      <c r="AE128" s="11" t="n">
+        <v>-3064.645058823529</v>
+      </c>
+      <c r="AF128" s="11" t="n">
+        <v>-275655.9047619047</v>
+      </c>
       <c r="AG128" s="11" t="n">
-        <v>-1110398013</v>
+        <v>-1162496979</v>
       </c>
       <c r="AH128" s="11" t="n">
-        <v>-65317.53017647059</v>
+        <v>-68382.17523529413</v>
       </c>
       <c r="AI128" s="11" t="n">
-        <v>-5875121.76190476</v>
+        <v>-6150777.666666665</v>
       </c>
     </row>
     <row r="129">
@@ -10390,22 +10402,22 @@
         <v>-132568430.7276719</v>
       </c>
       <c r="AD129" s="15" t="n">
-        <v>-15362300</v>
+        <v>-67461266</v>
       </c>
       <c r="AE129" s="15" t="n">
-        <v>-903.6647058823529</v>
+        <v>-3968.309764705883</v>
       </c>
       <c r="AF129" s="15" t="n">
-        <v>-81282.01058201058</v>
+        <v>-356937.9153439153</v>
       </c>
       <c r="AG129" s="15" t="n">
-        <v>-25070795707.53</v>
+        <v>-25122894673.53</v>
       </c>
       <c r="AH129" s="15" t="n">
-        <v>-1474752.688678235</v>
+        <v>-1477817.333737059</v>
       </c>
       <c r="AI129" s="15" t="n">
-        <v>-132649712.738254</v>
+        <v>-132925368.6430158</v>
       </c>
     </row>
     <row r="130">
@@ -11140,40 +11152,40 @@
         <v>-21392963.58698413</v>
       </c>
       <c r="X138" s="15" t="n">
-        <v>-3255746622.12</v>
+        <v>-3232210122.12</v>
       </c>
       <c r="Y138" s="15" t="n">
-        <v>-191514.5071835294</v>
+        <v>-190130.0071835294</v>
       </c>
       <c r="Z138" s="15" t="n">
-        <v>-17226172.60380952</v>
+        <v>-17101640.85777778</v>
       </c>
       <c r="AA138" s="15" t="n">
-        <v>-43545687844.43001</v>
+        <v>-43522151344.43001</v>
       </c>
       <c r="AB138" s="15" t="n">
-        <v>-2561511.049672353</v>
+        <v>-2560126.549672353</v>
       </c>
       <c r="AC138" s="15" t="n">
-        <v>-230400464.7853439</v>
+        <v>-230275933.0393122</v>
       </c>
       <c r="AD138" s="15" t="n">
-        <v>-18312300</v>
+        <v>-70411266</v>
       </c>
       <c r="AE138" s="15" t="n">
-        <v>-1077.194117647059</v>
+        <v>-4141.839176470588</v>
       </c>
       <c r="AF138" s="15" t="n">
-        <v>-96890.47619047618</v>
+        <v>-372546.3809523809</v>
       </c>
       <c r="AG138" s="15" t="n">
-        <v>-43564000144.43001</v>
+        <v>-43592562610.43001</v>
       </c>
       <c r="AH138" s="15" t="n">
-        <v>-2562588.24379</v>
+        <v>-2564268.388848823</v>
       </c>
       <c r="AI138" s="15" t="n">
-        <v>-230497355.2615344</v>
+        <v>-230648479.4202645</v>
       </c>
     </row>
     <row r="139">
@@ -12352,22 +12364,22 @@
         <v>-1529478500.653757</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-365870498</v>
+        <v>-432595564</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-21521.794</v>
+        <v>-25446.79788235294</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-1935822.740740741</v>
+        <v>-2288865.417989418</v>
       </c>
       <c r="AG153" s="19" t="n">
-        <v>-289437307121.5599</v>
+        <v>-289504032187.5599</v>
       </c>
       <c r="AH153" s="19" t="n">
-        <v>-17025723.94832706</v>
+        <v>-17029648.95220941</v>
       </c>
       <c r="AI153" s="19" t="n">
-        <v>-1531414323.394497</v>
+        <v>-1531767366.071746</v>
       </c>
     </row>
     <row r="154">
@@ -12458,22 +12470,22 @@
         <v>-349256107.4480425</v>
       </c>
       <c r="AD154" s="19" t="n">
-        <v>3500783835</v>
+        <v>3442000269</v>
       </c>
       <c r="AE154" s="19" t="n">
-        <v>205928.4608823529</v>
+        <v>202470.6040588235</v>
       </c>
       <c r="AF154" s="19" t="n">
-        <v>18522665.79365079</v>
+        <v>18211641.63492063</v>
       </c>
       <c r="AG154" s="19" t="n">
-        <v>-62508620472.68</v>
+        <v>-62567404038.68</v>
       </c>
       <c r="AH154" s="19" t="n">
-        <v>-3676977.67486353</v>
+        <v>-3680435.531687059</v>
       </c>
       <c r="AI154" s="19" t="n">
-        <v>-330733441.6543916</v>
+        <v>-331044465.8131218</v>
       </c>
     </row>
     <row r="155">
@@ -12564,22 +12576,22 @@
         <v>7747388.987724859</v>
       </c>
       <c r="AD155" s="7" t="n">
-        <v>4965040353.679998</v>
+        <v>4906256787.679998</v>
       </c>
       <c r="AE155" s="7" t="n">
-        <v>292061.197275294</v>
+        <v>288603.3404517646</v>
       </c>
       <c r="AF155" s="7" t="n">
-        <v>26270054.78137565</v>
+        <v>25959030.62264549</v>
       </c>
       <c r="AG155" s="7" t="n">
-        <v>4965040353.679998</v>
+        <v>4906256787.679998</v>
       </c>
       <c r="AH155" s="7" t="n">
-        <v>292061.197275294</v>
+        <v>288603.3404517646</v>
       </c>
       <c r="AI155" s="7" t="n">
-        <v>26270054.78137565</v>
+        <v>25959030.62264549</v>
       </c>
     </row>
   </sheetData>
@@ -13140,16 +13152,16 @@
         <v>172976399.24</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>-13405800</v>
+        <v>-72189366</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>159570599.24</v>
+        <v>100787033.24</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>9386.505837647059</v>
+        <v>5928.649014117647</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>844288.884867725</v>
+        <v>533264.7261375661</v>
       </c>
     </row>
     <row r="10">
@@ -13259,13 +13271,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>4965040355.679999</v>
+        <v>4906256789.679999</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>292061.1973929412</v>
+        <v>288603.3405694118</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>26270054.79195767</v>
+        <v>25959030.63322751</v>
       </c>
     </row>
   </sheetData>
@@ -13335,7 +13347,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 09 Sep 2026 11:45 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 09 Sep 2026 16:19 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -14795,22 +14807,22 @@
         <v>2.321849073439154</v>
       </c>
       <c r="AD20" s="13" t="n">
-        <v>5.934</v>
+        <v>13.8755</v>
       </c>
       <c r="AE20" s="13" t="n">
-        <v>0.0003490588235294118</v>
+        <v>0.0008162058823529412</v>
       </c>
       <c r="AF20" s="13" t="n">
-        <v>0.0313968253968254</v>
+        <v>0.07341534391534392</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>444.76347488</v>
+        <v>452.70497488</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>0.02616255734588235</v>
+        <v>0.02662970440470588</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>2.353245898835979</v>
+        <v>2.395264417354498</v>
       </c>
     </row>
     <row r="21">
@@ -15047,22 +15059,22 @@
         <v>0.332547619047619</v>
       </c>
       <c r="AD23" s="11" t="n">
-        <v>5.5615</v>
+        <v>13.503</v>
       </c>
       <c r="AE23" s="11" t="n">
-        <v>0.0003271470588235294</v>
+        <v>0.0007942941176470588</v>
       </c>
       <c r="AF23" s="11" t="n">
-        <v>0.02942592592592592</v>
+        <v>0.07144444444444445</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>68.413</v>
+        <v>76.3545</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>0.004024294117647059</v>
+        <v>0.004491441176470589</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>0.3619735449735449</v>
+        <v>0.4039920634920635</v>
       </c>
     </row>
     <row r="24">
@@ -16439,22 +16451,22 @@
         <v>1180.222393205714</v>
       </c>
       <c r="AD44" s="15" t="n">
-        <v>3866.654333</v>
+        <v>3874.595833</v>
       </c>
       <c r="AE44" s="15" t="n">
-        <v>0.2274502548823529</v>
+        <v>0.2279174019411765</v>
       </c>
       <c r="AF44" s="15" t="n">
-        <v>20.45848853439153</v>
+        <v>20.50050705291005</v>
       </c>
       <c r="AG44" s="15" t="n">
-        <v>226928.68664888</v>
+        <v>226936.62814888</v>
       </c>
       <c r="AH44" s="15" t="n">
-        <v>13.34874627346353</v>
+        <v>13.34921342052235</v>
       </c>
       <c r="AI44" s="15" t="n">
-        <v>1200.680881740106</v>
+        <v>1200.722900258624</v>
       </c>
     </row>
     <row r="45">
@@ -17103,34 +17115,34 @@
         <v>-1.644358121693122</v>
       </c>
       <c r="X54" s="13" t="n">
-        <v>-351.295896</v>
+        <v>-374.832396</v>
       </c>
       <c r="Y54" s="13" t="n">
-        <v>-0.02066446447058824</v>
+        <v>-0.02204896447058824</v>
       </c>
       <c r="Z54" s="13" t="n">
-        <v>-1.858708444444445</v>
+        <v>-1.98324019047619</v>
       </c>
       <c r="AA54" s="13" t="n">
-        <v>-1356.46441</v>
+        <v>-1380.00091</v>
       </c>
       <c r="AB54" s="13" t="n">
-        <v>-0.07979202411764706</v>
+        <v>-0.08117652411764706</v>
       </c>
       <c r="AC54" s="13" t="n">
-        <v>-7.177060370370371</v>
+        <v>-7.301592116402117</v>
       </c>
       <c r="AD54" s="13" t="n"/>
       <c r="AE54" s="13" t="n"/>
       <c r="AF54" s="13" t="n"/>
       <c r="AG54" s="13" t="n">
-        <v>-1356.46441</v>
+        <v>-1380.00091</v>
       </c>
       <c r="AH54" s="13" t="n">
-        <v>-0.07979202411764706</v>
+        <v>-0.08117652411764706</v>
       </c>
       <c r="AI54" s="13" t="n">
-        <v>-7.177060370370371</v>
+        <v>-7.301592116402117</v>
       </c>
     </row>
     <row r="55">
@@ -17753,34 +17765,34 @@
         <v>-4.972000248677248</v>
       </c>
       <c r="X62" s="15" t="n">
-        <v>-1669.45055</v>
+        <v>-1692.98705</v>
       </c>
       <c r="Y62" s="15" t="n">
-        <v>-0.09820297352941176</v>
+        <v>-0.09958747352941176</v>
       </c>
       <c r="Z62" s="15" t="n">
-        <v>-8.833071693121694</v>
+        <v>-8.95760343915344</v>
       </c>
       <c r="AA62" s="15" t="n">
-        <v>-15962.22468188</v>
+        <v>-15985.76118188</v>
       </c>
       <c r="AB62" s="15" t="n">
-        <v>-0.9389543930517646</v>
+        <v>-0.9403388930517647</v>
       </c>
       <c r="AC62" s="15" t="n">
-        <v>-84.45621524804233</v>
+        <v>-84.58074699407408</v>
       </c>
       <c r="AD62" s="15" t="n"/>
       <c r="AE62" s="15" t="n"/>
       <c r="AF62" s="15" t="n"/>
       <c r="AG62" s="15" t="n">
-        <v>-15962.22468188</v>
+        <v>-15985.76118188</v>
       </c>
       <c r="AH62" s="15" t="n">
-        <v>-0.9389543930517646</v>
+        <v>-0.9403388930517647</v>
       </c>
       <c r="AI62" s="15" t="n">
-        <v>-84.45621524804233</v>
+        <v>-84.58074699407408</v>
       </c>
     </row>
     <row r="63">
@@ -18938,17 +18950,23 @@
       <c r="AC81" s="13" t="n">
         <v>-48.83498968539683</v>
       </c>
-      <c r="AD81" s="13" t="n"/>
-      <c r="AE81" s="13" t="n"/>
-      <c r="AF81" s="13" t="n"/>
+      <c r="AD81" s="13" t="n">
+        <v>-14.6261</v>
+      </c>
+      <c r="AE81" s="13" t="n">
+        <v>-0.0008603588235294117</v>
+      </c>
+      <c r="AF81" s="13" t="n">
+        <v>-0.07738677248677248</v>
+      </c>
       <c r="AG81" s="13" t="n">
-        <v>-9229.813050539999</v>
+        <v>-9244.439150539998</v>
       </c>
       <c r="AH81" s="13" t="n">
-        <v>-0.5429301794435294</v>
+        <v>-0.5437905382670588</v>
       </c>
       <c r="AI81" s="13" t="n">
-        <v>-48.83498968539683</v>
+        <v>-48.9123764578836</v>
       </c>
     </row>
     <row r="82">
@@ -19239,22 +19257,22 @@
         <v>-126.3342242039153</v>
       </c>
       <c r="AD84" s="15" t="n">
-        <v>-286.804298</v>
+        <v>-301.430398</v>
       </c>
       <c r="AE84" s="15" t="n">
-        <v>-0.01687084105882353</v>
+        <v>-0.01773119988235294</v>
       </c>
       <c r="AF84" s="15" t="n">
-        <v>-1.517483058201058</v>
+        <v>-1.594869830687831</v>
       </c>
       <c r="AG84" s="15" t="n">
-        <v>-24163.97267254</v>
+        <v>-24178.59877254</v>
       </c>
       <c r="AH84" s="15" t="n">
-        <v>-1.421410157208235</v>
+        <v>-1.422270516031765</v>
       </c>
       <c r="AI84" s="15" t="n">
-        <v>-127.8517072621164</v>
+        <v>-127.9290940346032</v>
       </c>
     </row>
     <row r="85">
@@ -22085,22 +22103,22 @@
         <v>-3.58779708994709</v>
       </c>
       <c r="X119" s="11" t="n">
-        <v>-1090.252254</v>
+        <v>-1066.715754</v>
       </c>
       <c r="Y119" s="11" t="n">
-        <v>-0.06413248552941177</v>
+        <v>-0.06274798552941177</v>
       </c>
       <c r="Z119" s="11" t="n">
-        <v>-5.768530444444444</v>
+        <v>-5.643998698412699</v>
       </c>
       <c r="AA119" s="11" t="n">
-        <v>-5648.971481</v>
+        <v>-5625.434980999999</v>
       </c>
       <c r="AB119" s="11" t="n">
-        <v>-0.3322924400588235</v>
+        <v>-0.3309079400588235</v>
       </c>
       <c r="AC119" s="11" t="n">
-        <v>-29.888737994709</v>
+        <v>-29.76420624867725</v>
       </c>
       <c r="AD119" s="11" t="n">
         <v>-2.95</v>
@@ -22112,13 +22130,13 @@
         <v>-0.01560846560846561</v>
       </c>
       <c r="AG119" s="11" t="n">
-        <v>-5651.921480999999</v>
+        <v>-5628.384980999999</v>
       </c>
       <c r="AH119" s="11" t="n">
-        <v>-0.3324659694705882</v>
+        <v>-0.3310814694705882</v>
       </c>
       <c r="AI119" s="11" t="n">
-        <v>-29.90434646031746</v>
+        <v>-29.77981471428572</v>
       </c>
     </row>
     <row r="120">
@@ -22191,22 +22209,22 @@
         <v>-3.58779708994709</v>
       </c>
       <c r="X120" s="15" t="n">
-        <v>-1090.252254</v>
+        <v>-1066.715754</v>
       </c>
       <c r="Y120" s="15" t="n">
-        <v>-0.06413248552941177</v>
+        <v>-0.06274798552941177</v>
       </c>
       <c r="Z120" s="15" t="n">
-        <v>-5.768530444444444</v>
+        <v>-5.643998698412699</v>
       </c>
       <c r="AA120" s="15" t="n">
-        <v>-5648.971481</v>
+        <v>-5625.434980999999</v>
       </c>
       <c r="AB120" s="15" t="n">
-        <v>-0.3322924400588235</v>
+        <v>-0.3309079400588235</v>
       </c>
       <c r="AC120" s="15" t="n">
-        <v>-29.888737994709</v>
+        <v>-29.76420624867725</v>
       </c>
       <c r="AD120" s="15" t="n">
         <v>-2.95</v>
@@ -22218,13 +22236,13 @@
         <v>-0.01560846560846561</v>
       </c>
       <c r="AG120" s="15" t="n">
-        <v>-5651.921480999999</v>
+        <v>-5628.384980999999</v>
       </c>
       <c r="AH120" s="15" t="n">
-        <v>-0.3324659694705882</v>
+        <v>-0.3310814694705882</v>
       </c>
       <c r="AI120" s="15" t="n">
-        <v>-29.90434646031746</v>
+        <v>-29.77981471428572</v>
       </c>
     </row>
     <row r="121">
@@ -22894,17 +22912,23 @@
       <c r="AC128" s="11" t="n">
         <v>-5.875121761904762</v>
       </c>
-      <c r="AD128" s="11" t="n"/>
-      <c r="AE128" s="11" t="n"/>
-      <c r="AF128" s="11" t="n"/>
+      <c r="AD128" s="11" t="n">
+        <v>-52.098966</v>
+      </c>
+      <c r="AE128" s="11" t="n">
+        <v>-0.003064645058823529</v>
+      </c>
+      <c r="AF128" s="11" t="n">
+        <v>-0.2756559047619048</v>
+      </c>
       <c r="AG128" s="11" t="n">
-        <v>-1110.398013</v>
+        <v>-1162.496979</v>
       </c>
       <c r="AH128" s="11" t="n">
-        <v>-0.06531753017647059</v>
+        <v>-0.06838217523529412</v>
       </c>
       <c r="AI128" s="11" t="n">
-        <v>-5.875121761904762</v>
+        <v>-6.150777666666667</v>
       </c>
     </row>
     <row r="129">
@@ -22995,22 +23019,22 @@
         <v>-132.568430727672</v>
       </c>
       <c r="AD129" s="15" t="n">
-        <v>-15.3623</v>
+        <v>-67.46126599999999</v>
       </c>
       <c r="AE129" s="15" t="n">
-        <v>-0.0009036647058823529</v>
+        <v>-0.003968309764705882</v>
       </c>
       <c r="AF129" s="15" t="n">
-        <v>-0.08128201058201058</v>
+        <v>-0.3569379153439153</v>
       </c>
       <c r="AG129" s="15" t="n">
-        <v>-25070.79570753</v>
+        <v>-25122.89467353</v>
       </c>
       <c r="AH129" s="15" t="n">
-        <v>-1.474752688678236</v>
+        <v>-1.477817333737059</v>
       </c>
       <c r="AI129" s="15" t="n">
-        <v>-132.649712738254</v>
+        <v>-132.9253686430159</v>
       </c>
     </row>
     <row r="130">
@@ -23745,40 +23769,40 @@
         <v>-21.39296358698413</v>
       </c>
       <c r="X138" s="15" t="n">
-        <v>-3255.74662212</v>
+        <v>-3232.21012212</v>
       </c>
       <c r="Y138" s="15" t="n">
-        <v>-0.1915145071835294</v>
+        <v>-0.1901300071835294</v>
       </c>
       <c r="Z138" s="15" t="n">
-        <v>-17.22617260380952</v>
+        <v>-17.10164085777778</v>
       </c>
       <c r="AA138" s="15" t="n">
-        <v>-43545.68784443</v>
+        <v>-43522.15134443</v>
       </c>
       <c r="AB138" s="15" t="n">
-        <v>-2.561511049672353</v>
+        <v>-2.560126549672352</v>
       </c>
       <c r="AC138" s="15" t="n">
-        <v>-230.4004647853439</v>
+        <v>-230.2759330393122</v>
       </c>
       <c r="AD138" s="15" t="n">
-        <v>-18.3123</v>
+        <v>-70.411266</v>
       </c>
       <c r="AE138" s="15" t="n">
-        <v>-0.001077194117647059</v>
+        <v>-0.004141839176470588</v>
       </c>
       <c r="AF138" s="15" t="n">
-        <v>-0.09689047619047619</v>
+        <v>-0.372546380952381</v>
       </c>
       <c r="AG138" s="15" t="n">
-        <v>-43564.00014443</v>
+        <v>-43592.56261043</v>
       </c>
       <c r="AH138" s="15" t="n">
-        <v>-2.56258824379</v>
+        <v>-2.564268388848823</v>
       </c>
       <c r="AI138" s="15" t="n">
-        <v>-230.4973552615344</v>
+        <v>-230.6484794202645</v>
       </c>
     </row>
     <row r="139">
@@ -24957,22 +24981,22 @@
         <v>-1529.478500653756</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-365.870498</v>
+        <v>-432.595564</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-0.021521794</v>
+        <v>-0.02544679788235294</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-1.935822740740741</v>
+        <v>-2.288865417989418</v>
       </c>
       <c r="AG153" s="19" t="n">
-        <v>-289437.3071215599</v>
+        <v>-289504.0321875599</v>
       </c>
       <c r="AH153" s="19" t="n">
-        <v>-17.02572394832706</v>
+        <v>-17.02964895220941</v>
       </c>
       <c r="AI153" s="19" t="n">
-        <v>-1531.414323394497</v>
+        <v>-1531.767366071746</v>
       </c>
     </row>
     <row r="154">
@@ -25063,22 +25087,22 @@
         <v>-349.2561074480424</v>
       </c>
       <c r="AD154" s="19" t="n">
-        <v>3500.783835</v>
+        <v>3442.000269</v>
       </c>
       <c r="AE154" s="19" t="n">
-        <v>0.2059284608823529</v>
+        <v>0.2024706040588235</v>
       </c>
       <c r="AF154" s="19" t="n">
-        <v>18.52266579365079</v>
+        <v>18.21164163492064</v>
       </c>
       <c r="AG154" s="19" t="n">
-        <v>-62508.62047268001</v>
+        <v>-62567.40403868002</v>
       </c>
       <c r="AH154" s="19" t="n">
-        <v>-3.67697767486353</v>
+        <v>-3.68043553168706</v>
       </c>
       <c r="AI154" s="19" t="n">
-        <v>-330.7334416543916</v>
+        <v>-331.0444658131218</v>
       </c>
     </row>
     <row r="155">
@@ -25169,22 +25193,22 @@
         <v>7.747388987724859</v>
       </c>
       <c r="AD155" s="7" t="n">
-        <v>4965.040353679999</v>
+        <v>4906.256787679999</v>
       </c>
       <c r="AE155" s="7" t="n">
-        <v>0.2920611972752941</v>
+        <v>0.2886033404517646</v>
       </c>
       <c r="AF155" s="7" t="n">
-        <v>26.27005478137565</v>
+        <v>25.9590306226455</v>
       </c>
       <c r="AG155" s="7" t="n">
-        <v>4965.040353679999</v>
+        <v>4906.256787679999</v>
       </c>
       <c r="AH155" s="7" t="n">
-        <v>0.2920611972752941</v>
+        <v>0.2886033404517646</v>
       </c>
       <c r="AI155" s="7" t="n">
-        <v>26.27005478137565</v>
+        <v>25.9590306226455</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Fri 09/11/2026 16:51
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 09 Sep 2026 16:19</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 11 Sep 2026 16:51</t>
         </is>
       </c>
     </row>
@@ -805,14 +805,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 09 Sep 2026</t>
+          <t>MTD as of 11 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 09 Sep 2026</t>
+          <t>YTD as of 11 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
@@ -1220,22 +1220,22 @@
         <v>914323824.5555556</v>
       </c>
       <c r="AD7" s="11" t="n">
-        <v>3860720333</v>
+        <v>9886718086</v>
       </c>
       <c r="AE7" s="11" t="n">
-        <v>227101.1960588235</v>
+        <v>581571.6521176471</v>
       </c>
       <c r="AF7" s="11" t="n">
-        <v>20427091.70899471</v>
+        <v>52310677.7037037</v>
       </c>
       <c r="AG7" s="11" t="n">
-        <v>176667923174</v>
+        <v>182693920927</v>
       </c>
       <c r="AH7" s="11" t="n">
-        <v>10392230.77494118</v>
+        <v>10746701.231</v>
       </c>
       <c r="AI7" s="11" t="n">
-        <v>934750916.2645503</v>
+        <v>966634502.2592592</v>
       </c>
     </row>
     <row r="8">
@@ -1501,17 +1501,23 @@
       <c r="AC10" s="13" t="n">
         <v>183298395.3015873</v>
       </c>
-      <c r="AD10" s="13" t="n"/>
-      <c r="AE10" s="13" t="n"/>
-      <c r="AF10" s="13" t="n"/>
+      <c r="AD10" s="13" t="n">
+        <v>6025997753</v>
+      </c>
+      <c r="AE10" s="13" t="n">
+        <v>354470.4560588235</v>
+      </c>
+      <c r="AF10" s="13" t="n">
+        <v>31883585.994709</v>
+      </c>
       <c r="AG10" s="13" t="n">
-        <v>34643396712</v>
+        <v>40669394465</v>
       </c>
       <c r="AH10" s="13" t="n">
-        <v>2037846.865411765</v>
+        <v>2392317.321470588</v>
       </c>
       <c r="AI10" s="13" t="n">
-        <v>183298395.3015873</v>
+        <v>215181981.2962963</v>
       </c>
     </row>
     <row r="11">
@@ -2190,22 +2196,22 @@
         <v>2321849.073439153</v>
       </c>
       <c r="AD20" s="13" t="n">
-        <v>13875500</v>
+        <v>14901000</v>
       </c>
       <c r="AE20" s="13" t="n">
-        <v>816.2058823529412</v>
+        <v>876.5294117647059</v>
       </c>
       <c r="AF20" s="13" t="n">
-        <v>73415.34391534391</v>
+        <v>78841.26984126984</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>452704974.88</v>
+        <v>453730474.88</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>26629.70440470588</v>
+        <v>26690.02793411765</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>2395264.417354497</v>
+        <v>2400690.343280423</v>
       </c>
     </row>
     <row r="21">
@@ -2442,22 +2448,22 @@
         <v>332547.6190476191</v>
       </c>
       <c r="AD23" s="11" t="n">
-        <v>13503000</v>
+        <v>14528500</v>
       </c>
       <c r="AE23" s="11" t="n">
-        <v>794.2941176470588</v>
+        <v>854.6176470588235</v>
       </c>
       <c r="AF23" s="11" t="n">
-        <v>71444.44444444444</v>
+        <v>76870.37037037036</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>76354500</v>
+        <v>77380000</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>4491.441176470587</v>
+        <v>4551.764705882352</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>403992.0634920635</v>
+        <v>409417.9894179894</v>
       </c>
     </row>
     <row r="24">
@@ -3834,22 +3840,22 @@
         <v>1180222393.205714</v>
       </c>
       <c r="AD44" s="15" t="n">
-        <v>3874595833</v>
+        <v>9901619086</v>
       </c>
       <c r="AE44" s="15" t="n">
-        <v>227917.4019411765</v>
+        <v>582448.1815294118</v>
       </c>
       <c r="AF44" s="15" t="n">
-        <v>20500507.05291005</v>
+        <v>52389518.97354497</v>
       </c>
       <c r="AG44" s="15" t="n">
-        <v>226936628148.88</v>
+        <v>232963651401.88</v>
       </c>
       <c r="AH44" s="15" t="n">
-        <v>13349213.42052235</v>
+        <v>13703744.20011059</v>
       </c>
       <c r="AI44" s="15" t="n">
-        <v>1200722900.258625</v>
+        <v>1232611912.17926</v>
       </c>
     </row>
     <row r="45">
@@ -4083,17 +4089,23 @@
       <c r="AC48" s="13" t="n">
         <v>-825541.3492063492</v>
       </c>
-      <c r="AD48" s="13" t="n"/>
-      <c r="AE48" s="13" t="n"/>
-      <c r="AF48" s="13" t="n"/>
+      <c r="AD48" s="13" t="n">
+        <v>-4900000</v>
+      </c>
+      <c r="AE48" s="13" t="n">
+        <v>-288.2352941176471</v>
+      </c>
+      <c r="AF48" s="13" t="n">
+        <v>-25925.92592592593</v>
+      </c>
       <c r="AG48" s="13" t="n">
-        <v>-156027315</v>
+        <v>-160927315</v>
       </c>
       <c r="AH48" s="13" t="n">
-        <v>-9178.077352941176</v>
+        <v>-9466.312647058823</v>
       </c>
       <c r="AI48" s="13" t="n">
-        <v>-825541.3492063492</v>
+        <v>-851467.2751322752</v>
       </c>
     </row>
     <row r="49">
@@ -4235,17 +4247,23 @@
       <c r="AC50" s="13" t="n">
         <v>-9414012.693121692</v>
       </c>
-      <c r="AD50" s="13" t="n"/>
-      <c r="AE50" s="13" t="n"/>
-      <c r="AF50" s="13" t="n"/>
+      <c r="AD50" s="13" t="n">
+        <v>-278451550</v>
+      </c>
+      <c r="AE50" s="13" t="n">
+        <v>-16379.50294117647</v>
+      </c>
+      <c r="AF50" s="13" t="n">
+        <v>-1473288.624338624</v>
+      </c>
       <c r="AG50" s="13" t="n">
-        <v>-1779248399</v>
+        <v>-2057699949</v>
       </c>
       <c r="AH50" s="13" t="n">
-        <v>-104661.6705294118</v>
+        <v>-121041.1734705882</v>
       </c>
       <c r="AI50" s="13" t="n">
-        <v>-9414012.693121692</v>
+        <v>-10887301.31746032</v>
       </c>
     </row>
     <row r="51">
@@ -4515,17 +4533,23 @@
       <c r="AC54" s="13" t="n">
         <v>-7301592.116402116</v>
       </c>
-      <c r="AD54" s="13" t="n"/>
-      <c r="AE54" s="13" t="n"/>
-      <c r="AF54" s="13" t="n"/>
+      <c r="AD54" s="13" t="n">
+        <v>-522213844</v>
+      </c>
+      <c r="AE54" s="13" t="n">
+        <v>-30718.46141176471</v>
+      </c>
+      <c r="AF54" s="13" t="n">
+        <v>-2763036.211640212</v>
+      </c>
       <c r="AG54" s="13" t="n">
-        <v>-1380000910</v>
+        <v>-1902214754</v>
       </c>
       <c r="AH54" s="13" t="n">
-        <v>-81176.52411764706</v>
+        <v>-111894.9855294118</v>
       </c>
       <c r="AI54" s="13" t="n">
-        <v>-7301592.116402116</v>
+        <v>-10064628.32804233</v>
       </c>
     </row>
     <row r="55">
@@ -4755,17 +4779,23 @@
       <c r="AC57" s="11" t="n">
         <v>-1331501.074074074</v>
       </c>
-      <c r="AD57" s="11" t="n"/>
-      <c r="AE57" s="11" t="n"/>
-      <c r="AF57" s="11" t="n"/>
+      <c r="AD57" s="11" t="n">
+        <v>-19870000</v>
+      </c>
+      <c r="AE57" s="11" t="n">
+        <v>-1168.823529411765</v>
+      </c>
+      <c r="AF57" s="11" t="n">
+        <v>-105132.2751322751</v>
+      </c>
       <c r="AG57" s="11" t="n">
-        <v>-251653703</v>
+        <v>-271523703</v>
       </c>
       <c r="AH57" s="11" t="n">
-        <v>-14803.159</v>
+        <v>-15971.98252941176</v>
       </c>
       <c r="AI57" s="11" t="n">
-        <v>-1331501.074074074</v>
+        <v>-1436633.349206349</v>
       </c>
     </row>
     <row r="58">
@@ -4855,17 +4885,23 @@
       <c r="AC58" s="13" t="n">
         <v>-15896342.83005291</v>
       </c>
-      <c r="AD58" s="13" t="n"/>
-      <c r="AE58" s="13" t="n"/>
-      <c r="AF58" s="13" t="n"/>
+      <c r="AD58" s="13" t="n">
+        <v>-53391331</v>
+      </c>
+      <c r="AE58" s="13" t="n">
+        <v>-3140.666529411765</v>
+      </c>
+      <c r="AF58" s="13" t="n">
+        <v>-282493.8148148148</v>
+      </c>
       <c r="AG58" s="13" t="n">
-        <v>-3004408794.88</v>
+        <v>-3057800125.88</v>
       </c>
       <c r="AH58" s="13" t="n">
-        <v>-176729.9291105882</v>
+        <v>-179870.59564</v>
       </c>
       <c r="AI58" s="13" t="n">
-        <v>-15896342.83005291</v>
+        <v>-16178836.64486773</v>
       </c>
     </row>
     <row r="59">
@@ -5165,17 +5201,23 @@
       <c r="AC62" s="15" t="n">
         <v>-84580746.99407408</v>
       </c>
-      <c r="AD62" s="15" t="n"/>
-      <c r="AE62" s="15" t="n"/>
-      <c r="AF62" s="15" t="n"/>
+      <c r="AD62" s="15" t="n">
+        <v>-878826725</v>
+      </c>
+      <c r="AE62" s="15" t="n">
+        <v>-51695.68970588235</v>
+      </c>
+      <c r="AF62" s="15" t="n">
+        <v>-4649876.851851852</v>
+      </c>
       <c r="AG62" s="15" t="n">
-        <v>-15985761181.88</v>
+        <v>-16864587906.88</v>
       </c>
       <c r="AH62" s="15" t="n">
-        <v>-940338.8930517647</v>
+        <v>-992034.582757647</v>
       </c>
       <c r="AI62" s="15" t="n">
-        <v>-84580746.99407408</v>
+        <v>-89230623.84592593</v>
       </c>
     </row>
     <row r="63">
@@ -6228,22 +6270,22 @@
         <v>-35112264.4074074</v>
       </c>
       <c r="AD80" s="11" t="n">
-        <v>-286804298</v>
+        <v>-1088054516</v>
       </c>
       <c r="AE80" s="11" t="n">
-        <v>-16870.84105882353</v>
+        <v>-64003.20682352941</v>
       </c>
       <c r="AF80" s="11" t="n">
-        <v>-1517483.058201058</v>
+        <v>-5756902.201058201</v>
       </c>
       <c r="AG80" s="11" t="n">
-        <v>-6923022271</v>
+        <v>-7724272489</v>
       </c>
       <c r="AH80" s="11" t="n">
-        <v>-407236.6041764705</v>
+        <v>-454368.9699411764</v>
       </c>
       <c r="AI80" s="11" t="n">
-        <v>-36629747.46560846</v>
+        <v>-40869166.6084656</v>
       </c>
     </row>
     <row r="81">
@@ -6334,22 +6376,22 @@
         <v>-48834989.68539683</v>
       </c>
       <c r="AD81" s="13" t="n">
-        <v>-14626100</v>
+        <v>-1301257365</v>
       </c>
       <c r="AE81" s="13" t="n">
-        <v>-860.3588235294118</v>
+        <v>-76544.55088235294</v>
       </c>
       <c r="AF81" s="13" t="n">
-        <v>-77386.77248677249</v>
+        <v>-6884959.603174604</v>
       </c>
       <c r="AG81" s="13" t="n">
-        <v>-9244439150.540001</v>
+        <v>-10531070415.54</v>
       </c>
       <c r="AH81" s="13" t="n">
-        <v>-543790.5382670588</v>
+        <v>-619474.7303258823</v>
       </c>
       <c r="AI81" s="13" t="n">
-        <v>-48912376.4578836</v>
+        <v>-55719949.28857143</v>
       </c>
     </row>
     <row r="82">
@@ -6539,17 +6581,23 @@
       <c r="AC83" s="13" t="n">
         <v>-2053284.693121693</v>
       </c>
-      <c r="AD83" s="13" t="n"/>
-      <c r="AE83" s="13" t="n"/>
-      <c r="AF83" s="13" t="n"/>
+      <c r="AD83" s="13" t="n">
+        <v>-4255960</v>
+      </c>
+      <c r="AE83" s="13" t="n">
+        <v>-250.3505882352941</v>
+      </c>
+      <c r="AF83" s="13" t="n">
+        <v>-22518.30687830688</v>
+      </c>
       <c r="AG83" s="13" t="n">
-        <v>-388070807</v>
+        <v>-392326767</v>
       </c>
       <c r="AH83" s="13" t="n">
-        <v>-22827.69452941177</v>
+        <v>-23078.04511764706</v>
       </c>
       <c r="AI83" s="13" t="n">
-        <v>-2053284.693121693</v>
+        <v>-2075803</v>
       </c>
     </row>
     <row r="84">
@@ -6640,22 +6688,22 @@
         <v>-126334224.2039154</v>
       </c>
       <c r="AD84" s="15" t="n">
-        <v>-301430398</v>
+        <v>-2393567841</v>
       </c>
       <c r="AE84" s="15" t="n">
-        <v>-17731.19988235294</v>
+        <v>-140798.1082941176</v>
       </c>
       <c r="AF84" s="15" t="n">
-        <v>-1594869.830687831</v>
+        <v>-12664380.11111111</v>
       </c>
       <c r="AG84" s="15" t="n">
-        <v>-24178598772.54</v>
+        <v>-26270736215.54</v>
       </c>
       <c r="AH84" s="15" t="n">
-        <v>-1422270.516031765</v>
+        <v>-1545337.42444353</v>
       </c>
       <c r="AI84" s="15" t="n">
-        <v>-127929094.0346032</v>
+        <v>-138998604.3150265</v>
       </c>
     </row>
     <row r="85">
@@ -6825,17 +6873,23 @@
       <c r="AC87" s="11" t="n">
         <v>-716669.634920635</v>
       </c>
-      <c r="AD87" s="11" t="n"/>
-      <c r="AE87" s="11" t="n"/>
-      <c r="AF87" s="11" t="n"/>
+      <c r="AD87" s="11" t="n">
+        <v>-735172</v>
+      </c>
+      <c r="AE87" s="11" t="n">
+        <v>-43.24541176470589</v>
+      </c>
+      <c r="AF87" s="11" t="n">
+        <v>-3889.798941798942</v>
+      </c>
       <c r="AG87" s="11" t="n">
-        <v>-135450561</v>
+        <v>-136185733</v>
       </c>
       <c r="AH87" s="11" t="n">
-        <v>-7967.68005882353</v>
+        <v>-8010.925470588236</v>
       </c>
       <c r="AI87" s="11" t="n">
-        <v>-716669.634920635</v>
+        <v>-720559.433862434</v>
       </c>
     </row>
     <row r="88">
@@ -6959,17 +7013,23 @@
       <c r="AC89" s="11" t="n">
         <v>-42218.01587301587</v>
       </c>
-      <c r="AD89" s="11" t="n"/>
-      <c r="AE89" s="11" t="n"/>
-      <c r="AF89" s="11" t="n"/>
+      <c r="AD89" s="11" t="n">
+        <v>-5785771</v>
+      </c>
+      <c r="AE89" s="11" t="n">
+        <v>-340.3394705882353</v>
+      </c>
+      <c r="AF89" s="11" t="n">
+        <v>-30612.54497354497</v>
+      </c>
       <c r="AG89" s="11" t="n">
-        <v>-7979205</v>
+        <v>-13764976</v>
       </c>
       <c r="AH89" s="11" t="n">
-        <v>-469.3650000000001</v>
+        <v>-809.7044705882354</v>
       </c>
       <c r="AI89" s="11" t="n">
-        <v>-42218.01587301587</v>
+        <v>-72830.56084656084</v>
       </c>
     </row>
     <row r="90">
@@ -7029,17 +7089,23 @@
       <c r="AC90" s="13" t="n">
         <v>-8627.340952380953</v>
       </c>
-      <c r="AD90" s="13" t="n"/>
-      <c r="AE90" s="13" t="n"/>
-      <c r="AF90" s="13" t="n"/>
+      <c r="AD90" s="13" t="n">
+        <v>-40000</v>
+      </c>
+      <c r="AE90" s="13" t="n">
+        <v>-2.352941176470588</v>
+      </c>
+      <c r="AF90" s="13" t="n">
+        <v>-211.6402116402116</v>
+      </c>
       <c r="AG90" s="13" t="n">
-        <v>-1630567.44</v>
+        <v>-1670567.44</v>
       </c>
       <c r="AH90" s="13" t="n">
-        <v>-95.91573176470587</v>
+        <v>-98.26867294117646</v>
       </c>
       <c r="AI90" s="13" t="n">
-        <v>-8627.340952380953</v>
+        <v>-8838.981164021165</v>
       </c>
     </row>
     <row r="91">
@@ -7129,17 +7195,23 @@
       <c r="AC91" s="11" t="n">
         <v>-686517.0158730159</v>
       </c>
-      <c r="AD91" s="11" t="n"/>
-      <c r="AE91" s="11" t="n"/>
-      <c r="AF91" s="11" t="n"/>
+      <c r="AD91" s="11" t="n">
+        <v>-195400</v>
+      </c>
+      <c r="AE91" s="11" t="n">
+        <v>-11.49411764705882</v>
+      </c>
+      <c r="AF91" s="11" t="n">
+        <v>-1033.862433862434</v>
+      </c>
       <c r="AG91" s="11" t="n">
-        <v>-129751716</v>
+        <v>-129947116</v>
       </c>
       <c r="AH91" s="11" t="n">
-        <v>-7632.45388235294</v>
+        <v>-7643.947999999999</v>
       </c>
       <c r="AI91" s="11" t="n">
-        <v>-686517.0158730159</v>
+        <v>-687550.8783068783</v>
       </c>
     </row>
     <row r="92">
@@ -7217,17 +7289,23 @@
       <c r="AC92" s="13" t="n">
         <v>-11280.93121693122</v>
       </c>
-      <c r="AD92" s="13" t="n"/>
-      <c r="AE92" s="13" t="n"/>
-      <c r="AF92" s="13" t="n"/>
+      <c r="AD92" s="13" t="n">
+        <v>-185600</v>
+      </c>
+      <c r="AE92" s="13" t="n">
+        <v>-10.91764705882353</v>
+      </c>
+      <c r="AF92" s="13" t="n">
+        <v>-982.010582010582</v>
+      </c>
       <c r="AG92" s="13" t="n">
-        <v>-2132096</v>
+        <v>-2317696</v>
       </c>
       <c r="AH92" s="13" t="n">
-        <v>-125.4174117647059</v>
+        <v>-136.3350588235294</v>
       </c>
       <c r="AI92" s="13" t="n">
-        <v>-11280.93121693122</v>
+        <v>-12262.9417989418</v>
       </c>
     </row>
     <row r="93">
@@ -7317,17 +7395,23 @@
       <c r="AC93" s="15" t="n">
         <v>-1479210.293333333</v>
       </c>
-      <c r="AD93" s="15" t="n"/>
-      <c r="AE93" s="15" t="n"/>
-      <c r="AF93" s="15" t="n"/>
+      <c r="AD93" s="15" t="n">
+        <v>-6941943</v>
+      </c>
+      <c r="AE93" s="15" t="n">
+        <v>-408.3495882352941</v>
+      </c>
+      <c r="AF93" s="15" t="n">
+        <v>-36729.85714285714</v>
+      </c>
       <c r="AG93" s="15" t="n">
-        <v>-279570745.44</v>
+        <v>-286512688.44</v>
       </c>
       <c r="AH93" s="15" t="n">
-        <v>-16445.33796705883</v>
+        <v>-16853.68755529412</v>
       </c>
       <c r="AI93" s="15" t="n">
-        <v>-1479210.293333333</v>
+        <v>-1515940.15047619</v>
       </c>
     </row>
     <row r="94">
@@ -7539,17 +7623,23 @@
       <c r="AC96" s="13" t="n">
         <v>-1044235.444444444</v>
       </c>
-      <c r="AD96" s="13" t="n"/>
-      <c r="AE96" s="13" t="n"/>
-      <c r="AF96" s="13" t="n"/>
+      <c r="AD96" s="13" t="n">
+        <v>-62917000</v>
+      </c>
+      <c r="AE96" s="13" t="n">
+        <v>-3701</v>
+      </c>
+      <c r="AF96" s="13" t="n">
+        <v>-332894.1798941799</v>
+      </c>
       <c r="AG96" s="13" t="n">
-        <v>-197360499</v>
+        <v>-260277499</v>
       </c>
       <c r="AH96" s="13" t="n">
-        <v>-11609.44111764706</v>
+        <v>-15310.44111764706</v>
       </c>
       <c r="AI96" s="13" t="n">
-        <v>-1044235.444444444</v>
+        <v>-1377129.624338624</v>
       </c>
     </row>
     <row r="97">
@@ -7639,17 +7729,23 @@
       <c r="AC97" s="11" t="n">
         <v>-37066593.81195767</v>
       </c>
-      <c r="AD97" s="11" t="n"/>
-      <c r="AE97" s="11" t="n"/>
-      <c r="AF97" s="11" t="n"/>
+      <c r="AD97" s="11" t="n">
+        <v>-10078098</v>
+      </c>
+      <c r="AE97" s="11" t="n">
+        <v>-592.829294117647</v>
+      </c>
+      <c r="AF97" s="11" t="n">
+        <v>-53323.26984126984</v>
+      </c>
       <c r="AG97" s="11" t="n">
-        <v>-7005586230.46</v>
+        <v>-7015664328.46</v>
       </c>
       <c r="AH97" s="11" t="n">
-        <v>-412093.3076741177</v>
+        <v>-412686.1369682353</v>
       </c>
       <c r="AI97" s="11" t="n">
-        <v>-37066593.81195767</v>
+        <v>-37119917.08179894</v>
       </c>
     </row>
     <row r="98">
@@ -7739,17 +7835,23 @@
       <c r="AC98" s="13" t="n">
         <v>-1168025.571428571</v>
       </c>
-      <c r="AD98" s="13" t="n"/>
-      <c r="AE98" s="13" t="n"/>
-      <c r="AF98" s="13" t="n"/>
+      <c r="AD98" s="13" t="n">
+        <v>-63412411</v>
+      </c>
+      <c r="AE98" s="13" t="n">
+        <v>-3730.141823529412</v>
+      </c>
+      <c r="AF98" s="13" t="n">
+        <v>-335515.4021164021</v>
+      </c>
       <c r="AG98" s="13" t="n">
-        <v>-220756833</v>
+        <v>-284169244</v>
       </c>
       <c r="AH98" s="13" t="n">
-        <v>-12985.69605882353</v>
+        <v>-16715.83788235294</v>
       </c>
       <c r="AI98" s="13" t="n">
-        <v>-1168025.571428571</v>
+        <v>-1503540.973544973</v>
       </c>
     </row>
     <row r="99">
@@ -7839,17 +7941,23 @@
       <c r="AC99" s="11" t="n">
         <v>-1762867.232804233</v>
       </c>
-      <c r="AD99" s="11" t="n"/>
-      <c r="AE99" s="11" t="n"/>
-      <c r="AF99" s="11" t="n"/>
+      <c r="AD99" s="11" t="n">
+        <v>-9445000</v>
+      </c>
+      <c r="AE99" s="11" t="n">
+        <v>-555.5882352941177</v>
+      </c>
+      <c r="AF99" s="11" t="n">
+        <v>-49973.54497354497</v>
+      </c>
       <c r="AG99" s="11" t="n">
-        <v>-333181907</v>
+        <v>-342626907</v>
       </c>
       <c r="AH99" s="11" t="n">
-        <v>-19598.93570588235</v>
+        <v>-20154.52394117647</v>
       </c>
       <c r="AI99" s="11" t="n">
-        <v>-1762867.232804233</v>
+        <v>-1812840.777777778</v>
       </c>
     </row>
     <row r="100">
@@ -7939,17 +8047,23 @@
       <c r="AC100" s="15" t="n">
         <v>-41513173.38338625</v>
       </c>
-      <c r="AD100" s="15" t="n"/>
-      <c r="AE100" s="15" t="n"/>
-      <c r="AF100" s="15" t="n"/>
+      <c r="AD100" s="15" t="n">
+        <v>-145852509</v>
+      </c>
+      <c r="AE100" s="15" t="n">
+        <v>-8579.559352941176</v>
+      </c>
+      <c r="AF100" s="15" t="n">
+        <v>-771706.3968253968</v>
+      </c>
       <c r="AG100" s="15" t="n">
-        <v>-7845989769.46</v>
+        <v>-7991842278.46</v>
       </c>
       <c r="AH100" s="15" t="n">
-        <v>-461528.8099682353</v>
+        <v>-470108.3693211764</v>
       </c>
       <c r="AI100" s="15" t="n">
-        <v>-41513173.38338625</v>
+        <v>-42284879.78021164</v>
       </c>
     </row>
     <row r="101">
@@ -8079,17 +8193,23 @@
       <c r="AC102" s="11" t="n">
         <v>-1060289.031746032</v>
       </c>
-      <c r="AD102" s="11" t="n"/>
-      <c r="AE102" s="11" t="n"/>
-      <c r="AF102" s="11" t="n"/>
+      <c r="AD102" s="11" t="n">
+        <v>-15975200</v>
+      </c>
+      <c r="AE102" s="11" t="n">
+        <v>-939.7176470588236</v>
+      </c>
+      <c r="AF102" s="11" t="n">
+        <v>-84524.86772486773</v>
+      </c>
       <c r="AG102" s="11" t="n">
-        <v>-200394627</v>
+        <v>-216369827</v>
       </c>
       <c r="AH102" s="11" t="n">
-        <v>-11787.91923529412</v>
+        <v>-12727.63688235294</v>
       </c>
       <c r="AI102" s="11" t="n">
-        <v>-1060289.031746032</v>
+        <v>-1144813.899470899</v>
       </c>
     </row>
     <row r="103">
@@ -8179,17 +8299,23 @@
       <c r="AC103" s="13" t="n">
         <v>-1561337.105820106</v>
       </c>
-      <c r="AD103" s="13" t="n"/>
-      <c r="AE103" s="13" t="n"/>
-      <c r="AF103" s="13" t="n"/>
+      <c r="AD103" s="13" t="n">
+        <v>-32770247</v>
+      </c>
+      <c r="AE103" s="13" t="n">
+        <v>-1927.661588235294</v>
+      </c>
+      <c r="AF103" s="13" t="n">
+        <v>-173387.5502645503</v>
+      </c>
       <c r="AG103" s="13" t="n">
-        <v>-295092713</v>
+        <v>-327862960</v>
       </c>
       <c r="AH103" s="13" t="n">
-        <v>-17358.39488235294</v>
+        <v>-19286.05647058824</v>
       </c>
       <c r="AI103" s="13" t="n">
-        <v>-1561337.105820106</v>
+        <v>-1734724.656084656</v>
       </c>
     </row>
     <row r="104">
@@ -8279,17 +8405,23 @@
       <c r="AC104" s="11" t="n">
         <v>-7974517.291005291</v>
       </c>
-      <c r="AD104" s="11" t="n"/>
-      <c r="AE104" s="11" t="n"/>
-      <c r="AF104" s="11" t="n"/>
+      <c r="AD104" s="11" t="n">
+        <v>-37147399</v>
+      </c>
+      <c r="AE104" s="11" t="n">
+        <v>-2185.141117647059</v>
+      </c>
+      <c r="AF104" s="11" t="n">
+        <v>-196547.0846560847</v>
+      </c>
       <c r="AG104" s="11" t="n">
-        <v>-1507183768</v>
+        <v>-1544331167</v>
       </c>
       <c r="AH104" s="11" t="n">
-        <v>-88657.86870588236</v>
+        <v>-90843.00982352941</v>
       </c>
       <c r="AI104" s="11" t="n">
-        <v>-7974517.291005291</v>
+        <v>-8171064.375661376</v>
       </c>
     </row>
     <row r="105">
@@ -8473,17 +8605,23 @@
       <c r="AC106" s="15" t="n">
         <v>-11650057.79365079</v>
       </c>
-      <c r="AD106" s="15" t="n"/>
-      <c r="AE106" s="15" t="n"/>
-      <c r="AF106" s="15" t="n"/>
+      <c r="AD106" s="15" t="n">
+        <v>-85892846</v>
+      </c>
+      <c r="AE106" s="15" t="n">
+        <v>-5052.520352941176</v>
+      </c>
+      <c r="AF106" s="15" t="n">
+        <v>-454459.5026455026</v>
+      </c>
       <c r="AG106" s="15" t="n">
-        <v>-2201860923</v>
+        <v>-2287753769</v>
       </c>
       <c r="AH106" s="15" t="n">
-        <v>-129521.2307647059</v>
+        <v>-134573.7511176471</v>
       </c>
       <c r="AI106" s="15" t="n">
-        <v>-11650057.79365079</v>
+        <v>-12104517.2962963</v>
       </c>
     </row>
     <row r="107">
@@ -8671,17 +8809,23 @@
       <c r="AC109" s="13" t="n">
         <v>-43589.94708994709</v>
       </c>
-      <c r="AD109" s="13" t="n"/>
-      <c r="AE109" s="13" t="n"/>
-      <c r="AF109" s="13" t="n"/>
+      <c r="AD109" s="13" t="n">
+        <v>-487500</v>
+      </c>
+      <c r="AE109" s="13" t="n">
+        <v>-28.67647058823529</v>
+      </c>
+      <c r="AF109" s="13" t="n">
+        <v>-2579.36507936508</v>
+      </c>
       <c r="AG109" s="13" t="n">
-        <v>-8238500</v>
+        <v>-8726000</v>
       </c>
       <c r="AH109" s="13" t="n">
-        <v>-484.6176470588235</v>
+        <v>-513.2941176470588</v>
       </c>
       <c r="AI109" s="13" t="n">
-        <v>-43589.94708994709</v>
+        <v>-46169.31216931217</v>
       </c>
     </row>
     <row r="110">
@@ -8771,17 +8915,23 @@
       <c r="AC110" s="11" t="n">
         <v>-2481355.084656085</v>
       </c>
-      <c r="AD110" s="11" t="n"/>
-      <c r="AE110" s="11" t="n"/>
-      <c r="AF110" s="11" t="n"/>
+      <c r="AD110" s="11" t="n">
+        <v>-22442800</v>
+      </c>
+      <c r="AE110" s="11" t="n">
+        <v>-1320.164705882353</v>
+      </c>
+      <c r="AF110" s="11" t="n">
+        <v>-118744.9735449735</v>
+      </c>
       <c r="AG110" s="11" t="n">
-        <v>-468976111</v>
+        <v>-491418911</v>
       </c>
       <c r="AH110" s="11" t="n">
-        <v>-27586.83005882353</v>
+        <v>-28906.99476470588</v>
       </c>
       <c r="AI110" s="11" t="n">
-        <v>-2481355.084656085</v>
+        <v>-2600100.058201058</v>
       </c>
     </row>
     <row r="111">
@@ -8871,17 +9021,23 @@
       <c r="AC111" s="15" t="n">
         <v>-3272307.994708994</v>
       </c>
-      <c r="AD111" s="15" t="n"/>
-      <c r="AE111" s="15" t="n"/>
-      <c r="AF111" s="15" t="n"/>
+      <c r="AD111" s="15" t="n">
+        <v>-22930300</v>
+      </c>
+      <c r="AE111" s="15" t="n">
+        <v>-1348.841176470588</v>
+      </c>
+      <c r="AF111" s="15" t="n">
+        <v>-121324.3386243386</v>
+      </c>
       <c r="AG111" s="15" t="n">
-        <v>-618466211</v>
+        <v>-641396511</v>
       </c>
       <c r="AH111" s="15" t="n">
-        <v>-36380.36535294117</v>
+        <v>-37729.20652941176</v>
       </c>
       <c r="AI111" s="15" t="n">
-        <v>-3272307.994708994</v>
+        <v>-3393632.333333333</v>
       </c>
     </row>
     <row r="112">
@@ -9263,17 +9419,23 @@
       <c r="AC116" s="13" t="n">
         <v>-2608159.126984127</v>
       </c>
-      <c r="AD116" s="13" t="n"/>
-      <c r="AE116" s="13" t="n"/>
-      <c r="AF116" s="13" t="n"/>
+      <c r="AD116" s="13" t="n">
+        <v>-16713035</v>
+      </c>
+      <c r="AE116" s="13" t="n">
+        <v>-983.1197058823529</v>
+      </c>
+      <c r="AF116" s="13" t="n">
+        <v>-88428.75661375662</v>
+      </c>
       <c r="AG116" s="13" t="n">
-        <v>-492942075</v>
+        <v>-509655110</v>
       </c>
       <c r="AH116" s="13" t="n">
-        <v>-28996.59264705883</v>
+        <v>-29979.71235294118</v>
       </c>
       <c r="AI116" s="13" t="n">
-        <v>-2608159.126984127</v>
+        <v>-2696587.883597883</v>
       </c>
     </row>
     <row r="117">
@@ -9363,17 +9525,23 @@
       <c r="AC117" s="15" t="n">
         <v>-5476784.973544974</v>
       </c>
-      <c r="AD117" s="15" t="n"/>
-      <c r="AE117" s="15" t="n"/>
-      <c r="AF117" s="15" t="n"/>
+      <c r="AD117" s="15" t="n">
+        <v>-16713035</v>
+      </c>
+      <c r="AE117" s="15" t="n">
+        <v>-983.1197058823529</v>
+      </c>
+      <c r="AF117" s="15" t="n">
+        <v>-88428.75661375662</v>
+      </c>
       <c r="AG117" s="15" t="n">
-        <v>-1035112360</v>
+        <v>-1051825395</v>
       </c>
       <c r="AH117" s="15" t="n">
-        <v>-60888.96235294118</v>
+        <v>-61872.08205882353</v>
       </c>
       <c r="AI117" s="15" t="n">
-        <v>-5476784.973544974</v>
+        <v>-5565213.73015873</v>
       </c>
     </row>
     <row r="118">
@@ -9504,22 +9672,22 @@
         <v>-29764206.24867725</v>
       </c>
       <c r="AD119" s="11" t="n">
-        <v>-2950000</v>
+        <v>-377544050</v>
       </c>
       <c r="AE119" s="11" t="n">
-        <v>-173.5294117647059</v>
+        <v>-22208.47352941176</v>
       </c>
       <c r="AF119" s="11" t="n">
-        <v>-15608.46560846561</v>
+        <v>-1997587.566137566</v>
       </c>
       <c r="AG119" s="11" t="n">
-        <v>-5628384981</v>
+        <v>-6002979031</v>
       </c>
       <c r="AH119" s="11" t="n">
-        <v>-331081.4694705882</v>
+        <v>-353116.4135882353</v>
       </c>
       <c r="AI119" s="11" t="n">
-        <v>-29779814.71428572</v>
+        <v>-31761793.81481482</v>
       </c>
     </row>
     <row r="120">
@@ -9610,22 +9778,22 @@
         <v>-29764206.24867725</v>
       </c>
       <c r="AD120" s="15" t="n">
-        <v>-2950000</v>
+        <v>-377544050</v>
       </c>
       <c r="AE120" s="15" t="n">
-        <v>-173.5294117647059</v>
+        <v>-22208.47352941176</v>
       </c>
       <c r="AF120" s="15" t="n">
-        <v>-15608.46560846561</v>
+        <v>-1997587.566137566</v>
       </c>
       <c r="AG120" s="15" t="n">
-        <v>-5628384981</v>
+        <v>-6002979031</v>
       </c>
       <c r="AH120" s="15" t="n">
-        <v>-331081.4694705882</v>
+        <v>-353116.4135882353</v>
       </c>
       <c r="AI120" s="15" t="n">
-        <v>-29779814.71428572</v>
+        <v>-31761793.81481482</v>
       </c>
     </row>
     <row r="121">
@@ -9990,22 +10158,22 @@
         <v>-5069808.166825396</v>
       </c>
       <c r="AD125" s="13" t="n">
-        <v>-1548525</v>
+        <v>-123675500</v>
       </c>
       <c r="AE125" s="13" t="n">
-        <v>-91.08970588235294</v>
+        <v>-7275.029411764706</v>
       </c>
       <c r="AF125" s="13" t="n">
-        <v>-8193.253968253968</v>
+        <v>-654367.7248677248</v>
       </c>
       <c r="AG125" s="13" t="n">
-        <v>-959742268.5300001</v>
+        <v>-1081869243.53</v>
       </c>
       <c r="AH125" s="13" t="n">
-        <v>-56455.42756058824</v>
+        <v>-63639.3672664706</v>
       </c>
       <c r="AI125" s="13" t="n">
-        <v>-5078001.42079365</v>
+        <v>-5724175.891693121</v>
       </c>
     </row>
     <row r="126">
@@ -10190,22 +10358,22 @@
         <v>-75768803.29100528</v>
       </c>
       <c r="AD127" s="13" t="n">
-        <v>-6813775</v>
+        <v>-34298950</v>
       </c>
       <c r="AE127" s="13" t="n">
-        <v>-400.8102941176471</v>
+        <v>-2017.585294117647</v>
       </c>
       <c r="AF127" s="13" t="n">
-        <v>-36051.71957671957</v>
+        <v>-181475.9259259259</v>
       </c>
       <c r="AG127" s="13" t="n">
-        <v>-14327117597</v>
+        <v>-14354602772</v>
       </c>
       <c r="AH127" s="13" t="n">
-        <v>-842771.6233529412</v>
+        <v>-844388.3983529413</v>
       </c>
       <c r="AI127" s="13" t="n">
-        <v>-75804855.010582</v>
+        <v>-75950279.21693121</v>
       </c>
     </row>
     <row r="128">
@@ -10402,22 +10570,22 @@
         <v>-132568430.7276719</v>
       </c>
       <c r="AD129" s="15" t="n">
-        <v>-67461266</v>
+        <v>-217073416</v>
       </c>
       <c r="AE129" s="15" t="n">
-        <v>-3968.309764705883</v>
+        <v>-12769.02447058824</v>
       </c>
       <c r="AF129" s="15" t="n">
-        <v>-356937.9153439153</v>
+        <v>-1148536.592592593</v>
       </c>
       <c r="AG129" s="15" t="n">
-        <v>-25122894673.53</v>
+        <v>-25272506823.53</v>
       </c>
       <c r="AH129" s="15" t="n">
-        <v>-1477817.333737059</v>
+        <v>-1486618.048442941</v>
       </c>
       <c r="AI129" s="15" t="n">
-        <v>-132925368.6430158</v>
+        <v>-133716967.3202645</v>
       </c>
     </row>
     <row r="130">
@@ -10535,17 +10703,23 @@
       <c r="AC131" s="11" t="n">
         <v>-170588.9947089947</v>
       </c>
-      <c r="AD131" s="11" t="n"/>
-      <c r="AE131" s="11" t="n"/>
-      <c r="AF131" s="11" t="n"/>
+      <c r="AD131" s="11" t="n">
+        <v>-1513500</v>
+      </c>
+      <c r="AE131" s="11" t="n">
+        <v>-89.02941176470588</v>
+      </c>
+      <c r="AF131" s="11" t="n">
+        <v>-8007.936507936508</v>
+      </c>
       <c r="AG131" s="11" t="n">
-        <v>-32241320</v>
+        <v>-33754820</v>
       </c>
       <c r="AH131" s="11" t="n">
-        <v>-1896.548235294118</v>
+        <v>-1985.577647058823</v>
       </c>
       <c r="AI131" s="11" t="n">
-        <v>-170588.9947089947</v>
+        <v>-178596.9312169312</v>
       </c>
     </row>
     <row r="132">
@@ -10623,17 +10797,23 @@
       <c r="AC132" s="13" t="n">
         <v>-1669307.211640212</v>
       </c>
-      <c r="AD132" s="13" t="n"/>
-      <c r="AE132" s="13" t="n"/>
-      <c r="AF132" s="13" t="n"/>
+      <c r="AD132" s="13" t="n">
+        <v>-88418129</v>
+      </c>
+      <c r="AE132" s="13" t="n">
+        <v>-5201.066411764706</v>
+      </c>
+      <c r="AF132" s="13" t="n">
+        <v>-467820.7883597884</v>
+      </c>
       <c r="AG132" s="13" t="n">
-        <v>-315499063</v>
+        <v>-403917192</v>
       </c>
       <c r="AH132" s="13" t="n">
-        <v>-18558.76841176471</v>
+        <v>-23759.83482352941</v>
       </c>
       <c r="AI132" s="13" t="n">
-        <v>-1669307.211640212</v>
+        <v>-2137128</v>
       </c>
     </row>
     <row r="133">
@@ -10811,17 +10991,23 @@
       <c r="AC134" s="13" t="n">
         <v>-555076.6825396825</v>
       </c>
-      <c r="AD134" s="13" t="n"/>
-      <c r="AE134" s="13" t="n"/>
-      <c r="AF134" s="13" t="n"/>
+      <c r="AD134" s="13" t="n">
+        <v>-4345000</v>
+      </c>
+      <c r="AE134" s="13" t="n">
+        <v>-255.5882352941177</v>
+      </c>
+      <c r="AF134" s="13" t="n">
+        <v>-22989.41798941799</v>
+      </c>
       <c r="AG134" s="13" t="n">
-        <v>-104909493</v>
+        <v>-109254493</v>
       </c>
       <c r="AH134" s="13" t="n">
-        <v>-6171.146647058823</v>
+        <v>-6426.734882352941</v>
       </c>
       <c r="AI134" s="13" t="n">
-        <v>-555076.6825396825</v>
+        <v>-578066.1005291005</v>
       </c>
     </row>
     <row r="135">
@@ -10905,17 +11091,23 @@
       <c r="AC135" s="11" t="n">
         <v>-1057244.523809524</v>
       </c>
-      <c r="AD135" s="11" t="n"/>
-      <c r="AE135" s="11" t="n"/>
-      <c r="AF135" s="11" t="n"/>
+      <c r="AD135" s="11" t="n">
+        <v>-882612</v>
+      </c>
+      <c r="AE135" s="11" t="n">
+        <v>-51.91835294117647</v>
+      </c>
+      <c r="AF135" s="11" t="n">
+        <v>-4669.904761904761</v>
+      </c>
       <c r="AG135" s="11" t="n">
-        <v>-199819215</v>
+        <v>-200701827</v>
       </c>
       <c r="AH135" s="11" t="n">
-        <v>-11754.07147058823</v>
+        <v>-11805.98982352941</v>
       </c>
       <c r="AI135" s="11" t="n">
-        <v>-1057244.523809524</v>
+        <v>-1061914.428571429</v>
       </c>
     </row>
     <row r="136">
@@ -10969,17 +11161,23 @@
       <c r="AC136" s="13" t="n">
         <v>-6195.767195767196</v>
       </c>
-      <c r="AD136" s="13" t="n"/>
-      <c r="AE136" s="13" t="n"/>
-      <c r="AF136" s="13" t="n"/>
+      <c r="AD136" s="13" t="n">
+        <v>-578500</v>
+      </c>
+      <c r="AE136" s="13" t="n">
+        <v>-34.02941176470588</v>
+      </c>
+      <c r="AF136" s="13" t="n">
+        <v>-3060.846560846561</v>
+      </c>
       <c r="AG136" s="13" t="n">
-        <v>-1171000</v>
+        <v>-1749500</v>
       </c>
       <c r="AH136" s="13" t="n">
-        <v>-68.88235294117646</v>
+        <v>-102.9117647058823</v>
       </c>
       <c r="AI136" s="13" t="n">
-        <v>-6195.767195767196</v>
+        <v>-9256.613756613757</v>
       </c>
     </row>
     <row r="137">
@@ -11069,17 +11267,23 @@
       <c r="AC137" s="15" t="n">
         <v>-4551761.624338624</v>
       </c>
-      <c r="AD137" s="15" t="n"/>
-      <c r="AE137" s="15" t="n"/>
-      <c r="AF137" s="15" t="n"/>
+      <c r="AD137" s="15" t="n">
+        <v>-95737741</v>
+      </c>
+      <c r="AE137" s="15" t="n">
+        <v>-5631.631823529412</v>
+      </c>
+      <c r="AF137" s="15" t="n">
+        <v>-506548.8941798942</v>
+      </c>
       <c r="AG137" s="15" t="n">
-        <v>-860282947</v>
+        <v>-956020688</v>
       </c>
       <c r="AH137" s="15" t="n">
-        <v>-50604.87923529411</v>
+        <v>-56236.51105882352</v>
       </c>
       <c r="AI137" s="15" t="n">
-        <v>-4551761.624338624</v>
+        <v>-5058310.518518519</v>
       </c>
     </row>
     <row r="138">
@@ -11170,22 +11374,22 @@
         <v>-230275933.0393122</v>
       </c>
       <c r="AD138" s="15" t="n">
-        <v>-70411266</v>
+        <v>-968685840</v>
       </c>
       <c r="AE138" s="15" t="n">
-        <v>-4141.839176470588</v>
+        <v>-56981.52</v>
       </c>
       <c r="AF138" s="15" t="n">
-        <v>-372546.3809523809</v>
+        <v>-5125321.904761905</v>
       </c>
       <c r="AG138" s="15" t="n">
-        <v>-43592562610.43001</v>
+        <v>-44490837184.43001</v>
       </c>
       <c r="AH138" s="15" t="n">
-        <v>-2564268.388848823</v>
+        <v>-2617108.069672353</v>
       </c>
       <c r="AI138" s="15" t="n">
-        <v>-230648479.4202645</v>
+        <v>-235401254.9440741</v>
       </c>
     </row>
     <row r="139">
@@ -11398,22 +11602,22 @@
         <v>-4894589.497354497</v>
       </c>
       <c r="AD141" s="13" t="n">
-        <v>-60751400</v>
+        <v>-61751400</v>
       </c>
       <c r="AE141" s="13" t="n">
-        <v>-3573.611764705882</v>
+        <v>-3632.435294117647</v>
       </c>
       <c r="AF141" s="13" t="n">
-        <v>-321435.9788359788</v>
+        <v>-326726.9841269841</v>
       </c>
       <c r="AG141" s="13" t="n">
-        <v>-985828815</v>
+        <v>-986828815</v>
       </c>
       <c r="AH141" s="13" t="n">
-        <v>-57989.93029411765</v>
+        <v>-58048.75382352941</v>
       </c>
       <c r="AI141" s="13" t="n">
-        <v>-5216025.476190476</v>
+        <v>-5221316.481481481</v>
       </c>
     </row>
     <row r="142">
@@ -11620,22 +11824,22 @@
         <v>-13736457.22222222</v>
       </c>
       <c r="AD144" s="15" t="n">
-        <v>-60751400</v>
+        <v>-61751400</v>
       </c>
       <c r="AE144" s="15" t="n">
-        <v>-3573.611764705882</v>
+        <v>-3632.435294117647</v>
       </c>
       <c r="AF144" s="15" t="n">
-        <v>-321435.9788359788</v>
+        <v>-326726.9841269841</v>
       </c>
       <c r="AG144" s="15" t="n">
-        <v>-2656941815</v>
+        <v>-2657941815</v>
       </c>
       <c r="AH144" s="15" t="n">
-        <v>-156290.695</v>
+        <v>-156349.5185294118</v>
       </c>
       <c r="AI144" s="15" t="n">
-        <v>-14057893.2010582</v>
+        <v>-14063184.20634921</v>
       </c>
     </row>
     <row r="145">
@@ -11766,22 +11970,22 @@
         <v>-99449.19407407405</v>
       </c>
       <c r="AD146" s="11" t="n">
-        <v>-2500</v>
+        <v>-49500</v>
       </c>
       <c r="AE146" s="11" t="n">
-        <v>-0.1470588235294118</v>
+        <v>-2.911764705882353</v>
       </c>
       <c r="AF146" s="11" t="n">
-        <v>-13.22751322751323</v>
+        <v>-261.9047619047619</v>
       </c>
       <c r="AG146" s="11" t="n">
-        <v>-18798397.68</v>
+        <v>-18845397.68</v>
       </c>
       <c r="AH146" s="11" t="n">
-        <v>-1105.788098823529</v>
+        <v>-1108.552804705882</v>
       </c>
       <c r="AI146" s="11" t="n">
-        <v>-99462.42158730156</v>
+        <v>-99711.09883597882</v>
       </c>
     </row>
     <row r="147">
@@ -12258,22 +12462,22 @@
         <v>-31583868.07253968</v>
       </c>
       <c r="AD152" s="15" t="n">
-        <v>-2500</v>
+        <v>-49500</v>
       </c>
       <c r="AE152" s="15" t="n">
-        <v>-0.1470588235294118</v>
+        <v>-2.911764705882353</v>
       </c>
       <c r="AF152" s="15" t="n">
-        <v>-13.22751322751323</v>
+        <v>-261.9047619047619</v>
       </c>
       <c r="AG152" s="15" t="n">
-        <v>-5969353565.710001</v>
+        <v>-5969400565.710001</v>
       </c>
       <c r="AH152" s="15" t="n">
-        <v>-351138.4450417647</v>
+        <v>-351141.2097476471</v>
       </c>
       <c r="AI152" s="15" t="n">
-        <v>-31583881.30005291</v>
+        <v>-31584129.97730159</v>
       </c>
     </row>
     <row r="153">
@@ -12364,22 +12568,22 @@
         <v>-1529478500.653757</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-432595564</v>
+        <v>-4302881306</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-25446.79788235294</v>
+        <v>-253110.6650588235</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-2288865.417989418</v>
+        <v>-22766567.75661376</v>
       </c>
       <c r="AG153" s="19" t="n">
-        <v>-289504032187.5599</v>
+        <v>-293374317929.5599</v>
       </c>
       <c r="AH153" s="19" t="n">
-        <v>-17029648.95220941</v>
+        <v>-17257312.81938588</v>
       </c>
       <c r="AI153" s="19" t="n">
-        <v>-1531767366.071746</v>
+        <v>-1552245068.41037</v>
       </c>
     </row>
     <row r="154">
@@ -12470,22 +12674,22 @@
         <v>-349256107.4480425</v>
       </c>
       <c r="AD154" s="19" t="n">
-        <v>3442000269</v>
+        <v>5598737780</v>
       </c>
       <c r="AE154" s="19" t="n">
-        <v>202470.6040588235</v>
+        <v>329337.5164705882</v>
       </c>
       <c r="AF154" s="19" t="n">
-        <v>18211641.63492063</v>
+        <v>29622951.21693122</v>
       </c>
       <c r="AG154" s="19" t="n">
-        <v>-62567404038.68</v>
+        <v>-60410666527.68</v>
       </c>
       <c r="AH154" s="19" t="n">
-        <v>-3680435.531687059</v>
+        <v>-3553568.619275295</v>
       </c>
       <c r="AI154" s="19" t="n">
-        <v>-331044465.8131218</v>
+        <v>-319633156.2311112</v>
       </c>
     </row>
     <row r="155">
@@ -12576,22 +12780,22 @@
         <v>7747388.987724859</v>
       </c>
       <c r="AD155" s="7" t="n">
-        <v>4906256787.679998</v>
+        <v>7062994298.679998</v>
       </c>
       <c r="AE155" s="7" t="n">
-        <v>288603.3404517646</v>
+        <v>415470.2528635293</v>
       </c>
       <c r="AF155" s="7" t="n">
-        <v>25959030.62264549</v>
+        <v>37370340.20465608</v>
       </c>
       <c r="AG155" s="7" t="n">
-        <v>4906256787.679998</v>
+        <v>7062994298.679998</v>
       </c>
       <c r="AH155" s="7" t="n">
-        <v>288603.3404517646</v>
+        <v>415470.2528635293</v>
       </c>
       <c r="AI155" s="7" t="n">
-        <v>25959030.62264549</v>
+        <v>37370340.20465608</v>
       </c>
     </row>
   </sheetData>
@@ -13056,16 +13260,16 @@
         <v>1136676704</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>3514164635</v>
+        <v>5476861296</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>4650841339</v>
+        <v>6613538000</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>273578.9022941177</v>
+        <v>389031.6470588236</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>24607626.13227513</v>
+        <v>34992264.55026455</v>
       </c>
     </row>
     <row r="7">
@@ -13088,16 +13292,16 @@
         <v>7894080</v>
       </c>
       <c r="E7" s="13" t="n">
-        <v>0</v>
+        <v>185000000</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>7894080</v>
+        <v>192894080</v>
       </c>
       <c r="G7" s="24" t="n">
-        <v>464.3576470588235</v>
+        <v>11346.71058823529</v>
       </c>
       <c r="H7" s="24" t="n">
-        <v>41767.61904761905</v>
+        <v>1020603.597883598</v>
       </c>
     </row>
     <row r="8">
@@ -13152,16 +13356,16 @@
         <v>172976399.24</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>-72189366</v>
+        <v>-63148516</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>100787033.24</v>
+        <v>109827883.24</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>5928.649014117647</v>
+        <v>6460.463720000001</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>533264.7261375661</v>
+        <v>581099.9113227513</v>
       </c>
     </row>
     <row r="10">
@@ -13271,13 +13475,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>4906256789.679999</v>
+        <v>7062994300.679999</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>288603.3405694118</v>
+        <v>415470.2529811764</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>25959030.63322751</v>
+        <v>37370340.21523809</v>
       </c>
     </row>
   </sheetData>
@@ -13347,7 +13551,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 09 Sep 2026 16:19 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 11 Sep 2026 16:51 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -13422,14 +13626,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 09 Sep 2026</t>
+          <t>MTD as of 11 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 09 Sep 2026</t>
+          <t>YTD as of 11 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
@@ -13837,22 +14041,22 @@
         <v>914.3238245555556</v>
       </c>
       <c r="AD7" s="11" t="n">
-        <v>3860.720333</v>
+        <v>9886.718086000001</v>
       </c>
       <c r="AE7" s="11" t="n">
-        <v>0.2271011960588235</v>
+        <v>0.5815716521176471</v>
       </c>
       <c r="AF7" s="11" t="n">
-        <v>20.42709170899471</v>
+        <v>52.31067770370371</v>
       </c>
       <c r="AG7" s="11" t="n">
-        <v>176667.923174</v>
+        <v>182693.920927</v>
       </c>
       <c r="AH7" s="11" t="n">
-        <v>10.39223077494118</v>
+        <v>10.746701231</v>
       </c>
       <c r="AI7" s="11" t="n">
-        <v>934.7509162645503</v>
+        <v>966.6345022592593</v>
       </c>
     </row>
     <row r="8">
@@ -14118,17 +14322,23 @@
       <c r="AC10" s="13" t="n">
         <v>183.2983953015873</v>
       </c>
-      <c r="AD10" s="13" t="n"/>
-      <c r="AE10" s="13" t="n"/>
-      <c r="AF10" s="13" t="n"/>
+      <c r="AD10" s="13" t="n">
+        <v>6025.997753</v>
+      </c>
+      <c r="AE10" s="13" t="n">
+        <v>0.3544704560588235</v>
+      </c>
+      <c r="AF10" s="13" t="n">
+        <v>31.88358599470899</v>
+      </c>
       <c r="AG10" s="13" t="n">
-        <v>34643.396712</v>
+        <v>40669.394465</v>
       </c>
       <c r="AH10" s="13" t="n">
-        <v>2.037846865411765</v>
+        <v>2.392317321470588</v>
       </c>
       <c r="AI10" s="13" t="n">
-        <v>183.2983953015873</v>
+        <v>215.1819812962963</v>
       </c>
     </row>
     <row r="11">
@@ -14807,22 +15017,22 @@
         <v>2.321849073439154</v>
       </c>
       <c r="AD20" s="13" t="n">
-        <v>13.8755</v>
+        <v>14.901</v>
       </c>
       <c r="AE20" s="13" t="n">
-        <v>0.0008162058823529412</v>
+        <v>0.0008765294117647059</v>
       </c>
       <c r="AF20" s="13" t="n">
-        <v>0.07341534391534392</v>
+        <v>0.07884126984126984</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>452.70497488</v>
+        <v>453.73047488</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>0.02662970440470588</v>
+        <v>0.02669002793411765</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>2.395264417354498</v>
+        <v>2.400690343280424</v>
       </c>
     </row>
     <row r="21">
@@ -15059,22 +15269,22 @@
         <v>0.332547619047619</v>
       </c>
       <c r="AD23" s="11" t="n">
-        <v>13.503</v>
+        <v>14.5285</v>
       </c>
       <c r="AE23" s="11" t="n">
-        <v>0.0007942941176470588</v>
+        <v>0.0008546176470588235</v>
       </c>
       <c r="AF23" s="11" t="n">
-        <v>0.07144444444444445</v>
+        <v>0.07687037037037037</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>76.3545</v>
+        <v>77.38</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>0.004491441176470589</v>
+        <v>0.004551764705882353</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>0.4039920634920635</v>
+        <v>0.4094179894179894</v>
       </c>
     </row>
     <row r="24">
@@ -16451,22 +16661,22 @@
         <v>1180.222393205714</v>
       </c>
       <c r="AD44" s="15" t="n">
-        <v>3874.595833</v>
+        <v>9901.619086000001</v>
       </c>
       <c r="AE44" s="15" t="n">
-        <v>0.2279174019411765</v>
+        <v>0.5824481815294118</v>
       </c>
       <c r="AF44" s="15" t="n">
-        <v>20.50050705291005</v>
+        <v>52.38951897354497</v>
       </c>
       <c r="AG44" s="15" t="n">
-        <v>226936.62814888</v>
+        <v>232963.65140188</v>
       </c>
       <c r="AH44" s="15" t="n">
-        <v>13.34921342052235</v>
+        <v>13.70374420011059</v>
       </c>
       <c r="AI44" s="15" t="n">
-        <v>1200.722900258624</v>
+        <v>1232.611912179259</v>
       </c>
     </row>
     <row r="45">
@@ -16700,17 +16910,23 @@
       <c r="AC48" s="13" t="n">
         <v>-0.8255413492063493</v>
       </c>
-      <c r="AD48" s="13" t="n"/>
-      <c r="AE48" s="13" t="n"/>
-      <c r="AF48" s="13" t="n"/>
+      <c r="AD48" s="13" t="n">
+        <v>-4.9</v>
+      </c>
+      <c r="AE48" s="13" t="n">
+        <v>-0.0002882352941176471</v>
+      </c>
+      <c r="AF48" s="13" t="n">
+        <v>-0.02592592592592593</v>
+      </c>
       <c r="AG48" s="13" t="n">
-        <v>-156.027315</v>
+        <v>-160.927315</v>
       </c>
       <c r="AH48" s="13" t="n">
-        <v>-0.009178077352941178</v>
+        <v>-0.009466312647058824</v>
       </c>
       <c r="AI48" s="13" t="n">
-        <v>-0.8255413492063493</v>
+        <v>-0.8514672751322752</v>
       </c>
     </row>
     <row r="49">
@@ -16852,17 +17068,23 @@
       <c r="AC50" s="13" t="n">
         <v>-9.414012693121693</v>
       </c>
-      <c r="AD50" s="13" t="n"/>
-      <c r="AE50" s="13" t="n"/>
-      <c r="AF50" s="13" t="n"/>
+      <c r="AD50" s="13" t="n">
+        <v>-278.45155</v>
+      </c>
+      <c r="AE50" s="13" t="n">
+        <v>-0.01637950294117647</v>
+      </c>
+      <c r="AF50" s="13" t="n">
+        <v>-1.473288624338624</v>
+      </c>
       <c r="AG50" s="13" t="n">
-        <v>-1779.248399</v>
+        <v>-2057.699949</v>
       </c>
       <c r="AH50" s="13" t="n">
-        <v>-0.1046616705294118</v>
+        <v>-0.1210411734705883</v>
       </c>
       <c r="AI50" s="13" t="n">
-        <v>-9.414012693121693</v>
+        <v>-10.88730131746032</v>
       </c>
     </row>
     <row r="51">
@@ -17132,17 +17354,23 @@
       <c r="AC54" s="13" t="n">
         <v>-7.301592116402117</v>
       </c>
-      <c r="AD54" s="13" t="n"/>
-      <c r="AE54" s="13" t="n"/>
-      <c r="AF54" s="13" t="n"/>
+      <c r="AD54" s="13" t="n">
+        <v>-522.213844</v>
+      </c>
+      <c r="AE54" s="13" t="n">
+        <v>-0.0307184614117647</v>
+      </c>
+      <c r="AF54" s="13" t="n">
+        <v>-2.763036211640212</v>
+      </c>
       <c r="AG54" s="13" t="n">
-        <v>-1380.00091</v>
+        <v>-1902.214754</v>
       </c>
       <c r="AH54" s="13" t="n">
-        <v>-0.08117652411764706</v>
+        <v>-0.1118949855294118</v>
       </c>
       <c r="AI54" s="13" t="n">
-        <v>-7.301592116402117</v>
+        <v>-10.06462832804233</v>
       </c>
     </row>
     <row r="55">
@@ -17372,17 +17600,23 @@
       <c r="AC57" s="11" t="n">
         <v>-1.331501074074074</v>
       </c>
-      <c r="AD57" s="11" t="n"/>
-      <c r="AE57" s="11" t="n"/>
-      <c r="AF57" s="11" t="n"/>
+      <c r="AD57" s="11" t="n">
+        <v>-19.87</v>
+      </c>
+      <c r="AE57" s="11" t="n">
+        <v>-0.001168823529411765</v>
+      </c>
+      <c r="AF57" s="11" t="n">
+        <v>-0.1051322751322751</v>
+      </c>
       <c r="AG57" s="11" t="n">
-        <v>-251.653703</v>
+        <v>-271.523703</v>
       </c>
       <c r="AH57" s="11" t="n">
-        <v>-0.014803159</v>
+        <v>-0.01597198252941176</v>
       </c>
       <c r="AI57" s="11" t="n">
-        <v>-1.331501074074074</v>
+        <v>-1.436633349206349</v>
       </c>
     </row>
     <row r="58">
@@ -17472,17 +17706,23 @@
       <c r="AC58" s="13" t="n">
         <v>-15.89634283005291</v>
       </c>
-      <c r="AD58" s="13" t="n"/>
-      <c r="AE58" s="13" t="n"/>
-      <c r="AF58" s="13" t="n"/>
+      <c r="AD58" s="13" t="n">
+        <v>-53.391331</v>
+      </c>
+      <c r="AE58" s="13" t="n">
+        <v>-0.003140666529411765</v>
+      </c>
+      <c r="AF58" s="13" t="n">
+        <v>-0.2824938148148148</v>
+      </c>
       <c r="AG58" s="13" t="n">
-        <v>-3004.40879488</v>
+        <v>-3057.80012588</v>
       </c>
       <c r="AH58" s="13" t="n">
-        <v>-0.1767299291105882</v>
+        <v>-0.17987059564</v>
       </c>
       <c r="AI58" s="13" t="n">
-        <v>-15.89634283005291</v>
+        <v>-16.17883664486773</v>
       </c>
     </row>
     <row r="59">
@@ -17782,17 +18022,23 @@
       <c r="AC62" s="15" t="n">
         <v>-84.58074699407408</v>
       </c>
-      <c r="AD62" s="15" t="n"/>
-      <c r="AE62" s="15" t="n"/>
-      <c r="AF62" s="15" t="n"/>
+      <c r="AD62" s="15" t="n">
+        <v>-878.826725</v>
+      </c>
+      <c r="AE62" s="15" t="n">
+        <v>-0.05169568970588236</v>
+      </c>
+      <c r="AF62" s="15" t="n">
+        <v>-4.649876851851852</v>
+      </c>
       <c r="AG62" s="15" t="n">
-        <v>-15985.76118188</v>
+        <v>-16864.58790688</v>
       </c>
       <c r="AH62" s="15" t="n">
-        <v>-0.9403388930517647</v>
+        <v>-0.992034582757647</v>
       </c>
       <c r="AI62" s="15" t="n">
-        <v>-84.58074699407408</v>
+        <v>-89.23062384592593</v>
       </c>
     </row>
     <row r="63">
@@ -18845,22 +19091,22 @@
         <v>-35.11226440740741</v>
       </c>
       <c r="AD80" s="11" t="n">
-        <v>-286.804298</v>
+        <v>-1088.054516</v>
       </c>
       <c r="AE80" s="11" t="n">
-        <v>-0.01687084105882353</v>
+        <v>-0.0640032068235294</v>
       </c>
       <c r="AF80" s="11" t="n">
-        <v>-1.517483058201058</v>
+        <v>-5.7569022010582</v>
       </c>
       <c r="AG80" s="11" t="n">
-        <v>-6923.022271000001</v>
+        <v>-7724.272489000001</v>
       </c>
       <c r="AH80" s="11" t="n">
-        <v>-0.4072366041764707</v>
+        <v>-0.4543689699411765</v>
       </c>
       <c r="AI80" s="11" t="n">
-        <v>-36.62974746560847</v>
+        <v>-40.86916660846561</v>
       </c>
     </row>
     <row r="81">
@@ -18951,22 +19197,22 @@
         <v>-48.83498968539683</v>
       </c>
       <c r="AD81" s="13" t="n">
-        <v>-14.6261</v>
+        <v>-1301.257365</v>
       </c>
       <c r="AE81" s="13" t="n">
-        <v>-0.0008603588235294117</v>
+        <v>-0.07654455088235294</v>
       </c>
       <c r="AF81" s="13" t="n">
-        <v>-0.07738677248677248</v>
+        <v>-6.884959603174603</v>
       </c>
       <c r="AG81" s="13" t="n">
-        <v>-9244.439150539998</v>
+        <v>-10531.07041554</v>
       </c>
       <c r="AH81" s="13" t="n">
-        <v>-0.5437905382670588</v>
+        <v>-0.6194747303258823</v>
       </c>
       <c r="AI81" s="13" t="n">
-        <v>-48.9123764578836</v>
+        <v>-55.71994928857143</v>
       </c>
     </row>
     <row r="82">
@@ -19156,17 +19402,23 @@
       <c r="AC83" s="13" t="n">
         <v>-2.053284693121693</v>
       </c>
-      <c r="AD83" s="13" t="n"/>
-      <c r="AE83" s="13" t="n"/>
-      <c r="AF83" s="13" t="n"/>
+      <c r="AD83" s="13" t="n">
+        <v>-4.25596</v>
+      </c>
+      <c r="AE83" s="13" t="n">
+        <v>-0.0002503505882352941</v>
+      </c>
+      <c r="AF83" s="13" t="n">
+        <v>-0.02251830687830688</v>
+      </c>
       <c r="AG83" s="13" t="n">
-        <v>-388.0708070000001</v>
+        <v>-392.3267670000001</v>
       </c>
       <c r="AH83" s="13" t="n">
-        <v>-0.02282769452941177</v>
+        <v>-0.02307804511764706</v>
       </c>
       <c r="AI83" s="13" t="n">
-        <v>-2.053284693121693</v>
+        <v>-2.075803</v>
       </c>
     </row>
     <row r="84">
@@ -19257,22 +19509,22 @@
         <v>-126.3342242039153</v>
       </c>
       <c r="AD84" s="15" t="n">
-        <v>-301.430398</v>
+        <v>-2393.567841</v>
       </c>
       <c r="AE84" s="15" t="n">
-        <v>-0.01773119988235294</v>
+        <v>-0.1407981082941177</v>
       </c>
       <c r="AF84" s="15" t="n">
-        <v>-1.594869830687831</v>
+        <v>-12.66438011111111</v>
       </c>
       <c r="AG84" s="15" t="n">
-        <v>-24178.59877254</v>
+        <v>-26270.73621554</v>
       </c>
       <c r="AH84" s="15" t="n">
-        <v>-1.422270516031765</v>
+        <v>-1.545337424443529</v>
       </c>
       <c r="AI84" s="15" t="n">
-        <v>-127.9290940346032</v>
+        <v>-138.9986043150264</v>
       </c>
     </row>
     <row r="85">
@@ -19442,17 +19694,23 @@
       <c r="AC87" s="11" t="n">
         <v>-0.716669634920635</v>
       </c>
-      <c r="AD87" s="11" t="n"/>
-      <c r="AE87" s="11" t="n"/>
-      <c r="AF87" s="11" t="n"/>
+      <c r="AD87" s="11" t="n">
+        <v>-0.735172</v>
+      </c>
+      <c r="AE87" s="11" t="n">
+        <v>-4.324541176470589e-05</v>
+      </c>
+      <c r="AF87" s="11" t="n">
+        <v>-0.003889798941798942</v>
+      </c>
       <c r="AG87" s="11" t="n">
-        <v>-135.450561</v>
+        <v>-136.185733</v>
       </c>
       <c r="AH87" s="11" t="n">
-        <v>-0.007967680058823529</v>
+        <v>-0.008010925470588235</v>
       </c>
       <c r="AI87" s="11" t="n">
-        <v>-0.716669634920635</v>
+        <v>-0.7205594338624339</v>
       </c>
     </row>
     <row r="88">
@@ -19576,17 +19834,23 @@
       <c r="AC89" s="11" t="n">
         <v>-0.04221801587301587</v>
       </c>
-      <c r="AD89" s="11" t="n"/>
-      <c r="AE89" s="11" t="n"/>
-      <c r="AF89" s="11" t="n"/>
+      <c r="AD89" s="11" t="n">
+        <v>-5.785771</v>
+      </c>
+      <c r="AE89" s="11" t="n">
+        <v>-0.0003403394705882353</v>
+      </c>
+      <c r="AF89" s="11" t="n">
+        <v>-0.03061254497354498</v>
+      </c>
       <c r="AG89" s="11" t="n">
-        <v>-7.979205</v>
+        <v>-13.764976</v>
       </c>
       <c r="AH89" s="11" t="n">
-        <v>-0.000469365</v>
+        <v>-0.0008097044705882353</v>
       </c>
       <c r="AI89" s="11" t="n">
-        <v>-0.04221801587301587</v>
+        <v>-0.07283056084656084</v>
       </c>
     </row>
     <row r="90">
@@ -19646,17 +19910,23 @@
       <c r="AC90" s="13" t="n">
         <v>-0.008627340952380951</v>
       </c>
-      <c r="AD90" s="13" t="n"/>
-      <c r="AE90" s="13" t="n"/>
-      <c r="AF90" s="13" t="n"/>
+      <c r="AD90" s="13" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="AE90" s="13" t="n">
+        <v>-2.352941176470588e-06</v>
+      </c>
+      <c r="AF90" s="13" t="n">
+        <v>-0.0002116402116402116</v>
+      </c>
       <c r="AG90" s="13" t="n">
-        <v>-1.63056744</v>
+        <v>-1.67056744</v>
       </c>
       <c r="AH90" s="13" t="n">
-        <v>-9.591573176470588e-05</v>
+        <v>-9.826867294117647e-05</v>
       </c>
       <c r="AI90" s="13" t="n">
-        <v>-0.008627340952380951</v>
+        <v>-0.008838981164021162</v>
       </c>
     </row>
     <row r="91">
@@ -19746,17 +20016,23 @@
       <c r="AC91" s="11" t="n">
         <v>-0.6865170158730159</v>
       </c>
-      <c r="AD91" s="11" t="n"/>
-      <c r="AE91" s="11" t="n"/>
-      <c r="AF91" s="11" t="n"/>
+      <c r="AD91" s="11" t="n">
+        <v>-0.1954</v>
+      </c>
+      <c r="AE91" s="11" t="n">
+        <v>-1.149411764705882e-05</v>
+      </c>
+      <c r="AF91" s="11" t="n">
+        <v>-0.001033862433862434</v>
+      </c>
       <c r="AG91" s="11" t="n">
-        <v>-129.751716</v>
+        <v>-129.947116</v>
       </c>
       <c r="AH91" s="11" t="n">
-        <v>-0.007632453882352942</v>
+        <v>-0.007643948</v>
       </c>
       <c r="AI91" s="11" t="n">
-        <v>-0.6865170158730159</v>
+        <v>-0.6875508783068783</v>
       </c>
     </row>
     <row r="92">
@@ -19834,17 +20110,23 @@
       <c r="AC92" s="13" t="n">
         <v>-0.01128093121693122</v>
       </c>
-      <c r="AD92" s="13" t="n"/>
-      <c r="AE92" s="13" t="n"/>
-      <c r="AF92" s="13" t="n"/>
+      <c r="AD92" s="13" t="n">
+        <v>-0.1856</v>
+      </c>
+      <c r="AE92" s="13" t="n">
+        <v>-1.091764705882353e-05</v>
+      </c>
+      <c r="AF92" s="13" t="n">
+        <v>-0.000982010582010582</v>
+      </c>
       <c r="AG92" s="13" t="n">
-        <v>-2.132096</v>
+        <v>-2.317696</v>
       </c>
       <c r="AH92" s="13" t="n">
-        <v>-0.0001254174117647059</v>
+        <v>-0.0001363350588235294</v>
       </c>
       <c r="AI92" s="13" t="n">
-        <v>-0.01128093121693122</v>
+        <v>-0.0122629417989418</v>
       </c>
     </row>
     <row r="93">
@@ -19934,17 +20216,23 @@
       <c r="AC93" s="15" t="n">
         <v>-1.479210293333333</v>
       </c>
-      <c r="AD93" s="15" t="n"/>
-      <c r="AE93" s="15" t="n"/>
-      <c r="AF93" s="15" t="n"/>
+      <c r="AD93" s="15" t="n">
+        <v>-6.941943</v>
+      </c>
+      <c r="AE93" s="15" t="n">
+        <v>-0.0004083495882352941</v>
+      </c>
+      <c r="AF93" s="15" t="n">
+        <v>-0.03672985714285714</v>
+      </c>
       <c r="AG93" s="15" t="n">
-        <v>-279.5707454400001</v>
+        <v>-286.51268844</v>
       </c>
       <c r="AH93" s="15" t="n">
-        <v>-0.01644533796705882</v>
+        <v>-0.01685368755529412</v>
       </c>
       <c r="AI93" s="15" t="n">
-        <v>-1.479210293333333</v>
+        <v>-1.51594015047619</v>
       </c>
     </row>
     <row r="94">
@@ -20156,17 +20444,23 @@
       <c r="AC96" s="13" t="n">
         <v>-1.044235444444444</v>
       </c>
-      <c r="AD96" s="13" t="n"/>
-      <c r="AE96" s="13" t="n"/>
-      <c r="AF96" s="13" t="n"/>
+      <c r="AD96" s="13" t="n">
+        <v>-62.917</v>
+      </c>
+      <c r="AE96" s="13" t="n">
+        <v>-0.003701</v>
+      </c>
+      <c r="AF96" s="13" t="n">
+        <v>-0.3328941798941799</v>
+      </c>
       <c r="AG96" s="13" t="n">
-        <v>-197.360499</v>
+        <v>-260.277499</v>
       </c>
       <c r="AH96" s="13" t="n">
-        <v>-0.01160944111764706</v>
+        <v>-0.01531044111764706</v>
       </c>
       <c r="AI96" s="13" t="n">
-        <v>-1.044235444444444</v>
+        <v>-1.377129624338624</v>
       </c>
     </row>
     <row r="97">
@@ -20256,17 +20550,23 @@
       <c r="AC97" s="11" t="n">
         <v>-37.06659381195767</v>
       </c>
-      <c r="AD97" s="11" t="n"/>
-      <c r="AE97" s="11" t="n"/>
-      <c r="AF97" s="11" t="n"/>
+      <c r="AD97" s="11" t="n">
+        <v>-10.078098</v>
+      </c>
+      <c r="AE97" s="11" t="n">
+        <v>-0.0005928292941176471</v>
+      </c>
+      <c r="AF97" s="11" t="n">
+        <v>-0.05332326984126984</v>
+      </c>
       <c r="AG97" s="11" t="n">
-        <v>-7005.58623046</v>
+        <v>-7015.66432846</v>
       </c>
       <c r="AH97" s="11" t="n">
-        <v>-0.4120933076741176</v>
+        <v>-0.4126861369682353</v>
       </c>
       <c r="AI97" s="11" t="n">
-        <v>-37.06659381195767</v>
+        <v>-37.11991708179895</v>
       </c>
     </row>
     <row r="98">
@@ -20356,17 +20656,23 @@
       <c r="AC98" s="13" t="n">
         <v>-1.168025571428572</v>
       </c>
-      <c r="AD98" s="13" t="n"/>
-      <c r="AE98" s="13" t="n"/>
-      <c r="AF98" s="13" t="n"/>
+      <c r="AD98" s="13" t="n">
+        <v>-63.412411</v>
+      </c>
+      <c r="AE98" s="13" t="n">
+        <v>-0.003730141823529412</v>
+      </c>
+      <c r="AF98" s="13" t="n">
+        <v>-0.3355154021164021</v>
+      </c>
       <c r="AG98" s="13" t="n">
-        <v>-220.756833</v>
+        <v>-284.169244</v>
       </c>
       <c r="AH98" s="13" t="n">
-        <v>-0.01298569605882353</v>
+        <v>-0.01671583788235294</v>
       </c>
       <c r="AI98" s="13" t="n">
-        <v>-1.168025571428572</v>
+        <v>-1.503540973544974</v>
       </c>
     </row>
     <row r="99">
@@ -20456,17 +20762,23 @@
       <c r="AC99" s="11" t="n">
         <v>-1.762867232804233</v>
       </c>
-      <c r="AD99" s="11" t="n"/>
-      <c r="AE99" s="11" t="n"/>
-      <c r="AF99" s="11" t="n"/>
+      <c r="AD99" s="11" t="n">
+        <v>-9.445</v>
+      </c>
+      <c r="AE99" s="11" t="n">
+        <v>-0.0005555882352941176</v>
+      </c>
+      <c r="AF99" s="11" t="n">
+        <v>-0.04997354497354498</v>
+      </c>
       <c r="AG99" s="11" t="n">
-        <v>-333.181907</v>
+        <v>-342.626907</v>
       </c>
       <c r="AH99" s="11" t="n">
-        <v>-0.01959893570588235</v>
+        <v>-0.02015452394117647</v>
       </c>
       <c r="AI99" s="11" t="n">
-        <v>-1.762867232804233</v>
+        <v>-1.812840777777778</v>
       </c>
     </row>
     <row r="100">
@@ -20556,17 +20868,23 @@
       <c r="AC100" s="15" t="n">
         <v>-41.51317338338624</v>
       </c>
-      <c r="AD100" s="15" t="n"/>
-      <c r="AE100" s="15" t="n"/>
-      <c r="AF100" s="15" t="n"/>
+      <c r="AD100" s="15" t="n">
+        <v>-145.852509</v>
+      </c>
+      <c r="AE100" s="15" t="n">
+        <v>-0.008579559352941177</v>
+      </c>
+      <c r="AF100" s="15" t="n">
+        <v>-0.7717063968253968</v>
+      </c>
       <c r="AG100" s="15" t="n">
-        <v>-7845.98976946</v>
+        <v>-7991.842278460001</v>
       </c>
       <c r="AH100" s="15" t="n">
-        <v>-0.4615288099682353</v>
+        <v>-0.4701083693211765</v>
       </c>
       <c r="AI100" s="15" t="n">
-        <v>-41.51317338338624</v>
+        <v>-42.28487978021163</v>
       </c>
     </row>
     <row r="101">
@@ -20696,17 +21014,23 @@
       <c r="AC102" s="11" t="n">
         <v>-1.060289031746032</v>
       </c>
-      <c r="AD102" s="11" t="n"/>
-      <c r="AE102" s="11" t="n"/>
-      <c r="AF102" s="11" t="n"/>
+      <c r="AD102" s="11" t="n">
+        <v>-15.9752</v>
+      </c>
+      <c r="AE102" s="11" t="n">
+        <v>-0.0009397176470588235</v>
+      </c>
+      <c r="AF102" s="11" t="n">
+        <v>-0.08452486772486772</v>
+      </c>
       <c r="AG102" s="11" t="n">
-        <v>-200.394627</v>
+        <v>-216.369827</v>
       </c>
       <c r="AH102" s="11" t="n">
-        <v>-0.01178791923529412</v>
+        <v>-0.01272763688235294</v>
       </c>
       <c r="AI102" s="11" t="n">
-        <v>-1.060289031746032</v>
+        <v>-1.144813899470899</v>
       </c>
     </row>
     <row r="103">
@@ -20796,17 +21120,23 @@
       <c r="AC103" s="13" t="n">
         <v>-1.561337105820106</v>
       </c>
-      <c r="AD103" s="13" t="n"/>
-      <c r="AE103" s="13" t="n"/>
-      <c r="AF103" s="13" t="n"/>
+      <c r="AD103" s="13" t="n">
+        <v>-32.770247</v>
+      </c>
+      <c r="AE103" s="13" t="n">
+        <v>-0.001927661588235294</v>
+      </c>
+      <c r="AF103" s="13" t="n">
+        <v>-0.1733875502645502</v>
+      </c>
       <c r="AG103" s="13" t="n">
-        <v>-295.092713</v>
+        <v>-327.86296</v>
       </c>
       <c r="AH103" s="13" t="n">
-        <v>-0.01735839488235294</v>
+        <v>-0.01928605647058823</v>
       </c>
       <c r="AI103" s="13" t="n">
-        <v>-1.561337105820106</v>
+        <v>-1.734724656084656</v>
       </c>
     </row>
     <row r="104">
@@ -20896,17 +21226,23 @@
       <c r="AC104" s="11" t="n">
         <v>-7.974517291005291</v>
       </c>
-      <c r="AD104" s="11" t="n"/>
-      <c r="AE104" s="11" t="n"/>
-      <c r="AF104" s="11" t="n"/>
+      <c r="AD104" s="11" t="n">
+        <v>-37.147399</v>
+      </c>
+      <c r="AE104" s="11" t="n">
+        <v>-0.002185141117647059</v>
+      </c>
+      <c r="AF104" s="11" t="n">
+        <v>-0.1965470846560847</v>
+      </c>
       <c r="AG104" s="11" t="n">
-        <v>-1507.183768</v>
+        <v>-1544.331167</v>
       </c>
       <c r="AH104" s="11" t="n">
-        <v>-0.08865786870588234</v>
+        <v>-0.0908430098235294</v>
       </c>
       <c r="AI104" s="11" t="n">
-        <v>-7.974517291005291</v>
+        <v>-8.171064375661377</v>
       </c>
     </row>
     <row r="105">
@@ -21090,17 +21426,23 @@
       <c r="AC106" s="15" t="n">
         <v>-11.65005779365079</v>
       </c>
-      <c r="AD106" s="15" t="n"/>
-      <c r="AE106" s="15" t="n"/>
-      <c r="AF106" s="15" t="n"/>
+      <c r="AD106" s="15" t="n">
+        <v>-85.89284600000001</v>
+      </c>
+      <c r="AE106" s="15" t="n">
+        <v>-0.005052520352941177</v>
+      </c>
+      <c r="AF106" s="15" t="n">
+        <v>-0.4544595026455027</v>
+      </c>
       <c r="AG106" s="15" t="n">
-        <v>-2201.860923</v>
+        <v>-2287.753769</v>
       </c>
       <c r="AH106" s="15" t="n">
-        <v>-0.1295212307647059</v>
+        <v>-0.1345737511176471</v>
       </c>
       <c r="AI106" s="15" t="n">
-        <v>-11.65005779365079</v>
+        <v>-12.10451729629629</v>
       </c>
     </row>
     <row r="107">
@@ -21288,17 +21630,23 @@
       <c r="AC109" s="13" t="n">
         <v>-0.0435899470899471</v>
       </c>
-      <c r="AD109" s="13" t="n"/>
-      <c r="AE109" s="13" t="n"/>
-      <c r="AF109" s="13" t="n"/>
+      <c r="AD109" s="13" t="n">
+        <v>-0.4875</v>
+      </c>
+      <c r="AE109" s="13" t="n">
+        <v>-2.867647058823529e-05</v>
+      </c>
+      <c r="AF109" s="13" t="n">
+        <v>-0.002579365079365079</v>
+      </c>
       <c r="AG109" s="13" t="n">
-        <v>-8.2385</v>
+        <v>-8.726000000000001</v>
       </c>
       <c r="AH109" s="13" t="n">
-        <v>-0.0004846176470588235</v>
+        <v>-0.0005132941176470588</v>
       </c>
       <c r="AI109" s="13" t="n">
-        <v>-0.0435899470899471</v>
+        <v>-0.04616931216931217</v>
       </c>
     </row>
     <row r="110">
@@ -21388,17 +21736,23 @@
       <c r="AC110" s="11" t="n">
         <v>-2.481355084656085</v>
       </c>
-      <c r="AD110" s="11" t="n"/>
-      <c r="AE110" s="11" t="n"/>
-      <c r="AF110" s="11" t="n"/>
+      <c r="AD110" s="11" t="n">
+        <v>-22.4428</v>
+      </c>
+      <c r="AE110" s="11" t="n">
+        <v>-0.001320164705882353</v>
+      </c>
+      <c r="AF110" s="11" t="n">
+        <v>-0.1187449735449735</v>
+      </c>
       <c r="AG110" s="11" t="n">
-        <v>-468.9761110000001</v>
+        <v>-491.418911</v>
       </c>
       <c r="AH110" s="11" t="n">
-        <v>-0.02758683005882353</v>
+        <v>-0.02890699476470588</v>
       </c>
       <c r="AI110" s="11" t="n">
-        <v>-2.481355084656085</v>
+        <v>-2.600100058201058</v>
       </c>
     </row>
     <row r="111">
@@ -21488,17 +21842,23 @@
       <c r="AC111" s="15" t="n">
         <v>-3.272307994708995</v>
       </c>
-      <c r="AD111" s="15" t="n"/>
-      <c r="AE111" s="15" t="n"/>
-      <c r="AF111" s="15" t="n"/>
+      <c r="AD111" s="15" t="n">
+        <v>-22.9303</v>
+      </c>
+      <c r="AE111" s="15" t="n">
+        <v>-0.001348841176470588</v>
+      </c>
+      <c r="AF111" s="15" t="n">
+        <v>-0.1213243386243386</v>
+      </c>
       <c r="AG111" s="15" t="n">
-        <v>-618.4662109999999</v>
+        <v>-641.3965109999999</v>
       </c>
       <c r="AH111" s="15" t="n">
-        <v>-0.03638036535294117</v>
+        <v>-0.03772920652941177</v>
       </c>
       <c r="AI111" s="15" t="n">
-        <v>-3.272307994708995</v>
+        <v>-3.393632333333334</v>
       </c>
     </row>
     <row r="112">
@@ -21880,17 +22240,23 @@
       <c r="AC116" s="13" t="n">
         <v>-2.608159126984127</v>
       </c>
-      <c r="AD116" s="13" t="n"/>
-      <c r="AE116" s="13" t="n"/>
-      <c r="AF116" s="13" t="n"/>
+      <c r="AD116" s="13" t="n">
+        <v>-16.713035</v>
+      </c>
+      <c r="AE116" s="13" t="n">
+        <v>-0.000983119705882353</v>
+      </c>
+      <c r="AF116" s="13" t="n">
+        <v>-0.08842875661375663</v>
+      </c>
       <c r="AG116" s="13" t="n">
-        <v>-492.942075</v>
+        <v>-509.65511</v>
       </c>
       <c r="AH116" s="13" t="n">
-        <v>-0.02899659264705882</v>
+        <v>-0.02997971235294118</v>
       </c>
       <c r="AI116" s="13" t="n">
-        <v>-2.608159126984127</v>
+        <v>-2.696587883597883</v>
       </c>
     </row>
     <row r="117">
@@ -21980,17 +22346,23 @@
       <c r="AC117" s="15" t="n">
         <v>-5.476784973544974</v>
       </c>
-      <c r="AD117" s="15" t="n"/>
-      <c r="AE117" s="15" t="n"/>
-      <c r="AF117" s="15" t="n"/>
+      <c r="AD117" s="15" t="n">
+        <v>-16.713035</v>
+      </c>
+      <c r="AE117" s="15" t="n">
+        <v>-0.000983119705882353</v>
+      </c>
+      <c r="AF117" s="15" t="n">
+        <v>-0.08842875661375663</v>
+      </c>
       <c r="AG117" s="15" t="n">
-        <v>-1035.11236</v>
+        <v>-1051.825395</v>
       </c>
       <c r="AH117" s="15" t="n">
-        <v>-0.06088896235294118</v>
+        <v>-0.06187208205882353</v>
       </c>
       <c r="AI117" s="15" t="n">
-        <v>-5.476784973544974</v>
+        <v>-5.565213730158731</v>
       </c>
     </row>
     <row r="118">
@@ -22121,22 +22493,22 @@
         <v>-29.76420624867725</v>
       </c>
       <c r="AD119" s="11" t="n">
-        <v>-2.95</v>
+        <v>-377.54405</v>
       </c>
       <c r="AE119" s="11" t="n">
-        <v>-0.0001735294117647059</v>
+        <v>-0.02220847352941177</v>
       </c>
       <c r="AF119" s="11" t="n">
-        <v>-0.01560846560846561</v>
+        <v>-1.997587566137566</v>
       </c>
       <c r="AG119" s="11" t="n">
-        <v>-5628.384980999999</v>
+        <v>-6002.979031</v>
       </c>
       <c r="AH119" s="11" t="n">
-        <v>-0.3310814694705882</v>
+        <v>-0.3531164135882353</v>
       </c>
       <c r="AI119" s="11" t="n">
-        <v>-29.77981471428572</v>
+        <v>-31.76179381481482</v>
       </c>
     </row>
     <row r="120">
@@ -22227,22 +22599,22 @@
         <v>-29.76420624867725</v>
       </c>
       <c r="AD120" s="15" t="n">
-        <v>-2.95</v>
+        <v>-377.54405</v>
       </c>
       <c r="AE120" s="15" t="n">
-        <v>-0.0001735294117647059</v>
+        <v>-0.02220847352941177</v>
       </c>
       <c r="AF120" s="15" t="n">
-        <v>-0.01560846560846561</v>
+        <v>-1.997587566137566</v>
       </c>
       <c r="AG120" s="15" t="n">
-        <v>-5628.384980999999</v>
+        <v>-6002.979031</v>
       </c>
       <c r="AH120" s="15" t="n">
-        <v>-0.3310814694705882</v>
+        <v>-0.3531164135882353</v>
       </c>
       <c r="AI120" s="15" t="n">
-        <v>-29.77981471428572</v>
+        <v>-31.76179381481482</v>
       </c>
     </row>
     <row r="121">
@@ -22607,22 +22979,22 @@
         <v>-5.069808166825397</v>
       </c>
       <c r="AD125" s="13" t="n">
-        <v>-1.548525</v>
+        <v>-123.6755</v>
       </c>
       <c r="AE125" s="13" t="n">
-        <v>-9.108970588235293e-05</v>
+        <v>-0.007275029411764706</v>
       </c>
       <c r="AF125" s="13" t="n">
-        <v>-0.008193253968253968</v>
+        <v>-0.6543677248677249</v>
       </c>
       <c r="AG125" s="13" t="n">
-        <v>-959.74226853</v>
+        <v>-1081.86924353</v>
       </c>
       <c r="AH125" s="13" t="n">
-        <v>-0.05645542756058824</v>
+        <v>-0.06363936726647058</v>
       </c>
       <c r="AI125" s="13" t="n">
-        <v>-5.078001420793651</v>
+        <v>-5.724175891693122</v>
       </c>
     </row>
     <row r="126">
@@ -22807,22 +23179,22 @@
         <v>-75.76880329100528</v>
       </c>
       <c r="AD127" s="13" t="n">
-        <v>-6.813775</v>
+        <v>-34.29895</v>
       </c>
       <c r="AE127" s="13" t="n">
-        <v>-0.000400810294117647</v>
+        <v>-0.002017585294117647</v>
       </c>
       <c r="AF127" s="13" t="n">
-        <v>-0.03605171957671958</v>
+        <v>-0.1814759259259259</v>
       </c>
       <c r="AG127" s="13" t="n">
-        <v>-14327.117597</v>
+        <v>-14354.602772</v>
       </c>
       <c r="AH127" s="13" t="n">
-        <v>-0.8427716233529411</v>
+        <v>-0.8443883983529411</v>
       </c>
       <c r="AI127" s="13" t="n">
-        <v>-75.804855010582</v>
+        <v>-75.95027921693121</v>
       </c>
     </row>
     <row r="128">
@@ -23019,22 +23391,22 @@
         <v>-132.568430727672</v>
       </c>
       <c r="AD129" s="15" t="n">
-        <v>-67.46126599999999</v>
+        <v>-217.073416</v>
       </c>
       <c r="AE129" s="15" t="n">
-        <v>-0.003968309764705882</v>
+        <v>-0.01276902447058824</v>
       </c>
       <c r="AF129" s="15" t="n">
-        <v>-0.3569379153439153</v>
+        <v>-1.148536592592593</v>
       </c>
       <c r="AG129" s="15" t="n">
-        <v>-25122.89467353</v>
+        <v>-25272.50682353</v>
       </c>
       <c r="AH129" s="15" t="n">
-        <v>-1.477817333737059</v>
+        <v>-1.486618048442941</v>
       </c>
       <c r="AI129" s="15" t="n">
-        <v>-132.9253686430159</v>
+        <v>-133.7169673202646</v>
       </c>
     </row>
     <row r="130">
@@ -23152,17 +23524,23 @@
       <c r="AC131" s="11" t="n">
         <v>-0.1705889947089947</v>
       </c>
-      <c r="AD131" s="11" t="n"/>
-      <c r="AE131" s="11" t="n"/>
-      <c r="AF131" s="11" t="n"/>
+      <c r="AD131" s="11" t="n">
+        <v>-1.5135</v>
+      </c>
+      <c r="AE131" s="11" t="n">
+        <v>-8.902941176470589e-05</v>
+      </c>
+      <c r="AF131" s="11" t="n">
+        <v>-0.008007936507936509</v>
+      </c>
       <c r="AG131" s="11" t="n">
-        <v>-32.24132</v>
+        <v>-33.75482</v>
       </c>
       <c r="AH131" s="11" t="n">
-        <v>-0.001896548235294118</v>
+        <v>-0.001985577647058824</v>
       </c>
       <c r="AI131" s="11" t="n">
-        <v>-0.1705889947089947</v>
+        <v>-0.1785969312169312</v>
       </c>
     </row>
     <row r="132">
@@ -23240,17 +23618,23 @@
       <c r="AC132" s="13" t="n">
         <v>-1.669307211640212</v>
       </c>
-      <c r="AD132" s="13" t="n"/>
-      <c r="AE132" s="13" t="n"/>
-      <c r="AF132" s="13" t="n"/>
+      <c r="AD132" s="13" t="n">
+        <v>-88.41812899999999</v>
+      </c>
+      <c r="AE132" s="13" t="n">
+        <v>-0.005201066411764706</v>
+      </c>
+      <c r="AF132" s="13" t="n">
+        <v>-0.4678207883597883</v>
+      </c>
       <c r="AG132" s="13" t="n">
-        <v>-315.499063</v>
+        <v>-403.917192</v>
       </c>
       <c r="AH132" s="13" t="n">
-        <v>-0.01855876841176471</v>
+        <v>-0.02375983482352942</v>
       </c>
       <c r="AI132" s="13" t="n">
-        <v>-1.669307211640212</v>
+        <v>-2.137128</v>
       </c>
     </row>
     <row r="133">
@@ -23428,17 +23812,23 @@
       <c r="AC134" s="13" t="n">
         <v>-0.5550766825396826</v>
       </c>
-      <c r="AD134" s="13" t="n"/>
-      <c r="AE134" s="13" t="n"/>
-      <c r="AF134" s="13" t="n"/>
+      <c r="AD134" s="13" t="n">
+        <v>-4.345</v>
+      </c>
+      <c r="AE134" s="13" t="n">
+        <v>-0.0002555882352941176</v>
+      </c>
+      <c r="AF134" s="13" t="n">
+        <v>-0.02298941798941799</v>
+      </c>
       <c r="AG134" s="13" t="n">
-        <v>-104.909493</v>
+        <v>-109.254493</v>
       </c>
       <c r="AH134" s="13" t="n">
-        <v>-0.006171146647058824</v>
+        <v>-0.006426734882352941</v>
       </c>
       <c r="AI134" s="13" t="n">
-        <v>-0.5550766825396826</v>
+        <v>-0.5780661005291006</v>
       </c>
     </row>
     <row r="135">
@@ -23522,17 +23912,23 @@
       <c r="AC135" s="11" t="n">
         <v>-1.057244523809524</v>
       </c>
-      <c r="AD135" s="11" t="n"/>
-      <c r="AE135" s="11" t="n"/>
-      <c r="AF135" s="11" t="n"/>
+      <c r="AD135" s="11" t="n">
+        <v>-0.882612</v>
+      </c>
+      <c r="AE135" s="11" t="n">
+        <v>-5.191835294117647e-05</v>
+      </c>
+      <c r="AF135" s="11" t="n">
+        <v>-0.004669904761904761</v>
+      </c>
       <c r="AG135" s="11" t="n">
-        <v>-199.819215</v>
+        <v>-200.701827</v>
       </c>
       <c r="AH135" s="11" t="n">
-        <v>-0.01175407147058824</v>
+        <v>-0.01180598982352941</v>
       </c>
       <c r="AI135" s="11" t="n">
-        <v>-1.057244523809524</v>
+        <v>-1.061914428571429</v>
       </c>
     </row>
     <row r="136">
@@ -23586,17 +23982,23 @@
       <c r="AC136" s="13" t="n">
         <v>-0.006195767195767196</v>
       </c>
-      <c r="AD136" s="13" t="n"/>
-      <c r="AE136" s="13" t="n"/>
-      <c r="AF136" s="13" t="n"/>
+      <c r="AD136" s="13" t="n">
+        <v>-0.5785</v>
+      </c>
+      <c r="AE136" s="13" t="n">
+        <v>-3.402941176470588e-05</v>
+      </c>
+      <c r="AF136" s="13" t="n">
+        <v>-0.003060846560846561</v>
+      </c>
       <c r="AG136" s="13" t="n">
-        <v>-1.171</v>
+        <v>-1.7495</v>
       </c>
       <c r="AH136" s="13" t="n">
-        <v>-6.888235294117648e-05</v>
+        <v>-0.0001029117647058824</v>
       </c>
       <c r="AI136" s="13" t="n">
-        <v>-0.006195767195767196</v>
+        <v>-0.009256613756613758</v>
       </c>
     </row>
     <row r="137">
@@ -23686,17 +24088,23 @@
       <c r="AC137" s="15" t="n">
         <v>-4.551761624338624</v>
       </c>
-      <c r="AD137" s="15" t="n"/>
-      <c r="AE137" s="15" t="n"/>
-      <c r="AF137" s="15" t="n"/>
+      <c r="AD137" s="15" t="n">
+        <v>-95.737741</v>
+      </c>
+      <c r="AE137" s="15" t="n">
+        <v>-0.005631631823529412</v>
+      </c>
+      <c r="AF137" s="15" t="n">
+        <v>-0.5065488941798941</v>
+      </c>
       <c r="AG137" s="15" t="n">
-        <v>-860.282947</v>
+        <v>-956.0206880000001</v>
       </c>
       <c r="AH137" s="15" t="n">
-        <v>-0.05060487923529412</v>
+        <v>-0.05623651105882353</v>
       </c>
       <c r="AI137" s="15" t="n">
-        <v>-4.551761624338624</v>
+        <v>-5.058310518518518</v>
       </c>
     </row>
     <row r="138">
@@ -23787,22 +24195,22 @@
         <v>-230.2759330393122</v>
       </c>
       <c r="AD138" s="15" t="n">
-        <v>-70.411266</v>
+        <v>-968.68584</v>
       </c>
       <c r="AE138" s="15" t="n">
-        <v>-0.004141839176470588</v>
+        <v>-0.05698152</v>
       </c>
       <c r="AF138" s="15" t="n">
-        <v>-0.372546380952381</v>
+        <v>-5.125321904761905</v>
       </c>
       <c r="AG138" s="15" t="n">
-        <v>-43592.56261043</v>
+        <v>-44490.83718443</v>
       </c>
       <c r="AH138" s="15" t="n">
-        <v>-2.564268388848823</v>
+        <v>-2.617108069672352</v>
       </c>
       <c r="AI138" s="15" t="n">
-        <v>-230.6484794202645</v>
+        <v>-235.4012549440741</v>
       </c>
     </row>
     <row r="139">
@@ -24015,22 +24423,22 @@
         <v>-4.894589497354497</v>
       </c>
       <c r="AD141" s="13" t="n">
-        <v>-60.7514</v>
+        <v>-61.7514</v>
       </c>
       <c r="AE141" s="13" t="n">
-        <v>-0.003573611764705882</v>
+        <v>-0.003632435294117647</v>
       </c>
       <c r="AF141" s="13" t="n">
-        <v>-0.3214359788359788</v>
+        <v>-0.3267269841269841</v>
       </c>
       <c r="AG141" s="13" t="n">
-        <v>-985.8288150000001</v>
+        <v>-986.8288150000001</v>
       </c>
       <c r="AH141" s="13" t="n">
-        <v>-0.05798993029411766</v>
+        <v>-0.05804875382352942</v>
       </c>
       <c r="AI141" s="13" t="n">
-        <v>-5.216025476190476</v>
+        <v>-5.221316481481481</v>
       </c>
     </row>
     <row r="142">
@@ -24237,22 +24645,22 @@
         <v>-13.73645722222222</v>
       </c>
       <c r="AD144" s="15" t="n">
-        <v>-60.7514</v>
+        <v>-61.7514</v>
       </c>
       <c r="AE144" s="15" t="n">
-        <v>-0.003573611764705882</v>
+        <v>-0.003632435294117647</v>
       </c>
       <c r="AF144" s="15" t="n">
-        <v>-0.3214359788359788</v>
+        <v>-0.3267269841269841</v>
       </c>
       <c r="AG144" s="15" t="n">
-        <v>-2656.941815</v>
+        <v>-2657.941815</v>
       </c>
       <c r="AH144" s="15" t="n">
-        <v>-0.156290695</v>
+        <v>-0.1563495185294118</v>
       </c>
       <c r="AI144" s="15" t="n">
-        <v>-14.0578932010582</v>
+        <v>-14.06318420634921</v>
       </c>
     </row>
     <row r="145">
@@ -24383,22 +24791,22 @@
         <v>-0.09944919407407407</v>
       </c>
       <c r="AD146" s="11" t="n">
-        <v>-0.0025</v>
+        <v>-0.0495</v>
       </c>
       <c r="AE146" s="11" t="n">
-        <v>-1.470588235294118e-07</v>
+        <v>-2.911764705882353e-06</v>
       </c>
       <c r="AF146" s="11" t="n">
-        <v>-1.322751322751323e-05</v>
+        <v>-0.0002619047619047619</v>
       </c>
       <c r="AG146" s="11" t="n">
-        <v>-18.79839768</v>
+        <v>-18.84539768</v>
       </c>
       <c r="AH146" s="11" t="n">
-        <v>-0.00110578809882353</v>
+        <v>-0.001108552804705883</v>
       </c>
       <c r="AI146" s="11" t="n">
-        <v>-0.09946242158730158</v>
+        <v>-0.09971109883597884</v>
       </c>
     </row>
     <row r="147">
@@ -24875,22 +25283,22 @@
         <v>-31.58386807253968</v>
       </c>
       <c r="AD152" s="15" t="n">
-        <v>-0.0025</v>
+        <v>-0.0495</v>
       </c>
       <c r="AE152" s="15" t="n">
-        <v>-1.470588235294118e-07</v>
+        <v>-2.911764705882353e-06</v>
       </c>
       <c r="AF152" s="15" t="n">
-        <v>-1.322751322751323e-05</v>
+        <v>-0.0002619047619047619</v>
       </c>
       <c r="AG152" s="15" t="n">
-        <v>-5969.35356571</v>
+        <v>-5969.400565710001</v>
       </c>
       <c r="AH152" s="15" t="n">
-        <v>-0.3511384450417648</v>
+        <v>-0.3511412097476472</v>
       </c>
       <c r="AI152" s="15" t="n">
-        <v>-31.58388130005291</v>
+        <v>-31.58412997730159</v>
       </c>
     </row>
     <row r="153">
@@ -24981,22 +25389,22 @@
         <v>-1529.478500653756</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-432.595564</v>
+        <v>-4302.881306</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-0.02544679788235294</v>
+        <v>-0.2531106650588236</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-2.288865417989418</v>
+        <v>-22.76656775661376</v>
       </c>
       <c r="AG153" s="19" t="n">
-        <v>-289504.0321875599</v>
+        <v>-293374.3179295599</v>
       </c>
       <c r="AH153" s="19" t="n">
-        <v>-17.02964895220941</v>
+        <v>-17.25731281938588</v>
       </c>
       <c r="AI153" s="19" t="n">
-        <v>-1531.767366071746</v>
+        <v>-1552.24506841037</v>
       </c>
     </row>
     <row r="154">
@@ -25087,22 +25495,22 @@
         <v>-349.2561074480424</v>
       </c>
       <c r="AD154" s="19" t="n">
-        <v>3442.000269</v>
+        <v>5598.73778</v>
       </c>
       <c r="AE154" s="19" t="n">
-        <v>0.2024706040588235</v>
+        <v>0.3293375164705882</v>
       </c>
       <c r="AF154" s="19" t="n">
-        <v>18.21164163492064</v>
+        <v>29.62295121693122</v>
       </c>
       <c r="AG154" s="19" t="n">
-        <v>-62567.40403868002</v>
+        <v>-60410.66652768001</v>
       </c>
       <c r="AH154" s="19" t="n">
-        <v>-3.68043553168706</v>
+        <v>-3.553568619275295</v>
       </c>
       <c r="AI154" s="19" t="n">
-        <v>-331.0444658131218</v>
+        <v>-319.6331562311112</v>
       </c>
     </row>
     <row r="155">
@@ -25193,22 +25601,22 @@
         <v>7.747388987724859</v>
       </c>
       <c r="AD155" s="7" t="n">
-        <v>4906.256787679999</v>
+        <v>7062.994298679999</v>
       </c>
       <c r="AE155" s="7" t="n">
-        <v>0.2886033404517646</v>
+        <v>0.4154702528635293</v>
       </c>
       <c r="AF155" s="7" t="n">
-        <v>25.9590306226455</v>
+        <v>37.37034020465608</v>
       </c>
       <c r="AG155" s="7" t="n">
-        <v>4906.256787679999</v>
+        <v>7062.994298679999</v>
       </c>
       <c r="AH155" s="7" t="n">
-        <v>0.2886033404517646</v>
+        <v>0.4154702528635293</v>
       </c>
       <c r="AI155" s="7" t="n">
-        <v>25.9590306226455</v>
+        <v>37.37034020465608</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Mon 09/14/2026 17:34
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 11 Sep 2026 16:51</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 14 Sep 2026 17:34</t>
         </is>
       </c>
     </row>
@@ -805,14 +805,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 11 Sep 2026</t>
+          <t>MTD as of 14 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 11 Sep 2026</t>
+          <t>YTD as of 14 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
@@ -1220,22 +1220,22 @@
         <v>914323824.5555556</v>
       </c>
       <c r="AD7" s="11" t="n">
-        <v>9886718086</v>
+        <v>9914560879</v>
       </c>
       <c r="AE7" s="11" t="n">
-        <v>581571.6521176471</v>
+        <v>583209.4634705882</v>
       </c>
       <c r="AF7" s="11" t="n">
-        <v>52310677.7037037</v>
+        <v>52457994.06878307</v>
       </c>
       <c r="AG7" s="11" t="n">
-        <v>182693920927</v>
+        <v>182721763720</v>
       </c>
       <c r="AH7" s="11" t="n">
-        <v>10746701.231</v>
+        <v>10748339.04235294</v>
       </c>
       <c r="AI7" s="11" t="n">
-        <v>966634502.2592592</v>
+        <v>966781818.6243386</v>
       </c>
     </row>
     <row r="8">
@@ -1402,22 +1402,22 @@
         <v>198819750.8201058</v>
       </c>
       <c r="AD9" s="11" t="n">
-        <v>3785340879</v>
+        <v>3813183672</v>
       </c>
       <c r="AE9" s="11" t="n">
-        <v>222667.1105294118</v>
+        <v>224304.9218823529</v>
       </c>
       <c r="AF9" s="11" t="n">
-        <v>20028258.61904762</v>
+        <v>20175574.98412699</v>
       </c>
       <c r="AG9" s="11" t="n">
-        <v>41362273784</v>
+        <v>41390116577</v>
       </c>
       <c r="AH9" s="11" t="n">
-        <v>2433074.928470588</v>
+        <v>2434712.739823529</v>
       </c>
       <c r="AI9" s="11" t="n">
-        <v>218848009.4391534</v>
+        <v>218995325.8042328</v>
       </c>
     </row>
     <row r="10">
@@ -2196,22 +2196,22 @@
         <v>2321849.073439153</v>
       </c>
       <c r="AD20" s="13" t="n">
-        <v>14901000</v>
+        <v>16017500</v>
       </c>
       <c r="AE20" s="13" t="n">
-        <v>876.5294117647059</v>
+        <v>942.2058823529412</v>
       </c>
       <c r="AF20" s="13" t="n">
-        <v>78841.26984126984</v>
+        <v>84748.67724867725</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>453730474.88</v>
+        <v>454846974.88</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>26690.02793411765</v>
+        <v>26755.70440470588</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>2400690.343280423</v>
+        <v>2406597.750687831</v>
       </c>
     </row>
     <row r="21">
@@ -2448,22 +2448,22 @@
         <v>332547.6190476191</v>
       </c>
       <c r="AD23" s="11" t="n">
-        <v>14528500</v>
+        <v>15645000</v>
       </c>
       <c r="AE23" s="11" t="n">
-        <v>854.6176470588235</v>
+        <v>920.2941176470588</v>
       </c>
       <c r="AF23" s="11" t="n">
-        <v>76870.37037037036</v>
+        <v>82777.77777777778</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>77380000</v>
+        <v>78496500</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>4551.764705882352</v>
+        <v>4617.441176470587</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>409417.9894179894</v>
+        <v>415325.3968253968</v>
       </c>
     </row>
     <row r="24">
@@ -3840,22 +3840,22 @@
         <v>1180222393.205714</v>
       </c>
       <c r="AD44" s="15" t="n">
-        <v>9901619086</v>
+        <v>9930578379</v>
       </c>
       <c r="AE44" s="15" t="n">
-        <v>582448.1815294118</v>
+        <v>584151.6693529412</v>
       </c>
       <c r="AF44" s="15" t="n">
-        <v>52389518.97354497</v>
+        <v>52542742.74603175</v>
       </c>
       <c r="AG44" s="15" t="n">
-        <v>232963651401.88</v>
+        <v>232992610694.88</v>
       </c>
       <c r="AH44" s="15" t="n">
-        <v>13703744.20011059</v>
+        <v>13705447.68793412</v>
       </c>
       <c r="AI44" s="15" t="n">
-        <v>1232611912.17926</v>
+        <v>1232765135.951746</v>
       </c>
     </row>
     <row r="45">
@@ -10252,22 +10252,22 @@
         <v>-1736052.91005291</v>
       </c>
       <c r="AD126" s="11" t="n">
-        <v>-7000000</v>
+        <v>-14000000</v>
       </c>
       <c r="AE126" s="11" t="n">
-        <v>-411.7647058823529</v>
+        <v>-823.5294117647059</v>
       </c>
       <c r="AF126" s="11" t="n">
-        <v>-37037.03703703704</v>
+        <v>-74074.07407407407</v>
       </c>
       <c r="AG126" s="11" t="n">
-        <v>-335114000</v>
+        <v>-342114000</v>
       </c>
       <c r="AH126" s="11" t="n">
-        <v>-19712.58823529412</v>
+        <v>-20124.35294117647</v>
       </c>
       <c r="AI126" s="11" t="n">
-        <v>-1773089.947089947</v>
+        <v>-1810126.984126984</v>
       </c>
     </row>
     <row r="127">
@@ -10570,22 +10570,22 @@
         <v>-132568430.7276719</v>
       </c>
       <c r="AD129" s="15" t="n">
-        <v>-217073416</v>
+        <v>-224073416</v>
       </c>
       <c r="AE129" s="15" t="n">
-        <v>-12769.02447058824</v>
+        <v>-13180.78917647059</v>
       </c>
       <c r="AF129" s="15" t="n">
-        <v>-1148536.592592593</v>
+        <v>-1185573.62962963</v>
       </c>
       <c r="AG129" s="15" t="n">
-        <v>-25272506823.53</v>
+        <v>-25279506823.53</v>
       </c>
       <c r="AH129" s="15" t="n">
-        <v>-1486618.048442941</v>
+        <v>-1487029.813148824</v>
       </c>
       <c r="AI129" s="15" t="n">
-        <v>-133716967.3202645</v>
+        <v>-133754004.3573016</v>
       </c>
     </row>
     <row r="130">
@@ -11374,22 +11374,22 @@
         <v>-230275933.0393122</v>
       </c>
       <c r="AD138" s="15" t="n">
-        <v>-968685840</v>
+        <v>-975685840</v>
       </c>
       <c r="AE138" s="15" t="n">
-        <v>-56981.52</v>
+        <v>-57393.28470588235</v>
       </c>
       <c r="AF138" s="15" t="n">
-        <v>-5125321.904761905</v>
+        <v>-5162358.941798942</v>
       </c>
       <c r="AG138" s="15" t="n">
-        <v>-44490837184.43001</v>
+        <v>-44497837184.43001</v>
       </c>
       <c r="AH138" s="15" t="n">
-        <v>-2617108.069672353</v>
+        <v>-2617519.834378236</v>
       </c>
       <c r="AI138" s="15" t="n">
-        <v>-235401254.9440741</v>
+        <v>-235438291.9811111</v>
       </c>
     </row>
     <row r="139">
@@ -12215,17 +12215,23 @@
       <c r="AC149" s="13" t="n">
         <v>-22574233.60544973</v>
       </c>
-      <c r="AD149" s="13" t="n"/>
-      <c r="AE149" s="13" t="n"/>
-      <c r="AF149" s="13" t="n"/>
+      <c r="AD149" s="13" t="n">
+        <v>-182522142</v>
+      </c>
+      <c r="AE149" s="13" t="n">
+        <v>-10736.59658823529</v>
+      </c>
+      <c r="AF149" s="13" t="n">
+        <v>-965725.6190476191</v>
+      </c>
       <c r="AG149" s="13" t="n">
-        <v>-4266530151.43</v>
+        <v>-4449052293.43</v>
       </c>
       <c r="AH149" s="13" t="n">
-        <v>-250972.3618488236</v>
+        <v>-261708.9584370588</v>
       </c>
       <c r="AI149" s="13" t="n">
-        <v>-22574233.60544973</v>
+        <v>-23539959.22449735</v>
       </c>
     </row>
     <row r="150">
@@ -12462,22 +12468,22 @@
         <v>-31583868.07253968</v>
       </c>
       <c r="AD152" s="15" t="n">
-        <v>-49500</v>
+        <v>-182571642</v>
       </c>
       <c r="AE152" s="15" t="n">
-        <v>-2.911764705882353</v>
+        <v>-10739.50835294118</v>
       </c>
       <c r="AF152" s="15" t="n">
-        <v>-261.9047619047619</v>
+        <v>-965987.5238095238</v>
       </c>
       <c r="AG152" s="15" t="n">
-        <v>-5969400565.710001</v>
+        <v>-6151922707.710001</v>
       </c>
       <c r="AH152" s="15" t="n">
-        <v>-351141.2097476471</v>
+        <v>-361877.8063358823</v>
       </c>
       <c r="AI152" s="15" t="n">
-        <v>-31584129.97730159</v>
+        <v>-32549855.59634921</v>
       </c>
     </row>
     <row r="153">
@@ -12568,22 +12574,22 @@
         <v>-1529478500.653757</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-4302881306</v>
+        <v>-4492403448</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-253110.6650588235</v>
+        <v>-264259.0263529412</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-22766567.75661376</v>
+        <v>-23769330.41269841</v>
       </c>
       <c r="AG153" s="19" t="n">
-        <v>-293374317929.5599</v>
+        <v>-293563840071.5599</v>
       </c>
       <c r="AH153" s="19" t="n">
-        <v>-17257312.81938588</v>
+        <v>-17268461.18068</v>
       </c>
       <c r="AI153" s="19" t="n">
-        <v>-1552245068.41037</v>
+        <v>-1553247831.066455</v>
       </c>
     </row>
     <row r="154">
@@ -12674,22 +12680,22 @@
         <v>-349256107.4480425</v>
       </c>
       <c r="AD154" s="19" t="n">
-        <v>5598737780</v>
+        <v>5438174931</v>
       </c>
       <c r="AE154" s="19" t="n">
-        <v>329337.5164705882</v>
+        <v>319892.643</v>
       </c>
       <c r="AF154" s="19" t="n">
-        <v>29622951.21693122</v>
+        <v>28773412.33333333</v>
       </c>
       <c r="AG154" s="19" t="n">
-        <v>-60410666527.68</v>
+        <v>-60571229376.68</v>
       </c>
       <c r="AH154" s="19" t="n">
-        <v>-3553568.619275295</v>
+        <v>-3563013.492745883</v>
       </c>
       <c r="AI154" s="19" t="n">
-        <v>-319633156.2311112</v>
+        <v>-320482695.1147091</v>
       </c>
     </row>
     <row r="155">
@@ -12780,22 +12786,22 @@
         <v>7747388.987724859</v>
       </c>
       <c r="AD155" s="7" t="n">
-        <v>7062994298.679998</v>
+        <v>6902431449.679998</v>
       </c>
       <c r="AE155" s="7" t="n">
-        <v>415470.2528635293</v>
+        <v>406025.3793929411</v>
       </c>
       <c r="AF155" s="7" t="n">
-        <v>37370340.20465608</v>
+        <v>36520801.32105819</v>
       </c>
       <c r="AG155" s="7" t="n">
-        <v>7062994298.679998</v>
+        <v>6902431449.679998</v>
       </c>
       <c r="AH155" s="7" t="n">
-        <v>415470.2528635293</v>
+        <v>406025.3793929411</v>
       </c>
       <c r="AI155" s="7" t="n">
-        <v>37370340.20465608</v>
+        <v>36520801.32105819</v>
       </c>
     </row>
   </sheetData>
@@ -13260,16 +13266,16 @@
         <v>1136676704</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>5476861296</v>
+        <v>5504704089</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>6613538000</v>
+        <v>6641380793</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>389031.6470588236</v>
+        <v>390669.4584117647</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>34992264.55026455</v>
+        <v>35139580.91534392</v>
       </c>
     </row>
     <row r="7">
@@ -13292,16 +13298,16 @@
         <v>7894080</v>
       </c>
       <c r="E7" s="13" t="n">
-        <v>185000000</v>
+        <v>2477858</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>192894080</v>
+        <v>10371938</v>
       </c>
       <c r="G7" s="24" t="n">
-        <v>11346.71058823529</v>
+        <v>610.114</v>
       </c>
       <c r="H7" s="24" t="n">
-        <v>1020603.597883598</v>
+        <v>54877.97883597884</v>
       </c>
     </row>
     <row r="8">
@@ -13356,16 +13362,16 @@
         <v>172976399.24</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>-63148516</v>
+        <v>-69032016</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>109827883.24</v>
+        <v>103944383.24</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>6460.463720000001</v>
+        <v>6114.375484705883</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>581099.9113227513</v>
+        <v>549970.2816931218</v>
       </c>
     </row>
     <row r="10">
@@ -13475,13 +13481,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>7062994300.679999</v>
+        <v>6902431451.679999</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>415470.2529811764</v>
+        <v>406025.3795105882</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>37370340.21523809</v>
+        <v>36520801.33164021</v>
       </c>
     </row>
   </sheetData>
@@ -13551,7 +13557,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 11 Sep 2026 16:51 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 14 Sep 2026 17:34 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -13626,14 +13632,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 11 Sep 2026</t>
+          <t>MTD as of 14 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 11 Sep 2026</t>
+          <t>YTD as of 14 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
@@ -14041,22 +14047,22 @@
         <v>914.3238245555556</v>
       </c>
       <c r="AD7" s="11" t="n">
-        <v>9886.718086000001</v>
+        <v>9914.560879000001</v>
       </c>
       <c r="AE7" s="11" t="n">
-        <v>0.5815716521176471</v>
+        <v>0.5832094634705882</v>
       </c>
       <c r="AF7" s="11" t="n">
-        <v>52.31067770370371</v>
+        <v>52.45799406878307</v>
       </c>
       <c r="AG7" s="11" t="n">
-        <v>182693.920927</v>
+        <v>182721.76372</v>
       </c>
       <c r="AH7" s="11" t="n">
-        <v>10.746701231</v>
+        <v>10.74833904235294</v>
       </c>
       <c r="AI7" s="11" t="n">
-        <v>966.6345022592593</v>
+        <v>966.7818186243386</v>
       </c>
     </row>
     <row r="8">
@@ -14223,22 +14229,22 @@
         <v>198.8197508201058</v>
       </c>
       <c r="AD9" s="11" t="n">
-        <v>3785.340879</v>
+        <v>3813.183672</v>
       </c>
       <c r="AE9" s="11" t="n">
-        <v>0.2226671105294118</v>
+        <v>0.224304921882353</v>
       </c>
       <c r="AF9" s="11" t="n">
-        <v>20.02825861904762</v>
+        <v>20.17557498412699</v>
       </c>
       <c r="AG9" s="11" t="n">
-        <v>41362.273784</v>
+        <v>41390.116577</v>
       </c>
       <c r="AH9" s="11" t="n">
-        <v>2.433074928470588</v>
+        <v>2.434712739823529</v>
       </c>
       <c r="AI9" s="11" t="n">
-        <v>218.8480094391534</v>
+        <v>218.9953258042328</v>
       </c>
     </row>
     <row r="10">
@@ -15017,22 +15023,22 @@
         <v>2.321849073439154</v>
       </c>
       <c r="AD20" s="13" t="n">
-        <v>14.901</v>
+        <v>16.0175</v>
       </c>
       <c r="AE20" s="13" t="n">
-        <v>0.0008765294117647059</v>
+        <v>0.000942205882352941</v>
       </c>
       <c r="AF20" s="13" t="n">
-        <v>0.07884126984126984</v>
+        <v>0.08474867724867724</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>453.73047488</v>
+        <v>454.8469748799999</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>0.02669002793411765</v>
+        <v>0.02675570440470589</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>2.400690343280424</v>
+        <v>2.406597750687831</v>
       </c>
     </row>
     <row r="21">
@@ -15269,22 +15275,22 @@
         <v>0.332547619047619</v>
       </c>
       <c r="AD23" s="11" t="n">
-        <v>14.5285</v>
+        <v>15.645</v>
       </c>
       <c r="AE23" s="11" t="n">
-        <v>0.0008546176470588235</v>
+        <v>0.0009202941176470588</v>
       </c>
       <c r="AF23" s="11" t="n">
-        <v>0.07687037037037037</v>
+        <v>0.08277777777777777</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>77.38</v>
+        <v>78.4965</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>0.004551764705882353</v>
+        <v>0.004617441176470589</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>0.4094179894179894</v>
+        <v>0.4153253968253968</v>
       </c>
     </row>
     <row r="24">
@@ -16661,22 +16667,22 @@
         <v>1180.222393205714</v>
       </c>
       <c r="AD44" s="15" t="n">
-        <v>9901.619086000001</v>
+        <v>9930.578379</v>
       </c>
       <c r="AE44" s="15" t="n">
-        <v>0.5824481815294118</v>
+        <v>0.5841516693529412</v>
       </c>
       <c r="AF44" s="15" t="n">
-        <v>52.38951897354497</v>
+        <v>52.54274274603175</v>
       </c>
       <c r="AG44" s="15" t="n">
-        <v>232963.65140188</v>
+        <v>232992.61069488</v>
       </c>
       <c r="AH44" s="15" t="n">
-        <v>13.70374420011059</v>
+        <v>13.70544768793412</v>
       </c>
       <c r="AI44" s="15" t="n">
-        <v>1232.611912179259</v>
+        <v>1232.765135951746</v>
       </c>
     </row>
     <row r="45">
@@ -23073,22 +23079,22 @@
         <v>-1.73605291005291</v>
       </c>
       <c r="AD126" s="11" t="n">
-        <v>-7</v>
+        <v>-14</v>
       </c>
       <c r="AE126" s="11" t="n">
-        <v>-0.000411764705882353</v>
+        <v>-0.0008235294117647059</v>
       </c>
       <c r="AF126" s="11" t="n">
-        <v>-0.03703703703703703</v>
+        <v>-0.07407407407407407</v>
       </c>
       <c r="AG126" s="11" t="n">
-        <v>-335.114</v>
+        <v>-342.114</v>
       </c>
       <c r="AH126" s="11" t="n">
-        <v>-0.01971258823529412</v>
+        <v>-0.02012435294117647</v>
       </c>
       <c r="AI126" s="11" t="n">
-        <v>-1.773089947089947</v>
+        <v>-1.810126984126984</v>
       </c>
     </row>
     <row r="127">
@@ -23391,22 +23397,22 @@
         <v>-132.568430727672</v>
       </c>
       <c r="AD129" s="15" t="n">
-        <v>-217.073416</v>
+        <v>-224.073416</v>
       </c>
       <c r="AE129" s="15" t="n">
-        <v>-0.01276902447058824</v>
+        <v>-0.01318078917647059</v>
       </c>
       <c r="AF129" s="15" t="n">
-        <v>-1.148536592592593</v>
+        <v>-1.18557362962963</v>
       </c>
       <c r="AG129" s="15" t="n">
-        <v>-25272.50682353</v>
+        <v>-25279.50682353</v>
       </c>
       <c r="AH129" s="15" t="n">
-        <v>-1.486618048442941</v>
+        <v>-1.487029813148824</v>
       </c>
       <c r="AI129" s="15" t="n">
-        <v>-133.7169673202646</v>
+        <v>-133.7540043573016</v>
       </c>
     </row>
     <row r="130">
@@ -24195,22 +24201,22 @@
         <v>-230.2759330393122</v>
       </c>
       <c r="AD138" s="15" t="n">
-        <v>-968.68584</v>
+        <v>-975.68584</v>
       </c>
       <c r="AE138" s="15" t="n">
-        <v>-0.05698152</v>
+        <v>-0.05739328470588236</v>
       </c>
       <c r="AF138" s="15" t="n">
-        <v>-5.125321904761905</v>
+        <v>-5.162358941798941</v>
       </c>
       <c r="AG138" s="15" t="n">
-        <v>-44490.83718443</v>
+        <v>-44497.83718443</v>
       </c>
       <c r="AH138" s="15" t="n">
-        <v>-2.617108069672352</v>
+        <v>-2.617519834378235</v>
       </c>
       <c r="AI138" s="15" t="n">
-        <v>-235.4012549440741</v>
+        <v>-235.4382919811111</v>
       </c>
     </row>
     <row r="139">
@@ -25036,17 +25042,23 @@
       <c r="AC149" s="13" t="n">
         <v>-22.57423360544974</v>
       </c>
-      <c r="AD149" s="13" t="n"/>
-      <c r="AE149" s="13" t="n"/>
-      <c r="AF149" s="13" t="n"/>
+      <c r="AD149" s="13" t="n">
+        <v>-182.522142</v>
+      </c>
+      <c r="AE149" s="13" t="n">
+        <v>-0.01073659658823529</v>
+      </c>
+      <c r="AF149" s="13" t="n">
+        <v>-0.9657256190476191</v>
+      </c>
       <c r="AG149" s="13" t="n">
-        <v>-4266.53015143</v>
+        <v>-4449.05229343</v>
       </c>
       <c r="AH149" s="13" t="n">
-        <v>-0.2509723618488235</v>
+        <v>-0.2617089584370588</v>
       </c>
       <c r="AI149" s="13" t="n">
-        <v>-22.57423360544974</v>
+        <v>-23.53995922449736</v>
       </c>
     </row>
     <row r="150">
@@ -25283,22 +25295,22 @@
         <v>-31.58386807253968</v>
       </c>
       <c r="AD152" s="15" t="n">
-        <v>-0.0495</v>
+        <v>-182.571642</v>
       </c>
       <c r="AE152" s="15" t="n">
-        <v>-2.911764705882353e-06</v>
+        <v>-0.01073950835294118</v>
       </c>
       <c r="AF152" s="15" t="n">
-        <v>-0.0002619047619047619</v>
+        <v>-0.9659875238095238</v>
       </c>
       <c r="AG152" s="15" t="n">
-        <v>-5969.400565710001</v>
+        <v>-6151.92270771</v>
       </c>
       <c r="AH152" s="15" t="n">
-        <v>-0.3511412097476472</v>
+        <v>-0.3618778063358825</v>
       </c>
       <c r="AI152" s="15" t="n">
-        <v>-31.58412997730159</v>
+        <v>-32.5498555963492</v>
       </c>
     </row>
     <row r="153">
@@ -25389,22 +25401,22 @@
         <v>-1529.478500653756</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-4302.881306</v>
+        <v>-4492.403448</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-0.2531106650588236</v>
+        <v>-0.2642590263529412</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-22.76656775661376</v>
+        <v>-23.76933041269841</v>
       </c>
       <c r="AG153" s="19" t="n">
-        <v>-293374.3179295599</v>
+        <v>-293563.8400715599</v>
       </c>
       <c r="AH153" s="19" t="n">
-        <v>-17.25731281938588</v>
+        <v>-17.26846118068</v>
       </c>
       <c r="AI153" s="19" t="n">
-        <v>-1552.24506841037</v>
+        <v>-1553.247831066455</v>
       </c>
     </row>
     <row r="154">
@@ -25495,22 +25507,22 @@
         <v>-349.2561074480424</v>
       </c>
       <c r="AD154" s="19" t="n">
-        <v>5598.73778</v>
+        <v>5438.174931</v>
       </c>
       <c r="AE154" s="19" t="n">
-        <v>0.3293375164705882</v>
+        <v>0.319892643</v>
       </c>
       <c r="AF154" s="19" t="n">
-        <v>29.62295121693122</v>
+        <v>28.77341233333333</v>
       </c>
       <c r="AG154" s="19" t="n">
-        <v>-60410.66652768001</v>
+        <v>-60571.22937668001</v>
       </c>
       <c r="AH154" s="19" t="n">
-        <v>-3.553568619275295</v>
+        <v>-3.563013492745883</v>
       </c>
       <c r="AI154" s="19" t="n">
-        <v>-319.6331562311112</v>
+        <v>-320.4826951147091</v>
       </c>
     </row>
     <row r="155">
@@ -25601,22 +25613,22 @@
         <v>7.747388987724859</v>
       </c>
       <c r="AD155" s="7" t="n">
-        <v>7062.994298679999</v>
+        <v>6902.431449679998</v>
       </c>
       <c r="AE155" s="7" t="n">
-        <v>0.4154702528635293</v>
+        <v>0.406025379392941</v>
       </c>
       <c r="AF155" s="7" t="n">
-        <v>37.37034020465608</v>
+        <v>36.52080132105819</v>
       </c>
       <c r="AG155" s="7" t="n">
-        <v>7062.994298679999</v>
+        <v>6902.431449679998</v>
       </c>
       <c r="AH155" s="7" t="n">
-        <v>0.4154702528635293</v>
+        <v>0.406025379392941</v>
       </c>
       <c r="AI155" s="7" t="n">
-        <v>37.37034020465608</v>
+        <v>36.52080132105819</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard 09/15/26 13:23
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 14 Sep 2026 17:34</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 15 Sep 2026 13:23</t>
         </is>
       </c>
     </row>
@@ -805,14 +805,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 14 Sep 2026</t>
+          <t>MTD as of 15 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 14 Sep 2026</t>
+          <t>YTD as of 15 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
@@ -13557,7 +13557,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 14 Sep 2026 17:34 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 15 Sep 2026 13:23 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -13632,14 +13632,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 14 Sep 2026</t>
+          <t>MTD as of 15 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 14 Sep 2026</t>
+          <t>YTD as of 15 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>

</xml_diff>

<commit_message>
Refresh dashboard 09/15/26 16:58
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 15 Sep 2026 13:23</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 15 Sep 2026 16:58</t>
         </is>
       </c>
     </row>
@@ -2196,22 +2196,22 @@
         <v>2321849.073439153</v>
       </c>
       <c r="AD20" s="13" t="n">
-        <v>16017500</v>
+        <v>17331270</v>
       </c>
       <c r="AE20" s="13" t="n">
-        <v>942.2058823529412</v>
+        <v>1019.486470588235</v>
       </c>
       <c r="AF20" s="13" t="n">
-        <v>84748.67724867725</v>
+        <v>91699.84126984127</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>454846974.88</v>
+        <v>456160744.88</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>26755.70440470588</v>
+        <v>26832.98499294118</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>2406597.750687831</v>
+        <v>2413548.914708995</v>
       </c>
     </row>
     <row r="21">
@@ -2448,22 +2448,22 @@
         <v>332547.6190476191</v>
       </c>
       <c r="AD23" s="11" t="n">
-        <v>15645000</v>
+        <v>16838500</v>
       </c>
       <c r="AE23" s="11" t="n">
-        <v>920.2941176470588</v>
+        <v>990.5</v>
       </c>
       <c r="AF23" s="11" t="n">
-        <v>82777.77777777778</v>
+        <v>89092.5925925926</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>78496500</v>
+        <v>79690000</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>4617.441176470587</v>
+        <v>4687.647058823529</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>415325.3968253968</v>
+        <v>421640.2116402116</v>
       </c>
     </row>
     <row r="24">
@@ -2780,22 +2780,22 @@
         <v>62858.95238095238</v>
       </c>
       <c r="AD28" s="13" t="n">
-        <v>372500</v>
+        <v>492770</v>
       </c>
       <c r="AE28" s="13" t="n">
-        <v>21.91176470588235</v>
+        <v>28.9864705882353</v>
       </c>
       <c r="AF28" s="13" t="n">
-        <v>1970.899470899471</v>
+        <v>2607.248677248677</v>
       </c>
       <c r="AG28" s="13" t="n">
-        <v>12252842</v>
+        <v>12373112</v>
       </c>
       <c r="AH28" s="13" t="n">
-        <v>720.7554117647057</v>
+        <v>727.8301176470587</v>
       </c>
       <c r="AI28" s="13" t="n">
-        <v>64829.85185185185</v>
+        <v>65466.20105820106</v>
       </c>
     </row>
     <row r="29">
@@ -3840,22 +3840,22 @@
         <v>1180222393.205714</v>
       </c>
       <c r="AD44" s="15" t="n">
-        <v>9930578379</v>
+        <v>9931892149</v>
       </c>
       <c r="AE44" s="15" t="n">
-        <v>584151.6693529412</v>
+        <v>584228.9499411765</v>
       </c>
       <c r="AF44" s="15" t="n">
-        <v>52542742.74603175</v>
+        <v>52549693.91005291</v>
       </c>
       <c r="AG44" s="15" t="n">
-        <v>232992610694.88</v>
+        <v>232993924464.88</v>
       </c>
       <c r="AH44" s="15" t="n">
-        <v>13705447.68793412</v>
+        <v>13705524.96852235</v>
       </c>
       <c r="AI44" s="15" t="n">
-        <v>1232765135.951746</v>
+        <v>1232772087.115767</v>
       </c>
     </row>
     <row r="45">
@@ -6376,22 +6376,22 @@
         <v>-48834989.68539683</v>
       </c>
       <c r="AD81" s="13" t="n">
-        <v>-1301257365</v>
+        <v>-1336140329</v>
       </c>
       <c r="AE81" s="13" t="n">
-        <v>-76544.55088235294</v>
+        <v>-78596.48994117646</v>
       </c>
       <c r="AF81" s="13" t="n">
-        <v>-6884959.603174604</v>
+        <v>-7069525.55026455</v>
       </c>
       <c r="AG81" s="13" t="n">
-        <v>-10531070415.54</v>
+        <v>-10565953379.54</v>
       </c>
       <c r="AH81" s="13" t="n">
-        <v>-619474.7303258823</v>
+        <v>-621526.6693847058</v>
       </c>
       <c r="AI81" s="13" t="n">
-        <v>-55719949.28857143</v>
+        <v>-55904515.23566138</v>
       </c>
     </row>
     <row r="82">
@@ -6688,22 +6688,22 @@
         <v>-126334224.2039154</v>
       </c>
       <c r="AD84" s="15" t="n">
-        <v>-2393567841</v>
+        <v>-2428450805</v>
       </c>
       <c r="AE84" s="15" t="n">
-        <v>-140798.1082941176</v>
+        <v>-142850.0473529412</v>
       </c>
       <c r="AF84" s="15" t="n">
-        <v>-12664380.11111111</v>
+        <v>-12848946.05820106</v>
       </c>
       <c r="AG84" s="15" t="n">
-        <v>-26270736215.54</v>
+        <v>-26305619179.54</v>
       </c>
       <c r="AH84" s="15" t="n">
-        <v>-1545337.42444353</v>
+        <v>-1547389.363502353</v>
       </c>
       <c r="AI84" s="15" t="n">
-        <v>-138998604.3150265</v>
+        <v>-139183170.2621164</v>
       </c>
     </row>
     <row r="85">
@@ -7836,22 +7836,22 @@
         <v>-1168025.571428571</v>
       </c>
       <c r="AD98" s="13" t="n">
-        <v>-63412411</v>
+        <v>-28529447</v>
       </c>
       <c r="AE98" s="13" t="n">
-        <v>-3730.141823529412</v>
+        <v>-1678.202764705882</v>
       </c>
       <c r="AF98" s="13" t="n">
-        <v>-335515.4021164021</v>
+        <v>-150949.455026455</v>
       </c>
       <c r="AG98" s="13" t="n">
-        <v>-284169244</v>
+        <v>-249286280</v>
       </c>
       <c r="AH98" s="13" t="n">
-        <v>-16715.83788235294</v>
+        <v>-14663.89882352941</v>
       </c>
       <c r="AI98" s="13" t="n">
-        <v>-1503540.973544973</v>
+        <v>-1318975.026455026</v>
       </c>
     </row>
     <row r="99">
@@ -8048,22 +8048,22 @@
         <v>-41513173.38338625</v>
       </c>
       <c r="AD100" s="15" t="n">
-        <v>-145852509</v>
+        <v>-110969545</v>
       </c>
       <c r="AE100" s="15" t="n">
-        <v>-8579.559352941176</v>
+        <v>-6527.620294117647</v>
       </c>
       <c r="AF100" s="15" t="n">
-        <v>-771706.3968253968</v>
+        <v>-587140.4497354497</v>
       </c>
       <c r="AG100" s="15" t="n">
-        <v>-7991842278.46</v>
+        <v>-7956959314.46</v>
       </c>
       <c r="AH100" s="15" t="n">
-        <v>-470108.3693211764</v>
+        <v>-468056.4302623529</v>
       </c>
       <c r="AI100" s="15" t="n">
-        <v>-42284879.78021164</v>
+        <v>-42100313.83312169</v>
       </c>
     </row>
     <row r="101">
@@ -10358,22 +10358,22 @@
         <v>-75768803.29100528</v>
       </c>
       <c r="AD127" s="13" t="n">
-        <v>-34298950</v>
+        <v>-34798950</v>
       </c>
       <c r="AE127" s="13" t="n">
-        <v>-2017.585294117647</v>
+        <v>-2046.997058823529</v>
       </c>
       <c r="AF127" s="13" t="n">
-        <v>-181475.9259259259</v>
+        <v>-184121.4285714286</v>
       </c>
       <c r="AG127" s="13" t="n">
-        <v>-14354602772</v>
+        <v>-14355102772</v>
       </c>
       <c r="AH127" s="13" t="n">
-        <v>-844388.3983529413</v>
+        <v>-844417.8101176471</v>
       </c>
       <c r="AI127" s="13" t="n">
-        <v>-75950279.21693121</v>
+        <v>-75952924.71957672</v>
       </c>
     </row>
     <row r="128">
@@ -10570,22 +10570,22 @@
         <v>-132568430.7276719</v>
       </c>
       <c r="AD129" s="15" t="n">
-        <v>-224073416</v>
+        <v>-224573416</v>
       </c>
       <c r="AE129" s="15" t="n">
-        <v>-13180.78917647059</v>
+        <v>-13210.20094117647</v>
       </c>
       <c r="AF129" s="15" t="n">
-        <v>-1185573.62962963</v>
+        <v>-1188219.132275132</v>
       </c>
       <c r="AG129" s="15" t="n">
-        <v>-25279506823.53</v>
+        <v>-25280006823.53</v>
       </c>
       <c r="AH129" s="15" t="n">
-        <v>-1487029.813148824</v>
+        <v>-1487059.224913529</v>
       </c>
       <c r="AI129" s="15" t="n">
-        <v>-133754004.3573016</v>
+        <v>-133756649.8599471</v>
       </c>
     </row>
     <row r="130">
@@ -11374,22 +11374,22 @@
         <v>-230275933.0393122</v>
       </c>
       <c r="AD138" s="15" t="n">
-        <v>-975685840</v>
+        <v>-941302876</v>
       </c>
       <c r="AE138" s="15" t="n">
-        <v>-57393.28470588235</v>
+        <v>-55370.75741176471</v>
       </c>
       <c r="AF138" s="15" t="n">
-        <v>-5162358.941798942</v>
+        <v>-4980438.497354497</v>
       </c>
       <c r="AG138" s="15" t="n">
-        <v>-44497837184.43001</v>
+        <v>-44463454220.43001</v>
       </c>
       <c r="AH138" s="15" t="n">
-        <v>-2617519.834378236</v>
+        <v>-2615497.307084118</v>
       </c>
       <c r="AI138" s="15" t="n">
-        <v>-235438291.9811111</v>
+        <v>-235256371.5366667</v>
       </c>
     </row>
     <row r="139">
@@ -12574,22 +12574,22 @@
         <v>-1529478500.653757</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-4492403448</v>
+        <v>-4492903448</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-264259.0263529412</v>
+        <v>-264288.4381176471</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-23769330.41269841</v>
+        <v>-23771975.91534391</v>
       </c>
       <c r="AG153" s="19" t="n">
-        <v>-293563840071.5599</v>
+        <v>-293564340071.5599</v>
       </c>
       <c r="AH153" s="19" t="n">
-        <v>-17268461.18068</v>
+        <v>-17268490.5924447</v>
       </c>
       <c r="AI153" s="19" t="n">
-        <v>-1553247831.066455</v>
+        <v>-1553250476.569101</v>
       </c>
     </row>
     <row r="154">
@@ -12680,22 +12680,22 @@
         <v>-349256107.4480425</v>
       </c>
       <c r="AD154" s="19" t="n">
-        <v>5438174931</v>
+        <v>5438988701</v>
       </c>
       <c r="AE154" s="19" t="n">
-        <v>319892.643</v>
+        <v>319940.5118235294</v>
       </c>
       <c r="AF154" s="19" t="n">
-        <v>28773412.33333333</v>
+        <v>28777717.994709</v>
       </c>
       <c r="AG154" s="19" t="n">
-        <v>-60571229376.68</v>
+        <v>-60570415606.68</v>
       </c>
       <c r="AH154" s="19" t="n">
-        <v>-3563013.492745883</v>
+        <v>-3562965.623922354</v>
       </c>
       <c r="AI154" s="19" t="n">
-        <v>-320482695.1147091</v>
+        <v>-320478389.4533334</v>
       </c>
     </row>
     <row r="155">
@@ -12786,22 +12786,22 @@
         <v>7747388.987724859</v>
       </c>
       <c r="AD155" s="7" t="n">
-        <v>6902431449.679998</v>
+        <v>6903245219.679998</v>
       </c>
       <c r="AE155" s="7" t="n">
-        <v>406025.3793929411</v>
+        <v>406073.2482164705</v>
       </c>
       <c r="AF155" s="7" t="n">
-        <v>36520801.32105819</v>
+        <v>36525106.98243386</v>
       </c>
       <c r="AG155" s="7" t="n">
-        <v>6902431449.679998</v>
+        <v>6903245219.679998</v>
       </c>
       <c r="AH155" s="7" t="n">
-        <v>406025.3793929411</v>
+        <v>406073.2482164705</v>
       </c>
       <c r="AI155" s="7" t="n">
-        <v>36520801.32105819</v>
+        <v>36525106.98243386</v>
       </c>
     </row>
   </sheetData>
@@ -13362,16 +13362,16 @@
         <v>172976399.24</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>-69032016</v>
+        <v>-68218246</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>103944383.24</v>
+        <v>104758153.24</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>6114.375484705883</v>
+        <v>6162.244308235295</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>549970.2816931218</v>
+        <v>554275.9430687831</v>
       </c>
     </row>
     <row r="10">
@@ -13481,13 +13481,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>6902431451.679999</v>
+        <v>6903245221.679999</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>406025.3795105882</v>
+        <v>406073.2483341176</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>36520801.33164021</v>
+        <v>36525106.99301587</v>
       </c>
     </row>
   </sheetData>
@@ -13557,7 +13557,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 15 Sep 2026 13:23 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 15 Sep 2026 16:58 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -15023,22 +15023,22 @@
         <v>2.321849073439154</v>
       </c>
       <c r="AD20" s="13" t="n">
-        <v>16.0175</v>
+        <v>17.33127</v>
       </c>
       <c r="AE20" s="13" t="n">
-        <v>0.000942205882352941</v>
+        <v>0.001019486470588235</v>
       </c>
       <c r="AF20" s="13" t="n">
-        <v>0.08474867724867724</v>
+        <v>0.09169984126984126</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>454.8469748799999</v>
+        <v>456.16074488</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>0.02675570440470589</v>
+        <v>0.02683298499294118</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>2.406597750687831</v>
+        <v>2.413548914708995</v>
       </c>
     </row>
     <row r="21">
@@ -15275,22 +15275,22 @@
         <v>0.332547619047619</v>
       </c>
       <c r="AD23" s="11" t="n">
-        <v>15.645</v>
+        <v>16.8385</v>
       </c>
       <c r="AE23" s="11" t="n">
-        <v>0.0009202941176470588</v>
+        <v>0.0009905000000000001</v>
       </c>
       <c r="AF23" s="11" t="n">
-        <v>0.08277777777777777</v>
+        <v>0.0890925925925926</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>78.4965</v>
+        <v>79.69</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>0.004617441176470589</v>
+        <v>0.00468764705882353</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>0.4153253968253968</v>
+        <v>0.4216402116402116</v>
       </c>
     </row>
     <row r="24">
@@ -15607,22 +15607,22 @@
         <v>0.06285895238095238</v>
       </c>
       <c r="AD28" s="13" t="n">
-        <v>0.3725</v>
+        <v>0.49277</v>
       </c>
       <c r="AE28" s="13" t="n">
-        <v>2.191176470588235e-05</v>
+        <v>2.898647058823529e-05</v>
       </c>
       <c r="AF28" s="13" t="n">
-        <v>0.001970899470899471</v>
+        <v>0.002607248677248677</v>
       </c>
       <c r="AG28" s="13" t="n">
-        <v>12.252842</v>
+        <v>12.373112</v>
       </c>
       <c r="AH28" s="13" t="n">
-        <v>0.0007207554117647059</v>
+        <v>0.0007278301176470588</v>
       </c>
       <c r="AI28" s="13" t="n">
-        <v>0.06482985185185185</v>
+        <v>0.06546620105820106</v>
       </c>
     </row>
     <row r="29">
@@ -16667,22 +16667,22 @@
         <v>1180.222393205714</v>
       </c>
       <c r="AD44" s="15" t="n">
-        <v>9930.578379</v>
+        <v>9931.892148999999</v>
       </c>
       <c r="AE44" s="15" t="n">
-        <v>0.5841516693529412</v>
+        <v>0.5842289499411765</v>
       </c>
       <c r="AF44" s="15" t="n">
-        <v>52.54274274603175</v>
+        <v>52.54969391005291</v>
       </c>
       <c r="AG44" s="15" t="n">
-        <v>232992.61069488</v>
+        <v>232993.92446488</v>
       </c>
       <c r="AH44" s="15" t="n">
-        <v>13.70544768793412</v>
+        <v>13.70552496852235</v>
       </c>
       <c r="AI44" s="15" t="n">
-        <v>1232.765135951746</v>
+        <v>1232.772087115767</v>
       </c>
     </row>
     <row r="45">
@@ -19203,22 +19203,22 @@
         <v>-48.83498968539683</v>
       </c>
       <c r="AD81" s="13" t="n">
-        <v>-1301.257365</v>
+        <v>-1336.140329</v>
       </c>
       <c r="AE81" s="13" t="n">
-        <v>-0.07654455088235294</v>
+        <v>-0.07859648994117648</v>
       </c>
       <c r="AF81" s="13" t="n">
-        <v>-6.884959603174603</v>
+        <v>-7.069525550264551</v>
       </c>
       <c r="AG81" s="13" t="n">
-        <v>-10531.07041554</v>
+        <v>-10565.95337954</v>
       </c>
       <c r="AH81" s="13" t="n">
-        <v>-0.6194747303258823</v>
+        <v>-0.6215266693847059</v>
       </c>
       <c r="AI81" s="13" t="n">
-        <v>-55.71994928857143</v>
+        <v>-55.90451523566138</v>
       </c>
     </row>
     <row r="82">
@@ -19515,22 +19515,22 @@
         <v>-126.3342242039153</v>
       </c>
       <c r="AD84" s="15" t="n">
-        <v>-2393.567841</v>
+        <v>-2428.450805</v>
       </c>
       <c r="AE84" s="15" t="n">
-        <v>-0.1407981082941177</v>
+        <v>-0.1428500473529412</v>
       </c>
       <c r="AF84" s="15" t="n">
-        <v>-12.66438011111111</v>
+        <v>-12.84894605820106</v>
       </c>
       <c r="AG84" s="15" t="n">
-        <v>-26270.73621554</v>
+        <v>-26305.61917954</v>
       </c>
       <c r="AH84" s="15" t="n">
-        <v>-1.545337424443529</v>
+        <v>-1.547389363502353</v>
       </c>
       <c r="AI84" s="15" t="n">
-        <v>-138.9986043150264</v>
+        <v>-139.1831702621164</v>
       </c>
     </row>
     <row r="85">
@@ -20663,22 +20663,22 @@
         <v>-1.168025571428572</v>
       </c>
       <c r="AD98" s="13" t="n">
-        <v>-63.412411</v>
+        <v>-28.529447</v>
       </c>
       <c r="AE98" s="13" t="n">
-        <v>-0.003730141823529412</v>
+        <v>-0.001678202764705882</v>
       </c>
       <c r="AF98" s="13" t="n">
-        <v>-0.3355154021164021</v>
+        <v>-0.150949455026455</v>
       </c>
       <c r="AG98" s="13" t="n">
-        <v>-284.169244</v>
+        <v>-249.28628</v>
       </c>
       <c r="AH98" s="13" t="n">
-        <v>-0.01671583788235294</v>
+        <v>-0.01466389882352941</v>
       </c>
       <c r="AI98" s="13" t="n">
-        <v>-1.503540973544974</v>
+        <v>-1.318975026455027</v>
       </c>
     </row>
     <row r="99">
@@ -20875,22 +20875,22 @@
         <v>-41.51317338338624</v>
       </c>
       <c r="AD100" s="15" t="n">
-        <v>-145.852509</v>
+        <v>-110.969545</v>
       </c>
       <c r="AE100" s="15" t="n">
-        <v>-0.008579559352941177</v>
+        <v>-0.006527620294117647</v>
       </c>
       <c r="AF100" s="15" t="n">
-        <v>-0.7717063968253968</v>
+        <v>-0.5871404497354498</v>
       </c>
       <c r="AG100" s="15" t="n">
-        <v>-7991.842278460001</v>
+        <v>-7956.95931446</v>
       </c>
       <c r="AH100" s="15" t="n">
-        <v>-0.4701083693211765</v>
+        <v>-0.4680564302623529</v>
       </c>
       <c r="AI100" s="15" t="n">
-        <v>-42.28487978021163</v>
+        <v>-42.10031383312169</v>
       </c>
     </row>
     <row r="101">
@@ -23185,22 +23185,22 @@
         <v>-75.76880329100528</v>
       </c>
       <c r="AD127" s="13" t="n">
-        <v>-34.29895</v>
+        <v>-34.79895</v>
       </c>
       <c r="AE127" s="13" t="n">
-        <v>-0.002017585294117647</v>
+        <v>-0.002046997058823529</v>
       </c>
       <c r="AF127" s="13" t="n">
-        <v>-0.1814759259259259</v>
+        <v>-0.1841214285714285</v>
       </c>
       <c r="AG127" s="13" t="n">
-        <v>-14354.602772</v>
+        <v>-14355.102772</v>
       </c>
       <c r="AH127" s="13" t="n">
-        <v>-0.8443883983529411</v>
+        <v>-0.8444178101176469</v>
       </c>
       <c r="AI127" s="13" t="n">
-        <v>-75.95027921693121</v>
+        <v>-75.95292471957671</v>
       </c>
     </row>
     <row r="128">
@@ -23397,22 +23397,22 @@
         <v>-132.568430727672</v>
       </c>
       <c r="AD129" s="15" t="n">
-        <v>-224.073416</v>
+        <v>-224.573416</v>
       </c>
       <c r="AE129" s="15" t="n">
-        <v>-0.01318078917647059</v>
+        <v>-0.01321020094117647</v>
       </c>
       <c r="AF129" s="15" t="n">
-        <v>-1.18557362962963</v>
+        <v>-1.188219132275132</v>
       </c>
       <c r="AG129" s="15" t="n">
-        <v>-25279.50682353</v>
+        <v>-25280.00682353</v>
       </c>
       <c r="AH129" s="15" t="n">
-        <v>-1.487029813148824</v>
+        <v>-1.48705922491353</v>
       </c>
       <c r="AI129" s="15" t="n">
-        <v>-133.7540043573016</v>
+        <v>-133.7566498599471</v>
       </c>
     </row>
     <row r="130">
@@ -24201,22 +24201,22 @@
         <v>-230.2759330393122</v>
       </c>
       <c r="AD138" s="15" t="n">
-        <v>-975.68584</v>
+        <v>-941.302876</v>
       </c>
       <c r="AE138" s="15" t="n">
-        <v>-0.05739328470588236</v>
+        <v>-0.05537075741176471</v>
       </c>
       <c r="AF138" s="15" t="n">
-        <v>-5.162358941798941</v>
+        <v>-4.980438497354498</v>
       </c>
       <c r="AG138" s="15" t="n">
-        <v>-44497.83718443</v>
+        <v>-44463.45422043</v>
       </c>
       <c r="AH138" s="15" t="n">
-        <v>-2.617519834378235</v>
+        <v>-2.615497307084117</v>
       </c>
       <c r="AI138" s="15" t="n">
-        <v>-235.4382919811111</v>
+        <v>-235.2563715366666</v>
       </c>
     </row>
     <row r="139">
@@ -25401,22 +25401,22 @@
         <v>-1529.478500653756</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-4492.403448</v>
+        <v>-4492.903448</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-0.2642590263529412</v>
+        <v>-0.2642884381176471</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-23.76933041269841</v>
+        <v>-23.77197591534392</v>
       </c>
       <c r="AG153" s="19" t="n">
-        <v>-293563.8400715599</v>
+        <v>-293564.3400715599</v>
       </c>
       <c r="AH153" s="19" t="n">
-        <v>-17.26846118068</v>
+        <v>-17.26849059244471</v>
       </c>
       <c r="AI153" s="19" t="n">
-        <v>-1553.247831066455</v>
+        <v>-1553.2504765691</v>
       </c>
     </row>
     <row r="154">
@@ -25507,22 +25507,22 @@
         <v>-349.2561074480424</v>
       </c>
       <c r="AD154" s="19" t="n">
-        <v>5438.174931</v>
+        <v>5438.988701</v>
       </c>
       <c r="AE154" s="19" t="n">
-        <v>0.319892643</v>
+        <v>0.3199405118235294</v>
       </c>
       <c r="AF154" s="19" t="n">
-        <v>28.77341233333333</v>
+        <v>28.777717994709</v>
       </c>
       <c r="AG154" s="19" t="n">
-        <v>-60571.22937668001</v>
+        <v>-60570.41560668001</v>
       </c>
       <c r="AH154" s="19" t="n">
-        <v>-3.563013492745883</v>
+        <v>-3.562965623922354</v>
       </c>
       <c r="AI154" s="19" t="n">
-        <v>-320.4826951147091</v>
+        <v>-320.4783894533334</v>
       </c>
     </row>
     <row r="155">
@@ -25613,22 +25613,22 @@
         <v>7.747388987724859</v>
       </c>
       <c r="AD155" s="7" t="n">
-        <v>6902.431449679998</v>
+        <v>6903.245219679999</v>
       </c>
       <c r="AE155" s="7" t="n">
-        <v>0.406025379392941</v>
+        <v>0.4060732482164705</v>
       </c>
       <c r="AF155" s="7" t="n">
-        <v>36.52080132105819</v>
+        <v>36.52510698243385</v>
       </c>
       <c r="AG155" s="7" t="n">
-        <v>6902.431449679998</v>
+        <v>6903.245219679999</v>
       </c>
       <c r="AH155" s="7" t="n">
-        <v>0.406025379392941</v>
+        <v>0.4060732482164705</v>
       </c>
       <c r="AI155" s="7" t="n">
-        <v>36.52080132105819</v>
+        <v>36.52510698243385</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard 09/16/26 21:18
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 15 Sep 2026 16:58</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 16 Sep 2026 21:18</t>
         </is>
       </c>
     </row>
@@ -805,14 +805,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 15 Sep 2026</t>
+          <t>MTD as of 16 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 15 Sep 2026</t>
+          <t>YTD as of 16 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
@@ -1220,22 +1220,22 @@
         <v>914323824.5555556</v>
       </c>
       <c r="AD7" s="11" t="n">
-        <v>9914560879</v>
+        <v>9958920879</v>
       </c>
       <c r="AE7" s="11" t="n">
-        <v>583209.4634705882</v>
+        <v>585818.8752352941</v>
       </c>
       <c r="AF7" s="11" t="n">
-        <v>52457994.06878307</v>
+        <v>52692703.06349207</v>
       </c>
       <c r="AG7" s="11" t="n">
-        <v>182721763720</v>
+        <v>182766123720</v>
       </c>
       <c r="AH7" s="11" t="n">
-        <v>10748339.04235294</v>
+        <v>10750948.45411765</v>
       </c>
       <c r="AI7" s="11" t="n">
-        <v>966781818.6243386</v>
+        <v>967016527.6190476</v>
       </c>
     </row>
     <row r="8">
@@ -1805,17 +1805,23 @@
       <c r="AC14" s="13" t="n">
         <v>497629.6296296297</v>
       </c>
-      <c r="AD14" s="13" t="n"/>
-      <c r="AE14" s="13" t="n"/>
-      <c r="AF14" s="13" t="n"/>
+      <c r="AD14" s="13" t="n">
+        <v>44360000</v>
+      </c>
+      <c r="AE14" s="13" t="n">
+        <v>2609.411764705882</v>
+      </c>
+      <c r="AF14" s="13" t="n">
+        <v>234708.9947089947</v>
+      </c>
       <c r="AG14" s="13" t="n">
-        <v>94052000</v>
+        <v>138412000</v>
       </c>
       <c r="AH14" s="13" t="n">
-        <v>5532.470588235294</v>
+        <v>8141.882352941177</v>
       </c>
       <c r="AI14" s="13" t="n">
-        <v>497629.6296296297</v>
+        <v>732338.6243386243</v>
       </c>
     </row>
     <row r="15">
@@ -2196,22 +2202,22 @@
         <v>2321849.073439153</v>
       </c>
       <c r="AD20" s="13" t="n">
-        <v>17331270</v>
+        <v>18216770</v>
       </c>
       <c r="AE20" s="13" t="n">
-        <v>1019.486470588235</v>
+        <v>1071.574705882353</v>
       </c>
       <c r="AF20" s="13" t="n">
-        <v>91699.84126984127</v>
+        <v>96385.02645502645</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>456160744.88</v>
+        <v>457046244.88</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>26832.98499294118</v>
+        <v>26885.0732282353</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>2413548.914708995</v>
+        <v>2418234.09989418</v>
       </c>
     </row>
     <row r="21">
@@ -2448,22 +2454,22 @@
         <v>332547.6190476191</v>
       </c>
       <c r="AD23" s="11" t="n">
-        <v>16838500</v>
+        <v>17724000</v>
       </c>
       <c r="AE23" s="11" t="n">
-        <v>990.5</v>
+        <v>1042.588235294118</v>
       </c>
       <c r="AF23" s="11" t="n">
-        <v>89092.5925925926</v>
+        <v>93777.77777777778</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>79690000</v>
+        <v>80575500</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>4687.647058823529</v>
+        <v>4739.735294117647</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>421640.2116402116</v>
+        <v>426325.3968253968</v>
       </c>
     </row>
     <row r="24">
@@ -3840,22 +3846,22 @@
         <v>1180222393.205714</v>
       </c>
       <c r="AD44" s="15" t="n">
-        <v>9931892149</v>
+        <v>9977137649</v>
       </c>
       <c r="AE44" s="15" t="n">
-        <v>584228.9499411765</v>
+        <v>586890.4499411765</v>
       </c>
       <c r="AF44" s="15" t="n">
-        <v>52549693.91005291</v>
+        <v>52789088.08994709</v>
       </c>
       <c r="AG44" s="15" t="n">
-        <v>232993924464.88</v>
+        <v>233039169964.88</v>
       </c>
       <c r="AH44" s="15" t="n">
-        <v>13705524.96852235</v>
+        <v>13708186.46852235</v>
       </c>
       <c r="AI44" s="15" t="n">
-        <v>1232772087.115767</v>
+        <v>1233011481.295661</v>
       </c>
     </row>
     <row r="45">
@@ -6185,7 +6191,7 @@
     <row r="80">
       <c r="B80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">        CNG</t>
+          <t xml:space="preserve">        CNG/Candlenut/Firewoods</t>
         </is>
       </c>
       <c r="C80" s="11" t="n">
@@ -6270,22 +6276,22 @@
         <v>-35112264.4074074</v>
       </c>
       <c r="AD80" s="11" t="n">
-        <v>-1088054516</v>
+        <v>-1120554516</v>
       </c>
       <c r="AE80" s="11" t="n">
-        <v>-64003.20682352941</v>
+        <v>-65914.97152941176</v>
       </c>
       <c r="AF80" s="11" t="n">
-        <v>-5756902.201058201</v>
+        <v>-5928859.873015873</v>
       </c>
       <c r="AG80" s="11" t="n">
-        <v>-7724272489</v>
+        <v>-7756772489</v>
       </c>
       <c r="AH80" s="11" t="n">
-        <v>-454368.9699411764</v>
+        <v>-456280.7346470588</v>
       </c>
       <c r="AI80" s="11" t="n">
-        <v>-40869166.6084656</v>
+        <v>-41041124.28042328</v>
       </c>
     </row>
     <row r="81">
@@ -6688,22 +6694,22 @@
         <v>-126334224.2039154</v>
       </c>
       <c r="AD84" s="15" t="n">
-        <v>-2428450805</v>
+        <v>-2460950805</v>
       </c>
       <c r="AE84" s="15" t="n">
-        <v>-142850.0473529412</v>
+        <v>-144761.8120588235</v>
       </c>
       <c r="AF84" s="15" t="n">
-        <v>-12848946.05820106</v>
+        <v>-13020903.73015873</v>
       </c>
       <c r="AG84" s="15" t="n">
-        <v>-26305619179.54</v>
+        <v>-26338119179.54</v>
       </c>
       <c r="AH84" s="15" t="n">
-        <v>-1547389.363502353</v>
+        <v>-1549301.128208235</v>
       </c>
       <c r="AI84" s="15" t="n">
-        <v>-139183170.2621164</v>
+        <v>-139355127.9340741</v>
       </c>
     </row>
     <row r="85">
@@ -11970,22 +11976,22 @@
         <v>-99449.19407407405</v>
       </c>
       <c r="AD146" s="11" t="n">
-        <v>-49500</v>
+        <v>-52000</v>
       </c>
       <c r="AE146" s="11" t="n">
-        <v>-2.911764705882353</v>
+        <v>-3.058823529411764</v>
       </c>
       <c r="AF146" s="11" t="n">
-        <v>-261.9047619047619</v>
+        <v>-275.1322751322751</v>
       </c>
       <c r="AG146" s="11" t="n">
-        <v>-18845397.68</v>
+        <v>-18847897.68</v>
       </c>
       <c r="AH146" s="11" t="n">
-        <v>-1108.552804705882</v>
+        <v>-1108.699863529412</v>
       </c>
       <c r="AI146" s="11" t="n">
-        <v>-99711.09883597882</v>
+        <v>-99724.32634920633</v>
       </c>
     </row>
     <row r="147">
@@ -12468,22 +12474,22 @@
         <v>-31583868.07253968</v>
       </c>
       <c r="AD152" s="15" t="n">
-        <v>-182571642</v>
+        <v>-182574142</v>
       </c>
       <c r="AE152" s="15" t="n">
-        <v>-10739.50835294118</v>
+        <v>-10739.65541176471</v>
       </c>
       <c r="AF152" s="15" t="n">
-        <v>-965987.5238095238</v>
+        <v>-966000.7513227513</v>
       </c>
       <c r="AG152" s="15" t="n">
-        <v>-6151922707.710001</v>
+        <v>-6151925207.710001</v>
       </c>
       <c r="AH152" s="15" t="n">
-        <v>-361877.8063358823</v>
+        <v>-361877.9533947058</v>
       </c>
       <c r="AI152" s="15" t="n">
-        <v>-32549855.59634921</v>
+        <v>-32549868.82386243</v>
       </c>
     </row>
     <row r="153">
@@ -12574,22 +12580,22 @@
         <v>-1529478500.653757</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-4492903448</v>
+        <v>-4525405948</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-264288.4381176471</v>
+        <v>-266200.3498823529</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-23771975.91534391</v>
+        <v>-23943946.81481481</v>
       </c>
       <c r="AG153" s="19" t="n">
-        <v>-293564340071.5599</v>
+        <v>-293596842571.5599</v>
       </c>
       <c r="AH153" s="19" t="n">
-        <v>-17268490.5924447</v>
+        <v>-17270402.50420941</v>
       </c>
       <c r="AI153" s="19" t="n">
-        <v>-1553250476.569101</v>
+        <v>-1553422447.468571</v>
       </c>
     </row>
     <row r="154">
@@ -12680,22 +12686,22 @@
         <v>-349256107.4480425</v>
       </c>
       <c r="AD154" s="19" t="n">
-        <v>5438988701</v>
+        <v>5451731701</v>
       </c>
       <c r="AE154" s="19" t="n">
-        <v>319940.5118235294</v>
+        <v>320690.1000588235</v>
       </c>
       <c r="AF154" s="19" t="n">
-        <v>28777717.994709</v>
+        <v>28845141.27513228</v>
       </c>
       <c r="AG154" s="19" t="n">
-        <v>-60570415606.68</v>
+        <v>-60557672606.68</v>
       </c>
       <c r="AH154" s="19" t="n">
-        <v>-3562965.623922354</v>
+        <v>-3562216.03568706</v>
       </c>
       <c r="AI154" s="19" t="n">
-        <v>-320478389.4533334</v>
+        <v>-320410966.1729102</v>
       </c>
     </row>
     <row r="155">
@@ -12786,22 +12792,22 @@
         <v>7747388.987724859</v>
       </c>
       <c r="AD155" s="7" t="n">
-        <v>6903245219.679998</v>
+        <v>6915988219.679998</v>
       </c>
       <c r="AE155" s="7" t="n">
-        <v>406073.2482164705</v>
+        <v>406822.8364517646</v>
       </c>
       <c r="AF155" s="7" t="n">
-        <v>36525106.98243386</v>
+        <v>36592530.26285713</v>
       </c>
       <c r="AG155" s="7" t="n">
-        <v>6903245219.679998</v>
+        <v>6915988219.679998</v>
       </c>
       <c r="AH155" s="7" t="n">
-        <v>406073.2482164705</v>
+        <v>406822.8364517646</v>
       </c>
       <c r="AI155" s="7" t="n">
-        <v>36525106.98243386</v>
+        <v>36592530.26285713</v>
       </c>
     </row>
   </sheetData>
@@ -13362,16 +13368,16 @@
         <v>172976399.24</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>-68218246</v>
+        <v>-99835246</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>104758153.24</v>
+        <v>73141153.24000001</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>6162.244308235295</v>
+        <v>4302.42077882353</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>554275.9430687831</v>
+        <v>386990.2287830688</v>
       </c>
     </row>
     <row r="10">
@@ -13426,16 +13432,16 @@
         <v>112155332.96</v>
       </c>
       <c r="E11" s="13" t="n">
-        <v>0</v>
+        <v>44360000</v>
       </c>
       <c r="F11" s="13" t="n">
-        <v>112155332.96</v>
+        <v>156515332.96</v>
       </c>
       <c r="G11" s="24" t="n">
-        <v>6597.372527058823</v>
+        <v>9206.784291764705</v>
       </c>
       <c r="H11" s="24" t="n">
-        <v>593414.4601058201</v>
+        <v>828123.4548148147</v>
       </c>
     </row>
     <row r="12">
@@ -13481,13 +13487,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>6903245221.679999</v>
+        <v>6915988221.679999</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>406073.2483341176</v>
+        <v>406822.8365694117</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>36525106.99301587</v>
+        <v>36592530.27343915</v>
       </c>
     </row>
   </sheetData>
@@ -13557,7 +13563,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 15 Sep 2026 16:58 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 16 Sep 2026 21:18 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -13632,14 +13638,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 15 Sep 2026</t>
+          <t>MTD as of 16 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 15 Sep 2026</t>
+          <t>YTD as of 16 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
@@ -14047,22 +14053,22 @@
         <v>914.3238245555556</v>
       </c>
       <c r="AD7" s="11" t="n">
-        <v>9914.560879000001</v>
+        <v>9958.920878999999</v>
       </c>
       <c r="AE7" s="11" t="n">
-        <v>0.5832094634705882</v>
+        <v>0.5858188752352941</v>
       </c>
       <c r="AF7" s="11" t="n">
-        <v>52.45799406878307</v>
+        <v>52.69270306349206</v>
       </c>
       <c r="AG7" s="11" t="n">
-        <v>182721.76372</v>
+        <v>182766.12372</v>
       </c>
       <c r="AH7" s="11" t="n">
-        <v>10.74833904235294</v>
+        <v>10.75094845411765</v>
       </c>
       <c r="AI7" s="11" t="n">
-        <v>966.7818186243386</v>
+        <v>967.0165276190477</v>
       </c>
     </row>
     <row r="8">
@@ -14632,17 +14638,23 @@
       <c r="AC14" s="13" t="n">
         <v>0.4976296296296296</v>
       </c>
-      <c r="AD14" s="13" t="n"/>
-      <c r="AE14" s="13" t="n"/>
-      <c r="AF14" s="13" t="n"/>
+      <c r="AD14" s="13" t="n">
+        <v>44.36</v>
+      </c>
+      <c r="AE14" s="13" t="n">
+        <v>0.002609411764705882</v>
+      </c>
+      <c r="AF14" s="13" t="n">
+        <v>0.2347089947089947</v>
+      </c>
       <c r="AG14" s="13" t="n">
-        <v>94.05200000000001</v>
+        <v>138.412</v>
       </c>
       <c r="AH14" s="13" t="n">
-        <v>0.005532470588235295</v>
+        <v>0.008141882352941178</v>
       </c>
       <c r="AI14" s="13" t="n">
-        <v>0.4976296296296296</v>
+        <v>0.7323386243386243</v>
       </c>
     </row>
     <row r="15">
@@ -15023,22 +15035,22 @@
         <v>2.321849073439154</v>
       </c>
       <c r="AD20" s="13" t="n">
-        <v>17.33127</v>
+        <v>18.21677</v>
       </c>
       <c r="AE20" s="13" t="n">
-        <v>0.001019486470588235</v>
+        <v>0.001071574705882353</v>
       </c>
       <c r="AF20" s="13" t="n">
-        <v>0.09169984126984126</v>
+        <v>0.09638502645502646</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>456.16074488</v>
+        <v>457.04624488</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>0.02683298499294118</v>
+        <v>0.02688507322823529</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>2.413548914708995</v>
+        <v>2.41823409989418</v>
       </c>
     </row>
     <row r="21">
@@ -15275,22 +15287,22 @@
         <v>0.332547619047619</v>
       </c>
       <c r="AD23" s="11" t="n">
-        <v>16.8385</v>
+        <v>17.724</v>
       </c>
       <c r="AE23" s="11" t="n">
-        <v>0.0009905000000000001</v>
+        <v>0.001042588235294118</v>
       </c>
       <c r="AF23" s="11" t="n">
-        <v>0.0890925925925926</v>
+        <v>0.09377777777777778</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>79.69</v>
+        <v>80.57550000000001</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>0.00468764705882353</v>
+        <v>0.004739735294117647</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>0.4216402116402116</v>
+        <v>0.4263253968253968</v>
       </c>
     </row>
     <row r="24">
@@ -16667,22 +16679,22 @@
         <v>1180.222393205714</v>
       </c>
       <c r="AD44" s="15" t="n">
-        <v>9931.892148999999</v>
+        <v>9977.137649</v>
       </c>
       <c r="AE44" s="15" t="n">
-        <v>0.5842289499411765</v>
+        <v>0.5868904499411765</v>
       </c>
       <c r="AF44" s="15" t="n">
-        <v>52.54969391005291</v>
+        <v>52.78908808994709</v>
       </c>
       <c r="AG44" s="15" t="n">
-        <v>232993.92446488</v>
+        <v>233039.16996488</v>
       </c>
       <c r="AH44" s="15" t="n">
-        <v>13.70552496852235</v>
+        <v>13.70818646852235</v>
       </c>
       <c r="AI44" s="15" t="n">
-        <v>1232.772087115767</v>
+        <v>1233.011481295661</v>
       </c>
     </row>
     <row r="45">
@@ -19012,7 +19024,7 @@
     <row r="80">
       <c r="B80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">        CNG</t>
+          <t xml:space="preserve">        CNG/Candlenut/Firewoods</t>
         </is>
       </c>
       <c r="C80" s="11" t="n">
@@ -19097,22 +19109,22 @@
         <v>-35.11226440740741</v>
       </c>
       <c r="AD80" s="11" t="n">
-        <v>-1088.054516</v>
+        <v>-1120.554516</v>
       </c>
       <c r="AE80" s="11" t="n">
-        <v>-0.0640032068235294</v>
+        <v>-0.06591497152941175</v>
       </c>
       <c r="AF80" s="11" t="n">
-        <v>-5.7569022010582</v>
+        <v>-5.928859873015873</v>
       </c>
       <c r="AG80" s="11" t="n">
-        <v>-7724.272489000001</v>
+        <v>-7756.772489000001</v>
       </c>
       <c r="AH80" s="11" t="n">
-        <v>-0.4543689699411765</v>
+        <v>-0.4562807346470589</v>
       </c>
       <c r="AI80" s="11" t="n">
-        <v>-40.86916660846561</v>
+        <v>-41.04112428042328</v>
       </c>
     </row>
     <row r="81">
@@ -19515,22 +19527,22 @@
         <v>-126.3342242039153</v>
       </c>
       <c r="AD84" s="15" t="n">
-        <v>-2428.450805</v>
+        <v>-2460.950805</v>
       </c>
       <c r="AE84" s="15" t="n">
-        <v>-0.1428500473529412</v>
+        <v>-0.1447618120588235</v>
       </c>
       <c r="AF84" s="15" t="n">
-        <v>-12.84894605820106</v>
+        <v>-13.02090373015873</v>
       </c>
       <c r="AG84" s="15" t="n">
-        <v>-26305.61917954</v>
+        <v>-26338.11917954</v>
       </c>
       <c r="AH84" s="15" t="n">
-        <v>-1.547389363502353</v>
+        <v>-1.549301128208235</v>
       </c>
       <c r="AI84" s="15" t="n">
-        <v>-139.1831702621164</v>
+        <v>-139.3551279340741</v>
       </c>
     </row>
     <row r="85">
@@ -24797,22 +24809,22 @@
         <v>-0.09944919407407407</v>
       </c>
       <c r="AD146" s="11" t="n">
-        <v>-0.0495</v>
+        <v>-0.052</v>
       </c>
       <c r="AE146" s="11" t="n">
-        <v>-2.911764705882353e-06</v>
+        <v>-3.058823529411765e-06</v>
       </c>
       <c r="AF146" s="11" t="n">
-        <v>-0.0002619047619047619</v>
+        <v>-0.0002751322751322751</v>
       </c>
       <c r="AG146" s="11" t="n">
-        <v>-18.84539768</v>
+        <v>-18.84789768</v>
       </c>
       <c r="AH146" s="11" t="n">
-        <v>-0.001108552804705883</v>
+        <v>-0.001108699863529412</v>
       </c>
       <c r="AI146" s="11" t="n">
-        <v>-0.09971109883597884</v>
+        <v>-0.09972432634920635</v>
       </c>
     </row>
     <row r="147">
@@ -25295,22 +25307,22 @@
         <v>-31.58386807253968</v>
       </c>
       <c r="AD152" s="15" t="n">
-        <v>-182.571642</v>
+        <v>-182.574142</v>
       </c>
       <c r="AE152" s="15" t="n">
-        <v>-0.01073950835294118</v>
+        <v>-0.01073965541176471</v>
       </c>
       <c r="AF152" s="15" t="n">
-        <v>-0.9659875238095238</v>
+        <v>-0.9660007513227513</v>
       </c>
       <c r="AG152" s="15" t="n">
-        <v>-6151.92270771</v>
+        <v>-6151.925207710001</v>
       </c>
       <c r="AH152" s="15" t="n">
-        <v>-0.3618778063358825</v>
+        <v>-0.361877953394706</v>
       </c>
       <c r="AI152" s="15" t="n">
-        <v>-32.5498555963492</v>
+        <v>-32.54986882386243</v>
       </c>
     </row>
     <row r="153">
@@ -25401,22 +25413,22 @@
         <v>-1529.478500653756</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-4492.903448</v>
+        <v>-4525.405948</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-0.2642884381176471</v>
+        <v>-0.2662003498823529</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-23.77197591534392</v>
+        <v>-23.94394681481481</v>
       </c>
       <c r="AG153" s="19" t="n">
-        <v>-293564.3400715599</v>
+        <v>-293596.8425715599</v>
       </c>
       <c r="AH153" s="19" t="n">
-        <v>-17.26849059244471</v>
+        <v>-17.27040250420941</v>
       </c>
       <c r="AI153" s="19" t="n">
-        <v>-1553.2504765691</v>
+        <v>-1553.422447468571</v>
       </c>
     </row>
     <row r="154">
@@ -25507,22 +25519,22 @@
         <v>-349.2561074480424</v>
       </c>
       <c r="AD154" s="19" t="n">
-        <v>5438.988701</v>
+        <v>5451.731701</v>
       </c>
       <c r="AE154" s="19" t="n">
-        <v>0.3199405118235294</v>
+        <v>0.3206901000588235</v>
       </c>
       <c r="AF154" s="19" t="n">
-        <v>28.777717994709</v>
+        <v>28.84514127513227</v>
       </c>
       <c r="AG154" s="19" t="n">
-        <v>-60570.41560668001</v>
+        <v>-60557.67260668002</v>
       </c>
       <c r="AH154" s="19" t="n">
-        <v>-3.562965623922354</v>
+        <v>-3.56221603568706</v>
       </c>
       <c r="AI154" s="19" t="n">
-        <v>-320.4783894533334</v>
+        <v>-320.4109661729102</v>
       </c>
     </row>
     <row r="155">
@@ -25613,22 +25625,22 @@
         <v>7.747388987724859</v>
       </c>
       <c r="AD155" s="7" t="n">
-        <v>6903.245219679999</v>
+        <v>6915.988219679998</v>
       </c>
       <c r="AE155" s="7" t="n">
-        <v>0.4060732482164705</v>
+        <v>0.4068228364517646</v>
       </c>
       <c r="AF155" s="7" t="n">
-        <v>36.52510698243385</v>
+        <v>36.59253026285713</v>
       </c>
       <c r="AG155" s="7" t="n">
-        <v>6903.245219679999</v>
+        <v>6915.988219679998</v>
       </c>
       <c r="AH155" s="7" t="n">
-        <v>0.4060732482164705</v>
+        <v>0.4068228364517646</v>
       </c>
       <c r="AI155" s="7" t="n">
-        <v>36.52510698243385</v>
+        <v>36.59253026285713</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Wed 09/23/2026 16:10
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 22 Sep 2026 11:06</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 23 Sep 2026 16:10</t>
         </is>
       </c>
     </row>
@@ -805,14 +805,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 22 Sep 2026</t>
+          <t>MTD as of 23 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 22 Sep 2026</t>
+          <t>YTD as of 23 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
@@ -2260,22 +2260,22 @@
         <v>2321849.073439153</v>
       </c>
       <c r="AD21" s="11" t="n">
-        <v>26050170</v>
+        <v>29728211</v>
       </c>
       <c r="AE21" s="11" t="n">
-        <v>1532.36294117647</v>
+        <v>1748.718294117647</v>
       </c>
       <c r="AF21" s="11" t="n">
-        <v>137831.5873015873</v>
+        <v>157292.1216931217</v>
       </c>
       <c r="AG21" s="11" t="n">
-        <v>464879644.88</v>
+        <v>468557685.88</v>
       </c>
       <c r="AH21" s="11" t="n">
-        <v>27345.86146352941</v>
+        <v>27562.21681647059</v>
       </c>
       <c r="AI21" s="11" t="n">
-        <v>2459680.660740741</v>
+        <v>2479141.195132275</v>
       </c>
     </row>
     <row r="22">
@@ -2512,22 +2512,22 @@
         <v>332547.6190476191</v>
       </c>
       <c r="AD24" s="13" t="n">
-        <v>21422500</v>
+        <v>24569000</v>
       </c>
       <c r="AE24" s="13" t="n">
-        <v>1260.14705882353</v>
+        <v>1445.235294117647</v>
       </c>
       <c r="AF24" s="13" t="n">
-        <v>113346.5608465609</v>
+        <v>129994.708994709</v>
       </c>
       <c r="AG24" s="13" t="n">
-        <v>84274000</v>
+        <v>87420500</v>
       </c>
       <c r="AH24" s="13" t="n">
-        <v>4957.294117647059</v>
+        <v>5142.382352941176</v>
       </c>
       <c r="AI24" s="13" t="n">
-        <v>445894.1798941799</v>
+        <v>462542.3280423281</v>
       </c>
     </row>
     <row r="25">
@@ -3295,153 +3295,159 @@
     <row r="37">
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Foreign Fluctuation Gain Or Loss</t>
+          <t xml:space="preserve">        PT. Asuransi Allianz Utama Indonesia</t>
         </is>
       </c>
       <c r="C37" s="11" t="n"/>
       <c r="D37" s="11" t="n"/>
       <c r="E37" s="11" t="n"/>
       <c r="F37" s="11" t="n">
-        <v>605432.6800000001</v>
+        <v>283992</v>
       </c>
       <c r="G37" s="11" t="n">
-        <v>35.61368705882353</v>
+        <v>16.70541176470588</v>
       </c>
       <c r="H37" s="11" t="n">
-        <v>3203.347513227513</v>
-      </c>
-      <c r="I37" s="11" t="n">
-        <v>19977.84</v>
-      </c>
-      <c r="J37" s="11" t="n">
-        <v>1.175167058823529</v>
-      </c>
-      <c r="K37" s="11" t="n">
-        <v>105.7028571428571</v>
-      </c>
-      <c r="L37" s="11" t="n">
-        <v>391627.25</v>
-      </c>
-      <c r="M37" s="11" t="n">
-        <v>23.03689705882353</v>
-      </c>
-      <c r="N37" s="11" t="n">
-        <v>2072.101851851852</v>
-      </c>
-      <c r="O37" s="11" t="n">
-        <v>756578.6799999999</v>
-      </c>
-      <c r="P37" s="11" t="n">
-        <v>44.50462823529411</v>
-      </c>
-      <c r="Q37" s="11" t="n">
-        <v>4003.061798941799</v>
-      </c>
-      <c r="R37" s="11" t="n">
-        <v>55799.61</v>
-      </c>
-      <c r="S37" s="11" t="n">
-        <v>3.28233</v>
-      </c>
-      <c r="T37" s="11" t="n">
-        <v>295.2360317460318</v>
-      </c>
-      <c r="U37" s="11" t="n"/>
-      <c r="V37" s="11" t="n"/>
-      <c r="W37" s="11" t="n"/>
-      <c r="X37" s="11" t="n">
-        <v>291720</v>
-      </c>
-      <c r="Y37" s="11" t="n">
-        <v>17.16</v>
-      </c>
-      <c r="Z37" s="11" t="n">
-        <v>1543.492063492063</v>
-      </c>
+        <v>1502.603174603175</v>
+      </c>
+      <c r="I37" s="11" t="n"/>
+      <c r="J37" s="11" t="n"/>
+      <c r="K37" s="11" t="n"/>
+      <c r="L37" s="11" t="n"/>
+      <c r="M37" s="11" t="n"/>
+      <c r="N37" s="11" t="n"/>
+      <c r="O37" s="11" t="n"/>
+      <c r="P37" s="11" t="n"/>
+      <c r="Q37" s="11" t="n"/>
+      <c r="R37" s="11" t="n"/>
+      <c r="S37" s="11" t="n"/>
+      <c r="T37" s="11" t="n"/>
+      <c r="U37" s="11" t="n">
+        <v>1360300</v>
+      </c>
+      <c r="V37" s="11" t="n">
+        <v>80.01764705882353</v>
+      </c>
+      <c r="W37" s="11" t="n">
+        <v>7197.354497354498</v>
+      </c>
+      <c r="X37" s="11" t="n"/>
+      <c r="Y37" s="11" t="n"/>
+      <c r="Z37" s="11" t="n"/>
       <c r="AA37" s="11" t="n">
-        <v>2121136.06</v>
+        <v>1644292</v>
       </c>
       <c r="AB37" s="11" t="n">
-        <v>124.7727094117647</v>
+        <v>96.72305882352941</v>
       </c>
       <c r="AC37" s="11" t="n">
-        <v>11222.94211640212</v>
-      </c>
-      <c r="AD37" s="11" t="n"/>
-      <c r="AE37" s="11" t="n"/>
-      <c r="AF37" s="11" t="n"/>
+        <v>8699.957671957673</v>
+      </c>
+      <c r="AD37" s="11" t="n">
+        <v>531541</v>
+      </c>
+      <c r="AE37" s="11" t="n">
+        <v>31.26711764705883</v>
+      </c>
+      <c r="AF37" s="11" t="n">
+        <v>2812.386243386243</v>
+      </c>
       <c r="AG37" s="11" t="n">
-        <v>2121136.06</v>
+        <v>2175833</v>
       </c>
       <c r="AH37" s="11" t="n">
-        <v>124.7727094117647</v>
+        <v>127.9901764705882</v>
       </c>
       <c r="AI37" s="11" t="n">
-        <v>11222.94211640212</v>
+        <v>11512.34391534392</v>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">        PT. Asuransi Allianz Utama Indonesia</t>
+          <t xml:space="preserve">        Foreign Fluctuation Gain Or Loss</t>
         </is>
       </c>
       <c r="C38" s="13" t="n"/>
       <c r="D38" s="13" t="n"/>
       <c r="E38" s="13" t="n"/>
       <c r="F38" s="13" t="n">
-        <v>283992</v>
+        <v>605432.6800000001</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>16.70541176470588</v>
+        <v>35.61368705882353</v>
       </c>
       <c r="H38" s="13" t="n">
-        <v>1502.603174603175</v>
-      </c>
-      <c r="I38" s="13" t="n"/>
-      <c r="J38" s="13" t="n"/>
-      <c r="K38" s="13" t="n"/>
-      <c r="L38" s="13" t="n"/>
-      <c r="M38" s="13" t="n"/>
-      <c r="N38" s="13" t="n"/>
-      <c r="O38" s="13" t="n"/>
-      <c r="P38" s="13" t="n"/>
-      <c r="Q38" s="13" t="n"/>
-      <c r="R38" s="13" t="n"/>
-      <c r="S38" s="13" t="n"/>
-      <c r="T38" s="13" t="n"/>
-      <c r="U38" s="13" t="n">
-        <v>1360300</v>
-      </c>
-      <c r="V38" s="13" t="n">
-        <v>80.01764705882353</v>
-      </c>
-      <c r="W38" s="13" t="n">
-        <v>7197.354497354498</v>
-      </c>
-      <c r="X38" s="13" t="n"/>
-      <c r="Y38" s="13" t="n"/>
-      <c r="Z38" s="13" t="n"/>
+        <v>3203.347513227513</v>
+      </c>
+      <c r="I38" s="13" t="n">
+        <v>19977.84</v>
+      </c>
+      <c r="J38" s="13" t="n">
+        <v>1.175167058823529</v>
+      </c>
+      <c r="K38" s="13" t="n">
+        <v>105.7028571428571</v>
+      </c>
+      <c r="L38" s="13" t="n">
+        <v>391627.25</v>
+      </c>
+      <c r="M38" s="13" t="n">
+        <v>23.03689705882353</v>
+      </c>
+      <c r="N38" s="13" t="n">
+        <v>2072.101851851852</v>
+      </c>
+      <c r="O38" s="13" t="n">
+        <v>756578.6799999999</v>
+      </c>
+      <c r="P38" s="13" t="n">
+        <v>44.50462823529411</v>
+      </c>
+      <c r="Q38" s="13" t="n">
+        <v>4003.061798941799</v>
+      </c>
+      <c r="R38" s="13" t="n">
+        <v>55799.61</v>
+      </c>
+      <c r="S38" s="13" t="n">
+        <v>3.28233</v>
+      </c>
+      <c r="T38" s="13" t="n">
+        <v>295.2360317460318</v>
+      </c>
+      <c r="U38" s="13" t="n"/>
+      <c r="V38" s="13" t="n"/>
+      <c r="W38" s="13" t="n"/>
+      <c r="X38" s="13" t="n">
+        <v>291720</v>
+      </c>
+      <c r="Y38" s="13" t="n">
+        <v>17.16</v>
+      </c>
+      <c r="Z38" s="13" t="n">
+        <v>1543.492063492063</v>
+      </c>
       <c r="AA38" s="13" t="n">
-        <v>1644292</v>
+        <v>2121136.06</v>
       </c>
       <c r="AB38" s="13" t="n">
-        <v>96.72305882352941</v>
+        <v>124.7727094117647</v>
       </c>
       <c r="AC38" s="13" t="n">
-        <v>8699.957671957673</v>
+        <v>11222.94211640212</v>
       </c>
       <c r="AD38" s="13" t="n"/>
       <c r="AE38" s="13" t="n"/>
       <c r="AF38" s="13" t="n"/>
       <c r="AG38" s="13" t="n">
-        <v>1644292</v>
+        <v>2121136.06</v>
       </c>
       <c r="AH38" s="13" t="n">
-        <v>96.72305882352941</v>
+        <v>124.7727094117647</v>
       </c>
       <c r="AI38" s="13" t="n">
-        <v>8699.957671957673</v>
+        <v>11222.94211640212</v>
       </c>
     </row>
     <row r="39">
@@ -3962,22 +3968,22 @@
         <v>1180222393.205714</v>
       </c>
       <c r="AD46" s="15" t="n">
-        <v>15729020815</v>
+        <v>15732698856</v>
       </c>
       <c r="AE46" s="15" t="n">
-        <v>925236.5185294118</v>
+        <v>925452.873882353</v>
       </c>
       <c r="AF46" s="15" t="n">
-        <v>83222332.35449736</v>
+        <v>83241792.8888889</v>
       </c>
       <c r="AG46" s="15" t="n">
-        <v>238791053130.88</v>
+        <v>238794731171.88</v>
       </c>
       <c r="AH46" s="15" t="n">
-        <v>14046532.53711059</v>
+        <v>14046748.89246353</v>
       </c>
       <c r="AI46" s="15" t="n">
-        <v>1263444725.560212</v>
+        <v>1263464186.094603</v>
       </c>
     </row>
     <row r="47">
@@ -10414,22 +10420,22 @@
         <v>-5069808.166825396</v>
       </c>
       <c r="AD129" s="13" t="n">
-        <v>-123675500</v>
+        <v>-166617666</v>
       </c>
       <c r="AE129" s="13" t="n">
-        <v>-7275.029411764706</v>
+        <v>-9801.039176470587</v>
       </c>
       <c r="AF129" s="13" t="n">
-        <v>-654367.7248677248</v>
+        <v>-881574.9523809524</v>
       </c>
       <c r="AG129" s="13" t="n">
-        <v>-1081869243.53</v>
+        <v>-1124811409.53</v>
       </c>
       <c r="AH129" s="13" t="n">
-        <v>-63639.3672664706</v>
+        <v>-66165.37703117648</v>
       </c>
       <c r="AI129" s="13" t="n">
-        <v>-5724175.891693121</v>
+        <v>-5951383.119206348</v>
       </c>
     </row>
     <row r="130">
@@ -10826,22 +10832,22 @@
         <v>-132568430.7276719</v>
       </c>
       <c r="AD133" s="15" t="n">
-        <v>-226301416</v>
+        <v>-269243582</v>
       </c>
       <c r="AE133" s="15" t="n">
-        <v>-13311.848</v>
+        <v>-15837.85776470588</v>
       </c>
       <c r="AF133" s="15" t="n">
-        <v>-1197361.98941799</v>
+        <v>-1424569.216931217</v>
       </c>
       <c r="AG133" s="15" t="n">
-        <v>-25281734823.53</v>
+        <v>-25324676989.53</v>
       </c>
       <c r="AH133" s="15" t="n">
-        <v>-1487160.871972353</v>
+        <v>-1489686.881737059</v>
       </c>
       <c r="AI133" s="15" t="n">
-        <v>-133765792.7170899</v>
+        <v>-133992999.9446032</v>
       </c>
     </row>
     <row r="134">
@@ -11630,22 +11636,22 @@
         <v>-230275933.0393122</v>
       </c>
       <c r="AD142" s="15" t="n">
-        <v>-1169198561</v>
+        <v>-1212140727</v>
       </c>
       <c r="AE142" s="15" t="n">
-        <v>-68776.38594117647</v>
+        <v>-71302.39570588236</v>
       </c>
       <c r="AF142" s="15" t="n">
-        <v>-6186235.772486772</v>
+        <v>-6413443</v>
       </c>
       <c r="AG142" s="15" t="n">
-        <v>-44691349905.43001</v>
+        <v>-44734292071.43001</v>
       </c>
       <c r="AH142" s="15" t="n">
-        <v>-2628902.93561353</v>
+        <v>-2631428.945378236</v>
       </c>
       <c r="AI142" s="15" t="n">
-        <v>-236462168.8117989</v>
+        <v>-236689376.0393122</v>
       </c>
     </row>
     <row r="143">
@@ -12226,22 +12232,22 @@
         <v>-99449.19407407405</v>
       </c>
       <c r="AD150" s="11" t="n">
-        <v>-222500</v>
+        <v>-1250800</v>
       </c>
       <c r="AE150" s="11" t="n">
-        <v>-13.08823529411765</v>
+        <v>-73.5764705882353</v>
       </c>
       <c r="AF150" s="11" t="n">
-        <v>-1177.248677248677</v>
+        <v>-6617.989417989418</v>
       </c>
       <c r="AG150" s="11" t="n">
-        <v>-19018397.68</v>
+        <v>-20046697.68</v>
       </c>
       <c r="AH150" s="11" t="n">
-        <v>-1118.729275294118</v>
+        <v>-1179.217510588235</v>
       </c>
       <c r="AI150" s="11" t="n">
-        <v>-100626.4427513227</v>
+        <v>-106067.1834920635</v>
       </c>
     </row>
     <row r="151">
@@ -12724,22 +12730,22 @@
         <v>-31583868.07253968</v>
       </c>
       <c r="AD156" s="15" t="n">
-        <v>-182744642</v>
+        <v>-183772942</v>
       </c>
       <c r="AE156" s="15" t="n">
-        <v>-10749.68482352941</v>
+        <v>-10810.17305882353</v>
       </c>
       <c r="AF156" s="15" t="n">
-        <v>-966902.8677248678</v>
+        <v>-972343.6084656084</v>
       </c>
       <c r="AG156" s="15" t="n">
-        <v>-6152095707.710001</v>
+        <v>-6153124007.710001</v>
       </c>
       <c r="AH156" s="15" t="n">
-        <v>-361887.9828064705</v>
+        <v>-361948.4710417647</v>
       </c>
       <c r="AI156" s="15" t="n">
-        <v>-32550770.94026455</v>
+        <v>-32556211.68100529</v>
       </c>
     </row>
     <row r="157">
@@ -12830,22 +12836,22 @@
         <v>-1529478500.653757</v>
       </c>
       <c r="AD157" s="19" t="n">
-        <v>-9475645340</v>
+        <v>-9519615806</v>
       </c>
       <c r="AE157" s="19" t="n">
-        <v>-557390.9023529412</v>
+        <v>-559977.4003529411</v>
       </c>
       <c r="AF157" s="19" t="n">
-        <v>-50135689.62962963</v>
+        <v>-50368337.5978836</v>
       </c>
       <c r="AG157" s="19" t="n">
-        <v>-298547081963.5599</v>
+        <v>-298591052429.5599</v>
       </c>
       <c r="AH157" s="19" t="n">
-        <v>-17561593.05668</v>
+        <v>-17564179.55468</v>
       </c>
       <c r="AI157" s="19" t="n">
-        <v>-1579614190.283386</v>
+        <v>-1579846838.25164</v>
       </c>
     </row>
     <row r="158">
@@ -12936,22 +12942,22 @@
         <v>-349256107.4480425</v>
       </c>
       <c r="AD158" s="19" t="n">
-        <v>6253375475</v>
+        <v>6213083050</v>
       </c>
       <c r="AE158" s="19" t="n">
-        <v>367845.6161764706</v>
+        <v>365475.4735294118</v>
       </c>
       <c r="AF158" s="19" t="n">
-        <v>33086642.72486772</v>
+        <v>32873455.29100529</v>
       </c>
       <c r="AG158" s="19" t="n">
-        <v>-59756028832.68</v>
+        <v>-59796321257.68</v>
       </c>
       <c r="AH158" s="19" t="n">
-        <v>-3515060.519569412</v>
+        <v>-3517430.662216471</v>
       </c>
       <c r="AI158" s="19" t="n">
-        <v>-316169464.7231748</v>
+        <v>-316382652.1570371</v>
       </c>
     </row>
     <row r="159">
@@ -13042,22 +13048,22 @@
         <v>7747388.987724859</v>
       </c>
       <c r="AD159" s="7" t="n">
-        <v>7717631993.68</v>
+        <v>7677339568.68</v>
       </c>
       <c r="AE159" s="7" t="n">
-        <v>453978.3525694118</v>
+        <v>451608.209922353</v>
       </c>
       <c r="AF159" s="7" t="n">
-        <v>40834031.71259259</v>
+        <v>40620844.27873016</v>
       </c>
       <c r="AG159" s="7" t="n">
-        <v>7717631993.68</v>
+        <v>7677339568.68</v>
       </c>
       <c r="AH159" s="7" t="n">
-        <v>453978.3525694118</v>
+        <v>451608.209922353</v>
       </c>
       <c r="AI159" s="7" t="n">
-        <v>40834031.71259259</v>
+        <v>40620844.27873016</v>
       </c>
     </row>
   </sheetData>
@@ -13522,16 +13528,16 @@
         <v>1136676704</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>5220063987</v>
+        <v>5219042187</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>6356740691</v>
+        <v>6355718891</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>373925.923</v>
+        <v>373865.817117647</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>33633548.62962963</v>
+        <v>33628142.28042328</v>
       </c>
     </row>
     <row r="7">
@@ -13618,16 +13624,16 @@
         <v>172976399.24</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>957998154</v>
+        <v>918195988</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>1130974553.24</v>
+        <v>1091172387.24</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>66527.91489647058</v>
+        <v>64186.61101411765</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>5983992.345185185</v>
+        <v>5773398.874285715</v>
       </c>
     </row>
     <row r="10">
@@ -13682,16 +13688,16 @@
         <v>112155332.96</v>
       </c>
       <c r="E11" s="13" t="n">
-        <v>65083039</v>
+        <v>65614580</v>
       </c>
       <c r="F11" s="13" t="n">
-        <v>177238371.96</v>
+        <v>177769912.96</v>
       </c>
       <c r="G11" s="24" t="n">
-        <v>10425.78658588235</v>
+        <v>10457.05370352941</v>
       </c>
       <c r="H11" s="24" t="n">
-        <v>937769.1638095237</v>
+        <v>940581.55005291</v>
       </c>
     </row>
     <row r="12">
@@ -13737,13 +13743,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>7717631995.679999</v>
+        <v>7677339570.679999</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>453978.3526870588</v>
+        <v>451608.21004</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>40834031.7231746</v>
+        <v>40620844.28931217</v>
       </c>
     </row>
   </sheetData>
@@ -13813,7 +13819,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 22 Sep 2026 11:06 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 23 Sep 2026 16:10 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -13888,14 +13894,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 22 Sep 2026</t>
+          <t>MTD as of 23 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 22 Sep 2026</t>
+          <t>YTD as of 23 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
@@ -15343,22 +15349,22 @@
         <v>2.321849073439154</v>
       </c>
       <c r="AD21" s="11" t="n">
-        <v>26.05017</v>
+        <v>29.728211</v>
       </c>
       <c r="AE21" s="11" t="n">
-        <v>0.001532362941176471</v>
+        <v>0.001748718294117647</v>
       </c>
       <c r="AF21" s="11" t="n">
-        <v>0.1378315873015873</v>
+        <v>0.1572921216931217</v>
       </c>
       <c r="AG21" s="11" t="n">
-        <v>464.8796448799999</v>
+        <v>468.55768588</v>
       </c>
       <c r="AH21" s="11" t="n">
-        <v>0.02734586146352942</v>
+        <v>0.02756221681647059</v>
       </c>
       <c r="AI21" s="11" t="n">
-        <v>2.459680660740741</v>
+        <v>2.479141195132275</v>
       </c>
     </row>
     <row r="22">
@@ -15595,22 +15601,22 @@
         <v>0.332547619047619</v>
       </c>
       <c r="AD24" s="13" t="n">
-        <v>21.4225</v>
+        <v>24.569</v>
       </c>
       <c r="AE24" s="13" t="n">
-        <v>0.001260147058823529</v>
+        <v>0.001445235294117647</v>
       </c>
       <c r="AF24" s="13" t="n">
-        <v>0.1133465608465608</v>
+        <v>0.129994708994709</v>
       </c>
       <c r="AG24" s="13" t="n">
-        <v>84.274</v>
+        <v>87.4205</v>
       </c>
       <c r="AH24" s="13" t="n">
-        <v>0.00495729411764706</v>
+        <v>0.005142382352941177</v>
       </c>
       <c r="AI24" s="13" t="n">
-        <v>0.4458941798941799</v>
+        <v>0.462542328042328</v>
       </c>
     </row>
     <row r="25">
@@ -16378,153 +16384,159 @@
     <row r="37">
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Foreign Fluctuation Gain Or Loss</t>
+          <t xml:space="preserve">        PT. Asuransi Allianz Utama Indonesia</t>
         </is>
       </c>
       <c r="C37" s="11" t="n"/>
       <c r="D37" s="11" t="n"/>
       <c r="E37" s="11" t="n"/>
       <c r="F37" s="11" t="n">
-        <v>0.6054326800000001</v>
+        <v>0.283992</v>
       </c>
       <c r="G37" s="11" t="n">
-        <v>3.561368705882353e-05</v>
+        <v>1.670541176470588e-05</v>
       </c>
       <c r="H37" s="11" t="n">
-        <v>0.003203347513227513</v>
-      </c>
-      <c r="I37" s="11" t="n">
-        <v>0.01997784</v>
-      </c>
-      <c r="J37" s="11" t="n">
-        <v>1.175167058823529e-06</v>
-      </c>
-      <c r="K37" s="11" t="n">
-        <v>0.0001057028571428571</v>
-      </c>
-      <c r="L37" s="11" t="n">
-        <v>0.39162725</v>
-      </c>
-      <c r="M37" s="11" t="n">
-        <v>2.303689705882353e-05</v>
-      </c>
-      <c r="N37" s="11" t="n">
-        <v>0.002072101851851852</v>
-      </c>
-      <c r="O37" s="11" t="n">
-        <v>0.7565786799999999</v>
-      </c>
-      <c r="P37" s="11" t="n">
-        <v>4.450462823529412e-05</v>
-      </c>
-      <c r="Q37" s="11" t="n">
-        <v>0.004003061798941799</v>
-      </c>
-      <c r="R37" s="11" t="n">
-        <v>0.05579961</v>
-      </c>
-      <c r="S37" s="11" t="n">
-        <v>3.28233e-06</v>
-      </c>
-      <c r="T37" s="11" t="n">
-        <v>0.0002952360317460317</v>
-      </c>
-      <c r="U37" s="11" t="n"/>
-      <c r="V37" s="11" t="n"/>
-      <c r="W37" s="11" t="n"/>
-      <c r="X37" s="11" t="n">
-        <v>0.29172</v>
-      </c>
-      <c r="Y37" s="11" t="n">
-        <v>1.716e-05</v>
-      </c>
-      <c r="Z37" s="11" t="n">
-        <v>0.001543492063492063</v>
-      </c>
+        <v>0.001502603174603175</v>
+      </c>
+      <c r="I37" s="11" t="n"/>
+      <c r="J37" s="11" t="n"/>
+      <c r="K37" s="11" t="n"/>
+      <c r="L37" s="11" t="n"/>
+      <c r="M37" s="11" t="n"/>
+      <c r="N37" s="11" t="n"/>
+      <c r="O37" s="11" t="n"/>
+      <c r="P37" s="11" t="n"/>
+      <c r="Q37" s="11" t="n"/>
+      <c r="R37" s="11" t="n"/>
+      <c r="S37" s="11" t="n"/>
+      <c r="T37" s="11" t="n"/>
+      <c r="U37" s="11" t="n">
+        <v>1.3603</v>
+      </c>
+      <c r="V37" s="11" t="n">
+        <v>8.001764705882353e-05</v>
+      </c>
+      <c r="W37" s="11" t="n">
+        <v>0.007197354497354497</v>
+      </c>
+      <c r="X37" s="11" t="n"/>
+      <c r="Y37" s="11" t="n"/>
+      <c r="Z37" s="11" t="n"/>
       <c r="AA37" s="11" t="n">
-        <v>2.12113606</v>
+        <v>1.644292</v>
       </c>
       <c r="AB37" s="11" t="n">
-        <v>0.0001247727094117647</v>
+        <v>9.672305882352941e-05</v>
       </c>
       <c r="AC37" s="11" t="n">
-        <v>0.01122294211640212</v>
-      </c>
-      <c r="AD37" s="11" t="n"/>
-      <c r="AE37" s="11" t="n"/>
-      <c r="AF37" s="11" t="n"/>
+        <v>0.008699957671957671</v>
+      </c>
+      <c r="AD37" s="11" t="n">
+        <v>0.531541</v>
+      </c>
+      <c r="AE37" s="11" t="n">
+        <v>3.126711764705883e-05</v>
+      </c>
+      <c r="AF37" s="11" t="n">
+        <v>0.002812386243386244</v>
+      </c>
       <c r="AG37" s="11" t="n">
-        <v>2.12113606</v>
+        <v>2.175833</v>
       </c>
       <c r="AH37" s="11" t="n">
-        <v>0.0001247727094117647</v>
+        <v>0.0001279901764705882</v>
       </c>
       <c r="AI37" s="11" t="n">
-        <v>0.01122294211640212</v>
+        <v>0.01151234391534391</v>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">        PT. Asuransi Allianz Utama Indonesia</t>
+          <t xml:space="preserve">        Foreign Fluctuation Gain Or Loss</t>
         </is>
       </c>
       <c r="C38" s="13" t="n"/>
       <c r="D38" s="13" t="n"/>
       <c r="E38" s="13" t="n"/>
       <c r="F38" s="13" t="n">
-        <v>0.283992</v>
+        <v>0.6054326800000001</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>1.670541176470588e-05</v>
+        <v>3.561368705882353e-05</v>
       </c>
       <c r="H38" s="13" t="n">
-        <v>0.001502603174603175</v>
-      </c>
-      <c r="I38" s="13" t="n"/>
-      <c r="J38" s="13" t="n"/>
-      <c r="K38" s="13" t="n"/>
-      <c r="L38" s="13" t="n"/>
-      <c r="M38" s="13" t="n"/>
-      <c r="N38" s="13" t="n"/>
-      <c r="O38" s="13" t="n"/>
-      <c r="P38" s="13" t="n"/>
-      <c r="Q38" s="13" t="n"/>
-      <c r="R38" s="13" t="n"/>
-      <c r="S38" s="13" t="n"/>
-      <c r="T38" s="13" t="n"/>
-      <c r="U38" s="13" t="n">
-        <v>1.3603</v>
-      </c>
-      <c r="V38" s="13" t="n">
-        <v>8.001764705882353e-05</v>
-      </c>
-      <c r="W38" s="13" t="n">
-        <v>0.007197354497354497</v>
-      </c>
-      <c r="X38" s="13" t="n"/>
-      <c r="Y38" s="13" t="n"/>
-      <c r="Z38" s="13" t="n"/>
+        <v>0.003203347513227513</v>
+      </c>
+      <c r="I38" s="13" t="n">
+        <v>0.01997784</v>
+      </c>
+      <c r="J38" s="13" t="n">
+        <v>1.175167058823529e-06</v>
+      </c>
+      <c r="K38" s="13" t="n">
+        <v>0.0001057028571428571</v>
+      </c>
+      <c r="L38" s="13" t="n">
+        <v>0.39162725</v>
+      </c>
+      <c r="M38" s="13" t="n">
+        <v>2.303689705882353e-05</v>
+      </c>
+      <c r="N38" s="13" t="n">
+        <v>0.002072101851851852</v>
+      </c>
+      <c r="O38" s="13" t="n">
+        <v>0.7565786799999999</v>
+      </c>
+      <c r="P38" s="13" t="n">
+        <v>4.450462823529412e-05</v>
+      </c>
+      <c r="Q38" s="13" t="n">
+        <v>0.004003061798941799</v>
+      </c>
+      <c r="R38" s="13" t="n">
+        <v>0.05579961</v>
+      </c>
+      <c r="S38" s="13" t="n">
+        <v>3.28233e-06</v>
+      </c>
+      <c r="T38" s="13" t="n">
+        <v>0.0002952360317460317</v>
+      </c>
+      <c r="U38" s="13" t="n"/>
+      <c r="V38" s="13" t="n"/>
+      <c r="W38" s="13" t="n"/>
+      <c r="X38" s="13" t="n">
+        <v>0.29172</v>
+      </c>
+      <c r="Y38" s="13" t="n">
+        <v>1.716e-05</v>
+      </c>
+      <c r="Z38" s="13" t="n">
+        <v>0.001543492063492063</v>
+      </c>
       <c r="AA38" s="13" t="n">
-        <v>1.644292</v>
+        <v>2.12113606</v>
       </c>
       <c r="AB38" s="13" t="n">
-        <v>9.672305882352941e-05</v>
+        <v>0.0001247727094117647</v>
       </c>
       <c r="AC38" s="13" t="n">
-        <v>0.008699957671957671</v>
+        <v>0.01122294211640212</v>
       </c>
       <c r="AD38" s="13" t="n"/>
       <c r="AE38" s="13" t="n"/>
       <c r="AF38" s="13" t="n"/>
       <c r="AG38" s="13" t="n">
-        <v>1.644292</v>
+        <v>2.12113606</v>
       </c>
       <c r="AH38" s="13" t="n">
-        <v>9.672305882352941e-05</v>
+        <v>0.0001247727094117647</v>
       </c>
       <c r="AI38" s="13" t="n">
-        <v>0.008699957671957671</v>
+        <v>0.01122294211640212</v>
       </c>
     </row>
     <row r="39">
@@ -17045,22 +17057,22 @@
         <v>1180.222393205714</v>
       </c>
       <c r="AD46" s="15" t="n">
-        <v>15729.020815</v>
+        <v>15732.698856</v>
       </c>
       <c r="AE46" s="15" t="n">
-        <v>0.9252365185294118</v>
+        <v>0.925452873882353</v>
       </c>
       <c r="AF46" s="15" t="n">
-        <v>83.22233235449735</v>
+        <v>83.2417928888889</v>
       </c>
       <c r="AG46" s="15" t="n">
-        <v>238791.05313088</v>
+        <v>238794.73117188</v>
       </c>
       <c r="AH46" s="15" t="n">
-        <v>14.04653253711059</v>
+        <v>14.04674889246353</v>
       </c>
       <c r="AI46" s="15" t="n">
-        <v>1263.444725560212</v>
+        <v>1263.464186094603</v>
       </c>
     </row>
     <row r="47">
@@ -23497,22 +23509,22 @@
         <v>-5.069808166825397</v>
       </c>
       <c r="AD129" s="13" t="n">
-        <v>-123.6755</v>
+        <v>-166.617666</v>
       </c>
       <c r="AE129" s="13" t="n">
-        <v>-0.007275029411764706</v>
+        <v>-0.009801039176470589</v>
       </c>
       <c r="AF129" s="13" t="n">
-        <v>-0.6543677248677249</v>
+        <v>-0.8815749523809524</v>
       </c>
       <c r="AG129" s="13" t="n">
-        <v>-1081.86924353</v>
+        <v>-1124.81140953</v>
       </c>
       <c r="AH129" s="13" t="n">
-        <v>-0.06363936726647058</v>
+        <v>-0.06616537703117648</v>
       </c>
       <c r="AI129" s="13" t="n">
-        <v>-5.724175891693122</v>
+        <v>-5.95138311920635</v>
       </c>
     </row>
     <row r="130">
@@ -23909,22 +23921,22 @@
         <v>-132.568430727672</v>
       </c>
       <c r="AD133" s="15" t="n">
-        <v>-226.301416</v>
+        <v>-269.243582</v>
       </c>
       <c r="AE133" s="15" t="n">
-        <v>-0.013311848</v>
+        <v>-0.01583785776470588</v>
       </c>
       <c r="AF133" s="15" t="n">
-        <v>-1.197361989417989</v>
+        <v>-1.424569216931217</v>
       </c>
       <c r="AG133" s="15" t="n">
-        <v>-25281.73482353</v>
+        <v>-25324.67698953</v>
       </c>
       <c r="AH133" s="15" t="n">
-        <v>-1.487160871972353</v>
+        <v>-1.489686881737059</v>
       </c>
       <c r="AI133" s="15" t="n">
-        <v>-133.76579271709</v>
+        <v>-133.9929999446032</v>
       </c>
     </row>
     <row r="134">
@@ -24713,22 +24725,22 @@
         <v>-230.2759330393122</v>
       </c>
       <c r="AD142" s="15" t="n">
-        <v>-1169.198561</v>
+        <v>-1212.140727</v>
       </c>
       <c r="AE142" s="15" t="n">
-        <v>-0.06877638594117647</v>
+        <v>-0.07130239570588236</v>
       </c>
       <c r="AF142" s="15" t="n">
-        <v>-6.186235772486772</v>
+        <v>-6.413443</v>
       </c>
       <c r="AG142" s="15" t="n">
-        <v>-44691.34990543</v>
+        <v>-44734.29207143</v>
       </c>
       <c r="AH142" s="15" t="n">
-        <v>-2.628902935613529</v>
+        <v>-2.631428945378235</v>
       </c>
       <c r="AI142" s="15" t="n">
-        <v>-236.4621688117989</v>
+        <v>-236.6893760393122</v>
       </c>
     </row>
     <row r="143">
@@ -25309,22 +25321,22 @@
         <v>-0.09944919407407407</v>
       </c>
       <c r="AD150" s="11" t="n">
-        <v>-0.2225</v>
+        <v>-1.2508</v>
       </c>
       <c r="AE150" s="11" t="n">
-        <v>-1.308823529411765e-05</v>
+        <v>-7.357647058823529e-05</v>
       </c>
       <c r="AF150" s="11" t="n">
-        <v>-0.001177248677248677</v>
+        <v>-0.006617989417989418</v>
       </c>
       <c r="AG150" s="11" t="n">
-        <v>-19.01839768</v>
+        <v>-20.04669768</v>
       </c>
       <c r="AH150" s="11" t="n">
-        <v>-0.001118729275294118</v>
+        <v>-0.001179217510588236</v>
       </c>
       <c r="AI150" s="11" t="n">
-        <v>-0.1006264427513228</v>
+        <v>-0.1060671834920635</v>
       </c>
     </row>
     <row r="151">
@@ -25807,22 +25819,22 @@
         <v>-31.58386807253968</v>
       </c>
       <c r="AD156" s="15" t="n">
-        <v>-182.744642</v>
+        <v>-183.772942</v>
       </c>
       <c r="AE156" s="15" t="n">
-        <v>-0.01074968482352941</v>
+        <v>-0.01081017305882353</v>
       </c>
       <c r="AF156" s="15" t="n">
-        <v>-0.9669028677248677</v>
+        <v>-0.9723436084656085</v>
       </c>
       <c r="AG156" s="15" t="n">
-        <v>-6152.09570771</v>
+        <v>-6153.12400771</v>
       </c>
       <c r="AH156" s="15" t="n">
-        <v>-0.3618879828064707</v>
+        <v>-0.3619484710417648</v>
       </c>
       <c r="AI156" s="15" t="n">
-        <v>-32.55077094026455</v>
+        <v>-32.55621168100529</v>
       </c>
     </row>
     <row r="157">
@@ -25913,22 +25925,22 @@
         <v>-1529.478500653756</v>
       </c>
       <c r="AD157" s="19" t="n">
-        <v>-9475.645339999999</v>
+        <v>-9519.615806</v>
       </c>
       <c r="AE157" s="19" t="n">
-        <v>-0.5573909023529411</v>
+        <v>-0.5599774003529412</v>
       </c>
       <c r="AF157" s="19" t="n">
-        <v>-50.13568962962962</v>
+        <v>-50.3683375978836</v>
       </c>
       <c r="AG157" s="19" t="n">
-        <v>-298547.0819635599</v>
+        <v>-298591.0524295599</v>
       </c>
       <c r="AH157" s="19" t="n">
-        <v>-17.56159305668</v>
+        <v>-17.56417955468</v>
       </c>
       <c r="AI157" s="19" t="n">
-        <v>-1579.614190283386</v>
+        <v>-1579.84683825164</v>
       </c>
     </row>
     <row r="158">
@@ -26019,22 +26031,22 @@
         <v>-349.2561074480424</v>
       </c>
       <c r="AD158" s="19" t="n">
-        <v>6253.375475</v>
+        <v>6213.08305</v>
       </c>
       <c r="AE158" s="19" t="n">
-        <v>0.3678456161764706</v>
+        <v>0.3654754735294118</v>
       </c>
       <c r="AF158" s="19" t="n">
-        <v>33.08664272486772</v>
+        <v>32.87345529100529</v>
       </c>
       <c r="AG158" s="19" t="n">
-        <v>-59756.02883268001</v>
+        <v>-59796.32125768001</v>
       </c>
       <c r="AH158" s="19" t="n">
-        <v>-3.515060519569412</v>
+        <v>-3.517430662216471</v>
       </c>
       <c r="AI158" s="19" t="n">
-        <v>-316.1694647231747</v>
+        <v>-316.3826521570371</v>
       </c>
     </row>
     <row r="159">
@@ -26125,22 +26137,22 @@
         <v>7.747388987724859</v>
       </c>
       <c r="AD159" s="7" t="n">
-        <v>7717.63199368</v>
+        <v>7677.33956868</v>
       </c>
       <c r="AE159" s="7" t="n">
-        <v>0.4539783525694118</v>
+        <v>0.451608209922353</v>
       </c>
       <c r="AF159" s="7" t="n">
-        <v>40.83403171259259</v>
+        <v>40.62084427873016</v>
       </c>
       <c r="AG159" s="7" t="n">
-        <v>7717.63199368</v>
+        <v>7677.33956868</v>
       </c>
       <c r="AH159" s="7" t="n">
-        <v>0.4539783525694118</v>
+        <v>0.451608209922353</v>
       </c>
       <c r="AI159" s="7" t="n">
-        <v>40.83403171259259</v>
+        <v>40.62084427873016</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Mon 09/28/2026 16:32
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 25 Sep 2026 16:20</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Sep 2026 16:32</t>
         </is>
       </c>
     </row>
@@ -805,14 +805,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 25 Sep 2026</t>
+          <t>MTD as of 28 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 25 Sep 2026</t>
+          <t>YTD as of 28 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
@@ -2208,22 +2208,22 @@
         <v>2321849.073439153</v>
       </c>
       <c r="AD20" s="13" t="n">
-        <v>33857211</v>
+        <v>36231211</v>
       </c>
       <c r="AE20" s="13" t="n">
-        <v>1991.600647058824</v>
+        <v>2131.247705882353</v>
       </c>
       <c r="AF20" s="13" t="n">
-        <v>179138.6825396825</v>
+        <v>191699.5291005291</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>472686685.88</v>
+        <v>475060685.88</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>27805.09916941177</v>
+        <v>27944.7462282353</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>2500987.755978836</v>
+        <v>2513548.602539682</v>
       </c>
     </row>
     <row r="21">
@@ -2460,22 +2460,22 @@
         <v>332547.6190476191</v>
       </c>
       <c r="AD23" s="11" t="n">
-        <v>27384500</v>
+        <v>29365500</v>
       </c>
       <c r="AE23" s="11" t="n">
-        <v>1610.85294117647</v>
+        <v>1727.382352941177</v>
       </c>
       <c r="AF23" s="11" t="n">
-        <v>144891.5343915344</v>
+        <v>155373.0158730159</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>90236000</v>
+        <v>92217000</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>5307.999999999999</v>
+        <v>5424.529411764705</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>477439.1534391535</v>
+        <v>487920.6349206349</v>
       </c>
     </row>
     <row r="24">
@@ -2855,17 +2855,23 @@
       <c r="AC29" s="11" t="n">
         <v>39765.75132275133</v>
       </c>
-      <c r="AD29" s="11" t="n"/>
-      <c r="AE29" s="11" t="n"/>
-      <c r="AF29" s="11" t="n"/>
+      <c r="AD29" s="11" t="n">
+        <v>393000</v>
+      </c>
+      <c r="AE29" s="11" t="n">
+        <v>23.11764705882353</v>
+      </c>
+      <c r="AF29" s="11" t="n">
+        <v>2079.36507936508</v>
+      </c>
       <c r="AG29" s="11" t="n">
-        <v>7515727</v>
+        <v>7908727</v>
       </c>
       <c r="AH29" s="11" t="n">
-        <v>442.1015882352941</v>
+        <v>465.2192352941177</v>
       </c>
       <c r="AI29" s="11" t="n">
-        <v>39765.75132275133</v>
+        <v>41845.11640211641</v>
       </c>
     </row>
     <row r="30">
@@ -3916,22 +3922,22 @@
         <v>1180222393.205714</v>
       </c>
       <c r="AD45" s="15" t="n">
-        <v>15825096771</v>
+        <v>15827470771</v>
       </c>
       <c r="AE45" s="15" t="n">
-        <v>930888.0453529411</v>
+        <v>931027.6924117648</v>
       </c>
       <c r="AF45" s="15" t="n">
-        <v>83730670.74603175</v>
+        <v>83743231.5925926</v>
       </c>
       <c r="AG45" s="15" t="n">
-        <v>238887129086.88</v>
+        <v>238889503086.88</v>
       </c>
       <c r="AH45" s="15" t="n">
-        <v>14052184.06393412</v>
+        <v>14052323.71099294</v>
       </c>
       <c r="AI45" s="15" t="n">
-        <v>1263953063.951746</v>
+        <v>1263965624.798307</v>
       </c>
     </row>
     <row r="46">
@@ -11836,22 +11842,22 @@
         <v>-4894589.497354497</v>
       </c>
       <c r="AD144" s="13" t="n">
-        <v>-73082868</v>
+        <v>-105582868</v>
       </c>
       <c r="AE144" s="13" t="n">
-        <v>-4298.992235294118</v>
+        <v>-6210.756941176471</v>
       </c>
       <c r="AF144" s="13" t="n">
-        <v>-386681.8412698412</v>
+        <v>-558639.5132275132</v>
       </c>
       <c r="AG144" s="13" t="n">
-        <v>-998160283</v>
+        <v>-1030660283</v>
       </c>
       <c r="AH144" s="13" t="n">
-        <v>-58715.31076470588</v>
+        <v>-60627.07547058824</v>
       </c>
       <c r="AI144" s="13" t="n">
-        <v>-5281271.338624339</v>
+        <v>-5453229.01058201</v>
       </c>
     </row>
     <row r="145">
@@ -12058,22 +12064,22 @@
         <v>-13736457.22222222</v>
       </c>
       <c r="AD147" s="15" t="n">
-        <v>-73082868</v>
+        <v>-105582868</v>
       </c>
       <c r="AE147" s="15" t="n">
-        <v>-4298.992235294118</v>
+        <v>-6210.756941176471</v>
       </c>
       <c r="AF147" s="15" t="n">
-        <v>-386681.8412698412</v>
+        <v>-558639.5132275132</v>
       </c>
       <c r="AG147" s="15" t="n">
-        <v>-2669273283</v>
+        <v>-2701773283</v>
       </c>
       <c r="AH147" s="15" t="n">
-        <v>-157016.0754705882</v>
+        <v>-158927.8401764706</v>
       </c>
       <c r="AI147" s="15" t="n">
-        <v>-14123139.06349206</v>
+        <v>-14295096.73544974</v>
       </c>
     </row>
     <row r="148">
@@ -12204,22 +12210,22 @@
         <v>-99449.19407407405</v>
       </c>
       <c r="AD149" s="11" t="n">
-        <v>-1265800</v>
+        <v>-1268300</v>
       </c>
       <c r="AE149" s="11" t="n">
-        <v>-74.45882352941176</v>
+        <v>-74.60588235294118</v>
       </c>
       <c r="AF149" s="11" t="n">
-        <v>-6697.354497354498</v>
+        <v>-6710.58201058201</v>
       </c>
       <c r="AG149" s="11" t="n">
-        <v>-20061697.68</v>
+        <v>-20064197.68</v>
       </c>
       <c r="AH149" s="11" t="n">
-        <v>-1180.099863529412</v>
+        <v>-1180.246922352941</v>
       </c>
       <c r="AI149" s="11" t="n">
-        <v>-106146.5485714285</v>
+        <v>-106159.7760846561</v>
       </c>
     </row>
     <row r="150">
@@ -12702,22 +12708,22 @@
         <v>-31583868.07253968</v>
       </c>
       <c r="AD155" s="15" t="n">
-        <v>-183787942</v>
+        <v>-183790442</v>
       </c>
       <c r="AE155" s="15" t="n">
-        <v>-10811.05541176471</v>
+        <v>-10811.20247058824</v>
       </c>
       <c r="AF155" s="15" t="n">
-        <v>-972422.9735449735</v>
+        <v>-972436.201058201</v>
       </c>
       <c r="AG155" s="15" t="n">
-        <v>-6153139007.710001</v>
+        <v>-6153141507.710001</v>
       </c>
       <c r="AH155" s="15" t="n">
-        <v>-361949.3533947059</v>
+        <v>-361949.5004535294</v>
       </c>
       <c r="AI155" s="15" t="n">
-        <v>-32556291.04608466</v>
+        <v>-32556304.27359788</v>
       </c>
     </row>
     <row r="156">
@@ -12808,22 +12814,22 @@
         <v>-1529478500.653757</v>
       </c>
       <c r="AD156" s="19" t="n">
-        <v>-14676196553</v>
+        <v>-14708699053</v>
       </c>
       <c r="AE156" s="19" t="n">
-        <v>-863305.6795882353</v>
+        <v>-865217.5913529411</v>
       </c>
       <c r="AF156" s="19" t="n">
-        <v>-77651833.61375661</v>
+        <v>-77823804.51322751</v>
       </c>
       <c r="AG156" s="19" t="n">
-        <v>-303747633176.5599</v>
+        <v>-303780135676.5599</v>
       </c>
       <c r="AH156" s="19" t="n">
-        <v>-17867507.83391529</v>
+        <v>-17869419.74568</v>
       </c>
       <c r="AI156" s="19" t="n">
-        <v>-1607130334.267513</v>
+        <v>-1607302305.166984</v>
       </c>
     </row>
     <row r="157">
@@ -12914,22 +12920,22 @@
         <v>-349256107.4480425</v>
       </c>
       <c r="AD157" s="19" t="n">
-        <v>1148900218</v>
+        <v>1118771718</v>
       </c>
       <c r="AE157" s="19" t="n">
-        <v>67582.36576470589</v>
+        <v>65810.10105882352</v>
       </c>
       <c r="AF157" s="19" t="n">
-        <v>6078837.132275132</v>
+        <v>5919427.079365079</v>
       </c>
       <c r="AG157" s="19" t="n">
-        <v>-64860504089.68</v>
+        <v>-64890632589.68</v>
       </c>
       <c r="AH157" s="19" t="n">
-        <v>-3815323.769981177</v>
+        <v>-3817096.034687059</v>
       </c>
       <c r="AI157" s="19" t="n">
-        <v>-343177270.3157673</v>
+        <v>-343336680.3686774</v>
       </c>
     </row>
     <row r="158">
@@ -13020,22 +13026,22 @@
         <v>7747388.987724859</v>
       </c>
       <c r="AD158" s="7" t="n">
-        <v>2613156736.68</v>
+        <v>2583028236.68</v>
       </c>
       <c r="AE158" s="7" t="n">
-        <v>153715.1021576471</v>
+        <v>151942.8374517647</v>
       </c>
       <c r="AF158" s="7" t="n">
-        <v>13826226.12</v>
+        <v>13666816.06708995</v>
       </c>
       <c r="AG158" s="7" t="n">
-        <v>2613156736.68</v>
+        <v>2583028236.68</v>
       </c>
       <c r="AH158" s="7" t="n">
-        <v>153715.1021576471</v>
+        <v>151942.8374517647</v>
       </c>
       <c r="AI158" s="7" t="n">
-        <v>13826226.12</v>
+        <v>13666816.06708995</v>
       </c>
     </row>
   </sheetData>
@@ -13596,16 +13602,16 @@
         <v>172976399.24</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>-93299332</v>
+        <v>-123427832</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>79677067.24000001</v>
+        <v>49548567.24000001</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>4686.886308235295</v>
+        <v>2914.621602352942</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>421571.7843386244</v>
+        <v>262161.7314285715</v>
       </c>
     </row>
     <row r="10">
@@ -13715,13 +13721,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>2613156738.68</v>
+        <v>2583028238.68</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>153715.1022752941</v>
+        <v>151942.8375694118</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>13826226.13058201</v>
+        <v>13666816.07767196</v>
       </c>
     </row>
   </sheetData>
@@ -13791,7 +13797,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 25 Sep 2026 16:20 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Sep 2026 16:32 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -13866,14 +13872,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 25 Sep 2026</t>
+          <t>MTD as of 28 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 25 Sep 2026</t>
+          <t>YTD as of 28 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
@@ -15269,22 +15275,22 @@
         <v>2.321849073439154</v>
       </c>
       <c r="AD20" s="13" t="n">
-        <v>33.857211</v>
+        <v>36.231211</v>
       </c>
       <c r="AE20" s="13" t="n">
-        <v>0.001991600647058824</v>
+        <v>0.002131247705882353</v>
       </c>
       <c r="AF20" s="13" t="n">
-        <v>0.1791386825396825</v>
+        <v>0.1916995291005291</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>472.68668588</v>
+        <v>475.0606858799999</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>0.02780509916941177</v>
+        <v>0.02794474622823529</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>2.500987755978836</v>
+        <v>2.513548602539683</v>
       </c>
     </row>
     <row r="21">
@@ -15521,22 +15527,22 @@
         <v>0.332547619047619</v>
       </c>
       <c r="AD23" s="11" t="n">
-        <v>27.3845</v>
+        <v>29.3655</v>
       </c>
       <c r="AE23" s="11" t="n">
-        <v>0.001610852941176471</v>
+        <v>0.001727382352941176</v>
       </c>
       <c r="AF23" s="11" t="n">
-        <v>0.1448915343915344</v>
+        <v>0.1553730158730159</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>90.236</v>
+        <v>92.217</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>0.005308</v>
+        <v>0.005424529411764707</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>0.4774391534391534</v>
+        <v>0.4879206349206349</v>
       </c>
     </row>
     <row r="24">
@@ -15916,17 +15922,23 @@
       <c r="AC29" s="11" t="n">
         <v>0.03976575132275132</v>
       </c>
-      <c r="AD29" s="11" t="n"/>
-      <c r="AE29" s="11" t="n"/>
-      <c r="AF29" s="11" t="n"/>
+      <c r="AD29" s="11" t="n">
+        <v>0.393</v>
+      </c>
+      <c r="AE29" s="11" t="n">
+        <v>2.311764705882353e-05</v>
+      </c>
+      <c r="AF29" s="11" t="n">
+        <v>0.002079365079365079</v>
+      </c>
       <c r="AG29" s="11" t="n">
-        <v>7.515727</v>
+        <v>7.908727</v>
       </c>
       <c r="AH29" s="11" t="n">
-        <v>0.0004421015882352941</v>
+        <v>0.0004652192352941176</v>
       </c>
       <c r="AI29" s="11" t="n">
-        <v>0.03976575132275132</v>
+        <v>0.0418451164021164</v>
       </c>
     </row>
     <row r="30">
@@ -16977,22 +16989,22 @@
         <v>1180.222393205714</v>
       </c>
       <c r="AD45" s="15" t="n">
-        <v>15825.096771</v>
+        <v>15827.470771</v>
       </c>
       <c r="AE45" s="15" t="n">
-        <v>0.9308880453529412</v>
+        <v>0.9310276924117648</v>
       </c>
       <c r="AF45" s="15" t="n">
-        <v>83.73067074603175</v>
+        <v>83.74323159259259</v>
       </c>
       <c r="AG45" s="15" t="n">
-        <v>238887.12908688</v>
+        <v>238889.50308688</v>
       </c>
       <c r="AH45" s="15" t="n">
-        <v>14.05218406393412</v>
+        <v>14.05232371099294</v>
       </c>
       <c r="AI45" s="15" t="n">
-        <v>1263.953063951746</v>
+        <v>1263.965624798307</v>
       </c>
     </row>
     <row r="46">
@@ -24897,22 +24909,22 @@
         <v>-4.894589497354497</v>
       </c>
       <c r="AD144" s="13" t="n">
-        <v>-73.082868</v>
+        <v>-105.582868</v>
       </c>
       <c r="AE144" s="13" t="n">
-        <v>-0.004298992235294118</v>
+        <v>-0.006210756941176471</v>
       </c>
       <c r="AF144" s="13" t="n">
-        <v>-0.3866818412698413</v>
+        <v>-0.5586395132275133</v>
       </c>
       <c r="AG144" s="13" t="n">
-        <v>-998.160283</v>
+        <v>-1030.660283</v>
       </c>
       <c r="AH144" s="13" t="n">
-        <v>-0.0587153107647059</v>
+        <v>-0.06062707547058824</v>
       </c>
       <c r="AI144" s="13" t="n">
-        <v>-5.281271338624339</v>
+        <v>-5.45322901058201</v>
       </c>
     </row>
     <row r="145">
@@ -25119,22 +25131,22 @@
         <v>-13.73645722222222</v>
       </c>
       <c r="AD147" s="15" t="n">
-        <v>-73.082868</v>
+        <v>-105.582868</v>
       </c>
       <c r="AE147" s="15" t="n">
-        <v>-0.004298992235294118</v>
+        <v>-0.006210756941176471</v>
       </c>
       <c r="AF147" s="15" t="n">
-        <v>-0.3866818412698413</v>
+        <v>-0.5586395132275133</v>
       </c>
       <c r="AG147" s="15" t="n">
-        <v>-2669.273283</v>
+        <v>-2701.773283</v>
       </c>
       <c r="AH147" s="15" t="n">
-        <v>-0.1570160754705882</v>
+        <v>-0.1589278401764706</v>
       </c>
       <c r="AI147" s="15" t="n">
-        <v>-14.12313906349206</v>
+        <v>-14.29509673544974</v>
       </c>
     </row>
     <row r="148">
@@ -25265,22 +25277,22 @@
         <v>-0.09944919407407407</v>
       </c>
       <c r="AD149" s="11" t="n">
-        <v>-1.2658</v>
+        <v>-1.2683</v>
       </c>
       <c r="AE149" s="11" t="n">
-        <v>-7.445882352941176e-05</v>
+        <v>-7.460588235294118e-05</v>
       </c>
       <c r="AF149" s="11" t="n">
-        <v>-0.006697354497354498</v>
+        <v>-0.006710582010582011</v>
       </c>
       <c r="AG149" s="11" t="n">
-        <v>-20.06169768</v>
+        <v>-20.06419768</v>
       </c>
       <c r="AH149" s="11" t="n">
-        <v>-0.001180099863529412</v>
+        <v>-0.001180246922352941</v>
       </c>
       <c r="AI149" s="11" t="n">
-        <v>-0.1061465485714286</v>
+        <v>-0.1061597760846561</v>
       </c>
     </row>
     <row r="150">
@@ -25763,22 +25775,22 @@
         <v>-31.58386807253968</v>
       </c>
       <c r="AD155" s="15" t="n">
-        <v>-183.787942</v>
+        <v>-183.790442</v>
       </c>
       <c r="AE155" s="15" t="n">
-        <v>-0.01081105541176471</v>
+        <v>-0.01081120247058824</v>
       </c>
       <c r="AF155" s="15" t="n">
-        <v>-0.9724229735449734</v>
+        <v>-0.9724362010582012</v>
       </c>
       <c r="AG155" s="15" t="n">
-        <v>-6153.13900771</v>
+        <v>-6153.141507710001</v>
       </c>
       <c r="AH155" s="15" t="n">
-        <v>-0.361949353394706</v>
+        <v>-0.3619495004535295</v>
       </c>
       <c r="AI155" s="15" t="n">
-        <v>-32.55629104608465</v>
+        <v>-32.55630427359788</v>
       </c>
     </row>
     <row r="156">
@@ -25869,22 +25881,22 @@
         <v>-1529.478500653756</v>
       </c>
       <c r="AD156" s="19" t="n">
-        <v>-14676.196553</v>
+        <v>-14708.699053</v>
       </c>
       <c r="AE156" s="19" t="n">
-        <v>-0.8633056795882352</v>
+        <v>-0.8652175913529412</v>
       </c>
       <c r="AF156" s="19" t="n">
-        <v>-77.65183361375661</v>
+        <v>-77.82380451322751</v>
       </c>
       <c r="AG156" s="19" t="n">
-        <v>-303747.6331765599</v>
+        <v>-303780.1356765599</v>
       </c>
       <c r="AH156" s="19" t="n">
-        <v>-17.8675078339153</v>
+        <v>-17.86941974568</v>
       </c>
       <c r="AI156" s="19" t="n">
-        <v>-1607.130334267513</v>
+        <v>-1607.302305166984</v>
       </c>
     </row>
     <row r="157">
@@ -25975,22 +25987,22 @@
         <v>-349.2561074480424</v>
       </c>
       <c r="AD157" s="19" t="n">
-        <v>1148.900218</v>
+        <v>1118.771718</v>
       </c>
       <c r="AE157" s="19" t="n">
-        <v>0.06758236576470589</v>
+        <v>0.06581010105882353</v>
       </c>
       <c r="AF157" s="19" t="n">
-        <v>6.078837132275132</v>
+        <v>5.91942707936508</v>
       </c>
       <c r="AG157" s="19" t="n">
-        <v>-64860.50408968001</v>
+        <v>-64890.63258968001</v>
       </c>
       <c r="AH157" s="19" t="n">
-        <v>-3.815323769981177</v>
+        <v>-3.81709603468706</v>
       </c>
       <c r="AI157" s="19" t="n">
-        <v>-343.1772703157673</v>
+        <v>-343.3366803686773</v>
       </c>
     </row>
     <row r="158">
@@ -26081,22 +26093,22 @@
         <v>7.747388987724859</v>
       </c>
       <c r="AD158" s="7" t="n">
-        <v>2613.15673668</v>
+        <v>2583.02823668</v>
       </c>
       <c r="AE158" s="7" t="n">
-        <v>0.1537151021576471</v>
+        <v>0.1519428374517647</v>
       </c>
       <c r="AF158" s="7" t="n">
-        <v>13.82622612</v>
+        <v>13.66681606708995</v>
       </c>
       <c r="AG158" s="7" t="n">
-        <v>2613.15673668</v>
+        <v>2583.02823668</v>
       </c>
       <c r="AH158" s="7" t="n">
-        <v>0.1537151021576471</v>
+        <v>0.1519428374517647</v>
       </c>
       <c r="AI158" s="7" t="n">
-        <v>13.82622612</v>
+        <v>13.66681606708995</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Mon 09/28/2026 16:48
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Sep 2026 16:32</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Sep 2026 16:48</t>
         </is>
       </c>
     </row>
@@ -13797,7 +13797,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Sep 2026 16:32 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Sep 2026 16:48 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Mon 09/28/2026 20:27
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Sep 2026 16:48</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Sep 2026 20:27</t>
         </is>
       </c>
     </row>
@@ -13797,7 +13797,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Sep 2026 16:48 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Sep 2026 20:27 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Mon 09/28/2026 20:43
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Sep 2026 20:27</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Sep 2026 20:43</t>
         </is>
       </c>
     </row>
@@ -13797,7 +13797,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Sep 2026 20:27 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Sep 2026 20:43 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Tue 09/29/2026 10:19
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Sep 2026 20:43</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 10:19</t>
         </is>
       </c>
     </row>
@@ -805,14 +805,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 28 Sep 2026</t>
+          <t>MTD as of 29 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 28 Sep 2026</t>
+          <t>YTD as of 29 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
@@ -13797,7 +13797,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Sep 2026 20:43 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 10:19 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -13872,14 +13872,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 28 Sep 2026</t>
+          <t>MTD as of 29 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 28 Sep 2026</t>
+          <t>YTD as of 29 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>

</xml_diff>

<commit_message>
Refresh dashboard Tue 09/29/2026 10:26
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 10:19</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 10:25</t>
         </is>
       </c>
     </row>
@@ -13797,7 +13797,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 10:19 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 10:25 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Tue 09/29/2026 10:32
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 10:25</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 10:32</t>
         </is>
       </c>
     </row>
@@ -13797,7 +13797,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 10:25 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 10:32 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Tue 09/29/2026 12:15
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 10:32</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 12:15</t>
         </is>
       </c>
     </row>
@@ -13797,7 +13797,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 10:32 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 12:15 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Tue 09/29/2026 13:23
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 12:15</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 13:23</t>
         </is>
       </c>
     </row>
@@ -13797,7 +13797,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 12:15 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 13:23 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Tue 09/29/2026 14:35
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 13:23</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 14:35</t>
         </is>
       </c>
     </row>
@@ -13797,7 +13797,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 13:23 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 14:35 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Tue 09/29/2026 14:46
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 14:35</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 14:46</t>
         </is>
       </c>
     </row>
@@ -13797,7 +13797,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 14:35 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 14:46 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Tue 09/29/2026 15:28
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 14:46</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 15:28</t>
         </is>
       </c>
     </row>
@@ -13797,7 +13797,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 14:46 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 15:28 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Tue 09/29/2026 16:18
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 15:28</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 16:18</t>
         </is>
       </c>
     </row>
@@ -4336,22 +4336,22 @@
         <v>-9414012.693121692</v>
       </c>
       <c r="AD51" s="13" t="n">
-        <v>-728083558</v>
+        <v>-804381250</v>
       </c>
       <c r="AE51" s="13" t="n">
-        <v>-42828.4445882353</v>
+        <v>-47316.54411764706</v>
       </c>
       <c r="AF51" s="13" t="n">
-        <v>-3852293.957671958</v>
+        <v>-4255985.44973545</v>
       </c>
       <c r="AG51" s="13" t="n">
-        <v>-2507331957</v>
+        <v>-2583629649</v>
       </c>
       <c r="AH51" s="13" t="n">
-        <v>-147490.115117647</v>
+        <v>-151978.2146470588</v>
       </c>
       <c r="AI51" s="13" t="n">
-        <v>-13266306.65079365</v>
+        <v>-13669998.14285714</v>
       </c>
     </row>
     <row r="52">
@@ -5302,22 +5302,22 @@
         <v>-84580746.99407408</v>
       </c>
       <c r="AD63" s="15" t="n">
-        <v>-1867385778</v>
+        <v>-1943683470</v>
       </c>
       <c r="AE63" s="15" t="n">
-        <v>-109846.2222352941</v>
+        <v>-114334.3217647059</v>
       </c>
       <c r="AF63" s="15" t="n">
-        <v>-9880348.031746032</v>
+        <v>-10284039.52380952</v>
       </c>
       <c r="AG63" s="15" t="n">
-        <v>-17853146959.88</v>
+        <v>-17929444651.88</v>
       </c>
       <c r="AH63" s="15" t="n">
-        <v>-1050185.115287059</v>
+        <v>-1054673.214816471</v>
       </c>
       <c r="AI63" s="15" t="n">
-        <v>-94461095.02582011</v>
+        <v>-94864786.5178836</v>
       </c>
     </row>
     <row r="64">
@@ -7120,22 +7120,22 @@
         <v>-42218.01587301587</v>
       </c>
       <c r="AD90" s="11" t="n">
-        <v>-7427656</v>
+        <v>-187727656</v>
       </c>
       <c r="AE90" s="11" t="n">
-        <v>-436.9209411764706</v>
+        <v>-11042.80329411765</v>
       </c>
       <c r="AF90" s="11" t="n">
-        <v>-39299.7671957672</v>
+        <v>-993268.0211640212</v>
       </c>
       <c r="AG90" s="11" t="n">
-        <v>-15406861</v>
+        <v>-195706861</v>
       </c>
       <c r="AH90" s="11" t="n">
-        <v>-906.2859411764707</v>
+        <v>-11512.16829411765</v>
       </c>
       <c r="AI90" s="11" t="n">
-        <v>-81517.78306878307</v>
+        <v>-1035486.037037037</v>
       </c>
     </row>
     <row r="91">
@@ -7502,22 +7502,22 @@
         <v>-1479210.293333333</v>
       </c>
       <c r="AD94" s="15" t="n">
-        <v>-38376805</v>
+        <v>-218676805</v>
       </c>
       <c r="AE94" s="15" t="n">
-        <v>-2257.459117647059</v>
+        <v>-12863.34147058824</v>
       </c>
       <c r="AF94" s="15" t="n">
-        <v>-203051.8783068783</v>
+        <v>-1157020.132275132</v>
       </c>
       <c r="AG94" s="15" t="n">
-        <v>-317947550.44</v>
+        <v>-498247550.44</v>
       </c>
       <c r="AH94" s="15" t="n">
-        <v>-18702.79708470589</v>
+        <v>-29308.67943764706</v>
       </c>
       <c r="AI94" s="15" t="n">
-        <v>-1682262.171640211</v>
+        <v>-2636230.425608465</v>
       </c>
     </row>
     <row r="95">
@@ -11614,22 +11614,22 @@
         <v>-230275933.0393122</v>
       </c>
       <c r="AD141" s="15" t="n">
-        <v>-4242161434.27</v>
+        <v>-4422461434.27</v>
       </c>
       <c r="AE141" s="15" t="n">
-        <v>-249538.9078982353</v>
+        <v>-260144.7902511765</v>
       </c>
       <c r="AF141" s="15" t="n">
-        <v>-22445298.59402116</v>
+        <v>-23399266.84798942</v>
       </c>
       <c r="AG141" s="15" t="n">
-        <v>-47764312778.7</v>
+        <v>-47944612778.70001</v>
       </c>
       <c r="AH141" s="15" t="n">
-        <v>-2809665.457570588</v>
+        <v>-2820271.339923529</v>
       </c>
       <c r="AI141" s="15" t="n">
-        <v>-252721231.6333333</v>
+        <v>-253675199.8873016</v>
       </c>
     </row>
     <row r="142">
@@ -12814,22 +12814,22 @@
         <v>-1529478500.653757</v>
       </c>
       <c r="AD156" s="19" t="n">
-        <v>-14708699053</v>
+        <v>-14965296745</v>
       </c>
       <c r="AE156" s="19" t="n">
-        <v>-865217.5913529411</v>
+        <v>-880311.5732352941</v>
       </c>
       <c r="AF156" s="19" t="n">
-        <v>-77823804.51322751</v>
+        <v>-79181464.25925925</v>
       </c>
       <c r="AG156" s="19" t="n">
-        <v>-303780135676.5599</v>
+        <v>-304036733368.5599</v>
       </c>
       <c r="AH156" s="19" t="n">
-        <v>-17869419.74568</v>
+        <v>-17884513.72756235</v>
       </c>
       <c r="AI156" s="19" t="n">
-        <v>-1607302305.166984</v>
+        <v>-1608659964.913016</v>
       </c>
     </row>
     <row r="157">
@@ -12920,22 +12920,22 @@
         <v>-349256107.4480425</v>
       </c>
       <c r="AD157" s="19" t="n">
-        <v>1118771718</v>
+        <v>862174026</v>
       </c>
       <c r="AE157" s="19" t="n">
-        <v>65810.10105882352</v>
+        <v>50716.11917647059</v>
       </c>
       <c r="AF157" s="19" t="n">
-        <v>5919427.079365079</v>
+        <v>4561767.333333333</v>
       </c>
       <c r="AG157" s="19" t="n">
-        <v>-64890632589.68</v>
+        <v>-65147230281.68</v>
       </c>
       <c r="AH157" s="19" t="n">
-        <v>-3817096.034687059</v>
+        <v>-3832190.016569412</v>
       </c>
       <c r="AI157" s="19" t="n">
-        <v>-343336680.3686774</v>
+        <v>-344694340.1147091</v>
       </c>
     </row>
     <row r="158">
@@ -13026,22 +13026,22 @@
         <v>7747388.987724859</v>
       </c>
       <c r="AD158" s="7" t="n">
-        <v>2583028236.68</v>
+        <v>2326430544.68</v>
       </c>
       <c r="AE158" s="7" t="n">
-        <v>151942.8374517647</v>
+        <v>136848.8555694118</v>
       </c>
       <c r="AF158" s="7" t="n">
-        <v>13666816.06708995</v>
+        <v>12309156.3210582</v>
       </c>
       <c r="AG158" s="7" t="n">
-        <v>2583028236.68</v>
+        <v>2326430544.68</v>
       </c>
       <c r="AH158" s="7" t="n">
-        <v>151942.8374517647</v>
+        <v>136848.8555694118</v>
       </c>
       <c r="AI158" s="7" t="n">
-        <v>13666816.06708995</v>
+        <v>12309156.3210582</v>
       </c>
     </row>
   </sheetData>
@@ -13506,16 +13506,16 @@
         <v>1136676704</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>1196259617</v>
+        <v>1019961925</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>2332936321</v>
+        <v>2156638629</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>137231.5482941176</v>
+        <v>126861.0958235294</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>12343578.41798942</v>
+        <v>11410786.3968254</v>
       </c>
     </row>
     <row r="7">
@@ -13666,16 +13666,16 @@
         <v>112155332.96</v>
       </c>
       <c r="E11" s="13" t="n">
-        <v>35709638</v>
+        <v>-44590362</v>
       </c>
       <c r="F11" s="13" t="n">
-        <v>147864970.96</v>
+        <v>67564970.95999999</v>
       </c>
       <c r="G11" s="24" t="n">
-        <v>8697.939468235292</v>
+        <v>3974.410056470588</v>
       </c>
       <c r="H11" s="24" t="n">
-        <v>782354.3437037036</v>
+        <v>357486.6188359788</v>
       </c>
     </row>
     <row r="12">
@@ -13721,13 +13721,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>2583028238.68</v>
+        <v>2326430546.68</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>151942.8375694118</v>
+        <v>136848.8556870588</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>13666816.07767196</v>
+        <v>12309156.33164021</v>
       </c>
     </row>
   </sheetData>
@@ -13797,7 +13797,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 15:28 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 16:18 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -17403,22 +17403,22 @@
         <v>-9.414012693121693</v>
       </c>
       <c r="AD51" s="13" t="n">
-        <v>-728.083558</v>
+        <v>-804.38125</v>
       </c>
       <c r="AE51" s="13" t="n">
-        <v>-0.04282844458823529</v>
+        <v>-0.04731654411764706</v>
       </c>
       <c r="AF51" s="13" t="n">
-        <v>-3.852293957671958</v>
+        <v>-4.25598544973545</v>
       </c>
       <c r="AG51" s="13" t="n">
-        <v>-2507.331957</v>
+        <v>-2583.629649</v>
       </c>
       <c r="AH51" s="13" t="n">
-        <v>-0.1474901151176471</v>
+        <v>-0.1519782146470589</v>
       </c>
       <c r="AI51" s="13" t="n">
-        <v>-13.26630665079365</v>
+        <v>-13.66999814285714</v>
       </c>
     </row>
     <row r="52">
@@ -18369,22 +18369,22 @@
         <v>-84.58074699407408</v>
       </c>
       <c r="AD63" s="15" t="n">
-        <v>-1867.385778</v>
+        <v>-1943.68347</v>
       </c>
       <c r="AE63" s="15" t="n">
-        <v>-0.1098462222352941</v>
+        <v>-0.1143343217647059</v>
       </c>
       <c r="AF63" s="15" t="n">
-        <v>-9.880348031746031</v>
+        <v>-10.28403952380952</v>
       </c>
       <c r="AG63" s="15" t="n">
-        <v>-17853.14695988</v>
+        <v>-17929.44465188</v>
       </c>
       <c r="AH63" s="15" t="n">
-        <v>-1.050185115287059</v>
+        <v>-1.054673214816471</v>
       </c>
       <c r="AI63" s="15" t="n">
-        <v>-94.4610950258201</v>
+        <v>-94.8647865178836</v>
       </c>
     </row>
     <row r="64">
@@ -20187,22 +20187,22 @@
         <v>-0.04221801587301587</v>
       </c>
       <c r="AD90" s="11" t="n">
-        <v>-7.427656</v>
+        <v>-187.727656</v>
       </c>
       <c r="AE90" s="11" t="n">
-        <v>-0.0004369209411764706</v>
+        <v>-0.01104280329411765</v>
       </c>
       <c r="AF90" s="11" t="n">
-        <v>-0.03929976719576719</v>
+        <v>-0.9932680211640211</v>
       </c>
       <c r="AG90" s="11" t="n">
-        <v>-15.406861</v>
+        <v>-195.706861</v>
       </c>
       <c r="AH90" s="11" t="n">
-        <v>-0.0009062859411764706</v>
+        <v>-0.01151216829411765</v>
       </c>
       <c r="AI90" s="11" t="n">
-        <v>-0.08151778306878306</v>
+        <v>-1.035486037037037</v>
       </c>
     </row>
     <row r="91">
@@ -20569,22 +20569,22 @@
         <v>-1.479210293333333</v>
       </c>
       <c r="AD94" s="15" t="n">
-        <v>-38.376805</v>
+        <v>-218.676805</v>
       </c>
       <c r="AE94" s="15" t="n">
-        <v>-0.002257459117647059</v>
+        <v>-0.01286334147058824</v>
       </c>
       <c r="AF94" s="15" t="n">
-        <v>-0.2030518783068783</v>
+        <v>-1.157020132275132</v>
       </c>
       <c r="AG94" s="15" t="n">
-        <v>-317.94755044</v>
+        <v>-498.2475504400001</v>
       </c>
       <c r="AH94" s="15" t="n">
-        <v>-0.01870279708470588</v>
+        <v>-0.02930867943764706</v>
       </c>
       <c r="AI94" s="15" t="n">
-        <v>-1.682262171640212</v>
+        <v>-2.636230425608466</v>
       </c>
     </row>
     <row r="95">
@@ -24681,22 +24681,22 @@
         <v>-230.2759330393122</v>
       </c>
       <c r="AD141" s="15" t="n">
-        <v>-4242.16143427</v>
+        <v>-4422.461434270001</v>
       </c>
       <c r="AE141" s="15" t="n">
-        <v>-0.2495389078982353</v>
+        <v>-0.2601447902511765</v>
       </c>
       <c r="AF141" s="15" t="n">
-        <v>-22.44529859402117</v>
+        <v>-23.39926684798942</v>
       </c>
       <c r="AG141" s="15" t="n">
-        <v>-47764.3127787</v>
+        <v>-47944.6127787</v>
       </c>
       <c r="AH141" s="15" t="n">
-        <v>-2.809665457570588</v>
+        <v>-2.820271339923529</v>
       </c>
       <c r="AI141" s="15" t="n">
-        <v>-252.7212316333333</v>
+        <v>-253.6751998873016</v>
       </c>
     </row>
     <row r="142">
@@ -25881,22 +25881,22 @@
         <v>-1529.478500653756</v>
       </c>
       <c r="AD156" s="19" t="n">
-        <v>-14708.699053</v>
+        <v>-14965.296745</v>
       </c>
       <c r="AE156" s="19" t="n">
-        <v>-0.8652175913529412</v>
+        <v>-0.8803115732352941</v>
       </c>
       <c r="AF156" s="19" t="n">
-        <v>-77.82380451322751</v>
+        <v>-79.18146425925926</v>
       </c>
       <c r="AG156" s="19" t="n">
-        <v>-303780.1356765599</v>
+        <v>-304036.7333685599</v>
       </c>
       <c r="AH156" s="19" t="n">
-        <v>-17.86941974568</v>
+        <v>-17.88451372756235</v>
       </c>
       <c r="AI156" s="19" t="n">
-        <v>-1607.302305166984</v>
+        <v>-1608.659964913016</v>
       </c>
     </row>
     <row r="157">
@@ -25987,22 +25987,22 @@
         <v>-349.2561074480424</v>
       </c>
       <c r="AD157" s="19" t="n">
-        <v>1118.771718</v>
+        <v>862.174026</v>
       </c>
       <c r="AE157" s="19" t="n">
-        <v>0.06581010105882353</v>
+        <v>0.05071611917647059</v>
       </c>
       <c r="AF157" s="19" t="n">
-        <v>5.91942707936508</v>
+        <v>4.561767333333333</v>
       </c>
       <c r="AG157" s="19" t="n">
-        <v>-64890.63258968001</v>
+        <v>-65147.23028168001</v>
       </c>
       <c r="AH157" s="19" t="n">
-        <v>-3.81709603468706</v>
+        <v>-3.832190016569413</v>
       </c>
       <c r="AI157" s="19" t="n">
-        <v>-343.3366803686773</v>
+        <v>-344.6943401147091</v>
       </c>
     </row>
     <row r="158">
@@ -26093,22 +26093,22 @@
         <v>7.747388987724859</v>
       </c>
       <c r="AD158" s="7" t="n">
-        <v>2583.02823668</v>
+        <v>2326.43054468</v>
       </c>
       <c r="AE158" s="7" t="n">
-        <v>0.1519428374517647</v>
+        <v>0.1368488555694118</v>
       </c>
       <c r="AF158" s="7" t="n">
-        <v>13.66681606708995</v>
+        <v>12.3091563210582</v>
       </c>
       <c r="AG158" s="7" t="n">
-        <v>2583.02823668</v>
+        <v>2326.43054468</v>
       </c>
       <c r="AH158" s="7" t="n">
-        <v>0.1519428374517647</v>
+        <v>0.1368488555694118</v>
       </c>
       <c r="AI158" s="7" t="n">
-        <v>13.66681606708995</v>
+        <v>12.3091563210582</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Wed 09/30/2026 10:07
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 16:18</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 30 Sep 2026 10:07</t>
         </is>
       </c>
     </row>
@@ -805,14 +805,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 29 Sep 2026</t>
+          <t>MTD as of 30 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 29 Sep 2026</t>
+          <t>YTD as of 30 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
@@ -13797,7 +13797,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Sep 2026 16:18 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 30 Sep 2026 10:07 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -13872,14 +13872,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 29 Sep 2026</t>
+          <t>MTD as of 30 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 29 Sep 2026</t>
+          <t>YTD as of 30 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>

</xml_diff>

<commit_message>
Refresh dashboard Wed 09/30/2026 16:27
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 30 Sep 2026 10:07</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 30 Sep 2026 16:27</t>
         </is>
       </c>
     </row>
@@ -1220,22 +1220,22 @@
         <v>914323824.5555556</v>
       </c>
       <c r="AD7" s="11" t="n">
-        <v>15791239560</v>
+        <v>28574573153</v>
       </c>
       <c r="AE7" s="11" t="n">
-        <v>928896.4447058823</v>
+        <v>1680857.244294118</v>
       </c>
       <c r="AF7" s="11" t="n">
-        <v>83551532.06349206</v>
+        <v>151188217.7407407</v>
       </c>
       <c r="AG7" s="11" t="n">
-        <v>188598442401</v>
+        <v>201381775994</v>
       </c>
       <c r="AH7" s="11" t="n">
-        <v>11094026.02358824</v>
+        <v>11845986.82317647</v>
       </c>
       <c r="AI7" s="11" t="n">
-        <v>997875356.6190476</v>
+        <v>1065512042.296296</v>
       </c>
     </row>
     <row r="8">
@@ -1317,207 +1317,207 @@
     <row r="9">
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">        PT Syngenta Seed Indonesia</t>
+          <t xml:space="preserve">        PT Corteva Agriscience Seeds Indonesia</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>4917371048</v>
+        <v>14774062032</v>
       </c>
       <c r="D9" s="11" t="n">
-        <v>289257.1204705882</v>
+        <v>869062.4724705883</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>26017836.23280423</v>
-      </c>
-      <c r="F9" s="11" t="n">
-        <v>377499498</v>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>22205.85282352941</v>
-      </c>
-      <c r="H9" s="11" t="n">
-        <v>1997351.841269841</v>
-      </c>
+        <v>78169640.38095239</v>
+      </c>
+      <c r="F9" s="11" t="n"/>
+      <c r="G9" s="11" t="n"/>
+      <c r="H9" s="11" t="n"/>
       <c r="I9" s="11" t="n">
-        <v>5249034721</v>
+        <v>3060445998</v>
       </c>
       <c r="J9" s="11" t="n">
-        <v>308766.7482941176</v>
+        <v>180026.2351764706</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>27772670.48148148</v>
+        <v>16192835.96825397</v>
       </c>
       <c r="L9" s="11" t="n">
-        <v>5409395616</v>
+        <v>2647239849</v>
       </c>
       <c r="M9" s="11" t="n">
-        <v>318199.7421176471</v>
+        <v>155719.9911176471</v>
       </c>
       <c r="N9" s="11" t="n">
-        <v>28621140.82539682</v>
+        <v>14006560.04761905</v>
       </c>
       <c r="O9" s="11" t="n">
-        <v>7986730445</v>
+        <v>4342041733</v>
       </c>
       <c r="P9" s="11" t="n">
-        <v>469807.6732352941</v>
+        <v>255414.2195882353</v>
       </c>
       <c r="Q9" s="11" t="n">
-        <v>42257833.04232804</v>
+        <v>22973765.78306878</v>
       </c>
       <c r="R9" s="11" t="n">
-        <v>5293583677</v>
+        <v>2142139150</v>
       </c>
       <c r="S9" s="11" t="n">
-        <v>311387.2751176471</v>
+        <v>126008.1852941176</v>
       </c>
       <c r="T9" s="11" t="n">
-        <v>28008379.24338624</v>
+        <v>11334069.57671958</v>
       </c>
       <c r="U9" s="11" t="n">
-        <v>3590241514</v>
+        <v>4939206340</v>
       </c>
       <c r="V9" s="11" t="n">
-        <v>211190.6772941177</v>
+        <v>290541.5494117647</v>
       </c>
       <c r="W9" s="11" t="n">
-        <v>18995986.84656085</v>
+        <v>26133366.87830688</v>
       </c>
       <c r="X9" s="11" t="n">
-        <v>4753076386</v>
+        <v>2738261610</v>
       </c>
       <c r="Y9" s="11" t="n">
-        <v>279592.7285882353</v>
+        <v>161074.2123529412</v>
       </c>
       <c r="Z9" s="11" t="n">
-        <v>25148552.30687831</v>
+        <v>14488156.66666667</v>
       </c>
       <c r="AA9" s="11" t="n">
-        <v>37576932905</v>
+        <v>34643396712</v>
       </c>
       <c r="AB9" s="11" t="n">
-        <v>2210407.817941176</v>
+        <v>2037846.865411765</v>
       </c>
       <c r="AC9" s="11" t="n">
-        <v>198819750.8201058</v>
+        <v>183298395.3015873</v>
       </c>
       <c r="AD9" s="11" t="n">
-        <v>7099446001</v>
+        <v>18886221373</v>
       </c>
       <c r="AE9" s="11" t="n">
-        <v>417614.4706470588</v>
+        <v>1110954.198411765</v>
       </c>
       <c r="AF9" s="11" t="n">
-        <v>37563206.35449736</v>
+        <v>99927097.21164021</v>
       </c>
       <c r="AG9" s="11" t="n">
-        <v>44676378906</v>
+        <v>53529618085</v>
       </c>
       <c r="AH9" s="11" t="n">
-        <v>2628022.288588235</v>
+        <v>3148801.06382353</v>
       </c>
       <c r="AI9" s="11" t="n">
-        <v>236382957.1746032</v>
+        <v>283225492.5132275</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">        PT Corteva Agriscience Seeds Indonesia</t>
+          <t xml:space="preserve">        PT Syngenta Seed Indonesia</t>
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>14774062032</v>
+        <v>4917371048</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>869062.4724705883</v>
+        <v>289257.1204705882</v>
       </c>
       <c r="E10" s="13" t="n">
-        <v>78169640.38095239</v>
-      </c>
-      <c r="F10" s="13" t="n"/>
-      <c r="G10" s="13" t="n"/>
-      <c r="H10" s="13" t="n"/>
+        <v>26017836.23280423</v>
+      </c>
+      <c r="F10" s="13" t="n">
+        <v>377499498</v>
+      </c>
+      <c r="G10" s="13" t="n">
+        <v>22205.85282352941</v>
+      </c>
+      <c r="H10" s="13" t="n">
+        <v>1997351.841269841</v>
+      </c>
       <c r="I10" s="13" t="n">
-        <v>3060445998</v>
+        <v>5249034721</v>
       </c>
       <c r="J10" s="13" t="n">
-        <v>180026.2351764706</v>
+        <v>308766.7482941176</v>
       </c>
       <c r="K10" s="13" t="n">
-        <v>16192835.96825397</v>
+        <v>27772670.48148148</v>
       </c>
       <c r="L10" s="13" t="n">
-        <v>2647239849</v>
+        <v>5409395616</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>155719.9911176471</v>
+        <v>318199.7421176471</v>
       </c>
       <c r="N10" s="13" t="n">
-        <v>14006560.04761905</v>
+        <v>28621140.82539682</v>
       </c>
       <c r="O10" s="13" t="n">
-        <v>4342041733</v>
+        <v>7986730445</v>
       </c>
       <c r="P10" s="13" t="n">
-        <v>255414.2195882353</v>
+        <v>469807.6732352941</v>
       </c>
       <c r="Q10" s="13" t="n">
-        <v>22973765.78306878</v>
+        <v>42257833.04232804</v>
       </c>
       <c r="R10" s="13" t="n">
-        <v>2142139150</v>
+        <v>5293583677</v>
       </c>
       <c r="S10" s="13" t="n">
-        <v>126008.1852941176</v>
+        <v>311387.2751176471</v>
       </c>
       <c r="T10" s="13" t="n">
-        <v>11334069.57671958</v>
+        <v>28008379.24338624</v>
       </c>
       <c r="U10" s="13" t="n">
-        <v>4939206340</v>
+        <v>3590241514</v>
       </c>
       <c r="V10" s="13" t="n">
-        <v>290541.5494117647</v>
+        <v>211190.6772941177</v>
       </c>
       <c r="W10" s="13" t="n">
-        <v>26133366.87830688</v>
+        <v>18995986.84656085</v>
       </c>
       <c r="X10" s="13" t="n">
-        <v>2738261610</v>
+        <v>4753076386</v>
       </c>
       <c r="Y10" s="13" t="n">
-        <v>161074.2123529412</v>
+        <v>279592.7285882353</v>
       </c>
       <c r="Z10" s="13" t="n">
-        <v>14488156.66666667</v>
+        <v>25148552.30687831</v>
       </c>
       <c r="AA10" s="13" t="n">
-        <v>34643396712</v>
+        <v>37576932905</v>
       </c>
       <c r="AB10" s="13" t="n">
-        <v>2037846.865411765</v>
+        <v>2210407.817941176</v>
       </c>
       <c r="AC10" s="13" t="n">
-        <v>183298395.3015873</v>
+        <v>198819750.8201058</v>
       </c>
       <c r="AD10" s="13" t="n">
-        <v>6114266668</v>
+        <v>7099446001</v>
       </c>
       <c r="AE10" s="13" t="n">
-        <v>359662.7451764706</v>
+        <v>417614.4706470588</v>
       </c>
       <c r="AF10" s="13" t="n">
-        <v>32350617.29100529</v>
+        <v>37563206.35449736</v>
       </c>
       <c r="AG10" s="13" t="n">
-        <v>40757663380</v>
+        <v>44676378906</v>
       </c>
       <c r="AH10" s="13" t="n">
-        <v>2397509.610588236</v>
+        <v>2628022.288588235</v>
       </c>
       <c r="AI10" s="13" t="n">
-        <v>215649012.5925926</v>
+        <v>236382957.1746032</v>
       </c>
     </row>
     <row r="11">
@@ -1885,7 +1885,7 @@
     <row r="16">
       <c r="B16" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Kariono</t>
+          <t xml:space="preserve">        PT Shriram Genetics</t>
         </is>
       </c>
       <c r="C16" s="13" t="n"/>
@@ -1900,56 +1900,56 @@
       <c r="L16" s="13" t="n"/>
       <c r="M16" s="13" t="n"/>
       <c r="N16" s="13" t="n"/>
-      <c r="O16" s="13" t="n">
-        <v>28188000</v>
-      </c>
-      <c r="P16" s="13" t="n">
-        <v>1658.117647058823</v>
-      </c>
-      <c r="Q16" s="13" t="n">
-        <v>149142.8571428571</v>
-      </c>
+      <c r="O16" s="13" t="n"/>
+      <c r="P16" s="13" t="n"/>
+      <c r="Q16" s="13" t="n"/>
       <c r="R16" s="13" t="n"/>
       <c r="S16" s="13" t="n"/>
       <c r="T16" s="13" t="n"/>
-      <c r="U16" s="13" t="n">
-        <v>12720000</v>
-      </c>
-      <c r="V16" s="13" t="n">
-        <v>748.2352941176471</v>
-      </c>
-      <c r="W16" s="13" t="n">
-        <v>67301.58730158731</v>
-      </c>
-      <c r="X16" s="13" t="n"/>
-      <c r="Y16" s="13" t="n"/>
-      <c r="Z16" s="13" t="n"/>
+      <c r="U16" s="13" t="n"/>
+      <c r="V16" s="13" t="n"/>
+      <c r="W16" s="13" t="n"/>
+      <c r="X16" s="13" t="n">
+        <v>35440700</v>
+      </c>
+      <c r="Y16" s="13" t="n">
+        <v>2084.747058823529</v>
+      </c>
+      <c r="Z16" s="13" t="n">
+        <v>187516.9312169312</v>
+      </c>
       <c r="AA16" s="13" t="n">
-        <v>40908000</v>
+        <v>35440700</v>
       </c>
       <c r="AB16" s="13" t="n">
-        <v>2406.35294117647</v>
+        <v>2084.747058823529</v>
       </c>
       <c r="AC16" s="13" t="n">
-        <v>216444.4444444444</v>
-      </c>
-      <c r="AD16" s="13" t="n"/>
-      <c r="AE16" s="13" t="n"/>
-      <c r="AF16" s="13" t="n"/>
+        <v>187516.9312169312</v>
+      </c>
+      <c r="AD16" s="13" t="n">
+        <v>11378888</v>
+      </c>
+      <c r="AE16" s="13" t="n">
+        <v>669.3463529411765</v>
+      </c>
+      <c r="AF16" s="13" t="n">
+        <v>60205.75661375662</v>
+      </c>
       <c r="AG16" s="13" t="n">
-        <v>40908000</v>
+        <v>46819588</v>
       </c>
       <c r="AH16" s="13" t="n">
-        <v>2406.35294117647</v>
+        <v>2754.093411764706</v>
       </c>
       <c r="AI16" s="13" t="n">
-        <v>216444.4444444444</v>
+        <v>247722.6878306878</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">        PT Shriram Genetics</t>
+          <t xml:space="preserve">        Kariono</t>
         </is>
       </c>
       <c r="C17" s="11" t="n"/>
@@ -1964,44 +1964,50 @@
       <c r="L17" s="11" t="n"/>
       <c r="M17" s="11" t="n"/>
       <c r="N17" s="11" t="n"/>
-      <c r="O17" s="11" t="n"/>
-      <c r="P17" s="11" t="n"/>
-      <c r="Q17" s="11" t="n"/>
+      <c r="O17" s="11" t="n">
+        <v>28188000</v>
+      </c>
+      <c r="P17" s="11" t="n">
+        <v>1658.117647058823</v>
+      </c>
+      <c r="Q17" s="11" t="n">
+        <v>149142.8571428571</v>
+      </c>
       <c r="R17" s="11" t="n"/>
       <c r="S17" s="11" t="n"/>
       <c r="T17" s="11" t="n"/>
-      <c r="U17" s="11" t="n"/>
-      <c r="V17" s="11" t="n"/>
-      <c r="W17" s="11" t="n"/>
-      <c r="X17" s="11" t="n">
-        <v>35440700</v>
-      </c>
-      <c r="Y17" s="11" t="n">
-        <v>2084.747058823529</v>
-      </c>
-      <c r="Z17" s="11" t="n">
-        <v>187516.9312169312</v>
-      </c>
+      <c r="U17" s="11" t="n">
+        <v>12720000</v>
+      </c>
+      <c r="V17" s="11" t="n">
+        <v>748.2352941176471</v>
+      </c>
+      <c r="W17" s="11" t="n">
+        <v>67301.58730158731</v>
+      </c>
+      <c r="X17" s="11" t="n"/>
+      <c r="Y17" s="11" t="n"/>
+      <c r="Z17" s="11" t="n"/>
       <c r="AA17" s="11" t="n">
-        <v>35440700</v>
+        <v>40908000</v>
       </c>
       <c r="AB17" s="11" t="n">
-        <v>2084.747058823529</v>
+        <v>2406.35294117647</v>
       </c>
       <c r="AC17" s="11" t="n">
-        <v>187516.9312169312</v>
+        <v>216444.4444444444</v>
       </c>
       <c r="AD17" s="11" t="n"/>
       <c r="AE17" s="11" t="n"/>
       <c r="AF17" s="11" t="n"/>
       <c r="AG17" s="11" t="n">
-        <v>35440700</v>
+        <v>40908000</v>
       </c>
       <c r="AH17" s="11" t="n">
-        <v>2084.747058823529</v>
+        <v>2406.35294117647</v>
       </c>
       <c r="AI17" s="11" t="n">
-        <v>187516.9312169312</v>
+        <v>216444.4444444444</v>
       </c>
     </row>
     <row r="18">
@@ -3922,22 +3928,22 @@
         <v>1180222393.205714</v>
       </c>
       <c r="AD45" s="15" t="n">
-        <v>15827470771</v>
+        <v>28610804364</v>
       </c>
       <c r="AE45" s="15" t="n">
-        <v>931027.6924117648</v>
+        <v>1682988.492</v>
       </c>
       <c r="AF45" s="15" t="n">
-        <v>83743231.5925926</v>
+        <v>151379917.2698413</v>
       </c>
       <c r="AG45" s="15" t="n">
-        <v>238889503086.88</v>
+        <v>251672836679.88</v>
       </c>
       <c r="AH45" s="15" t="n">
-        <v>14052323.71099294</v>
+        <v>14804284.51058118</v>
       </c>
       <c r="AI45" s="15" t="n">
-        <v>1263965624.798307</v>
+        <v>1331602310.475556</v>
       </c>
     </row>
     <row r="46">
@@ -10398,22 +10404,22 @@
         <v>-5069808.166825396</v>
       </c>
       <c r="AD128" s="13" t="n">
-        <v>-334290078</v>
+        <v>-373713050</v>
       </c>
       <c r="AE128" s="13" t="n">
-        <v>-19664.12223529412</v>
+        <v>-21983.1205882353</v>
       </c>
       <c r="AF128" s="13" t="n">
-        <v>-1768730.571428571</v>
+        <v>-1977317.724867725</v>
       </c>
       <c r="AG128" s="13" t="n">
-        <v>-1292483821.53</v>
+        <v>-1331906793.53</v>
       </c>
       <c r="AH128" s="13" t="n">
-        <v>-76028.46009000001</v>
+        <v>-78347.45844294119</v>
       </c>
       <c r="AI128" s="13" t="n">
-        <v>-6838538.738253968</v>
+        <v>-7047125.891693121</v>
       </c>
     </row>
     <row r="129">
@@ -10810,22 +10816,22 @@
         <v>-132568430.7276719</v>
       </c>
       <c r="AD132" s="15" t="n">
-        <v>-1624570063</v>
+        <v>-1663993035</v>
       </c>
       <c r="AE132" s="15" t="n">
-        <v>-95562.94488235294</v>
+        <v>-97881.94323529412</v>
       </c>
       <c r="AF132" s="15" t="n">
-        <v>-8595608.798941799</v>
+        <v>-8804195.952380951</v>
       </c>
       <c r="AG132" s="15" t="n">
-        <v>-26680003470.53</v>
+        <v>-26719426442.53</v>
       </c>
       <c r="AH132" s="15" t="n">
-        <v>-1569411.968854706</v>
+        <v>-1571730.967207647</v>
       </c>
       <c r="AI132" s="15" t="n">
-        <v>-141164039.5266137</v>
+        <v>-141372626.6800529</v>
       </c>
     </row>
     <row r="133">
@@ -11614,22 +11620,22 @@
         <v>-230275933.0393122</v>
       </c>
       <c r="AD141" s="15" t="n">
-        <v>-4422461434.27</v>
+        <v>-4461884406.27</v>
       </c>
       <c r="AE141" s="15" t="n">
-        <v>-260144.7902511765</v>
+        <v>-262463.7886041177</v>
       </c>
       <c r="AF141" s="15" t="n">
-        <v>-23399266.84798942</v>
+        <v>-23607854.00142857</v>
       </c>
       <c r="AG141" s="15" t="n">
-        <v>-47944612778.70001</v>
+        <v>-47984035750.70001</v>
       </c>
       <c r="AH141" s="15" t="n">
-        <v>-2820271.339923529</v>
+        <v>-2822590.338276471</v>
       </c>
       <c r="AI141" s="15" t="n">
-        <v>-253675199.8873016</v>
+        <v>-253883787.0407407</v>
       </c>
     </row>
     <row r="142">
@@ -12549,17 +12555,23 @@
       <c r="AC153" s="11" t="n">
         <v>-4490419.042328042</v>
       </c>
-      <c r="AD153" s="11" t="n"/>
-      <c r="AE153" s="11" t="n"/>
-      <c r="AF153" s="11" t="n"/>
+      <c r="AD153" s="11" t="n">
+        <v>-99710427</v>
+      </c>
+      <c r="AE153" s="11" t="n">
+        <v>-5865.319235294118</v>
+      </c>
+      <c r="AF153" s="11" t="n">
+        <v>-527568.3968253968</v>
+      </c>
       <c r="AG153" s="11" t="n">
-        <v>-848689199</v>
+        <v>-948399626</v>
       </c>
       <c r="AH153" s="11" t="n">
-        <v>-49922.89405882353</v>
+        <v>-55788.21329411765</v>
       </c>
       <c r="AI153" s="11" t="n">
-        <v>-4490419.042328042</v>
+        <v>-5017987.439153438</v>
       </c>
     </row>
     <row r="154">
@@ -12708,22 +12720,22 @@
         <v>-31583868.07253968</v>
       </c>
       <c r="AD155" s="15" t="n">
-        <v>-183790442</v>
+        <v>-283500869</v>
       </c>
       <c r="AE155" s="15" t="n">
-        <v>-10811.20247058824</v>
+        <v>-16676.52170588235</v>
       </c>
       <c r="AF155" s="15" t="n">
-        <v>-972436.201058201</v>
+        <v>-1500004.597883598</v>
       </c>
       <c r="AG155" s="15" t="n">
-        <v>-6153141507.710001</v>
+        <v>-6252851934.710001</v>
       </c>
       <c r="AH155" s="15" t="n">
-        <v>-361949.5004535294</v>
+        <v>-367814.8196888235</v>
       </c>
       <c r="AI155" s="15" t="n">
-        <v>-32556304.27359788</v>
+        <v>-33083872.67042328</v>
       </c>
     </row>
     <row r="156">
@@ -12814,22 +12826,22 @@
         <v>-1529478500.653757</v>
       </c>
       <c r="AD156" s="19" t="n">
-        <v>-14965296745</v>
+        <v>-15104430144</v>
       </c>
       <c r="AE156" s="19" t="n">
-        <v>-880311.5732352941</v>
+        <v>-888495.8908235295</v>
       </c>
       <c r="AF156" s="19" t="n">
-        <v>-79181464.25925925</v>
+        <v>-79917619.80952381</v>
       </c>
       <c r="AG156" s="19" t="n">
-        <v>-304036733368.5599</v>
+        <v>-304175866767.5599</v>
       </c>
       <c r="AH156" s="19" t="n">
-        <v>-17884513.72756235</v>
+        <v>-17892698.04515059</v>
       </c>
       <c r="AI156" s="19" t="n">
-        <v>-1608659964.913016</v>
+        <v>-1609396120.46328</v>
       </c>
     </row>
     <row r="157">
@@ -12920,22 +12932,22 @@
         <v>-349256107.4480425</v>
       </c>
       <c r="AD157" s="19" t="n">
-        <v>862174026</v>
+        <v>13506374220</v>
       </c>
       <c r="AE157" s="19" t="n">
-        <v>50716.11917647059</v>
+        <v>794492.6011764706</v>
       </c>
       <c r="AF157" s="19" t="n">
-        <v>4561767.333333333</v>
+        <v>71462297.46031746</v>
       </c>
       <c r="AG157" s="19" t="n">
-        <v>-65147230281.68</v>
+        <v>-52503030087.68</v>
       </c>
       <c r="AH157" s="19" t="n">
-        <v>-3832190.016569412</v>
+        <v>-3088413.534569412</v>
       </c>
       <c r="AI157" s="19" t="n">
-        <v>-344694340.1147091</v>
+        <v>-277793809.987725</v>
       </c>
     </row>
     <row r="158">
@@ -13026,22 +13038,22 @@
         <v>7747388.987724859</v>
       </c>
       <c r="AD158" s="7" t="n">
-        <v>2326430544.68</v>
+        <v>14970630738.68</v>
       </c>
       <c r="AE158" s="7" t="n">
-        <v>136848.8555694118</v>
+        <v>880625.3375694117</v>
       </c>
       <c r="AF158" s="7" t="n">
-        <v>12309156.3210582</v>
+        <v>79209686.44804233</v>
       </c>
       <c r="AG158" s="7" t="n">
-        <v>2326430544.68</v>
+        <v>14970630738.68</v>
       </c>
       <c r="AH158" s="7" t="n">
-        <v>136848.8555694118</v>
+        <v>880625.3375694117</v>
       </c>
       <c r="AI158" s="7" t="n">
-        <v>12309156.3210582</v>
+        <v>79209686.44804233</v>
       </c>
     </row>
   </sheetData>
@@ -13506,16 +13518,16 @@
         <v>1136676704</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>1019961925</v>
+        <v>13692206203</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>2156638629</v>
+        <v>14828882907</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>126861.0958235294</v>
+        <v>872287.2298235294</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>11410786.3968254</v>
+        <v>78459697.92063493</v>
       </c>
     </row>
     <row r="7">
@@ -13602,16 +13614,16 @@
         <v>172976399.24</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>-123427832</v>
+        <v>-151471916</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>49548567.24000001</v>
+        <v>21504483.24000001</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>2914.621602352942</v>
+        <v>1264.969602352942</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>262161.7314285715</v>
+        <v>113780.3346031746</v>
       </c>
     </row>
     <row r="10">
@@ -13721,13 +13733,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>2326430546.68</v>
+        <v>14970630740.68</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>136848.8556870588</v>
+        <v>880625.3376870587</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>12309156.33164021</v>
+        <v>79209686.45862433</v>
       </c>
     </row>
   </sheetData>
@@ -13797,7 +13809,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 30 Sep 2026 10:07 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 30 Sep 2026 16:27 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -14287,22 +14299,22 @@
         <v>914.3238245555556</v>
       </c>
       <c r="AD7" s="11" t="n">
-        <v>15791.23956</v>
+        <v>28574.573153</v>
       </c>
       <c r="AE7" s="11" t="n">
-        <v>0.9288964447058824</v>
+        <v>1.680857244294118</v>
       </c>
       <c r="AF7" s="11" t="n">
-        <v>83.55153206349206</v>
+        <v>151.1882177407408</v>
       </c>
       <c r="AG7" s="11" t="n">
-        <v>188598.442401</v>
+        <v>201381.775994</v>
       </c>
       <c r="AH7" s="11" t="n">
-        <v>11.09402602358823</v>
+        <v>11.84598682317647</v>
       </c>
       <c r="AI7" s="11" t="n">
-        <v>997.8753566190476</v>
+        <v>1065.512042296296</v>
       </c>
     </row>
     <row r="8">
@@ -14384,207 +14396,207 @@
     <row r="9">
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">        PT Syngenta Seed Indonesia</t>
+          <t xml:space="preserve">        PT Corteva Agriscience Seeds Indonesia</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>4917.371048</v>
+        <v>14774.062032</v>
       </c>
       <c r="D9" s="11" t="n">
-        <v>0.2892571204705882</v>
+        <v>0.8690624724705882</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>26.01783623280423</v>
-      </c>
-      <c r="F9" s="11" t="n">
-        <v>377.499498</v>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>0.02220585282352941</v>
-      </c>
-      <c r="H9" s="11" t="n">
-        <v>1.997351841269841</v>
-      </c>
+        <v>78.16964038095237</v>
+      </c>
+      <c r="F9" s="11" t="n"/>
+      <c r="G9" s="11" t="n"/>
+      <c r="H9" s="11" t="n"/>
       <c r="I9" s="11" t="n">
-        <v>5249.034721</v>
+        <v>3060.445998</v>
       </c>
       <c r="J9" s="11" t="n">
-        <v>0.3087667482941177</v>
+        <v>0.1800262351764706</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>27.77267048148148</v>
+        <v>16.19283596825397</v>
       </c>
       <c r="L9" s="11" t="n">
-        <v>5409.395616</v>
+        <v>2647.239849</v>
       </c>
       <c r="M9" s="11" t="n">
-        <v>0.3181997421176471</v>
+        <v>0.1557199911176471</v>
       </c>
       <c r="N9" s="11" t="n">
-        <v>28.62114082539683</v>
+        <v>14.00656004761905</v>
       </c>
       <c r="O9" s="11" t="n">
-        <v>7986.730445</v>
+        <v>4342.041733</v>
       </c>
       <c r="P9" s="11" t="n">
-        <v>0.4698076732352941</v>
+        <v>0.2554142195882353</v>
       </c>
       <c r="Q9" s="11" t="n">
-        <v>42.25783304232804</v>
+        <v>22.97376578306878</v>
       </c>
       <c r="R9" s="11" t="n">
-        <v>5293.583677</v>
+        <v>2142.13915</v>
       </c>
       <c r="S9" s="11" t="n">
-        <v>0.311387275117647</v>
+        <v>0.1260081852941176</v>
       </c>
       <c r="T9" s="11" t="n">
-        <v>28.00837924338624</v>
+        <v>11.33406957671958</v>
       </c>
       <c r="U9" s="11" t="n">
-        <v>3590.241514</v>
+        <v>4939.20634</v>
       </c>
       <c r="V9" s="11" t="n">
-        <v>0.2111906772941176</v>
+        <v>0.2905415494117647</v>
       </c>
       <c r="W9" s="11" t="n">
-        <v>18.99598684656085</v>
+        <v>26.13336687830688</v>
       </c>
       <c r="X9" s="11" t="n">
-        <v>4753.076386</v>
+        <v>2738.26161</v>
       </c>
       <c r="Y9" s="11" t="n">
-        <v>0.2795927285882353</v>
+        <v>0.1610742123529412</v>
       </c>
       <c r="Z9" s="11" t="n">
-        <v>25.1485523068783</v>
+        <v>14.48815666666667</v>
       </c>
       <c r="AA9" s="11" t="n">
-        <v>37576.932905</v>
+        <v>34643.396712</v>
       </c>
       <c r="AB9" s="11" t="n">
-        <v>2.210407817941176</v>
+        <v>2.037846865411765</v>
       </c>
       <c r="AC9" s="11" t="n">
-        <v>198.8197508201058</v>
+        <v>183.2983953015873</v>
       </c>
       <c r="AD9" s="11" t="n">
-        <v>7099.446001</v>
+        <v>18886.221373</v>
       </c>
       <c r="AE9" s="11" t="n">
-        <v>0.4176144706470588</v>
+        <v>1.110954198411765</v>
       </c>
       <c r="AF9" s="11" t="n">
-        <v>37.56320635449735</v>
+        <v>99.92709721164022</v>
       </c>
       <c r="AG9" s="11" t="n">
-        <v>44676.378906</v>
+        <v>53529.618085</v>
       </c>
       <c r="AH9" s="11" t="n">
-        <v>2.628022288588235</v>
+        <v>3.148801063823529</v>
       </c>
       <c r="AI9" s="11" t="n">
-        <v>236.3829571746032</v>
+        <v>283.2254925132275</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">        PT Corteva Agriscience Seeds Indonesia</t>
+          <t xml:space="preserve">        PT Syngenta Seed Indonesia</t>
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>14774.062032</v>
+        <v>4917.371048</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>0.8690624724705882</v>
+        <v>0.2892571204705882</v>
       </c>
       <c r="E10" s="13" t="n">
-        <v>78.16964038095237</v>
-      </c>
-      <c r="F10" s="13" t="n"/>
-      <c r="G10" s="13" t="n"/>
-      <c r="H10" s="13" t="n"/>
+        <v>26.01783623280423</v>
+      </c>
+      <c r="F10" s="13" t="n">
+        <v>377.499498</v>
+      </c>
+      <c r="G10" s="13" t="n">
+        <v>0.02220585282352941</v>
+      </c>
+      <c r="H10" s="13" t="n">
+        <v>1.997351841269841</v>
+      </c>
       <c r="I10" s="13" t="n">
-        <v>3060.445998</v>
+        <v>5249.034721</v>
       </c>
       <c r="J10" s="13" t="n">
-        <v>0.1800262351764706</v>
+        <v>0.3087667482941177</v>
       </c>
       <c r="K10" s="13" t="n">
-        <v>16.19283596825397</v>
+        <v>27.77267048148148</v>
       </c>
       <c r="L10" s="13" t="n">
-        <v>2647.239849</v>
+        <v>5409.395616</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>0.1557199911176471</v>
+        <v>0.3181997421176471</v>
       </c>
       <c r="N10" s="13" t="n">
-        <v>14.00656004761905</v>
+        <v>28.62114082539683</v>
       </c>
       <c r="O10" s="13" t="n">
-        <v>4342.041733</v>
+        <v>7986.730445</v>
       </c>
       <c r="P10" s="13" t="n">
-        <v>0.2554142195882353</v>
+        <v>0.4698076732352941</v>
       </c>
       <c r="Q10" s="13" t="n">
-        <v>22.97376578306878</v>
+        <v>42.25783304232804</v>
       </c>
       <c r="R10" s="13" t="n">
-        <v>2142.13915</v>
+        <v>5293.583677</v>
       </c>
       <c r="S10" s="13" t="n">
-        <v>0.1260081852941176</v>
+        <v>0.311387275117647</v>
       </c>
       <c r="T10" s="13" t="n">
-        <v>11.33406957671958</v>
+        <v>28.00837924338624</v>
       </c>
       <c r="U10" s="13" t="n">
-        <v>4939.20634</v>
+        <v>3590.241514</v>
       </c>
       <c r="V10" s="13" t="n">
-        <v>0.2905415494117647</v>
+        <v>0.2111906772941176</v>
       </c>
       <c r="W10" s="13" t="n">
-        <v>26.13336687830688</v>
+        <v>18.99598684656085</v>
       </c>
       <c r="X10" s="13" t="n">
-        <v>2738.26161</v>
+        <v>4753.076386</v>
       </c>
       <c r="Y10" s="13" t="n">
-        <v>0.1610742123529412</v>
+        <v>0.2795927285882353</v>
       </c>
       <c r="Z10" s="13" t="n">
-        <v>14.48815666666667</v>
+        <v>25.1485523068783</v>
       </c>
       <c r="AA10" s="13" t="n">
-        <v>34643.396712</v>
+        <v>37576.932905</v>
       </c>
       <c r="AB10" s="13" t="n">
-        <v>2.037846865411765</v>
+        <v>2.210407817941176</v>
       </c>
       <c r="AC10" s="13" t="n">
-        <v>183.2983953015873</v>
+        <v>198.8197508201058</v>
       </c>
       <c r="AD10" s="13" t="n">
-        <v>6114.266668</v>
+        <v>7099.446001</v>
       </c>
       <c r="AE10" s="13" t="n">
-        <v>0.3596627451764706</v>
+        <v>0.4176144706470588</v>
       </c>
       <c r="AF10" s="13" t="n">
-        <v>32.35061729100529</v>
+        <v>37.56320635449735</v>
       </c>
       <c r="AG10" s="13" t="n">
-        <v>40757.66338</v>
+        <v>44676.378906</v>
       </c>
       <c r="AH10" s="13" t="n">
-        <v>2.397509610588235</v>
+        <v>2.628022288588235</v>
       </c>
       <c r="AI10" s="13" t="n">
-        <v>215.6490125925926</v>
+        <v>236.3829571746032</v>
       </c>
     </row>
     <row r="11">
@@ -14952,7 +14964,7 @@
     <row r="16">
       <c r="B16" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Kariono</t>
+          <t xml:space="preserve">        PT Shriram Genetics</t>
         </is>
       </c>
       <c r="C16" s="13" t="n"/>
@@ -14967,56 +14979,56 @@
       <c r="L16" s="13" t="n"/>
       <c r="M16" s="13" t="n"/>
       <c r="N16" s="13" t="n"/>
-      <c r="O16" s="13" t="n">
-        <v>28.188</v>
-      </c>
-      <c r="P16" s="13" t="n">
-        <v>0.001658117647058823</v>
-      </c>
-      <c r="Q16" s="13" t="n">
-        <v>0.1491428571428571</v>
-      </c>
+      <c r="O16" s="13" t="n"/>
+      <c r="P16" s="13" t="n"/>
+      <c r="Q16" s="13" t="n"/>
       <c r="R16" s="13" t="n"/>
       <c r="S16" s="13" t="n"/>
       <c r="T16" s="13" t="n"/>
-      <c r="U16" s="13" t="n">
-        <v>12.72</v>
-      </c>
-      <c r="V16" s="13" t="n">
-        <v>0.0007482352941176471</v>
-      </c>
-      <c r="W16" s="13" t="n">
-        <v>0.06730158730158731</v>
-      </c>
-      <c r="X16" s="13" t="n"/>
-      <c r="Y16" s="13" t="n"/>
-      <c r="Z16" s="13" t="n"/>
+      <c r="U16" s="13" t="n"/>
+      <c r="V16" s="13" t="n"/>
+      <c r="W16" s="13" t="n"/>
+      <c r="X16" s="13" t="n">
+        <v>35.4407</v>
+      </c>
+      <c r="Y16" s="13" t="n">
+        <v>0.002084747058823529</v>
+      </c>
+      <c r="Z16" s="13" t="n">
+        <v>0.1875169312169312</v>
+      </c>
       <c r="AA16" s="13" t="n">
-        <v>40.908</v>
+        <v>35.4407</v>
       </c>
       <c r="AB16" s="13" t="n">
-        <v>0.002406352941176471</v>
+        <v>0.002084747058823529</v>
       </c>
       <c r="AC16" s="13" t="n">
-        <v>0.2164444444444444</v>
-      </c>
-      <c r="AD16" s="13" t="n"/>
-      <c r="AE16" s="13" t="n"/>
-      <c r="AF16" s="13" t="n"/>
+        <v>0.1875169312169312</v>
+      </c>
+      <c r="AD16" s="13" t="n">
+        <v>11.378888</v>
+      </c>
+      <c r="AE16" s="13" t="n">
+        <v>0.0006693463529411764</v>
+      </c>
+      <c r="AF16" s="13" t="n">
+        <v>0.06020575661375661</v>
+      </c>
       <c r="AG16" s="13" t="n">
-        <v>40.908</v>
+        <v>46.819588</v>
       </c>
       <c r="AH16" s="13" t="n">
-        <v>0.002406352941176471</v>
+        <v>0.002754093411764706</v>
       </c>
       <c r="AI16" s="13" t="n">
-        <v>0.2164444444444444</v>
+        <v>0.2477226878306878</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">        PT Shriram Genetics</t>
+          <t xml:space="preserve">        Kariono</t>
         </is>
       </c>
       <c r="C17" s="11" t="n"/>
@@ -15031,44 +15043,50 @@
       <c r="L17" s="11" t="n"/>
       <c r="M17" s="11" t="n"/>
       <c r="N17" s="11" t="n"/>
-      <c r="O17" s="11" t="n"/>
-      <c r="P17" s="11" t="n"/>
-      <c r="Q17" s="11" t="n"/>
+      <c r="O17" s="11" t="n">
+        <v>28.188</v>
+      </c>
+      <c r="P17" s="11" t="n">
+        <v>0.001658117647058823</v>
+      </c>
+      <c r="Q17" s="11" t="n">
+        <v>0.1491428571428571</v>
+      </c>
       <c r="R17" s="11" t="n"/>
       <c r="S17" s="11" t="n"/>
       <c r="T17" s="11" t="n"/>
-      <c r="U17" s="11" t="n"/>
-      <c r="V17" s="11" t="n"/>
-      <c r="W17" s="11" t="n"/>
-      <c r="X17" s="11" t="n">
-        <v>35.4407</v>
-      </c>
-      <c r="Y17" s="11" t="n">
-        <v>0.002084747058823529</v>
-      </c>
-      <c r="Z17" s="11" t="n">
-        <v>0.1875169312169312</v>
-      </c>
+      <c r="U17" s="11" t="n">
+        <v>12.72</v>
+      </c>
+      <c r="V17" s="11" t="n">
+        <v>0.0007482352941176471</v>
+      </c>
+      <c r="W17" s="11" t="n">
+        <v>0.06730158730158731</v>
+      </c>
+      <c r="X17" s="11" t="n"/>
+      <c r="Y17" s="11" t="n"/>
+      <c r="Z17" s="11" t="n"/>
       <c r="AA17" s="11" t="n">
-        <v>35.4407</v>
+        <v>40.908</v>
       </c>
       <c r="AB17" s="11" t="n">
-        <v>0.002084747058823529</v>
+        <v>0.002406352941176471</v>
       </c>
       <c r="AC17" s="11" t="n">
-        <v>0.1875169312169312</v>
+        <v>0.2164444444444444</v>
       </c>
       <c r="AD17" s="11" t="n"/>
       <c r="AE17" s="11" t="n"/>
       <c r="AF17" s="11" t="n"/>
       <c r="AG17" s="11" t="n">
-        <v>35.4407</v>
+        <v>40.908</v>
       </c>
       <c r="AH17" s="11" t="n">
-        <v>0.002084747058823529</v>
+        <v>0.002406352941176471</v>
       </c>
       <c r="AI17" s="11" t="n">
-        <v>0.1875169312169312</v>
+        <v>0.2164444444444444</v>
       </c>
     </row>
     <row r="18">
@@ -16989,22 +17007,22 @@
         <v>1180.222393205714</v>
       </c>
       <c r="AD45" s="15" t="n">
-        <v>15827.470771</v>
+        <v>28610.804364</v>
       </c>
       <c r="AE45" s="15" t="n">
-        <v>0.9310276924117648</v>
+        <v>1.682988492</v>
       </c>
       <c r="AF45" s="15" t="n">
-        <v>83.74323159259259</v>
+        <v>151.3799172698413</v>
       </c>
       <c r="AG45" s="15" t="n">
-        <v>238889.50308688</v>
+        <v>251672.83667988</v>
       </c>
       <c r="AH45" s="15" t="n">
-        <v>14.05232371099294</v>
+        <v>14.80428451058117</v>
       </c>
       <c r="AI45" s="15" t="n">
-        <v>1263.965624798307</v>
+        <v>1331.602310475555</v>
       </c>
     </row>
     <row r="46">
@@ -23465,22 +23483,22 @@
         <v>-5.069808166825397</v>
       </c>
       <c r="AD128" s="13" t="n">
-        <v>-334.290078</v>
+        <v>-373.71305</v>
       </c>
       <c r="AE128" s="13" t="n">
-        <v>-0.01966412223529412</v>
+        <v>-0.0219831205882353</v>
       </c>
       <c r="AF128" s="13" t="n">
-        <v>-1.768730571428571</v>
+        <v>-1.977317724867725</v>
       </c>
       <c r="AG128" s="13" t="n">
-        <v>-1292.48382153</v>
+        <v>-1331.90679353</v>
       </c>
       <c r="AH128" s="13" t="n">
-        <v>-0.07602846009</v>
+        <v>-0.07834745844294118</v>
       </c>
       <c r="AI128" s="13" t="n">
-        <v>-6.838538738253969</v>
+        <v>-7.047125891693122</v>
       </c>
     </row>
     <row r="129">
@@ -23877,22 +23895,22 @@
         <v>-132.568430727672</v>
       </c>
       <c r="AD132" s="15" t="n">
-        <v>-1624.570063</v>
+        <v>-1663.993035</v>
       </c>
       <c r="AE132" s="15" t="n">
-        <v>-0.09556294488235294</v>
+        <v>-0.09788194323529412</v>
       </c>
       <c r="AF132" s="15" t="n">
-        <v>-8.595608798941798</v>
+        <v>-8.804195952380953</v>
       </c>
       <c r="AG132" s="15" t="n">
-        <v>-26680.00347053</v>
+        <v>-26719.42644253</v>
       </c>
       <c r="AH132" s="15" t="n">
-        <v>-1.569411968854706</v>
+        <v>-1.571730967207647</v>
       </c>
       <c r="AI132" s="15" t="n">
-        <v>-141.1640395266138</v>
+        <v>-141.3726266800529</v>
       </c>
     </row>
     <row r="133">
@@ -24681,22 +24699,22 @@
         <v>-230.2759330393122</v>
       </c>
       <c r="AD141" s="15" t="n">
-        <v>-4422.461434270001</v>
+        <v>-4461.884406270001</v>
       </c>
       <c r="AE141" s="15" t="n">
-        <v>-0.2601447902511765</v>
+        <v>-0.2624637886041177</v>
       </c>
       <c r="AF141" s="15" t="n">
-        <v>-23.39926684798942</v>
+        <v>-23.60785400142858</v>
       </c>
       <c r="AG141" s="15" t="n">
-        <v>-47944.6127787</v>
+        <v>-47984.0357507</v>
       </c>
       <c r="AH141" s="15" t="n">
-        <v>-2.820271339923529</v>
+        <v>-2.82259033827647</v>
       </c>
       <c r="AI141" s="15" t="n">
-        <v>-253.6751998873016</v>
+        <v>-253.8837870407407</v>
       </c>
     </row>
     <row r="142">
@@ -25616,17 +25634,23 @@
       <c r="AC153" s="11" t="n">
         <v>-4.490419042328043</v>
       </c>
-      <c r="AD153" s="11" t="n"/>
-      <c r="AE153" s="11" t="n"/>
-      <c r="AF153" s="11" t="n"/>
+      <c r="AD153" s="11" t="n">
+        <v>-99.710427</v>
+      </c>
+      <c r="AE153" s="11" t="n">
+        <v>-0.005865319235294117</v>
+      </c>
+      <c r="AF153" s="11" t="n">
+        <v>-0.5275683968253968</v>
+      </c>
       <c r="AG153" s="11" t="n">
-        <v>-848.6891990000001</v>
+        <v>-948.3996260000001</v>
       </c>
       <c r="AH153" s="11" t="n">
-        <v>-0.04992289405882353</v>
+        <v>-0.05578821329411765</v>
       </c>
       <c r="AI153" s="11" t="n">
-        <v>-4.490419042328043</v>
+        <v>-5.01798743915344</v>
       </c>
     </row>
     <row r="154">
@@ -25775,22 +25799,22 @@
         <v>-31.58386807253968</v>
       </c>
       <c r="AD155" s="15" t="n">
-        <v>-183.790442</v>
+        <v>-283.500869</v>
       </c>
       <c r="AE155" s="15" t="n">
-        <v>-0.01081120247058824</v>
+        <v>-0.01667652170588236</v>
       </c>
       <c r="AF155" s="15" t="n">
-        <v>-0.9724362010582012</v>
+        <v>-1.500004597883598</v>
       </c>
       <c r="AG155" s="15" t="n">
-        <v>-6153.141507710001</v>
+        <v>-6252.851934710001</v>
       </c>
       <c r="AH155" s="15" t="n">
-        <v>-0.3619495004535295</v>
+        <v>-0.3678148196888236</v>
       </c>
       <c r="AI155" s="15" t="n">
-        <v>-32.55630427359788</v>
+        <v>-33.08387267042328</v>
       </c>
     </row>
     <row r="156">
@@ -25881,22 +25905,22 @@
         <v>-1529.478500653756</v>
       </c>
       <c r="AD156" s="19" t="n">
-        <v>-14965.296745</v>
+        <v>-15104.430144</v>
       </c>
       <c r="AE156" s="19" t="n">
-        <v>-0.8803115732352941</v>
+        <v>-0.8884958908235294</v>
       </c>
       <c r="AF156" s="19" t="n">
-        <v>-79.18146425925926</v>
+        <v>-79.91761980952381</v>
       </c>
       <c r="AG156" s="19" t="n">
-        <v>-304036.7333685599</v>
+        <v>-304175.8667675599</v>
       </c>
       <c r="AH156" s="19" t="n">
-        <v>-17.88451372756235</v>
+        <v>-17.89269804515059</v>
       </c>
       <c r="AI156" s="19" t="n">
-        <v>-1608.659964913016</v>
+        <v>-1609.39612046328</v>
       </c>
     </row>
     <row r="157">
@@ -25987,22 +26011,22 @@
         <v>-349.2561074480424</v>
       </c>
       <c r="AD157" s="19" t="n">
-        <v>862.174026</v>
+        <v>13506.37422</v>
       </c>
       <c r="AE157" s="19" t="n">
-        <v>0.05071611917647059</v>
+        <v>0.7944926011764706</v>
       </c>
       <c r="AF157" s="19" t="n">
-        <v>4.561767333333333</v>
+        <v>71.46229746031746</v>
       </c>
       <c r="AG157" s="19" t="n">
-        <v>-65147.23028168001</v>
+        <v>-52503.03008768002</v>
       </c>
       <c r="AH157" s="19" t="n">
-        <v>-3.832190016569413</v>
+        <v>-3.088413534569413</v>
       </c>
       <c r="AI157" s="19" t="n">
-        <v>-344.6943401147091</v>
+        <v>-277.793809987725</v>
       </c>
     </row>
     <row r="158">
@@ -26093,22 +26117,22 @@
         <v>7.747388987724859</v>
       </c>
       <c r="AD158" s="7" t="n">
-        <v>2326.43054468</v>
+        <v>14970.63073868</v>
       </c>
       <c r="AE158" s="7" t="n">
-        <v>0.1368488555694118</v>
+        <v>0.8806253375694117</v>
       </c>
       <c r="AF158" s="7" t="n">
-        <v>12.3091563210582</v>
+        <v>79.20968644804233</v>
       </c>
       <c r="AG158" s="7" t="n">
-        <v>2326.43054468</v>
+        <v>14970.63073868</v>
       </c>
       <c r="AH158" s="7" t="n">
-        <v>0.1368488555694118</v>
+        <v>0.8806253375694117</v>
       </c>
       <c r="AI158" s="7" t="n">
-        <v>12.3091563210582</v>
+        <v>79.20968644804233</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Fri 10/02/2026 17:26
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -734,7 +734,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 01 Oct 2026 20:32</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 02 Oct 2026 17:26</t>
         </is>
       </c>
     </row>
@@ -816,14 +816,14 @@
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 01 Oct 2026</t>
+          <t>MTD as of 02 Oct 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
       <c r="AI3" s="4" t="n"/>
       <c r="AJ3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 01 Oct 2026</t>
+          <t>YTD as of 02 Oct 2026</t>
         </is>
       </c>
       <c r="AK3" s="4" t="n"/>
@@ -1266,17 +1266,23 @@
       <c r="AF7" s="11" t="n">
         <v>1066081968.222222</v>
       </c>
-      <c r="AG7" s="11" t="n"/>
-      <c r="AH7" s="11" t="n"/>
-      <c r="AI7" s="11" t="n"/>
+      <c r="AG7" s="11" t="n">
+        <v>1739093256</v>
+      </c>
+      <c r="AH7" s="11" t="n">
+        <v>102299.6032941177</v>
+      </c>
+      <c r="AI7" s="11" t="n">
+        <v>9201551.619047619</v>
+      </c>
       <c r="AJ7" s="11" t="n">
-        <v>201489491994</v>
+        <v>203228585250</v>
       </c>
       <c r="AK7" s="11" t="n">
-        <v>11852323.05847059</v>
+        <v>11954622.66176471</v>
       </c>
       <c r="AL7" s="11" t="n">
-        <v>1066081968.222222</v>
+        <v>1075283519.84127</v>
       </c>
     </row>
     <row r="8">
@@ -1448,17 +1454,23 @@
       <c r="AF9" s="11" t="n">
         <v>283225492.5132275</v>
       </c>
-      <c r="AG9" s="11" t="n"/>
-      <c r="AH9" s="11" t="n"/>
-      <c r="AI9" s="11" t="n"/>
+      <c r="AG9" s="11" t="n">
+        <v>1739093256</v>
+      </c>
+      <c r="AH9" s="11" t="n">
+        <v>102299.6032941177</v>
+      </c>
+      <c r="AI9" s="11" t="n">
+        <v>9201551.619047619</v>
+      </c>
       <c r="AJ9" s="11" t="n">
-        <v>53529618085</v>
+        <v>55268711341</v>
       </c>
       <c r="AK9" s="11" t="n">
-        <v>3148801.06382353</v>
+        <v>3251100.667117647</v>
       </c>
       <c r="AL9" s="11" t="n">
-        <v>283225492.5132275</v>
+        <v>292427044.1322751</v>
       </c>
     </row>
     <row r="10">
@@ -2306,22 +2318,22 @@
         <v>2521134.965502645</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>623000</v>
+        <v>1529500</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>36.64705882352941</v>
+        <v>89.97058823529412</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>3296.296296296296</v>
+        <v>8092.592592592592</v>
       </c>
       <c r="AJ20" s="13" t="n">
-        <v>477117508.48</v>
+        <v>478024008.48</v>
       </c>
       <c r="AK20" s="13" t="n">
-        <v>28065.73579294118</v>
+        <v>28119.05932235294</v>
       </c>
       <c r="AL20" s="13" t="n">
-        <v>2524431.261798942</v>
+        <v>2529227.558095238</v>
       </c>
     </row>
     <row r="21">
@@ -2579,22 +2591,22 @@
         <v>491976.1904761905</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>623000</v>
+        <v>1529500</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>36.64705882352941</v>
+        <v>89.97058823529412</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>3296.296296296296</v>
+        <v>8092.592592592592</v>
       </c>
       <c r="AJ23" s="11" t="n">
-        <v>93606500</v>
+        <v>94513000</v>
       </c>
       <c r="AK23" s="11" t="n">
-        <v>5506.264705882353</v>
+        <v>5559.588235294117</v>
       </c>
       <c r="AL23" s="11" t="n">
-        <v>495272.4867724868</v>
+        <v>500068.7830687831</v>
       </c>
     </row>
     <row r="24">
@@ -4119,22 +4131,22 @@
         <v>1332179822.764445</v>
       </c>
       <c r="AG45" s="15" t="n">
-        <v>623000</v>
+        <v>1740622756</v>
       </c>
       <c r="AH45" s="15" t="n">
-        <v>36.64705882352941</v>
+        <v>102389.5738823529</v>
       </c>
       <c r="AI45" s="15" t="n">
-        <v>3296.296296296296</v>
+        <v>9209644.211640211</v>
       </c>
       <c r="AJ45" s="15" t="n">
-        <v>251782609502.48</v>
+        <v>253522609258.48</v>
       </c>
       <c r="AK45" s="15" t="n">
-        <v>14810741.73544</v>
+        <v>14913094.66226353</v>
       </c>
       <c r="AL45" s="15" t="n">
-        <v>1332183119.060741</v>
+        <v>1341389466.976085</v>
       </c>
     </row>
     <row r="46">
@@ -6680,17 +6692,23 @@
       <c r="AF81" s="11" t="n">
         <v>-52843398.14285713</v>
       </c>
-      <c r="AG81" s="11" t="n"/>
-      <c r="AH81" s="11" t="n"/>
-      <c r="AI81" s="11" t="n"/>
+      <c r="AG81" s="11" t="n">
+        <v>-870978933</v>
+      </c>
+      <c r="AH81" s="11" t="n">
+        <v>-51234.05488235294</v>
+      </c>
+      <c r="AI81" s="11" t="n">
+        <v>-4608354.142857143</v>
+      </c>
       <c r="AJ81" s="11" t="n">
-        <v>-9987402249</v>
+        <v>-10858381182</v>
       </c>
       <c r="AK81" s="11" t="n">
-        <v>-587494.2499411764</v>
+        <v>-638728.3048235293</v>
       </c>
       <c r="AL81" s="11" t="n">
-        <v>-52843398.14285713</v>
+        <v>-57451752.28571428</v>
       </c>
     </row>
     <row r="82">
@@ -6789,17 +6807,23 @@
       <c r="AF82" s="13" t="n">
         <v>-58934229.3347619</v>
       </c>
-      <c r="AG82" s="13" t="n"/>
-      <c r="AH82" s="13" t="n"/>
-      <c r="AI82" s="13" t="n"/>
+      <c r="AG82" s="13" t="n">
+        <v>-897917960</v>
+      </c>
+      <c r="AH82" s="13" t="n">
+        <v>-52818.70352941177</v>
+      </c>
+      <c r="AI82" s="13" t="n">
+        <v>-4750888.677248677</v>
+      </c>
       <c r="AJ82" s="13" t="n">
-        <v>-11138569344.27</v>
+        <v>-12036487304.27</v>
       </c>
       <c r="AK82" s="13" t="n">
-        <v>-655209.961427647</v>
+        <v>-708028.6649570588</v>
       </c>
       <c r="AL82" s="13" t="n">
-        <v>-58934229.3347619</v>
+        <v>-63685118.01201058</v>
       </c>
     </row>
     <row r="83">
@@ -7007,17 +7031,23 @@
       <c r="AF84" s="13" t="n">
         <v>-2427178.873015873</v>
       </c>
-      <c r="AG84" s="13" t="n"/>
-      <c r="AH84" s="13" t="n"/>
-      <c r="AI84" s="13" t="n"/>
+      <c r="AG84" s="13" t="n">
+        <v>-800000</v>
+      </c>
+      <c r="AH84" s="13" t="n">
+        <v>-47.05882352941177</v>
+      </c>
+      <c r="AI84" s="13" t="n">
+        <v>-4232.804232804233</v>
+      </c>
       <c r="AJ84" s="13" t="n">
-        <v>-458736807</v>
+        <v>-459536807</v>
       </c>
       <c r="AK84" s="13" t="n">
-        <v>-26984.51805882353</v>
+        <v>-27031.57688235295</v>
       </c>
       <c r="AL84" s="13" t="n">
-        <v>-2427178.873015873</v>
+        <v>-2431411.677248677</v>
       </c>
     </row>
     <row r="85">
@@ -7116,17 +7146,23 @@
       <c r="AF85" s="15" t="n">
         <v>-170301306.3770899</v>
       </c>
-      <c r="AG85" s="15" t="n"/>
-      <c r="AH85" s="15" t="n"/>
-      <c r="AI85" s="15" t="n"/>
+      <c r="AG85" s="15" t="n">
+        <v>-1769696893</v>
+      </c>
+      <c r="AH85" s="15" t="n">
+        <v>-104099.8172352941</v>
+      </c>
+      <c r="AI85" s="15" t="n">
+        <v>-9363475.624338625</v>
+      </c>
       <c r="AJ85" s="15" t="n">
-        <v>-32186946905.27</v>
+        <v>-33956643798.27</v>
       </c>
       <c r="AK85" s="15" t="n">
-        <v>-1893349.817957059</v>
+        <v>-1997449.635192353</v>
       </c>
       <c r="AL85" s="15" t="n">
-        <v>-170301306.3770899</v>
+        <v>-179664782.0014286</v>
       </c>
     </row>
     <row r="86">
@@ -7311,17 +7347,23 @@
       <c r="AF88" s="11" t="n">
         <v>-778818.2539682541</v>
       </c>
-      <c r="AG88" s="11" t="n"/>
-      <c r="AH88" s="11" t="n"/>
-      <c r="AI88" s="11" t="n"/>
+      <c r="AG88" s="11" t="n">
+        <v>-294372</v>
+      </c>
+      <c r="AH88" s="11" t="n">
+        <v>-17.316</v>
+      </c>
+      <c r="AI88" s="11" t="n">
+        <v>-1557.52380952381</v>
+      </c>
       <c r="AJ88" s="11" t="n">
-        <v>-147196650</v>
+        <v>-147491022</v>
       </c>
       <c r="AK88" s="11" t="n">
-        <v>-8658.626470588237</v>
+        <v>-8675.942470588237</v>
       </c>
       <c r="AL88" s="11" t="n">
-        <v>-778818.2539682541</v>
+        <v>-780375.7777777779</v>
       </c>
     </row>
     <row r="89">
@@ -7372,17 +7414,23 @@
       <c r="AF89" s="13" t="n">
         <v>-13897.3544973545</v>
       </c>
-      <c r="AG89" s="13" t="n"/>
-      <c r="AH89" s="13" t="n"/>
-      <c r="AI89" s="13" t="n"/>
+      <c r="AG89" s="13" t="n">
+        <v>-772500</v>
+      </c>
+      <c r="AH89" s="13" t="n">
+        <v>-45.44117647058823</v>
+      </c>
+      <c r="AI89" s="13" t="n">
+        <v>-4087.301587301587</v>
+      </c>
       <c r="AJ89" s="13" t="n">
-        <v>-2626600</v>
+        <v>-3399100</v>
       </c>
       <c r="AK89" s="13" t="n">
-        <v>-154.5058823529412</v>
+        <v>-199.9470588235294</v>
       </c>
       <c r="AL89" s="13" t="n">
-        <v>-13897.3544973545</v>
+        <v>-17984.65608465609</v>
       </c>
     </row>
     <row r="90">
@@ -7645,17 +7693,23 @@
       <c r="AF92" s="11" t="n">
         <v>-786410.9841269841</v>
       </c>
-      <c r="AG92" s="11" t="n"/>
-      <c r="AH92" s="11" t="n"/>
-      <c r="AI92" s="11" t="n"/>
+      <c r="AG92" s="11" t="n">
+        <v>-1078200</v>
+      </c>
+      <c r="AH92" s="11" t="n">
+        <v>-63.4235294117647</v>
+      </c>
+      <c r="AI92" s="11" t="n">
+        <v>-5704.761904761905</v>
+      </c>
       <c r="AJ92" s="11" t="n">
-        <v>-148631676</v>
+        <v>-149709876</v>
       </c>
       <c r="AK92" s="11" t="n">
-        <v>-8743.039764705882</v>
+        <v>-8806.463294117646</v>
       </c>
       <c r="AL92" s="11" t="n">
-        <v>-786410.9841269841</v>
+        <v>-792115.746031746</v>
       </c>
     </row>
     <row r="93">
@@ -7851,17 +7905,23 @@
       <c r="AF94" s="15" t="n">
         <v>-2636230.425608465</v>
       </c>
-      <c r="AG94" s="15" t="n"/>
-      <c r="AH94" s="15" t="n"/>
-      <c r="AI94" s="15" t="n"/>
+      <c r="AG94" s="15" t="n">
+        <v>-2145072</v>
+      </c>
+      <c r="AH94" s="15" t="n">
+        <v>-126.1807058823529</v>
+      </c>
+      <c r="AI94" s="15" t="n">
+        <v>-11349.5873015873</v>
+      </c>
       <c r="AJ94" s="15" t="n">
-        <v>-498247550.44</v>
+        <v>-500392622.44</v>
       </c>
       <c r="AK94" s="15" t="n">
-        <v>-29308.67943764706</v>
+        <v>-29434.86014352941</v>
       </c>
       <c r="AL94" s="15" t="n">
-        <v>-2636230.425608465</v>
+        <v>-2647580.012910053</v>
       </c>
     </row>
     <row r="95">
@@ -8040,17 +8100,23 @@
       <c r="AF97" s="13" t="n">
         <v>-471451.3227513228</v>
       </c>
-      <c r="AG97" s="13" t="n"/>
-      <c r="AH97" s="13" t="n"/>
-      <c r="AI97" s="13" t="n"/>
+      <c r="AG97" s="13" t="n">
+        <v>-531541</v>
+      </c>
+      <c r="AH97" s="13" t="n">
+        <v>-31.26711764705883</v>
+      </c>
+      <c r="AI97" s="13" t="n">
+        <v>-2812.386243386243</v>
+      </c>
       <c r="AJ97" s="13" t="n">
-        <v>-89104300</v>
+        <v>-89635841</v>
       </c>
       <c r="AK97" s="13" t="n">
-        <v>-5241.429411764706</v>
+        <v>-5272.696529411764</v>
       </c>
       <c r="AL97" s="13" t="n">
-        <v>-471451.3227513228</v>
+        <v>-474263.708994709</v>
       </c>
     </row>
     <row r="98">
@@ -8149,17 +8215,23 @@
       <c r="AF98" s="11" t="n">
         <v>-1418156.079365079</v>
       </c>
-      <c r="AG98" s="11" t="n"/>
-      <c r="AH98" s="11" t="n"/>
-      <c r="AI98" s="11" t="n"/>
+      <c r="AG98" s="11" t="n">
+        <v>-1248500</v>
+      </c>
+      <c r="AH98" s="11" t="n">
+        <v>-73.44117647058823</v>
+      </c>
+      <c r="AI98" s="11" t="n">
+        <v>-6605.820105820106</v>
+      </c>
       <c r="AJ98" s="11" t="n">
-        <v>-268031499</v>
+        <v>-269279999</v>
       </c>
       <c r="AK98" s="11" t="n">
-        <v>-15766.55876470588</v>
+        <v>-15839.99994117647</v>
       </c>
       <c r="AL98" s="11" t="n">
-        <v>-1418156.079365079</v>
+        <v>-1424761.899470899</v>
       </c>
     </row>
     <row r="99">
@@ -8258,17 +8330,23 @@
       <c r="AF99" s="13" t="n">
         <v>-40893236.55941799</v>
       </c>
-      <c r="AG99" s="13" t="n"/>
-      <c r="AH99" s="13" t="n"/>
-      <c r="AI99" s="13" t="n"/>
+      <c r="AG99" s="13" t="n">
+        <v>-82401009</v>
+      </c>
+      <c r="AH99" s="13" t="n">
+        <v>-4847.118176470588</v>
+      </c>
+      <c r="AI99" s="13" t="n">
+        <v>-435984.1746031746</v>
+      </c>
       <c r="AJ99" s="13" t="n">
-        <v>-7728821709.73</v>
+        <v>-7811222718.73</v>
       </c>
       <c r="AK99" s="13" t="n">
-        <v>-454636.5711605883</v>
+        <v>-459483.6893370589</v>
       </c>
       <c r="AL99" s="13" t="n">
-        <v>-40893236.55941799</v>
+        <v>-41329220.73402116</v>
       </c>
     </row>
     <row r="100">
@@ -8476,17 +8554,23 @@
       <c r="AF101" s="13" t="n">
         <v>-1927101.095238095</v>
       </c>
-      <c r="AG101" s="13" t="n"/>
-      <c r="AH101" s="13" t="n"/>
-      <c r="AI101" s="13" t="n"/>
+      <c r="AG101" s="13" t="n">
+        <v>-1109400</v>
+      </c>
+      <c r="AH101" s="13" t="n">
+        <v>-65.25882352941177</v>
+      </c>
+      <c r="AI101" s="13" t="n">
+        <v>-5869.841269841269</v>
+      </c>
       <c r="AJ101" s="13" t="n">
-        <v>-364222107</v>
+        <v>-365331507</v>
       </c>
       <c r="AK101" s="13" t="n">
-        <v>-21424.82982352941</v>
+        <v>-21490.08864705882</v>
       </c>
       <c r="AL101" s="13" t="n">
-        <v>-1927101.095238095</v>
+        <v>-1932970.936507936</v>
       </c>
     </row>
     <row r="102">
@@ -8585,17 +8669,23 @@
       <c r="AF102" s="15" t="n">
         <v>-46202465.05677249</v>
       </c>
-      <c r="AG102" s="15" t="n"/>
-      <c r="AH102" s="15" t="n"/>
-      <c r="AI102" s="15" t="n"/>
+      <c r="AG102" s="15" t="n">
+        <v>-85290450</v>
+      </c>
+      <c r="AH102" s="15" t="n">
+        <v>-5017.085294117647</v>
+      </c>
+      <c r="AI102" s="15" t="n">
+        <v>-451272.2222222222</v>
+      </c>
       <c r="AJ102" s="15" t="n">
-        <v>-8732265895.73</v>
+        <v>-8817556345.73</v>
       </c>
       <c r="AK102" s="15" t="n">
-        <v>-513662.6997488235</v>
+        <v>-518679.7850429411</v>
       </c>
       <c r="AL102" s="15" t="n">
-        <v>-46202465.05677249</v>
+        <v>-46653737.27899472</v>
       </c>
     </row>
     <row r="103">
@@ -8737,17 +8827,23 @@
       <c r="AF104" s="11" t="n">
         <v>-1237435.248677249</v>
       </c>
-      <c r="AG104" s="11" t="n"/>
-      <c r="AH104" s="11" t="n"/>
-      <c r="AI104" s="11" t="n"/>
+      <c r="AG104" s="11" t="n">
+        <v>-544500</v>
+      </c>
+      <c r="AH104" s="11" t="n">
+        <v>-32.02941176470588</v>
+      </c>
+      <c r="AI104" s="11" t="n">
+        <v>-2880.952380952381</v>
+      </c>
       <c r="AJ104" s="11" t="n">
-        <v>-233875262</v>
+        <v>-234419762</v>
       </c>
       <c r="AK104" s="11" t="n">
-        <v>-13757.36835294118</v>
+        <v>-13789.39776470588</v>
       </c>
       <c r="AL104" s="11" t="n">
-        <v>-1237435.248677249</v>
+        <v>-1240316.201058201</v>
       </c>
     </row>
     <row r="105">
@@ -8846,17 +8942,23 @@
       <c r="AF105" s="13" t="n">
         <v>-1864747.592592593</v>
       </c>
-      <c r="AG105" s="13" t="n"/>
-      <c r="AH105" s="13" t="n"/>
-      <c r="AI105" s="13" t="n"/>
+      <c r="AG105" s="13" t="n">
+        <v>-587000</v>
+      </c>
+      <c r="AH105" s="13" t="n">
+        <v>-34.52941176470588</v>
+      </c>
+      <c r="AI105" s="13" t="n">
+        <v>-3105.820105820106</v>
+      </c>
       <c r="AJ105" s="13" t="n">
-        <v>-352437295</v>
+        <v>-353024295</v>
       </c>
       <c r="AK105" s="13" t="n">
-        <v>-20731.6055882353</v>
+        <v>-20766.135</v>
       </c>
       <c r="AL105" s="13" t="n">
-        <v>-1864747.592592593</v>
+        <v>-1867853.412698413</v>
       </c>
     </row>
     <row r="106">
@@ -9167,17 +9269,23 @@
       <c r="AF108" s="15" t="n">
         <v>-13088081.45502646</v>
       </c>
-      <c r="AG108" s="15" t="n"/>
-      <c r="AH108" s="15" t="n"/>
-      <c r="AI108" s="15" t="n"/>
+      <c r="AG108" s="15" t="n">
+        <v>-1131500</v>
+      </c>
+      <c r="AH108" s="15" t="n">
+        <v>-66.55882352941177</v>
+      </c>
+      <c r="AI108" s="15" t="n">
+        <v>-5986.772486772486</v>
+      </c>
       <c r="AJ108" s="15" t="n">
-        <v>-2473647395</v>
+        <v>-2474778895</v>
       </c>
       <c r="AK108" s="15" t="n">
-        <v>-145508.6702941176</v>
+        <v>-145575.229117647</v>
       </c>
       <c r="AL108" s="15" t="n">
-        <v>-13088081.45502646</v>
+        <v>-13094068.22751323</v>
       </c>
     </row>
     <row r="109">
@@ -9495,17 +9603,23 @@
       <c r="AF112" s="11" t="n">
         <v>-2628936.037037037</v>
       </c>
-      <c r="AG112" s="11" t="n"/>
-      <c r="AH112" s="11" t="n"/>
-      <c r="AI112" s="11" t="n"/>
+      <c r="AG112" s="11" t="n">
+        <v>-16087500</v>
+      </c>
+      <c r="AH112" s="11" t="n">
+        <v>-946.3235294117648</v>
+      </c>
+      <c r="AI112" s="11" t="n">
+        <v>-85119.04761904762</v>
+      </c>
       <c r="AJ112" s="11" t="n">
-        <v>-496868911</v>
+        <v>-512956411</v>
       </c>
       <c r="AK112" s="11" t="n">
-        <v>-29227.583</v>
+        <v>-30173.90652941176</v>
       </c>
       <c r="AL112" s="11" t="n">
-        <v>-2628936.037037037</v>
+        <v>-2714055.084656085</v>
       </c>
     </row>
     <row r="113">
@@ -9604,17 +9718,23 @@
       <c r="AF113" s="15" t="n">
         <v>-3443791.063492063</v>
       </c>
-      <c r="AG113" s="15" t="n"/>
-      <c r="AH113" s="15" t="n"/>
-      <c r="AI113" s="15" t="n"/>
+      <c r="AG113" s="15" t="n">
+        <v>-16087500</v>
+      </c>
+      <c r="AH113" s="15" t="n">
+        <v>-946.3235294117648</v>
+      </c>
+      <c r="AI113" s="15" t="n">
+        <v>-85119.04761904762</v>
+      </c>
       <c r="AJ113" s="15" t="n">
-        <v>-650876511</v>
+        <v>-666964011</v>
       </c>
       <c r="AK113" s="15" t="n">
-        <v>-38286.8535882353</v>
+        <v>-39233.17711764706</v>
       </c>
       <c r="AL113" s="15" t="n">
-        <v>-3443791.063492063</v>
+        <v>-3528910.111111111</v>
       </c>
     </row>
     <row r="114">
@@ -10351,17 +10471,23 @@
       <c r="AF122" s="13" t="n">
         <v>-34751144.73015873</v>
       </c>
-      <c r="AG122" s="13" t="n"/>
-      <c r="AH122" s="13" t="n"/>
-      <c r="AI122" s="13" t="n"/>
+      <c r="AG122" s="13" t="n">
+        <v>-3836159</v>
+      </c>
+      <c r="AH122" s="13" t="n">
+        <v>-225.6564117647059</v>
+      </c>
+      <c r="AI122" s="13" t="n">
+        <v>-20297.13756613757</v>
+      </c>
       <c r="AJ122" s="13" t="n">
-        <v>-6567966354</v>
+        <v>-6571802513</v>
       </c>
       <c r="AK122" s="13" t="n">
-        <v>-386350.9619999999</v>
+        <v>-386576.6184117646</v>
       </c>
       <c r="AL122" s="13" t="n">
-        <v>-34751144.73015873</v>
+        <v>-34771441.86772487</v>
       </c>
     </row>
     <row r="123">
@@ -10460,17 +10586,23 @@
       <c r="AF123" s="15" t="n">
         <v>-35391244.26984127</v>
       </c>
-      <c r="AG123" s="15" t="n"/>
-      <c r="AH123" s="15" t="n"/>
-      <c r="AI123" s="15" t="n"/>
+      <c r="AG123" s="15" t="n">
+        <v>-3836159</v>
+      </c>
+      <c r="AH123" s="15" t="n">
+        <v>-225.6564117647059</v>
+      </c>
+      <c r="AI123" s="15" t="n">
+        <v>-20297.13756613757</v>
+      </c>
       <c r="AJ123" s="15" t="n">
-        <v>-6688945167</v>
+        <v>-6692781326</v>
       </c>
       <c r="AK123" s="15" t="n">
-        <v>-393467.3627647058</v>
+        <v>-393693.0191764705</v>
       </c>
       <c r="AL123" s="15" t="n">
-        <v>-35391244.26984127</v>
+        <v>-35411541.4074074</v>
       </c>
     </row>
     <row r="124">
@@ -11425,17 +11557,23 @@
       <c r="AF134" s="11" t="n">
         <v>-197258.3068783069</v>
       </c>
-      <c r="AG134" s="11" t="n"/>
-      <c r="AH134" s="11" t="n"/>
-      <c r="AI134" s="11" t="n"/>
+      <c r="AG134" s="11" t="n">
+        <v>-91000</v>
+      </c>
+      <c r="AH134" s="11" t="n">
+        <v>-5.352941176470588</v>
+      </c>
+      <c r="AI134" s="11" t="n">
+        <v>-481.4814814814815</v>
+      </c>
       <c r="AJ134" s="11" t="n">
-        <v>-37281820</v>
+        <v>-37372820</v>
       </c>
       <c r="AK134" s="11" t="n">
-        <v>-2193.048235294118</v>
+        <v>-2198.401176470588</v>
       </c>
       <c r="AL134" s="11" t="n">
-        <v>-197258.3068783069</v>
+        <v>-197739.7883597884</v>
       </c>
     </row>
     <row r="135">
@@ -11722,17 +11860,23 @@
       <c r="AF137" s="13" t="n">
         <v>-620735.5185185184</v>
       </c>
-      <c r="AG137" s="13" t="n"/>
-      <c r="AH137" s="13" t="n"/>
-      <c r="AI137" s="13" t="n"/>
+      <c r="AG137" s="13" t="n">
+        <v>-1866000</v>
+      </c>
+      <c r="AH137" s="13" t="n">
+        <v>-109.7647058823529</v>
+      </c>
+      <c r="AI137" s="13" t="n">
+        <v>-9873.015873015873</v>
+      </c>
       <c r="AJ137" s="13" t="n">
-        <v>-117319013</v>
+        <v>-119185013</v>
       </c>
       <c r="AK137" s="13" t="n">
-        <v>-6901.118411764705</v>
+        <v>-7010.883117647058</v>
       </c>
       <c r="AL137" s="13" t="n">
-        <v>-620735.5185185184</v>
+        <v>-630608.5343915343</v>
       </c>
     </row>
     <row r="138">
@@ -11898,17 +12042,23 @@
       <c r="AF139" s="13" t="n">
         <v>-9978.835978835979</v>
       </c>
-      <c r="AG139" s="13" t="n"/>
-      <c r="AH139" s="13" t="n"/>
-      <c r="AI139" s="13" t="n"/>
+      <c r="AG139" s="13" t="n">
+        <v>-89000</v>
+      </c>
+      <c r="AH139" s="13" t="n">
+        <v>-5.235294117647059</v>
+      </c>
+      <c r="AI139" s="13" t="n">
+        <v>-470.8994708994709</v>
+      </c>
       <c r="AJ139" s="13" t="n">
-        <v>-1886000</v>
+        <v>-1975000</v>
       </c>
       <c r="AK139" s="13" t="n">
-        <v>-110.9411764705882</v>
+        <v>-116.1764705882353</v>
       </c>
       <c r="AL139" s="13" t="n">
-        <v>-9978.835978835979</v>
+        <v>-10449.73544973545</v>
       </c>
     </row>
     <row r="140">
@@ -12007,17 +12157,23 @@
       <c r="AF140" s="15" t="n">
         <v>-5569215.973544973</v>
       </c>
-      <c r="AG140" s="15" t="n"/>
-      <c r="AH140" s="15" t="n"/>
-      <c r="AI140" s="15" t="n"/>
+      <c r="AG140" s="15" t="n">
+        <v>-2046000</v>
+      </c>
+      <c r="AH140" s="15" t="n">
+        <v>-120.3529411764706</v>
+      </c>
+      <c r="AI140" s="15" t="n">
+        <v>-10825.39682539683</v>
+      </c>
       <c r="AJ140" s="15" t="n">
-        <v>-1052581819</v>
+        <v>-1054627819</v>
       </c>
       <c r="AK140" s="15" t="n">
-        <v>-61916.57758823529</v>
+        <v>-62036.93052941176</v>
       </c>
       <c r="AL140" s="15" t="n">
-        <v>-5569215.973544973</v>
+        <v>-5580041.370370369</v>
       </c>
     </row>
     <row r="141">
@@ -12116,17 +12272,23 @@
       <c r="AF141" s="15" t="n">
         <v>-253884225.9834391</v>
       </c>
-      <c r="AG141" s="15" t="n"/>
-      <c r="AH141" s="15" t="n"/>
-      <c r="AI141" s="15" t="n"/>
+      <c r="AG141" s="15" t="n">
+        <v>-110536681</v>
+      </c>
+      <c r="AH141" s="15" t="n">
+        <v>-6502.157705882353</v>
+      </c>
+      <c r="AI141" s="15" t="n">
+        <v>-584850.1640211641</v>
+      </c>
       <c r="AJ141" s="15" t="n">
-        <v>-47984118710.87001</v>
+        <v>-48094655391.87001</v>
       </c>
       <c r="AK141" s="15" t="n">
-        <v>-2822595.218286471</v>
+        <v>-2829097.375992353</v>
       </c>
       <c r="AL141" s="15" t="n">
-        <v>-253884225.9834391</v>
+        <v>-254469076.1474603</v>
       </c>
     </row>
     <row r="142">
@@ -12736,17 +12898,23 @@
       <c r="AF149" s="11" t="n">
         <v>-107075.0670899471</v>
       </c>
-      <c r="AG149" s="11" t="n"/>
-      <c r="AH149" s="11" t="n"/>
-      <c r="AI149" s="11" t="n"/>
+      <c r="AG149" s="11" t="n">
+        <v>-15700</v>
+      </c>
+      <c r="AH149" s="11" t="n">
+        <v>-0.9235294117647059</v>
+      </c>
+      <c r="AI149" s="11" t="n">
+        <v>-83.06878306878306</v>
+      </c>
       <c r="AJ149" s="11" t="n">
-        <v>-20237187.68</v>
+        <v>-20252887.68</v>
       </c>
       <c r="AK149" s="11" t="n">
-        <v>-1190.422804705882</v>
+        <v>-1191.346334117647</v>
       </c>
       <c r="AL149" s="11" t="n">
-        <v>-107075.0670899471</v>
+        <v>-107158.1358730159</v>
       </c>
     </row>
     <row r="150">
@@ -13258,17 +13426,23 @@
       <c r="AF155" s="15" t="n">
         <v>-33085054.60883598</v>
       </c>
-      <c r="AG155" s="15" t="n"/>
-      <c r="AH155" s="15" t="n"/>
-      <c r="AI155" s="15" t="n"/>
+      <c r="AG155" s="15" t="n">
+        <v>-15700</v>
+      </c>
+      <c r="AH155" s="15" t="n">
+        <v>-0.9235294117647059</v>
+      </c>
+      <c r="AI155" s="15" t="n">
+        <v>-83.06878306878306</v>
+      </c>
       <c r="AJ155" s="15" t="n">
-        <v>-6253075321.070001</v>
+        <v>-6253091021.070001</v>
       </c>
       <c r="AK155" s="15" t="n">
-        <v>-367827.9600629411</v>
+        <v>-367828.8835923529</v>
       </c>
       <c r="AL155" s="15" t="n">
-        <v>-33085054.60883598</v>
+        <v>-33085137.67761905</v>
       </c>
     </row>
     <row r="156">
@@ -13367,17 +13541,23 @@
       <c r="AF156" s="19" t="n">
         <v>-1609397741.344392</v>
       </c>
-      <c r="AG156" s="19" t="n"/>
-      <c r="AH156" s="19" t="n"/>
-      <c r="AI156" s="19" t="n"/>
+      <c r="AG156" s="19" t="n">
+        <v>-1880249274</v>
+      </c>
+      <c r="AH156" s="19" t="n">
+        <v>-110602.8984705882</v>
+      </c>
+      <c r="AI156" s="19" t="n">
+        <v>-9948408.857142856</v>
+      </c>
       <c r="AJ156" s="19" t="n">
-        <v>-304176173114.09</v>
+        <v>-306056422388.09</v>
       </c>
       <c r="AK156" s="19" t="n">
-        <v>-17892716.0655347</v>
+        <v>-18003318.96400529</v>
       </c>
       <c r="AL156" s="19" t="n">
-        <v>-1609397741.344392</v>
+        <v>-1619346150.201535</v>
       </c>
     </row>
     <row r="157">
@@ -13477,22 +13657,22 @@
         <v>-277217918.5799472</v>
       </c>
       <c r="AG157" s="19" t="n">
-        <v>623000</v>
+        <v>-139626518</v>
       </c>
       <c r="AH157" s="19" t="n">
-        <v>36.64705882352941</v>
+        <v>-8213.324588235295</v>
       </c>
       <c r="AI157" s="19" t="n">
-        <v>3296.296296296296</v>
+        <v>-738764.6455026455</v>
       </c>
       <c r="AJ157" s="19" t="n">
-        <v>-52393563611.61</v>
+        <v>-52533813129.61</v>
       </c>
       <c r="AK157" s="19" t="n">
-        <v>-3081974.330094707</v>
+        <v>-3090224.301741766</v>
       </c>
       <c r="AL157" s="19" t="n">
-        <v>-277214622.2836509</v>
+        <v>-277956683.2254499</v>
       </c>
     </row>
     <row r="158">
@@ -13592,22 +13772,22 @@
         <v>79785577.85582009</v>
       </c>
       <c r="AG158" s="7" t="n">
-        <v>15080097214.75</v>
+        <v>14939847696.75</v>
       </c>
       <c r="AH158" s="7" t="n">
-        <v>887064.5420441176</v>
+        <v>878814.5703970587</v>
       </c>
       <c r="AI158" s="7" t="n">
-        <v>79788874.15211639</v>
+        <v>79046813.21031745</v>
       </c>
       <c r="AJ158" s="7" t="n">
-        <v>15080097214.75</v>
+        <v>14939847696.75</v>
       </c>
       <c r="AK158" s="7" t="n">
-        <v>887064.5420441176</v>
+        <v>878814.5703970587</v>
       </c>
       <c r="AL158" s="7" t="n">
-        <v>79788874.15211639</v>
+        <v>79046813.21031745</v>
       </c>
     </row>
   </sheetData>
@@ -14410,16 +14590,16 @@
         <v>14828882907</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>0</v>
+        <v>-141156018</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>14828882907</v>
+        <v>14687726889</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>872287.2298235294</v>
+        <v>863983.9346470588</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>78459697.92063493</v>
+        <v>77712840.68253969</v>
       </c>
     </row>
     <row r="7">
@@ -14471,10 +14651,10 @@
         </is>
       </c>
       <c r="D8" s="11" t="n">
-        <v>2000000</v>
+        <v>1975000</v>
       </c>
       <c r="E8" s="11" t="n">
-        <v>0</v>
+        <v>25000</v>
       </c>
       <c r="F8" s="11" t="n">
         <v>2000000</v>
@@ -14506,16 +14686,16 @@
         <v>22400563.84000001</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>623000</v>
+        <v>1504500</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>23023563.84000001</v>
+        <v>23905063.84000001</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>1354.327284705883</v>
+        <v>1406.180225882354</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>121817.7980952381</v>
+        <v>126481.8192592593</v>
       </c>
     </row>
     <row r="10">
@@ -14625,13 +14805,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>15080122216.75</v>
+        <v>14939847698.75</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>887066.0127499999</v>
+        <v>878814.5705147057</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>79789006.43783067</v>
+        <v>79046813.22089946</v>
       </c>
     </row>
   </sheetData>
@@ -14704,7 +14884,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 01 Oct 2026 20:32 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 02 Oct 2026 17:26 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -14786,14 +14966,14 @@
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 01 Oct 2026</t>
+          <t>MTD as of 02 Oct 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
       <c r="AI3" s="4" t="n"/>
       <c r="AJ3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 01 Oct 2026</t>
+          <t>YTD as of 02 Oct 2026</t>
         </is>
       </c>
       <c r="AK3" s="4" t="n"/>
@@ -15236,17 +15416,23 @@
       <c r="AF7" s="11" t="n">
         <v>1066.081968222222</v>
       </c>
-      <c r="AG7" s="11" t="n"/>
-      <c r="AH7" s="11" t="n"/>
-      <c r="AI7" s="11" t="n"/>
+      <c r="AG7" s="11" t="n">
+        <v>1739.093256</v>
+      </c>
+      <c r="AH7" s="11" t="n">
+        <v>0.1022996032941176</v>
+      </c>
+      <c r="AI7" s="11" t="n">
+        <v>9.201551619047619</v>
+      </c>
       <c r="AJ7" s="11" t="n">
-        <v>201489.491994</v>
+        <v>203228.58525</v>
       </c>
       <c r="AK7" s="11" t="n">
-        <v>11.85232305847059</v>
+        <v>11.9546226617647</v>
       </c>
       <c r="AL7" s="11" t="n">
-        <v>1066.081968222222</v>
+        <v>1075.28351984127</v>
       </c>
     </row>
     <row r="8">
@@ -15418,17 +15604,23 @@
       <c r="AF9" s="11" t="n">
         <v>283.2254925132275</v>
       </c>
-      <c r="AG9" s="11" t="n"/>
-      <c r="AH9" s="11" t="n"/>
-      <c r="AI9" s="11" t="n"/>
+      <c r="AG9" s="11" t="n">
+        <v>1739.093256</v>
+      </c>
+      <c r="AH9" s="11" t="n">
+        <v>0.1022996032941176</v>
+      </c>
+      <c r="AI9" s="11" t="n">
+        <v>9.201551619047619</v>
+      </c>
       <c r="AJ9" s="11" t="n">
-        <v>53529.618085</v>
+        <v>55268.711341</v>
       </c>
       <c r="AK9" s="11" t="n">
-        <v>3.148801063823529</v>
+        <v>3.251100667117647</v>
       </c>
       <c r="AL9" s="11" t="n">
-        <v>283.2254925132275</v>
+        <v>292.4270441322751</v>
       </c>
     </row>
     <row r="10">
@@ -16276,22 +16468,22 @@
         <v>2.521134965502646</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>0.623</v>
+        <v>1.5295</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>3.664705882352941e-05</v>
+        <v>8.997058823529413e-05</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>0.003296296296296296</v>
+        <v>0.008092592592592592</v>
       </c>
       <c r="AJ20" s="13" t="n">
-        <v>477.11750848</v>
+        <v>478.02400848</v>
       </c>
       <c r="AK20" s="13" t="n">
-        <v>0.02806573579294118</v>
+        <v>0.02811905932235294</v>
       </c>
       <c r="AL20" s="13" t="n">
-        <v>2.524431261798942</v>
+        <v>2.529227558095239</v>
       </c>
     </row>
     <row r="21">
@@ -16549,22 +16741,22 @@
         <v>0.4919761904761905</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>0.623</v>
+        <v>1.5295</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>3.664705882352941e-05</v>
+        <v>8.997058823529413e-05</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>0.003296296296296296</v>
+        <v>0.008092592592592592</v>
       </c>
       <c r="AJ23" s="11" t="n">
-        <v>93.60650000000001</v>
+        <v>94.51300000000001</v>
       </c>
       <c r="AK23" s="11" t="n">
-        <v>0.005506264705882354</v>
+        <v>0.005559588235294118</v>
       </c>
       <c r="AL23" s="11" t="n">
-        <v>0.4952724867724868</v>
+        <v>0.500068783068783</v>
       </c>
     </row>
     <row r="24">
@@ -18089,22 +18281,22 @@
         <v>1332.179822764444</v>
       </c>
       <c r="AG45" s="15" t="n">
-        <v>0.623</v>
+        <v>1740.622756</v>
       </c>
       <c r="AH45" s="15" t="n">
-        <v>3.664705882352941e-05</v>
+        <v>0.1023895738823529</v>
       </c>
       <c r="AI45" s="15" t="n">
-        <v>0.003296296296296296</v>
+        <v>9.209644211640212</v>
       </c>
       <c r="AJ45" s="15" t="n">
-        <v>251782.60950248</v>
+        <v>253522.60925848</v>
       </c>
       <c r="AK45" s="15" t="n">
-        <v>14.81074173544</v>
+        <v>14.91309466226353</v>
       </c>
       <c r="AL45" s="15" t="n">
-        <v>1332.183119060741</v>
+        <v>1341.389466976085</v>
       </c>
     </row>
     <row r="46">
@@ -20650,17 +20842,23 @@
       <c r="AF81" s="11" t="n">
         <v>-52.84339814285714</v>
       </c>
-      <c r="AG81" s="11" t="n"/>
-      <c r="AH81" s="11" t="n"/>
-      <c r="AI81" s="11" t="n"/>
+      <c r="AG81" s="11" t="n">
+        <v>-870.978933</v>
+      </c>
+      <c r="AH81" s="11" t="n">
+        <v>-0.05123405488235294</v>
+      </c>
+      <c r="AI81" s="11" t="n">
+        <v>-4.608354142857142</v>
+      </c>
       <c r="AJ81" s="11" t="n">
-        <v>-9987.402249000001</v>
+        <v>-10858.381182</v>
       </c>
       <c r="AK81" s="11" t="n">
-        <v>-0.5874942499411766</v>
+        <v>-0.6387283048235295</v>
       </c>
       <c r="AL81" s="11" t="n">
-        <v>-52.84339814285714</v>
+        <v>-57.45175228571429</v>
       </c>
     </row>
     <row r="82">
@@ -20759,17 +20957,23 @@
       <c r="AF82" s="13" t="n">
         <v>-58.93422933476191</v>
       </c>
-      <c r="AG82" s="13" t="n"/>
-      <c r="AH82" s="13" t="n"/>
-      <c r="AI82" s="13" t="n"/>
+      <c r="AG82" s="13" t="n">
+        <v>-897.91796</v>
+      </c>
+      <c r="AH82" s="13" t="n">
+        <v>-0.05281870352941177</v>
+      </c>
+      <c r="AI82" s="13" t="n">
+        <v>-4.750888677248677</v>
+      </c>
       <c r="AJ82" s="13" t="n">
-        <v>-11138.56934427</v>
+        <v>-12036.48730427</v>
       </c>
       <c r="AK82" s="13" t="n">
-        <v>-0.655209961427647</v>
+        <v>-0.7080286649570587</v>
       </c>
       <c r="AL82" s="13" t="n">
-        <v>-58.93422933476191</v>
+        <v>-63.68511801201058</v>
       </c>
     </row>
     <row r="83">
@@ -20977,17 +21181,23 @@
       <c r="AF84" s="13" t="n">
         <v>-2.427178873015873</v>
       </c>
-      <c r="AG84" s="13" t="n"/>
-      <c r="AH84" s="13" t="n"/>
-      <c r="AI84" s="13" t="n"/>
+      <c r="AG84" s="13" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="AH84" s="13" t="n">
+        <v>-4.705882352941177e-05</v>
+      </c>
+      <c r="AI84" s="13" t="n">
+        <v>-0.004232804232804233</v>
+      </c>
       <c r="AJ84" s="13" t="n">
-        <v>-458.7368070000001</v>
+        <v>-459.5368070000001</v>
       </c>
       <c r="AK84" s="13" t="n">
-        <v>-0.02698451805882354</v>
+        <v>-0.02703157688235295</v>
       </c>
       <c r="AL84" s="13" t="n">
-        <v>-2.427178873015873</v>
+        <v>-2.431411677248677</v>
       </c>
     </row>
     <row r="85">
@@ -21086,17 +21296,23 @@
       <c r="AF85" s="15" t="n">
         <v>-170.3013063770899</v>
       </c>
-      <c r="AG85" s="15" t="n"/>
-      <c r="AH85" s="15" t="n"/>
-      <c r="AI85" s="15" t="n"/>
+      <c r="AG85" s="15" t="n">
+        <v>-1769.696893</v>
+      </c>
+      <c r="AH85" s="15" t="n">
+        <v>-0.1040998172352941</v>
+      </c>
+      <c r="AI85" s="15" t="n">
+        <v>-9.363475624338625</v>
+      </c>
       <c r="AJ85" s="15" t="n">
-        <v>-32186.94690527</v>
+        <v>-33956.64379827</v>
       </c>
       <c r="AK85" s="15" t="n">
-        <v>-1.893349817957059</v>
+        <v>-1.997449635192353</v>
       </c>
       <c r="AL85" s="15" t="n">
-        <v>-170.3013063770899</v>
+        <v>-179.6647820014286</v>
       </c>
     </row>
     <row r="86">
@@ -21281,17 +21497,23 @@
       <c r="AF88" s="11" t="n">
         <v>-0.778818253968254</v>
       </c>
-      <c r="AG88" s="11" t="n"/>
-      <c r="AH88" s="11" t="n"/>
-      <c r="AI88" s="11" t="n"/>
+      <c r="AG88" s="11" t="n">
+        <v>-0.294372</v>
+      </c>
+      <c r="AH88" s="11" t="n">
+        <v>-1.7316e-05</v>
+      </c>
+      <c r="AI88" s="11" t="n">
+        <v>-0.00155752380952381</v>
+      </c>
       <c r="AJ88" s="11" t="n">
-        <v>-147.19665</v>
+        <v>-147.491022</v>
       </c>
       <c r="AK88" s="11" t="n">
-        <v>-0.008658626470588234</v>
+        <v>-0.008675942470588234</v>
       </c>
       <c r="AL88" s="11" t="n">
-        <v>-0.778818253968254</v>
+        <v>-0.7803757777777778</v>
       </c>
     </row>
     <row r="89">
@@ -21342,17 +21564,23 @@
       <c r="AF89" s="13" t="n">
         <v>-0.0138973544973545</v>
       </c>
-      <c r="AG89" s="13" t="n"/>
-      <c r="AH89" s="13" t="n"/>
-      <c r="AI89" s="13" t="n"/>
+      <c r="AG89" s="13" t="n">
+        <v>-0.7725</v>
+      </c>
+      <c r="AH89" s="13" t="n">
+        <v>-4.544117647058823e-05</v>
+      </c>
+      <c r="AI89" s="13" t="n">
+        <v>-0.004087301587301587</v>
+      </c>
       <c r="AJ89" s="13" t="n">
-        <v>-2.6266</v>
+        <v>-3.3991</v>
       </c>
       <c r="AK89" s="13" t="n">
-        <v>-0.0001545058823529412</v>
+        <v>-0.0001999470588235294</v>
       </c>
       <c r="AL89" s="13" t="n">
-        <v>-0.0138973544973545</v>
+        <v>-0.01798465608465608</v>
       </c>
     </row>
     <row r="90">
@@ -21615,17 +21843,23 @@
       <c r="AF92" s="11" t="n">
         <v>-0.7864109841269842</v>
       </c>
-      <c r="AG92" s="11" t="n"/>
-      <c r="AH92" s="11" t="n"/>
-      <c r="AI92" s="11" t="n"/>
+      <c r="AG92" s="11" t="n">
+        <v>-1.0782</v>
+      </c>
+      <c r="AH92" s="11" t="n">
+        <v>-6.34235294117647e-05</v>
+      </c>
+      <c r="AI92" s="11" t="n">
+        <v>-0.005704761904761905</v>
+      </c>
       <c r="AJ92" s="11" t="n">
-        <v>-148.631676</v>
+        <v>-149.709876</v>
       </c>
       <c r="AK92" s="11" t="n">
-        <v>-0.008743039764705883</v>
+        <v>-0.008806463294117647</v>
       </c>
       <c r="AL92" s="11" t="n">
-        <v>-0.7864109841269842</v>
+        <v>-0.7921157460317461</v>
       </c>
     </row>
     <row r="93">
@@ -21821,17 +22055,23 @@
       <c r="AF94" s="15" t="n">
         <v>-2.636230425608466</v>
       </c>
-      <c r="AG94" s="15" t="n"/>
-      <c r="AH94" s="15" t="n"/>
-      <c r="AI94" s="15" t="n"/>
+      <c r="AG94" s="15" t="n">
+        <v>-2.145072</v>
+      </c>
+      <c r="AH94" s="15" t="n">
+        <v>-0.0001261807058823529</v>
+      </c>
+      <c r="AI94" s="15" t="n">
+        <v>-0.0113495873015873</v>
+      </c>
       <c r="AJ94" s="15" t="n">
-        <v>-498.2475504400001</v>
+        <v>-500.3926224400001</v>
       </c>
       <c r="AK94" s="15" t="n">
-        <v>-0.02930867943764706</v>
+        <v>-0.02943486014352941</v>
       </c>
       <c r="AL94" s="15" t="n">
-        <v>-2.636230425608466</v>
+        <v>-2.647580012910053</v>
       </c>
     </row>
     <row r="95">
@@ -22010,17 +22250,23 @@
       <c r="AF97" s="13" t="n">
         <v>-0.4714513227513227</v>
       </c>
-      <c r="AG97" s="13" t="n"/>
-      <c r="AH97" s="13" t="n"/>
-      <c r="AI97" s="13" t="n"/>
+      <c r="AG97" s="13" t="n">
+        <v>-0.531541</v>
+      </c>
+      <c r="AH97" s="13" t="n">
+        <v>-3.126711764705883e-05</v>
+      </c>
+      <c r="AI97" s="13" t="n">
+        <v>-0.002812386243386244</v>
+      </c>
       <c r="AJ97" s="13" t="n">
-        <v>-89.10430000000001</v>
+        <v>-89.63584100000001</v>
       </c>
       <c r="AK97" s="13" t="n">
-        <v>-0.005241429411764707</v>
+        <v>-0.005272696529411766</v>
       </c>
       <c r="AL97" s="13" t="n">
-        <v>-0.4714513227513227</v>
+        <v>-0.474263708994709</v>
       </c>
     </row>
     <row r="98">
@@ -22119,17 +22365,23 @@
       <c r="AF98" s="11" t="n">
         <v>-1.418156079365079</v>
       </c>
-      <c r="AG98" s="11" t="n"/>
-      <c r="AH98" s="11" t="n"/>
-      <c r="AI98" s="11" t="n"/>
+      <c r="AG98" s="11" t="n">
+        <v>-1.2485</v>
+      </c>
+      <c r="AH98" s="11" t="n">
+        <v>-7.344117647058823e-05</v>
+      </c>
+      <c r="AI98" s="11" t="n">
+        <v>-0.006605820105820105</v>
+      </c>
       <c r="AJ98" s="11" t="n">
-        <v>-268.031499</v>
+        <v>-269.279999</v>
       </c>
       <c r="AK98" s="11" t="n">
-        <v>-0.01576655876470588</v>
+        <v>-0.01583999994117647</v>
       </c>
       <c r="AL98" s="11" t="n">
-        <v>-1.418156079365079</v>
+        <v>-1.424761899470899</v>
       </c>
     </row>
     <row r="99">
@@ -22228,17 +22480,23 @@
       <c r="AF99" s="13" t="n">
         <v>-40.89323655941799</v>
       </c>
-      <c r="AG99" s="13" t="n"/>
-      <c r="AH99" s="13" t="n"/>
-      <c r="AI99" s="13" t="n"/>
+      <c r="AG99" s="13" t="n">
+        <v>-82.401009</v>
+      </c>
+      <c r="AH99" s="13" t="n">
+        <v>-0.004847118176470588</v>
+      </c>
+      <c r="AI99" s="13" t="n">
+        <v>-0.4359841746031746</v>
+      </c>
       <c r="AJ99" s="13" t="n">
-        <v>-7728.82170973</v>
+        <v>-7811.22271873</v>
       </c>
       <c r="AK99" s="13" t="n">
-        <v>-0.4546365711605882</v>
+        <v>-0.4594836893370588</v>
       </c>
       <c r="AL99" s="13" t="n">
-        <v>-40.89323655941799</v>
+        <v>-41.32922073402117</v>
       </c>
     </row>
     <row r="100">
@@ -22446,17 +22704,23 @@
       <c r="AF101" s="13" t="n">
         <v>-1.927101095238095</v>
       </c>
-      <c r="AG101" s="13" t="n"/>
-      <c r="AH101" s="13" t="n"/>
-      <c r="AI101" s="13" t="n"/>
+      <c r="AG101" s="13" t="n">
+        <v>-1.1094</v>
+      </c>
+      <c r="AH101" s="13" t="n">
+        <v>-6.525882352941176e-05</v>
+      </c>
+      <c r="AI101" s="13" t="n">
+        <v>-0.00586984126984127</v>
+      </c>
       <c r="AJ101" s="13" t="n">
-        <v>-364.2221070000001</v>
+        <v>-365.331507</v>
       </c>
       <c r="AK101" s="13" t="n">
-        <v>-0.02142482982352941</v>
+        <v>-0.02149008864705883</v>
       </c>
       <c r="AL101" s="13" t="n">
-        <v>-1.927101095238095</v>
+        <v>-1.932970936507936</v>
       </c>
     </row>
     <row r="102">
@@ -22555,17 +22819,23 @@
       <c r="AF102" s="15" t="n">
         <v>-46.20246505677248</v>
       </c>
-      <c r="AG102" s="15" t="n"/>
-      <c r="AH102" s="15" t="n"/>
-      <c r="AI102" s="15" t="n"/>
+      <c r="AG102" s="15" t="n">
+        <v>-85.29045000000001</v>
+      </c>
+      <c r="AH102" s="15" t="n">
+        <v>-0.005017085294117648</v>
+      </c>
+      <c r="AI102" s="15" t="n">
+        <v>-0.4512722222222222</v>
+      </c>
       <c r="AJ102" s="15" t="n">
-        <v>-8732.265895730001</v>
+        <v>-8817.556345730001</v>
       </c>
       <c r="AK102" s="15" t="n">
-        <v>-0.5136626997488235</v>
+        <v>-0.5186797850429411</v>
       </c>
       <c r="AL102" s="15" t="n">
-        <v>-46.20246505677248</v>
+        <v>-46.6537372789947</v>
       </c>
     </row>
     <row r="103">
@@ -22707,17 +22977,23 @@
       <c r="AF104" s="11" t="n">
         <v>-1.237435248677249</v>
       </c>
-      <c r="AG104" s="11" t="n"/>
-      <c r="AH104" s="11" t="n"/>
-      <c r="AI104" s="11" t="n"/>
+      <c r="AG104" s="11" t="n">
+        <v>-0.5445</v>
+      </c>
+      <c r="AH104" s="11" t="n">
+        <v>-3.202941176470588e-05</v>
+      </c>
+      <c r="AI104" s="11" t="n">
+        <v>-0.002880952380952381</v>
+      </c>
       <c r="AJ104" s="11" t="n">
-        <v>-233.875262</v>
+        <v>-234.419762</v>
       </c>
       <c r="AK104" s="11" t="n">
-        <v>-0.01375736835294118</v>
+        <v>-0.01378939776470588</v>
       </c>
       <c r="AL104" s="11" t="n">
-        <v>-1.237435248677249</v>
+        <v>-1.240316201058201</v>
       </c>
     </row>
     <row r="105">
@@ -22816,17 +23092,23 @@
       <c r="AF105" s="13" t="n">
         <v>-1.864747592592592</v>
       </c>
-      <c r="AG105" s="13" t="n"/>
-      <c r="AH105" s="13" t="n"/>
-      <c r="AI105" s="13" t="n"/>
+      <c r="AG105" s="13" t="n">
+        <v>-0.587</v>
+      </c>
+      <c r="AH105" s="13" t="n">
+        <v>-3.452941176470588e-05</v>
+      </c>
+      <c r="AI105" s="13" t="n">
+        <v>-0.003105820105820106</v>
+      </c>
       <c r="AJ105" s="13" t="n">
-        <v>-352.437295</v>
+        <v>-353.024295</v>
       </c>
       <c r="AK105" s="13" t="n">
-        <v>-0.02073160558823529</v>
+        <v>-0.020766135</v>
       </c>
       <c r="AL105" s="13" t="n">
-        <v>-1.864747592592592</v>
+        <v>-1.867853412698413</v>
       </c>
     </row>
     <row r="106">
@@ -23137,17 +23419,23 @@
       <c r="AF108" s="15" t="n">
         <v>-13.08808145502645</v>
       </c>
-      <c r="AG108" s="15" t="n"/>
-      <c r="AH108" s="15" t="n"/>
-      <c r="AI108" s="15" t="n"/>
+      <c r="AG108" s="15" t="n">
+        <v>-1.1315</v>
+      </c>
+      <c r="AH108" s="15" t="n">
+        <v>-6.655882352941176e-05</v>
+      </c>
+      <c r="AI108" s="15" t="n">
+        <v>-0.005986772486772486</v>
+      </c>
       <c r="AJ108" s="15" t="n">
-        <v>-2473.647395</v>
+        <v>-2474.778895</v>
       </c>
       <c r="AK108" s="15" t="n">
-        <v>-0.1455086702941176</v>
+        <v>-0.145575229117647</v>
       </c>
       <c r="AL108" s="15" t="n">
-        <v>-13.08808145502645</v>
+        <v>-13.09406822751323</v>
       </c>
     </row>
     <row r="109">
@@ -23465,17 +23753,23 @@
       <c r="AF112" s="11" t="n">
         <v>-2.628936037037037</v>
       </c>
-      <c r="AG112" s="11" t="n"/>
-      <c r="AH112" s="11" t="n"/>
-      <c r="AI112" s="11" t="n"/>
+      <c r="AG112" s="11" t="n">
+        <v>-16.0875</v>
+      </c>
+      <c r="AH112" s="11" t="n">
+        <v>-0.0009463235294117646</v>
+      </c>
+      <c r="AI112" s="11" t="n">
+        <v>-0.08511904761904761</v>
+      </c>
       <c r="AJ112" s="11" t="n">
-        <v>-496.8689110000001</v>
+        <v>-512.9564110000001</v>
       </c>
       <c r="AK112" s="11" t="n">
-        <v>-0.029227583</v>
+        <v>-0.03017390652941176</v>
       </c>
       <c r="AL112" s="11" t="n">
-        <v>-2.628936037037037</v>
+        <v>-2.714055084656084</v>
       </c>
     </row>
     <row r="113">
@@ -23574,17 +23868,23 @@
       <c r="AF113" s="15" t="n">
         <v>-3.443791063492064</v>
       </c>
-      <c r="AG113" s="15" t="n"/>
-      <c r="AH113" s="15" t="n"/>
-      <c r="AI113" s="15" t="n"/>
+      <c r="AG113" s="15" t="n">
+        <v>-16.0875</v>
+      </c>
+      <c r="AH113" s="15" t="n">
+        <v>-0.0009463235294117646</v>
+      </c>
+      <c r="AI113" s="15" t="n">
+        <v>-0.08511904761904761</v>
+      </c>
       <c r="AJ113" s="15" t="n">
-        <v>-650.8765109999999</v>
+        <v>-666.9640109999999</v>
       </c>
       <c r="AK113" s="15" t="n">
-        <v>-0.03828685358823529</v>
+        <v>-0.03923317711764705</v>
       </c>
       <c r="AL113" s="15" t="n">
-        <v>-3.443791063492064</v>
+        <v>-3.528910111111111</v>
       </c>
     </row>
     <row r="114">
@@ -24321,17 +24621,23 @@
       <c r="AF122" s="13" t="n">
         <v>-34.75114473015874</v>
       </c>
-      <c r="AG122" s="13" t="n"/>
-      <c r="AH122" s="13" t="n"/>
-      <c r="AI122" s="13" t="n"/>
+      <c r="AG122" s="13" t="n">
+        <v>-3.836159</v>
+      </c>
+      <c r="AH122" s="13" t="n">
+        <v>-0.0002256564117647059</v>
+      </c>
+      <c r="AI122" s="13" t="n">
+        <v>-0.02029713756613757</v>
+      </c>
       <c r="AJ122" s="13" t="n">
-        <v>-6567.966353999999</v>
+        <v>-6571.802513</v>
       </c>
       <c r="AK122" s="13" t="n">
-        <v>-0.386350962</v>
+        <v>-0.3865766184117647</v>
       </c>
       <c r="AL122" s="13" t="n">
-        <v>-34.75114473015874</v>
+        <v>-34.77144186772487</v>
       </c>
     </row>
     <row r="123">
@@ -24430,17 +24736,23 @@
       <c r="AF123" s="15" t="n">
         <v>-35.39124426984127</v>
       </c>
-      <c r="AG123" s="15" t="n"/>
-      <c r="AH123" s="15" t="n"/>
-      <c r="AI123" s="15" t="n"/>
+      <c r="AG123" s="15" t="n">
+        <v>-3.836159</v>
+      </c>
+      <c r="AH123" s="15" t="n">
+        <v>-0.0002256564117647059</v>
+      </c>
+      <c r="AI123" s="15" t="n">
+        <v>-0.02029713756613757</v>
+      </c>
       <c r="AJ123" s="15" t="n">
-        <v>-6688.945167</v>
+        <v>-6692.781326</v>
       </c>
       <c r="AK123" s="15" t="n">
-        <v>-0.3934673627647058</v>
+        <v>-0.3936930191764705</v>
       </c>
       <c r="AL123" s="15" t="n">
-        <v>-35.39124426984127</v>
+        <v>-35.41154140740741</v>
       </c>
     </row>
     <row r="124">
@@ -25395,17 +25707,23 @@
       <c r="AF134" s="11" t="n">
         <v>-0.1972583068783069</v>
       </c>
-      <c r="AG134" s="11" t="n"/>
-      <c r="AH134" s="11" t="n"/>
-      <c r="AI134" s="11" t="n"/>
+      <c r="AG134" s="11" t="n">
+        <v>-0.091</v>
+      </c>
+      <c r="AH134" s="11" t="n">
+        <v>-5.352941176470588e-06</v>
+      </c>
+      <c r="AI134" s="11" t="n">
+        <v>-0.0004814814814814815</v>
+      </c>
       <c r="AJ134" s="11" t="n">
-        <v>-37.28182</v>
+        <v>-37.37282</v>
       </c>
       <c r="AK134" s="11" t="n">
-        <v>-0.002193048235294118</v>
+        <v>-0.002198401176470589</v>
       </c>
       <c r="AL134" s="11" t="n">
-        <v>-0.1972583068783069</v>
+        <v>-0.1977397883597883</v>
       </c>
     </row>
     <row r="135">
@@ -25692,17 +26010,23 @@
       <c r="AF137" s="13" t="n">
         <v>-0.6207355185185186</v>
       </c>
-      <c r="AG137" s="13" t="n"/>
-      <c r="AH137" s="13" t="n"/>
-      <c r="AI137" s="13" t="n"/>
+      <c r="AG137" s="13" t="n">
+        <v>-1.866</v>
+      </c>
+      <c r="AH137" s="13" t="n">
+        <v>-0.000109764705882353</v>
+      </c>
+      <c r="AI137" s="13" t="n">
+        <v>-0.009873015873015874</v>
+      </c>
       <c r="AJ137" s="13" t="n">
-        <v>-117.319013</v>
+        <v>-119.185013</v>
       </c>
       <c r="AK137" s="13" t="n">
-        <v>-0.006901118411764706</v>
+        <v>-0.007010883117647059</v>
       </c>
       <c r="AL137" s="13" t="n">
-        <v>-0.6207355185185186</v>
+        <v>-0.6306085343915345</v>
       </c>
     </row>
     <row r="138">
@@ -25868,17 +26192,23 @@
       <c r="AF139" s="13" t="n">
         <v>-0.009978835978835979</v>
       </c>
-      <c r="AG139" s="13" t="n"/>
-      <c r="AH139" s="13" t="n"/>
-      <c r="AI139" s="13" t="n"/>
+      <c r="AG139" s="13" t="n">
+        <v>-0.089</v>
+      </c>
+      <c r="AH139" s="13" t="n">
+        <v>-5.235294117647059e-06</v>
+      </c>
+      <c r="AI139" s="13" t="n">
+        <v>-0.0004708994708994709</v>
+      </c>
       <c r="AJ139" s="13" t="n">
-        <v>-1.886</v>
+        <v>-1.975</v>
       </c>
       <c r="AK139" s="13" t="n">
-        <v>-0.0001109411764705882</v>
+        <v>-0.0001161764705882353</v>
       </c>
       <c r="AL139" s="13" t="n">
-        <v>-0.009978835978835979</v>
+        <v>-0.01044973544973545</v>
       </c>
     </row>
     <row r="140">
@@ -25977,17 +26307,23 @@
       <c r="AF140" s="15" t="n">
         <v>-5.569215973544973</v>
       </c>
-      <c r="AG140" s="15" t="n"/>
-      <c r="AH140" s="15" t="n"/>
-      <c r="AI140" s="15" t="n"/>
+      <c r="AG140" s="15" t="n">
+        <v>-2.046</v>
+      </c>
+      <c r="AH140" s="15" t="n">
+        <v>-0.0001203529411764706</v>
+      </c>
+      <c r="AI140" s="15" t="n">
+        <v>-0.01082539682539682</v>
+      </c>
       <c r="AJ140" s="15" t="n">
-        <v>-1052.581819</v>
+        <v>-1054.627819</v>
       </c>
       <c r="AK140" s="15" t="n">
-        <v>-0.06191657758823529</v>
+        <v>-0.06203693052941176</v>
       </c>
       <c r="AL140" s="15" t="n">
-        <v>-5.569215973544973</v>
+        <v>-5.58004137037037</v>
       </c>
     </row>
     <row r="141">
@@ -26086,17 +26422,23 @@
       <c r="AF141" s="15" t="n">
         <v>-253.8842259834391</v>
       </c>
-      <c r="AG141" s="15" t="n"/>
-      <c r="AH141" s="15" t="n"/>
-      <c r="AI141" s="15" t="n"/>
+      <c r="AG141" s="15" t="n">
+        <v>-110.536681</v>
+      </c>
+      <c r="AH141" s="15" t="n">
+        <v>-0.006502157705882353</v>
+      </c>
+      <c r="AI141" s="15" t="n">
+        <v>-0.5848501640211641</v>
+      </c>
       <c r="AJ141" s="15" t="n">
-        <v>-47984.11871087</v>
+        <v>-48094.65539187</v>
       </c>
       <c r="AK141" s="15" t="n">
-        <v>-2.82259521828647</v>
+        <v>-2.829097375992352</v>
       </c>
       <c r="AL141" s="15" t="n">
-        <v>-253.8842259834391</v>
+        <v>-254.4690761474603</v>
       </c>
     </row>
     <row r="142">
@@ -26706,17 +27048,23 @@
       <c r="AF149" s="11" t="n">
         <v>-0.1070750670899471</v>
       </c>
-      <c r="AG149" s="11" t="n"/>
-      <c r="AH149" s="11" t="n"/>
-      <c r="AI149" s="11" t="n"/>
+      <c r="AG149" s="11" t="n">
+        <v>-0.0157</v>
+      </c>
+      <c r="AH149" s="11" t="n">
+        <v>-9.235294117647058e-07</v>
+      </c>
+      <c r="AI149" s="11" t="n">
+        <v>-8.306878306878306e-05</v>
+      </c>
       <c r="AJ149" s="11" t="n">
-        <v>-20.23718768</v>
+        <v>-20.25288768</v>
       </c>
       <c r="AK149" s="11" t="n">
-        <v>-0.001190422804705882</v>
+        <v>-0.001191346334117647</v>
       </c>
       <c r="AL149" s="11" t="n">
-        <v>-0.1070750670899471</v>
+        <v>-0.1071581358730159</v>
       </c>
     </row>
     <row r="150">
@@ -27228,17 +27576,23 @@
       <c r="AF155" s="15" t="n">
         <v>-33.08505460883597</v>
       </c>
-      <c r="AG155" s="15" t="n"/>
-      <c r="AH155" s="15" t="n"/>
-      <c r="AI155" s="15" t="n"/>
+      <c r="AG155" s="15" t="n">
+        <v>-0.0157</v>
+      </c>
+      <c r="AH155" s="15" t="n">
+        <v>-9.235294117647058e-07</v>
+      </c>
+      <c r="AI155" s="15" t="n">
+        <v>-8.306878306878306e-05</v>
+      </c>
       <c r="AJ155" s="15" t="n">
-        <v>-6253.07532107</v>
+        <v>-6253.09102107</v>
       </c>
       <c r="AK155" s="15" t="n">
-        <v>-0.3678279600629413</v>
+        <v>-0.3678288835923531</v>
       </c>
       <c r="AL155" s="15" t="n">
-        <v>-33.08505460883597</v>
+        <v>-33.08513767761904</v>
       </c>
     </row>
     <row r="156">
@@ -27337,17 +27691,23 @@
       <c r="AF156" s="19" t="n">
         <v>-1609.397741344391</v>
       </c>
-      <c r="AG156" s="19" t="n"/>
-      <c r="AH156" s="19" t="n"/>
-      <c r="AI156" s="19" t="n"/>
+      <c r="AG156" s="19" t="n">
+        <v>-1880.249274</v>
+      </c>
+      <c r="AH156" s="19" t="n">
+        <v>-0.1106028984705882</v>
+      </c>
+      <c r="AI156" s="19" t="n">
+        <v>-9.948408857142857</v>
+      </c>
       <c r="AJ156" s="19" t="n">
-        <v>-304176.1731140899</v>
+        <v>-306056.4223880899</v>
       </c>
       <c r="AK156" s="19" t="n">
-        <v>-17.89271606553471</v>
+        <v>-18.0033189640053</v>
       </c>
       <c r="AL156" s="19" t="n">
-        <v>-1609.397741344391</v>
+        <v>-1619.346150201534</v>
       </c>
     </row>
     <row r="157">
@@ -27447,22 +27807,22 @@
         <v>-277.2179185799472</v>
       </c>
       <c r="AG157" s="19" t="n">
-        <v>0.623</v>
+        <v>-139.626518</v>
       </c>
       <c r="AH157" s="19" t="n">
-        <v>3.664705882352941e-05</v>
+        <v>-0.008213324588235295</v>
       </c>
       <c r="AI157" s="19" t="n">
-        <v>0.003296296296296296</v>
+        <v>-0.7387646455026455</v>
       </c>
       <c r="AJ157" s="19" t="n">
-        <v>-52393.56361161001</v>
+        <v>-52533.81312961001</v>
       </c>
       <c r="AK157" s="19" t="n">
-        <v>-3.081974330094707</v>
+        <v>-3.090224301741766</v>
       </c>
       <c r="AL157" s="19" t="n">
-        <v>-277.2146222836509</v>
+        <v>-277.9566832254499</v>
       </c>
     </row>
     <row r="158">
@@ -27562,22 +27922,22 @@
         <v>79.78557785582009</v>
       </c>
       <c r="AG158" s="7" t="n">
-        <v>15080.09721475</v>
+        <v>14939.84769675</v>
       </c>
       <c r="AH158" s="7" t="n">
-        <v>0.8870645420441176</v>
+        <v>0.8788145703970587</v>
       </c>
       <c r="AI158" s="7" t="n">
-        <v>79.78887415211639</v>
+        <v>79.04681321031745</v>
       </c>
       <c r="AJ158" s="7" t="n">
-        <v>15080.09721475</v>
+        <v>14939.84769675</v>
       </c>
       <c r="AK158" s="7" t="n">
-        <v>0.8870645420441176</v>
+        <v>0.8788145703970587</v>
       </c>
       <c r="AL158" s="7" t="n">
-        <v>79.78887415211639</v>
+        <v>79.04681321031745</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Tue 10/06/2026  9:50
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -734,7 +734,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 02 Oct 2026 17:26</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 06 Oct 2026 09:50</t>
         </is>
       </c>
     </row>
@@ -816,14 +816,14 @@
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 02 Oct 2026</t>
+          <t>MTD as of 06 Oct 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
       <c r="AI3" s="4" t="n"/>
       <c r="AJ3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 02 Oct 2026</t>
+          <t>YTD as of 06 Oct 2026</t>
         </is>
       </c>
       <c r="AK3" s="4" t="n"/>
@@ -1267,22 +1267,22 @@
         <v>1066081968.222222</v>
       </c>
       <c r="AG7" s="11" t="n">
-        <v>1739093256</v>
+        <v>6339231148</v>
       </c>
       <c r="AH7" s="11" t="n">
-        <v>102299.6032941177</v>
+        <v>372895.949882353</v>
       </c>
       <c r="AI7" s="11" t="n">
-        <v>9201551.619047619</v>
+        <v>33540905.54497354</v>
       </c>
       <c r="AJ7" s="11" t="n">
-        <v>203228585250</v>
+        <v>207828723142</v>
       </c>
       <c r="AK7" s="11" t="n">
-        <v>11954622.66176471</v>
+        <v>12225219.00835294</v>
       </c>
       <c r="AL7" s="11" t="n">
-        <v>1075283519.84127</v>
+        <v>1099622873.767196</v>
       </c>
     </row>
     <row r="8">
@@ -1569,17 +1569,23 @@
       <c r="AF10" s="13" t="n">
         <v>236382957.1746032</v>
       </c>
-      <c r="AG10" s="13" t="n"/>
-      <c r="AH10" s="13" t="n"/>
-      <c r="AI10" s="13" t="n"/>
+      <c r="AG10" s="13" t="n">
+        <v>4600137892</v>
+      </c>
+      <c r="AH10" s="13" t="n">
+        <v>270596.3465882353</v>
+      </c>
+      <c r="AI10" s="13" t="n">
+        <v>24339353.92592593</v>
+      </c>
       <c r="AJ10" s="13" t="n">
-        <v>44676378906</v>
+        <v>49276516798</v>
       </c>
       <c r="AK10" s="13" t="n">
-        <v>2628022.288588235</v>
+        <v>2898618.635176471</v>
       </c>
       <c r="AL10" s="13" t="n">
-        <v>236382957.1746032</v>
+        <v>260722311.1005291</v>
       </c>
     </row>
     <row r="11">
@@ -2318,22 +2324,22 @@
         <v>2521134.965502645</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>1529500</v>
+        <v>2649500</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>89.97058823529412</v>
+        <v>155.8529411764706</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>8092.592592592592</v>
+        <v>14018.51851851852</v>
       </c>
       <c r="AJ20" s="13" t="n">
-        <v>478024008.48</v>
+        <v>479144008.48</v>
       </c>
       <c r="AK20" s="13" t="n">
-        <v>28119.05932235294</v>
+        <v>28184.94167529412</v>
       </c>
       <c r="AL20" s="13" t="n">
-        <v>2529227.558095238</v>
+        <v>2535153.484021164</v>
       </c>
     </row>
     <row r="21">
@@ -2591,22 +2597,22 @@
         <v>491976.1904761905</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>1529500</v>
+        <v>2649500</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>89.97058823529412</v>
+        <v>155.8529411764706</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>8092.592592592592</v>
+        <v>14018.51851851852</v>
       </c>
       <c r="AJ23" s="11" t="n">
-        <v>94513000</v>
+        <v>95633000</v>
       </c>
       <c r="AK23" s="11" t="n">
-        <v>5559.588235294117</v>
+        <v>5625.470588235294</v>
       </c>
       <c r="AL23" s="11" t="n">
-        <v>500068.7830687831</v>
+        <v>505994.708994709</v>
       </c>
     </row>
     <row r="24">
@@ -4131,22 +4137,22 @@
         <v>1332179822.764445</v>
       </c>
       <c r="AG45" s="15" t="n">
-        <v>1740622756</v>
+        <v>6341880648</v>
       </c>
       <c r="AH45" s="15" t="n">
-        <v>102389.5738823529</v>
+        <v>373051.8028235294</v>
       </c>
       <c r="AI45" s="15" t="n">
-        <v>9209644.211640211</v>
+        <v>33554924.06349207</v>
       </c>
       <c r="AJ45" s="15" t="n">
-        <v>253522609258.48</v>
+        <v>258123867150.48</v>
       </c>
       <c r="AK45" s="15" t="n">
-        <v>14913094.66226353</v>
+        <v>15183756.89120471</v>
       </c>
       <c r="AL45" s="15" t="n">
-        <v>1341389466.976085</v>
+        <v>1365734746.827937</v>
       </c>
     </row>
     <row r="46">
@@ -13657,22 +13663,22 @@
         <v>-277217918.5799472</v>
       </c>
       <c r="AG157" s="19" t="n">
-        <v>-139626518</v>
+        <v>4461631374</v>
       </c>
       <c r="AH157" s="19" t="n">
-        <v>-8213.324588235295</v>
+        <v>262448.9043529412</v>
       </c>
       <c r="AI157" s="19" t="n">
-        <v>-738764.6455026455</v>
+        <v>23606515.20634921</v>
       </c>
       <c r="AJ157" s="19" t="n">
-        <v>-52533813129.61</v>
+        <v>-47932555237.61</v>
       </c>
       <c r="AK157" s="19" t="n">
-        <v>-3090224.301741766</v>
+        <v>-2819562.072800589</v>
       </c>
       <c r="AL157" s="19" t="n">
-        <v>-277956683.2254499</v>
+        <v>-253611403.373598</v>
       </c>
     </row>
     <row r="158">
@@ -13772,22 +13778,22 @@
         <v>79785577.85582009</v>
       </c>
       <c r="AG158" s="7" t="n">
-        <v>14939847696.75</v>
+        <v>19541105588.75</v>
       </c>
       <c r="AH158" s="7" t="n">
-        <v>878814.5703970587</v>
+        <v>1149476.799338235</v>
       </c>
       <c r="AI158" s="7" t="n">
-        <v>79046813.21031745</v>
+        <v>103392093.0621693</v>
       </c>
       <c r="AJ158" s="7" t="n">
-        <v>14939847696.75</v>
+        <v>19541105588.75</v>
       </c>
       <c r="AK158" s="7" t="n">
-        <v>878814.5703970587</v>
+        <v>1149476.799338235</v>
       </c>
       <c r="AL158" s="7" t="n">
-        <v>79046813.21031745</v>
+        <v>103392093.0621693</v>
       </c>
     </row>
   </sheetData>
@@ -14590,16 +14596,16 @@
         <v>14828882907</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>-141156018</v>
+        <v>4458981874</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>14687726889</v>
+        <v>19287864781</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>863983.9346470588</v>
+        <v>1134580.281235294</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>77712840.68253969</v>
+        <v>102052194.6084656</v>
       </c>
     </row>
     <row r="7">
@@ -14686,16 +14692,16 @@
         <v>22400563.84000001</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>1504500</v>
+        <v>2624500</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>23905063.84000001</v>
+        <v>25025063.84000001</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>1406.180225882354</v>
+        <v>1472.06257882353</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>126481.8192592593</v>
+        <v>132407.7451851853</v>
       </c>
     </row>
     <row r="10">
@@ -14805,13 +14811,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>14939847698.75</v>
+        <v>19541105590.75</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>878814.5705147057</v>
+        <v>1149476.799455883</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>79046813.22089946</v>
+        <v>103392093.0727513</v>
       </c>
     </row>
   </sheetData>
@@ -14884,7 +14890,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 02 Oct 2026 17:26 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 06 Oct 2026 09:50 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -14966,14 +14972,14 @@
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 02 Oct 2026</t>
+          <t>MTD as of 06 Oct 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
       <c r="AI3" s="4" t="n"/>
       <c r="AJ3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 02 Oct 2026</t>
+          <t>YTD as of 06 Oct 2026</t>
         </is>
       </c>
       <c r="AK3" s="4" t="n"/>
@@ -15417,22 +15423,22 @@
         <v>1066.081968222222</v>
       </c>
       <c r="AG7" s="11" t="n">
-        <v>1739.093256</v>
+        <v>6339.231148</v>
       </c>
       <c r="AH7" s="11" t="n">
-        <v>0.1022996032941176</v>
+        <v>0.3728959498823529</v>
       </c>
       <c r="AI7" s="11" t="n">
-        <v>9.201551619047619</v>
+        <v>33.54090554497355</v>
       </c>
       <c r="AJ7" s="11" t="n">
-        <v>203228.58525</v>
+        <v>207828.723142</v>
       </c>
       <c r="AK7" s="11" t="n">
-        <v>11.9546226617647</v>
+        <v>12.22521900835294</v>
       </c>
       <c r="AL7" s="11" t="n">
-        <v>1075.28351984127</v>
+        <v>1099.622873767196</v>
       </c>
     </row>
     <row r="8">
@@ -15719,17 +15725,23 @@
       <c r="AF10" s="13" t="n">
         <v>236.3829571746032</v>
       </c>
-      <c r="AG10" s="13" t="n"/>
-      <c r="AH10" s="13" t="n"/>
-      <c r="AI10" s="13" t="n"/>
+      <c r="AG10" s="13" t="n">
+        <v>4600.137892</v>
+      </c>
+      <c r="AH10" s="13" t="n">
+        <v>0.2705963465882353</v>
+      </c>
+      <c r="AI10" s="13" t="n">
+        <v>24.33935392592592</v>
+      </c>
       <c r="AJ10" s="13" t="n">
-        <v>44676.378906</v>
+        <v>49276.516798</v>
       </c>
       <c r="AK10" s="13" t="n">
-        <v>2.628022288588235</v>
+        <v>2.89861863517647</v>
       </c>
       <c r="AL10" s="13" t="n">
-        <v>236.3829571746032</v>
+        <v>260.7223111005291</v>
       </c>
     </row>
     <row r="11">
@@ -16468,22 +16480,22 @@
         <v>2.521134965502646</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>1.5295</v>
+        <v>2.6495</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>8.997058823529413e-05</v>
+        <v>0.0001558529411764706</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>0.008092592592592592</v>
+        <v>0.01401851851851852</v>
       </c>
       <c r="AJ20" s="13" t="n">
-        <v>478.02400848</v>
+        <v>479.14400848</v>
       </c>
       <c r="AK20" s="13" t="n">
-        <v>0.02811905932235294</v>
+        <v>0.02818494167529412</v>
       </c>
       <c r="AL20" s="13" t="n">
-        <v>2.529227558095239</v>
+        <v>2.535153484021164</v>
       </c>
     </row>
     <row r="21">
@@ -16741,22 +16753,22 @@
         <v>0.4919761904761905</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>1.5295</v>
+        <v>2.6495</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>8.997058823529413e-05</v>
+        <v>0.0001558529411764706</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>0.008092592592592592</v>
+        <v>0.01401851851851852</v>
       </c>
       <c r="AJ23" s="11" t="n">
-        <v>94.51300000000001</v>
+        <v>95.63300000000001</v>
       </c>
       <c r="AK23" s="11" t="n">
-        <v>0.005559588235294118</v>
+        <v>0.005625470588235295</v>
       </c>
       <c r="AL23" s="11" t="n">
-        <v>0.500068783068783</v>
+        <v>0.505994708994709</v>
       </c>
     </row>
     <row r="24">
@@ -18281,22 +18293,22 @@
         <v>1332.179822764444</v>
       </c>
       <c r="AG45" s="15" t="n">
-        <v>1740.622756</v>
+        <v>6341.880648</v>
       </c>
       <c r="AH45" s="15" t="n">
-        <v>0.1023895738823529</v>
+        <v>0.3730518028235295</v>
       </c>
       <c r="AI45" s="15" t="n">
-        <v>9.209644211640212</v>
+        <v>33.55492406349207</v>
       </c>
       <c r="AJ45" s="15" t="n">
-        <v>253522.60925848</v>
+        <v>258123.86715048</v>
       </c>
       <c r="AK45" s="15" t="n">
-        <v>14.91309466226353</v>
+        <v>15.1837568912047</v>
       </c>
       <c r="AL45" s="15" t="n">
-        <v>1341.389466976085</v>
+        <v>1365.734746827937</v>
       </c>
     </row>
     <row r="46">
@@ -27807,22 +27819,22 @@
         <v>-277.2179185799472</v>
       </c>
       <c r="AG157" s="19" t="n">
-        <v>-139.626518</v>
+        <v>4461.631374</v>
       </c>
       <c r="AH157" s="19" t="n">
-        <v>-0.008213324588235295</v>
+        <v>0.2624489043529412</v>
       </c>
       <c r="AI157" s="19" t="n">
-        <v>-0.7387646455026455</v>
+        <v>23.6065152063492</v>
       </c>
       <c r="AJ157" s="19" t="n">
-        <v>-52533.81312961001</v>
+        <v>-47932.55523761002</v>
       </c>
       <c r="AK157" s="19" t="n">
-        <v>-3.090224301741766</v>
+        <v>-2.819562072800589</v>
       </c>
       <c r="AL157" s="19" t="n">
-        <v>-277.9566832254499</v>
+        <v>-253.611403373598</v>
       </c>
     </row>
     <row r="158">
@@ -27922,22 +27934,22 @@
         <v>79.78557785582009</v>
       </c>
       <c r="AG158" s="7" t="n">
-        <v>14939.84769675</v>
+        <v>19541.10558875</v>
       </c>
       <c r="AH158" s="7" t="n">
-        <v>0.8788145703970587</v>
+        <v>1.149476799338235</v>
       </c>
       <c r="AI158" s="7" t="n">
-        <v>79.04681321031745</v>
+        <v>103.3920930621693</v>
       </c>
       <c r="AJ158" s="7" t="n">
-        <v>14939.84769675</v>
+        <v>19541.10558875</v>
       </c>
       <c r="AK158" s="7" t="n">
-        <v>0.8788145703970587</v>
+        <v>1.149476799338235</v>
       </c>
       <c r="AL158" s="7" t="n">
-        <v>79.04681321031745</v>
+        <v>103.3920930621693</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Tue 10/06/2026 10:05
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -734,7 +734,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 06 Oct 2026 09:50</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 06 Oct 2026 10:05</t>
         </is>
       </c>
     </row>
@@ -14890,7 +14890,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 06 Oct 2026 09:50 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 06 Oct 2026 10:05 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Tue 10/06/2026 16:19
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -681,7 +681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:AL158"/>
+  <dimension ref="B1:AL159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -734,7 +734,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 06 Oct 2026 10:05</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 06 Oct 2026 16:19</t>
         </is>
       </c>
     </row>
@@ -2324,22 +2324,22 @@
         <v>2521134.965502645</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>2649500</v>
+        <v>3223500</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>155.8529411764706</v>
+        <v>189.6176470588235</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>14018.51851851852</v>
+        <v>17055.55555555555</v>
       </c>
       <c r="AJ20" s="13" t="n">
-        <v>479144008.48</v>
+        <v>479718008.48</v>
       </c>
       <c r="AK20" s="13" t="n">
-        <v>28184.94167529412</v>
+        <v>28218.70638117647</v>
       </c>
       <c r="AL20" s="13" t="n">
-        <v>2535153.484021164</v>
+        <v>2538190.521058201</v>
       </c>
     </row>
     <row r="21">
@@ -2597,22 +2597,22 @@
         <v>491976.1904761905</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>2649500</v>
+        <v>3223500</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>155.8529411764706</v>
+        <v>189.6176470588235</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>14018.51851851852</v>
+        <v>17055.55555555555</v>
       </c>
       <c r="AJ23" s="11" t="n">
-        <v>95633000</v>
+        <v>96207000</v>
       </c>
       <c r="AK23" s="11" t="n">
-        <v>5625.470588235294</v>
+        <v>5659.235294117647</v>
       </c>
       <c r="AL23" s="11" t="n">
-        <v>505994.708994709</v>
+        <v>509031.746031746</v>
       </c>
     </row>
     <row r="24">
@@ -4137,22 +4137,22 @@
         <v>1332179822.764445</v>
       </c>
       <c r="AG45" s="15" t="n">
-        <v>6341880648</v>
+        <v>6342454648</v>
       </c>
       <c r="AH45" s="15" t="n">
-        <v>373051.8028235294</v>
+        <v>373085.5675294118</v>
       </c>
       <c r="AI45" s="15" t="n">
-        <v>33554924.06349207</v>
+        <v>33557961.1005291</v>
       </c>
       <c r="AJ45" s="15" t="n">
-        <v>258123867150.48</v>
+        <v>258124441150.48</v>
       </c>
       <c r="AK45" s="15" t="n">
-        <v>15183756.89120471</v>
+        <v>15183790.65591059</v>
       </c>
       <c r="AL45" s="15" t="n">
-        <v>1365734746.827937</v>
+        <v>1365737783.864974</v>
       </c>
     </row>
     <row r="46">
@@ -6681,40 +6681,40 @@
         <v>-2937621.931216931</v>
       </c>
       <c r="AA81" s="11" t="n">
-        <v>-3351184276</v>
+        <v>-3383684276</v>
       </c>
       <c r="AB81" s="11" t="n">
-        <v>-197128.4868235294</v>
+        <v>-199040.2515294118</v>
       </c>
       <c r="AC81" s="11" t="n">
-        <v>-17731133.73544974</v>
+        <v>-17903091.40740741</v>
       </c>
       <c r="AD81" s="11" t="n">
-        <v>-9987402249</v>
+        <v>-10019902249</v>
       </c>
       <c r="AE81" s="11" t="n">
-        <v>-587494.2499411764</v>
+        <v>-589406.0146470587</v>
       </c>
       <c r="AF81" s="11" t="n">
-        <v>-52843398.14285713</v>
+        <v>-53015355.81481481</v>
       </c>
       <c r="AG81" s="11" t="n">
-        <v>-870978933</v>
+        <v>-890478933</v>
       </c>
       <c r="AH81" s="11" t="n">
-        <v>-51234.05488235294</v>
+        <v>-52381.11370588235</v>
       </c>
       <c r="AI81" s="11" t="n">
-        <v>-4608354.142857143</v>
+        <v>-4711528.746031746</v>
       </c>
       <c r="AJ81" s="11" t="n">
-        <v>-10858381182</v>
+        <v>-10910381182</v>
       </c>
       <c r="AK81" s="11" t="n">
-        <v>-638728.3048235293</v>
+        <v>-641787.128352941</v>
       </c>
       <c r="AL81" s="11" t="n">
-        <v>-57451752.28571428</v>
+        <v>-57726884.56084655</v>
       </c>
     </row>
     <row r="82">
@@ -7135,40 +7135,40 @@
         <v>-21921095.57671958</v>
       </c>
       <c r="AA85" s="15" t="n">
-        <v>-8309778530.73</v>
+        <v>-8342278530.73</v>
       </c>
       <c r="AB85" s="15" t="n">
-        <v>-488810.5018076471</v>
+        <v>-490722.2665135294</v>
       </c>
       <c r="AC85" s="15" t="n">
-        <v>-43967082.1731746</v>
+        <v>-44139039.84513228</v>
       </c>
       <c r="AD85" s="15" t="n">
-        <v>-32186946905.27</v>
+        <v>-32219446905.27</v>
       </c>
       <c r="AE85" s="15" t="n">
-        <v>-1893349.817957059</v>
+        <v>-1895261.582662941</v>
       </c>
       <c r="AF85" s="15" t="n">
-        <v>-170301306.3770899</v>
+        <v>-170473264.0490476</v>
       </c>
       <c r="AG85" s="15" t="n">
-        <v>-1769696893</v>
+        <v>-1789196893</v>
       </c>
       <c r="AH85" s="15" t="n">
-        <v>-104099.8172352941</v>
+        <v>-105246.8760588235</v>
       </c>
       <c r="AI85" s="15" t="n">
-        <v>-9363475.624338625</v>
+        <v>-9466650.227513228</v>
       </c>
       <c r="AJ85" s="15" t="n">
-        <v>-33956643798.27</v>
+        <v>-34008643798.27</v>
       </c>
       <c r="AK85" s="15" t="n">
-        <v>-1997449.635192353</v>
+        <v>-2000508.458721765</v>
       </c>
       <c r="AL85" s="15" t="n">
-        <v>-179664782.0014286</v>
+        <v>-179939914.2765609</v>
       </c>
     </row>
     <row r="86">
@@ -10910,106 +10910,106 @@
         </is>
       </c>
       <c r="C128" s="13" t="n">
-        <v>-22722669.31</v>
+        <v>-22591057</v>
       </c>
       <c r="D128" s="13" t="n">
-        <v>-1336.627606470588</v>
+        <v>-1328.885705882353</v>
       </c>
       <c r="E128" s="13" t="n">
-        <v>-120225.7635449735</v>
+        <v>-119529.4021164021</v>
       </c>
       <c r="F128" s="13" t="n">
-        <v>-216848378.34</v>
+        <v>-216595653</v>
       </c>
       <c r="G128" s="13" t="n">
-        <v>-12755.78696117647</v>
+        <v>-12740.92076470588</v>
       </c>
       <c r="H128" s="13" t="n">
-        <v>-1147345.917142857</v>
+        <v>-1146008.746031746</v>
       </c>
       <c r="I128" s="13" t="n">
-        <v>-1486783</v>
+        <v>-1408413</v>
       </c>
       <c r="J128" s="13" t="n">
-        <v>-87.45782352941177</v>
+        <v>-82.84782352941177</v>
       </c>
       <c r="K128" s="13" t="n">
-        <v>-7866.576719576719</v>
+        <v>-7451.920634920635</v>
       </c>
       <c r="L128" s="13" t="n">
-        <v>-218357245.06</v>
+        <v>-218312249</v>
       </c>
       <c r="M128" s="13" t="n">
-        <v>-12844.54382705882</v>
+        <v>-12841.897</v>
       </c>
       <c r="N128" s="13" t="n">
-        <v>-1155329.338941799</v>
+        <v>-1155091.264550264</v>
       </c>
       <c r="O128" s="13" t="n">
-        <v>-1552948.4</v>
+        <v>-1549043</v>
       </c>
       <c r="P128" s="13" t="n">
-        <v>-91.34990588235294</v>
+        <v>-91.12017647058823</v>
       </c>
       <c r="Q128" s="13" t="n">
-        <v>-8216.658201058201</v>
+        <v>-8195.994708994709</v>
       </c>
       <c r="R128" s="13" t="n">
-        <v>-242858353.36</v>
+        <v>-242651498</v>
       </c>
       <c r="S128" s="13" t="n">
-        <v>-14285.78549176471</v>
+        <v>-14273.61752941176</v>
       </c>
       <c r="T128" s="13" t="n">
-        <v>-1284964.832592593</v>
+        <v>-1283870.35978836</v>
       </c>
       <c r="U128" s="13" t="n">
-        <v>-243434747.94</v>
+        <v>-243375606</v>
       </c>
       <c r="V128" s="13" t="n">
-        <v>-14319.69105529412</v>
+        <v>-14316.21211764706</v>
       </c>
       <c r="W128" s="13" t="n">
-        <v>-1288014.539365079</v>
+        <v>-1287701.619047619</v>
       </c>
       <c r="X128" s="13" t="n">
-        <v>-10932618.12</v>
+        <v>-10873033</v>
       </c>
       <c r="Y128" s="13" t="n">
-        <v>-643.0951835294118</v>
+        <v>-639.5901764705883</v>
       </c>
       <c r="Z128" s="13" t="n">
-        <v>-57844.54031746032</v>
+        <v>-57529.27513227514</v>
       </c>
       <c r="AA128" s="13" t="n">
-        <v>-373796010.17</v>
+        <v>-373713050</v>
       </c>
       <c r="AB128" s="13" t="n">
-        <v>-21988.00059823529</v>
+        <v>-21983.1205882353</v>
       </c>
       <c r="AC128" s="13" t="n">
-        <v>-1977756.667566137</v>
+        <v>-1977317.724867725</v>
       </c>
       <c r="AD128" s="13" t="n">
-        <v>-1331989753.7</v>
+        <v>-1331069602</v>
       </c>
       <c r="AE128" s="13" t="n">
-        <v>-78352.33845294119</v>
+        <v>-78298.21188235295</v>
       </c>
       <c r="AF128" s="13" t="n">
-        <v>-7047564.834391533</v>
+        <v>-7042696.306878306</v>
       </c>
       <c r="AG128" s="13" t="n"/>
       <c r="AH128" s="13" t="n"/>
       <c r="AI128" s="13" t="n"/>
       <c r="AJ128" s="13" t="n">
-        <v>-1331989753.7</v>
+        <v>-1331069602</v>
       </c>
       <c r="AK128" s="13" t="n">
-        <v>-78352.33845294119</v>
+        <v>-78298.21188235295</v>
       </c>
       <c r="AL128" s="13" t="n">
-        <v>-7047564.834391533</v>
+        <v>-7042696.306878306</v>
       </c>
     </row>
     <row r="129">
@@ -11334,106 +11334,106 @@
         </is>
       </c>
       <c r="C132" s="15" t="n">
-        <v>-5923487425.309999</v>
+        <v>-5923355813</v>
       </c>
       <c r="D132" s="15" t="n">
-        <v>-348440.4367829412</v>
+        <v>-348432.694882353</v>
       </c>
       <c r="E132" s="15" t="n">
-        <v>-31341203.30851851</v>
+        <v>-31340506.94708995</v>
       </c>
       <c r="F132" s="15" t="n">
-        <v>-7548948538.34</v>
+        <v>-7548695813</v>
       </c>
       <c r="G132" s="15" t="n">
-        <v>-444055.7963729412</v>
+        <v>-444040.9301764706</v>
       </c>
       <c r="H132" s="15" t="n">
-        <v>-39941526.6578836</v>
+        <v>-39940189.48677249</v>
       </c>
       <c r="I132" s="15" t="n">
-        <v>-961200171</v>
+        <v>-961121801</v>
       </c>
       <c r="J132" s="15" t="n">
-        <v>-56541.18652941177</v>
+        <v>-56536.57652941177</v>
       </c>
       <c r="K132" s="15" t="n">
-        <v>-5085715.19047619</v>
+        <v>-5085300.534391535</v>
       </c>
       <c r="L132" s="15" t="n">
-        <v>-6466021878.059999</v>
+        <v>-6465976882</v>
       </c>
       <c r="M132" s="15" t="n">
-        <v>-380354.2281211764</v>
+        <v>-380351.5812941177</v>
       </c>
       <c r="N132" s="15" t="n">
-        <v>-34211755.96857142</v>
+        <v>-34211517.8941799</v>
       </c>
       <c r="O132" s="15" t="n">
-        <v>-1318812959.4</v>
+        <v>-1318809054</v>
       </c>
       <c r="P132" s="15" t="n">
-        <v>-77577.23290588235</v>
+        <v>-77577.00317647059</v>
       </c>
       <c r="Q132" s="15" t="n">
-        <v>-6977846.346031747</v>
+        <v>-6977825.682539683</v>
       </c>
       <c r="R132" s="15" t="n">
-        <v>-416258006.36</v>
+        <v>-416051151</v>
       </c>
       <c r="S132" s="15" t="n">
-        <v>-24485.76508</v>
+        <v>-24473.59711764706</v>
       </c>
       <c r="T132" s="15" t="n">
-        <v>-2202423.314074074</v>
+        <v>-2201328.841269841</v>
       </c>
       <c r="U132" s="15" t="n">
-        <v>-1929030552.94</v>
+        <v>-1928971411</v>
       </c>
       <c r="V132" s="15" t="n">
-        <v>-113472.3854670588</v>
+        <v>-113468.9065294118</v>
       </c>
       <c r="W132" s="15" t="n">
-        <v>-10206510.8621164</v>
+        <v>-10206197.94179894</v>
       </c>
       <c r="X132" s="15" t="n">
-        <v>-491673876.12</v>
+        <v>-491614291</v>
       </c>
       <c r="Y132" s="15" t="n">
-        <v>-28921.99271294118</v>
+        <v>-28918.48770588235</v>
       </c>
       <c r="Z132" s="15" t="n">
-        <v>-2601449.08</v>
+        <v>-2601133.814814815</v>
       </c>
       <c r="AA132" s="15" t="n">
-        <v>-1664075995.17</v>
+        <v>-1663993035</v>
       </c>
       <c r="AB132" s="15" t="n">
-        <v>-97886.82324529412</v>
+        <v>-97881.94323529412</v>
       </c>
       <c r="AC132" s="15" t="n">
-        <v>-8804634.895079365</v>
+        <v>-8804195.952380951</v>
       </c>
       <c r="AD132" s="15" t="n">
-        <v>-26719509402.7</v>
+        <v>-26718589251</v>
       </c>
       <c r="AE132" s="15" t="n">
-        <v>-1571735.847217647</v>
+        <v>-1571681.720647059</v>
       </c>
       <c r="AF132" s="15" t="n">
-        <v>-141373065.6227513</v>
+        <v>-141368197.0952381</v>
       </c>
       <c r="AG132" s="15" t="n"/>
       <c r="AH132" s="15" t="n"/>
       <c r="AI132" s="15" t="n"/>
       <c r="AJ132" s="15" t="n">
-        <v>-26719509402.7</v>
+        <v>-26718589251</v>
       </c>
       <c r="AK132" s="15" t="n">
-        <v>-1571735.847217647</v>
+        <v>-1571681.720647059</v>
       </c>
       <c r="AL132" s="15" t="n">
-        <v>-141373065.6227513</v>
+        <v>-141368197.0952381</v>
       </c>
     </row>
     <row r="133">
@@ -12189,94 +12189,94 @@
         </is>
       </c>
       <c r="C141" s="15" t="n">
-        <v>-8603850102.309999</v>
+        <v>-8603718490</v>
       </c>
       <c r="D141" s="15" t="n">
-        <v>-506108.829547647</v>
+        <v>-506101.0876470588</v>
       </c>
       <c r="E141" s="15" t="n">
-        <v>-45523016.41433862</v>
+        <v>-45522320.05291005</v>
       </c>
       <c r="F141" s="15" t="n">
-        <v>-10106099580.34</v>
+        <v>-10105846855</v>
       </c>
       <c r="G141" s="15" t="n">
-        <v>-594476.4459023529</v>
+        <v>-594461.5797058824</v>
       </c>
       <c r="H141" s="15" t="n">
-        <v>-53471426.35100529</v>
+        <v>-53470089.17989418</v>
       </c>
       <c r="I141" s="15" t="n">
-        <v>-2763428661</v>
+        <v>-2763350291</v>
       </c>
       <c r="J141" s="15" t="n">
-        <v>-162554.6271176471</v>
+        <v>-162550.017117647</v>
       </c>
       <c r="K141" s="15" t="n">
-        <v>-14621315.66666667</v>
+        <v>-14620901.01058201</v>
       </c>
       <c r="L141" s="15" t="n">
-        <v>-8658626831.059999</v>
+        <v>-8658581835</v>
       </c>
       <c r="M141" s="15" t="n">
-        <v>-509330.9900623529</v>
+        <v>-509328.3432352941</v>
       </c>
       <c r="N141" s="15" t="n">
-        <v>-45812840.37597883</v>
+        <v>-45812602.3015873</v>
       </c>
       <c r="O141" s="15" t="n">
-        <v>-2654292760.86</v>
+        <v>-2654288855.46</v>
       </c>
       <c r="P141" s="15" t="n">
-        <v>-156134.8682858824</v>
+        <v>-156134.6385564706</v>
       </c>
       <c r="Q141" s="15" t="n">
-        <v>-14043877.0415873</v>
+        <v>-14043856.37809524</v>
       </c>
       <c r="R141" s="15" t="n">
-        <v>-3460373168.8</v>
+        <v>-3460166313.44</v>
       </c>
       <c r="S141" s="15" t="n">
-        <v>-203551.3628705883</v>
+        <v>-203539.1949082353</v>
       </c>
       <c r="T141" s="15" t="n">
-        <v>-18308852.74497355</v>
+        <v>-18307758.27216931</v>
       </c>
       <c r="U141" s="15" t="n">
-        <v>-4043270117.94</v>
+        <v>-4043210976</v>
       </c>
       <c r="V141" s="15" t="n">
-        <v>-237839.4187023529</v>
+        <v>-237835.9397647059</v>
       </c>
       <c r="W141" s="15" t="n">
-        <v>-21392963.58698413</v>
+        <v>-21392650.66666667</v>
       </c>
       <c r="X141" s="15" t="n">
-        <v>-3232210122.12</v>
+        <v>-3232150537</v>
       </c>
       <c r="Y141" s="15" t="n">
-        <v>-190130.0071835294</v>
+        <v>-190126.5021764706</v>
       </c>
       <c r="Z141" s="15" t="n">
-        <v>-17101640.85777778</v>
+        <v>-17101325.59259259</v>
       </c>
       <c r="AA141" s="15" t="n">
-        <v>-4461967366.440001</v>
+        <v>-4461884406.27</v>
       </c>
       <c r="AB141" s="15" t="n">
-        <v>-262468.6686141177</v>
+        <v>-262463.7886041177</v>
       </c>
       <c r="AC141" s="15" t="n">
-        <v>-23608292.94412699</v>
+        <v>-23607854.00142857</v>
       </c>
       <c r="AD141" s="15" t="n">
-        <v>-47984118710.87001</v>
+        <v>-47983198559.17</v>
       </c>
       <c r="AE141" s="15" t="n">
-        <v>-2822595.218286471</v>
+        <v>-2822541.091715883</v>
       </c>
       <c r="AF141" s="15" t="n">
-        <v>-253884225.9834391</v>
+        <v>-253879357.4559259</v>
       </c>
       <c r="AG141" s="15" t="n">
         <v>-110536681</v>
@@ -12288,13 +12288,13 @@
         <v>-584850.1640211641</v>
       </c>
       <c r="AJ141" s="15" t="n">
-        <v>-48094655391.87001</v>
+        <v>-48093735240.17</v>
       </c>
       <c r="AK141" s="15" t="n">
-        <v>-2829097.375992353</v>
+        <v>-2829043.249421765</v>
       </c>
       <c r="AL141" s="15" t="n">
-        <v>-254469076.1474603</v>
+        <v>-254464207.6199471</v>
       </c>
     </row>
     <row r="142">
@@ -12504,34 +12504,34 @@
         <v>-1038657.989417989</v>
       </c>
       <c r="AA144" s="13" t="n">
-        <v>-105582868</v>
+        <v>-73082868</v>
       </c>
       <c r="AB144" s="13" t="n">
-        <v>-6210.756941176471</v>
+        <v>-4298.992235294118</v>
       </c>
       <c r="AC144" s="13" t="n">
-        <v>-558639.5132275132</v>
+        <v>-386681.8412698412</v>
       </c>
       <c r="AD144" s="13" t="n">
-        <v>-1030660283</v>
+        <v>-998160283</v>
       </c>
       <c r="AE144" s="13" t="n">
-        <v>-60627.07547058824</v>
+        <v>-58715.31076470588</v>
       </c>
       <c r="AF144" s="13" t="n">
-        <v>-5453229.01058201</v>
+        <v>-5281271.338624339</v>
       </c>
       <c r="AG144" s="13" t="n"/>
       <c r="AH144" s="13" t="n"/>
       <c r="AI144" s="13" t="n"/>
       <c r="AJ144" s="13" t="n">
-        <v>-1030660283</v>
+        <v>-998160283</v>
       </c>
       <c r="AK144" s="13" t="n">
-        <v>-60627.07547058824</v>
+        <v>-58715.31076470588</v>
       </c>
       <c r="AL144" s="13" t="n">
-        <v>-5453229.01058201</v>
+        <v>-5281271.338624339</v>
       </c>
     </row>
     <row r="145">
@@ -12735,34 +12735,34 @@
         <v>-1038657.989417989</v>
       </c>
       <c r="AA147" s="15" t="n">
-        <v>-105582868</v>
+        <v>-73082868</v>
       </c>
       <c r="AB147" s="15" t="n">
-        <v>-6210.756941176471</v>
+        <v>-4298.992235294118</v>
       </c>
       <c r="AC147" s="15" t="n">
-        <v>-558639.5132275132</v>
+        <v>-386681.8412698412</v>
       </c>
       <c r="AD147" s="15" t="n">
-        <v>-2701773283</v>
+        <v>-2669273283</v>
       </c>
       <c r="AE147" s="15" t="n">
-        <v>-158927.8401764706</v>
+        <v>-157016.0754705882</v>
       </c>
       <c r="AF147" s="15" t="n">
-        <v>-14295096.73544974</v>
+        <v>-14123139.06349206</v>
       </c>
       <c r="AG147" s="15" t="n"/>
       <c r="AH147" s="15" t="n"/>
       <c r="AI147" s="15" t="n"/>
       <c r="AJ147" s="15" t="n">
-        <v>-2701773283</v>
+        <v>-2669273283</v>
       </c>
       <c r="AK147" s="15" t="n">
-        <v>-158927.8401764706</v>
+        <v>-157016.0754705882</v>
       </c>
       <c r="AL147" s="15" t="n">
-        <v>-14295096.73544974</v>
+        <v>-14123139.06349206</v>
       </c>
     </row>
     <row r="148">
@@ -12905,138 +12905,168 @@
         <v>-107075.0670899471</v>
       </c>
       <c r="AG149" s="11" t="n">
-        <v>-15700</v>
+        <v>-18200</v>
       </c>
       <c r="AH149" s="11" t="n">
-        <v>-0.9235294117647059</v>
+        <v>-1.070588235294118</v>
       </c>
       <c r="AI149" s="11" t="n">
-        <v>-83.06878306878306</v>
+        <v>-96.29629629629629</v>
       </c>
       <c r="AJ149" s="11" t="n">
-        <v>-20252887.68</v>
+        <v>-20255387.68</v>
       </c>
       <c r="AK149" s="11" t="n">
-        <v>-1191.346334117647</v>
+        <v>-1191.493392941176</v>
       </c>
       <c r="AL149" s="11" t="n">
-        <v>-107158.1358730159</v>
+        <v>-107171.3633862434</v>
       </c>
     </row>
     <row r="150">
       <c r="B150" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Bank Provision Charges</t>
-        </is>
-      </c>
-      <c r="C150" s="13" t="n"/>
-      <c r="D150" s="13" t="n"/>
-      <c r="E150" s="13" t="n"/>
-      <c r="F150" s="13" t="n"/>
-      <c r="G150" s="13" t="n"/>
-      <c r="H150" s="13" t="n"/>
+          <t xml:space="preserve">        Bank Interest Income</t>
+        </is>
+      </c>
+      <c r="C150" s="13" t="n">
+        <v>-10741389.75</v>
+      </c>
+      <c r="D150" s="13" t="n">
+        <v>-631.8464558823531</v>
+      </c>
+      <c r="E150" s="13" t="n">
+        <v>-56832.75000000001</v>
+      </c>
+      <c r="F150" s="13" t="n">
+        <v>-13598083.25</v>
+      </c>
+      <c r="G150" s="13" t="n">
+        <v>-799.88725</v>
+      </c>
+      <c r="H150" s="13" t="n">
+        <v>-71947.53042328042</v>
+      </c>
       <c r="I150" s="13" t="n">
-        <v>-19344233</v>
+        <v>-364732.99</v>
       </c>
       <c r="J150" s="13" t="n">
-        <v>-1137.896058823529</v>
+        <v>-21.45488176470588</v>
       </c>
       <c r="K150" s="13" t="n">
-        <v>-102350.4391534391</v>
-      </c>
-      <c r="L150" s="13" t="n"/>
-      <c r="M150" s="13" t="n"/>
-      <c r="N150" s="13" t="n"/>
-      <c r="O150" s="13" t="n"/>
-      <c r="P150" s="13" t="n"/>
-      <c r="Q150" s="13" t="n"/>
+        <v>-1929.80417989418</v>
+      </c>
+      <c r="L150" s="13" t="n">
+        <v>-163549.2</v>
+      </c>
+      <c r="M150" s="13" t="n">
+        <v>-9.620541176470589</v>
+      </c>
+      <c r="N150" s="13" t="n">
+        <v>-865.3396825396826</v>
+      </c>
+      <c r="O150" s="13" t="n">
+        <v>-131477.82</v>
+      </c>
+      <c r="P150" s="13" t="n">
+        <v>-7.733989411764706</v>
+      </c>
+      <c r="Q150" s="13" t="n">
+        <v>-695.6498412698413</v>
+      </c>
       <c r="R150" s="13" t="n">
-        <v>-32669440</v>
+        <v>-395579.03</v>
       </c>
       <c r="S150" s="13" t="n">
-        <v>-1921.731764705882</v>
+        <v>-23.26935470588235</v>
       </c>
       <c r="T150" s="13" t="n">
-        <v>-172854.1798941799</v>
-      </c>
-      <c r="U150" s="13" t="n"/>
-      <c r="V150" s="13" t="n"/>
-      <c r="W150" s="13" t="n"/>
-      <c r="X150" s="13" t="n"/>
-      <c r="Y150" s="13" t="n"/>
-      <c r="Z150" s="13" t="n"/>
-      <c r="AA150" s="13" t="n"/>
-      <c r="AB150" s="13" t="n"/>
-      <c r="AC150" s="13" t="n"/>
+        <v>-2093.01074074074</v>
+      </c>
+      <c r="U150" s="13" t="n">
+        <v>-158551.2</v>
+      </c>
+      <c r="V150" s="13" t="n">
+        <v>-9.326541176470588</v>
+      </c>
+      <c r="W150" s="13" t="n">
+        <v>-838.8952380952381</v>
+      </c>
+      <c r="X150" s="13" t="n">
+        <v>-202489.72</v>
+      </c>
+      <c r="Y150" s="13" t="n">
+        <v>-11.91116</v>
+      </c>
+      <c r="Z150" s="13" t="n">
+        <v>-1071.37417989418</v>
+      </c>
+      <c r="AA150" s="13" t="n">
+        <v>-133356.53</v>
+      </c>
+      <c r="AB150" s="13" t="n">
+        <v>-7.844501764705882</v>
+      </c>
+      <c r="AC150" s="13" t="n">
+        <v>-705.5901058201058</v>
+      </c>
       <c r="AD150" s="13" t="n">
-        <v>-52013673</v>
+        <v>-25889209.49</v>
       </c>
       <c r="AE150" s="13" t="n">
-        <v>-3059.627823529412</v>
+        <v>-1522.894675882353</v>
       </c>
       <c r="AF150" s="13" t="n">
-        <v>-275204.6190476191</v>
+        <v>-136979.9443915344</v>
       </c>
       <c r="AG150" s="13" t="n"/>
       <c r="AH150" s="13" t="n"/>
       <c r="AI150" s="13" t="n"/>
       <c r="AJ150" s="13" t="n">
-        <v>-52013673</v>
+        <v>-25889209.49</v>
       </c>
       <c r="AK150" s="13" t="n">
-        <v>-3059.627823529412</v>
+        <v>-1522.894675882353</v>
       </c>
       <c r="AL150" s="13" t="n">
-        <v>-275204.6190476191</v>
+        <v>-136979.9443915344</v>
       </c>
     </row>
     <row r="151">
       <c r="B151" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Forex</t>
-        </is>
-      </c>
-      <c r="C151" s="11" t="n">
-        <v>-502398.6</v>
-      </c>
-      <c r="D151" s="11" t="n">
-        <v>-29.55285882352941</v>
-      </c>
-      <c r="E151" s="11" t="n">
-        <v>-2658.193650793651</v>
-      </c>
+          <t xml:space="preserve">        Bank Provision Charges</t>
+        </is>
+      </c>
+      <c r="C151" s="11" t="n"/>
+      <c r="D151" s="11" t="n"/>
+      <c r="E151" s="11" t="n"/>
       <c r="F151" s="11" t="n"/>
       <c r="G151" s="11" t="n"/>
       <c r="H151" s="11" t="n"/>
       <c r="I151" s="11" t="n">
-        <v>-237149</v>
+        <v>-19344233</v>
       </c>
       <c r="J151" s="11" t="n">
-        <v>-13.94994117647059</v>
+        <v>-1137.896058823529</v>
       </c>
       <c r="K151" s="11" t="n">
-        <v>-1254.756613756614</v>
+        <v>-102350.4391534391</v>
       </c>
       <c r="L151" s="11" t="n"/>
       <c r="M151" s="11" t="n"/>
       <c r="N151" s="11" t="n"/>
-      <c r="O151" s="11" t="n">
-        <v>-476000</v>
-      </c>
-      <c r="P151" s="11" t="n">
-        <v>-28</v>
-      </c>
-      <c r="Q151" s="11" t="n">
-        <v>-2518.518518518519</v>
-      </c>
+      <c r="O151" s="11" t="n"/>
+      <c r="P151" s="11" t="n"/>
+      <c r="Q151" s="11" t="n"/>
       <c r="R151" s="11" t="n">
-        <v>-8215065</v>
+        <v>-32669440</v>
       </c>
       <c r="S151" s="11" t="n">
-        <v>-483.2391176470588</v>
+        <v>-1921.731764705882</v>
       </c>
       <c r="T151" s="11" t="n">
-        <v>-43465.95238095238</v>
+        <v>-172854.1798941799</v>
       </c>
       <c r="U151" s="11" t="n"/>
       <c r="V151" s="11" t="n"/>
@@ -13048,752 +13078,831 @@
       <c r="AB151" s="11" t="n"/>
       <c r="AC151" s="11" t="n"/>
       <c r="AD151" s="11" t="n">
-        <v>-9430612.6</v>
+        <v>-52013673</v>
       </c>
       <c r="AE151" s="11" t="n">
-        <v>-554.7419176470588</v>
+        <v>-3059.627823529412</v>
       </c>
       <c r="AF151" s="11" t="n">
-        <v>-49897.42116402117</v>
+        <v>-275204.6190476191</v>
       </c>
       <c r="AG151" s="11" t="n"/>
       <c r="AH151" s="11" t="n"/>
       <c r="AI151" s="11" t="n"/>
       <c r="AJ151" s="11" t="n">
-        <v>-9430612.6</v>
+        <v>-52013673</v>
       </c>
       <c r="AK151" s="11" t="n">
-        <v>-554.7419176470588</v>
+        <v>-3059.627823529412</v>
       </c>
       <c r="AL151" s="11" t="n">
-        <v>-49897.42116402117</v>
+        <v>-275204.6190476191</v>
       </c>
     </row>
     <row r="152">
       <c r="B152" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Interest on Bank Term Loans</t>
+          <t xml:space="preserve">        Forex</t>
         </is>
       </c>
       <c r="C152" s="13" t="n">
-        <v>-304089642.44</v>
+        <v>-502398.6</v>
       </c>
       <c r="D152" s="13" t="n">
-        <v>-17887.62602588235</v>
+        <v>-29.55285882352941</v>
       </c>
       <c r="E152" s="13" t="n">
-        <v>-1608939.907089947</v>
-      </c>
-      <c r="F152" s="13" t="n">
-        <v>-192548915.91</v>
-      </c>
-      <c r="G152" s="13" t="n">
-        <v>-11326.40681823529</v>
-      </c>
-      <c r="H152" s="13" t="n">
-        <v>-1018777.332857143</v>
-      </c>
+        <v>-2658.193650793651</v>
+      </c>
+      <c r="F152" s="13" t="n"/>
+      <c r="G152" s="13" t="n"/>
+      <c r="H152" s="13" t="n"/>
       <c r="I152" s="13" t="n">
-        <v>-154772188.99</v>
+        <v>-237149</v>
       </c>
       <c r="J152" s="13" t="n">
-        <v>-9104.246411176471</v>
+        <v>-13.94994117647059</v>
       </c>
       <c r="K152" s="13" t="n">
-        <v>-818900.4708465609</v>
-      </c>
-      <c r="L152" s="13" t="n">
-        <v>-185501545.14</v>
-      </c>
-      <c r="M152" s="13" t="n">
-        <v>-10911.85559647059</v>
-      </c>
-      <c r="N152" s="13" t="n">
-        <v>-981489.6568253967</v>
-      </c>
+        <v>-1254.756613756614</v>
+      </c>
+      <c r="L152" s="13" t="n"/>
+      <c r="M152" s="13" t="n"/>
+      <c r="N152" s="13" t="n"/>
       <c r="O152" s="13" t="n">
-        <v>-2857131528.42</v>
+        <v>-476000</v>
       </c>
       <c r="P152" s="13" t="n">
-        <v>-168066.5604952941</v>
+        <v>-28</v>
       </c>
       <c r="Q152" s="13" t="n">
-        <v>-15117098.03396825</v>
+        <v>-2518.518518518519</v>
       </c>
       <c r="R152" s="13" t="n">
-        <v>-185571714.67</v>
+        <v>-8215065</v>
       </c>
       <c r="S152" s="13" t="n">
-        <v>-10915.98321588235</v>
+        <v>-483.2391176470588</v>
       </c>
       <c r="T152" s="13" t="n">
-        <v>-981860.9241798942</v>
-      </c>
-      <c r="U152" s="13" t="n">
-        <v>-191661834.26</v>
-      </c>
-      <c r="V152" s="13" t="n">
-        <v>-11274.22554470588</v>
-      </c>
-      <c r="W152" s="13" t="n">
-        <v>-1014083.779153439</v>
-      </c>
-      <c r="X152" s="13" t="n">
-        <v>-195252781.6</v>
-      </c>
-      <c r="Y152" s="13" t="n">
-        <v>-11485.45774117647</v>
-      </c>
-      <c r="Z152" s="13" t="n">
-        <v>-1033083.500529101</v>
-      </c>
-      <c r="AA152" s="13" t="n">
-        <v>-182572538.36</v>
-      </c>
-      <c r="AB152" s="13" t="n">
-        <v>-10739.56108</v>
-      </c>
-      <c r="AC152" s="13" t="n">
-        <v>-965992.2664550266</v>
-      </c>
+        <v>-43465.95238095238</v>
+      </c>
+      <c r="U152" s="13" t="n"/>
+      <c r="V152" s="13" t="n"/>
+      <c r="W152" s="13" t="n"/>
+      <c r="X152" s="13" t="n"/>
+      <c r="Y152" s="13" t="n"/>
+      <c r="Z152" s="13" t="n"/>
+      <c r="AA152" s="13" t="n"/>
+      <c r="AB152" s="13" t="n"/>
+      <c r="AC152" s="13" t="n"/>
       <c r="AD152" s="13" t="n">
-        <v>-4449102689.79</v>
+        <v>-9430612.6</v>
       </c>
       <c r="AE152" s="13" t="n">
-        <v>-261711.9229288236</v>
+        <v>-554.7419176470588</v>
       </c>
       <c r="AF152" s="13" t="n">
-        <v>-23540225.87190476</v>
+        <v>-49897.42116402117</v>
       </c>
       <c r="AG152" s="13" t="n"/>
       <c r="AH152" s="13" t="n"/>
       <c r="AI152" s="13" t="n"/>
       <c r="AJ152" s="13" t="n">
-        <v>-4449102689.79</v>
+        <v>-9430612.6</v>
       </c>
       <c r="AK152" s="13" t="n">
-        <v>-261711.9229288236</v>
+        <v>-554.7419176470588</v>
       </c>
       <c r="AL152" s="13" t="n">
-        <v>-23540225.87190476</v>
+        <v>-49897.42116402117</v>
       </c>
     </row>
     <row r="153">
       <c r="B153" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Interest on Bank Working Capital Loans</t>
-        </is>
-      </c>
-      <c r="C153" s="11" t="n"/>
-      <c r="D153" s="11" t="n"/>
-      <c r="E153" s="11" t="n"/>
-      <c r="F153" s="11" t="n"/>
-      <c r="G153" s="11" t="n"/>
-      <c r="H153" s="11" t="n"/>
+          <t xml:space="preserve">        Interest on Bank Term Loans</t>
+        </is>
+      </c>
+      <c r="C153" s="11" t="n">
+        <v>-293479865</v>
+      </c>
+      <c r="D153" s="11" t="n">
+        <v>-17263.52147058824</v>
+      </c>
+      <c r="E153" s="11" t="n">
+        <v>-1552803.518518518</v>
+      </c>
+      <c r="F153" s="11" t="n">
+        <v>-179203558</v>
+      </c>
+      <c r="G153" s="11" t="n">
+        <v>-10541.38576470588</v>
+      </c>
+      <c r="H153" s="11" t="n">
+        <v>-948166.9735449735</v>
+      </c>
       <c r="I153" s="11" t="n">
-        <v>-268756578</v>
+        <v>-154485826</v>
       </c>
       <c r="J153" s="11" t="n">
-        <v>-15809.21047058824</v>
+        <v>-9087.401529411765</v>
       </c>
       <c r="K153" s="11" t="n">
-        <v>-1421992.476190476</v>
+        <v>-817385.3227513228</v>
       </c>
       <c r="L153" s="11" t="n">
-        <v>-171119871</v>
+        <v>-185382992</v>
       </c>
       <c r="M153" s="11" t="n">
-        <v>-10065.87476470588</v>
+        <v>-10904.88188235294</v>
       </c>
       <c r="N153" s="11" t="n">
-        <v>-905396.1428571428</v>
+        <v>-980862.3915343916</v>
       </c>
       <c r="O153" s="11" t="n">
-        <v>-96386746</v>
+        <v>-2857003956</v>
       </c>
       <c r="P153" s="11" t="n">
-        <v>-5669.808588235294</v>
+        <v>-168059.0562352941</v>
       </c>
       <c r="Q153" s="11" t="n">
-        <v>-509982.7830687831</v>
+        <v>-15116423.04761905</v>
       </c>
       <c r="R153" s="11" t="n">
-        <v>-106357788</v>
+        <v>-185382991</v>
       </c>
       <c r="S153" s="11" t="n">
-        <v>-6256.340470588235</v>
+        <v>-10904.88182352941</v>
       </c>
       <c r="T153" s="11" t="n">
-        <v>-562739.6190476191</v>
+        <v>-980862.3862433862</v>
       </c>
       <c r="U153" s="11" t="n">
-        <v>-103034108</v>
+        <v>-191562425</v>
       </c>
       <c r="V153" s="11" t="n">
-        <v>-6060.829882352941</v>
+        <v>-11268.37794117647</v>
       </c>
       <c r="W153" s="11" t="n">
-        <v>-545154.0105820106</v>
+        <v>-1013557.804232804</v>
       </c>
       <c r="X153" s="11" t="n">
-        <v>-103034108</v>
+        <v>-195109877</v>
       </c>
       <c r="Y153" s="11" t="n">
-        <v>-6060.829882352941</v>
+        <v>-11477.05158823529</v>
       </c>
       <c r="Z153" s="11" t="n">
-        <v>-545154.0105820106</v>
+        <v>-1032327.391534392</v>
       </c>
       <c r="AA153" s="11" t="n">
-        <v>-99710427</v>
+        <v>-182522142</v>
       </c>
       <c r="AB153" s="11" t="n">
-        <v>-5865.319235294118</v>
+        <v>-10736.59658823529</v>
       </c>
       <c r="AC153" s="11" t="n">
-        <v>-527568.3968253968</v>
+        <v>-965725.6190476191</v>
       </c>
       <c r="AD153" s="11" t="n">
-        <v>-948399626</v>
+        <v>-4424133632</v>
       </c>
       <c r="AE153" s="11" t="n">
-        <v>-55788.21329411765</v>
+        <v>-260243.1548235294</v>
       </c>
       <c r="AF153" s="11" t="n">
-        <v>-5017987.439153438</v>
+        <v>-23408114.45502646</v>
       </c>
       <c r="AG153" s="11" t="n"/>
       <c r="AH153" s="11" t="n"/>
       <c r="AI153" s="11" t="n"/>
       <c r="AJ153" s="11" t="n">
-        <v>-948399626</v>
+        <v>-4424133632</v>
       </c>
       <c r="AK153" s="11" t="n">
-        <v>-55788.21329411765</v>
+        <v>-260243.1548235294</v>
       </c>
       <c r="AL153" s="11" t="n">
-        <v>-5017987.439153438</v>
+        <v>-23408114.45502646</v>
       </c>
     </row>
     <row r="154">
       <c r="B154" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Loan Related Charges</t>
+          <t xml:space="preserve">        Interest on Bank Working Capital Loans</t>
         </is>
       </c>
       <c r="C154" s="13" t="n"/>
       <c r="D154" s="13" t="n"/>
       <c r="E154" s="13" t="n"/>
-      <c r="F154" s="13" t="n">
-        <v>-773891532</v>
-      </c>
-      <c r="G154" s="13" t="n">
-        <v>-45523.03129411765</v>
-      </c>
-      <c r="H154" s="13" t="n">
-        <v>-4094664.19047619</v>
-      </c>
-      <c r="I154" s="13" t="n"/>
-      <c r="J154" s="13" t="n"/>
-      <c r="K154" s="13" t="n"/>
-      <c r="L154" s="13" t="n"/>
-      <c r="M154" s="13" t="n"/>
-      <c r="N154" s="13" t="n"/>
-      <c r="O154" s="13" t="n"/>
-      <c r="P154" s="13" t="n"/>
-      <c r="Q154" s="13" t="n"/>
-      <c r="R154" s="13" t="n"/>
-      <c r="S154" s="13" t="n"/>
-      <c r="T154" s="13" t="n"/>
-      <c r="U154" s="13" t="n"/>
-      <c r="V154" s="13" t="n"/>
-      <c r="W154" s="13" t="n"/>
-      <c r="X154" s="13" t="n"/>
-      <c r="Y154" s="13" t="n"/>
-      <c r="Z154" s="13" t="n"/>
-      <c r="AA154" s="13" t="n"/>
-      <c r="AB154" s="13" t="n"/>
-      <c r="AC154" s="13" t="n"/>
+      <c r="F154" s="13" t="n"/>
+      <c r="G154" s="13" t="n"/>
+      <c r="H154" s="13" t="n"/>
+      <c r="I154" s="13" t="n">
+        <v>-268756578</v>
+      </c>
+      <c r="J154" s="13" t="n">
+        <v>-15809.21047058824</v>
+      </c>
+      <c r="K154" s="13" t="n">
+        <v>-1421992.476190476</v>
+      </c>
+      <c r="L154" s="13" t="n">
+        <v>-171119871</v>
+      </c>
+      <c r="M154" s="13" t="n">
+        <v>-10065.87476470588</v>
+      </c>
+      <c r="N154" s="13" t="n">
+        <v>-905396.1428571428</v>
+      </c>
+      <c r="O154" s="13" t="n">
+        <v>-96386746</v>
+      </c>
+      <c r="P154" s="13" t="n">
+        <v>-5669.808588235294</v>
+      </c>
+      <c r="Q154" s="13" t="n">
+        <v>-509982.7830687831</v>
+      </c>
+      <c r="R154" s="13" t="n">
+        <v>-106357788</v>
+      </c>
+      <c r="S154" s="13" t="n">
+        <v>-6256.340470588235</v>
+      </c>
+      <c r="T154" s="13" t="n">
+        <v>-562739.6190476191</v>
+      </c>
+      <c r="U154" s="13" t="n">
+        <v>-103034108</v>
+      </c>
+      <c r="V154" s="13" t="n">
+        <v>-6060.829882352941</v>
+      </c>
+      <c r="W154" s="13" t="n">
+        <v>-545154.0105820106</v>
+      </c>
+      <c r="X154" s="13" t="n">
+        <v>-103034108</v>
+      </c>
+      <c r="Y154" s="13" t="n">
+        <v>-6060.829882352941</v>
+      </c>
+      <c r="Z154" s="13" t="n">
+        <v>-545154.0105820106</v>
+      </c>
+      <c r="AA154" s="13" t="n">
+        <v>-99710427</v>
+      </c>
+      <c r="AB154" s="13" t="n">
+        <v>-5865.319235294118</v>
+      </c>
+      <c r="AC154" s="13" t="n">
+        <v>-527568.3968253968</v>
+      </c>
       <c r="AD154" s="13" t="n">
-        <v>-773891532</v>
+        <v>-948399626</v>
       </c>
       <c r="AE154" s="13" t="n">
-        <v>-45523.03129411765</v>
+        <v>-55788.21329411765</v>
       </c>
       <c r="AF154" s="13" t="n">
-        <v>-4094664.19047619</v>
+        <v>-5017987.439153438</v>
       </c>
       <c r="AG154" s="13" t="n"/>
       <c r="AH154" s="13" t="n"/>
       <c r="AI154" s="13" t="n"/>
       <c r="AJ154" s="13" t="n">
+        <v>-948399626</v>
+      </c>
+      <c r="AK154" s="13" t="n">
+        <v>-55788.21329411765</v>
+      </c>
+      <c r="AL154" s="13" t="n">
+        <v>-5017987.439153438</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="B155" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        Loan Related Charges</t>
+        </is>
+      </c>
+      <c r="C155" s="11" t="n"/>
+      <c r="D155" s="11" t="n"/>
+      <c r="E155" s="11" t="n"/>
+      <c r="F155" s="11" t="n">
         <v>-773891532</v>
       </c>
-      <c r="AK154" s="13" t="n">
+      <c r="G155" s="11" t="n">
         <v>-45523.03129411765</v>
       </c>
-      <c r="AL154" s="13" t="n">
+      <c r="H155" s="11" t="n">
         <v>-4094664.19047619</v>
       </c>
-    </row>
-    <row r="155">
-      <c r="B155" s="14" t="inlineStr">
+      <c r="I155" s="11" t="n"/>
+      <c r="J155" s="11" t="n"/>
+      <c r="K155" s="11" t="n"/>
+      <c r="L155" s="11" t="n"/>
+      <c r="M155" s="11" t="n"/>
+      <c r="N155" s="11" t="n"/>
+      <c r="O155" s="11" t="n"/>
+      <c r="P155" s="11" t="n"/>
+      <c r="Q155" s="11" t="n"/>
+      <c r="R155" s="11" t="n"/>
+      <c r="S155" s="11" t="n"/>
+      <c r="T155" s="11" t="n"/>
+      <c r="U155" s="11" t="n"/>
+      <c r="V155" s="11" t="n"/>
+      <c r="W155" s="11" t="n"/>
+      <c r="X155" s="11" t="n"/>
+      <c r="Y155" s="11" t="n"/>
+      <c r="Z155" s="11" t="n"/>
+      <c r="AA155" s="11" t="n"/>
+      <c r="AB155" s="11" t="n"/>
+      <c r="AC155" s="11" t="n"/>
+      <c r="AD155" s="11" t="n">
+        <v>-773891532</v>
+      </c>
+      <c r="AE155" s="11" t="n">
+        <v>-45523.03129411765</v>
+      </c>
+      <c r="AF155" s="11" t="n">
+        <v>-4094664.19047619</v>
+      </c>
+      <c r="AG155" s="11" t="n"/>
+      <c r="AH155" s="11" t="n"/>
+      <c r="AI155" s="11" t="n"/>
+      <c r="AJ155" s="11" t="n">
+        <v>-773891532</v>
+      </c>
+      <c r="AK155" s="11" t="n">
+        <v>-45523.03129411765</v>
+      </c>
+      <c r="AL155" s="11" t="n">
+        <v>-4094664.19047619</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="B156" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    TOTAL FINANCE COST</t>
         </is>
       </c>
-      <c r="C155" s="15" t="n">
-        <v>-308685541.72</v>
-      </c>
-      <c r="D155" s="15" t="n">
-        <v>-18157.97304235294</v>
-      </c>
-      <c r="E155" s="15" t="n">
-        <v>-1633256.834497355</v>
-      </c>
-      <c r="F155" s="15" t="n">
-        <v>-967365147.91</v>
-      </c>
-      <c r="G155" s="15" t="n">
-        <v>-56903.83223</v>
-      </c>
-      <c r="H155" s="15" t="n">
-        <v>-5118334.115925926</v>
-      </c>
-      <c r="I155" s="15" t="n">
-        <v>-446674688.99</v>
-      </c>
-      <c r="J155" s="15" t="n">
-        <v>-26274.98170529412</v>
-      </c>
-      <c r="K155" s="15" t="n">
-        <v>-2363358.142804233</v>
-      </c>
-      <c r="L155" s="15" t="n">
-        <v>-358180514.14</v>
-      </c>
-      <c r="M155" s="15" t="n">
-        <v>-21069.44200823529</v>
-      </c>
-      <c r="N155" s="15" t="n">
-        <v>-1895134.995449735</v>
-      </c>
-      <c r="O155" s="15" t="n">
-        <v>-2956572690.42</v>
-      </c>
-      <c r="P155" s="15" t="n">
-        <v>-173916.0406129412</v>
-      </c>
-      <c r="Q155" s="15" t="n">
-        <v>-15643241.74825397</v>
-      </c>
-      <c r="R155" s="15" t="n">
-        <v>-334287230.67</v>
-      </c>
-      <c r="S155" s="15" t="n">
-        <v>-19663.95474529412</v>
-      </c>
-      <c r="T155" s="15" t="n">
-        <v>-1768715.506190476</v>
-      </c>
-      <c r="U155" s="15" t="n">
-        <v>-296979086.26</v>
-      </c>
-      <c r="V155" s="15" t="n">
-        <v>-17469.35801529412</v>
-      </c>
-      <c r="W155" s="15" t="n">
-        <v>-1571317.916719577</v>
-      </c>
-      <c r="X155" s="15" t="n">
-        <v>-300606165.6</v>
-      </c>
-      <c r="Y155" s="15" t="n">
-        <v>-17682.71562352941</v>
-      </c>
-      <c r="Z155" s="15" t="n">
-        <v>-1590508.812698413</v>
-      </c>
-      <c r="AA155" s="15" t="n">
-        <v>-283724255.36</v>
-      </c>
-      <c r="AB155" s="15" t="n">
-        <v>-16689.66208</v>
-      </c>
-      <c r="AC155" s="15" t="n">
-        <v>-1501186.536296296</v>
-      </c>
-      <c r="AD155" s="15" t="n">
-        <v>-6253075321.070001</v>
-      </c>
-      <c r="AE155" s="15" t="n">
-        <v>-367827.9600629411</v>
-      </c>
-      <c r="AF155" s="15" t="n">
-        <v>-33085054.60883598</v>
-      </c>
-      <c r="AG155" s="15" t="n">
-        <v>-15700</v>
-      </c>
-      <c r="AH155" s="15" t="n">
-        <v>-0.9235294117647059</v>
-      </c>
-      <c r="AI155" s="15" t="n">
-        <v>-83.06878306878306</v>
-      </c>
-      <c r="AJ155" s="15" t="n">
-        <v>-6253091021.070001</v>
-      </c>
-      <c r="AK155" s="15" t="n">
-        <v>-367828.8835923529</v>
-      </c>
-      <c r="AL155" s="15" t="n">
-        <v>-33085137.67761905</v>
-      </c>
-    </row>
-    <row r="156">
-      <c r="B156" s="18" t="inlineStr">
-        <is>
-          <t>TOTAL OUTFLOW</t>
-        </is>
-      </c>
-      <c r="C156" s="19" t="n">
-        <v>-44493158195.03</v>
-      </c>
-      <c r="D156" s="19" t="n">
-        <v>-2617244.599707647</v>
-      </c>
-      <c r="E156" s="19" t="n">
-        <v>-235413535.4234391</v>
-      </c>
-      <c r="F156" s="19" t="n">
-        <v>-87290805698.13</v>
-      </c>
-      <c r="G156" s="19" t="n">
-        <v>-5134753.276360588</v>
-      </c>
-      <c r="H156" s="19" t="n">
-        <v>-461856114.8049207</v>
-      </c>
-      <c r="I156" s="19" t="n">
-        <v>-56595919771.99</v>
-      </c>
-      <c r="J156" s="19" t="n">
-        <v>-3329171.751293529</v>
-      </c>
-      <c r="K156" s="19" t="n">
-        <v>-299449310.9629101</v>
-      </c>
-      <c r="L156" s="19" t="n">
-        <v>-47009379649.2</v>
-      </c>
-      <c r="M156" s="19" t="n">
-        <v>-2765257.626423529</v>
-      </c>
-      <c r="N156" s="19" t="n">
-        <v>-248726876.4507936</v>
-      </c>
-      <c r="O156" s="19" t="n">
-        <v>-27914586083.82</v>
-      </c>
-      <c r="P156" s="19" t="n">
-        <v>-1642034.475518824</v>
-      </c>
-      <c r="Q156" s="19" t="n">
-        <v>-147696222.6657143</v>
-      </c>
-      <c r="R156" s="19" t="n">
-        <v>-7977840953.47</v>
-      </c>
-      <c r="S156" s="19" t="n">
-        <v>-469284.7619688236</v>
-      </c>
-      <c r="T156" s="19" t="n">
-        <v>-42210798.69560847</v>
-      </c>
-      <c r="U156" s="19" t="n">
-        <v>-8224549510.2</v>
-      </c>
-      <c r="V156" s="19" t="n">
-        <v>-483797.0300117647</v>
-      </c>
-      <c r="W156" s="19" t="n">
-        <v>-43516134.97460318</v>
-      </c>
-      <c r="X156" s="19" t="n">
-        <v>-9565196761.719999</v>
-      </c>
-      <c r="Y156" s="19" t="n">
-        <v>-562658.6330423529</v>
-      </c>
-      <c r="Z156" s="19" t="n">
-        <v>-50609506.67576719</v>
-      </c>
-      <c r="AA156" s="19" t="n">
-        <v>-15104736490.53</v>
-      </c>
-      <c r="AB156" s="19" t="n">
-        <v>-888513.9112076471</v>
-      </c>
-      <c r="AC156" s="19" t="n">
-        <v>-79919240.69063492</v>
-      </c>
-      <c r="AD156" s="19" t="n">
-        <v>-304176173114.09</v>
-      </c>
-      <c r="AE156" s="19" t="n">
-        <v>-17892716.0655347</v>
-      </c>
-      <c r="AF156" s="19" t="n">
-        <v>-1609397741.344392</v>
-      </c>
-      <c r="AG156" s="19" t="n">
-        <v>-1880249274</v>
-      </c>
-      <c r="AH156" s="19" t="n">
-        <v>-110602.8984705882</v>
-      </c>
-      <c r="AI156" s="19" t="n">
-        <v>-9948408.857142856</v>
-      </c>
-      <c r="AJ156" s="19" t="n">
-        <v>-306056422388.09</v>
-      </c>
-      <c r="AK156" s="19" t="n">
-        <v>-18003318.96400529</v>
-      </c>
-      <c r="AL156" s="19" t="n">
-        <v>-1619346150.201535</v>
+      <c r="C156" s="15" t="n">
+        <v>-308817154.03</v>
+      </c>
+      <c r="D156" s="15" t="n">
+        <v>-18165.71494294118</v>
+      </c>
+      <c r="E156" s="15" t="n">
+        <v>-1633953.195925926</v>
+      </c>
+      <c r="F156" s="15" t="n">
+        <v>-967617873.25</v>
+      </c>
+      <c r="G156" s="15" t="n">
+        <v>-56918.69842647059</v>
+      </c>
+      <c r="H156" s="15" t="n">
+        <v>-5119671.287037037</v>
+      </c>
+      <c r="I156" s="15" t="n">
+        <v>-446753058.99</v>
+      </c>
+      <c r="J156" s="15" t="n">
+        <v>-26279.59170529412</v>
+      </c>
+      <c r="K156" s="15" t="n">
+        <v>-2363772.798888889</v>
+      </c>
+      <c r="L156" s="15" t="n">
+        <v>-358225510.2</v>
+      </c>
+      <c r="M156" s="15" t="n">
+        <v>-21072.08883529412</v>
+      </c>
+      <c r="N156" s="15" t="n">
+        <v>-1895373.06984127</v>
+      </c>
+      <c r="O156" s="15" t="n">
+        <v>-2956576595.82</v>
+      </c>
+      <c r="P156" s="15" t="n">
+        <v>-173916.2703423529</v>
+      </c>
+      <c r="Q156" s="15" t="n">
+        <v>-15643262.41174603</v>
+      </c>
+      <c r="R156" s="15" t="n">
+        <v>-334494086.03</v>
+      </c>
+      <c r="S156" s="15" t="n">
+        <v>-19676.12270764706</v>
+      </c>
+      <c r="T156" s="15" t="n">
+        <v>-1769809.978994709</v>
+      </c>
+      <c r="U156" s="15" t="n">
+        <v>-297038228.2</v>
+      </c>
+      <c r="V156" s="15" t="n">
+        <v>-17472.83695294118</v>
+      </c>
+      <c r="W156" s="15" t="n">
+        <v>-1571630.837037037</v>
+      </c>
+      <c r="X156" s="15" t="n">
+        <v>-300665750.72</v>
+      </c>
+      <c r="Y156" s="15" t="n">
+        <v>-17686.22063058824</v>
+      </c>
+      <c r="Z156" s="15" t="n">
+        <v>-1590824.077883598</v>
+      </c>
+      <c r="AA156" s="15" t="n">
+        <v>-283807215.53</v>
+      </c>
+      <c r="AB156" s="15" t="n">
+        <v>-16694.54209</v>
+      </c>
+      <c r="AC156" s="15" t="n">
+        <v>-1501625.478994709</v>
+      </c>
+      <c r="AD156" s="15" t="n">
+        <v>-6253995472.77</v>
+      </c>
+      <c r="AE156" s="15" t="n">
+        <v>-367882.0866335295</v>
+      </c>
+      <c r="AF156" s="15" t="n">
+        <v>-33089923.13634921</v>
+      </c>
+      <c r="AG156" s="15" t="n">
+        <v>-18200</v>
+      </c>
+      <c r="AH156" s="15" t="n">
+        <v>-1.070588235294118</v>
+      </c>
+      <c r="AI156" s="15" t="n">
+        <v>-96.29629629629629</v>
+      </c>
+      <c r="AJ156" s="15" t="n">
+        <v>-6254013672.77</v>
+      </c>
+      <c r="AK156" s="15" t="n">
+        <v>-367883.1572217647</v>
+      </c>
+      <c r="AL156" s="15" t="n">
+        <v>-33090019.4326455</v>
       </c>
     </row>
     <row r="157">
       <c r="B157" s="18" t="inlineStr">
         <is>
+          <t>TOTAL OUTFLOW</t>
+        </is>
+      </c>
+      <c r="C157" s="19" t="n">
+        <v>-44493158195.03</v>
+      </c>
+      <c r="D157" s="19" t="n">
+        <v>-2617244.599707647</v>
+      </c>
+      <c r="E157" s="19" t="n">
+        <v>-235413535.4234391</v>
+      </c>
+      <c r="F157" s="19" t="n">
+        <v>-87290805698.13</v>
+      </c>
+      <c r="G157" s="19" t="n">
+        <v>-5134753.276360588</v>
+      </c>
+      <c r="H157" s="19" t="n">
+        <v>-461856114.8049207</v>
+      </c>
+      <c r="I157" s="19" t="n">
+        <v>-56595919771.99</v>
+      </c>
+      <c r="J157" s="19" t="n">
+        <v>-3329171.751293529</v>
+      </c>
+      <c r="K157" s="19" t="n">
+        <v>-299449310.9629101</v>
+      </c>
+      <c r="L157" s="19" t="n">
+        <v>-47009379649.2</v>
+      </c>
+      <c r="M157" s="19" t="n">
+        <v>-2765257.626423529</v>
+      </c>
+      <c r="N157" s="19" t="n">
+        <v>-248726876.4507936</v>
+      </c>
+      <c r="O157" s="19" t="n">
+        <v>-27914586083.82</v>
+      </c>
+      <c r="P157" s="19" t="n">
+        <v>-1642034.475518824</v>
+      </c>
+      <c r="Q157" s="19" t="n">
+        <v>-147696222.6657143</v>
+      </c>
+      <c r="R157" s="19" t="n">
+        <v>-7977840953.469999</v>
+      </c>
+      <c r="S157" s="19" t="n">
+        <v>-469284.7619688235</v>
+      </c>
+      <c r="T157" s="19" t="n">
+        <v>-42210798.69560846</v>
+      </c>
+      <c r="U157" s="19" t="n">
+        <v>-8224549510.2</v>
+      </c>
+      <c r="V157" s="19" t="n">
+        <v>-483797.0300117647</v>
+      </c>
+      <c r="W157" s="19" t="n">
+        <v>-43516134.97460318</v>
+      </c>
+      <c r="X157" s="19" t="n">
+        <v>-9565196761.720001</v>
+      </c>
+      <c r="Y157" s="19" t="n">
+        <v>-562658.633042353</v>
+      </c>
+      <c r="Z157" s="19" t="n">
+        <v>-50609506.67576721</v>
+      </c>
+      <c r="AA157" s="19" t="n">
+        <v>-15104736490.53</v>
+      </c>
+      <c r="AB157" s="19" t="n">
+        <v>-888513.9112076471</v>
+      </c>
+      <c r="AC157" s="19" t="n">
+        <v>-79919240.69063492</v>
+      </c>
+      <c r="AD157" s="19" t="n">
+        <v>-304176173114.09</v>
+      </c>
+      <c r="AE157" s="19" t="n">
+        <v>-17892716.0655347</v>
+      </c>
+      <c r="AF157" s="19" t="n">
+        <v>-1609397741.344392</v>
+      </c>
+      <c r="AG157" s="19" t="n">
+        <v>-1899751774</v>
+      </c>
+      <c r="AH157" s="19" t="n">
+        <v>-111750.1043529412</v>
+      </c>
+      <c r="AI157" s="19" t="n">
+        <v>-10051596.68783069</v>
+      </c>
+      <c r="AJ157" s="19" t="n">
+        <v>-306075924888.09</v>
+      </c>
+      <c r="AK157" s="19" t="n">
+        <v>-18004466.16988764</v>
+      </c>
+      <c r="AL157" s="19" t="n">
+        <v>-1619449338.032222</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="B158" s="18" t="inlineStr">
+        <is>
           <t>NET CASH SURPLUS (LOSS)</t>
         </is>
       </c>
-      <c r="C157" s="19" t="n">
+      <c r="C158" s="19" t="n">
         <v>11812902160.24</v>
       </c>
-      <c r="D157" s="19" t="n">
+      <c r="D158" s="19" t="n">
         <v>694876.5976611763</v>
       </c>
-      <c r="E157" s="19" t="n">
+      <c r="E158" s="19" t="n">
         <v>62502127.83195766</v>
       </c>
-      <c r="F157" s="19" t="n">
+      <c r="F158" s="19" t="n">
         <v>-75526959730.20001</v>
       </c>
-      <c r="G157" s="19" t="n">
+      <c r="G158" s="19" t="n">
         <v>-4442762.337070589</v>
       </c>
-      <c r="H157" s="19" t="n">
+      <c r="H158" s="19" t="n">
         <v>-399613543.5460318</v>
       </c>
-      <c r="I157" s="19" t="n">
+      <c r="I158" s="19" t="n">
         <v>2573810161.360001</v>
       </c>
-      <c r="J157" s="19" t="n">
+      <c r="J158" s="19" t="n">
         <v>151400.5977270589</v>
       </c>
-      <c r="K157" s="19" t="n">
+      <c r="K158" s="19" t="n">
         <v>13618043.18179894</v>
       </c>
-      <c r="L157" s="19" t="n">
+      <c r="L158" s="19" t="n">
         <v>11041904011.41</v>
       </c>
-      <c r="M157" s="19" t="n">
+      <c r="M158" s="19" t="n">
         <v>649523.765377059</v>
       </c>
-      <c r="N157" s="19" t="n">
+      <c r="N158" s="19" t="n">
         <v>58422772.54714288</v>
       </c>
-      <c r="O157" s="19" t="n">
+      <c r="O158" s="19" t="n">
         <v>-15435413590.8</v>
       </c>
-      <c r="P157" s="19" t="n">
+      <c r="P158" s="19" t="n">
         <v>-907965.5053411764</v>
       </c>
-      <c r="Q157" s="19" t="n">
+      <c r="Q158" s="19" t="n">
         <v>-81668854.97777778</v>
       </c>
-      <c r="R157" s="19" t="n">
-        <v>-114348822.1300001</v>
-      </c>
-      <c r="S157" s="19" t="n">
-        <v>-6726.401301764713</v>
-      </c>
-      <c r="T157" s="19" t="n">
-        <v>-605020.2229100536</v>
-      </c>
-      <c r="U157" s="19" t="n">
+      <c r="R158" s="19" t="n">
+        <v>-114348822.1299992</v>
+      </c>
+      <c r="S158" s="19" t="n">
+        <v>-6726.401301764657</v>
+      </c>
+      <c r="T158" s="19" t="n">
+        <v>-605020.2229100484</v>
+      </c>
+      <c r="U158" s="19" t="n">
         <v>1367972765.69</v>
       </c>
-      <c r="V157" s="19" t="n">
+      <c r="V158" s="19" t="n">
         <v>80468.9862170588</v>
       </c>
-      <c r="W157" s="19" t="n">
+      <c r="W158" s="19" t="n">
         <v>7237951.141216929</v>
       </c>
-      <c r="X157" s="19" t="n">
-        <v>-1729271263.249999</v>
-      </c>
-      <c r="Y157" s="19" t="n">
-        <v>-101721.8390147058</v>
-      </c>
-      <c r="Z157" s="19" t="n">
-        <v>-9149583.403439149</v>
-      </c>
-      <c r="AA157" s="19" t="n">
+      <c r="X158" s="19" t="n">
+        <v>-1729271263.250001</v>
+      </c>
+      <c r="Y158" s="19" t="n">
+        <v>-101721.8390147059</v>
+      </c>
+      <c r="Z158" s="19" t="n">
+        <v>-9149583.403439159</v>
+      </c>
+      <c r="AA158" s="19" t="n">
         <v>13615217696.07</v>
       </c>
-      <c r="AB157" s="19" t="n">
+      <c r="AB158" s="19" t="n">
         <v>800895.1585923528</v>
       </c>
-      <c r="AC157" s="19" t="n">
+      <c r="AC158" s="19" t="n">
         <v>72038188.86809522</v>
       </c>
-      <c r="AD157" s="19" t="n">
+      <c r="AD158" s="19" t="n">
         <v>-52394186611.61</v>
       </c>
-      <c r="AE157" s="19" t="n">
+      <c r="AE158" s="19" t="n">
         <v>-3082010.97715353</v>
       </c>
-      <c r="AF157" s="19" t="n">
+      <c r="AF158" s="19" t="n">
         <v>-277217918.5799472</v>
       </c>
-      <c r="AG157" s="19" t="n">
-        <v>4461631374</v>
-      </c>
-      <c r="AH157" s="19" t="n">
-        <v>262448.9043529412</v>
-      </c>
-      <c r="AI157" s="19" t="n">
-        <v>23606515.20634921</v>
-      </c>
-      <c r="AJ157" s="19" t="n">
-        <v>-47932555237.61</v>
-      </c>
-      <c r="AK157" s="19" t="n">
-        <v>-2819562.072800589</v>
-      </c>
-      <c r="AL157" s="19" t="n">
-        <v>-253611403.373598</v>
-      </c>
-    </row>
-    <row r="158">
-      <c r="B158" s="6" t="inlineStr">
+      <c r="AG158" s="19" t="n">
+        <v>4442702874</v>
+      </c>
+      <c r="AH158" s="19" t="n">
+        <v>261335.4631764706</v>
+      </c>
+      <c r="AI158" s="19" t="n">
+        <v>23506364.41269841</v>
+      </c>
+      <c r="AJ158" s="19" t="n">
+        <v>-47951483737.61</v>
+      </c>
+      <c r="AK158" s="19" t="n">
+        <v>-2820675.51397706</v>
+      </c>
+      <c r="AL158" s="19" t="n">
+        <v>-253711554.1672488</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="B159" s="6" t="inlineStr">
         <is>
           <t>ENDING BALANCE</t>
         </is>
       </c>
-      <c r="C158" s="7" t="n">
+      <c r="C159" s="7" t="n">
         <v>79286562986.60001</v>
       </c>
-      <c r="D158" s="7" t="n">
+      <c r="D159" s="7" t="n">
         <v>4663915.4698</v>
       </c>
-      <c r="E158" s="7" t="n">
+      <c r="E159" s="7" t="n">
         <v>419505624.2677249</v>
       </c>
-      <c r="F158" s="7" t="n">
+      <c r="F159" s="7" t="n">
         <v>3759603256.399994</v>
       </c>
-      <c r="G158" s="7" t="n">
+      <c r="G159" s="7" t="n">
         <v>221153.1327294114</v>
       </c>
-      <c r="H158" s="7" t="n">
+      <c r="H159" s="7" t="n">
         <v>19892080.72169309</v>
       </c>
-      <c r="I158" s="7" t="n">
+      <c r="I159" s="7" t="n">
         <v>6333413417.759995</v>
       </c>
-      <c r="J158" s="7" t="n">
+      <c r="J159" s="7" t="n">
         <v>372553.7304564703</v>
       </c>
-      <c r="K158" s="7" t="n">
+      <c r="K159" s="7" t="n">
         <v>33510123.90349203</v>
       </c>
-      <c r="L158" s="7" t="n">
+      <c r="L159" s="7" t="n">
         <v>17375317429.17</v>
       </c>
-      <c r="M158" s="7" t="n">
+      <c r="M159" s="7" t="n">
         <v>1022077.495833529</v>
       </c>
-      <c r="N158" s="7" t="n">
+      <c r="N159" s="7" t="n">
         <v>91932896.45063491</v>
       </c>
-      <c r="O158" s="7" t="n">
+      <c r="O159" s="7" t="n">
         <v>1939903838.369999</v>
       </c>
-      <c r="P158" s="7" t="n">
+      <c r="P159" s="7" t="n">
         <v>114111.9904923529</v>
       </c>
-      <c r="Q158" s="7" t="n">
+      <c r="Q159" s="7" t="n">
         <v>10264041.47285714</v>
       </c>
-      <c r="R158" s="7" t="n">
-        <v>1825555016.239999</v>
-      </c>
-      <c r="S158" s="7" t="n">
+      <c r="R159" s="7" t="n">
+        <v>1825555016.24</v>
+      </c>
+      <c r="S159" s="7" t="n">
         <v>107385.5891905882</v>
       </c>
-      <c r="T158" s="7" t="n">
-        <v>9659021.249947084</v>
-      </c>
-      <c r="U158" s="7" t="n">
-        <v>3193527781.929997</v>
-      </c>
-      <c r="V158" s="7" t="n">
-        <v>187854.5754076469</v>
-      </c>
-      <c r="W158" s="7" t="n">
-        <v>16896972.39116401</v>
-      </c>
-      <c r="X158" s="7" t="n">
+      <c r="T159" s="7" t="n">
+        <v>9659021.249947088</v>
+      </c>
+      <c r="U159" s="7" t="n">
+        <v>3193527781.929999</v>
+      </c>
+      <c r="V159" s="7" t="n">
+        <v>187854.575407647</v>
+      </c>
+      <c r="W159" s="7" t="n">
+        <v>16896972.39116402</v>
+      </c>
+      <c r="X159" s="7" t="n">
         <v>1464256518.679998</v>
       </c>
-      <c r="Y158" s="7" t="n">
+      <c r="Y159" s="7" t="n">
         <v>86132.73639294108</v>
       </c>
-      <c r="Z158" s="7" t="n">
+      <c r="Z159" s="7" t="n">
         <v>7747388.987724859</v>
       </c>
-      <c r="AA158" s="7" t="n">
+      <c r="AA159" s="7" t="n">
         <v>15079474214.75</v>
       </c>
-      <c r="AB158" s="7" t="n">
+      <c r="AB159" s="7" t="n">
         <v>887027.894985294</v>
       </c>
-      <c r="AC158" s="7" t="n">
+      <c r="AC159" s="7" t="n">
         <v>79785577.85582009</v>
       </c>
-      <c r="AD158" s="7" t="n">
+      <c r="AD159" s="7" t="n">
         <v>15079474214.75</v>
       </c>
-      <c r="AE158" s="7" t="n">
+      <c r="AE159" s="7" t="n">
         <v>887027.894985294</v>
       </c>
-      <c r="AF158" s="7" t="n">
+      <c r="AF159" s="7" t="n">
         <v>79785577.85582009</v>
       </c>
-      <c r="AG158" s="7" t="n">
-        <v>19541105588.75</v>
-      </c>
-      <c r="AH158" s="7" t="n">
-        <v>1149476.799338235</v>
-      </c>
-      <c r="AI158" s="7" t="n">
-        <v>103392093.0621693</v>
-      </c>
-      <c r="AJ158" s="7" t="n">
-        <v>19541105588.75</v>
-      </c>
-      <c r="AK158" s="7" t="n">
-        <v>1149476.799338235</v>
-      </c>
-      <c r="AL158" s="7" t="n">
-        <v>103392093.0621693</v>
+      <c r="AG159" s="7" t="n">
+        <v>19522177088.75</v>
+      </c>
+      <c r="AH159" s="7" t="n">
+        <v>1148363.358161765</v>
+      </c>
+      <c r="AI159" s="7" t="n">
+        <v>103291942.2685185</v>
+      </c>
+      <c r="AJ159" s="7" t="n">
+        <v>19522177088.75</v>
+      </c>
+      <c r="AK159" s="7" t="n">
+        <v>1148363.358161765</v>
+      </c>
+      <c r="AL159" s="7" t="n">
+        <v>103291942.2685185</v>
       </c>
     </row>
   </sheetData>
@@ -14692,16 +14801,16 @@
         <v>22400563.84000001</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>2624500</v>
+        <v>-16304000</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>25025063.84000001</v>
+        <v>6096563.840000011</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>1472.06257882353</v>
+        <v>358.6214023529418</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>132407.7451851853</v>
+        <v>32256.95153439159</v>
       </c>
     </row>
     <row r="10">
@@ -14811,13 +14920,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>19541105590.75</v>
+        <v>19522177090.75</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>1149476.799455883</v>
+        <v>1148363.358279412</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>103392093.0727513</v>
+        <v>103291942.2791006</v>
       </c>
     </row>
   </sheetData>
@@ -14837,7 +14946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:AL158"/>
+  <dimension ref="B1:AL159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -14890,7 +14999,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 06 Oct 2026 10:05 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 06 Oct 2026 16:19 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -16480,22 +16589,22 @@
         <v>2.521134965502646</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>2.6495</v>
+        <v>3.2235</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>0.0001558529411764706</v>
+        <v>0.0001896176470588235</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>0.01401851851851852</v>
+        <v>0.01705555555555556</v>
       </c>
       <c r="AJ20" s="13" t="n">
-        <v>479.14400848</v>
+        <v>479.71800848</v>
       </c>
       <c r="AK20" s="13" t="n">
-        <v>0.02818494167529412</v>
+        <v>0.02821870638117647</v>
       </c>
       <c r="AL20" s="13" t="n">
-        <v>2.535153484021164</v>
+        <v>2.538190521058201</v>
       </c>
     </row>
     <row r="21">
@@ -16753,22 +16862,22 @@
         <v>0.4919761904761905</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>2.6495</v>
+        <v>3.2235</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>0.0001558529411764706</v>
+        <v>0.0001896176470588235</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>0.01401851851851852</v>
+        <v>0.01705555555555556</v>
       </c>
       <c r="AJ23" s="11" t="n">
-        <v>95.63300000000001</v>
+        <v>96.20700000000001</v>
       </c>
       <c r="AK23" s="11" t="n">
-        <v>0.005625470588235295</v>
+        <v>0.005659235294117648</v>
       </c>
       <c r="AL23" s="11" t="n">
-        <v>0.505994708994709</v>
+        <v>0.5090317460317461</v>
       </c>
     </row>
     <row r="24">
@@ -18293,22 +18402,22 @@
         <v>1332.179822764444</v>
       </c>
       <c r="AG45" s="15" t="n">
-        <v>6341.880648</v>
+        <v>6342.454648</v>
       </c>
       <c r="AH45" s="15" t="n">
-        <v>0.3730518028235295</v>
+        <v>0.3730855675294117</v>
       </c>
       <c r="AI45" s="15" t="n">
-        <v>33.55492406349207</v>
+        <v>33.5579611005291</v>
       </c>
       <c r="AJ45" s="15" t="n">
-        <v>258123.86715048</v>
+        <v>258124.44115048</v>
       </c>
       <c r="AK45" s="15" t="n">
-        <v>15.1837568912047</v>
+        <v>15.18379065591059</v>
       </c>
       <c r="AL45" s="15" t="n">
-        <v>1365.734746827937</v>
+        <v>1365.737783864974</v>
       </c>
     </row>
     <row r="46">
@@ -20837,40 +20946,40 @@
         <v>-2.937621931216931</v>
       </c>
       <c r="AA81" s="11" t="n">
-        <v>-3351.184276</v>
+        <v>-3383.684276</v>
       </c>
       <c r="AB81" s="11" t="n">
-        <v>-0.1971284868235294</v>
+        <v>-0.1990402515294118</v>
       </c>
       <c r="AC81" s="11" t="n">
-        <v>-17.73113373544973</v>
+        <v>-17.90309140740741</v>
       </c>
       <c r="AD81" s="11" t="n">
-        <v>-9987.402249000001</v>
+        <v>-10019.902249</v>
       </c>
       <c r="AE81" s="11" t="n">
-        <v>-0.5874942499411766</v>
+        <v>-0.5894060146470589</v>
       </c>
       <c r="AF81" s="11" t="n">
-        <v>-52.84339814285714</v>
+        <v>-53.01535581481481</v>
       </c>
       <c r="AG81" s="11" t="n">
-        <v>-870.978933</v>
+        <v>-890.478933</v>
       </c>
       <c r="AH81" s="11" t="n">
-        <v>-0.05123405488235294</v>
+        <v>-0.05238111370588235</v>
       </c>
       <c r="AI81" s="11" t="n">
-        <v>-4.608354142857142</v>
+        <v>-4.711528746031746</v>
       </c>
       <c r="AJ81" s="11" t="n">
-        <v>-10858.381182</v>
+        <v>-10910.381182</v>
       </c>
       <c r="AK81" s="11" t="n">
-        <v>-0.6387283048235295</v>
+        <v>-0.6417871283529413</v>
       </c>
       <c r="AL81" s="11" t="n">
-        <v>-57.45175228571429</v>
+        <v>-57.72688456084656</v>
       </c>
     </row>
     <row r="82">
@@ -21291,40 +21400,40 @@
         <v>-21.92109557671958</v>
       </c>
       <c r="AA85" s="15" t="n">
-        <v>-8309.77853073</v>
+        <v>-8342.27853073</v>
       </c>
       <c r="AB85" s="15" t="n">
-        <v>-0.4888105018076471</v>
+        <v>-0.4907222665135294</v>
       </c>
       <c r="AC85" s="15" t="n">
-        <v>-43.9670821731746</v>
+        <v>-44.13903984513227</v>
       </c>
       <c r="AD85" s="15" t="n">
-        <v>-32186.94690527</v>
+        <v>-32219.44690527</v>
       </c>
       <c r="AE85" s="15" t="n">
-        <v>-1.893349817957059</v>
+        <v>-1.895261582662941</v>
       </c>
       <c r="AF85" s="15" t="n">
-        <v>-170.3013063770899</v>
+        <v>-170.4732640490476</v>
       </c>
       <c r="AG85" s="15" t="n">
-        <v>-1769.696893</v>
+        <v>-1789.196893</v>
       </c>
       <c r="AH85" s="15" t="n">
-        <v>-0.1040998172352941</v>
+        <v>-0.1052468760588235</v>
       </c>
       <c r="AI85" s="15" t="n">
-        <v>-9.363475624338625</v>
+        <v>-9.466650227513227</v>
       </c>
       <c r="AJ85" s="15" t="n">
-        <v>-33956.64379827</v>
+        <v>-34008.64379827</v>
       </c>
       <c r="AK85" s="15" t="n">
-        <v>-1.997449635192353</v>
+        <v>-2.000508458721765</v>
       </c>
       <c r="AL85" s="15" t="n">
-        <v>-179.6647820014286</v>
+        <v>-179.9399142765608</v>
       </c>
     </row>
     <row r="86">
@@ -25066,106 +25175,106 @@
         </is>
       </c>
       <c r="C128" s="13" t="n">
-        <v>-22.72266931</v>
+        <v>-22.591057</v>
       </c>
       <c r="D128" s="13" t="n">
-        <v>-0.001336627606470588</v>
+        <v>-0.001328885705882353</v>
       </c>
       <c r="E128" s="13" t="n">
-        <v>-0.1202257635449735</v>
+        <v>-0.1195294021164021</v>
       </c>
       <c r="F128" s="13" t="n">
-        <v>-216.84837834</v>
+        <v>-216.595653</v>
       </c>
       <c r="G128" s="13" t="n">
-        <v>-0.01275578696117647</v>
+        <v>-0.01274092076470588</v>
       </c>
       <c r="H128" s="13" t="n">
-        <v>-1.147345917142857</v>
+        <v>-1.146008746031746</v>
       </c>
       <c r="I128" s="13" t="n">
-        <v>-1.486783</v>
+        <v>-1.408413</v>
       </c>
       <c r="J128" s="13" t="n">
-        <v>-8.745782352941176e-05</v>
+        <v>-8.284782352941177e-05</v>
       </c>
       <c r="K128" s="13" t="n">
-        <v>-0.00786657671957672</v>
+        <v>-0.007451920634920634</v>
       </c>
       <c r="L128" s="13" t="n">
-        <v>-218.35724506</v>
+        <v>-218.312249</v>
       </c>
       <c r="M128" s="13" t="n">
-        <v>-0.01284454382705882</v>
+        <v>-0.012841897</v>
       </c>
       <c r="N128" s="13" t="n">
-        <v>-1.155329338941799</v>
+        <v>-1.155091264550265</v>
       </c>
       <c r="O128" s="13" t="n">
-        <v>-1.5529484</v>
+        <v>-1.549043</v>
       </c>
       <c r="P128" s="13" t="n">
-        <v>-9.134990588235295e-05</v>
+        <v>-9.112017647058823e-05</v>
       </c>
       <c r="Q128" s="13" t="n">
-        <v>-0.008216658201058201</v>
+        <v>-0.008195994708994708</v>
       </c>
       <c r="R128" s="13" t="n">
-        <v>-242.85835336</v>
+        <v>-242.651498</v>
       </c>
       <c r="S128" s="13" t="n">
-        <v>-0.01428578549176471</v>
+        <v>-0.01427361752941177</v>
       </c>
       <c r="T128" s="13" t="n">
-        <v>-1.284964832592593</v>
+        <v>-1.28387035978836</v>
       </c>
       <c r="U128" s="13" t="n">
-        <v>-243.43474794</v>
+        <v>-243.375606</v>
       </c>
       <c r="V128" s="13" t="n">
-        <v>-0.01431969105529412</v>
+        <v>-0.01431621211764706</v>
       </c>
       <c r="W128" s="13" t="n">
-        <v>-1.288014539365079</v>
+        <v>-1.287701619047619</v>
       </c>
       <c r="X128" s="13" t="n">
-        <v>-10.93261812</v>
+        <v>-10.873033</v>
       </c>
       <c r="Y128" s="13" t="n">
-        <v>-0.0006430951835294118</v>
+        <v>-0.0006395901764705882</v>
       </c>
       <c r="Z128" s="13" t="n">
-        <v>-0.05784454031746032</v>
+        <v>-0.05752927513227513</v>
       </c>
       <c r="AA128" s="13" t="n">
-        <v>-373.7960101699999</v>
+        <v>-373.71305</v>
       </c>
       <c r="AB128" s="13" t="n">
-        <v>-0.02198800059823529</v>
+        <v>-0.0219831205882353</v>
       </c>
       <c r="AC128" s="13" t="n">
-        <v>-1.977756667566137</v>
+        <v>-1.977317724867725</v>
       </c>
       <c r="AD128" s="13" t="n">
-        <v>-1331.9897537</v>
+        <v>-1331.069602</v>
       </c>
       <c r="AE128" s="13" t="n">
-        <v>-0.07835233845294118</v>
+        <v>-0.07829821188235295</v>
       </c>
       <c r="AF128" s="13" t="n">
-        <v>-7.047564834391534</v>
+        <v>-7.042696306878308</v>
       </c>
       <c r="AG128" s="13" t="n"/>
       <c r="AH128" s="13" t="n"/>
       <c r="AI128" s="13" t="n"/>
       <c r="AJ128" s="13" t="n">
-        <v>-1331.9897537</v>
+        <v>-1331.069602</v>
       </c>
       <c r="AK128" s="13" t="n">
-        <v>-0.07835233845294118</v>
+        <v>-0.07829821188235295</v>
       </c>
       <c r="AL128" s="13" t="n">
-        <v>-7.047564834391534</v>
+        <v>-7.042696306878308</v>
       </c>
     </row>
     <row r="129">
@@ -25490,106 +25599,106 @@
         </is>
       </c>
       <c r="C132" s="15" t="n">
-        <v>-5923.48742531</v>
+        <v>-5923.355813</v>
       </c>
       <c r="D132" s="15" t="n">
-        <v>-0.3484404367829412</v>
+        <v>-0.348432694882353</v>
       </c>
       <c r="E132" s="15" t="n">
-        <v>-31.34120330851852</v>
+        <v>-31.34050694708995</v>
       </c>
       <c r="F132" s="15" t="n">
-        <v>-7548.948538340001</v>
+        <v>-7548.695813</v>
       </c>
       <c r="G132" s="15" t="n">
-        <v>-0.4440557963729412</v>
+        <v>-0.4440409301764706</v>
       </c>
       <c r="H132" s="15" t="n">
-        <v>-39.9415266578836</v>
+        <v>-39.94018948677249</v>
       </c>
       <c r="I132" s="15" t="n">
-        <v>-961.200171</v>
+        <v>-961.121801</v>
       </c>
       <c r="J132" s="15" t="n">
-        <v>-0.05654118652941176</v>
+        <v>-0.05653657652941176</v>
       </c>
       <c r="K132" s="15" t="n">
-        <v>-5.08571519047619</v>
+        <v>-5.085300534391535</v>
       </c>
       <c r="L132" s="15" t="n">
-        <v>-6466.02187806</v>
+        <v>-6465.976882</v>
       </c>
       <c r="M132" s="15" t="n">
-        <v>-0.3803542281211765</v>
+        <v>-0.3803515812941177</v>
       </c>
       <c r="N132" s="15" t="n">
-        <v>-34.21175596857143</v>
+        <v>-34.21151789417989</v>
       </c>
       <c r="O132" s="15" t="n">
-        <v>-1318.8129594</v>
+        <v>-1318.809054</v>
       </c>
       <c r="P132" s="15" t="n">
-        <v>-0.07757723290588237</v>
+        <v>-0.07757700317647059</v>
       </c>
       <c r="Q132" s="15" t="n">
-        <v>-6.977846346031747</v>
+        <v>-6.977825682539683</v>
       </c>
       <c r="R132" s="15" t="n">
-        <v>-416.25800636</v>
+        <v>-416.051151</v>
       </c>
       <c r="S132" s="15" t="n">
-        <v>-0.02448576508</v>
+        <v>-0.02447359711764706</v>
       </c>
       <c r="T132" s="15" t="n">
-        <v>-2.202423314074074</v>
+        <v>-2.201328841269841</v>
       </c>
       <c r="U132" s="15" t="n">
-        <v>-1929.03055294</v>
+        <v>-1928.971411</v>
       </c>
       <c r="V132" s="15" t="n">
-        <v>-0.1134723854670588</v>
+        <v>-0.1134689065294118</v>
       </c>
       <c r="W132" s="15" t="n">
-        <v>-10.2065108621164</v>
+        <v>-10.20619794179894</v>
       </c>
       <c r="X132" s="15" t="n">
-        <v>-491.67387612</v>
+        <v>-491.614291</v>
       </c>
       <c r="Y132" s="15" t="n">
-        <v>-0.02892199271294118</v>
+        <v>-0.02891848770588235</v>
       </c>
       <c r="Z132" s="15" t="n">
-        <v>-2.60144908</v>
+        <v>-2.601133814814815</v>
       </c>
       <c r="AA132" s="15" t="n">
-        <v>-1664.07599517</v>
+        <v>-1663.993035</v>
       </c>
       <c r="AB132" s="15" t="n">
-        <v>-0.09788682324529413</v>
+        <v>-0.09788194323529412</v>
       </c>
       <c r="AC132" s="15" t="n">
-        <v>-8.804634895079365</v>
+        <v>-8.804195952380953</v>
       </c>
       <c r="AD132" s="15" t="n">
-        <v>-26719.5094027</v>
+        <v>-26718.589251</v>
       </c>
       <c r="AE132" s="15" t="n">
-        <v>-1.571735847217647</v>
+        <v>-1.571681720647059</v>
       </c>
       <c r="AF132" s="15" t="n">
-        <v>-141.3730656227513</v>
+        <v>-141.3681970952381</v>
       </c>
       <c r="AG132" s="15" t="n"/>
       <c r="AH132" s="15" t="n"/>
       <c r="AI132" s="15" t="n"/>
       <c r="AJ132" s="15" t="n">
-        <v>-26719.5094027</v>
+        <v>-26718.589251</v>
       </c>
       <c r="AK132" s="15" t="n">
-        <v>-1.571735847217647</v>
+        <v>-1.571681720647059</v>
       </c>
       <c r="AL132" s="15" t="n">
-        <v>-141.3730656227513</v>
+        <v>-141.3681970952381</v>
       </c>
     </row>
     <row r="133">
@@ -26345,94 +26454,94 @@
         </is>
       </c>
       <c r="C141" s="15" t="n">
-        <v>-8603.85010231</v>
+        <v>-8603.718489999999</v>
       </c>
       <c r="D141" s="15" t="n">
-        <v>-0.506108829547647</v>
+        <v>-0.5061010876470587</v>
       </c>
       <c r="E141" s="15" t="n">
-        <v>-45.52301641433862</v>
+        <v>-45.52232005291005</v>
       </c>
       <c r="F141" s="15" t="n">
-        <v>-10106.09958034</v>
+        <v>-10105.846855</v>
       </c>
       <c r="G141" s="15" t="n">
-        <v>-0.5944764459023529</v>
+        <v>-0.5944615797058823</v>
       </c>
       <c r="H141" s="15" t="n">
-        <v>-53.47142635100529</v>
+        <v>-53.47008917989418</v>
       </c>
       <c r="I141" s="15" t="n">
-        <v>-2763.428661</v>
+        <v>-2763.350291</v>
       </c>
       <c r="J141" s="15" t="n">
-        <v>-0.1625546271176471</v>
+        <v>-0.1625500171176471</v>
       </c>
       <c r="K141" s="15" t="n">
-        <v>-14.62131566666667</v>
+        <v>-14.62090101058201</v>
       </c>
       <c r="L141" s="15" t="n">
-        <v>-8658.626831059999</v>
+        <v>-8658.581835000001</v>
       </c>
       <c r="M141" s="15" t="n">
-        <v>-0.5093309900623528</v>
+        <v>-0.5093283432352942</v>
       </c>
       <c r="N141" s="15" t="n">
-        <v>-45.81284037597883</v>
+        <v>-45.8126023015873</v>
       </c>
       <c r="O141" s="15" t="n">
-        <v>-2654.29276086</v>
+        <v>-2654.28885546</v>
       </c>
       <c r="P141" s="15" t="n">
-        <v>-0.1561348682858824</v>
+        <v>-0.1561346385564706</v>
       </c>
       <c r="Q141" s="15" t="n">
-        <v>-14.0438770415873</v>
+        <v>-14.04385637809524</v>
       </c>
       <c r="R141" s="15" t="n">
-        <v>-3460.3731688</v>
+        <v>-3460.16631344</v>
       </c>
       <c r="S141" s="15" t="n">
-        <v>-0.2035513628705883</v>
+        <v>-0.2035391949082353</v>
       </c>
       <c r="T141" s="15" t="n">
-        <v>-18.30885274497355</v>
+        <v>-18.30775827216931</v>
       </c>
       <c r="U141" s="15" t="n">
-        <v>-4043.27011794</v>
+        <v>-4043.210976</v>
       </c>
       <c r="V141" s="15" t="n">
-        <v>-0.237839418702353</v>
+        <v>-0.2378359397647059</v>
       </c>
       <c r="W141" s="15" t="n">
-        <v>-21.39296358698413</v>
+        <v>-21.39265066666666</v>
       </c>
       <c r="X141" s="15" t="n">
-        <v>-3232.21012212</v>
+        <v>-3232.150537</v>
       </c>
       <c r="Y141" s="15" t="n">
-        <v>-0.1901300071835294</v>
+        <v>-0.1901265021764706</v>
       </c>
       <c r="Z141" s="15" t="n">
-        <v>-17.10164085777778</v>
+        <v>-17.10132559259259</v>
       </c>
       <c r="AA141" s="15" t="n">
-        <v>-4461.967366440001</v>
+        <v>-4461.884406270001</v>
       </c>
       <c r="AB141" s="15" t="n">
-        <v>-0.2624686686141177</v>
+        <v>-0.2624637886041177</v>
       </c>
       <c r="AC141" s="15" t="n">
-        <v>-23.60829294412699</v>
+        <v>-23.60785400142858</v>
       </c>
       <c r="AD141" s="15" t="n">
-        <v>-47984.11871087</v>
+        <v>-47983.19855917001</v>
       </c>
       <c r="AE141" s="15" t="n">
-        <v>-2.82259521828647</v>
+        <v>-2.822541091715882</v>
       </c>
       <c r="AF141" s="15" t="n">
-        <v>-253.8842259834391</v>
+        <v>-253.8793574559259</v>
       </c>
       <c r="AG141" s="15" t="n">
         <v>-110.536681</v>
@@ -26444,13 +26553,13 @@
         <v>-0.5848501640211641</v>
       </c>
       <c r="AJ141" s="15" t="n">
-        <v>-48094.65539187</v>
+        <v>-48093.73524017</v>
       </c>
       <c r="AK141" s="15" t="n">
-        <v>-2.829097375992352</v>
+        <v>-2.829043249421765</v>
       </c>
       <c r="AL141" s="15" t="n">
-        <v>-254.4690761474603</v>
+        <v>-254.4642076199471</v>
       </c>
     </row>
     <row r="142">
@@ -26660,34 +26769,34 @@
         <v>-1.038657989417989</v>
       </c>
       <c r="AA144" s="13" t="n">
-        <v>-105.582868</v>
+        <v>-73.082868</v>
       </c>
       <c r="AB144" s="13" t="n">
-        <v>-0.006210756941176471</v>
+        <v>-0.004298992235294118</v>
       </c>
       <c r="AC144" s="13" t="n">
-        <v>-0.5586395132275133</v>
+        <v>-0.3866818412698413</v>
       </c>
       <c r="AD144" s="13" t="n">
-        <v>-1030.660283</v>
+        <v>-998.160283</v>
       </c>
       <c r="AE144" s="13" t="n">
-        <v>-0.06062707547058824</v>
+        <v>-0.0587153107647059</v>
       </c>
       <c r="AF144" s="13" t="n">
-        <v>-5.45322901058201</v>
+        <v>-5.281271338624339</v>
       </c>
       <c r="AG144" s="13" t="n"/>
       <c r="AH144" s="13" t="n"/>
       <c r="AI144" s="13" t="n"/>
       <c r="AJ144" s="13" t="n">
-        <v>-1030.660283</v>
+        <v>-998.160283</v>
       </c>
       <c r="AK144" s="13" t="n">
-        <v>-0.06062707547058824</v>
+        <v>-0.0587153107647059</v>
       </c>
       <c r="AL144" s="13" t="n">
-        <v>-5.45322901058201</v>
+        <v>-5.281271338624339</v>
       </c>
     </row>
     <row r="145">
@@ -26891,34 +27000,34 @@
         <v>-1.038657989417989</v>
       </c>
       <c r="AA147" s="15" t="n">
-        <v>-105.582868</v>
+        <v>-73.082868</v>
       </c>
       <c r="AB147" s="15" t="n">
-        <v>-0.006210756941176471</v>
+        <v>-0.004298992235294118</v>
       </c>
       <c r="AC147" s="15" t="n">
-        <v>-0.5586395132275133</v>
+        <v>-0.3866818412698413</v>
       </c>
       <c r="AD147" s="15" t="n">
-        <v>-2701.773283</v>
+        <v>-2669.273283</v>
       </c>
       <c r="AE147" s="15" t="n">
-        <v>-0.1589278401764706</v>
+        <v>-0.1570160754705882</v>
       </c>
       <c r="AF147" s="15" t="n">
-        <v>-14.29509673544974</v>
+        <v>-14.12313906349206</v>
       </c>
       <c r="AG147" s="15" t="n"/>
       <c r="AH147" s="15" t="n"/>
       <c r="AI147" s="15" t="n"/>
       <c r="AJ147" s="15" t="n">
-        <v>-2701.773283</v>
+        <v>-2669.273283</v>
       </c>
       <c r="AK147" s="15" t="n">
-        <v>-0.1589278401764706</v>
+        <v>-0.1570160754705882</v>
       </c>
       <c r="AL147" s="15" t="n">
-        <v>-14.29509673544974</v>
+        <v>-14.12313906349206</v>
       </c>
     </row>
     <row r="148">
@@ -27061,138 +27170,168 @@
         <v>-0.1070750670899471</v>
       </c>
       <c r="AG149" s="11" t="n">
-        <v>-0.0157</v>
+        <v>-0.0182</v>
       </c>
       <c r="AH149" s="11" t="n">
-        <v>-9.235294117647058e-07</v>
+        <v>-1.070588235294118e-06</v>
       </c>
       <c r="AI149" s="11" t="n">
-        <v>-8.306878306878306e-05</v>
+        <v>-9.62962962962963e-05</v>
       </c>
       <c r="AJ149" s="11" t="n">
-        <v>-20.25288768</v>
+        <v>-20.25538768</v>
       </c>
       <c r="AK149" s="11" t="n">
-        <v>-0.001191346334117647</v>
+        <v>-0.001191493392941177</v>
       </c>
       <c r="AL149" s="11" t="n">
-        <v>-0.1071581358730159</v>
+        <v>-0.1071713633862434</v>
       </c>
     </row>
     <row r="150">
       <c r="B150" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Bank Provision Charges</t>
-        </is>
-      </c>
-      <c r="C150" s="13" t="n"/>
-      <c r="D150" s="13" t="n"/>
-      <c r="E150" s="13" t="n"/>
-      <c r="F150" s="13" t="n"/>
-      <c r="G150" s="13" t="n"/>
-      <c r="H150" s="13" t="n"/>
+          <t xml:space="preserve">        Bank Interest Income</t>
+        </is>
+      </c>
+      <c r="C150" s="13" t="n">
+        <v>-10.74138975</v>
+      </c>
+      <c r="D150" s="13" t="n">
+        <v>-0.0006318464558823531</v>
+      </c>
+      <c r="E150" s="13" t="n">
+        <v>-0.05683275000000001</v>
+      </c>
+      <c r="F150" s="13" t="n">
+        <v>-13.59808325</v>
+      </c>
+      <c r="G150" s="13" t="n">
+        <v>-0.00079988725</v>
+      </c>
+      <c r="H150" s="13" t="n">
+        <v>-0.07194753042328042</v>
+      </c>
       <c r="I150" s="13" t="n">
-        <v>-19.344233</v>
+        <v>-0.36473299</v>
       </c>
       <c r="J150" s="13" t="n">
-        <v>-0.001137896058823529</v>
+        <v>-2.145488176470588e-05</v>
       </c>
       <c r="K150" s="13" t="n">
-        <v>-0.1023504391534392</v>
-      </c>
-      <c r="L150" s="13" t="n"/>
-      <c r="M150" s="13" t="n"/>
-      <c r="N150" s="13" t="n"/>
-      <c r="O150" s="13" t="n"/>
-      <c r="P150" s="13" t="n"/>
-      <c r="Q150" s="13" t="n"/>
+        <v>-0.00192980417989418</v>
+      </c>
+      <c r="L150" s="13" t="n">
+        <v>-0.1635492</v>
+      </c>
+      <c r="M150" s="13" t="n">
+        <v>-9.620541176470589e-06</v>
+      </c>
+      <c r="N150" s="13" t="n">
+        <v>-0.0008653396825396826</v>
+      </c>
+      <c r="O150" s="13" t="n">
+        <v>-0.13147782</v>
+      </c>
+      <c r="P150" s="13" t="n">
+        <v>-7.733989411764705e-06</v>
+      </c>
+      <c r="Q150" s="13" t="n">
+        <v>-0.0006956498412698412</v>
+      </c>
       <c r="R150" s="13" t="n">
-        <v>-32.66944</v>
+        <v>-0.3955790299999999</v>
       </c>
       <c r="S150" s="13" t="n">
-        <v>-0.001921731764705882</v>
+        <v>-2.326935470588235e-05</v>
       </c>
       <c r="T150" s="13" t="n">
-        <v>-0.1728541798941799</v>
-      </c>
-      <c r="U150" s="13" t="n"/>
-      <c r="V150" s="13" t="n"/>
-      <c r="W150" s="13" t="n"/>
-      <c r="X150" s="13" t="n"/>
-      <c r="Y150" s="13" t="n"/>
-      <c r="Z150" s="13" t="n"/>
-      <c r="AA150" s="13" t="n"/>
-      <c r="AB150" s="13" t="n"/>
-      <c r="AC150" s="13" t="n"/>
+        <v>-0.002093010740740741</v>
+      </c>
+      <c r="U150" s="13" t="n">
+        <v>-0.1585512</v>
+      </c>
+      <c r="V150" s="13" t="n">
+        <v>-9.326541176470588e-06</v>
+      </c>
+      <c r="W150" s="13" t="n">
+        <v>-0.0008388952380952381</v>
+      </c>
+      <c r="X150" s="13" t="n">
+        <v>-0.20248972</v>
+      </c>
+      <c r="Y150" s="13" t="n">
+        <v>-1.191116e-05</v>
+      </c>
+      <c r="Z150" s="13" t="n">
+        <v>-0.00107137417989418</v>
+      </c>
+      <c r="AA150" s="13" t="n">
+        <v>-0.13335653</v>
+      </c>
+      <c r="AB150" s="13" t="n">
+        <v>-7.844501764705882e-06</v>
+      </c>
+      <c r="AC150" s="13" t="n">
+        <v>-0.0007055901058201058</v>
+      </c>
       <c r="AD150" s="13" t="n">
-        <v>-52.013673</v>
+        <v>-25.88920949</v>
       </c>
       <c r="AE150" s="13" t="n">
-        <v>-0.003059627823529412</v>
+        <v>-0.001522894675882353</v>
       </c>
       <c r="AF150" s="13" t="n">
-        <v>-0.2752046190476191</v>
+        <v>-0.1369799443915344</v>
       </c>
       <c r="AG150" s="13" t="n"/>
       <c r="AH150" s="13" t="n"/>
       <c r="AI150" s="13" t="n"/>
       <c r="AJ150" s="13" t="n">
-        <v>-52.013673</v>
+        <v>-25.88920949</v>
       </c>
       <c r="AK150" s="13" t="n">
-        <v>-0.003059627823529412</v>
+        <v>-0.001522894675882353</v>
       </c>
       <c r="AL150" s="13" t="n">
-        <v>-0.2752046190476191</v>
+        <v>-0.1369799443915344</v>
       </c>
     </row>
     <row r="151">
       <c r="B151" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Forex</t>
-        </is>
-      </c>
-      <c r="C151" s="11" t="n">
-        <v>-0.5023986</v>
-      </c>
-      <c r="D151" s="11" t="n">
-        <v>-2.955285882352941e-05</v>
-      </c>
-      <c r="E151" s="11" t="n">
-        <v>-0.002658193650793651</v>
-      </c>
+          <t xml:space="preserve">        Bank Provision Charges</t>
+        </is>
+      </c>
+      <c r="C151" s="11" t="n"/>
+      <c r="D151" s="11" t="n"/>
+      <c r="E151" s="11" t="n"/>
       <c r="F151" s="11" t="n"/>
       <c r="G151" s="11" t="n"/>
       <c r="H151" s="11" t="n"/>
       <c r="I151" s="11" t="n">
-        <v>-0.237149</v>
+        <v>-19.344233</v>
       </c>
       <c r="J151" s="11" t="n">
-        <v>-1.394994117647059e-05</v>
+        <v>-0.001137896058823529</v>
       </c>
       <c r="K151" s="11" t="n">
-        <v>-0.001254756613756614</v>
+        <v>-0.1023504391534392</v>
       </c>
       <c r="L151" s="11" t="n"/>
       <c r="M151" s="11" t="n"/>
       <c r="N151" s="11" t="n"/>
-      <c r="O151" s="11" t="n">
-        <v>-0.476</v>
-      </c>
-      <c r="P151" s="11" t="n">
-        <v>-2.8e-05</v>
-      </c>
-      <c r="Q151" s="11" t="n">
-        <v>-0.002518518518518518</v>
-      </c>
+      <c r="O151" s="11" t="n"/>
+      <c r="P151" s="11" t="n"/>
+      <c r="Q151" s="11" t="n"/>
       <c r="R151" s="11" t="n">
-        <v>-8.215064999999999</v>
+        <v>-32.66944</v>
       </c>
       <c r="S151" s="11" t="n">
-        <v>-0.0004832391176470588</v>
+        <v>-0.001921731764705882</v>
       </c>
       <c r="T151" s="11" t="n">
-        <v>-0.04346595238095238</v>
+        <v>-0.1728541798941799</v>
       </c>
       <c r="U151" s="11" t="n"/>
       <c r="V151" s="11" t="n"/>
@@ -27204,752 +27343,831 @@
       <c r="AB151" s="11" t="n"/>
       <c r="AC151" s="11" t="n"/>
       <c r="AD151" s="11" t="n">
-        <v>-9.4306126</v>
+        <v>-52.013673</v>
       </c>
       <c r="AE151" s="11" t="n">
-        <v>-0.0005547419176470588</v>
+        <v>-0.003059627823529412</v>
       </c>
       <c r="AF151" s="11" t="n">
-        <v>-0.04989742116402116</v>
+        <v>-0.2752046190476191</v>
       </c>
       <c r="AG151" s="11" t="n"/>
       <c r="AH151" s="11" t="n"/>
       <c r="AI151" s="11" t="n"/>
       <c r="AJ151" s="11" t="n">
-        <v>-9.4306126</v>
+        <v>-52.013673</v>
       </c>
       <c r="AK151" s="11" t="n">
-        <v>-0.0005547419176470588</v>
+        <v>-0.003059627823529412</v>
       </c>
       <c r="AL151" s="11" t="n">
-        <v>-0.04989742116402116</v>
+        <v>-0.2752046190476191</v>
       </c>
     </row>
     <row r="152">
       <c r="B152" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Interest on Bank Term Loans</t>
+          <t xml:space="preserve">        Forex</t>
         </is>
       </c>
       <c r="C152" s="13" t="n">
-        <v>-304.08964244</v>
+        <v>-0.5023986</v>
       </c>
       <c r="D152" s="13" t="n">
-        <v>-0.01788762602588235</v>
+        <v>-2.955285882352941e-05</v>
       </c>
       <c r="E152" s="13" t="n">
-        <v>-1.608939907089947</v>
-      </c>
-      <c r="F152" s="13" t="n">
-        <v>-192.54891591</v>
-      </c>
-      <c r="G152" s="13" t="n">
-        <v>-0.01132640681823529</v>
-      </c>
-      <c r="H152" s="13" t="n">
-        <v>-1.018777332857143</v>
-      </c>
+        <v>-0.002658193650793651</v>
+      </c>
+      <c r="F152" s="13" t="n"/>
+      <c r="G152" s="13" t="n"/>
+      <c r="H152" s="13" t="n"/>
       <c r="I152" s="13" t="n">
-        <v>-154.77218899</v>
+        <v>-0.237149</v>
       </c>
       <c r="J152" s="13" t="n">
-        <v>-0.009104246411176471</v>
+        <v>-1.394994117647059e-05</v>
       </c>
       <c r="K152" s="13" t="n">
-        <v>-0.8189004708465609</v>
-      </c>
-      <c r="L152" s="13" t="n">
-        <v>-185.50154514</v>
-      </c>
-      <c r="M152" s="13" t="n">
-        <v>-0.01091185559647059</v>
-      </c>
-      <c r="N152" s="13" t="n">
-        <v>-0.9814896568253968</v>
-      </c>
+        <v>-0.001254756613756614</v>
+      </c>
+      <c r="L152" s="13" t="n"/>
+      <c r="M152" s="13" t="n"/>
+      <c r="N152" s="13" t="n"/>
       <c r="O152" s="13" t="n">
-        <v>-2857.13152842</v>
+        <v>-0.476</v>
       </c>
       <c r="P152" s="13" t="n">
-        <v>-0.1680665604952941</v>
+        <v>-2.8e-05</v>
       </c>
       <c r="Q152" s="13" t="n">
-        <v>-15.11709803396825</v>
+        <v>-0.002518518518518518</v>
       </c>
       <c r="R152" s="13" t="n">
-        <v>-185.57171467</v>
+        <v>-8.215064999999999</v>
       </c>
       <c r="S152" s="13" t="n">
-        <v>-0.01091598321588235</v>
+        <v>-0.0004832391176470588</v>
       </c>
       <c r="T152" s="13" t="n">
-        <v>-0.981860924179894</v>
-      </c>
-      <c r="U152" s="13" t="n">
-        <v>-191.66183426</v>
-      </c>
-      <c r="V152" s="13" t="n">
-        <v>-0.01127422554470588</v>
-      </c>
-      <c r="W152" s="13" t="n">
-        <v>-1.014083779153439</v>
-      </c>
-      <c r="X152" s="13" t="n">
-        <v>-195.2527816</v>
-      </c>
-      <c r="Y152" s="13" t="n">
-        <v>-0.01148545774117647</v>
-      </c>
-      <c r="Z152" s="13" t="n">
-        <v>-1.033083500529101</v>
-      </c>
-      <c r="AA152" s="13" t="n">
-        <v>-182.57253836</v>
-      </c>
-      <c r="AB152" s="13" t="n">
-        <v>-0.01073956108</v>
-      </c>
-      <c r="AC152" s="13" t="n">
-        <v>-0.9659922664550266</v>
-      </c>
+        <v>-0.04346595238095238</v>
+      </c>
+      <c r="U152" s="13" t="n"/>
+      <c r="V152" s="13" t="n"/>
+      <c r="W152" s="13" t="n"/>
+      <c r="X152" s="13" t="n"/>
+      <c r="Y152" s="13" t="n"/>
+      <c r="Z152" s="13" t="n"/>
+      <c r="AA152" s="13" t="n"/>
+      <c r="AB152" s="13" t="n"/>
+      <c r="AC152" s="13" t="n"/>
       <c r="AD152" s="13" t="n">
-        <v>-4449.10268979</v>
+        <v>-9.4306126</v>
       </c>
       <c r="AE152" s="13" t="n">
-        <v>-0.2617119229288236</v>
+        <v>-0.0005547419176470588</v>
       </c>
       <c r="AF152" s="13" t="n">
-        <v>-23.54022587190476</v>
+        <v>-0.04989742116402116</v>
       </c>
       <c r="AG152" s="13" t="n"/>
       <c r="AH152" s="13" t="n"/>
       <c r="AI152" s="13" t="n"/>
       <c r="AJ152" s="13" t="n">
-        <v>-4449.10268979</v>
+        <v>-9.4306126</v>
       </c>
       <c r="AK152" s="13" t="n">
-        <v>-0.2617119229288236</v>
+        <v>-0.0005547419176470588</v>
       </c>
       <c r="AL152" s="13" t="n">
-        <v>-23.54022587190476</v>
+        <v>-0.04989742116402116</v>
       </c>
     </row>
     <row r="153">
       <c r="B153" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Interest on Bank Working Capital Loans</t>
-        </is>
-      </c>
-      <c r="C153" s="11" t="n"/>
-      <c r="D153" s="11" t="n"/>
-      <c r="E153" s="11" t="n"/>
-      <c r="F153" s="11" t="n"/>
-      <c r="G153" s="11" t="n"/>
-      <c r="H153" s="11" t="n"/>
+          <t xml:space="preserve">        Interest on Bank Term Loans</t>
+        </is>
+      </c>
+      <c r="C153" s="11" t="n">
+        <v>-293.479865</v>
+      </c>
+      <c r="D153" s="11" t="n">
+        <v>-0.01726352147058824</v>
+      </c>
+      <c r="E153" s="11" t="n">
+        <v>-1.552803518518519</v>
+      </c>
+      <c r="F153" s="11" t="n">
+        <v>-179.203558</v>
+      </c>
+      <c r="G153" s="11" t="n">
+        <v>-0.01054138576470588</v>
+      </c>
+      <c r="H153" s="11" t="n">
+        <v>-0.9481669735449735</v>
+      </c>
       <c r="I153" s="11" t="n">
-        <v>-268.756578</v>
+        <v>-154.485826</v>
       </c>
       <c r="J153" s="11" t="n">
-        <v>-0.01580921047058824</v>
+        <v>-0.009087401529411765</v>
       </c>
       <c r="K153" s="11" t="n">
-        <v>-1.421992476190476</v>
+        <v>-0.8173853227513228</v>
       </c>
       <c r="L153" s="11" t="n">
-        <v>-171.119871</v>
+        <v>-185.382992</v>
       </c>
       <c r="M153" s="11" t="n">
-        <v>-0.01006587476470588</v>
+        <v>-0.01090488188235294</v>
       </c>
       <c r="N153" s="11" t="n">
-        <v>-0.9053961428571428</v>
+        <v>-0.9808623915343916</v>
       </c>
       <c r="O153" s="11" t="n">
-        <v>-96.386746</v>
+        <v>-2857.003956</v>
       </c>
       <c r="P153" s="11" t="n">
-        <v>-0.005669808588235294</v>
+        <v>-0.1680590562352941</v>
       </c>
       <c r="Q153" s="11" t="n">
-        <v>-0.5099827830687831</v>
+        <v>-15.11642304761905</v>
       </c>
       <c r="R153" s="11" t="n">
-        <v>-106.357788</v>
+        <v>-185.382991</v>
       </c>
       <c r="S153" s="11" t="n">
-        <v>-0.006256340470588235</v>
+        <v>-0.01090488182352941</v>
       </c>
       <c r="T153" s="11" t="n">
-        <v>-0.562739619047619</v>
+        <v>-0.9808623862433863</v>
       </c>
       <c r="U153" s="11" t="n">
-        <v>-103.034108</v>
+        <v>-191.562425</v>
       </c>
       <c r="V153" s="11" t="n">
-        <v>-0.006060829882352942</v>
+        <v>-0.01126837794117647</v>
       </c>
       <c r="W153" s="11" t="n">
-        <v>-0.5451540105820106</v>
+        <v>-1.013557804232804</v>
       </c>
       <c r="X153" s="11" t="n">
-        <v>-103.034108</v>
+        <v>-195.109877</v>
       </c>
       <c r="Y153" s="11" t="n">
-        <v>-0.006060829882352942</v>
+        <v>-0.01147705158823529</v>
       </c>
       <c r="Z153" s="11" t="n">
-        <v>-0.5451540105820106</v>
+        <v>-1.032327391534392</v>
       </c>
       <c r="AA153" s="11" t="n">
-        <v>-99.710427</v>
+        <v>-182.522142</v>
       </c>
       <c r="AB153" s="11" t="n">
-        <v>-0.005865319235294117</v>
+        <v>-0.01073659658823529</v>
       </c>
       <c r="AC153" s="11" t="n">
-        <v>-0.5275683968253968</v>
+        <v>-0.9657256190476191</v>
       </c>
       <c r="AD153" s="11" t="n">
-        <v>-948.3996260000001</v>
+        <v>-4424.133632</v>
       </c>
       <c r="AE153" s="11" t="n">
-        <v>-0.05578821329411765</v>
+        <v>-0.2602431548235294</v>
       </c>
       <c r="AF153" s="11" t="n">
-        <v>-5.01798743915344</v>
+        <v>-23.40811445502645</v>
       </c>
       <c r="AG153" s="11" t="n"/>
       <c r="AH153" s="11" t="n"/>
       <c r="AI153" s="11" t="n"/>
       <c r="AJ153" s="11" t="n">
-        <v>-948.3996260000001</v>
+        <v>-4424.133632</v>
       </c>
       <c r="AK153" s="11" t="n">
-        <v>-0.05578821329411765</v>
+        <v>-0.2602431548235294</v>
       </c>
       <c r="AL153" s="11" t="n">
-        <v>-5.01798743915344</v>
+        <v>-23.40811445502645</v>
       </c>
     </row>
     <row r="154">
       <c r="B154" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Loan Related Charges</t>
+          <t xml:space="preserve">        Interest on Bank Working Capital Loans</t>
         </is>
       </c>
       <c r="C154" s="13" t="n"/>
       <c r="D154" s="13" t="n"/>
       <c r="E154" s="13" t="n"/>
-      <c r="F154" s="13" t="n">
-        <v>-773.891532</v>
-      </c>
-      <c r="G154" s="13" t="n">
-        <v>-0.04552303129411765</v>
-      </c>
-      <c r="H154" s="13" t="n">
-        <v>-4.09466419047619</v>
-      </c>
-      <c r="I154" s="13" t="n"/>
-      <c r="J154" s="13" t="n"/>
-      <c r="K154" s="13" t="n"/>
-      <c r="L154" s="13" t="n"/>
-      <c r="M154" s="13" t="n"/>
-      <c r="N154" s="13" t="n"/>
-      <c r="O154" s="13" t="n"/>
-      <c r="P154" s="13" t="n"/>
-      <c r="Q154" s="13" t="n"/>
-      <c r="R154" s="13" t="n"/>
-      <c r="S154" s="13" t="n"/>
-      <c r="T154" s="13" t="n"/>
-      <c r="U154" s="13" t="n"/>
-      <c r="V154" s="13" t="n"/>
-      <c r="W154" s="13" t="n"/>
-      <c r="X154" s="13" t="n"/>
-      <c r="Y154" s="13" t="n"/>
-      <c r="Z154" s="13" t="n"/>
-      <c r="AA154" s="13" t="n"/>
-      <c r="AB154" s="13" t="n"/>
-      <c r="AC154" s="13" t="n"/>
+      <c r="F154" s="13" t="n"/>
+      <c r="G154" s="13" t="n"/>
+      <c r="H154" s="13" t="n"/>
+      <c r="I154" s="13" t="n">
+        <v>-268.756578</v>
+      </c>
+      <c r="J154" s="13" t="n">
+        <v>-0.01580921047058824</v>
+      </c>
+      <c r="K154" s="13" t="n">
+        <v>-1.421992476190476</v>
+      </c>
+      <c r="L154" s="13" t="n">
+        <v>-171.119871</v>
+      </c>
+      <c r="M154" s="13" t="n">
+        <v>-0.01006587476470588</v>
+      </c>
+      <c r="N154" s="13" t="n">
+        <v>-0.9053961428571428</v>
+      </c>
+      <c r="O154" s="13" t="n">
+        <v>-96.386746</v>
+      </c>
+      <c r="P154" s="13" t="n">
+        <v>-0.005669808588235294</v>
+      </c>
+      <c r="Q154" s="13" t="n">
+        <v>-0.5099827830687831</v>
+      </c>
+      <c r="R154" s="13" t="n">
+        <v>-106.357788</v>
+      </c>
+      <c r="S154" s="13" t="n">
+        <v>-0.006256340470588235</v>
+      </c>
+      <c r="T154" s="13" t="n">
+        <v>-0.562739619047619</v>
+      </c>
+      <c r="U154" s="13" t="n">
+        <v>-103.034108</v>
+      </c>
+      <c r="V154" s="13" t="n">
+        <v>-0.006060829882352942</v>
+      </c>
+      <c r="W154" s="13" t="n">
+        <v>-0.5451540105820106</v>
+      </c>
+      <c r="X154" s="13" t="n">
+        <v>-103.034108</v>
+      </c>
+      <c r="Y154" s="13" t="n">
+        <v>-0.006060829882352942</v>
+      </c>
+      <c r="Z154" s="13" t="n">
+        <v>-0.5451540105820106</v>
+      </c>
+      <c r="AA154" s="13" t="n">
+        <v>-99.710427</v>
+      </c>
+      <c r="AB154" s="13" t="n">
+        <v>-0.005865319235294117</v>
+      </c>
+      <c r="AC154" s="13" t="n">
+        <v>-0.5275683968253968</v>
+      </c>
       <c r="AD154" s="13" t="n">
-        <v>-773.891532</v>
+        <v>-948.3996260000001</v>
       </c>
       <c r="AE154" s="13" t="n">
-        <v>-0.04552303129411765</v>
+        <v>-0.05578821329411765</v>
       </c>
       <c r="AF154" s="13" t="n">
-        <v>-4.09466419047619</v>
+        <v>-5.01798743915344</v>
       </c>
       <c r="AG154" s="13" t="n"/>
       <c r="AH154" s="13" t="n"/>
       <c r="AI154" s="13" t="n"/>
       <c r="AJ154" s="13" t="n">
+        <v>-948.3996260000001</v>
+      </c>
+      <c r="AK154" s="13" t="n">
+        <v>-0.05578821329411765</v>
+      </c>
+      <c r="AL154" s="13" t="n">
+        <v>-5.01798743915344</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="B155" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        Loan Related Charges</t>
+        </is>
+      </c>
+      <c r="C155" s="11" t="n"/>
+      <c r="D155" s="11" t="n"/>
+      <c r="E155" s="11" t="n"/>
+      <c r="F155" s="11" t="n">
         <v>-773.891532</v>
       </c>
-      <c r="AK154" s="13" t="n">
+      <c r="G155" s="11" t="n">
         <v>-0.04552303129411765</v>
       </c>
-      <c r="AL154" s="13" t="n">
+      <c r="H155" s="11" t="n">
         <v>-4.09466419047619</v>
       </c>
-    </row>
-    <row r="155">
-      <c r="B155" s="14" t="inlineStr">
+      <c r="I155" s="11" t="n"/>
+      <c r="J155" s="11" t="n"/>
+      <c r="K155" s="11" t="n"/>
+      <c r="L155" s="11" t="n"/>
+      <c r="M155" s="11" t="n"/>
+      <c r="N155" s="11" t="n"/>
+      <c r="O155" s="11" t="n"/>
+      <c r="P155" s="11" t="n"/>
+      <c r="Q155" s="11" t="n"/>
+      <c r="R155" s="11" t="n"/>
+      <c r="S155" s="11" t="n"/>
+      <c r="T155" s="11" t="n"/>
+      <c r="U155" s="11" t="n"/>
+      <c r="V155" s="11" t="n"/>
+      <c r="W155" s="11" t="n"/>
+      <c r="X155" s="11" t="n"/>
+      <c r="Y155" s="11" t="n"/>
+      <c r="Z155" s="11" t="n"/>
+      <c r="AA155" s="11" t="n"/>
+      <c r="AB155" s="11" t="n"/>
+      <c r="AC155" s="11" t="n"/>
+      <c r="AD155" s="11" t="n">
+        <v>-773.891532</v>
+      </c>
+      <c r="AE155" s="11" t="n">
+        <v>-0.04552303129411765</v>
+      </c>
+      <c r="AF155" s="11" t="n">
+        <v>-4.09466419047619</v>
+      </c>
+      <c r="AG155" s="11" t="n"/>
+      <c r="AH155" s="11" t="n"/>
+      <c r="AI155" s="11" t="n"/>
+      <c r="AJ155" s="11" t="n">
+        <v>-773.891532</v>
+      </c>
+      <c r="AK155" s="11" t="n">
+        <v>-0.04552303129411765</v>
+      </c>
+      <c r="AL155" s="11" t="n">
+        <v>-4.09466419047619</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="B156" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    TOTAL FINANCE COST</t>
         </is>
       </c>
-      <c r="C155" s="15" t="n">
-        <v>-308.68554172</v>
-      </c>
-      <c r="D155" s="15" t="n">
-        <v>-0.01815797304235294</v>
-      </c>
-      <c r="E155" s="15" t="n">
-        <v>-1.633256834497355</v>
-      </c>
-      <c r="F155" s="15" t="n">
-        <v>-967.36514791</v>
-      </c>
-      <c r="G155" s="15" t="n">
-        <v>-0.05690383223</v>
-      </c>
-      <c r="H155" s="15" t="n">
-        <v>-5.118334115925926</v>
-      </c>
-      <c r="I155" s="15" t="n">
-        <v>-446.67468899</v>
-      </c>
-      <c r="J155" s="15" t="n">
-        <v>-0.02627498170529412</v>
-      </c>
-      <c r="K155" s="15" t="n">
-        <v>-2.363358142804233</v>
-      </c>
-      <c r="L155" s="15" t="n">
-        <v>-358.18051414</v>
-      </c>
-      <c r="M155" s="15" t="n">
-        <v>-0.0210694420082353</v>
-      </c>
-      <c r="N155" s="15" t="n">
-        <v>-1.895134995449736</v>
-      </c>
-      <c r="O155" s="15" t="n">
-        <v>-2956.57269042</v>
-      </c>
-      <c r="P155" s="15" t="n">
-        <v>-0.1739160406129412</v>
-      </c>
-      <c r="Q155" s="15" t="n">
-        <v>-15.64324174825397</v>
-      </c>
-      <c r="R155" s="15" t="n">
-        <v>-334.28723067</v>
-      </c>
-      <c r="S155" s="15" t="n">
-        <v>-0.01966395474529412</v>
-      </c>
-      <c r="T155" s="15" t="n">
-        <v>-1.768715506190476</v>
-      </c>
-      <c r="U155" s="15" t="n">
-        <v>-296.97908626</v>
-      </c>
-      <c r="V155" s="15" t="n">
-        <v>-0.01746935801529412</v>
-      </c>
-      <c r="W155" s="15" t="n">
-        <v>-1.571317916719577</v>
-      </c>
-      <c r="X155" s="15" t="n">
-        <v>-300.6061656</v>
-      </c>
-      <c r="Y155" s="15" t="n">
-        <v>-0.01768271562352941</v>
-      </c>
-      <c r="Z155" s="15" t="n">
-        <v>-1.590508812698413</v>
-      </c>
-      <c r="AA155" s="15" t="n">
-        <v>-283.72425536</v>
-      </c>
-      <c r="AB155" s="15" t="n">
-        <v>-0.01668966208</v>
-      </c>
-      <c r="AC155" s="15" t="n">
-        <v>-1.501186536296296</v>
-      </c>
-      <c r="AD155" s="15" t="n">
-        <v>-6253.07532107</v>
-      </c>
-      <c r="AE155" s="15" t="n">
-        <v>-0.3678279600629413</v>
-      </c>
-      <c r="AF155" s="15" t="n">
-        <v>-33.08505460883597</v>
-      </c>
-      <c r="AG155" s="15" t="n">
-        <v>-0.0157</v>
-      </c>
-      <c r="AH155" s="15" t="n">
-        <v>-9.235294117647058e-07</v>
-      </c>
-      <c r="AI155" s="15" t="n">
-        <v>-8.306878306878306e-05</v>
-      </c>
-      <c r="AJ155" s="15" t="n">
-        <v>-6253.09102107</v>
-      </c>
-      <c r="AK155" s="15" t="n">
-        <v>-0.3678288835923531</v>
-      </c>
-      <c r="AL155" s="15" t="n">
-        <v>-33.08513767761904</v>
-      </c>
-    </row>
-    <row r="156">
-      <c r="B156" s="18" t="inlineStr">
-        <is>
-          <t>TOTAL OUTFLOW</t>
-        </is>
-      </c>
-      <c r="C156" s="19" t="n">
-        <v>-44493.15819503</v>
-      </c>
-      <c r="D156" s="19" t="n">
-        <v>-2.617244599707647</v>
-      </c>
-      <c r="E156" s="19" t="n">
-        <v>-235.4135354234392</v>
-      </c>
-      <c r="F156" s="19" t="n">
-        <v>-87290.80569813</v>
-      </c>
-      <c r="G156" s="19" t="n">
-        <v>-5.134753276360589</v>
-      </c>
-      <c r="H156" s="19" t="n">
-        <v>-461.8561148049207</v>
-      </c>
-      <c r="I156" s="19" t="n">
-        <v>-56595.91977199</v>
-      </c>
-      <c r="J156" s="19" t="n">
-        <v>-3.329171751293529</v>
-      </c>
-      <c r="K156" s="19" t="n">
-        <v>-299.44931096291</v>
-      </c>
-      <c r="L156" s="19" t="n">
-        <v>-47009.3796492</v>
-      </c>
-      <c r="M156" s="19" t="n">
-        <v>-2.765257626423529</v>
-      </c>
-      <c r="N156" s="19" t="n">
-        <v>-248.7268764507936</v>
-      </c>
-      <c r="O156" s="19" t="n">
-        <v>-27914.58608382</v>
-      </c>
-      <c r="P156" s="19" t="n">
-        <v>-1.642034475518823</v>
-      </c>
-      <c r="Q156" s="19" t="n">
-        <v>-147.6962226657143</v>
-      </c>
-      <c r="R156" s="19" t="n">
-        <v>-7977.84095347</v>
-      </c>
-      <c r="S156" s="19" t="n">
-        <v>-0.4692847619688236</v>
-      </c>
-      <c r="T156" s="19" t="n">
-        <v>-42.21079869560847</v>
-      </c>
-      <c r="U156" s="19" t="n">
-        <v>-8224.5495102</v>
-      </c>
-      <c r="V156" s="19" t="n">
-        <v>-0.4837970300117647</v>
-      </c>
-      <c r="W156" s="19" t="n">
-        <v>-43.51613497460318</v>
-      </c>
-      <c r="X156" s="19" t="n">
-        <v>-9565.196761719999</v>
-      </c>
-      <c r="Y156" s="19" t="n">
-        <v>-0.5626586330423529</v>
-      </c>
-      <c r="Z156" s="19" t="n">
-        <v>-50.60950667576719</v>
-      </c>
-      <c r="AA156" s="19" t="n">
-        <v>-15104.73649053</v>
-      </c>
-      <c r="AB156" s="19" t="n">
-        <v>-0.8885139112076471</v>
-      </c>
-      <c r="AC156" s="19" t="n">
-        <v>-79.91924069063492</v>
-      </c>
-      <c r="AD156" s="19" t="n">
-        <v>-304176.1731140899</v>
-      </c>
-      <c r="AE156" s="19" t="n">
-        <v>-17.89271606553471</v>
-      </c>
-      <c r="AF156" s="19" t="n">
-        <v>-1609.397741344391</v>
-      </c>
-      <c r="AG156" s="19" t="n">
-        <v>-1880.249274</v>
-      </c>
-      <c r="AH156" s="19" t="n">
-        <v>-0.1106028984705882</v>
-      </c>
-      <c r="AI156" s="19" t="n">
-        <v>-9.948408857142857</v>
-      </c>
-      <c r="AJ156" s="19" t="n">
-        <v>-306056.4223880899</v>
-      </c>
-      <c r="AK156" s="19" t="n">
-        <v>-18.0033189640053</v>
-      </c>
-      <c r="AL156" s="19" t="n">
-        <v>-1619.346150201534</v>
+      <c r="C156" s="15" t="n">
+        <v>-308.81715403</v>
+      </c>
+      <c r="D156" s="15" t="n">
+        <v>-0.01816571494294118</v>
+      </c>
+      <c r="E156" s="15" t="n">
+        <v>-1.633953195925926</v>
+      </c>
+      <c r="F156" s="15" t="n">
+        <v>-967.61787325</v>
+      </c>
+      <c r="G156" s="15" t="n">
+        <v>-0.05691869842647059</v>
+      </c>
+      <c r="H156" s="15" t="n">
+        <v>-5.119671287037037</v>
+      </c>
+      <c r="I156" s="15" t="n">
+        <v>-446.75305899</v>
+      </c>
+      <c r="J156" s="15" t="n">
+        <v>-0.02627959170529412</v>
+      </c>
+      <c r="K156" s="15" t="n">
+        <v>-2.363772798888889</v>
+      </c>
+      <c r="L156" s="15" t="n">
+        <v>-358.2255102</v>
+      </c>
+      <c r="M156" s="15" t="n">
+        <v>-0.02107208883529412</v>
+      </c>
+      <c r="N156" s="15" t="n">
+        <v>-1.89537306984127</v>
+      </c>
+      <c r="O156" s="15" t="n">
+        <v>-2956.57659582</v>
+      </c>
+      <c r="P156" s="15" t="n">
+        <v>-0.1739162703423529</v>
+      </c>
+      <c r="Q156" s="15" t="n">
+        <v>-15.64326241174603</v>
+      </c>
+      <c r="R156" s="15" t="n">
+        <v>-334.4940860299999</v>
+      </c>
+      <c r="S156" s="15" t="n">
+        <v>-0.01967612270764706</v>
+      </c>
+      <c r="T156" s="15" t="n">
+        <v>-1.769809978994709</v>
+      </c>
+      <c r="U156" s="15" t="n">
+        <v>-297.0382282</v>
+      </c>
+      <c r="V156" s="15" t="n">
+        <v>-0.01747283695294118</v>
+      </c>
+      <c r="W156" s="15" t="n">
+        <v>-1.571630837037037</v>
+      </c>
+      <c r="X156" s="15" t="n">
+        <v>-300.66575072</v>
+      </c>
+      <c r="Y156" s="15" t="n">
+        <v>-0.01768622063058824</v>
+      </c>
+      <c r="Z156" s="15" t="n">
+        <v>-1.590824077883598</v>
+      </c>
+      <c r="AA156" s="15" t="n">
+        <v>-283.80721553</v>
+      </c>
+      <c r="AB156" s="15" t="n">
+        <v>-0.01669454209</v>
+      </c>
+      <c r="AC156" s="15" t="n">
+        <v>-1.501625478994709</v>
+      </c>
+      <c r="AD156" s="15" t="n">
+        <v>-6253.99547277</v>
+      </c>
+      <c r="AE156" s="15" t="n">
+        <v>-0.3678820866335294</v>
+      </c>
+      <c r="AF156" s="15" t="n">
+        <v>-33.08992313634921</v>
+      </c>
+      <c r="AG156" s="15" t="n">
+        <v>-0.0182</v>
+      </c>
+      <c r="AH156" s="15" t="n">
+        <v>-1.070588235294118e-06</v>
+      </c>
+      <c r="AI156" s="15" t="n">
+        <v>-9.62962962962963e-05</v>
+      </c>
+      <c r="AJ156" s="15" t="n">
+        <v>-6254.01367277</v>
+      </c>
+      <c r="AK156" s="15" t="n">
+        <v>-0.3678831572217647</v>
+      </c>
+      <c r="AL156" s="15" t="n">
+        <v>-33.09001943264551</v>
       </c>
     </row>
     <row r="157">
       <c r="B157" s="18" t="inlineStr">
         <is>
+          <t>TOTAL OUTFLOW</t>
+        </is>
+      </c>
+      <c r="C157" s="19" t="n">
+        <v>-44493.15819503</v>
+      </c>
+      <c r="D157" s="19" t="n">
+        <v>-2.617244599707647</v>
+      </c>
+      <c r="E157" s="19" t="n">
+        <v>-235.4135354234392</v>
+      </c>
+      <c r="F157" s="19" t="n">
+        <v>-87290.80569813</v>
+      </c>
+      <c r="G157" s="19" t="n">
+        <v>-5.134753276360589</v>
+      </c>
+      <c r="H157" s="19" t="n">
+        <v>-461.8561148049207</v>
+      </c>
+      <c r="I157" s="19" t="n">
+        <v>-56595.91977199</v>
+      </c>
+      <c r="J157" s="19" t="n">
+        <v>-3.329171751293529</v>
+      </c>
+      <c r="K157" s="19" t="n">
+        <v>-299.44931096291</v>
+      </c>
+      <c r="L157" s="19" t="n">
+        <v>-47009.3796492</v>
+      </c>
+      <c r="M157" s="19" t="n">
+        <v>-2.765257626423529</v>
+      </c>
+      <c r="N157" s="19" t="n">
+        <v>-248.7268764507936</v>
+      </c>
+      <c r="O157" s="19" t="n">
+        <v>-27914.58608382</v>
+      </c>
+      <c r="P157" s="19" t="n">
+        <v>-1.642034475518823</v>
+      </c>
+      <c r="Q157" s="19" t="n">
+        <v>-147.6962226657143</v>
+      </c>
+      <c r="R157" s="19" t="n">
+        <v>-7977.840953469999</v>
+      </c>
+      <c r="S157" s="19" t="n">
+        <v>-0.4692847619688235</v>
+      </c>
+      <c r="T157" s="19" t="n">
+        <v>-42.21079869560846</v>
+      </c>
+      <c r="U157" s="19" t="n">
+        <v>-8224.5495102</v>
+      </c>
+      <c r="V157" s="19" t="n">
+        <v>-0.4837970300117647</v>
+      </c>
+      <c r="W157" s="19" t="n">
+        <v>-43.51613497460318</v>
+      </c>
+      <c r="X157" s="19" t="n">
+        <v>-9565.196761720001</v>
+      </c>
+      <c r="Y157" s="19" t="n">
+        <v>-0.562658633042353</v>
+      </c>
+      <c r="Z157" s="19" t="n">
+        <v>-50.6095066757672</v>
+      </c>
+      <c r="AA157" s="19" t="n">
+        <v>-15104.73649053</v>
+      </c>
+      <c r="AB157" s="19" t="n">
+        <v>-0.8885139112076471</v>
+      </c>
+      <c r="AC157" s="19" t="n">
+        <v>-79.91924069063492</v>
+      </c>
+      <c r="AD157" s="19" t="n">
+        <v>-304176.1731140899</v>
+      </c>
+      <c r="AE157" s="19" t="n">
+        <v>-17.89271606553471</v>
+      </c>
+      <c r="AF157" s="19" t="n">
+        <v>-1609.397741344392</v>
+      </c>
+      <c r="AG157" s="19" t="n">
+        <v>-1899.751774</v>
+      </c>
+      <c r="AH157" s="19" t="n">
+        <v>-0.1117501043529412</v>
+      </c>
+      <c r="AI157" s="19" t="n">
+        <v>-10.05159668783069</v>
+      </c>
+      <c r="AJ157" s="19" t="n">
+        <v>-306075.9248880899</v>
+      </c>
+      <c r="AK157" s="19" t="n">
+        <v>-18.00446616988765</v>
+      </c>
+      <c r="AL157" s="19" t="n">
+        <v>-1619.449338032222</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="B158" s="18" t="inlineStr">
+        <is>
           <t>NET CASH SURPLUS (LOSS)</t>
         </is>
       </c>
-      <c r="C157" s="19" t="n">
+      <c r="C158" s="19" t="n">
         <v>11812.90216024</v>
       </c>
-      <c r="D157" s="19" t="n">
+      <c r="D158" s="19" t="n">
         <v>0.6948765976611763</v>
       </c>
-      <c r="E157" s="19" t="n">
+      <c r="E158" s="19" t="n">
         <v>62.50212783195766</v>
       </c>
-      <c r="F157" s="19" t="n">
+      <c r="F158" s="19" t="n">
         <v>-75526.95973020002</v>
       </c>
-      <c r="G157" s="19" t="n">
+      <c r="G158" s="19" t="n">
         <v>-4.442762337070589</v>
       </c>
-      <c r="H157" s="19" t="n">
+      <c r="H158" s="19" t="n">
         <v>-399.6135435460318</v>
       </c>
-      <c r="I157" s="19" t="n">
+      <c r="I158" s="19" t="n">
         <v>2573.810161360001</v>
       </c>
-      <c r="J157" s="19" t="n">
+      <c r="J158" s="19" t="n">
         <v>0.1514005977270589</v>
       </c>
-      <c r="K157" s="19" t="n">
+      <c r="K158" s="19" t="n">
         <v>13.61804318179895</v>
       </c>
-      <c r="L157" s="19" t="n">
+      <c r="L158" s="19" t="n">
         <v>11041.90401141</v>
       </c>
-      <c r="M157" s="19" t="n">
+      <c r="M158" s="19" t="n">
         <v>0.6495237653770591</v>
       </c>
-      <c r="N157" s="19" t="n">
+      <c r="N158" s="19" t="n">
         <v>58.42277254714288</v>
       </c>
-      <c r="O157" s="19" t="n">
+      <c r="O158" s="19" t="n">
         <v>-15435.4135908</v>
       </c>
-      <c r="P157" s="19" t="n">
+      <c r="P158" s="19" t="n">
         <v>-0.9079655053411764</v>
       </c>
-      <c r="Q157" s="19" t="n">
+      <c r="Q158" s="19" t="n">
         <v>-81.66885497777777</v>
       </c>
-      <c r="R157" s="19" t="n">
-        <v>-114.3488221300001</v>
-      </c>
-      <c r="S157" s="19" t="n">
-        <v>-0.006726401301764713</v>
-      </c>
-      <c r="T157" s="19" t="n">
-        <v>-0.6050202229100535</v>
-      </c>
-      <c r="U157" s="19" t="n">
+      <c r="R158" s="19" t="n">
+        <v>-114.3488221299992</v>
+      </c>
+      <c r="S158" s="19" t="n">
+        <v>-0.006726401301764657</v>
+      </c>
+      <c r="T158" s="19" t="n">
+        <v>-0.6050202229100485</v>
+      </c>
+      <c r="U158" s="19" t="n">
         <v>1367.97276569</v>
       </c>
-      <c r="V157" s="19" t="n">
+      <c r="V158" s="19" t="n">
         <v>0.08046898621705879</v>
       </c>
-      <c r="W157" s="19" t="n">
+      <c r="W158" s="19" t="n">
         <v>7.237951141216929</v>
       </c>
-      <c r="X157" s="19" t="n">
-        <v>-1729.271263249999</v>
-      </c>
-      <c r="Y157" s="19" t="n">
-        <v>-0.1017218390147058</v>
-      </c>
-      <c r="Z157" s="19" t="n">
-        <v>-9.149583403439149</v>
-      </c>
-      <c r="AA157" s="19" t="n">
+      <c r="X158" s="19" t="n">
+        <v>-1729.271263250001</v>
+      </c>
+      <c r="Y158" s="19" t="n">
+        <v>-0.1017218390147059</v>
+      </c>
+      <c r="Z158" s="19" t="n">
+        <v>-9.149583403439157</v>
+      </c>
+      <c r="AA158" s="19" t="n">
         <v>13615.21769607</v>
       </c>
-      <c r="AB157" s="19" t="n">
+      <c r="AB158" s="19" t="n">
         <v>0.8008951585923528</v>
       </c>
-      <c r="AC157" s="19" t="n">
+      <c r="AC158" s="19" t="n">
         <v>72.03818886809523</v>
       </c>
-      <c r="AD157" s="19" t="n">
-        <v>-52394.18661161001</v>
-      </c>
-      <c r="AE157" s="19" t="n">
-        <v>-3.08201097715353</v>
-      </c>
-      <c r="AF157" s="19" t="n">
-        <v>-277.2179185799472</v>
-      </c>
-      <c r="AG157" s="19" t="n">
-        <v>4461.631374</v>
-      </c>
-      <c r="AH157" s="19" t="n">
-        <v>0.2624489043529412</v>
-      </c>
-      <c r="AI157" s="19" t="n">
-        <v>23.6065152063492</v>
-      </c>
-      <c r="AJ157" s="19" t="n">
-        <v>-47932.55523761002</v>
-      </c>
-      <c r="AK157" s="19" t="n">
-        <v>-2.819562072800589</v>
-      </c>
-      <c r="AL157" s="19" t="n">
-        <v>-253.611403373598</v>
-      </c>
-    </row>
-    <row r="158">
-      <c r="B158" s="6" t="inlineStr">
+      <c r="AD158" s="19" t="n">
+        <v>-52394.18661161</v>
+      </c>
+      <c r="AE158" s="19" t="n">
+        <v>-3.082010977153531</v>
+      </c>
+      <c r="AF158" s="19" t="n">
+        <v>-277.2179185799473</v>
+      </c>
+      <c r="AG158" s="19" t="n">
+        <v>4442.702874</v>
+      </c>
+      <c r="AH158" s="19" t="n">
+        <v>0.2613354631764706</v>
+      </c>
+      <c r="AI158" s="19" t="n">
+        <v>23.50636441269841</v>
+      </c>
+      <c r="AJ158" s="19" t="n">
+        <v>-47951.48373761</v>
+      </c>
+      <c r="AK158" s="19" t="n">
+        <v>-2.820675513977061</v>
+      </c>
+      <c r="AL158" s="19" t="n">
+        <v>-253.7115541672488</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="B159" s="6" t="inlineStr">
         <is>
           <t>ENDING BALANCE</t>
         </is>
       </c>
-      <c r="C158" s="7" t="n">
+      <c r="C159" s="7" t="n">
         <v>79286.56298660001</v>
       </c>
-      <c r="D158" s="7" t="n">
+      <c r="D159" s="7" t="n">
         <v>4.663915469800001</v>
       </c>
-      <c r="E158" s="7" t="n">
+      <c r="E159" s="7" t="n">
         <v>419.5056242677249</v>
       </c>
-      <c r="F158" s="7" t="n">
+      <c r="F159" s="7" t="n">
         <v>3759.603256399994</v>
       </c>
-      <c r="G158" s="7" t="n">
+      <c r="G159" s="7" t="n">
         <v>0.2211531327294114</v>
       </c>
-      <c r="H158" s="7" t="n">
+      <c r="H159" s="7" t="n">
         <v>19.89208072169309</v>
       </c>
-      <c r="I158" s="7" t="n">
+      <c r="I159" s="7" t="n">
         <v>6333.413417759994</v>
       </c>
-      <c r="J158" s="7" t="n">
+      <c r="J159" s="7" t="n">
         <v>0.3725537304564703</v>
       </c>
-      <c r="K158" s="7" t="n">
+      <c r="K159" s="7" t="n">
         <v>33.51012390349204</v>
       </c>
-      <c r="L158" s="7" t="n">
+      <c r="L159" s="7" t="n">
         <v>17375.31742917</v>
       </c>
-      <c r="M158" s="7" t="n">
+      <c r="M159" s="7" t="n">
         <v>1.022077495833529</v>
       </c>
-      <c r="N158" s="7" t="n">
+      <c r="N159" s="7" t="n">
         <v>91.93289645063491</v>
       </c>
-      <c r="O158" s="7" t="n">
+      <c r="O159" s="7" t="n">
         <v>1939.903838369999</v>
       </c>
-      <c r="P158" s="7" t="n">
+      <c r="P159" s="7" t="n">
         <v>0.1141119904923529</v>
       </c>
-      <c r="Q158" s="7" t="n">
+      <c r="Q159" s="7" t="n">
         <v>10.26404147285714</v>
       </c>
-      <c r="R158" s="7" t="n">
-        <v>1825.555016239999</v>
-      </c>
-      <c r="S158" s="7" t="n">
+      <c r="R159" s="7" t="n">
+        <v>1825.55501624</v>
+      </c>
+      <c r="S159" s="7" t="n">
         <v>0.1073855891905882</v>
       </c>
-      <c r="T158" s="7" t="n">
-        <v>9.659021249947084</v>
-      </c>
-      <c r="U158" s="7" t="n">
-        <v>3193.527781929997</v>
-      </c>
-      <c r="V158" s="7" t="n">
-        <v>0.1878545754076469</v>
-      </c>
-      <c r="W158" s="7" t="n">
-        <v>16.89697239116401</v>
-      </c>
-      <c r="X158" s="7" t="n">
+      <c r="T159" s="7" t="n">
+        <v>9.659021249947088</v>
+      </c>
+      <c r="U159" s="7" t="n">
+        <v>3193.527781929999</v>
+      </c>
+      <c r="V159" s="7" t="n">
+        <v>0.187854575407647</v>
+      </c>
+      <c r="W159" s="7" t="n">
+        <v>16.89697239116402</v>
+      </c>
+      <c r="X159" s="7" t="n">
         <v>1464.256518679998</v>
       </c>
-      <c r="Y158" s="7" t="n">
+      <c r="Y159" s="7" t="n">
         <v>0.08613273639294108</v>
       </c>
-      <c r="Z158" s="7" t="n">
+      <c r="Z159" s="7" t="n">
         <v>7.747388987724859</v>
       </c>
-      <c r="AA158" s="7" t="n">
+      <c r="AA159" s="7" t="n">
         <v>15079.47421475</v>
       </c>
-      <c r="AB158" s="7" t="n">
+      <c r="AB159" s="7" t="n">
         <v>0.887027894985294</v>
       </c>
-      <c r="AC158" s="7" t="n">
+      <c r="AC159" s="7" t="n">
         <v>79.78557785582009</v>
       </c>
-      <c r="AD158" s="7" t="n">
+      <c r="AD159" s="7" t="n">
         <v>15079.47421475</v>
       </c>
-      <c r="AE158" s="7" t="n">
+      <c r="AE159" s="7" t="n">
         <v>0.887027894985294</v>
       </c>
-      <c r="AF158" s="7" t="n">
+      <c r="AF159" s="7" t="n">
         <v>79.78557785582009</v>
       </c>
-      <c r="AG158" s="7" t="n">
-        <v>19541.10558875</v>
-      </c>
-      <c r="AH158" s="7" t="n">
-        <v>1.149476799338235</v>
-      </c>
-      <c r="AI158" s="7" t="n">
-        <v>103.3920930621693</v>
-      </c>
-      <c r="AJ158" s="7" t="n">
-        <v>19541.10558875</v>
-      </c>
-      <c r="AK158" s="7" t="n">
-        <v>1.149476799338235</v>
-      </c>
-      <c r="AL158" s="7" t="n">
-        <v>103.3920930621693</v>
+      <c r="AG159" s="7" t="n">
+        <v>19522.17708875</v>
+      </c>
+      <c r="AH159" s="7" t="n">
+        <v>1.148363358161765</v>
+      </c>
+      <c r="AI159" s="7" t="n">
+        <v>103.2919422685185</v>
+      </c>
+      <c r="AJ159" s="7" t="n">
+        <v>19522.17708875</v>
+      </c>
+      <c r="AK159" s="7" t="n">
+        <v>1.148363358161765</v>
+      </c>
+      <c r="AL159" s="7" t="n">
+        <v>103.2919422685185</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Fri 10/09/2026 16:19
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -734,7 +734,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 06 Oct 2026 16:19</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 09 Oct 2026 16:19</t>
         </is>
       </c>
     </row>
@@ -816,14 +816,14 @@
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 06 Oct 2026</t>
+          <t>MTD as of 09 Oct 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
       <c r="AI3" s="4" t="n"/>
       <c r="AJ3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 06 Oct 2026</t>
+          <t>YTD as of 09 Oct 2026</t>
         </is>
       </c>
       <c r="AK3" s="4" t="n"/>
@@ -1267,22 +1267,22 @@
         <v>1066081968.222222</v>
       </c>
       <c r="AG7" s="11" t="n">
-        <v>6339231148</v>
+        <v>6390025148</v>
       </c>
       <c r="AH7" s="11" t="n">
-        <v>372895.949882353</v>
+        <v>375883.8322352941</v>
       </c>
       <c r="AI7" s="11" t="n">
-        <v>33540905.54497354</v>
+        <v>33809656.86772487</v>
       </c>
       <c r="AJ7" s="11" t="n">
-        <v>207828723142</v>
+        <v>207879517142</v>
       </c>
       <c r="AK7" s="11" t="n">
-        <v>12225219.00835294</v>
+        <v>12228206.89070588</v>
       </c>
       <c r="AL7" s="11" t="n">
-        <v>1099622873.767196</v>
+        <v>1099891625.089947</v>
       </c>
     </row>
     <row r="8">
@@ -1958,17 +1958,23 @@
       <c r="AF15" s="11" t="n">
         <v>398833.08994709</v>
       </c>
-      <c r="AG15" s="11" t="n"/>
-      <c r="AH15" s="11" t="n"/>
-      <c r="AI15" s="11" t="n"/>
+      <c r="AG15" s="11" t="n">
+        <v>50794000</v>
+      </c>
+      <c r="AH15" s="11" t="n">
+        <v>2987.882352941177</v>
+      </c>
+      <c r="AI15" s="11" t="n">
+        <v>268751.3227513228</v>
+      </c>
       <c r="AJ15" s="11" t="n">
-        <v>75379454</v>
+        <v>126173454</v>
       </c>
       <c r="AK15" s="11" t="n">
-        <v>4434.085529411765</v>
+        <v>7421.967882352941</v>
       </c>
       <c r="AL15" s="11" t="n">
-        <v>398833.08994709</v>
+        <v>667584.4126984128</v>
       </c>
     </row>
     <row r="16">
@@ -2324,22 +2330,22 @@
         <v>2521134.965502645</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>3223500</v>
+        <v>6304000</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>189.6176470588235</v>
+        <v>370.8235294117647</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>17055.55555555555</v>
+        <v>33354.49735449735</v>
       </c>
       <c r="AJ20" s="13" t="n">
-        <v>479718008.48</v>
+        <v>482798508.48</v>
       </c>
       <c r="AK20" s="13" t="n">
-        <v>28218.70638117647</v>
+        <v>28399.91226352942</v>
       </c>
       <c r="AL20" s="13" t="n">
-        <v>2538190.521058201</v>
+        <v>2554489.462857143</v>
       </c>
     </row>
     <row r="21">
@@ -2597,22 +2603,22 @@
         <v>491976.1904761905</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>3223500</v>
+        <v>5304000</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>189.6176470588235</v>
+        <v>312</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>17055.55555555555</v>
+        <v>28063.49206349206</v>
       </c>
       <c r="AJ23" s="11" t="n">
-        <v>96207000</v>
+        <v>98287500</v>
       </c>
       <c r="AK23" s="11" t="n">
-        <v>5659.235294117647</v>
+        <v>5781.617647058823</v>
       </c>
       <c r="AL23" s="11" t="n">
-        <v>509031.746031746</v>
+        <v>520039.6825396825</v>
       </c>
     </row>
     <row r="24">
@@ -3229,17 +3235,23 @@
       <c r="AF32" s="13" t="n">
         <v>23725.02645502645</v>
       </c>
-      <c r="AG32" s="13" t="n"/>
-      <c r="AH32" s="13" t="n"/>
-      <c r="AI32" s="13" t="n"/>
+      <c r="AG32" s="13" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="AH32" s="13" t="n">
+        <v>58.8235294117647</v>
+      </c>
+      <c r="AI32" s="13" t="n">
+        <v>5291.005291005291</v>
+      </c>
       <c r="AJ32" s="13" t="n">
-        <v>4484030</v>
+        <v>5484030</v>
       </c>
       <c r="AK32" s="13" t="n">
-        <v>263.7664705882353</v>
+        <v>322.59</v>
       </c>
       <c r="AL32" s="13" t="n">
-        <v>23725.02645502645</v>
+        <v>29016.03174603175</v>
       </c>
     </row>
     <row r="33">
@@ -4137,22 +4149,22 @@
         <v>1332179822.764445</v>
       </c>
       <c r="AG45" s="15" t="n">
-        <v>6342454648</v>
+        <v>6396329148</v>
       </c>
       <c r="AH45" s="15" t="n">
-        <v>373085.5675294118</v>
+        <v>376254.6557647059</v>
       </c>
       <c r="AI45" s="15" t="n">
-        <v>33557961.1005291</v>
+        <v>33843011.36507937</v>
       </c>
       <c r="AJ45" s="15" t="n">
-        <v>258124441150.48</v>
+        <v>258178315650.48</v>
       </c>
       <c r="AK45" s="15" t="n">
-        <v>15183790.65591059</v>
+        <v>15186959.74414588</v>
       </c>
       <c r="AL45" s="15" t="n">
-        <v>1365737783.864974</v>
+        <v>1366022834.129524</v>
       </c>
     </row>
     <row r="46">
@@ -4574,17 +4586,23 @@
       <c r="AF51" s="13" t="n">
         <v>-13669998.14285714</v>
       </c>
-      <c r="AG51" s="13" t="n"/>
-      <c r="AH51" s="13" t="n"/>
-      <c r="AI51" s="13" t="n"/>
+      <c r="AG51" s="13" t="n">
+        <v>-64097151</v>
+      </c>
+      <c r="AH51" s="13" t="n">
+        <v>-3770.420647058823</v>
+      </c>
+      <c r="AI51" s="13" t="n">
+        <v>-339138.3650793651</v>
+      </c>
       <c r="AJ51" s="13" t="n">
-        <v>-2583629649</v>
+        <v>-2647726800</v>
       </c>
       <c r="AK51" s="13" t="n">
-        <v>-151978.2146470588</v>
+        <v>-155748.6352941176</v>
       </c>
       <c r="AL51" s="13" t="n">
-        <v>-13669998.14285714</v>
+        <v>-14009136.50793651</v>
       </c>
     </row>
     <row r="52">
@@ -4653,17 +4671,23 @@
       <c r="AF52" s="11" t="n">
         <v>-986146.9047619047</v>
       </c>
-      <c r="AG52" s="11" t="n"/>
-      <c r="AH52" s="11" t="n"/>
-      <c r="AI52" s="11" t="n"/>
+      <c r="AG52" s="11" t="n">
+        <v>-46950780</v>
+      </c>
+      <c r="AH52" s="11" t="n">
+        <v>-2761.810588235294</v>
+      </c>
+      <c r="AI52" s="11" t="n">
+        <v>-248416.8253968254</v>
+      </c>
       <c r="AJ52" s="11" t="n">
-        <v>-186381765</v>
+        <v>-233332545</v>
       </c>
       <c r="AK52" s="11" t="n">
-        <v>-10963.63323529412</v>
+        <v>-13725.44382352941</v>
       </c>
       <c r="AL52" s="11" t="n">
-        <v>-986146.9047619047</v>
+        <v>-1234563.73015873</v>
       </c>
     </row>
     <row r="53">
@@ -4878,17 +4902,23 @@
       <c r="AF55" s="13" t="n">
         <v>-10237629.65079365</v>
       </c>
-      <c r="AG55" s="13" t="n"/>
-      <c r="AH55" s="13" t="n"/>
-      <c r="AI55" s="13" t="n"/>
+      <c r="AG55" s="13" t="n">
+        <v>-492540000</v>
+      </c>
+      <c r="AH55" s="13" t="n">
+        <v>-28972.94117647059</v>
+      </c>
+      <c r="AI55" s="13" t="n">
+        <v>-2606031.746031746</v>
+      </c>
       <c r="AJ55" s="13" t="n">
-        <v>-1934912004</v>
+        <v>-2427452004</v>
       </c>
       <c r="AK55" s="13" t="n">
-        <v>-113818.3531764706</v>
+        <v>-142791.2943529412</v>
       </c>
       <c r="AL55" s="13" t="n">
-        <v>-10237629.65079365</v>
+        <v>-12843661.3968254</v>
       </c>
     </row>
     <row r="56">
@@ -4957,17 +4987,23 @@
       <c r="AF56" s="11" t="n">
         <v>-512265</v>
       </c>
-      <c r="AG56" s="11" t="n"/>
-      <c r="AH56" s="11" t="n"/>
-      <c r="AI56" s="11" t="n"/>
+      <c r="AG56" s="11" t="n">
+        <v>-184850000</v>
+      </c>
+      <c r="AH56" s="11" t="n">
+        <v>-10873.52941176471</v>
+      </c>
+      <c r="AI56" s="11" t="n">
+        <v>-978042.328042328</v>
+      </c>
       <c r="AJ56" s="11" t="n">
-        <v>-96818085</v>
+        <v>-281668085</v>
       </c>
       <c r="AK56" s="11" t="n">
-        <v>-5695.181470588235</v>
+        <v>-16568.71088235294</v>
       </c>
       <c r="AL56" s="11" t="n">
-        <v>-512265</v>
+        <v>-1490307.328042328</v>
       </c>
     </row>
     <row r="57">
@@ -5133,17 +5169,23 @@
       <c r="AF58" s="11" t="n">
         <v>-1436633.349206349</v>
       </c>
-      <c r="AG58" s="11" t="n"/>
-      <c r="AH58" s="11" t="n"/>
-      <c r="AI58" s="11" t="n"/>
+      <c r="AG58" s="11" t="n">
+        <v>-7442175</v>
+      </c>
+      <c r="AH58" s="11" t="n">
+        <v>-437.775</v>
+      </c>
+      <c r="AI58" s="11" t="n">
+        <v>-39376.5873015873</v>
+      </c>
       <c r="AJ58" s="11" t="n">
-        <v>-271523703</v>
+        <v>-278965878</v>
       </c>
       <c r="AK58" s="11" t="n">
-        <v>-15971.98252941176</v>
+        <v>-16409.75752941176</v>
       </c>
       <c r="AL58" s="11" t="n">
-        <v>-1436633.349206349</v>
+        <v>-1476009.936507937</v>
       </c>
     </row>
     <row r="59">
@@ -5198,13 +5240,13 @@
         <v>-441719.5767195767</v>
       </c>
       <c r="R59" s="13" t="n">
-        <v>-9372406</v>
+        <v>-36077406</v>
       </c>
       <c r="S59" s="13" t="n">
-        <v>-551.318</v>
+        <v>-2122.200352941176</v>
       </c>
       <c r="T59" s="13" t="n">
-        <v>-49589.44973544974</v>
+        <v>-190885.746031746</v>
       </c>
       <c r="U59" s="13" t="n">
         <v>-64272988</v>
@@ -5234,25 +5276,31 @@
         <v>-1072042.687830688</v>
       </c>
       <c r="AD59" s="13" t="n">
-        <v>-3207024862.88</v>
+        <v>-3233729862.88</v>
       </c>
       <c r="AE59" s="13" t="n">
-        <v>-188648.5213458824</v>
+        <v>-190219.4036988235</v>
       </c>
       <c r="AF59" s="13" t="n">
-        <v>-16968385.5178836</v>
-      </c>
-      <c r="AG59" s="13" t="n"/>
-      <c r="AH59" s="13" t="n"/>
-      <c r="AI59" s="13" t="n"/>
+        <v>-17109681.81417989</v>
+      </c>
+      <c r="AG59" s="13" t="n">
+        <v>-59229205</v>
+      </c>
+      <c r="AH59" s="13" t="n">
+        <v>-3484.070882352941</v>
+      </c>
+      <c r="AI59" s="13" t="n">
+        <v>-313382.037037037</v>
+      </c>
       <c r="AJ59" s="13" t="n">
-        <v>-3207024862.88</v>
+        <v>-3292959067.88</v>
       </c>
       <c r="AK59" s="13" t="n">
-        <v>-188648.5213458824</v>
+        <v>-193703.4745811765</v>
       </c>
       <c r="AL59" s="13" t="n">
-        <v>-16968385.5178836</v>
+        <v>-17423063.85121693</v>
       </c>
     </row>
     <row r="60">
@@ -5364,17 +5412,23 @@
       <c r="AF61" s="13" t="n">
         <v>-10582.01058201058</v>
       </c>
-      <c r="AG61" s="13" t="n"/>
-      <c r="AH61" s="13" t="n"/>
-      <c r="AI61" s="13" t="n"/>
+      <c r="AG61" s="13" t="n">
+        <v>-36672000</v>
+      </c>
+      <c r="AH61" s="13" t="n">
+        <v>-2157.176470588235</v>
+      </c>
+      <c r="AI61" s="13" t="n">
+        <v>-194031.746031746</v>
+      </c>
       <c r="AJ61" s="13" t="n">
-        <v>-2000000</v>
+        <v>-38672000</v>
       </c>
       <c r="AK61" s="13" t="n">
-        <v>-117.6470588235294</v>
+        <v>-2274.823529411764</v>
       </c>
       <c r="AL61" s="13" t="n">
-        <v>-10582.01058201058</v>
+        <v>-204613.7566137566</v>
       </c>
     </row>
     <row r="62">
@@ -5532,13 +5586,13 @@
         <v>-11758772.45502646</v>
       </c>
       <c r="R63" s="15" t="n">
-        <v>-1116468582</v>
+        <v>-1143173582</v>
       </c>
       <c r="S63" s="15" t="n">
-        <v>-65674.62247058823</v>
+        <v>-67245.50482352941</v>
       </c>
       <c r="T63" s="15" t="n">
-        <v>-5907241.174603174</v>
+        <v>-6048537.470899471</v>
       </c>
       <c r="U63" s="15" t="n">
         <v>-939708047</v>
@@ -5568,25 +5622,31 @@
         <v>-10284039.52380952</v>
       </c>
       <c r="AD63" s="15" t="n">
-        <v>-17929444651.88</v>
+        <v>-17956149651.88</v>
       </c>
       <c r="AE63" s="15" t="n">
-        <v>-1054673.214816471</v>
+        <v>-1056244.097169412</v>
       </c>
       <c r="AF63" s="15" t="n">
-        <v>-94864786.5178836</v>
-      </c>
-      <c r="AG63" s="15" t="n"/>
-      <c r="AH63" s="15" t="n"/>
-      <c r="AI63" s="15" t="n"/>
+        <v>-95006082.8141799</v>
+      </c>
+      <c r="AG63" s="15" t="n">
+        <v>-891781311</v>
+      </c>
+      <c r="AH63" s="15" t="n">
+        <v>-52457.72417647059</v>
+      </c>
+      <c r="AI63" s="15" t="n">
+        <v>-4718419.634920635</v>
+      </c>
       <c r="AJ63" s="15" t="n">
-        <v>-17929444651.88</v>
+        <v>-18847930962.88</v>
       </c>
       <c r="AK63" s="15" t="n">
-        <v>-1054673.214816471</v>
+        <v>-1108701.821345882</v>
       </c>
       <c r="AL63" s="15" t="n">
-        <v>-94864786.5178836</v>
+        <v>-99724502.44910054</v>
       </c>
     </row>
     <row r="64">
@@ -6699,22 +6759,22 @@
         <v>-53015355.81481481</v>
       </c>
       <c r="AG81" s="11" t="n">
-        <v>-890478933</v>
+        <v>-903478933</v>
       </c>
       <c r="AH81" s="11" t="n">
-        <v>-52381.11370588235</v>
+        <v>-53145.8195882353</v>
       </c>
       <c r="AI81" s="11" t="n">
-        <v>-4711528.746031746</v>
+        <v>-4780311.814814814</v>
       </c>
       <c r="AJ81" s="11" t="n">
-        <v>-10910381182</v>
+        <v>-10923381182</v>
       </c>
       <c r="AK81" s="11" t="n">
-        <v>-641787.128352941</v>
+        <v>-642551.834235294</v>
       </c>
       <c r="AL81" s="11" t="n">
-        <v>-57726884.56084655</v>
+        <v>-57795667.62962962</v>
       </c>
     </row>
     <row r="82">
@@ -6814,22 +6874,22 @@
         <v>-58934229.3347619</v>
       </c>
       <c r="AG82" s="13" t="n">
-        <v>-897917960</v>
+        <v>-1752972535</v>
       </c>
       <c r="AH82" s="13" t="n">
-        <v>-52818.70352941177</v>
+        <v>-103116.0314705882</v>
       </c>
       <c r="AI82" s="13" t="n">
-        <v>-4750888.677248677</v>
+        <v>-9274986.957671957</v>
       </c>
       <c r="AJ82" s="13" t="n">
-        <v>-12036487304.27</v>
+        <v>-12891541879.27</v>
       </c>
       <c r="AK82" s="13" t="n">
-        <v>-708028.6649570588</v>
+        <v>-758325.9928982353</v>
       </c>
       <c r="AL82" s="13" t="n">
-        <v>-63685118.01201058</v>
+        <v>-68209216.29243386</v>
       </c>
     </row>
     <row r="83">
@@ -7038,22 +7098,22 @@
         <v>-2427178.873015873</v>
       </c>
       <c r="AG84" s="13" t="n">
-        <v>-800000</v>
+        <v>-6136120</v>
       </c>
       <c r="AH84" s="13" t="n">
-        <v>-47.05882352941177</v>
+        <v>-360.9482352941176</v>
       </c>
       <c r="AI84" s="13" t="n">
-        <v>-4232.804232804233</v>
+        <v>-32466.24338624339</v>
       </c>
       <c r="AJ84" s="13" t="n">
-        <v>-459536807</v>
+        <v>-464872927</v>
       </c>
       <c r="AK84" s="13" t="n">
-        <v>-27031.57688235295</v>
+        <v>-27345.46629411765</v>
       </c>
       <c r="AL84" s="13" t="n">
-        <v>-2431411.677248677</v>
+        <v>-2459645.116402117</v>
       </c>
     </row>
     <row r="85">
@@ -7153,22 +7213,22 @@
         <v>-170473264.0490476</v>
       </c>
       <c r="AG85" s="15" t="n">
-        <v>-1789196893</v>
+        <v>-2662587588</v>
       </c>
       <c r="AH85" s="15" t="n">
-        <v>-105246.8760588235</v>
+        <v>-156622.7992941176</v>
       </c>
       <c r="AI85" s="15" t="n">
-        <v>-9466650.227513228</v>
+        <v>-14087765.01587302</v>
       </c>
       <c r="AJ85" s="15" t="n">
-        <v>-34008643798.27</v>
+        <v>-34882034493.27</v>
       </c>
       <c r="AK85" s="15" t="n">
-        <v>-2000508.458721765</v>
+        <v>-2051884.381957059</v>
       </c>
       <c r="AL85" s="15" t="n">
-        <v>-179939914.2765609</v>
+        <v>-184561029.0649207</v>
       </c>
     </row>
     <row r="86">
@@ -7354,22 +7414,22 @@
         <v>-778818.2539682541</v>
       </c>
       <c r="AG88" s="11" t="n">
-        <v>-294372</v>
+        <v>-874372</v>
       </c>
       <c r="AH88" s="11" t="n">
-        <v>-17.316</v>
+        <v>-51.43364705882353</v>
       </c>
       <c r="AI88" s="11" t="n">
-        <v>-1557.52380952381</v>
+        <v>-4626.306878306878</v>
       </c>
       <c r="AJ88" s="11" t="n">
-        <v>-147491022</v>
+        <v>-148071022</v>
       </c>
       <c r="AK88" s="11" t="n">
-        <v>-8675.942470588237</v>
+        <v>-8710.060117647061</v>
       </c>
       <c r="AL88" s="11" t="n">
-        <v>-780375.7777777779</v>
+        <v>-783444.560846561</v>
       </c>
     </row>
     <row r="89">
@@ -7700,22 +7760,22 @@
         <v>-786410.9841269841</v>
       </c>
       <c r="AG92" s="11" t="n">
-        <v>-1078200</v>
+        <v>-1093200</v>
       </c>
       <c r="AH92" s="11" t="n">
-        <v>-63.4235294117647</v>
+        <v>-64.30588235294118</v>
       </c>
       <c r="AI92" s="11" t="n">
-        <v>-5704.761904761905</v>
+        <v>-5784.126984126984</v>
       </c>
       <c r="AJ92" s="11" t="n">
-        <v>-149709876</v>
+        <v>-149724876</v>
       </c>
       <c r="AK92" s="11" t="n">
-        <v>-8806.463294117646</v>
+        <v>-8807.345647058823</v>
       </c>
       <c r="AL92" s="11" t="n">
-        <v>-792115.746031746</v>
+        <v>-792195.1111111111</v>
       </c>
     </row>
     <row r="93">
@@ -7802,17 +7862,23 @@
       <c r="AF93" s="13" t="n">
         <v>-12778.81481481481</v>
       </c>
-      <c r="AG93" s="13" t="n"/>
-      <c r="AH93" s="13" t="n"/>
-      <c r="AI93" s="13" t="n"/>
+      <c r="AG93" s="13" t="n">
+        <v>-233600</v>
+      </c>
+      <c r="AH93" s="13" t="n">
+        <v>-13.74117647058823</v>
+      </c>
+      <c r="AI93" s="13" t="n">
+        <v>-1235.978835978836</v>
+      </c>
       <c r="AJ93" s="13" t="n">
-        <v>-2415196</v>
+        <v>-2648796</v>
       </c>
       <c r="AK93" s="13" t="n">
-        <v>-142.0703529411765</v>
+        <v>-155.8115294117647</v>
       </c>
       <c r="AL93" s="13" t="n">
-        <v>-12778.81481481481</v>
+        <v>-14014.79365079365</v>
       </c>
     </row>
     <row r="94">
@@ -7912,22 +7978,22 @@
         <v>-2636230.425608465</v>
       </c>
       <c r="AG94" s="15" t="n">
-        <v>-2145072</v>
+        <v>-2973672</v>
       </c>
       <c r="AH94" s="15" t="n">
-        <v>-126.1807058823529</v>
+        <v>-174.9218823529412</v>
       </c>
       <c r="AI94" s="15" t="n">
-        <v>-11349.5873015873</v>
+        <v>-15733.71428571429</v>
       </c>
       <c r="AJ94" s="15" t="n">
-        <v>-500392622.44</v>
+        <v>-501221222.44</v>
       </c>
       <c r="AK94" s="15" t="n">
-        <v>-29434.86014352941</v>
+        <v>-29483.60132</v>
       </c>
       <c r="AL94" s="15" t="n">
-        <v>-2647580.012910053</v>
+        <v>-2651964.13989418</v>
       </c>
     </row>
     <row r="95">
@@ -8222,22 +8288,22 @@
         <v>-1418156.079365079</v>
       </c>
       <c r="AG98" s="11" t="n">
-        <v>-1248500</v>
+        <v>-12640200</v>
       </c>
       <c r="AH98" s="11" t="n">
-        <v>-73.44117647058823</v>
+        <v>-743.5411764705882</v>
       </c>
       <c r="AI98" s="11" t="n">
-        <v>-6605.820105820106</v>
+        <v>-66879.36507936507</v>
       </c>
       <c r="AJ98" s="11" t="n">
-        <v>-269279999</v>
+        <v>-280671699</v>
       </c>
       <c r="AK98" s="11" t="n">
-        <v>-15839.99994117647</v>
+        <v>-16510.09994117647</v>
       </c>
       <c r="AL98" s="11" t="n">
-        <v>-1424761.899470899</v>
+        <v>-1485035.444444444</v>
       </c>
     </row>
     <row r="99">
@@ -8337,22 +8403,22 @@
         <v>-40893236.55941799</v>
       </c>
       <c r="AG99" s="13" t="n">
-        <v>-82401009</v>
+        <v>-151615974</v>
       </c>
       <c r="AH99" s="13" t="n">
-        <v>-4847.118176470588</v>
+        <v>-8918.586705882353</v>
       </c>
       <c r="AI99" s="13" t="n">
-        <v>-435984.1746031746</v>
+        <v>-802200.9206349206</v>
       </c>
       <c r="AJ99" s="13" t="n">
-        <v>-7811222718.73</v>
+        <v>-7880437683.73</v>
       </c>
       <c r="AK99" s="13" t="n">
-        <v>-459483.6893370589</v>
+        <v>-463555.1578664706</v>
       </c>
       <c r="AL99" s="13" t="n">
-        <v>-41329220.73402116</v>
+        <v>-41695437.48005291</v>
       </c>
     </row>
     <row r="100">
@@ -8451,17 +8517,23 @@
       <c r="AF100" s="11" t="n">
         <v>-1318975.026455026</v>
       </c>
-      <c r="AG100" s="11" t="n"/>
-      <c r="AH100" s="11" t="n"/>
-      <c r="AI100" s="11" t="n"/>
+      <c r="AG100" s="11" t="n">
+        <v>-7999429</v>
+      </c>
+      <c r="AH100" s="11" t="n">
+        <v>-470.5546470588235</v>
+      </c>
+      <c r="AI100" s="11" t="n">
+        <v>-42325.02116402116</v>
+      </c>
       <c r="AJ100" s="11" t="n">
-        <v>-249286280</v>
+        <v>-257285709</v>
       </c>
       <c r="AK100" s="11" t="n">
-        <v>-14663.89882352941</v>
+        <v>-15134.45347058824</v>
       </c>
       <c r="AL100" s="11" t="n">
-        <v>-1318975.026455026</v>
+        <v>-1361300.047619048</v>
       </c>
     </row>
     <row r="101">
@@ -8543,40 +8615,40 @@
         <v>-211897.4867724868</v>
       </c>
       <c r="AA101" s="13" t="n">
-        <v>-31040200</v>
+        <v>-31241950</v>
       </c>
       <c r="AB101" s="13" t="n">
-        <v>-1825.894117647059</v>
+        <v>-1837.761764705882</v>
       </c>
       <c r="AC101" s="13" t="n">
-        <v>-164233.8624338624</v>
+        <v>-165301.3227513228</v>
       </c>
       <c r="AD101" s="13" t="n">
-        <v>-364222107</v>
+        <v>-364423857</v>
       </c>
       <c r="AE101" s="13" t="n">
-        <v>-21424.82982352941</v>
+        <v>-21436.69747058823</v>
       </c>
       <c r="AF101" s="13" t="n">
-        <v>-1927101.095238095</v>
+        <v>-1928168.555555556</v>
       </c>
       <c r="AG101" s="13" t="n">
-        <v>-1109400</v>
+        <v>-4332150</v>
       </c>
       <c r="AH101" s="13" t="n">
-        <v>-65.25882352941177</v>
+        <v>-254.8323529411765</v>
       </c>
       <c r="AI101" s="13" t="n">
-        <v>-5869.841269841269</v>
+        <v>-22921.42857142857</v>
       </c>
       <c r="AJ101" s="13" t="n">
-        <v>-365331507</v>
+        <v>-368756007</v>
       </c>
       <c r="AK101" s="13" t="n">
-        <v>-21490.08864705882</v>
+        <v>-21691.52982352941</v>
       </c>
       <c r="AL101" s="13" t="n">
-        <v>-1932970.936507936</v>
+        <v>-1951089.984126984</v>
       </c>
     </row>
     <row r="102">
@@ -8658,40 +8730,40 @@
         <v>-3812258.455026455</v>
       </c>
       <c r="AA102" s="15" t="n">
-        <v>-886276126.27</v>
+        <v>-886477876.27</v>
       </c>
       <c r="AB102" s="15" t="n">
-        <v>-52133.88978058824</v>
+        <v>-52145.75742764706</v>
       </c>
       <c r="AC102" s="15" t="n">
-        <v>-4689291.673386243</v>
+        <v>-4690359.133703704</v>
       </c>
       <c r="AD102" s="15" t="n">
-        <v>-8732265895.73</v>
+        <v>-8732467645.73</v>
       </c>
       <c r="AE102" s="15" t="n">
-        <v>-513662.6997488235</v>
+        <v>-513674.5673958823</v>
       </c>
       <c r="AF102" s="15" t="n">
-        <v>-46202465.05677249</v>
+        <v>-46203532.51708995</v>
       </c>
       <c r="AG102" s="15" t="n">
-        <v>-85290450</v>
+        <v>-177119294</v>
       </c>
       <c r="AH102" s="15" t="n">
-        <v>-5017.085294117647</v>
+        <v>-10418.782</v>
       </c>
       <c r="AI102" s="15" t="n">
-        <v>-451272.2222222222</v>
+        <v>-937139.1216931217</v>
       </c>
       <c r="AJ102" s="15" t="n">
-        <v>-8817556345.73</v>
+        <v>-8909586939.73</v>
       </c>
       <c r="AK102" s="15" t="n">
-        <v>-518679.7850429411</v>
+        <v>-524093.3493958823</v>
       </c>
       <c r="AL102" s="15" t="n">
-        <v>-46653737.27899472</v>
+        <v>-47140671.63878307</v>
       </c>
     </row>
     <row r="103">
@@ -8834,22 +8906,22 @@
         <v>-1237435.248677249</v>
       </c>
       <c r="AG104" s="11" t="n">
-        <v>-544500</v>
+        <v>-17094600</v>
       </c>
       <c r="AH104" s="11" t="n">
-        <v>-32.02941176470588</v>
+        <v>-1005.564705882353</v>
       </c>
       <c r="AI104" s="11" t="n">
-        <v>-2880.952380952381</v>
+        <v>-90447.61904761905</v>
       </c>
       <c r="AJ104" s="11" t="n">
-        <v>-234419762</v>
+        <v>-250969862</v>
       </c>
       <c r="AK104" s="11" t="n">
-        <v>-13789.39776470588</v>
+        <v>-14762.93305882353</v>
       </c>
       <c r="AL104" s="11" t="n">
-        <v>-1240316.201058201</v>
+        <v>-1327882.867724868</v>
       </c>
     </row>
     <row r="105">
@@ -8949,22 +9021,22 @@
         <v>-1864747.592592593</v>
       </c>
       <c r="AG105" s="13" t="n">
-        <v>-587000</v>
+        <v>-161522493</v>
       </c>
       <c r="AH105" s="13" t="n">
-        <v>-34.52941176470588</v>
+        <v>-9501.323117647058</v>
       </c>
       <c r="AI105" s="13" t="n">
-        <v>-3105.820105820106</v>
+        <v>-854616.3650793651</v>
       </c>
       <c r="AJ105" s="13" t="n">
-        <v>-353024295</v>
+        <v>-513959788</v>
       </c>
       <c r="AK105" s="13" t="n">
-        <v>-20766.135</v>
+        <v>-30232.92870588235</v>
       </c>
       <c r="AL105" s="13" t="n">
-        <v>-1867853.412698413</v>
+        <v>-2719363.957671958</v>
       </c>
     </row>
     <row r="106">
@@ -9063,17 +9135,23 @@
       <c r="AF106" s="11" t="n">
         <v>-8926693.243386243</v>
       </c>
-      <c r="AG106" s="11" t="n"/>
-      <c r="AH106" s="11" t="n"/>
-      <c r="AI106" s="11" t="n"/>
+      <c r="AG106" s="11" t="n">
+        <v>-70776068</v>
+      </c>
+      <c r="AH106" s="11" t="n">
+        <v>-4163.298117647058</v>
+      </c>
+      <c r="AI106" s="11" t="n">
+        <v>-374476.5502645503</v>
+      </c>
       <c r="AJ106" s="11" t="n">
-        <v>-1687145023</v>
+        <v>-1757921091</v>
       </c>
       <c r="AK106" s="11" t="n">
-        <v>-99243.82488235294</v>
+        <v>-103407.123</v>
       </c>
       <c r="AL106" s="11" t="n">
-        <v>-8926693.243386243</v>
+        <v>-9301169.793650793</v>
       </c>
     </row>
     <row r="107">
@@ -9166,17 +9244,23 @@
       <c r="AF107" s="13" t="n">
         <v>-1059205.370370371</v>
       </c>
-      <c r="AG107" s="13" t="n"/>
-      <c r="AH107" s="13" t="n"/>
-      <c r="AI107" s="13" t="n"/>
+      <c r="AG107" s="13" t="n">
+        <v>-34937225</v>
+      </c>
+      <c r="AH107" s="13" t="n">
+        <v>-2055.130882352941</v>
+      </c>
+      <c r="AI107" s="13" t="n">
+        <v>-184853.0423280423</v>
+      </c>
       <c r="AJ107" s="13" t="n">
-        <v>-200189815</v>
+        <v>-235127040</v>
       </c>
       <c r="AK107" s="13" t="n">
-        <v>-11775.87147058824</v>
+        <v>-13831.00235294118</v>
       </c>
       <c r="AL107" s="13" t="n">
-        <v>-1059205.370370371</v>
+        <v>-1244058.412698413</v>
       </c>
     </row>
     <row r="108">
@@ -9276,22 +9360,22 @@
         <v>-13088081.45502646</v>
       </c>
       <c r="AG108" s="15" t="n">
-        <v>-1131500</v>
+        <v>-284330386</v>
       </c>
       <c r="AH108" s="15" t="n">
-        <v>-66.55882352941177</v>
+        <v>-16725.31682352941</v>
       </c>
       <c r="AI108" s="15" t="n">
-        <v>-5986.772486772486</v>
+        <v>-1504393.576719577</v>
       </c>
       <c r="AJ108" s="15" t="n">
-        <v>-2474778895</v>
+        <v>-2757977781</v>
       </c>
       <c r="AK108" s="15" t="n">
-        <v>-145575.229117647</v>
+        <v>-162233.987117647</v>
       </c>
       <c r="AL108" s="15" t="n">
-        <v>-13094068.22751323</v>
+        <v>-14592475.03174603</v>
       </c>
     </row>
     <row r="109">
@@ -9565,13 +9649,13 @@
         <v>-120145.5026455027</v>
       </c>
       <c r="R112" s="11" t="n">
-        <v>-81190650</v>
+        <v>-54485650</v>
       </c>
       <c r="S112" s="11" t="n">
-        <v>-4775.920588235294</v>
+        <v>-3205.038235294118</v>
       </c>
       <c r="T112" s="11" t="n">
-        <v>-429580.1587301588</v>
+        <v>-288283.8624338624</v>
       </c>
       <c r="U112" s="11" t="n">
         <v>-147792961</v>
@@ -9601,31 +9685,31 @@
         <v>-147580.9523809524</v>
       </c>
       <c r="AD112" s="11" t="n">
-        <v>-496868911</v>
+        <v>-470163911</v>
       </c>
       <c r="AE112" s="11" t="n">
-        <v>-29227.583</v>
+        <v>-27656.70064705882</v>
       </c>
       <c r="AF112" s="11" t="n">
-        <v>-2628936.037037037</v>
+        <v>-2487639.740740741</v>
       </c>
       <c r="AG112" s="11" t="n">
-        <v>-16087500</v>
+        <v>-21587500</v>
       </c>
       <c r="AH112" s="11" t="n">
-        <v>-946.3235294117648</v>
+        <v>-1269.85294117647</v>
       </c>
       <c r="AI112" s="11" t="n">
-        <v>-85119.04761904762</v>
+        <v>-114219.5767195767</v>
       </c>
       <c r="AJ112" s="11" t="n">
-        <v>-512956411</v>
+        <v>-491751411</v>
       </c>
       <c r="AK112" s="11" t="n">
-        <v>-30173.90652941176</v>
+        <v>-28926.5535882353</v>
       </c>
       <c r="AL112" s="11" t="n">
-        <v>-2714055.084656085</v>
+        <v>-2601859.317460317</v>
       </c>
     </row>
     <row r="113">
@@ -9680,13 +9764,13 @@
         <v>-194378.3068783069</v>
       </c>
       <c r="R113" s="15" t="n">
-        <v>-144562250</v>
+        <v>-117857250</v>
       </c>
       <c r="S113" s="15" t="n">
-        <v>-8503.661764705883</v>
+        <v>-6932.779411764706</v>
       </c>
       <c r="T113" s="15" t="n">
-        <v>-764879.6296296297</v>
+        <v>-623583.3333333334</v>
       </c>
       <c r="U113" s="15" t="n">
         <v>-157760461</v>
@@ -9716,31 +9800,31 @@
         <v>-171483.0687830688</v>
       </c>
       <c r="AD113" s="15" t="n">
-        <v>-650876511</v>
+        <v>-624171511</v>
       </c>
       <c r="AE113" s="15" t="n">
-        <v>-38286.8535882353</v>
+        <v>-36715.97123529412</v>
       </c>
       <c r="AF113" s="15" t="n">
-        <v>-3443791.063492063</v>
+        <v>-3302494.767195768</v>
       </c>
       <c r="AG113" s="15" t="n">
-        <v>-16087500</v>
+        <v>-21587500</v>
       </c>
       <c r="AH113" s="15" t="n">
-        <v>-946.3235294117648</v>
+        <v>-1269.85294117647</v>
       </c>
       <c r="AI113" s="15" t="n">
-        <v>-85119.04761904762</v>
+        <v>-114219.5767195767</v>
       </c>
       <c r="AJ113" s="15" t="n">
-        <v>-666964011</v>
+        <v>-645759011</v>
       </c>
       <c r="AK113" s="15" t="n">
-        <v>-39233.17711764706</v>
+        <v>-37985.82417647059</v>
       </c>
       <c r="AL113" s="15" t="n">
-        <v>-3528910.111111111</v>
+        <v>-3416714.343915344</v>
       </c>
     </row>
     <row r="114">
@@ -9876,17 +9960,23 @@
       <c r="AF115" s="11" t="n">
         <v>-2418823.142857143</v>
       </c>
-      <c r="AG115" s="11" t="n"/>
-      <c r="AH115" s="11" t="n"/>
-      <c r="AI115" s="11" t="n"/>
+      <c r="AG115" s="11" t="n">
+        <v>-37104000</v>
+      </c>
+      <c r="AH115" s="11" t="n">
+        <v>-2182.588235294118</v>
+      </c>
+      <c r="AI115" s="11" t="n">
+        <v>-196317.4603174603</v>
+      </c>
       <c r="AJ115" s="11" t="n">
-        <v>-457157574</v>
+        <v>-494261574</v>
       </c>
       <c r="AK115" s="11" t="n">
-        <v>-26891.622</v>
+        <v>-29074.21023529412</v>
       </c>
       <c r="AL115" s="11" t="n">
-        <v>-2418823.142857143</v>
+        <v>-2615140.603174603</v>
       </c>
     </row>
     <row r="116">
@@ -10046,17 +10136,23 @@
       <c r="AF117" s="11" t="n">
         <v>-715199.5291005292</v>
       </c>
-      <c r="AG117" s="11" t="n"/>
-      <c r="AH117" s="11" t="n"/>
-      <c r="AI117" s="11" t="n"/>
+      <c r="AG117" s="11" t="n">
+        <v>-12740000</v>
+      </c>
+      <c r="AH117" s="11" t="n">
+        <v>-749.4117647058823</v>
+      </c>
+      <c r="AI117" s="11" t="n">
+        <v>-67407.4074074074</v>
+      </c>
       <c r="AJ117" s="11" t="n">
-        <v>-135172711</v>
+        <v>-147912711</v>
       </c>
       <c r="AK117" s="11" t="n">
-        <v>-7951.335941176471</v>
+        <v>-8700.747705882353</v>
       </c>
       <c r="AL117" s="11" t="n">
-        <v>-715199.5291005292</v>
+        <v>-782606.9365079366</v>
       </c>
     </row>
     <row r="118">
@@ -10155,17 +10251,23 @@
       <c r="AF118" s="13" t="n">
         <v>-2977326.375661375</v>
       </c>
-      <c r="AG118" s="13" t="n"/>
-      <c r="AH118" s="13" t="n"/>
-      <c r="AI118" s="13" t="n"/>
+      <c r="AG118" s="13" t="n">
+        <v>-14652000</v>
+      </c>
+      <c r="AH118" s="13" t="n">
+        <v>-861.8823529411765</v>
+      </c>
+      <c r="AI118" s="13" t="n">
+        <v>-77523.80952380953</v>
+      </c>
       <c r="AJ118" s="13" t="n">
-        <v>-562714685</v>
+        <v>-577366685</v>
       </c>
       <c r="AK118" s="13" t="n">
-        <v>-33100.86382352941</v>
+        <v>-33962.74617647059</v>
       </c>
       <c r="AL118" s="13" t="n">
-        <v>-2977326.375661375</v>
+        <v>-3054850.185185185</v>
       </c>
     </row>
     <row r="119">
@@ -10264,17 +10366,23 @@
       <c r="AF119" s="15" t="n">
         <v>-6180132.116402117</v>
       </c>
-      <c r="AG119" s="15" t="n"/>
-      <c r="AH119" s="15" t="n"/>
-      <c r="AI119" s="15" t="n"/>
+      <c r="AG119" s="15" t="n">
+        <v>-64496000</v>
+      </c>
+      <c r="AH119" s="15" t="n">
+        <v>-3793.882352941177</v>
+      </c>
+      <c r="AI119" s="15" t="n">
+        <v>-341248.6772486772</v>
+      </c>
       <c r="AJ119" s="15" t="n">
-        <v>-1168044970</v>
+        <v>-1232540970</v>
       </c>
       <c r="AK119" s="15" t="n">
-        <v>-68708.52764705883</v>
+        <v>-72502.41</v>
       </c>
       <c r="AL119" s="15" t="n">
-        <v>-6180132.116402117</v>
+        <v>-6521380.793650794</v>
       </c>
     </row>
     <row r="120">
@@ -10433,13 +10541,13 @@
         <v>-1429808.666666667</v>
       </c>
       <c r="R122" s="13" t="n">
-        <v>-1626344861</v>
+        <v>-1601969861</v>
       </c>
       <c r="S122" s="13" t="n">
-        <v>-95667.34476470588</v>
+        <v>-94233.52123529412</v>
       </c>
       <c r="T122" s="13" t="n">
-        <v>-8604999.264550265</v>
+        <v>-8476031.010582011</v>
       </c>
       <c r="U122" s="13" t="n">
         <v>-678093650</v>
@@ -10460,40 +10568,40 @@
         <v>-5643998.698412699</v>
       </c>
       <c r="AA122" s="13" t="n">
-        <v>-942531373</v>
+        <v>-942329623</v>
       </c>
       <c r="AB122" s="13" t="n">
-        <v>-55443.02194117647</v>
+        <v>-55431.15429411764</v>
       </c>
       <c r="AC122" s="13" t="n">
-        <v>-4986938.481481481</v>
+        <v>-4985871.021164021</v>
       </c>
       <c r="AD122" s="13" t="n">
-        <v>-6567966354</v>
+        <v>-6543389604</v>
       </c>
       <c r="AE122" s="13" t="n">
-        <v>-386350.9619999999</v>
+        <v>-384905.2708235295</v>
       </c>
       <c r="AF122" s="13" t="n">
-        <v>-34751144.73015873</v>
+        <v>-34621109.01587301</v>
       </c>
       <c r="AG122" s="13" t="n">
-        <v>-3836159</v>
+        <v>-212354423</v>
       </c>
       <c r="AH122" s="13" t="n">
-        <v>-225.6564117647059</v>
+        <v>-12491.43664705882</v>
       </c>
       <c r="AI122" s="13" t="n">
-        <v>-20297.13756613757</v>
+        <v>-1123568.375661376</v>
       </c>
       <c r="AJ122" s="13" t="n">
-        <v>-6571802513</v>
+        <v>-6755744027</v>
       </c>
       <c r="AK122" s="13" t="n">
-        <v>-386576.6184117646</v>
+        <v>-397396.7074705883</v>
       </c>
       <c r="AL122" s="13" t="n">
-        <v>-34771441.86772487</v>
+        <v>-35744677.39153439</v>
       </c>
     </row>
     <row r="123">
@@ -10548,13 +10656,13 @@
         <v>-1429808.666666667</v>
       </c>
       <c r="R123" s="15" t="n">
-        <v>-1626344861</v>
+        <v>-1601969861</v>
       </c>
       <c r="S123" s="15" t="n">
-        <v>-95667.34476470588</v>
+        <v>-94233.52123529412</v>
       </c>
       <c r="T123" s="15" t="n">
-        <v>-8604999.264550265</v>
+        <v>-8476031.010582011</v>
       </c>
       <c r="U123" s="15" t="n">
         <v>-678093650</v>
@@ -10575,40 +10683,40 @@
         <v>-5643998.698412699</v>
       </c>
       <c r="AA123" s="15" t="n">
-        <v>-1063510186</v>
+        <v>-1063308436</v>
       </c>
       <c r="AB123" s="15" t="n">
-        <v>-62559.42270588235</v>
+        <v>-62547.55505882353</v>
       </c>
       <c r="AC123" s="15" t="n">
-        <v>-5627038.021164021</v>
+        <v>-5625970.560846561</v>
       </c>
       <c r="AD123" s="15" t="n">
-        <v>-6688945167</v>
+        <v>-6664368417</v>
       </c>
       <c r="AE123" s="15" t="n">
-        <v>-393467.3627647058</v>
+        <v>-392021.6715882354</v>
       </c>
       <c r="AF123" s="15" t="n">
-        <v>-35391244.26984127</v>
+        <v>-35261208.55555556</v>
       </c>
       <c r="AG123" s="15" t="n">
-        <v>-3836159</v>
+        <v>-212354423</v>
       </c>
       <c r="AH123" s="15" t="n">
-        <v>-225.6564117647059</v>
+        <v>-12491.43664705882</v>
       </c>
       <c r="AI123" s="15" t="n">
-        <v>-20297.13756613757</v>
+        <v>-1123568.375661376</v>
       </c>
       <c r="AJ123" s="15" t="n">
-        <v>-6692781326</v>
+        <v>-6876722840</v>
       </c>
       <c r="AK123" s="15" t="n">
-        <v>-393693.0191764705</v>
+        <v>-404513.1082352942</v>
       </c>
       <c r="AL123" s="15" t="n">
-        <v>-35411541.4074074</v>
+        <v>-36384776.93121693</v>
       </c>
     </row>
     <row r="124">
@@ -11052,13 +11160,13 @@
         <v>-558177.2486772487</v>
       </c>
       <c r="R129" s="11" t="n">
-        <v>-4900000</v>
+        <v>-29275000</v>
       </c>
       <c r="S129" s="11" t="n">
-        <v>-288.2352941176471</v>
+        <v>-1722.058823529412</v>
       </c>
       <c r="T129" s="11" t="n">
-        <v>-25925.92592592593</v>
+        <v>-154894.1798941799</v>
       </c>
       <c r="U129" s="11" t="n">
         <v>-119829000</v>
@@ -11088,25 +11196,25 @@
         <v>-142857.1428571429</v>
       </c>
       <c r="AD129" s="11" t="n">
-        <v>-355114000</v>
+        <v>-379489000</v>
       </c>
       <c r="AE129" s="11" t="n">
-        <v>-20889.05882352941</v>
+        <v>-22322.88235294118</v>
       </c>
       <c r="AF129" s="11" t="n">
-        <v>-1878910.052910053</v>
+        <v>-2007878.306878307</v>
       </c>
       <c r="AG129" s="11" t="n"/>
       <c r="AH129" s="11" t="n"/>
       <c r="AI129" s="11" t="n"/>
       <c r="AJ129" s="11" t="n">
-        <v>-355114000</v>
+        <v>-379489000</v>
       </c>
       <c r="AK129" s="11" t="n">
-        <v>-20889.05882352941</v>
+        <v>-22322.88235294118</v>
       </c>
       <c r="AL129" s="11" t="n">
-        <v>-1878910.052910053</v>
+        <v>-2007878.306878307</v>
       </c>
     </row>
     <row r="130">
@@ -11379,13 +11487,13 @@
         <v>-6977825.682539683</v>
       </c>
       <c r="R132" s="15" t="n">
-        <v>-416051151</v>
+        <v>-440426151</v>
       </c>
       <c r="S132" s="15" t="n">
-        <v>-24473.59711764706</v>
+        <v>-25907.42064705883</v>
       </c>
       <c r="T132" s="15" t="n">
-        <v>-2201328.841269841</v>
+        <v>-2330297.095238095</v>
       </c>
       <c r="U132" s="15" t="n">
         <v>-1928971411</v>
@@ -11415,25 +11523,25 @@
         <v>-8804195.952380951</v>
       </c>
       <c r="AD132" s="15" t="n">
-        <v>-26718589251</v>
+        <v>-26742964251</v>
       </c>
       <c r="AE132" s="15" t="n">
-        <v>-1571681.720647059</v>
+        <v>-1573115.54417647</v>
       </c>
       <c r="AF132" s="15" t="n">
-        <v>-141368197.0952381</v>
+        <v>-141497165.3492064</v>
       </c>
       <c r="AG132" s="15" t="n"/>
       <c r="AH132" s="15" t="n"/>
       <c r="AI132" s="15" t="n"/>
       <c r="AJ132" s="15" t="n">
-        <v>-26718589251</v>
+        <v>-26742964251</v>
       </c>
       <c r="AK132" s="15" t="n">
-        <v>-1571681.720647059</v>
+        <v>-1573115.54417647</v>
       </c>
       <c r="AL132" s="15" t="n">
-        <v>-141368197.0952381</v>
+        <v>-141497165.3492064</v>
       </c>
     </row>
     <row r="133">
@@ -11564,22 +11672,22 @@
         <v>-197258.3068783069</v>
       </c>
       <c r="AG134" s="11" t="n">
-        <v>-91000</v>
+        <v>-2404000</v>
       </c>
       <c r="AH134" s="11" t="n">
-        <v>-5.352941176470588</v>
+        <v>-141.4117647058823</v>
       </c>
       <c r="AI134" s="11" t="n">
-        <v>-481.4814814814815</v>
+        <v>-12719.57671957672</v>
       </c>
       <c r="AJ134" s="11" t="n">
-        <v>-37372820</v>
+        <v>-39685820</v>
       </c>
       <c r="AK134" s="11" t="n">
-        <v>-2198.401176470588</v>
+        <v>-2334.46</v>
       </c>
       <c r="AL134" s="11" t="n">
-        <v>-197739.7883597884</v>
+        <v>-209977.8835978836</v>
       </c>
     </row>
     <row r="135">
@@ -11666,17 +11774,23 @@
       <c r="AF135" s="13" t="n">
         <v>-2537128</v>
       </c>
-      <c r="AG135" s="13" t="n"/>
-      <c r="AH135" s="13" t="n"/>
-      <c r="AI135" s="13" t="n"/>
+      <c r="AG135" s="13" t="n">
+        <v>-59530720</v>
+      </c>
+      <c r="AH135" s="13" t="n">
+        <v>-3501.80705882353</v>
+      </c>
+      <c r="AI135" s="13" t="n">
+        <v>-314977.3544973545</v>
+      </c>
       <c r="AJ135" s="13" t="n">
-        <v>-479517192</v>
+        <v>-539047912</v>
       </c>
       <c r="AK135" s="13" t="n">
-        <v>-28206.89364705882</v>
+        <v>-31708.70070588235</v>
       </c>
       <c r="AL135" s="13" t="n">
-        <v>-2537128</v>
+        <v>-2852105.354497354</v>
       </c>
     </row>
     <row r="136">
@@ -11867,22 +11981,22 @@
         <v>-620735.5185185184</v>
       </c>
       <c r="AG137" s="13" t="n">
-        <v>-1866000</v>
+        <v>-4216900</v>
       </c>
       <c r="AH137" s="13" t="n">
-        <v>-109.7647058823529</v>
+        <v>-248.0529411764706</v>
       </c>
       <c r="AI137" s="13" t="n">
-        <v>-9873.015873015873</v>
+        <v>-22311.64021164021</v>
       </c>
       <c r="AJ137" s="13" t="n">
-        <v>-119185013</v>
+        <v>-121535913</v>
       </c>
       <c r="AK137" s="13" t="n">
-        <v>-7010.883117647058</v>
+        <v>-7149.171352941176</v>
       </c>
       <c r="AL137" s="13" t="n">
-        <v>-630608.5343915343</v>
+        <v>-643047.1587301586</v>
       </c>
     </row>
     <row r="138">
@@ -11975,17 +12089,23 @@
       <c r="AF138" s="11" t="n">
         <v>-1110766.867724868</v>
       </c>
-      <c r="AG138" s="11" t="n"/>
-      <c r="AH138" s="11" t="n"/>
-      <c r="AI138" s="11" t="n"/>
+      <c r="AG138" s="11" t="n">
+        <v>-2713124</v>
+      </c>
+      <c r="AH138" s="11" t="n">
+        <v>-159.5955294117647</v>
+      </c>
+      <c r="AI138" s="11" t="n">
+        <v>-14355.15343915344</v>
+      </c>
       <c r="AJ138" s="11" t="n">
-        <v>-209934938</v>
+        <v>-212648062</v>
       </c>
       <c r="AK138" s="11" t="n">
-        <v>-12349.114</v>
+        <v>-12508.70952941176</v>
       </c>
       <c r="AL138" s="11" t="n">
-        <v>-1110766.867724868</v>
+        <v>-1125122.021164021</v>
       </c>
     </row>
     <row r="139">
@@ -12049,22 +12169,22 @@
         <v>-9978.835978835979</v>
       </c>
       <c r="AG139" s="13" t="n">
-        <v>-89000</v>
+        <v>-144255</v>
       </c>
       <c r="AH139" s="13" t="n">
-        <v>-5.235294117647059</v>
+        <v>-8.485588235294118</v>
       </c>
       <c r="AI139" s="13" t="n">
-        <v>-470.8994708994709</v>
+        <v>-763.2539682539683</v>
       </c>
       <c r="AJ139" s="13" t="n">
-        <v>-1975000</v>
+        <v>-2030255</v>
       </c>
       <c r="AK139" s="13" t="n">
-        <v>-116.1764705882353</v>
+        <v>-119.4267647058823</v>
       </c>
       <c r="AL139" s="13" t="n">
-        <v>-10449.73544973545</v>
+        <v>-10742.08994708995</v>
       </c>
     </row>
     <row r="140">
@@ -12164,22 +12284,22 @@
         <v>-5569215.973544973</v>
       </c>
       <c r="AG140" s="15" t="n">
-        <v>-2046000</v>
+        <v>-69008999</v>
       </c>
       <c r="AH140" s="15" t="n">
-        <v>-120.3529411764706</v>
+        <v>-4059.352882352941</v>
       </c>
       <c r="AI140" s="15" t="n">
-        <v>-10825.39682539683</v>
+        <v>-365126.9788359788</v>
       </c>
       <c r="AJ140" s="15" t="n">
-        <v>-1054627819</v>
+        <v>-1121590818</v>
       </c>
       <c r="AK140" s="15" t="n">
-        <v>-62036.93052941176</v>
+        <v>-65975.93047058824</v>
       </c>
       <c r="AL140" s="15" t="n">
-        <v>-5580041.370370369</v>
+        <v>-5934342.952380951</v>
       </c>
     </row>
     <row r="141">
@@ -12234,13 +12354,13 @@
         <v>-14043856.37809524</v>
       </c>
       <c r="R141" s="15" t="n">
-        <v>-3460166313.44</v>
+        <v>-3433461313.44</v>
       </c>
       <c r="S141" s="15" t="n">
-        <v>-203539.1949082353</v>
+        <v>-201968.3125552941</v>
       </c>
       <c r="T141" s="15" t="n">
-        <v>-18307758.27216931</v>
+        <v>-18166461.97587302</v>
       </c>
       <c r="U141" s="15" t="n">
         <v>-4043210976</v>
@@ -12270,31 +12390,31 @@
         <v>-23607854.00142857</v>
       </c>
       <c r="AD141" s="15" t="n">
-        <v>-47983198559.17</v>
+        <v>-47956493559.17</v>
       </c>
       <c r="AE141" s="15" t="n">
-        <v>-2822541.091715883</v>
+        <v>-2820970.209362941</v>
       </c>
       <c r="AF141" s="15" t="n">
-        <v>-253879357.4559259</v>
+        <v>-253738061.1596296</v>
       </c>
       <c r="AG141" s="15" t="n">
-        <v>-110536681</v>
+        <v>-831870274</v>
       </c>
       <c r="AH141" s="15" t="n">
-        <v>-6502.157705882353</v>
+        <v>-48933.54552941176</v>
       </c>
       <c r="AI141" s="15" t="n">
-        <v>-584850.1640211641</v>
+        <v>-4401430.021164021</v>
       </c>
       <c r="AJ141" s="15" t="n">
-        <v>-48093735240.17</v>
+        <v>-48788363833.17</v>
       </c>
       <c r="AK141" s="15" t="n">
-        <v>-2829043.249421765</v>
+        <v>-2869903.754892353</v>
       </c>
       <c r="AL141" s="15" t="n">
-        <v>-254464207.6199471</v>
+        <v>-258139491.1807937</v>
       </c>
     </row>
     <row r="142">
@@ -12521,17 +12641,23 @@
       <c r="AF144" s="13" t="n">
         <v>-5281271.338624339</v>
       </c>
-      <c r="AG144" s="13" t="n"/>
-      <c r="AH144" s="13" t="n"/>
-      <c r="AI144" s="13" t="n"/>
+      <c r="AG144" s="13" t="n">
+        <v>-9500000</v>
+      </c>
+      <c r="AH144" s="13" t="n">
+        <v>-558.8235294117648</v>
+      </c>
+      <c r="AI144" s="13" t="n">
+        <v>-50264.55026455026</v>
+      </c>
       <c r="AJ144" s="13" t="n">
-        <v>-998160283</v>
+        <v>-1007660283</v>
       </c>
       <c r="AK144" s="13" t="n">
-        <v>-58715.31076470588</v>
+        <v>-59274.13429411764</v>
       </c>
       <c r="AL144" s="13" t="n">
-        <v>-5281271.338624339</v>
+        <v>-5331535.888888889</v>
       </c>
     </row>
     <row r="145">
@@ -12752,17 +12878,23 @@
       <c r="AF147" s="15" t="n">
         <v>-14123139.06349206</v>
       </c>
-      <c r="AG147" s="15" t="n"/>
-      <c r="AH147" s="15" t="n"/>
-      <c r="AI147" s="15" t="n"/>
+      <c r="AG147" s="15" t="n">
+        <v>-9500000</v>
+      </c>
+      <c r="AH147" s="15" t="n">
+        <v>-558.8235294117648</v>
+      </c>
+      <c r="AI147" s="15" t="n">
+        <v>-50264.55026455026</v>
+      </c>
       <c r="AJ147" s="15" t="n">
-        <v>-2669273283</v>
+        <v>-2678773283</v>
       </c>
       <c r="AK147" s="15" t="n">
-        <v>-157016.0754705882</v>
+        <v>-157574.899</v>
       </c>
       <c r="AL147" s="15" t="n">
-        <v>-14123139.06349206</v>
+        <v>-14173403.61375661</v>
       </c>
     </row>
     <row r="148">
@@ -12905,22 +13037,22 @@
         <v>-107075.0670899471</v>
       </c>
       <c r="AG149" s="11" t="n">
-        <v>-18200</v>
+        <v>-24700</v>
       </c>
       <c r="AH149" s="11" t="n">
-        <v>-1.070588235294118</v>
+        <v>-1.452941176470588</v>
       </c>
       <c r="AI149" s="11" t="n">
-        <v>-96.29629629629629</v>
+        <v>-130.6878306878307</v>
       </c>
       <c r="AJ149" s="11" t="n">
-        <v>-20255387.68</v>
+        <v>-20261887.68</v>
       </c>
       <c r="AK149" s="11" t="n">
-        <v>-1191.493392941176</v>
+        <v>-1191.875745882353</v>
       </c>
       <c r="AL149" s="11" t="n">
-        <v>-107171.3633862434</v>
+        <v>-107205.7549206349</v>
       </c>
     </row>
     <row r="150">
@@ -13542,22 +13674,22 @@
         <v>-33089923.13634921</v>
       </c>
       <c r="AG156" s="15" t="n">
-        <v>-18200</v>
+        <v>-24700</v>
       </c>
       <c r="AH156" s="15" t="n">
-        <v>-1.070588235294118</v>
+        <v>-1.452941176470588</v>
       </c>
       <c r="AI156" s="15" t="n">
-        <v>-96.29629629629629</v>
+        <v>-130.6878306878307</v>
       </c>
       <c r="AJ156" s="15" t="n">
-        <v>-6254013672.77</v>
+        <v>-6254020172.77</v>
       </c>
       <c r="AK156" s="15" t="n">
-        <v>-367883.1572217647</v>
+        <v>-367883.5395747059</v>
       </c>
       <c r="AL156" s="15" t="n">
-        <v>-33090019.4326455</v>
+        <v>-33090053.8241799</v>
       </c>
     </row>
     <row r="157">
@@ -13657,22 +13789,22 @@
         <v>-1609397741.344392</v>
       </c>
       <c r="AG157" s="19" t="n">
-        <v>-1899751774</v>
+        <v>-4395763873</v>
       </c>
       <c r="AH157" s="19" t="n">
-        <v>-111750.1043529412</v>
+        <v>-258574.3454705882</v>
       </c>
       <c r="AI157" s="19" t="n">
-        <v>-10051596.68783069</v>
+        <v>-23258009.91005291</v>
       </c>
       <c r="AJ157" s="19" t="n">
-        <v>-306075924888.09</v>
+        <v>-308571936987.09</v>
       </c>
       <c r="AK157" s="19" t="n">
-        <v>-18004466.16988764</v>
+        <v>-18151290.41100529</v>
       </c>
       <c r="AL157" s="19" t="n">
-        <v>-1619449338.032222</v>
+        <v>-1632655751.254445</v>
       </c>
     </row>
     <row r="158">
@@ -13772,22 +13904,22 @@
         <v>-277217918.5799472</v>
       </c>
       <c r="AG158" s="19" t="n">
-        <v>4442702874</v>
+        <v>2000565275</v>
       </c>
       <c r="AH158" s="19" t="n">
-        <v>261335.4631764706</v>
+        <v>117680.3102941176</v>
       </c>
       <c r="AI158" s="19" t="n">
-        <v>23506364.41269841</v>
+        <v>10585001.45502646</v>
       </c>
       <c r="AJ158" s="19" t="n">
-        <v>-47951483737.61</v>
+        <v>-50393621336.61</v>
       </c>
       <c r="AK158" s="19" t="n">
-        <v>-2820675.51397706</v>
+        <v>-2964330.666859413</v>
       </c>
       <c r="AL158" s="19" t="n">
-        <v>-253711554.1672488</v>
+        <v>-266632917.1249208</v>
       </c>
     </row>
     <row r="159">
@@ -13887,22 +14019,22 @@
         <v>79785577.85582009</v>
       </c>
       <c r="AG159" s="7" t="n">
-        <v>19522177088.75</v>
+        <v>17080039489.75</v>
       </c>
       <c r="AH159" s="7" t="n">
-        <v>1148363.358161765</v>
+        <v>1004708.205279412</v>
       </c>
       <c r="AI159" s="7" t="n">
-        <v>103291942.2685185</v>
+        <v>90370579.31084657</v>
       </c>
       <c r="AJ159" s="7" t="n">
-        <v>19522177088.75</v>
+        <v>17080039489.75</v>
       </c>
       <c r="AK159" s="7" t="n">
-        <v>1148363.358161765</v>
+        <v>1004708.205279412</v>
       </c>
       <c r="AL159" s="7" t="n">
-        <v>103291942.2685185</v>
+        <v>90370579.31084657</v>
       </c>
     </row>
   </sheetData>
@@ -14705,16 +14837,16 @@
         <v>14828882907</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>4458981874</v>
+        <v>421365900</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>19287864781</v>
+        <v>15250248807</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>1134580.281235294</v>
+        <v>897073.4592352941</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>102052194.6084656</v>
+        <v>80689147.12698413</v>
       </c>
     </row>
     <row r="7">
@@ -14737,16 +14869,16 @@
         <v>18099375</v>
       </c>
       <c r="E7" s="13" t="n">
-        <v>0</v>
+        <v>200000000</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>18099375</v>
+        <v>218099375</v>
       </c>
       <c r="G7" s="24" t="n">
-        <v>1064.669117647059</v>
+        <v>12829.375</v>
       </c>
       <c r="H7" s="24" t="n">
-        <v>95763.88888888889</v>
+        <v>1153964.947089947</v>
       </c>
     </row>
     <row r="8">
@@ -14801,16 +14933,16 @@
         <v>22400563.84000001</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>-16304000</v>
+        <v>55070136</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>6096563.840000011</v>
+        <v>77470699.84</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>358.6214023529418</v>
+        <v>4557.099990588235</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>32256.95153439159</v>
+        <v>409897.8827513228</v>
       </c>
     </row>
     <row r="10">
@@ -14920,13 +15052,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>19522177090.75</v>
+        <v>15755935252.75</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>1148363.358279412</v>
+        <v>926819.7207499999</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>103291942.2791006</v>
+        <v>83364736.78703703</v>
       </c>
     </row>
   </sheetData>
@@ -14999,7 +15131,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 06 Oct 2026 16:19 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 09 Oct 2026 16:19 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -15081,14 +15213,14 @@
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 06 Oct 2026</t>
+          <t>MTD as of 09 Oct 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
       <c r="AI3" s="4" t="n"/>
       <c r="AJ3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 06 Oct 2026</t>
+          <t>YTD as of 09 Oct 2026</t>
         </is>
       </c>
       <c r="AK3" s="4" t="n"/>
@@ -15532,22 +15664,22 @@
         <v>1066.081968222222</v>
       </c>
       <c r="AG7" s="11" t="n">
-        <v>6339.231148</v>
+        <v>6390.025148</v>
       </c>
       <c r="AH7" s="11" t="n">
-        <v>0.3728959498823529</v>
+        <v>0.3758838322352941</v>
       </c>
       <c r="AI7" s="11" t="n">
-        <v>33.54090554497355</v>
+        <v>33.80965686772487</v>
       </c>
       <c r="AJ7" s="11" t="n">
-        <v>207828.723142</v>
+        <v>207879.517142</v>
       </c>
       <c r="AK7" s="11" t="n">
-        <v>12.22521900835294</v>
+        <v>12.22820689070588</v>
       </c>
       <c r="AL7" s="11" t="n">
-        <v>1099.622873767196</v>
+        <v>1099.891625089947</v>
       </c>
     </row>
     <row r="8">
@@ -16223,17 +16355,23 @@
       <c r="AF15" s="11" t="n">
         <v>0.3988330899470899</v>
       </c>
-      <c r="AG15" s="11" t="n"/>
-      <c r="AH15" s="11" t="n"/>
-      <c r="AI15" s="11" t="n"/>
+      <c r="AG15" s="11" t="n">
+        <v>50.794</v>
+      </c>
+      <c r="AH15" s="11" t="n">
+        <v>0.002987882352941176</v>
+      </c>
+      <c r="AI15" s="11" t="n">
+        <v>0.2687513227513227</v>
+      </c>
       <c r="AJ15" s="11" t="n">
-        <v>75.379454</v>
+        <v>126.173454</v>
       </c>
       <c r="AK15" s="11" t="n">
-        <v>0.004434085529411764</v>
+        <v>0.007421967882352941</v>
       </c>
       <c r="AL15" s="11" t="n">
-        <v>0.3988330899470899</v>
+        <v>0.6675844126984127</v>
       </c>
     </row>
     <row r="16">
@@ -16589,22 +16727,22 @@
         <v>2.521134965502646</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>3.2235</v>
+        <v>6.304</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>0.0001896176470588235</v>
+        <v>0.0003708235294117647</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>0.01705555555555556</v>
+        <v>0.03335449735449736</v>
       </c>
       <c r="AJ20" s="13" t="n">
-        <v>479.71800848</v>
+        <v>482.79850848</v>
       </c>
       <c r="AK20" s="13" t="n">
-        <v>0.02821870638117647</v>
+        <v>0.02839991226352941</v>
       </c>
       <c r="AL20" s="13" t="n">
-        <v>2.538190521058201</v>
+        <v>2.554489462857143</v>
       </c>
     </row>
     <row r="21">
@@ -16862,22 +17000,22 @@
         <v>0.4919761904761905</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>3.2235</v>
+        <v>5.304</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>0.0001896176470588235</v>
+        <v>0.000312</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>0.01705555555555556</v>
+        <v>0.02806349206349206</v>
       </c>
       <c r="AJ23" s="11" t="n">
-        <v>96.20700000000001</v>
+        <v>98.28750000000001</v>
       </c>
       <c r="AK23" s="11" t="n">
-        <v>0.005659235294117648</v>
+        <v>0.005781617647058824</v>
       </c>
       <c r="AL23" s="11" t="n">
-        <v>0.5090317460317461</v>
+        <v>0.5200396825396825</v>
       </c>
     </row>
     <row r="24">
@@ -17494,17 +17632,23 @@
       <c r="AF32" s="13" t="n">
         <v>0.02372502645502645</v>
       </c>
-      <c r="AG32" s="13" t="n"/>
-      <c r="AH32" s="13" t="n"/>
-      <c r="AI32" s="13" t="n"/>
+      <c r="AG32" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH32" s="13" t="n">
+        <v>5.882352941176471e-05</v>
+      </c>
+      <c r="AI32" s="13" t="n">
+        <v>0.005291005291005291</v>
+      </c>
       <c r="AJ32" s="13" t="n">
-        <v>4.48403</v>
+        <v>5.48403</v>
       </c>
       <c r="AK32" s="13" t="n">
-        <v>0.0002637664705882353</v>
+        <v>0.00032259</v>
       </c>
       <c r="AL32" s="13" t="n">
-        <v>0.02372502645502645</v>
+        <v>0.02901603174603174</v>
       </c>
     </row>
     <row r="33">
@@ -18402,22 +18546,22 @@
         <v>1332.179822764444</v>
       </c>
       <c r="AG45" s="15" t="n">
-        <v>6342.454648</v>
+        <v>6396.329148</v>
       </c>
       <c r="AH45" s="15" t="n">
-        <v>0.3730855675294117</v>
+        <v>0.3762546557647058</v>
       </c>
       <c r="AI45" s="15" t="n">
-        <v>33.5579611005291</v>
+        <v>33.84301136507936</v>
       </c>
       <c r="AJ45" s="15" t="n">
-        <v>258124.44115048</v>
+        <v>258178.31565048</v>
       </c>
       <c r="AK45" s="15" t="n">
-        <v>15.18379065591059</v>
+        <v>15.18695974414588</v>
       </c>
       <c r="AL45" s="15" t="n">
-        <v>1365.737783864974</v>
+        <v>1366.022834129524</v>
       </c>
     </row>
     <row r="46">
@@ -18839,17 +18983,23 @@
       <c r="AF51" s="13" t="n">
         <v>-13.66999814285714</v>
       </c>
-      <c r="AG51" s="13" t="n"/>
-      <c r="AH51" s="13" t="n"/>
-      <c r="AI51" s="13" t="n"/>
+      <c r="AG51" s="13" t="n">
+        <v>-64.097151</v>
+      </c>
+      <c r="AH51" s="13" t="n">
+        <v>-0.003770420647058823</v>
+      </c>
+      <c r="AI51" s="13" t="n">
+        <v>-0.3391383650793651</v>
+      </c>
       <c r="AJ51" s="13" t="n">
-        <v>-2583.629649</v>
+        <v>-2647.7268</v>
       </c>
       <c r="AK51" s="13" t="n">
-        <v>-0.1519782146470589</v>
+        <v>-0.1557486352941177</v>
       </c>
       <c r="AL51" s="13" t="n">
-        <v>-13.66999814285714</v>
+        <v>-14.00913650793651</v>
       </c>
     </row>
     <row r="52">
@@ -18918,17 +19068,23 @@
       <c r="AF52" s="11" t="n">
         <v>-0.9861469047619047</v>
       </c>
-      <c r="AG52" s="11" t="n"/>
-      <c r="AH52" s="11" t="n"/>
-      <c r="AI52" s="11" t="n"/>
+      <c r="AG52" s="11" t="n">
+        <v>-46.95078</v>
+      </c>
+      <c r="AH52" s="11" t="n">
+        <v>-0.002761810588235294</v>
+      </c>
+      <c r="AI52" s="11" t="n">
+        <v>-0.2484168253968254</v>
+      </c>
       <c r="AJ52" s="11" t="n">
-        <v>-186.381765</v>
+        <v>-233.332545</v>
       </c>
       <c r="AK52" s="11" t="n">
-        <v>-0.01096363323529412</v>
+        <v>-0.01372544382352941</v>
       </c>
       <c r="AL52" s="11" t="n">
-        <v>-0.9861469047619047</v>
+        <v>-1.23456373015873</v>
       </c>
     </row>
     <row r="53">
@@ -19143,17 +19299,23 @@
       <c r="AF55" s="13" t="n">
         <v>-10.23762965079365</v>
       </c>
-      <c r="AG55" s="13" t="n"/>
-      <c r="AH55" s="13" t="n"/>
-      <c r="AI55" s="13" t="n"/>
+      <c r="AG55" s="13" t="n">
+        <v>-492.54</v>
+      </c>
+      <c r="AH55" s="13" t="n">
+        <v>-0.02897294117647059</v>
+      </c>
+      <c r="AI55" s="13" t="n">
+        <v>-2.606031746031746</v>
+      </c>
       <c r="AJ55" s="13" t="n">
-        <v>-1934.912004</v>
+        <v>-2427.452004</v>
       </c>
       <c r="AK55" s="13" t="n">
-        <v>-0.1138183531764706</v>
+        <v>-0.1427912943529412</v>
       </c>
       <c r="AL55" s="13" t="n">
-        <v>-10.23762965079365</v>
+        <v>-12.8436613968254</v>
       </c>
     </row>
     <row r="56">
@@ -19222,17 +19384,23 @@
       <c r="AF56" s="11" t="n">
         <v>-0.512265</v>
       </c>
-      <c r="AG56" s="11" t="n"/>
-      <c r="AH56" s="11" t="n"/>
-      <c r="AI56" s="11" t="n"/>
+      <c r="AG56" s="11" t="n">
+        <v>-184.85</v>
+      </c>
+      <c r="AH56" s="11" t="n">
+        <v>-0.01087352941176471</v>
+      </c>
+      <c r="AI56" s="11" t="n">
+        <v>-0.978042328042328</v>
+      </c>
       <c r="AJ56" s="11" t="n">
-        <v>-96.818085</v>
+        <v>-281.668085</v>
       </c>
       <c r="AK56" s="11" t="n">
-        <v>-0.005695181470588235</v>
+        <v>-0.01656871088235294</v>
       </c>
       <c r="AL56" s="11" t="n">
-        <v>-0.512265</v>
+        <v>-1.490307328042328</v>
       </c>
     </row>
     <row r="57">
@@ -19398,17 +19566,23 @@
       <c r="AF58" s="11" t="n">
         <v>-1.436633349206349</v>
       </c>
-      <c r="AG58" s="11" t="n"/>
-      <c r="AH58" s="11" t="n"/>
-      <c r="AI58" s="11" t="n"/>
+      <c r="AG58" s="11" t="n">
+        <v>-7.442175</v>
+      </c>
+      <c r="AH58" s="11" t="n">
+        <v>-0.000437775</v>
+      </c>
+      <c r="AI58" s="11" t="n">
+        <v>-0.0393765873015873</v>
+      </c>
       <c r="AJ58" s="11" t="n">
-        <v>-271.523703</v>
+        <v>-278.965878</v>
       </c>
       <c r="AK58" s="11" t="n">
-        <v>-0.01597198252941176</v>
+        <v>-0.01640975752941176</v>
       </c>
       <c r="AL58" s="11" t="n">
-        <v>-1.436633349206349</v>
+        <v>-1.476009936507936</v>
       </c>
     </row>
     <row r="59">
@@ -19463,13 +19637,13 @@
         <v>-0.4417195767195767</v>
       </c>
       <c r="R59" s="13" t="n">
-        <v>-9.372406</v>
+        <v>-36.077406</v>
       </c>
       <c r="S59" s="13" t="n">
-        <v>-0.000551318</v>
+        <v>-0.002122200352941177</v>
       </c>
       <c r="T59" s="13" t="n">
-        <v>-0.04958944973544974</v>
+        <v>-0.190885746031746</v>
       </c>
       <c r="U59" s="13" t="n">
         <v>-64.272988</v>
@@ -19499,25 +19673,31 @@
         <v>-1.072042687830688</v>
       </c>
       <c r="AD59" s="13" t="n">
-        <v>-3207.02486288</v>
+        <v>-3233.72986288</v>
       </c>
       <c r="AE59" s="13" t="n">
-        <v>-0.1886485213458823</v>
+        <v>-0.1902194036988235</v>
       </c>
       <c r="AF59" s="13" t="n">
-        <v>-16.9683855178836</v>
-      </c>
-      <c r="AG59" s="13" t="n"/>
-      <c r="AH59" s="13" t="n"/>
-      <c r="AI59" s="13" t="n"/>
+        <v>-17.10968181417989</v>
+      </c>
+      <c r="AG59" s="13" t="n">
+        <v>-59.229205</v>
+      </c>
+      <c r="AH59" s="13" t="n">
+        <v>-0.003484070882352941</v>
+      </c>
+      <c r="AI59" s="13" t="n">
+        <v>-0.313382037037037</v>
+      </c>
       <c r="AJ59" s="13" t="n">
-        <v>-3207.02486288</v>
+        <v>-3292.95906788</v>
       </c>
       <c r="AK59" s="13" t="n">
-        <v>-0.1886485213458823</v>
+        <v>-0.1937034745811765</v>
       </c>
       <c r="AL59" s="13" t="n">
-        <v>-16.9683855178836</v>
+        <v>-17.42306385121693</v>
       </c>
     </row>
     <row r="60">
@@ -19629,17 +19809,23 @@
       <c r="AF61" s="13" t="n">
         <v>-0.01058201058201058</v>
       </c>
-      <c r="AG61" s="13" t="n"/>
-      <c r="AH61" s="13" t="n"/>
-      <c r="AI61" s="13" t="n"/>
+      <c r="AG61" s="13" t="n">
+        <v>-36.672</v>
+      </c>
+      <c r="AH61" s="13" t="n">
+        <v>-0.002157176470588235</v>
+      </c>
+      <c r="AI61" s="13" t="n">
+        <v>-0.194031746031746</v>
+      </c>
       <c r="AJ61" s="13" t="n">
-        <v>-2</v>
+        <v>-38.672</v>
       </c>
       <c r="AK61" s="13" t="n">
-        <v>-0.0001176470588235294</v>
+        <v>-0.002274823529411765</v>
       </c>
       <c r="AL61" s="13" t="n">
-        <v>-0.01058201058201058</v>
+        <v>-0.2046137566137566</v>
       </c>
     </row>
     <row r="62">
@@ -19797,13 +19983,13 @@
         <v>-11.75877245502646</v>
       </c>
       <c r="R63" s="15" t="n">
-        <v>-1116.468582</v>
+        <v>-1143.173582</v>
       </c>
       <c r="S63" s="15" t="n">
-        <v>-0.06567462247058824</v>
+        <v>-0.06724550482352941</v>
       </c>
       <c r="T63" s="15" t="n">
-        <v>-5.907241174603175</v>
+        <v>-6.04853747089947</v>
       </c>
       <c r="U63" s="15" t="n">
         <v>-939.708047</v>
@@ -19833,25 +20019,31 @@
         <v>-10.28403952380952</v>
       </c>
       <c r="AD63" s="15" t="n">
-        <v>-17929.44465188</v>
+        <v>-17956.14965188</v>
       </c>
       <c r="AE63" s="15" t="n">
-        <v>-1.054673214816471</v>
+        <v>-1.056244097169412</v>
       </c>
       <c r="AF63" s="15" t="n">
-        <v>-94.8647865178836</v>
-      </c>
-      <c r="AG63" s="15" t="n"/>
-      <c r="AH63" s="15" t="n"/>
-      <c r="AI63" s="15" t="n"/>
+        <v>-95.0060828141799</v>
+      </c>
+      <c r="AG63" s="15" t="n">
+        <v>-891.781311</v>
+      </c>
+      <c r="AH63" s="15" t="n">
+        <v>-0.05245772417647059</v>
+      </c>
+      <c r="AI63" s="15" t="n">
+        <v>-4.718419634920635</v>
+      </c>
       <c r="AJ63" s="15" t="n">
-        <v>-17929.44465188</v>
+        <v>-18847.93096288</v>
       </c>
       <c r="AK63" s="15" t="n">
-        <v>-1.054673214816471</v>
+        <v>-1.108701821345882</v>
       </c>
       <c r="AL63" s="15" t="n">
-        <v>-94.8647865178836</v>
+        <v>-99.72450244910054</v>
       </c>
     </row>
     <row r="64">
@@ -20964,22 +21156,22 @@
         <v>-53.01535581481481</v>
       </c>
       <c r="AG81" s="11" t="n">
-        <v>-890.478933</v>
+        <v>-903.478933</v>
       </c>
       <c r="AH81" s="11" t="n">
-        <v>-0.05238111370588235</v>
+        <v>-0.05314581958823529</v>
       </c>
       <c r="AI81" s="11" t="n">
-        <v>-4.711528746031746</v>
+        <v>-4.780311814814815</v>
       </c>
       <c r="AJ81" s="11" t="n">
-        <v>-10910.381182</v>
+        <v>-10923.381182</v>
       </c>
       <c r="AK81" s="11" t="n">
-        <v>-0.6417871283529413</v>
+        <v>-0.6425518342352942</v>
       </c>
       <c r="AL81" s="11" t="n">
-        <v>-57.72688456084656</v>
+        <v>-57.79566762962963</v>
       </c>
     </row>
     <row r="82">
@@ -21079,22 +21271,22 @@
         <v>-58.93422933476191</v>
       </c>
       <c r="AG82" s="13" t="n">
-        <v>-897.91796</v>
+        <v>-1752.972535</v>
       </c>
       <c r="AH82" s="13" t="n">
-        <v>-0.05281870352941177</v>
+        <v>-0.1031160314705882</v>
       </c>
       <c r="AI82" s="13" t="n">
-        <v>-4.750888677248677</v>
+        <v>-9.274986957671958</v>
       </c>
       <c r="AJ82" s="13" t="n">
-        <v>-12036.48730427</v>
+        <v>-12891.54187927</v>
       </c>
       <c r="AK82" s="13" t="n">
-        <v>-0.7080286649570587</v>
+        <v>-0.7583259928982352</v>
       </c>
       <c r="AL82" s="13" t="n">
-        <v>-63.68511801201058</v>
+        <v>-68.20921629243387</v>
       </c>
     </row>
     <row r="83">
@@ -21303,22 +21495,22 @@
         <v>-2.427178873015873</v>
       </c>
       <c r="AG84" s="13" t="n">
-        <v>-0.8</v>
+        <v>-6.13612</v>
       </c>
       <c r="AH84" s="13" t="n">
-        <v>-4.705882352941177e-05</v>
+        <v>-0.0003609482352941177</v>
       </c>
       <c r="AI84" s="13" t="n">
-        <v>-0.004232804232804233</v>
+        <v>-0.03246624338624338</v>
       </c>
       <c r="AJ84" s="13" t="n">
-        <v>-459.5368070000001</v>
+        <v>-464.8729270000001</v>
       </c>
       <c r="AK84" s="13" t="n">
-        <v>-0.02703157688235295</v>
+        <v>-0.02734546629411765</v>
       </c>
       <c r="AL84" s="13" t="n">
-        <v>-2.431411677248677</v>
+        <v>-2.459645116402116</v>
       </c>
     </row>
     <row r="85">
@@ -21418,22 +21610,22 @@
         <v>-170.4732640490476</v>
       </c>
       <c r="AG85" s="15" t="n">
-        <v>-1789.196893</v>
+        <v>-2662.587588</v>
       </c>
       <c r="AH85" s="15" t="n">
-        <v>-0.1052468760588235</v>
+        <v>-0.1566227992941176</v>
       </c>
       <c r="AI85" s="15" t="n">
-        <v>-9.466650227513227</v>
+        <v>-14.08776501587302</v>
       </c>
       <c r="AJ85" s="15" t="n">
-        <v>-34008.64379827</v>
+        <v>-34882.03449327</v>
       </c>
       <c r="AK85" s="15" t="n">
-        <v>-2.000508458721765</v>
+        <v>-2.051884381957059</v>
       </c>
       <c r="AL85" s="15" t="n">
-        <v>-179.9399142765608</v>
+        <v>-184.5610290649206</v>
       </c>
     </row>
     <row r="86">
@@ -21619,22 +21811,22 @@
         <v>-0.778818253968254</v>
       </c>
       <c r="AG88" s="11" t="n">
-        <v>-0.294372</v>
+        <v>-0.874372</v>
       </c>
       <c r="AH88" s="11" t="n">
-        <v>-1.7316e-05</v>
+        <v>-5.143364705882353e-05</v>
       </c>
       <c r="AI88" s="11" t="n">
-        <v>-0.00155752380952381</v>
+        <v>-0.004626306878306879</v>
       </c>
       <c r="AJ88" s="11" t="n">
-        <v>-147.491022</v>
+        <v>-148.071022</v>
       </c>
       <c r="AK88" s="11" t="n">
-        <v>-0.008675942470588234</v>
+        <v>-0.008710060117647057</v>
       </c>
       <c r="AL88" s="11" t="n">
-        <v>-0.7803757777777778</v>
+        <v>-0.7834445608465609</v>
       </c>
     </row>
     <row r="89">
@@ -21965,22 +22157,22 @@
         <v>-0.7864109841269842</v>
       </c>
       <c r="AG92" s="11" t="n">
-        <v>-1.0782</v>
+        <v>-1.0932</v>
       </c>
       <c r="AH92" s="11" t="n">
-        <v>-6.34235294117647e-05</v>
+        <v>-6.430588235294117e-05</v>
       </c>
       <c r="AI92" s="11" t="n">
-        <v>-0.005704761904761905</v>
+        <v>-0.005784126984126984</v>
       </c>
       <c r="AJ92" s="11" t="n">
-        <v>-149.709876</v>
+        <v>-149.724876</v>
       </c>
       <c r="AK92" s="11" t="n">
-        <v>-0.008806463294117647</v>
+        <v>-0.008807345647058824</v>
       </c>
       <c r="AL92" s="11" t="n">
-        <v>-0.7921157460317461</v>
+        <v>-0.7921951111111112</v>
       </c>
     </row>
     <row r="93">
@@ -22067,17 +22259,23 @@
       <c r="AF93" s="13" t="n">
         <v>-0.01277881481481482</v>
       </c>
-      <c r="AG93" s="13" t="n"/>
-      <c r="AH93" s="13" t="n"/>
-      <c r="AI93" s="13" t="n"/>
+      <c r="AG93" s="13" t="n">
+        <v>-0.2336</v>
+      </c>
+      <c r="AH93" s="13" t="n">
+        <v>-1.374117647058823e-05</v>
+      </c>
+      <c r="AI93" s="13" t="n">
+        <v>-0.001235978835978836</v>
+      </c>
       <c r="AJ93" s="13" t="n">
-        <v>-2.415196</v>
+        <v>-2.648796</v>
       </c>
       <c r="AK93" s="13" t="n">
-        <v>-0.0001420703529411765</v>
+        <v>-0.0001558115294117647</v>
       </c>
       <c r="AL93" s="13" t="n">
-        <v>-0.01277881481481482</v>
+        <v>-0.01401479365079365</v>
       </c>
     </row>
     <row r="94">
@@ -22177,22 +22375,22 @@
         <v>-2.636230425608466</v>
       </c>
       <c r="AG94" s="15" t="n">
-        <v>-2.145072</v>
+        <v>-2.973672</v>
       </c>
       <c r="AH94" s="15" t="n">
-        <v>-0.0001261807058823529</v>
+        <v>-0.0001749218823529412</v>
       </c>
       <c r="AI94" s="15" t="n">
-        <v>-0.0113495873015873</v>
+        <v>-0.01573371428571428</v>
       </c>
       <c r="AJ94" s="15" t="n">
-        <v>-500.3926224400001</v>
+        <v>-501.2212224400001</v>
       </c>
       <c r="AK94" s="15" t="n">
-        <v>-0.02943486014352941</v>
+        <v>-0.02948360132</v>
       </c>
       <c r="AL94" s="15" t="n">
-        <v>-2.647580012910053</v>
+        <v>-2.65196413989418</v>
       </c>
     </row>
     <row r="95">
@@ -22487,22 +22685,22 @@
         <v>-1.418156079365079</v>
       </c>
       <c r="AG98" s="11" t="n">
-        <v>-1.2485</v>
+        <v>-12.6402</v>
       </c>
       <c r="AH98" s="11" t="n">
-        <v>-7.344117647058823e-05</v>
+        <v>-0.0007435411764705883</v>
       </c>
       <c r="AI98" s="11" t="n">
-        <v>-0.006605820105820105</v>
+        <v>-0.06687936507936508</v>
       </c>
       <c r="AJ98" s="11" t="n">
-        <v>-269.279999</v>
+        <v>-280.671699</v>
       </c>
       <c r="AK98" s="11" t="n">
-        <v>-0.01583999994117647</v>
+        <v>-0.01651009994117647</v>
       </c>
       <c r="AL98" s="11" t="n">
-        <v>-1.424761899470899</v>
+        <v>-1.485035444444444</v>
       </c>
     </row>
     <row r="99">
@@ -22602,22 +22800,22 @@
         <v>-40.89323655941799</v>
       </c>
       <c r="AG99" s="13" t="n">
-        <v>-82.401009</v>
+        <v>-151.615974</v>
       </c>
       <c r="AH99" s="13" t="n">
-        <v>-0.004847118176470588</v>
+        <v>-0.008918586705882352</v>
       </c>
       <c r="AI99" s="13" t="n">
-        <v>-0.4359841746031746</v>
+        <v>-0.8022009206349207</v>
       </c>
       <c r="AJ99" s="13" t="n">
-        <v>-7811.22271873</v>
+        <v>-7880.437683730001</v>
       </c>
       <c r="AK99" s="13" t="n">
-        <v>-0.4594836893370588</v>
+        <v>-0.4635551578664706</v>
       </c>
       <c r="AL99" s="13" t="n">
-        <v>-41.32922073402117</v>
+        <v>-41.69543748005292</v>
       </c>
     </row>
     <row r="100">
@@ -22716,17 +22914,23 @@
       <c r="AF100" s="11" t="n">
         <v>-1.318975026455027</v>
       </c>
-      <c r="AG100" s="11" t="n"/>
-      <c r="AH100" s="11" t="n"/>
-      <c r="AI100" s="11" t="n"/>
+      <c r="AG100" s="11" t="n">
+        <v>-7.999429</v>
+      </c>
+      <c r="AH100" s="11" t="n">
+        <v>-0.0004705546470588235</v>
+      </c>
+      <c r="AI100" s="11" t="n">
+        <v>-0.04232502116402116</v>
+      </c>
       <c r="AJ100" s="11" t="n">
-        <v>-249.28628</v>
+        <v>-257.285709</v>
       </c>
       <c r="AK100" s="11" t="n">
-        <v>-0.01466389882352941</v>
+        <v>-0.01513445347058823</v>
       </c>
       <c r="AL100" s="11" t="n">
-        <v>-1.318975026455027</v>
+        <v>-1.361300047619048</v>
       </c>
     </row>
     <row r="101">
@@ -22808,40 +23012,40 @@
         <v>-0.2118974867724868</v>
       </c>
       <c r="AA101" s="13" t="n">
-        <v>-31.0402</v>
+        <v>-31.24195</v>
       </c>
       <c r="AB101" s="13" t="n">
-        <v>-0.001825894117647059</v>
+        <v>-0.001837761764705882</v>
       </c>
       <c r="AC101" s="13" t="n">
-        <v>-0.1642338624338624</v>
+        <v>-0.1653013227513228</v>
       </c>
       <c r="AD101" s="13" t="n">
-        <v>-364.2221070000001</v>
+        <v>-364.423857</v>
       </c>
       <c r="AE101" s="13" t="n">
-        <v>-0.02142482982352941</v>
+        <v>-0.02143669747058824</v>
       </c>
       <c r="AF101" s="13" t="n">
-        <v>-1.927101095238095</v>
+        <v>-1.928168555555555</v>
       </c>
       <c r="AG101" s="13" t="n">
-        <v>-1.1094</v>
+        <v>-4.33215</v>
       </c>
       <c r="AH101" s="13" t="n">
-        <v>-6.525882352941176e-05</v>
+        <v>-0.0002548323529411765</v>
       </c>
       <c r="AI101" s="13" t="n">
-        <v>-0.00586984126984127</v>
+        <v>-0.02292142857142857</v>
       </c>
       <c r="AJ101" s="13" t="n">
-        <v>-365.331507</v>
+        <v>-368.756007</v>
       </c>
       <c r="AK101" s="13" t="n">
-        <v>-0.02149008864705883</v>
+        <v>-0.02169152982352941</v>
       </c>
       <c r="AL101" s="13" t="n">
-        <v>-1.932970936507936</v>
+        <v>-1.951089984126984</v>
       </c>
     </row>
     <row r="102">
@@ -22923,40 +23127,40 @@
         <v>-3.812258455026455</v>
       </c>
       <c r="AA102" s="15" t="n">
-        <v>-886.27612627</v>
+        <v>-886.47787627</v>
       </c>
       <c r="AB102" s="15" t="n">
-        <v>-0.05213388978058824</v>
+        <v>-0.05214575742764706</v>
       </c>
       <c r="AC102" s="15" t="n">
-        <v>-4.689291673386244</v>
+        <v>-4.690359133703704</v>
       </c>
       <c r="AD102" s="15" t="n">
-        <v>-8732.265895730001</v>
+        <v>-8732.467645730001</v>
       </c>
       <c r="AE102" s="15" t="n">
-        <v>-0.5136626997488235</v>
+        <v>-0.5136745673958824</v>
       </c>
       <c r="AF102" s="15" t="n">
-        <v>-46.20246505677248</v>
+        <v>-46.20353251708994</v>
       </c>
       <c r="AG102" s="15" t="n">
-        <v>-85.29045000000001</v>
+        <v>-177.119294</v>
       </c>
       <c r="AH102" s="15" t="n">
-        <v>-0.005017085294117648</v>
+        <v>-0.010418782</v>
       </c>
       <c r="AI102" s="15" t="n">
-        <v>-0.4512722222222222</v>
+        <v>-0.9371391216931216</v>
       </c>
       <c r="AJ102" s="15" t="n">
-        <v>-8817.556345730001</v>
+        <v>-8909.586939730001</v>
       </c>
       <c r="AK102" s="15" t="n">
-        <v>-0.5186797850429411</v>
+        <v>-0.5240933493958824</v>
       </c>
       <c r="AL102" s="15" t="n">
-        <v>-46.6537372789947</v>
+        <v>-47.14067163878306</v>
       </c>
     </row>
     <row r="103">
@@ -23099,22 +23303,22 @@
         <v>-1.237435248677249</v>
       </c>
       <c r="AG104" s="11" t="n">
-        <v>-0.5445</v>
+        <v>-17.0946</v>
       </c>
       <c r="AH104" s="11" t="n">
-        <v>-3.202941176470588e-05</v>
+        <v>-0.001005564705882353</v>
       </c>
       <c r="AI104" s="11" t="n">
-        <v>-0.002880952380952381</v>
+        <v>-0.09044761904761904</v>
       </c>
       <c r="AJ104" s="11" t="n">
-        <v>-234.419762</v>
+        <v>-250.969862</v>
       </c>
       <c r="AK104" s="11" t="n">
-        <v>-0.01378939776470588</v>
+        <v>-0.01476293305882353</v>
       </c>
       <c r="AL104" s="11" t="n">
-        <v>-1.240316201058201</v>
+        <v>-1.327882867724868</v>
       </c>
     </row>
     <row r="105">
@@ -23214,22 +23418,22 @@
         <v>-1.864747592592592</v>
       </c>
       <c r="AG105" s="13" t="n">
-        <v>-0.587</v>
+        <v>-161.522493</v>
       </c>
       <c r="AH105" s="13" t="n">
-        <v>-3.452941176470588e-05</v>
+        <v>-0.00950132311764706</v>
       </c>
       <c r="AI105" s="13" t="n">
-        <v>-0.003105820105820106</v>
+        <v>-0.8546163650793651</v>
       </c>
       <c r="AJ105" s="13" t="n">
-        <v>-353.024295</v>
+        <v>-513.959788</v>
       </c>
       <c r="AK105" s="13" t="n">
-        <v>-0.020766135</v>
+        <v>-0.03023292870588235</v>
       </c>
       <c r="AL105" s="13" t="n">
-        <v>-1.867853412698413</v>
+        <v>-2.719363957671958</v>
       </c>
     </row>
     <row r="106">
@@ -23328,17 +23532,23 @@
       <c r="AF106" s="11" t="n">
         <v>-8.926693243386243</v>
       </c>
-      <c r="AG106" s="11" t="n"/>
-      <c r="AH106" s="11" t="n"/>
-      <c r="AI106" s="11" t="n"/>
+      <c r="AG106" s="11" t="n">
+        <v>-70.776068</v>
+      </c>
+      <c r="AH106" s="11" t="n">
+        <v>-0.004163298117647059</v>
+      </c>
+      <c r="AI106" s="11" t="n">
+        <v>-0.3744765502645502</v>
+      </c>
       <c r="AJ106" s="11" t="n">
-        <v>-1687.145023</v>
+        <v>-1757.921091</v>
       </c>
       <c r="AK106" s="11" t="n">
-        <v>-0.09924382488235292</v>
+        <v>-0.103407123</v>
       </c>
       <c r="AL106" s="11" t="n">
-        <v>-8.926693243386243</v>
+        <v>-9.301169793650793</v>
       </c>
     </row>
     <row r="107">
@@ -23431,17 +23641,23 @@
       <c r="AF107" s="13" t="n">
         <v>-1.059205370370371</v>
       </c>
-      <c r="AG107" s="13" t="n"/>
-      <c r="AH107" s="13" t="n"/>
-      <c r="AI107" s="13" t="n"/>
+      <c r="AG107" s="13" t="n">
+        <v>-34.937225</v>
+      </c>
+      <c r="AH107" s="13" t="n">
+        <v>-0.002055130882352941</v>
+      </c>
+      <c r="AI107" s="13" t="n">
+        <v>-0.1848530423280423</v>
+      </c>
       <c r="AJ107" s="13" t="n">
-        <v>-200.189815</v>
+        <v>-235.12704</v>
       </c>
       <c r="AK107" s="13" t="n">
-        <v>-0.01177587147058824</v>
+        <v>-0.01383100235294118</v>
       </c>
       <c r="AL107" s="13" t="n">
-        <v>-1.059205370370371</v>
+        <v>-1.244058412698413</v>
       </c>
     </row>
     <row r="108">
@@ -23541,22 +23757,22 @@
         <v>-13.08808145502645</v>
       </c>
       <c r="AG108" s="15" t="n">
-        <v>-1.1315</v>
+        <v>-284.330386</v>
       </c>
       <c r="AH108" s="15" t="n">
-        <v>-6.655882352941176e-05</v>
+        <v>-0.01672531682352941</v>
       </c>
       <c r="AI108" s="15" t="n">
-        <v>-0.005986772486772486</v>
+        <v>-1.504393576719577</v>
       </c>
       <c r="AJ108" s="15" t="n">
-        <v>-2474.778895</v>
+        <v>-2757.977781</v>
       </c>
       <c r="AK108" s="15" t="n">
-        <v>-0.145575229117647</v>
+        <v>-0.162233987117647</v>
       </c>
       <c r="AL108" s="15" t="n">
-        <v>-13.09406822751323</v>
+        <v>-14.59247503174603</v>
       </c>
     </row>
     <row r="109">
@@ -23830,13 +24046,13 @@
         <v>-0.1201455026455026</v>
       </c>
       <c r="R112" s="11" t="n">
-        <v>-81.19065000000001</v>
+        <v>-54.48565</v>
       </c>
       <c r="S112" s="11" t="n">
-        <v>-0.004775920588235294</v>
+        <v>-0.003205038235294117</v>
       </c>
       <c r="T112" s="11" t="n">
-        <v>-0.4295801587301588</v>
+        <v>-0.2882838624338624</v>
       </c>
       <c r="U112" s="11" t="n">
         <v>-147.792961</v>
@@ -23866,31 +24082,31 @@
         <v>-0.1475809523809524</v>
       </c>
       <c r="AD112" s="11" t="n">
-        <v>-496.8689110000001</v>
+        <v>-470.163911</v>
       </c>
       <c r="AE112" s="11" t="n">
-        <v>-0.029227583</v>
+        <v>-0.02765670064705882</v>
       </c>
       <c r="AF112" s="11" t="n">
-        <v>-2.628936037037037</v>
+        <v>-2.48763974074074</v>
       </c>
       <c r="AG112" s="11" t="n">
-        <v>-16.0875</v>
+        <v>-21.5875</v>
       </c>
       <c r="AH112" s="11" t="n">
-        <v>-0.0009463235294117646</v>
+        <v>-0.00126985294117647</v>
       </c>
       <c r="AI112" s="11" t="n">
-        <v>-0.08511904761904761</v>
+        <v>-0.1142195767195767</v>
       </c>
       <c r="AJ112" s="11" t="n">
-        <v>-512.9564110000001</v>
+        <v>-491.751411</v>
       </c>
       <c r="AK112" s="11" t="n">
-        <v>-0.03017390652941176</v>
+        <v>-0.02892655358823529</v>
       </c>
       <c r="AL112" s="11" t="n">
-        <v>-2.714055084656084</v>
+        <v>-2.601859317460317</v>
       </c>
     </row>
     <row r="113">
@@ -23945,13 +24161,13 @@
         <v>-0.1943783068783069</v>
       </c>
       <c r="R113" s="15" t="n">
-        <v>-144.56225</v>
+        <v>-117.85725</v>
       </c>
       <c r="S113" s="15" t="n">
-        <v>-0.008503661764705883</v>
+        <v>-0.006932779411764706</v>
       </c>
       <c r="T113" s="15" t="n">
-        <v>-0.7648796296296296</v>
+        <v>-0.6235833333333333</v>
       </c>
       <c r="U113" s="15" t="n">
         <v>-157.760461</v>
@@ -23981,31 +24197,31 @@
         <v>-0.1714830687830688</v>
       </c>
       <c r="AD113" s="15" t="n">
-        <v>-650.8765109999999</v>
+        <v>-624.1715109999999</v>
       </c>
       <c r="AE113" s="15" t="n">
-        <v>-0.03828685358823529</v>
+        <v>-0.03671597123529411</v>
       </c>
       <c r="AF113" s="15" t="n">
-        <v>-3.443791063492064</v>
+        <v>-3.302494767195767</v>
       </c>
       <c r="AG113" s="15" t="n">
-        <v>-16.0875</v>
+        <v>-21.5875</v>
       </c>
       <c r="AH113" s="15" t="n">
-        <v>-0.0009463235294117646</v>
+        <v>-0.00126985294117647</v>
       </c>
       <c r="AI113" s="15" t="n">
-        <v>-0.08511904761904761</v>
+        <v>-0.1142195767195767</v>
       </c>
       <c r="AJ113" s="15" t="n">
-        <v>-666.9640109999999</v>
+        <v>-645.7590109999999</v>
       </c>
       <c r="AK113" s="15" t="n">
-        <v>-0.03923317711764705</v>
+        <v>-0.03798582417647058</v>
       </c>
       <c r="AL113" s="15" t="n">
-        <v>-3.528910111111111</v>
+        <v>-3.416714343915344</v>
       </c>
     </row>
     <row r="114">
@@ -24141,17 +24357,23 @@
       <c r="AF115" s="11" t="n">
         <v>-2.418823142857143</v>
       </c>
-      <c r="AG115" s="11" t="n"/>
-      <c r="AH115" s="11" t="n"/>
-      <c r="AI115" s="11" t="n"/>
+      <c r="AG115" s="11" t="n">
+        <v>-37.104</v>
+      </c>
+      <c r="AH115" s="11" t="n">
+        <v>-0.002182588235294118</v>
+      </c>
+      <c r="AI115" s="11" t="n">
+        <v>-0.1963174603174603</v>
+      </c>
       <c r="AJ115" s="11" t="n">
-        <v>-457.1575740000001</v>
+        <v>-494.2615740000001</v>
       </c>
       <c r="AK115" s="11" t="n">
-        <v>-0.026891622</v>
+        <v>-0.02907421023529412</v>
       </c>
       <c r="AL115" s="11" t="n">
-        <v>-2.418823142857143</v>
+        <v>-2.615140603174603</v>
       </c>
     </row>
     <row r="116">
@@ -24311,17 +24533,23 @@
       <c r="AF117" s="11" t="n">
         <v>-0.7151995291005291</v>
       </c>
-      <c r="AG117" s="11" t="n"/>
-      <c r="AH117" s="11" t="n"/>
-      <c r="AI117" s="11" t="n"/>
+      <c r="AG117" s="11" t="n">
+        <v>-12.74</v>
+      </c>
+      <c r="AH117" s="11" t="n">
+        <v>-0.0007494117647058823</v>
+      </c>
+      <c r="AI117" s="11" t="n">
+        <v>-0.0674074074074074</v>
+      </c>
       <c r="AJ117" s="11" t="n">
-        <v>-135.172711</v>
+        <v>-147.912711</v>
       </c>
       <c r="AK117" s="11" t="n">
-        <v>-0.00795133594117647</v>
+        <v>-0.008700747705882353</v>
       </c>
       <c r="AL117" s="11" t="n">
-        <v>-0.7151995291005291</v>
+        <v>-0.7826069365079364</v>
       </c>
     </row>
     <row r="118">
@@ -24420,17 +24648,23 @@
       <c r="AF118" s="13" t="n">
         <v>-2.977326375661375</v>
       </c>
-      <c r="AG118" s="13" t="n"/>
-      <c r="AH118" s="13" t="n"/>
-      <c r="AI118" s="13" t="n"/>
+      <c r="AG118" s="13" t="n">
+        <v>-14.652</v>
+      </c>
+      <c r="AH118" s="13" t="n">
+        <v>-0.0008618823529411764</v>
+      </c>
+      <c r="AI118" s="13" t="n">
+        <v>-0.07752380952380952</v>
+      </c>
       <c r="AJ118" s="13" t="n">
-        <v>-562.714685</v>
+        <v>-577.3666850000001</v>
       </c>
       <c r="AK118" s="13" t="n">
-        <v>-0.03310086382352941</v>
+        <v>-0.03396274617647059</v>
       </c>
       <c r="AL118" s="13" t="n">
-        <v>-2.977326375661375</v>
+        <v>-3.054850185185185</v>
       </c>
     </row>
     <row r="119">
@@ -24529,17 +24763,23 @@
       <c r="AF119" s="15" t="n">
         <v>-6.180132116402117</v>
       </c>
-      <c r="AG119" s="15" t="n"/>
-      <c r="AH119" s="15" t="n"/>
-      <c r="AI119" s="15" t="n"/>
+      <c r="AG119" s="15" t="n">
+        <v>-64.496</v>
+      </c>
+      <c r="AH119" s="15" t="n">
+        <v>-0.003793882352941176</v>
+      </c>
+      <c r="AI119" s="15" t="n">
+        <v>-0.3412486772486772</v>
+      </c>
       <c r="AJ119" s="15" t="n">
-        <v>-1168.04497</v>
+        <v>-1232.54097</v>
       </c>
       <c r="AK119" s="15" t="n">
-        <v>-0.06870852764705883</v>
+        <v>-0.07250241</v>
       </c>
       <c r="AL119" s="15" t="n">
-        <v>-6.180132116402117</v>
+        <v>-6.521380793650794</v>
       </c>
     </row>
     <row r="120">
@@ -24698,13 +24938,13 @@
         <v>-1.429808666666667</v>
       </c>
       <c r="R122" s="13" t="n">
-        <v>-1626.344861</v>
+        <v>-1601.969861</v>
       </c>
       <c r="S122" s="13" t="n">
-        <v>-0.09566734476470588</v>
+        <v>-0.09423352123529412</v>
       </c>
       <c r="T122" s="13" t="n">
-        <v>-8.604999264550266</v>
+        <v>-8.476031010582011</v>
       </c>
       <c r="U122" s="13" t="n">
         <v>-678.09365</v>
@@ -24725,40 +24965,40 @@
         <v>-5.643998698412699</v>
       </c>
       <c r="AA122" s="13" t="n">
-        <v>-942.531373</v>
+        <v>-942.329623</v>
       </c>
       <c r="AB122" s="13" t="n">
-        <v>-0.05544302194117647</v>
+        <v>-0.05543115429411764</v>
       </c>
       <c r="AC122" s="13" t="n">
-        <v>-4.986938481481482</v>
+        <v>-4.985871021164021</v>
       </c>
       <c r="AD122" s="13" t="n">
-        <v>-6567.966353999999</v>
+        <v>-6543.389603999999</v>
       </c>
       <c r="AE122" s="13" t="n">
-        <v>-0.386350962</v>
+        <v>-0.3849052708235294</v>
       </c>
       <c r="AF122" s="13" t="n">
-        <v>-34.75114473015874</v>
+        <v>-34.62110901587301</v>
       </c>
       <c r="AG122" s="13" t="n">
-        <v>-3.836159</v>
+        <v>-212.354423</v>
       </c>
       <c r="AH122" s="13" t="n">
-        <v>-0.0002256564117647059</v>
+        <v>-0.01249143664705882</v>
       </c>
       <c r="AI122" s="13" t="n">
-        <v>-0.02029713756613757</v>
+        <v>-1.123568375661376</v>
       </c>
       <c r="AJ122" s="13" t="n">
-        <v>-6571.802513</v>
+        <v>-6755.744026999999</v>
       </c>
       <c r="AK122" s="13" t="n">
-        <v>-0.3865766184117647</v>
+        <v>-0.3973967074705882</v>
       </c>
       <c r="AL122" s="13" t="n">
-        <v>-34.77144186772487</v>
+        <v>-35.74467739153439</v>
       </c>
     </row>
     <row r="123">
@@ -24813,13 +25053,13 @@
         <v>-1.429808666666667</v>
       </c>
       <c r="R123" s="15" t="n">
-        <v>-1626.344861</v>
+        <v>-1601.969861</v>
       </c>
       <c r="S123" s="15" t="n">
-        <v>-0.09566734476470588</v>
+        <v>-0.09423352123529412</v>
       </c>
       <c r="T123" s="15" t="n">
-        <v>-8.604999264550266</v>
+        <v>-8.476031010582011</v>
       </c>
       <c r="U123" s="15" t="n">
         <v>-678.09365</v>
@@ -24840,40 +25080,40 @@
         <v>-5.643998698412699</v>
       </c>
       <c r="AA123" s="15" t="n">
-        <v>-1063.510186</v>
+        <v>-1063.308436</v>
       </c>
       <c r="AB123" s="15" t="n">
-        <v>-0.06255942270588236</v>
+        <v>-0.06254755505882353</v>
       </c>
       <c r="AC123" s="15" t="n">
-        <v>-5.627038021164021</v>
+        <v>-5.625970560846561</v>
       </c>
       <c r="AD123" s="15" t="n">
-        <v>-6688.945167</v>
+        <v>-6664.368417</v>
       </c>
       <c r="AE123" s="15" t="n">
-        <v>-0.3934673627647058</v>
+        <v>-0.3920216715882353</v>
       </c>
       <c r="AF123" s="15" t="n">
-        <v>-35.39124426984127</v>
+        <v>-35.26120855555556</v>
       </c>
       <c r="AG123" s="15" t="n">
-        <v>-3.836159</v>
+        <v>-212.354423</v>
       </c>
       <c r="AH123" s="15" t="n">
-        <v>-0.0002256564117647059</v>
+        <v>-0.01249143664705882</v>
       </c>
       <c r="AI123" s="15" t="n">
-        <v>-0.02029713756613757</v>
+        <v>-1.123568375661376</v>
       </c>
       <c r="AJ123" s="15" t="n">
-        <v>-6692.781326</v>
+        <v>-6876.722839999999</v>
       </c>
       <c r="AK123" s="15" t="n">
-        <v>-0.3936930191764705</v>
+        <v>-0.4045131082352941</v>
       </c>
       <c r="AL123" s="15" t="n">
-        <v>-35.41154140740741</v>
+        <v>-36.38477693121693</v>
       </c>
     </row>
     <row r="124">
@@ -25317,13 +25557,13 @@
         <v>-0.5581772486772487</v>
       </c>
       <c r="R129" s="11" t="n">
-        <v>-4.9</v>
+        <v>-29.275</v>
       </c>
       <c r="S129" s="11" t="n">
-        <v>-0.0002882352941176471</v>
+        <v>-0.001722058823529412</v>
       </c>
       <c r="T129" s="11" t="n">
-        <v>-0.02592592592592593</v>
+        <v>-0.1548941798941799</v>
       </c>
       <c r="U129" s="11" t="n">
         <v>-119.829</v>
@@ -25353,25 +25593,25 @@
         <v>-0.1428571428571428</v>
       </c>
       <c r="AD129" s="11" t="n">
-        <v>-355.114</v>
+        <v>-379.489</v>
       </c>
       <c r="AE129" s="11" t="n">
-        <v>-0.02088905882352941</v>
+        <v>-0.02232288235294118</v>
       </c>
       <c r="AF129" s="11" t="n">
-        <v>-1.878910052910053</v>
+        <v>-2.007878306878307</v>
       </c>
       <c r="AG129" s="11" t="n"/>
       <c r="AH129" s="11" t="n"/>
       <c r="AI129" s="11" t="n"/>
       <c r="AJ129" s="11" t="n">
-        <v>-355.114</v>
+        <v>-379.489</v>
       </c>
       <c r="AK129" s="11" t="n">
-        <v>-0.02088905882352941</v>
+        <v>-0.02232288235294118</v>
       </c>
       <c r="AL129" s="11" t="n">
-        <v>-1.878910052910053</v>
+        <v>-2.007878306878307</v>
       </c>
     </row>
     <row r="130">
@@ -25644,13 +25884,13 @@
         <v>-6.977825682539683</v>
       </c>
       <c r="R132" s="15" t="n">
-        <v>-416.051151</v>
+        <v>-440.426151</v>
       </c>
       <c r="S132" s="15" t="n">
-        <v>-0.02447359711764706</v>
+        <v>-0.02590742064705882</v>
       </c>
       <c r="T132" s="15" t="n">
-        <v>-2.201328841269841</v>
+        <v>-2.330297095238095</v>
       </c>
       <c r="U132" s="15" t="n">
         <v>-1928.971411</v>
@@ -25680,25 +25920,25 @@
         <v>-8.804195952380953</v>
       </c>
       <c r="AD132" s="15" t="n">
-        <v>-26718.589251</v>
+        <v>-26742.964251</v>
       </c>
       <c r="AE132" s="15" t="n">
-        <v>-1.571681720647059</v>
+        <v>-1.573115544176471</v>
       </c>
       <c r="AF132" s="15" t="n">
-        <v>-141.3681970952381</v>
+        <v>-141.4971653492063</v>
       </c>
       <c r="AG132" s="15" t="n"/>
       <c r="AH132" s="15" t="n"/>
       <c r="AI132" s="15" t="n"/>
       <c r="AJ132" s="15" t="n">
-        <v>-26718.589251</v>
+        <v>-26742.964251</v>
       </c>
       <c r="AK132" s="15" t="n">
-        <v>-1.571681720647059</v>
+        <v>-1.573115544176471</v>
       </c>
       <c r="AL132" s="15" t="n">
-        <v>-141.3681970952381</v>
+        <v>-141.4971653492063</v>
       </c>
     </row>
     <row r="133">
@@ -25829,22 +26069,22 @@
         <v>-0.1972583068783069</v>
       </c>
       <c r="AG134" s="11" t="n">
-        <v>-0.091</v>
+        <v>-2.404</v>
       </c>
       <c r="AH134" s="11" t="n">
-        <v>-5.352941176470588e-06</v>
+        <v>-0.0001414117647058823</v>
       </c>
       <c r="AI134" s="11" t="n">
-        <v>-0.0004814814814814815</v>
+        <v>-0.01271957671957672</v>
       </c>
       <c r="AJ134" s="11" t="n">
-        <v>-37.37282</v>
+        <v>-39.68582000000001</v>
       </c>
       <c r="AK134" s="11" t="n">
-        <v>-0.002198401176470589</v>
+        <v>-0.00233446</v>
       </c>
       <c r="AL134" s="11" t="n">
-        <v>-0.1977397883597883</v>
+        <v>-0.2099778835978836</v>
       </c>
     </row>
     <row r="135">
@@ -25931,17 +26171,23 @@
       <c r="AF135" s="13" t="n">
         <v>-2.537128</v>
       </c>
-      <c r="AG135" s="13" t="n"/>
-      <c r="AH135" s="13" t="n"/>
-      <c r="AI135" s="13" t="n"/>
+      <c r="AG135" s="13" t="n">
+        <v>-59.53072</v>
+      </c>
+      <c r="AH135" s="13" t="n">
+        <v>-0.003501807058823529</v>
+      </c>
+      <c r="AI135" s="13" t="n">
+        <v>-0.3149773544973545</v>
+      </c>
       <c r="AJ135" s="13" t="n">
-        <v>-479.517192</v>
+        <v>-539.047912</v>
       </c>
       <c r="AK135" s="13" t="n">
-        <v>-0.02820689364705883</v>
+        <v>-0.03170870070588236</v>
       </c>
       <c r="AL135" s="13" t="n">
-        <v>-2.537128</v>
+        <v>-2.852105354497354</v>
       </c>
     </row>
     <row r="136">
@@ -26132,22 +26378,22 @@
         <v>-0.6207355185185186</v>
       </c>
       <c r="AG137" s="13" t="n">
-        <v>-1.866</v>
+        <v>-4.2169</v>
       </c>
       <c r="AH137" s="13" t="n">
-        <v>-0.000109764705882353</v>
+        <v>-0.0002480529411764706</v>
       </c>
       <c r="AI137" s="13" t="n">
-        <v>-0.009873015873015874</v>
+        <v>-0.02231164021164021</v>
       </c>
       <c r="AJ137" s="13" t="n">
-        <v>-119.185013</v>
+        <v>-121.535913</v>
       </c>
       <c r="AK137" s="13" t="n">
-        <v>-0.007010883117647059</v>
+        <v>-0.007149171352941176</v>
       </c>
       <c r="AL137" s="13" t="n">
-        <v>-0.6306085343915345</v>
+        <v>-0.6430471587301588</v>
       </c>
     </row>
     <row r="138">
@@ -26240,17 +26486,23 @@
       <c r="AF138" s="11" t="n">
         <v>-1.110766867724868</v>
       </c>
-      <c r="AG138" s="11" t="n"/>
-      <c r="AH138" s="11" t="n"/>
-      <c r="AI138" s="11" t="n"/>
+      <c r="AG138" s="11" t="n">
+        <v>-2.713124</v>
+      </c>
+      <c r="AH138" s="11" t="n">
+        <v>-0.0001595955294117647</v>
+      </c>
+      <c r="AI138" s="11" t="n">
+        <v>-0.01435515343915344</v>
+      </c>
       <c r="AJ138" s="11" t="n">
-        <v>-209.934938</v>
+        <v>-212.648062</v>
       </c>
       <c r="AK138" s="11" t="n">
-        <v>-0.012349114</v>
+        <v>-0.01250870952941177</v>
       </c>
       <c r="AL138" s="11" t="n">
-        <v>-1.110766867724868</v>
+        <v>-1.125122021164021</v>
       </c>
     </row>
     <row r="139">
@@ -26314,22 +26566,22 @@
         <v>-0.009978835978835979</v>
       </c>
       <c r="AG139" s="13" t="n">
-        <v>-0.089</v>
+        <v>-0.144255</v>
       </c>
       <c r="AH139" s="13" t="n">
-        <v>-5.235294117647059e-06</v>
+        <v>-8.485588235294117e-06</v>
       </c>
       <c r="AI139" s="13" t="n">
-        <v>-0.0004708994708994709</v>
+        <v>-0.0007632539682539682</v>
       </c>
       <c r="AJ139" s="13" t="n">
-        <v>-1.975</v>
+        <v>-2.030255</v>
       </c>
       <c r="AK139" s="13" t="n">
-        <v>-0.0001161764705882353</v>
+        <v>-0.0001194267647058824</v>
       </c>
       <c r="AL139" s="13" t="n">
-        <v>-0.01044973544973545</v>
+        <v>-0.01074208994708995</v>
       </c>
     </row>
     <row r="140">
@@ -26429,22 +26681,22 @@
         <v>-5.569215973544973</v>
       </c>
       <c r="AG140" s="15" t="n">
-        <v>-2.046</v>
+        <v>-69.008999</v>
       </c>
       <c r="AH140" s="15" t="n">
-        <v>-0.0001203529411764706</v>
+        <v>-0.004059352882352941</v>
       </c>
       <c r="AI140" s="15" t="n">
-        <v>-0.01082539682539682</v>
+        <v>-0.3651269788359788</v>
       </c>
       <c r="AJ140" s="15" t="n">
-        <v>-1054.627819</v>
+        <v>-1121.590818</v>
       </c>
       <c r="AK140" s="15" t="n">
-        <v>-0.06203693052941176</v>
+        <v>-0.06597593047058824</v>
       </c>
       <c r="AL140" s="15" t="n">
-        <v>-5.58004137037037</v>
+        <v>-5.934342952380952</v>
       </c>
     </row>
     <row r="141">
@@ -26499,13 +26751,13 @@
         <v>-14.04385637809524</v>
       </c>
       <c r="R141" s="15" t="n">
-        <v>-3460.16631344</v>
+        <v>-3433.46131344</v>
       </c>
       <c r="S141" s="15" t="n">
-        <v>-0.2035391949082353</v>
+        <v>-0.2019683125552941</v>
       </c>
       <c r="T141" s="15" t="n">
-        <v>-18.30775827216931</v>
+        <v>-18.16646197587302</v>
       </c>
       <c r="U141" s="15" t="n">
         <v>-4043.210976</v>
@@ -26535,31 +26787,31 @@
         <v>-23.60785400142858</v>
       </c>
       <c r="AD141" s="15" t="n">
-        <v>-47983.19855917001</v>
+        <v>-47956.49355917001</v>
       </c>
       <c r="AE141" s="15" t="n">
-        <v>-2.822541091715882</v>
+        <v>-2.820970209362941</v>
       </c>
       <c r="AF141" s="15" t="n">
-        <v>-253.8793574559259</v>
+        <v>-253.7380611596296</v>
       </c>
       <c r="AG141" s="15" t="n">
-        <v>-110.536681</v>
+        <v>-831.870274</v>
       </c>
       <c r="AH141" s="15" t="n">
-        <v>-0.006502157705882353</v>
+        <v>-0.04893354552941177</v>
       </c>
       <c r="AI141" s="15" t="n">
-        <v>-0.5848501640211641</v>
+        <v>-4.401430021164021</v>
       </c>
       <c r="AJ141" s="15" t="n">
-        <v>-48093.73524017</v>
+        <v>-48788.36383317001</v>
       </c>
       <c r="AK141" s="15" t="n">
-        <v>-2.829043249421765</v>
+        <v>-2.869903754892353</v>
       </c>
       <c r="AL141" s="15" t="n">
-        <v>-254.4642076199471</v>
+        <v>-258.1394911807936</v>
       </c>
     </row>
     <row r="142">
@@ -26786,17 +27038,23 @@
       <c r="AF144" s="13" t="n">
         <v>-5.281271338624339</v>
       </c>
-      <c r="AG144" s="13" t="n"/>
-      <c r="AH144" s="13" t="n"/>
-      <c r="AI144" s="13" t="n"/>
+      <c r="AG144" s="13" t="n">
+        <v>-9.5</v>
+      </c>
+      <c r="AH144" s="13" t="n">
+        <v>-0.0005588235294117647</v>
+      </c>
+      <c r="AI144" s="13" t="n">
+        <v>-0.05026455026455026</v>
+      </c>
       <c r="AJ144" s="13" t="n">
-        <v>-998.160283</v>
+        <v>-1007.660283</v>
       </c>
       <c r="AK144" s="13" t="n">
-        <v>-0.0587153107647059</v>
+        <v>-0.05927413429411766</v>
       </c>
       <c r="AL144" s="13" t="n">
-        <v>-5.281271338624339</v>
+        <v>-5.331535888888889</v>
       </c>
     </row>
     <row r="145">
@@ -27017,17 +27275,23 @@
       <c r="AF147" s="15" t="n">
         <v>-14.12313906349206</v>
       </c>
-      <c r="AG147" s="15" t="n"/>
-      <c r="AH147" s="15" t="n"/>
-      <c r="AI147" s="15" t="n"/>
+      <c r="AG147" s="15" t="n">
+        <v>-9.5</v>
+      </c>
+      <c r="AH147" s="15" t="n">
+        <v>-0.0005588235294117647</v>
+      </c>
+      <c r="AI147" s="15" t="n">
+        <v>-0.05026455026455026</v>
+      </c>
       <c r="AJ147" s="15" t="n">
-        <v>-2669.273283</v>
+        <v>-2678.773283</v>
       </c>
       <c r="AK147" s="15" t="n">
-        <v>-0.1570160754705882</v>
+        <v>-0.157574899</v>
       </c>
       <c r="AL147" s="15" t="n">
-        <v>-14.12313906349206</v>
+        <v>-14.17340361375661</v>
       </c>
     </row>
     <row r="148">
@@ -27170,22 +27434,22 @@
         <v>-0.1070750670899471</v>
       </c>
       <c r="AG149" s="11" t="n">
-        <v>-0.0182</v>
+        <v>-0.0247</v>
       </c>
       <c r="AH149" s="11" t="n">
-        <v>-1.070588235294118e-06</v>
+        <v>-1.452941176470588e-06</v>
       </c>
       <c r="AI149" s="11" t="n">
-        <v>-9.62962962962963e-05</v>
+        <v>-0.0001306878306878307</v>
       </c>
       <c r="AJ149" s="11" t="n">
-        <v>-20.25538768</v>
+        <v>-20.26188768</v>
       </c>
       <c r="AK149" s="11" t="n">
-        <v>-0.001191493392941177</v>
+        <v>-0.001191875745882353</v>
       </c>
       <c r="AL149" s="11" t="n">
-        <v>-0.1071713633862434</v>
+        <v>-0.1072057549206349</v>
       </c>
     </row>
     <row r="150">
@@ -27807,22 +28071,22 @@
         <v>-33.08992313634921</v>
       </c>
       <c r="AG156" s="15" t="n">
-        <v>-0.0182</v>
+        <v>-0.0247</v>
       </c>
       <c r="AH156" s="15" t="n">
-        <v>-1.070588235294118e-06</v>
+        <v>-1.452941176470588e-06</v>
       </c>
       <c r="AI156" s="15" t="n">
-        <v>-9.62962962962963e-05</v>
+        <v>-0.0001306878306878307</v>
       </c>
       <c r="AJ156" s="15" t="n">
-        <v>-6254.01367277</v>
+        <v>-6254.02017277</v>
       </c>
       <c r="AK156" s="15" t="n">
-        <v>-0.3678831572217647</v>
+        <v>-0.3678835395747059</v>
       </c>
       <c r="AL156" s="15" t="n">
-        <v>-33.09001943264551</v>
+        <v>-33.0900538241799</v>
       </c>
     </row>
     <row r="157">
@@ -27922,22 +28186,22 @@
         <v>-1609.397741344392</v>
       </c>
       <c r="AG157" s="19" t="n">
-        <v>-1899.751774</v>
+        <v>-4395.763873</v>
       </c>
       <c r="AH157" s="19" t="n">
-        <v>-0.1117501043529412</v>
+        <v>-0.2585743454705882</v>
       </c>
       <c r="AI157" s="19" t="n">
-        <v>-10.05159668783069</v>
+        <v>-23.25800991005291</v>
       </c>
       <c r="AJ157" s="19" t="n">
-        <v>-306075.9248880899</v>
+        <v>-308571.9369870899</v>
       </c>
       <c r="AK157" s="19" t="n">
-        <v>-18.00446616988765</v>
+        <v>-18.1512904110053</v>
       </c>
       <c r="AL157" s="19" t="n">
-        <v>-1619.449338032222</v>
+        <v>-1632.655751254444</v>
       </c>
     </row>
     <row r="158">
@@ -28037,22 +28301,22 @@
         <v>-277.2179185799473</v>
       </c>
       <c r="AG158" s="19" t="n">
-        <v>4442.702874</v>
+        <v>2000.565275</v>
       </c>
       <c r="AH158" s="19" t="n">
-        <v>0.2613354631764706</v>
+        <v>0.1176803102941176</v>
       </c>
       <c r="AI158" s="19" t="n">
-        <v>23.50636441269841</v>
+        <v>10.58500145502645</v>
       </c>
       <c r="AJ158" s="19" t="n">
-        <v>-47951.48373761</v>
+        <v>-50393.62133661</v>
       </c>
       <c r="AK158" s="19" t="n">
-        <v>-2.820675513977061</v>
+        <v>-2.964330666859413</v>
       </c>
       <c r="AL158" s="19" t="n">
-        <v>-253.7115541672488</v>
+        <v>-266.6329171249208</v>
       </c>
     </row>
     <row r="159">
@@ -28152,22 +28416,22 @@
         <v>79.78557785582009</v>
       </c>
       <c r="AG159" s="7" t="n">
-        <v>19522.17708875</v>
+        <v>17080.03948975</v>
       </c>
       <c r="AH159" s="7" t="n">
-        <v>1.148363358161765</v>
+        <v>1.004708205279412</v>
       </c>
       <c r="AI159" s="7" t="n">
-        <v>103.2919422685185</v>
+        <v>90.37057931084657</v>
       </c>
       <c r="AJ159" s="7" t="n">
-        <v>19522.17708875</v>
+        <v>17080.03948975</v>
       </c>
       <c r="AK159" s="7" t="n">
-        <v>1.148363358161765</v>
+        <v>1.004708205279412</v>
       </c>
       <c r="AL159" s="7" t="n">
-        <v>103.2919422685185</v>
+        <v>90.37057931084657</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Mon 10/12/2026 11:57
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -734,7 +734,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 09 Oct 2026 16:19</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 12 Oct 2026 11:57</t>
         </is>
       </c>
     </row>
@@ -816,14 +816,14 @@
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 09 Oct 2026</t>
+          <t>MTD as of 12 Oct 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
       <c r="AI3" s="4" t="n"/>
       <c r="AJ3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 09 Oct 2026</t>
+          <t>YTD as of 12 Oct 2026</t>
         </is>
       </c>
       <c r="AK3" s="4" t="n"/>
@@ -1267,22 +1267,22 @@
         <v>1066081968.222222</v>
       </c>
       <c r="AG7" s="11" t="n">
-        <v>6390025148</v>
+        <v>13517220283</v>
       </c>
       <c r="AH7" s="11" t="n">
-        <v>375883.8322352941</v>
+        <v>795130.604882353</v>
       </c>
       <c r="AI7" s="11" t="n">
-        <v>33809656.86772487</v>
+        <v>71519684.03703703</v>
       </c>
       <c r="AJ7" s="11" t="n">
-        <v>207879517142</v>
+        <v>215006712277</v>
       </c>
       <c r="AK7" s="11" t="n">
-        <v>12228206.89070588</v>
+        <v>12647453.66335294</v>
       </c>
       <c r="AL7" s="11" t="n">
-        <v>1099891625.089947</v>
+        <v>1137601652.259259</v>
       </c>
     </row>
     <row r="8">
@@ -1367,225 +1367,225 @@
     <row r="9">
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">        PT Corteva Agriscience Seeds Indonesia</t>
+          <t xml:space="preserve">        PT Syngenta Seed Indonesia</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>14774062032</v>
+        <v>4917371048</v>
       </c>
       <c r="D9" s="11" t="n">
-        <v>869062.4724705883</v>
+        <v>289257.1204705882</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>78169640.38095239</v>
-      </c>
-      <c r="F9" s="11" t="n"/>
-      <c r="G9" s="11" t="n"/>
-      <c r="H9" s="11" t="n"/>
+        <v>26017836.23280423</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>377499498</v>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>22205.85282352941</v>
+      </c>
+      <c r="H9" s="11" t="n">
+        <v>1997351.841269841</v>
+      </c>
       <c r="I9" s="11" t="n">
-        <v>3060445998</v>
+        <v>5249034721</v>
       </c>
       <c r="J9" s="11" t="n">
-        <v>180026.2351764706</v>
+        <v>308766.7482941176</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>16192835.96825397</v>
+        <v>27772670.48148148</v>
       </c>
       <c r="L9" s="11" t="n">
-        <v>2647239849</v>
+        <v>5409395616</v>
       </c>
       <c r="M9" s="11" t="n">
-        <v>155719.9911176471</v>
+        <v>318199.7421176471</v>
       </c>
       <c r="N9" s="11" t="n">
-        <v>14006560.04761905</v>
+        <v>28621140.82539682</v>
       </c>
       <c r="O9" s="11" t="n">
-        <v>4342041733</v>
+        <v>7986730445</v>
       </c>
       <c r="P9" s="11" t="n">
-        <v>255414.2195882353</v>
+        <v>469807.6732352941</v>
       </c>
       <c r="Q9" s="11" t="n">
-        <v>22973765.78306878</v>
+        <v>42257833.04232804</v>
       </c>
       <c r="R9" s="11" t="n">
-        <v>2142139150</v>
+        <v>5293583677</v>
       </c>
       <c r="S9" s="11" t="n">
-        <v>126008.1852941176</v>
+        <v>311387.2751176471</v>
       </c>
       <c r="T9" s="11" t="n">
-        <v>11334069.57671958</v>
+        <v>28008379.24338624</v>
       </c>
       <c r="U9" s="11" t="n">
-        <v>4939206340</v>
+        <v>3590241514</v>
       </c>
       <c r="V9" s="11" t="n">
-        <v>290541.5494117647</v>
+        <v>211190.6772941177</v>
       </c>
       <c r="W9" s="11" t="n">
-        <v>26133366.87830688</v>
+        <v>18995986.84656085</v>
       </c>
       <c r="X9" s="11" t="n">
-        <v>2738261610</v>
+        <v>4753076386</v>
       </c>
       <c r="Y9" s="11" t="n">
-        <v>161074.2123529412</v>
+        <v>279592.7285882353</v>
       </c>
       <c r="Z9" s="11" t="n">
-        <v>14488156.66666667</v>
+        <v>25148552.30687831</v>
       </c>
       <c r="AA9" s="11" t="n">
-        <v>18886221373</v>
+        <v>7099446001</v>
       </c>
       <c r="AB9" s="11" t="n">
-        <v>1110954.198411765</v>
+        <v>417614.4706470588</v>
       </c>
       <c r="AC9" s="11" t="n">
-        <v>99927097.21164021</v>
+        <v>37563206.35449736</v>
       </c>
       <c r="AD9" s="11" t="n">
-        <v>53529618085</v>
+        <v>44676378906</v>
       </c>
       <c r="AE9" s="11" t="n">
-        <v>3148801.06382353</v>
+        <v>2628022.288588235</v>
       </c>
       <c r="AF9" s="11" t="n">
-        <v>283225492.5132275</v>
+        <v>236382957.1746032</v>
       </c>
       <c r="AG9" s="11" t="n">
-        <v>1739093256</v>
+        <v>11727333027</v>
       </c>
       <c r="AH9" s="11" t="n">
-        <v>102299.6032941177</v>
+        <v>689843.1192352942</v>
       </c>
       <c r="AI9" s="11" t="n">
-        <v>9201551.619047619</v>
+        <v>62049381.0952381</v>
       </c>
       <c r="AJ9" s="11" t="n">
-        <v>55268711341</v>
+        <v>56403711933</v>
       </c>
       <c r="AK9" s="11" t="n">
-        <v>3251100.667117647</v>
+        <v>3317865.407823529</v>
       </c>
       <c r="AL9" s="11" t="n">
-        <v>292427044.1322751</v>
+        <v>298432338.2698413</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">        PT Syngenta Seed Indonesia</t>
+          <t xml:space="preserve">        PT Corteva Agriscience Seeds Indonesia</t>
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>4917371048</v>
+        <v>14774062032</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>289257.1204705882</v>
+        <v>869062.4724705883</v>
       </c>
       <c r="E10" s="13" t="n">
-        <v>26017836.23280423</v>
-      </c>
-      <c r="F10" s="13" t="n">
-        <v>377499498</v>
-      </c>
-      <c r="G10" s="13" t="n">
-        <v>22205.85282352941</v>
-      </c>
-      <c r="H10" s="13" t="n">
-        <v>1997351.841269841</v>
-      </c>
+        <v>78169640.38095239</v>
+      </c>
+      <c r="F10" s="13" t="n"/>
+      <c r="G10" s="13" t="n"/>
+      <c r="H10" s="13" t="n"/>
       <c r="I10" s="13" t="n">
-        <v>5249034721</v>
+        <v>3060445998</v>
       </c>
       <c r="J10" s="13" t="n">
-        <v>308766.7482941176</v>
+        <v>180026.2351764706</v>
       </c>
       <c r="K10" s="13" t="n">
-        <v>27772670.48148148</v>
+        <v>16192835.96825397</v>
       </c>
       <c r="L10" s="13" t="n">
-        <v>5409395616</v>
+        <v>2647239849</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>318199.7421176471</v>
+        <v>155719.9911176471</v>
       </c>
       <c r="N10" s="13" t="n">
-        <v>28621140.82539682</v>
+        <v>14006560.04761905</v>
       </c>
       <c r="O10" s="13" t="n">
-        <v>7986730445</v>
+        <v>4342041733</v>
       </c>
       <c r="P10" s="13" t="n">
-        <v>469807.6732352941</v>
+        <v>255414.2195882353</v>
       </c>
       <c r="Q10" s="13" t="n">
-        <v>42257833.04232804</v>
+        <v>22973765.78306878</v>
       </c>
       <c r="R10" s="13" t="n">
-        <v>5293583677</v>
+        <v>2142139150</v>
       </c>
       <c r="S10" s="13" t="n">
-        <v>311387.2751176471</v>
+        <v>126008.1852941176</v>
       </c>
       <c r="T10" s="13" t="n">
-        <v>28008379.24338624</v>
+        <v>11334069.57671958</v>
       </c>
       <c r="U10" s="13" t="n">
-        <v>3590241514</v>
+        <v>4939206340</v>
       </c>
       <c r="V10" s="13" t="n">
-        <v>211190.6772941177</v>
+        <v>290541.5494117647</v>
       </c>
       <c r="W10" s="13" t="n">
-        <v>18995986.84656085</v>
+        <v>26133366.87830688</v>
       </c>
       <c r="X10" s="13" t="n">
-        <v>4753076386</v>
+        <v>2738261610</v>
       </c>
       <c r="Y10" s="13" t="n">
-        <v>279592.7285882353</v>
+        <v>161074.2123529412</v>
       </c>
       <c r="Z10" s="13" t="n">
-        <v>25148552.30687831</v>
+        <v>14488156.66666667</v>
       </c>
       <c r="AA10" s="13" t="n">
-        <v>7099446001</v>
+        <v>18886221373</v>
       </c>
       <c r="AB10" s="13" t="n">
-        <v>417614.4706470588</v>
+        <v>1110954.198411765</v>
       </c>
       <c r="AC10" s="13" t="n">
-        <v>37563206.35449736</v>
+        <v>99927097.21164021</v>
       </c>
       <c r="AD10" s="13" t="n">
-        <v>44676378906</v>
+        <v>53529618085</v>
       </c>
       <c r="AE10" s="13" t="n">
-        <v>2628022.288588235</v>
+        <v>3148801.06382353</v>
       </c>
       <c r="AF10" s="13" t="n">
-        <v>236382957.1746032</v>
+        <v>283225492.5132275</v>
       </c>
       <c r="AG10" s="13" t="n">
-        <v>4600137892</v>
+        <v>1739093256</v>
       </c>
       <c r="AH10" s="13" t="n">
-        <v>270596.3465882353</v>
+        <v>102299.6032941177</v>
       </c>
       <c r="AI10" s="13" t="n">
-        <v>24339353.92592593</v>
+        <v>9201551.619047619</v>
       </c>
       <c r="AJ10" s="13" t="n">
-        <v>49276516798</v>
+        <v>55268711341</v>
       </c>
       <c r="AK10" s="13" t="n">
-        <v>2898618.635176471</v>
+        <v>3251100.667117647</v>
       </c>
       <c r="AL10" s="13" t="n">
-        <v>260722311.1005291</v>
+        <v>292427044.1322751</v>
       </c>
     </row>
     <row r="11">
@@ -2330,22 +2330,22 @@
         <v>2521134.965502645</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>6304000</v>
+        <v>9044500</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>370.8235294117647</v>
+        <v>532.0294117647059</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>33354.49735449735</v>
+        <v>47854.49735449735</v>
       </c>
       <c r="AJ20" s="13" t="n">
-        <v>482798508.48</v>
+        <v>485539008.48</v>
       </c>
       <c r="AK20" s="13" t="n">
-        <v>28399.91226352942</v>
+        <v>28561.11814588236</v>
       </c>
       <c r="AL20" s="13" t="n">
-        <v>2554489.462857143</v>
+        <v>2568989.462857143</v>
       </c>
     </row>
     <row r="21">
@@ -2603,22 +2603,22 @@
         <v>491976.1904761905</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>5304000</v>
+        <v>8044500</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>312</v>
+        <v>473.2058823529412</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>28063.49206349206</v>
+        <v>42563.49206349206</v>
       </c>
       <c r="AJ23" s="11" t="n">
-        <v>98287500</v>
+        <v>101028000</v>
       </c>
       <c r="AK23" s="11" t="n">
-        <v>5781.617647058823</v>
+        <v>5942.823529411765</v>
       </c>
       <c r="AL23" s="11" t="n">
-        <v>520039.6825396825</v>
+        <v>534539.6825396825</v>
       </c>
     </row>
     <row r="24">
@@ -4149,22 +4149,22 @@
         <v>1332179822.764445</v>
       </c>
       <c r="AG45" s="15" t="n">
-        <v>6396329148</v>
+        <v>13526264783</v>
       </c>
       <c r="AH45" s="15" t="n">
-        <v>376254.6557647059</v>
+        <v>795662.6342941177</v>
       </c>
       <c r="AI45" s="15" t="n">
-        <v>33843011.36507937</v>
+        <v>71567538.53439154</v>
       </c>
       <c r="AJ45" s="15" t="n">
-        <v>258178315650.48</v>
+        <v>265308251285.48</v>
       </c>
       <c r="AK45" s="15" t="n">
-        <v>15186959.74414588</v>
+        <v>15606367.72267529</v>
       </c>
       <c r="AL45" s="15" t="n">
-        <v>1366022834.129524</v>
+        <v>1403747361.298836</v>
       </c>
     </row>
     <row r="46">
@@ -13406,17 +13406,23 @@
       <c r="AF153" s="11" t="n">
         <v>-23408114.45502646</v>
       </c>
-      <c r="AG153" s="11" t="n"/>
-      <c r="AH153" s="11" t="n"/>
-      <c r="AI153" s="11" t="n"/>
+      <c r="AG153" s="11" t="n">
+        <v>-176228276</v>
+      </c>
+      <c r="AH153" s="11" t="n">
+        <v>-10366.36917647059</v>
+      </c>
+      <c r="AI153" s="11" t="n">
+        <v>-932424.7407407408</v>
+      </c>
       <c r="AJ153" s="11" t="n">
-        <v>-4424133632</v>
+        <v>-4600361908</v>
       </c>
       <c r="AK153" s="11" t="n">
-        <v>-260243.1548235294</v>
+        <v>-270609.524</v>
       </c>
       <c r="AL153" s="11" t="n">
-        <v>-23408114.45502646</v>
+        <v>-24340539.1957672</v>
       </c>
     </row>
     <row r="154">
@@ -13674,22 +13680,22 @@
         <v>-33089923.13634921</v>
       </c>
       <c r="AG156" s="15" t="n">
-        <v>-24700</v>
+        <v>-176252976</v>
       </c>
       <c r="AH156" s="15" t="n">
-        <v>-1.452941176470588</v>
+        <v>-10367.82211764706</v>
       </c>
       <c r="AI156" s="15" t="n">
-        <v>-130.6878306878307</v>
+        <v>-932555.4285714285</v>
       </c>
       <c r="AJ156" s="15" t="n">
-        <v>-6254020172.77</v>
+        <v>-6430248448.77</v>
       </c>
       <c r="AK156" s="15" t="n">
-        <v>-367883.5395747059</v>
+        <v>-378249.9087511765</v>
       </c>
       <c r="AL156" s="15" t="n">
-        <v>-33090053.8241799</v>
+        <v>-34022478.56492063</v>
       </c>
     </row>
     <row r="157">
@@ -13789,22 +13795,22 @@
         <v>-1609397741.344392</v>
       </c>
       <c r="AG157" s="19" t="n">
-        <v>-4395763873</v>
+        <v>-4571992149</v>
       </c>
       <c r="AH157" s="19" t="n">
-        <v>-258574.3454705882</v>
+        <v>-268940.7146470588</v>
       </c>
       <c r="AI157" s="19" t="n">
-        <v>-23258009.91005291</v>
+        <v>-24190434.65079365</v>
       </c>
       <c r="AJ157" s="19" t="n">
-        <v>-308571936987.09</v>
+        <v>-308748165263.09</v>
       </c>
       <c r="AK157" s="19" t="n">
-        <v>-18151290.41100529</v>
+        <v>-18161656.78018176</v>
       </c>
       <c r="AL157" s="19" t="n">
-        <v>-1632655751.254445</v>
+        <v>-1633588175.995185</v>
       </c>
     </row>
     <row r="158">
@@ -13904,22 +13910,22 @@
         <v>-277217918.5799472</v>
       </c>
       <c r="AG158" s="19" t="n">
-        <v>2000565275</v>
+        <v>8954272634</v>
       </c>
       <c r="AH158" s="19" t="n">
-        <v>117680.3102941176</v>
+        <v>526721.9196470588</v>
       </c>
       <c r="AI158" s="19" t="n">
-        <v>10585001.45502646</v>
+        <v>47377103.88359788</v>
       </c>
       <c r="AJ158" s="19" t="n">
-        <v>-50393621336.61</v>
+        <v>-43439913977.61</v>
       </c>
       <c r="AK158" s="19" t="n">
-        <v>-2964330.666859413</v>
+        <v>-2555289.057506471</v>
       </c>
       <c r="AL158" s="19" t="n">
-        <v>-266632917.1249208</v>
+        <v>-229840814.6963494</v>
       </c>
     </row>
     <row r="159">
@@ -14019,22 +14025,22 @@
         <v>79785577.85582009</v>
       </c>
       <c r="AG159" s="7" t="n">
-        <v>17080039489.75</v>
+        <v>24033746848.75</v>
       </c>
       <c r="AH159" s="7" t="n">
-        <v>1004708.205279412</v>
+        <v>1413749.814632353</v>
       </c>
       <c r="AI159" s="7" t="n">
-        <v>90370579.31084657</v>
+        <v>127162681.739418</v>
       </c>
       <c r="AJ159" s="7" t="n">
-        <v>17080039489.75</v>
+        <v>24033746848.75</v>
       </c>
       <c r="AK159" s="7" t="n">
-        <v>1004708.205279412</v>
+        <v>1413749.814632353</v>
       </c>
       <c r="AL159" s="7" t="n">
-        <v>90370579.31084657</v>
+        <v>127162681.739418</v>
       </c>
     </row>
   </sheetData>
@@ -14837,16 +14843,16 @@
         <v>14828882907</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>421365900</v>
+        <v>7548561035</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>15250248807</v>
+        <v>22377443942</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>897073.4592352941</v>
+        <v>1316320.231882353</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>80689147.12698413</v>
+        <v>118399174.2962963</v>
       </c>
     </row>
     <row r="7">
@@ -14869,16 +14875,16 @@
         <v>18099375</v>
       </c>
       <c r="E7" s="13" t="n">
-        <v>200000000</v>
+        <v>23771724</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>218099375</v>
+        <v>41871099</v>
       </c>
       <c r="G7" s="24" t="n">
-        <v>12829.375</v>
+        <v>2463.005823529412</v>
       </c>
       <c r="H7" s="24" t="n">
-        <v>1153964.947089947</v>
+        <v>221540.2063492064</v>
       </c>
     </row>
     <row r="8">
@@ -14933,16 +14939,16 @@
         <v>22400563.84000001</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>55070136</v>
+        <v>57810636</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>77470699.84</v>
+        <v>80211199.84</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>4557.099990588235</v>
+        <v>4718.305872941177</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>409897.8827513228</v>
+        <v>424397.8827513228</v>
       </c>
     </row>
     <row r="10">
@@ -15052,13 +15058,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>15755935252.75</v>
+        <v>22709642611.75</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>926819.7207499999</v>
+        <v>1335861.330102941</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>83364736.78703703</v>
+        <v>120156839.2156085</v>
       </c>
     </row>
   </sheetData>
@@ -15131,7 +15137,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 09 Oct 2026 16:19 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 12 Oct 2026 11:57 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -15213,14 +15219,14 @@
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 09 Oct 2026</t>
+          <t>MTD as of 12 Oct 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
       <c r="AI3" s="4" t="n"/>
       <c r="AJ3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 09 Oct 2026</t>
+          <t>YTD as of 12 Oct 2026</t>
         </is>
       </c>
       <c r="AK3" s="4" t="n"/>
@@ -15664,22 +15670,22 @@
         <v>1066.081968222222</v>
       </c>
       <c r="AG7" s="11" t="n">
-        <v>6390.025148</v>
+        <v>13517.220283</v>
       </c>
       <c r="AH7" s="11" t="n">
-        <v>0.3758838322352941</v>
+        <v>0.795130604882353</v>
       </c>
       <c r="AI7" s="11" t="n">
-        <v>33.80965686772487</v>
+        <v>71.51968403703704</v>
       </c>
       <c r="AJ7" s="11" t="n">
-        <v>207879.517142</v>
+        <v>215006.712277</v>
       </c>
       <c r="AK7" s="11" t="n">
-        <v>12.22820689070588</v>
+        <v>12.64745366335294</v>
       </c>
       <c r="AL7" s="11" t="n">
-        <v>1099.891625089947</v>
+        <v>1137.601652259259</v>
       </c>
     </row>
     <row r="8">
@@ -15764,225 +15770,225 @@
     <row r="9">
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">        PT Corteva Agriscience Seeds Indonesia</t>
+          <t xml:space="preserve">        PT Syngenta Seed Indonesia</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>14774.062032</v>
+        <v>4917.371048</v>
       </c>
       <c r="D9" s="11" t="n">
-        <v>0.8690624724705882</v>
+        <v>0.2892571204705882</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>78.16964038095237</v>
-      </c>
-      <c r="F9" s="11" t="n"/>
-      <c r="G9" s="11" t="n"/>
-      <c r="H9" s="11" t="n"/>
+        <v>26.01783623280423</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>377.499498</v>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>0.02220585282352941</v>
+      </c>
+      <c r="H9" s="11" t="n">
+        <v>1.997351841269841</v>
+      </c>
       <c r="I9" s="11" t="n">
-        <v>3060.445998</v>
+        <v>5249.034721</v>
       </c>
       <c r="J9" s="11" t="n">
-        <v>0.1800262351764706</v>
+        <v>0.3087667482941177</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>16.19283596825397</v>
+        <v>27.77267048148148</v>
       </c>
       <c r="L9" s="11" t="n">
-        <v>2647.239849</v>
+        <v>5409.395616</v>
       </c>
       <c r="M9" s="11" t="n">
-        <v>0.1557199911176471</v>
+        <v>0.3181997421176471</v>
       </c>
       <c r="N9" s="11" t="n">
-        <v>14.00656004761905</v>
+        <v>28.62114082539683</v>
       </c>
       <c r="O9" s="11" t="n">
-        <v>4342.041733</v>
+        <v>7986.730445</v>
       </c>
       <c r="P9" s="11" t="n">
-        <v>0.2554142195882353</v>
+        <v>0.4698076732352941</v>
       </c>
       <c r="Q9" s="11" t="n">
-        <v>22.97376578306878</v>
+        <v>42.25783304232804</v>
       </c>
       <c r="R9" s="11" t="n">
-        <v>2142.13915</v>
+        <v>5293.583677</v>
       </c>
       <c r="S9" s="11" t="n">
-        <v>0.1260081852941176</v>
+        <v>0.311387275117647</v>
       </c>
       <c r="T9" s="11" t="n">
-        <v>11.33406957671958</v>
+        <v>28.00837924338624</v>
       </c>
       <c r="U9" s="11" t="n">
-        <v>4939.20634</v>
+        <v>3590.241514</v>
       </c>
       <c r="V9" s="11" t="n">
-        <v>0.2905415494117647</v>
+        <v>0.2111906772941176</v>
       </c>
       <c r="W9" s="11" t="n">
-        <v>26.13336687830688</v>
+        <v>18.99598684656085</v>
       </c>
       <c r="X9" s="11" t="n">
-        <v>2738.26161</v>
+        <v>4753.076386</v>
       </c>
       <c r="Y9" s="11" t="n">
-        <v>0.1610742123529412</v>
+        <v>0.2795927285882353</v>
       </c>
       <c r="Z9" s="11" t="n">
-        <v>14.48815666666667</v>
+        <v>25.1485523068783</v>
       </c>
       <c r="AA9" s="11" t="n">
-        <v>18886.221373</v>
+        <v>7099.446001</v>
       </c>
       <c r="AB9" s="11" t="n">
-        <v>1.110954198411765</v>
+        <v>0.4176144706470588</v>
       </c>
       <c r="AC9" s="11" t="n">
-        <v>99.92709721164022</v>
+        <v>37.56320635449735</v>
       </c>
       <c r="AD9" s="11" t="n">
-        <v>53529.618085</v>
+        <v>44676.378906</v>
       </c>
       <c r="AE9" s="11" t="n">
-        <v>3.148801063823529</v>
+        <v>2.628022288588235</v>
       </c>
       <c r="AF9" s="11" t="n">
-        <v>283.2254925132275</v>
+        <v>236.3829571746032</v>
       </c>
       <c r="AG9" s="11" t="n">
-        <v>1739.093256</v>
+        <v>11727.333027</v>
       </c>
       <c r="AH9" s="11" t="n">
-        <v>0.1022996032941176</v>
+        <v>0.6898431192352942</v>
       </c>
       <c r="AI9" s="11" t="n">
-        <v>9.201551619047619</v>
+        <v>62.0493810952381</v>
       </c>
       <c r="AJ9" s="11" t="n">
-        <v>55268.711341</v>
+        <v>56403.711933</v>
       </c>
       <c r="AK9" s="11" t="n">
-        <v>3.251100667117647</v>
+        <v>3.317865407823529</v>
       </c>
       <c r="AL9" s="11" t="n">
-        <v>292.4270441322751</v>
+        <v>298.4323382698413</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">        PT Syngenta Seed Indonesia</t>
+          <t xml:space="preserve">        PT Corteva Agriscience Seeds Indonesia</t>
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>4917.371048</v>
+        <v>14774.062032</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>0.2892571204705882</v>
+        <v>0.8690624724705882</v>
       </c>
       <c r="E10" s="13" t="n">
-        <v>26.01783623280423</v>
-      </c>
-      <c r="F10" s="13" t="n">
-        <v>377.499498</v>
-      </c>
-      <c r="G10" s="13" t="n">
-        <v>0.02220585282352941</v>
-      </c>
-      <c r="H10" s="13" t="n">
-        <v>1.997351841269841</v>
-      </c>
+        <v>78.16964038095237</v>
+      </c>
+      <c r="F10" s="13" t="n"/>
+      <c r="G10" s="13" t="n"/>
+      <c r="H10" s="13" t="n"/>
       <c r="I10" s="13" t="n">
-        <v>5249.034721</v>
+        <v>3060.445998</v>
       </c>
       <c r="J10" s="13" t="n">
-        <v>0.3087667482941177</v>
+        <v>0.1800262351764706</v>
       </c>
       <c r="K10" s="13" t="n">
-        <v>27.77267048148148</v>
+        <v>16.19283596825397</v>
       </c>
       <c r="L10" s="13" t="n">
-        <v>5409.395616</v>
+        <v>2647.239849</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>0.3181997421176471</v>
+        <v>0.1557199911176471</v>
       </c>
       <c r="N10" s="13" t="n">
-        <v>28.62114082539683</v>
+        <v>14.00656004761905</v>
       </c>
       <c r="O10" s="13" t="n">
-        <v>7986.730445</v>
+        <v>4342.041733</v>
       </c>
       <c r="P10" s="13" t="n">
-        <v>0.4698076732352941</v>
+        <v>0.2554142195882353</v>
       </c>
       <c r="Q10" s="13" t="n">
-        <v>42.25783304232804</v>
+        <v>22.97376578306878</v>
       </c>
       <c r="R10" s="13" t="n">
-        <v>5293.583677</v>
+        <v>2142.13915</v>
       </c>
       <c r="S10" s="13" t="n">
-        <v>0.311387275117647</v>
+        <v>0.1260081852941176</v>
       </c>
       <c r="T10" s="13" t="n">
-        <v>28.00837924338624</v>
+        <v>11.33406957671958</v>
       </c>
       <c r="U10" s="13" t="n">
-        <v>3590.241514</v>
+        <v>4939.20634</v>
       </c>
       <c r="V10" s="13" t="n">
-        <v>0.2111906772941176</v>
+        <v>0.2905415494117647</v>
       </c>
       <c r="W10" s="13" t="n">
-        <v>18.99598684656085</v>
+        <v>26.13336687830688</v>
       </c>
       <c r="X10" s="13" t="n">
-        <v>4753.076386</v>
+        <v>2738.26161</v>
       </c>
       <c r="Y10" s="13" t="n">
-        <v>0.2795927285882353</v>
+        <v>0.1610742123529412</v>
       </c>
       <c r="Z10" s="13" t="n">
-        <v>25.1485523068783</v>
+        <v>14.48815666666667</v>
       </c>
       <c r="AA10" s="13" t="n">
-        <v>7099.446001</v>
+        <v>18886.221373</v>
       </c>
       <c r="AB10" s="13" t="n">
-        <v>0.4176144706470588</v>
+        <v>1.110954198411765</v>
       </c>
       <c r="AC10" s="13" t="n">
-        <v>37.56320635449735</v>
+        <v>99.92709721164022</v>
       </c>
       <c r="AD10" s="13" t="n">
-        <v>44676.378906</v>
+        <v>53529.618085</v>
       </c>
       <c r="AE10" s="13" t="n">
-        <v>2.628022288588235</v>
+        <v>3.148801063823529</v>
       </c>
       <c r="AF10" s="13" t="n">
-        <v>236.3829571746032</v>
+        <v>283.2254925132275</v>
       </c>
       <c r="AG10" s="13" t="n">
-        <v>4600.137892</v>
+        <v>1739.093256</v>
       </c>
       <c r="AH10" s="13" t="n">
-        <v>0.2705963465882353</v>
+        <v>0.1022996032941176</v>
       </c>
       <c r="AI10" s="13" t="n">
-        <v>24.33935392592592</v>
+        <v>9.201551619047619</v>
       </c>
       <c r="AJ10" s="13" t="n">
-        <v>49276.516798</v>
+        <v>55268.711341</v>
       </c>
       <c r="AK10" s="13" t="n">
-        <v>2.89861863517647</v>
+        <v>3.251100667117647</v>
       </c>
       <c r="AL10" s="13" t="n">
-        <v>260.7223111005291</v>
+        <v>292.4270441322751</v>
       </c>
     </row>
     <row r="11">
@@ -16727,22 +16733,22 @@
         <v>2.521134965502646</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>6.304</v>
+        <v>9.044499999999999</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>0.0003708235294117647</v>
+        <v>0.0005320294117647058</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>0.03335449735449736</v>
+        <v>0.04785449735449735</v>
       </c>
       <c r="AJ20" s="13" t="n">
-        <v>482.79850848</v>
+        <v>485.53900848</v>
       </c>
       <c r="AK20" s="13" t="n">
-        <v>0.02839991226352941</v>
+        <v>0.02856111814588235</v>
       </c>
       <c r="AL20" s="13" t="n">
-        <v>2.554489462857143</v>
+        <v>2.568989462857143</v>
       </c>
     </row>
     <row r="21">
@@ -17000,22 +17006,22 @@
         <v>0.4919761904761905</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>5.304</v>
+        <v>8.044499999999999</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>0.000312</v>
+        <v>0.0004732058823529411</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>0.02806349206349206</v>
+        <v>0.04256349206349206</v>
       </c>
       <c r="AJ23" s="11" t="n">
-        <v>98.28750000000001</v>
+        <v>101.028</v>
       </c>
       <c r="AK23" s="11" t="n">
-        <v>0.005781617647058824</v>
+        <v>0.005942823529411766</v>
       </c>
       <c r="AL23" s="11" t="n">
-        <v>0.5200396825396825</v>
+        <v>0.5345396825396825</v>
       </c>
     </row>
     <row r="24">
@@ -18546,22 +18552,22 @@
         <v>1332.179822764444</v>
       </c>
       <c r="AG45" s="15" t="n">
-        <v>6396.329148</v>
+        <v>13526.264783</v>
       </c>
       <c r="AH45" s="15" t="n">
-        <v>0.3762546557647058</v>
+        <v>0.7956626342941177</v>
       </c>
       <c r="AI45" s="15" t="n">
-        <v>33.84301136507936</v>
+        <v>71.56753853439153</v>
       </c>
       <c r="AJ45" s="15" t="n">
-        <v>258178.31565048</v>
+        <v>265308.25128548</v>
       </c>
       <c r="AK45" s="15" t="n">
-        <v>15.18695974414588</v>
+        <v>15.60636772267529</v>
       </c>
       <c r="AL45" s="15" t="n">
-        <v>1366.022834129524</v>
+        <v>1403.747361298836</v>
       </c>
     </row>
     <row r="46">
@@ -27803,17 +27809,23 @@
       <c r="AF153" s="11" t="n">
         <v>-23.40811445502645</v>
       </c>
-      <c r="AG153" s="11" t="n"/>
-      <c r="AH153" s="11" t="n"/>
-      <c r="AI153" s="11" t="n"/>
+      <c r="AG153" s="11" t="n">
+        <v>-176.228276</v>
+      </c>
+      <c r="AH153" s="11" t="n">
+        <v>-0.01036636917647059</v>
+      </c>
+      <c r="AI153" s="11" t="n">
+        <v>-0.9324247407407407</v>
+      </c>
       <c r="AJ153" s="11" t="n">
-        <v>-4424.133632</v>
+        <v>-4600.361908</v>
       </c>
       <c r="AK153" s="11" t="n">
-        <v>-0.2602431548235294</v>
+        <v>-0.270609524</v>
       </c>
       <c r="AL153" s="11" t="n">
-        <v>-23.40811445502645</v>
+        <v>-24.34053919576719</v>
       </c>
     </row>
     <row r="154">
@@ -28071,22 +28083,22 @@
         <v>-33.08992313634921</v>
       </c>
       <c r="AG156" s="15" t="n">
-        <v>-0.0247</v>
+        <v>-176.252976</v>
       </c>
       <c r="AH156" s="15" t="n">
-        <v>-1.452941176470588e-06</v>
+        <v>-0.01036782211764706</v>
       </c>
       <c r="AI156" s="15" t="n">
-        <v>-0.0001306878306878307</v>
+        <v>-0.9325554285714285</v>
       </c>
       <c r="AJ156" s="15" t="n">
-        <v>-6254.02017277</v>
+        <v>-6430.248448769999</v>
       </c>
       <c r="AK156" s="15" t="n">
-        <v>-0.3678835395747059</v>
+        <v>-0.3782499087511765</v>
       </c>
       <c r="AL156" s="15" t="n">
-        <v>-33.0900538241799</v>
+        <v>-34.02247856492063</v>
       </c>
     </row>
     <row r="157">
@@ -28186,22 +28198,22 @@
         <v>-1609.397741344392</v>
       </c>
       <c r="AG157" s="19" t="n">
-        <v>-4395.763873</v>
+        <v>-4571.992149</v>
       </c>
       <c r="AH157" s="19" t="n">
-        <v>-0.2585743454705882</v>
+        <v>-0.2689407146470588</v>
       </c>
       <c r="AI157" s="19" t="n">
-        <v>-23.25800991005291</v>
+        <v>-24.19043465079365</v>
       </c>
       <c r="AJ157" s="19" t="n">
-        <v>-308571.9369870899</v>
+        <v>-308748.1652630899</v>
       </c>
       <c r="AK157" s="19" t="n">
-        <v>-18.1512904110053</v>
+        <v>-18.16165678018177</v>
       </c>
       <c r="AL157" s="19" t="n">
-        <v>-1632.655751254444</v>
+        <v>-1633.588175995185</v>
       </c>
     </row>
     <row r="158">
@@ -28301,22 +28313,22 @@
         <v>-277.2179185799473</v>
       </c>
       <c r="AG158" s="19" t="n">
-        <v>2000.565275</v>
+        <v>8954.272634000001</v>
       </c>
       <c r="AH158" s="19" t="n">
-        <v>0.1176803102941176</v>
+        <v>0.5267219196470588</v>
       </c>
       <c r="AI158" s="19" t="n">
-        <v>10.58500145502645</v>
+        <v>47.37710388359789</v>
       </c>
       <c r="AJ158" s="19" t="n">
-        <v>-50393.62133661</v>
+        <v>-43439.91397761</v>
       </c>
       <c r="AK158" s="19" t="n">
-        <v>-2.964330666859413</v>
+        <v>-2.555289057506472</v>
       </c>
       <c r="AL158" s="19" t="n">
-        <v>-266.6329171249208</v>
+        <v>-229.8408146963494</v>
       </c>
     </row>
     <row r="159">
@@ -28416,22 +28428,22 @@
         <v>79.78557785582009</v>
       </c>
       <c r="AG159" s="7" t="n">
-        <v>17080.03948975</v>
+        <v>24033.74684875</v>
       </c>
       <c r="AH159" s="7" t="n">
-        <v>1.004708205279412</v>
+        <v>1.413749814632353</v>
       </c>
       <c r="AI159" s="7" t="n">
-        <v>90.37057931084657</v>
+        <v>127.162681739418</v>
       </c>
       <c r="AJ159" s="7" t="n">
-        <v>17080.03948975</v>
+        <v>24033.74684875</v>
       </c>
       <c r="AK159" s="7" t="n">
-        <v>1.004708205279412</v>
+        <v>1.413749814632353</v>
       </c>
       <c r="AL159" s="7" t="n">
-        <v>90.37057931084657</v>
+        <v>127.162681739418</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Mon 10/12/2026 13:51
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -734,7 +734,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 12 Oct 2026 11:57</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 12 Oct 2026 13:51</t>
         </is>
       </c>
     </row>
@@ -15137,7 +15137,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 12 Oct 2026 11:57 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 12 Oct 2026 13:51 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Mon 10/12/2026 17:09
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -734,7 +734,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 12 Oct 2026 13:51</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 12 Oct 2026 17:09</t>
         </is>
       </c>
     </row>
@@ -8288,22 +8288,22 @@
         <v>-1418156.079365079</v>
       </c>
       <c r="AG98" s="11" t="n">
-        <v>-12640200</v>
+        <v>-112897000</v>
       </c>
       <c r="AH98" s="11" t="n">
-        <v>-743.5411764705882</v>
+        <v>-6641</v>
       </c>
       <c r="AI98" s="11" t="n">
-        <v>-66879.36507936507</v>
+        <v>-597338.6243386243</v>
       </c>
       <c r="AJ98" s="11" t="n">
-        <v>-280671699</v>
+        <v>-380928499</v>
       </c>
       <c r="AK98" s="11" t="n">
-        <v>-16510.09994117647</v>
+        <v>-22407.55876470588</v>
       </c>
       <c r="AL98" s="11" t="n">
-        <v>-1485035.444444444</v>
+        <v>-2015494.703703704</v>
       </c>
     </row>
     <row r="99">
@@ -8748,22 +8748,22 @@
         <v>-46203532.51708995</v>
       </c>
       <c r="AG102" s="15" t="n">
-        <v>-177119294</v>
+        <v>-277376094</v>
       </c>
       <c r="AH102" s="15" t="n">
-        <v>-10418.782</v>
+        <v>-16316.24082352941</v>
       </c>
       <c r="AI102" s="15" t="n">
-        <v>-937139.1216931217</v>
+        <v>-1467598.380952381</v>
       </c>
       <c r="AJ102" s="15" t="n">
-        <v>-8909586939.73</v>
+        <v>-9009843739.73</v>
       </c>
       <c r="AK102" s="15" t="n">
-        <v>-524093.3493958823</v>
+        <v>-529990.8082194118</v>
       </c>
       <c r="AL102" s="15" t="n">
-        <v>-47140671.63878307</v>
+        <v>-47671130.89804233</v>
       </c>
     </row>
     <row r="103">
@@ -12399,22 +12399,22 @@
         <v>-253738061.1596296</v>
       </c>
       <c r="AG141" s="15" t="n">
-        <v>-831870274</v>
+        <v>-932127074</v>
       </c>
       <c r="AH141" s="15" t="n">
-        <v>-48933.54552941176</v>
+        <v>-54831.00435294118</v>
       </c>
       <c r="AI141" s="15" t="n">
-        <v>-4401430.021164021</v>
+        <v>-4931889.280423281</v>
       </c>
       <c r="AJ141" s="15" t="n">
-        <v>-48788363833.17</v>
+        <v>-48888620633.17</v>
       </c>
       <c r="AK141" s="15" t="n">
-        <v>-2869903.754892353</v>
+        <v>-2875801.213715882</v>
       </c>
       <c r="AL141" s="15" t="n">
-        <v>-258139491.1807937</v>
+        <v>-258669950.4400529</v>
       </c>
     </row>
     <row r="142">
@@ -13037,22 +13037,22 @@
         <v>-107075.0670899471</v>
       </c>
       <c r="AG149" s="11" t="n">
-        <v>-24700</v>
+        <v>-600042</v>
       </c>
       <c r="AH149" s="11" t="n">
-        <v>-1.452941176470588</v>
+        <v>-35.29658823529412</v>
       </c>
       <c r="AI149" s="11" t="n">
-        <v>-130.6878306878307</v>
+        <v>-3174.825396825397</v>
       </c>
       <c r="AJ149" s="11" t="n">
-        <v>-20261887.68</v>
+        <v>-20837229.68</v>
       </c>
       <c r="AK149" s="11" t="n">
-        <v>-1191.875745882353</v>
+        <v>-1225.719392941176</v>
       </c>
       <c r="AL149" s="11" t="n">
-        <v>-107205.7549206349</v>
+        <v>-110249.8924867725</v>
       </c>
     </row>
     <row r="150">
@@ -13680,22 +13680,22 @@
         <v>-33089923.13634921</v>
       </c>
       <c r="AG156" s="15" t="n">
-        <v>-176252976</v>
+        <v>-176828318</v>
       </c>
       <c r="AH156" s="15" t="n">
-        <v>-10367.82211764706</v>
+        <v>-10401.66576470588</v>
       </c>
       <c r="AI156" s="15" t="n">
-        <v>-932555.4285714285</v>
+        <v>-935599.5661375661</v>
       </c>
       <c r="AJ156" s="15" t="n">
-        <v>-6430248448.77</v>
+        <v>-6430823790.77</v>
       </c>
       <c r="AK156" s="15" t="n">
-        <v>-378249.9087511765</v>
+        <v>-378283.7523982353</v>
       </c>
       <c r="AL156" s="15" t="n">
-        <v>-34022478.56492063</v>
+        <v>-34025522.70248678</v>
       </c>
     </row>
     <row r="157">
@@ -13795,22 +13795,22 @@
         <v>-1609397741.344392</v>
       </c>
       <c r="AG157" s="19" t="n">
-        <v>-4571992149</v>
+        <v>-4672824291</v>
       </c>
       <c r="AH157" s="19" t="n">
-        <v>-268940.7146470588</v>
+        <v>-274872.017117647</v>
       </c>
       <c r="AI157" s="19" t="n">
-        <v>-24190434.65079365</v>
+        <v>-24723938.04761905</v>
       </c>
       <c r="AJ157" s="19" t="n">
-        <v>-308748165263.09</v>
+        <v>-308848997405.09</v>
       </c>
       <c r="AK157" s="19" t="n">
-        <v>-18161656.78018176</v>
+        <v>-18167588.08265235</v>
       </c>
       <c r="AL157" s="19" t="n">
-        <v>-1633588175.995185</v>
+        <v>-1634121679.392011</v>
       </c>
     </row>
     <row r="158">
@@ -13910,22 +13910,22 @@
         <v>-277217918.5799472</v>
       </c>
       <c r="AG158" s="19" t="n">
-        <v>8954272634</v>
+        <v>8853440492</v>
       </c>
       <c r="AH158" s="19" t="n">
-        <v>526721.9196470588</v>
+        <v>520790.6171764706</v>
       </c>
       <c r="AI158" s="19" t="n">
-        <v>47377103.88359788</v>
+        <v>46843600.48677249</v>
       </c>
       <c r="AJ158" s="19" t="n">
-        <v>-43439913977.61</v>
+        <v>-43540746119.61</v>
       </c>
       <c r="AK158" s="19" t="n">
-        <v>-2555289.057506471</v>
+        <v>-2561220.35997706</v>
       </c>
       <c r="AL158" s="19" t="n">
-        <v>-229840814.6963494</v>
+        <v>-230374318.0931748</v>
       </c>
     </row>
     <row r="159">
@@ -14025,22 +14025,22 @@
         <v>79785577.85582009</v>
       </c>
       <c r="AG159" s="7" t="n">
-        <v>24033746848.75</v>
+        <v>23932914706.75</v>
       </c>
       <c r="AH159" s="7" t="n">
-        <v>1413749.814632353</v>
+        <v>1407818.512161765</v>
       </c>
       <c r="AI159" s="7" t="n">
-        <v>127162681.739418</v>
+        <v>126629178.3425926</v>
       </c>
       <c r="AJ159" s="7" t="n">
-        <v>24033746848.75</v>
+        <v>23932914706.75</v>
       </c>
       <c r="AK159" s="7" t="n">
-        <v>1413749.814632353</v>
+        <v>1407818.512161765</v>
       </c>
       <c r="AL159" s="7" t="n">
-        <v>127162681.739418</v>
+        <v>126629178.3425926</v>
       </c>
     </row>
   </sheetData>
@@ -15003,16 +15003,16 @@
         <v>175445396.6500001</v>
       </c>
       <c r="E11" s="13" t="n">
-        <v>0</v>
+        <v>-100832142</v>
       </c>
       <c r="F11" s="13" t="n">
-        <v>175445396.6500001</v>
+        <v>74613254.65000007</v>
       </c>
       <c r="G11" s="24" t="n">
-        <v>10320.31745</v>
+        <v>4389.014979411769</v>
       </c>
       <c r="H11" s="24" t="n">
-        <v>928282.5219576723</v>
+        <v>394779.1251322755</v>
       </c>
     </row>
     <row r="12">
@@ -15058,13 +15058,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>22709642611.75</v>
+        <v>22608810469.75</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>1335861.330102941</v>
+        <v>1329930.027632353</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>120156839.2156085</v>
+        <v>119623335.8187831</v>
       </c>
     </row>
   </sheetData>
@@ -15137,7 +15137,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 12 Oct 2026 13:51 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 12 Oct 2026 17:09 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -22691,22 +22691,22 @@
         <v>-1.418156079365079</v>
       </c>
       <c r="AG98" s="11" t="n">
-        <v>-12.6402</v>
+        <v>-112.897</v>
       </c>
       <c r="AH98" s="11" t="n">
-        <v>-0.0007435411764705883</v>
+        <v>-0.006641</v>
       </c>
       <c r="AI98" s="11" t="n">
-        <v>-0.06687936507936508</v>
+        <v>-0.5973386243386244</v>
       </c>
       <c r="AJ98" s="11" t="n">
-        <v>-280.671699</v>
+        <v>-380.928499</v>
       </c>
       <c r="AK98" s="11" t="n">
-        <v>-0.01651009994117647</v>
+        <v>-0.02240755876470588</v>
       </c>
       <c r="AL98" s="11" t="n">
-        <v>-1.485035444444444</v>
+        <v>-2.015494703703704</v>
       </c>
     </row>
     <row r="99">
@@ -23151,22 +23151,22 @@
         <v>-46.20353251708994</v>
       </c>
       <c r="AG102" s="15" t="n">
-        <v>-177.119294</v>
+        <v>-277.376094</v>
       </c>
       <c r="AH102" s="15" t="n">
-        <v>-0.010418782</v>
+        <v>-0.01631624082352941</v>
       </c>
       <c r="AI102" s="15" t="n">
-        <v>-0.9371391216931216</v>
+        <v>-1.467598380952381</v>
       </c>
       <c r="AJ102" s="15" t="n">
-        <v>-8909.586939730001</v>
+        <v>-9009.84373973</v>
       </c>
       <c r="AK102" s="15" t="n">
-        <v>-0.5240933493958824</v>
+        <v>-0.5299908082194118</v>
       </c>
       <c r="AL102" s="15" t="n">
-        <v>-47.14067163878306</v>
+        <v>-47.67113089804232</v>
       </c>
     </row>
     <row r="103">
@@ -26802,22 +26802,22 @@
         <v>-253.7380611596296</v>
       </c>
       <c r="AG141" s="15" t="n">
-        <v>-831.870274</v>
+        <v>-932.127074</v>
       </c>
       <c r="AH141" s="15" t="n">
-        <v>-0.04893354552941177</v>
+        <v>-0.05483100435294118</v>
       </c>
       <c r="AI141" s="15" t="n">
-        <v>-4.401430021164021</v>
+        <v>-4.93188928042328</v>
       </c>
       <c r="AJ141" s="15" t="n">
-        <v>-48788.36383317001</v>
+        <v>-48888.62063317001</v>
       </c>
       <c r="AK141" s="15" t="n">
-        <v>-2.869903754892353</v>
+        <v>-2.875801213715882</v>
       </c>
       <c r="AL141" s="15" t="n">
-        <v>-258.1394911807936</v>
+        <v>-258.6699504400528</v>
       </c>
     </row>
     <row r="142">
@@ -27440,22 +27440,22 @@
         <v>-0.1070750670899471</v>
       </c>
       <c r="AG149" s="11" t="n">
-        <v>-0.0247</v>
+        <v>-0.600042</v>
       </c>
       <c r="AH149" s="11" t="n">
-        <v>-1.452941176470588e-06</v>
+        <v>-3.529658823529412e-05</v>
       </c>
       <c r="AI149" s="11" t="n">
-        <v>-0.0001306878306878307</v>
+        <v>-0.003174825396825397</v>
       </c>
       <c r="AJ149" s="11" t="n">
-        <v>-20.26188768</v>
+        <v>-20.83722968</v>
       </c>
       <c r="AK149" s="11" t="n">
-        <v>-0.001191875745882353</v>
+        <v>-0.001225719392941177</v>
       </c>
       <c r="AL149" s="11" t="n">
-        <v>-0.1072057549206349</v>
+        <v>-0.1102498924867725</v>
       </c>
     </row>
     <row r="150">
@@ -28083,22 +28083,22 @@
         <v>-33.08992313634921</v>
       </c>
       <c r="AG156" s="15" t="n">
-        <v>-176.252976</v>
+        <v>-176.828318</v>
       </c>
       <c r="AH156" s="15" t="n">
-        <v>-0.01036782211764706</v>
+        <v>-0.01040166576470588</v>
       </c>
       <c r="AI156" s="15" t="n">
-        <v>-0.9325554285714285</v>
+        <v>-0.9355995661375661</v>
       </c>
       <c r="AJ156" s="15" t="n">
-        <v>-6430.248448769999</v>
+        <v>-6430.82379077</v>
       </c>
       <c r="AK156" s="15" t="n">
-        <v>-0.3782499087511765</v>
+        <v>-0.3782837523982353</v>
       </c>
       <c r="AL156" s="15" t="n">
-        <v>-34.02247856492063</v>
+        <v>-34.02552270248678</v>
       </c>
     </row>
     <row r="157">
@@ -28198,22 +28198,22 @@
         <v>-1609.397741344392</v>
       </c>
       <c r="AG157" s="19" t="n">
-        <v>-4571.992149</v>
+        <v>-4672.824291</v>
       </c>
       <c r="AH157" s="19" t="n">
-        <v>-0.2689407146470588</v>
+        <v>-0.274872017117647</v>
       </c>
       <c r="AI157" s="19" t="n">
-        <v>-24.19043465079365</v>
+        <v>-24.72393804761905</v>
       </c>
       <c r="AJ157" s="19" t="n">
-        <v>-308748.1652630899</v>
+        <v>-308848.99740509</v>
       </c>
       <c r="AK157" s="19" t="n">
-        <v>-18.16165678018177</v>
+        <v>-18.16758808265235</v>
       </c>
       <c r="AL157" s="19" t="n">
-        <v>-1633.588175995185</v>
+        <v>-1634.12167939201</v>
       </c>
     </row>
     <row r="158">
@@ -28313,22 +28313,22 @@
         <v>-277.2179185799473</v>
       </c>
       <c r="AG158" s="19" t="n">
-        <v>8954.272634000001</v>
+        <v>8853.440492</v>
       </c>
       <c r="AH158" s="19" t="n">
-        <v>0.5267219196470588</v>
+        <v>0.5207906171764706</v>
       </c>
       <c r="AI158" s="19" t="n">
-        <v>47.37710388359789</v>
+        <v>46.84360048677249</v>
       </c>
       <c r="AJ158" s="19" t="n">
-        <v>-43439.91397761</v>
+        <v>-43540.74611961</v>
       </c>
       <c r="AK158" s="19" t="n">
-        <v>-2.555289057506472</v>
+        <v>-2.56122035997706</v>
       </c>
       <c r="AL158" s="19" t="n">
-        <v>-229.8408146963494</v>
+        <v>-230.3743180931748</v>
       </c>
     </row>
     <row r="159">
@@ -28428,22 +28428,22 @@
         <v>79.78557785582009</v>
       </c>
       <c r="AG159" s="7" t="n">
-        <v>24033.74684875</v>
+        <v>23932.91470675</v>
       </c>
       <c r="AH159" s="7" t="n">
-        <v>1.413749814632353</v>
+        <v>1.407818512161765</v>
       </c>
       <c r="AI159" s="7" t="n">
-        <v>127.162681739418</v>
+        <v>126.6291783425926</v>
       </c>
       <c r="AJ159" s="7" t="n">
-        <v>24033.74684875</v>
+        <v>23932.91470675</v>
       </c>
       <c r="AK159" s="7" t="n">
-        <v>1.413749814632353</v>
+        <v>1.407818512161765</v>
       </c>
       <c r="AL159" s="7" t="n">
-        <v>127.162681739418</v>
+        <v>126.6291783425926</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Tue 10/13/2026  9:33
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -734,7 +734,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 12 Oct 2026 17:09</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 13 Oct 2026 09:33</t>
         </is>
       </c>
     </row>
@@ -816,14 +816,14 @@
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 12 Oct 2026</t>
+          <t>MTD as of 13 Oct 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
       <c r="AI3" s="4" t="n"/>
       <c r="AJ3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 12 Oct 2026</t>
+          <t>YTD as of 13 Oct 2026</t>
         </is>
       </c>
       <c r="AK3" s="4" t="n"/>
@@ -15137,7 +15137,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 12 Oct 2026 17:09 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 13 Oct 2026 09:33 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -15219,14 +15219,14 @@
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 12 Oct 2026</t>
+          <t>MTD as of 13 Oct 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
       <c r="AI3" s="4" t="n"/>
       <c r="AJ3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 12 Oct 2026</t>
+          <t>YTD as of 13 Oct 2026</t>
         </is>
       </c>
       <c r="AK3" s="4" t="n"/>

</xml_diff>

<commit_message>
Refresh dashboard Thu 10/15/2026 17:02
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -734,7 +734,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 13 Oct 2026 09:33</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 15 Oct 2026 17:02</t>
         </is>
       </c>
     </row>
@@ -816,14 +816,14 @@
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 13 Oct 2026</t>
+          <t>MTD as of 15 Oct 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
       <c r="AI3" s="4" t="n"/>
       <c r="AJ3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 13 Oct 2026</t>
+          <t>YTD as of 15 Oct 2026</t>
         </is>
       </c>
       <c r="AK3" s="4" t="n"/>
@@ -2330,22 +2330,22 @@
         <v>2521134.965502645</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>9044500</v>
+        <v>12881400</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>532.0294117647059</v>
+        <v>757.7294117647059</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>47854.49735449735</v>
+        <v>68155.55555555556</v>
       </c>
       <c r="AJ20" s="13" t="n">
-        <v>485539008.48</v>
+        <v>489375908.48</v>
       </c>
       <c r="AK20" s="13" t="n">
-        <v>28561.11814588236</v>
+        <v>28786.81814588236</v>
       </c>
       <c r="AL20" s="13" t="n">
-        <v>2568989.462857143</v>
+        <v>2589290.521058201</v>
       </c>
     </row>
     <row r="21">
@@ -2603,22 +2603,22 @@
         <v>491976.1904761905</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>8044500</v>
+        <v>10249500</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>473.2058823529412</v>
+        <v>602.9117647058823</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>42563.49206349206</v>
+        <v>54230.15873015873</v>
       </c>
       <c r="AJ23" s="11" t="n">
-        <v>101028000</v>
+        <v>103233000</v>
       </c>
       <c r="AK23" s="11" t="n">
-        <v>5942.823529411765</v>
+        <v>6072.529411764705</v>
       </c>
       <c r="AL23" s="11" t="n">
-        <v>534539.6825396825</v>
+        <v>546206.3492063492</v>
       </c>
     </row>
     <row r="24">
@@ -2955,17 +2955,23 @@
       <c r="AF28" s="13" t="n">
         <v>65466.20105820106</v>
       </c>
-      <c r="AG28" s="13" t="n"/>
-      <c r="AH28" s="13" t="n"/>
-      <c r="AI28" s="13" t="n"/>
+      <c r="AG28" s="13" t="n">
+        <v>1631900</v>
+      </c>
+      <c r="AH28" s="13" t="n">
+        <v>95.99411764705883</v>
+      </c>
+      <c r="AI28" s="13" t="n">
+        <v>8634.391534391534</v>
+      </c>
       <c r="AJ28" s="13" t="n">
-        <v>12373112</v>
+        <v>14005012</v>
       </c>
       <c r="AK28" s="13" t="n">
-        <v>727.8301176470587</v>
+        <v>823.8242352941176</v>
       </c>
       <c r="AL28" s="13" t="n">
-        <v>65466.20105820106</v>
+        <v>74100.59259259258</v>
       </c>
     </row>
     <row r="29">
@@ -4149,22 +4155,22 @@
         <v>1332179822.764445</v>
       </c>
       <c r="AG45" s="15" t="n">
-        <v>13526264783</v>
+        <v>13530101683</v>
       </c>
       <c r="AH45" s="15" t="n">
-        <v>795662.6342941177</v>
+        <v>795888.3342941176</v>
       </c>
       <c r="AI45" s="15" t="n">
-        <v>71567538.53439154</v>
+        <v>71587839.5925926</v>
       </c>
       <c r="AJ45" s="15" t="n">
-        <v>265308251285.48</v>
+        <v>265312088185.48</v>
       </c>
       <c r="AK45" s="15" t="n">
-        <v>15606367.72267529</v>
+        <v>15606593.42267529</v>
       </c>
       <c r="AL45" s="15" t="n">
-        <v>1403747361.298836</v>
+        <v>1403767662.357037</v>
       </c>
     </row>
     <row r="46">
@@ -4489,17 +4495,23 @@
       <c r="AF50" s="11" t="n">
         <v>-4462156.708994709</v>
       </c>
-      <c r="AG50" s="11" t="n"/>
-      <c r="AH50" s="11" t="n"/>
-      <c r="AI50" s="11" t="n"/>
+      <c r="AG50" s="11" t="n">
+        <v>-398598156</v>
+      </c>
+      <c r="AH50" s="11" t="n">
+        <v>-23446.95035294118</v>
+      </c>
+      <c r="AI50" s="11" t="n">
+        <v>-2108984.952380952</v>
+      </c>
       <c r="AJ50" s="11" t="n">
-        <v>-843347618</v>
+        <v>-1241945774</v>
       </c>
       <c r="AK50" s="11" t="n">
-        <v>-49608.68341176471</v>
+        <v>-73055.63376470588</v>
       </c>
       <c r="AL50" s="11" t="n">
-        <v>-4462156.708994709</v>
+        <v>-6571141.661375661</v>
       </c>
     </row>
     <row r="51">
@@ -4672,22 +4684,22 @@
         <v>-986146.9047619047</v>
       </c>
       <c r="AG52" s="11" t="n">
-        <v>-46950780</v>
+        <v>-47904270</v>
       </c>
       <c r="AH52" s="11" t="n">
-        <v>-2761.810588235294</v>
+        <v>-2817.898235294118</v>
       </c>
       <c r="AI52" s="11" t="n">
-        <v>-248416.8253968254</v>
+        <v>-253461.746031746</v>
       </c>
       <c r="AJ52" s="11" t="n">
-        <v>-233332545</v>
+        <v>-234286035</v>
       </c>
       <c r="AK52" s="11" t="n">
-        <v>-13725.44382352941</v>
+        <v>-13781.53147058824</v>
       </c>
       <c r="AL52" s="11" t="n">
-        <v>-1234563.73015873</v>
+        <v>-1239608.650793651</v>
       </c>
     </row>
     <row r="53">
@@ -4903,22 +4915,22 @@
         <v>-10237629.65079365</v>
       </c>
       <c r="AG55" s="13" t="n">
-        <v>-492540000</v>
+        <v>-517416250</v>
       </c>
       <c r="AH55" s="13" t="n">
-        <v>-28972.94117647059</v>
+        <v>-30436.25</v>
       </c>
       <c r="AI55" s="13" t="n">
-        <v>-2606031.746031746</v>
+        <v>-2737652.116402117</v>
       </c>
       <c r="AJ55" s="13" t="n">
-        <v>-2427452004</v>
+        <v>-2452328254</v>
       </c>
       <c r="AK55" s="13" t="n">
-        <v>-142791.2943529412</v>
+        <v>-144254.6031764706</v>
       </c>
       <c r="AL55" s="13" t="n">
-        <v>-12843661.3968254</v>
+        <v>-12975281.76719576</v>
       </c>
     </row>
     <row r="56">
@@ -5631,22 +5643,22 @@
         <v>-95006082.8141799</v>
       </c>
       <c r="AG63" s="15" t="n">
-        <v>-891781311</v>
+        <v>-1316209207</v>
       </c>
       <c r="AH63" s="15" t="n">
-        <v>-52457.72417647059</v>
+        <v>-77424.071</v>
       </c>
       <c r="AI63" s="15" t="n">
-        <v>-4718419.634920635</v>
+        <v>-6964069.878306879</v>
       </c>
       <c r="AJ63" s="15" t="n">
-        <v>-18847930962.88</v>
+        <v>-19272358858.88</v>
       </c>
       <c r="AK63" s="15" t="n">
-        <v>-1108701.821345882</v>
+        <v>-1133668.168169412</v>
       </c>
       <c r="AL63" s="15" t="n">
-        <v>-99724502.44910054</v>
+        <v>-101970152.6924868</v>
       </c>
     </row>
     <row r="64">
@@ -6759,22 +6771,22 @@
         <v>-53015355.81481481</v>
       </c>
       <c r="AG81" s="11" t="n">
-        <v>-903478933</v>
+        <v>-4492646413</v>
       </c>
       <c r="AH81" s="11" t="n">
-        <v>-53145.8195882353</v>
+        <v>-264273.3184117647</v>
       </c>
       <c r="AI81" s="11" t="n">
-        <v>-4780311.814814814</v>
+        <v>-23770615.94179894</v>
       </c>
       <c r="AJ81" s="11" t="n">
-        <v>-10923381182</v>
+        <v>-14512548662</v>
       </c>
       <c r="AK81" s="11" t="n">
-        <v>-642551.834235294</v>
+        <v>-853679.3330588234</v>
       </c>
       <c r="AL81" s="11" t="n">
-        <v>-57795667.62962962</v>
+        <v>-76785971.75661375</v>
       </c>
     </row>
     <row r="82">
@@ -6874,22 +6886,22 @@
         <v>-58934229.3347619</v>
       </c>
       <c r="AG82" s="13" t="n">
-        <v>-1752972535</v>
+        <v>-2507660085</v>
       </c>
       <c r="AH82" s="13" t="n">
-        <v>-103116.0314705882</v>
+        <v>-147509.4167647059</v>
       </c>
       <c r="AI82" s="13" t="n">
-        <v>-9274986.957671957</v>
+        <v>-13268042.77777778</v>
       </c>
       <c r="AJ82" s="13" t="n">
-        <v>-12891541879.27</v>
+        <v>-13646229429.27</v>
       </c>
       <c r="AK82" s="13" t="n">
-        <v>-758325.9928982353</v>
+        <v>-802719.3781923529</v>
       </c>
       <c r="AL82" s="13" t="n">
-        <v>-68209216.29243386</v>
+        <v>-72202272.11253968</v>
       </c>
     </row>
     <row r="83">
@@ -6988,17 +7000,23 @@
       <c r="AF83" s="11" t="n">
         <v>-56096500.02645503</v>
       </c>
-      <c r="AG83" s="11" t="n"/>
-      <c r="AH83" s="11" t="n"/>
-      <c r="AI83" s="11" t="n"/>
+      <c r="AG83" s="11" t="n">
+        <v>-2411754594</v>
+      </c>
+      <c r="AH83" s="11" t="n">
+        <v>-141867.9172941177</v>
+      </c>
+      <c r="AI83" s="11" t="n">
+        <v>-12760606.31746032</v>
+      </c>
       <c r="AJ83" s="11" t="n">
-        <v>-10602238505</v>
+        <v>-13013993099</v>
       </c>
       <c r="AK83" s="11" t="n">
-        <v>-623661.0885294117</v>
+        <v>-765529.0058235293</v>
       </c>
       <c r="AL83" s="11" t="n">
-        <v>-56096500.02645503</v>
+        <v>-68857106.34391534</v>
       </c>
     </row>
     <row r="84">
@@ -7098,22 +7116,22 @@
         <v>-2427178.873015873</v>
       </c>
       <c r="AG84" s="13" t="n">
-        <v>-6136120</v>
+        <v>-11370640</v>
       </c>
       <c r="AH84" s="13" t="n">
-        <v>-360.9482352941176</v>
+        <v>-668.8611764705882</v>
       </c>
       <c r="AI84" s="13" t="n">
-        <v>-32466.24338624339</v>
+        <v>-60162.1164021164</v>
       </c>
       <c r="AJ84" s="13" t="n">
-        <v>-464872927</v>
+        <v>-470107447</v>
       </c>
       <c r="AK84" s="13" t="n">
-        <v>-27345.46629411765</v>
+        <v>-27653.37923529412</v>
       </c>
       <c r="AL84" s="13" t="n">
-        <v>-2459645.116402117</v>
+        <v>-2487340.98941799</v>
       </c>
     </row>
     <row r="85">
@@ -7213,22 +7231,22 @@
         <v>-170473264.0490476</v>
       </c>
       <c r="AG85" s="15" t="n">
-        <v>-2662587588</v>
+        <v>-9423431732</v>
       </c>
       <c r="AH85" s="15" t="n">
-        <v>-156622.7992941176</v>
+        <v>-554319.5136470589</v>
       </c>
       <c r="AI85" s="15" t="n">
-        <v>-14087765.01587302</v>
+        <v>-49859427.15343916</v>
       </c>
       <c r="AJ85" s="15" t="n">
-        <v>-34882034493.27</v>
+        <v>-41642878637.27</v>
       </c>
       <c r="AK85" s="15" t="n">
-        <v>-2051884.381957059</v>
+        <v>-2449581.09631</v>
       </c>
       <c r="AL85" s="15" t="n">
-        <v>-184561029.0649207</v>
+        <v>-220332691.2024868</v>
       </c>
     </row>
     <row r="86">
@@ -7414,22 +7432,22 @@
         <v>-778818.2539682541</v>
       </c>
       <c r="AG88" s="11" t="n">
-        <v>-874372</v>
+        <v>-10466372</v>
       </c>
       <c r="AH88" s="11" t="n">
-        <v>-51.43364705882353</v>
+        <v>-615.6689411764706</v>
       </c>
       <c r="AI88" s="11" t="n">
-        <v>-4626.306878306878</v>
+        <v>-55377.62962962963</v>
       </c>
       <c r="AJ88" s="11" t="n">
-        <v>-148071022</v>
+        <v>-157663022</v>
       </c>
       <c r="AK88" s="11" t="n">
-        <v>-8710.060117647061</v>
+        <v>-9274.295411764708</v>
       </c>
       <c r="AL88" s="11" t="n">
-        <v>-783444.560846561</v>
+        <v>-834195.8835978837</v>
       </c>
     </row>
     <row r="89">
@@ -7571,17 +7589,23 @@
       <c r="AF90" s="11" t="n">
         <v>-1035486.037037037</v>
       </c>
-      <c r="AG90" s="11" t="n"/>
-      <c r="AH90" s="11" t="n"/>
-      <c r="AI90" s="11" t="n"/>
+      <c r="AG90" s="11" t="n">
+        <v>-504700</v>
+      </c>
+      <c r="AH90" s="11" t="n">
+        <v>-29.68823529411765</v>
+      </c>
+      <c r="AI90" s="11" t="n">
+        <v>-2670.37037037037</v>
+      </c>
       <c r="AJ90" s="11" t="n">
-        <v>-195706861</v>
+        <v>-196211561</v>
       </c>
       <c r="AK90" s="11" t="n">
-        <v>-11512.16829411765</v>
+        <v>-11541.85652941177</v>
       </c>
       <c r="AL90" s="11" t="n">
-        <v>-1035486.037037037</v>
+        <v>-1038156.407407407</v>
       </c>
     </row>
     <row r="91">
@@ -7650,17 +7674,23 @@
       <c r="AF91" s="13" t="n">
         <v>-8838.981164021165</v>
       </c>
-      <c r="AG91" s="13" t="n"/>
-      <c r="AH91" s="13" t="n"/>
-      <c r="AI91" s="13" t="n"/>
+      <c r="AG91" s="13" t="n">
+        <v>-702500</v>
+      </c>
+      <c r="AH91" s="13" t="n">
+        <v>-41.3235294117647</v>
+      </c>
+      <c r="AI91" s="13" t="n">
+        <v>-3716.931216931217</v>
+      </c>
       <c r="AJ91" s="13" t="n">
-        <v>-1670567.44</v>
+        <v>-2373067.44</v>
       </c>
       <c r="AK91" s="13" t="n">
-        <v>-98.26867294117646</v>
+        <v>-139.5922023529412</v>
       </c>
       <c r="AL91" s="13" t="n">
-        <v>-8838.981164021165</v>
+        <v>-12555.91238095238</v>
       </c>
     </row>
     <row r="92">
@@ -7863,22 +7893,22 @@
         <v>-12778.81481481481</v>
       </c>
       <c r="AG93" s="13" t="n">
-        <v>-233600</v>
+        <v>-297600</v>
       </c>
       <c r="AH93" s="13" t="n">
-        <v>-13.74117647058823</v>
+        <v>-17.50588235294118</v>
       </c>
       <c r="AI93" s="13" t="n">
-        <v>-1235.978835978836</v>
+        <v>-1574.603174603175</v>
       </c>
       <c r="AJ93" s="13" t="n">
-        <v>-2648796</v>
+        <v>-2712796</v>
       </c>
       <c r="AK93" s="13" t="n">
-        <v>-155.8115294117647</v>
+        <v>-159.5762352941177</v>
       </c>
       <c r="AL93" s="13" t="n">
-        <v>-14014.79365079365</v>
+        <v>-14353.41798941799</v>
       </c>
     </row>
     <row r="94">
@@ -7978,22 +8008,22 @@
         <v>-2636230.425608465</v>
       </c>
       <c r="AG94" s="15" t="n">
-        <v>-2973672</v>
+        <v>-13836872</v>
       </c>
       <c r="AH94" s="15" t="n">
-        <v>-174.9218823529412</v>
+        <v>-813.9336470588236</v>
       </c>
       <c r="AI94" s="15" t="n">
-        <v>-15733.71428571429</v>
+        <v>-73210.96296296296</v>
       </c>
       <c r="AJ94" s="15" t="n">
-        <v>-501221222.44</v>
+        <v>-512084422.44</v>
       </c>
       <c r="AK94" s="15" t="n">
-        <v>-29483.60132</v>
+        <v>-30122.61308470588</v>
       </c>
       <c r="AL94" s="15" t="n">
-        <v>-2651964.13989418</v>
+        <v>-2709441.388571429</v>
       </c>
     </row>
     <row r="95">
@@ -8173,22 +8203,22 @@
         <v>-471451.3227513228</v>
       </c>
       <c r="AG97" s="13" t="n">
-        <v>-531541</v>
+        <v>-76331541</v>
       </c>
       <c r="AH97" s="13" t="n">
-        <v>-31.26711764705883</v>
+        <v>-4490.090647058823</v>
       </c>
       <c r="AI97" s="13" t="n">
-        <v>-2812.386243386243</v>
+        <v>-403870.5873015873</v>
       </c>
       <c r="AJ97" s="13" t="n">
-        <v>-89635841</v>
+        <v>-165435841</v>
       </c>
       <c r="AK97" s="13" t="n">
-        <v>-5272.696529411764</v>
+        <v>-9731.520058823529</v>
       </c>
       <c r="AL97" s="13" t="n">
-        <v>-474263.708994709</v>
+        <v>-875321.91005291</v>
       </c>
     </row>
     <row r="98">
@@ -8288,22 +8318,22 @@
         <v>-1418156.079365079</v>
       </c>
       <c r="AG98" s="11" t="n">
-        <v>-112897000</v>
+        <v>-128353307</v>
       </c>
       <c r="AH98" s="11" t="n">
-        <v>-6641</v>
+        <v>-7550.194529411765</v>
       </c>
       <c r="AI98" s="11" t="n">
-        <v>-597338.6243386243</v>
+        <v>-679118.0264550265</v>
       </c>
       <c r="AJ98" s="11" t="n">
-        <v>-380928499</v>
+        <v>-396384806</v>
       </c>
       <c r="AK98" s="11" t="n">
-        <v>-22407.55876470588</v>
+        <v>-23316.75329411765</v>
       </c>
       <c r="AL98" s="11" t="n">
-        <v>-2015494.703703704</v>
+        <v>-2097274.105820106</v>
       </c>
     </row>
     <row r="99">
@@ -8518,22 +8548,22 @@
         <v>-1318975.026455026</v>
       </c>
       <c r="AG100" s="11" t="n">
-        <v>-7999429</v>
+        <v>-51709011</v>
       </c>
       <c r="AH100" s="11" t="n">
-        <v>-470.5546470588235</v>
+        <v>-3041.706529411765</v>
       </c>
       <c r="AI100" s="11" t="n">
-        <v>-42325.02116402116</v>
+        <v>-273592.6507936508</v>
       </c>
       <c r="AJ100" s="11" t="n">
-        <v>-257285709</v>
+        <v>-300995291</v>
       </c>
       <c r="AK100" s="11" t="n">
-        <v>-15134.45347058824</v>
+        <v>-17705.60535294118</v>
       </c>
       <c r="AL100" s="11" t="n">
-        <v>-1361300.047619048</v>
+        <v>-1592567.677248677</v>
       </c>
     </row>
     <row r="101">
@@ -8633,22 +8663,22 @@
         <v>-1928168.555555556</v>
       </c>
       <c r="AG101" s="13" t="n">
-        <v>-4332150</v>
+        <v>-4725650</v>
       </c>
       <c r="AH101" s="13" t="n">
-        <v>-254.8323529411765</v>
+        <v>-277.9794117647059</v>
       </c>
       <c r="AI101" s="13" t="n">
-        <v>-22921.42857142857</v>
+        <v>-25003.43915343915</v>
       </c>
       <c r="AJ101" s="13" t="n">
-        <v>-368756007</v>
+        <v>-369149507</v>
       </c>
       <c r="AK101" s="13" t="n">
-        <v>-21691.52982352941</v>
+        <v>-21714.67688235294</v>
       </c>
       <c r="AL101" s="13" t="n">
-        <v>-1951089.984126984</v>
+        <v>-1953171.994708995</v>
       </c>
     </row>
     <row r="102">
@@ -8748,22 +8778,22 @@
         <v>-46203532.51708995</v>
       </c>
       <c r="AG102" s="15" t="n">
-        <v>-277376094</v>
+        <v>-412735483</v>
       </c>
       <c r="AH102" s="15" t="n">
-        <v>-16316.24082352941</v>
+        <v>-24278.55782352941</v>
       </c>
       <c r="AI102" s="15" t="n">
-        <v>-1467598.380952381</v>
+        <v>-2183785.624338625</v>
       </c>
       <c r="AJ102" s="15" t="n">
-        <v>-9009843739.73</v>
+        <v>-9145203128.73</v>
       </c>
       <c r="AK102" s="15" t="n">
-        <v>-529990.8082194118</v>
+        <v>-537953.1252194118</v>
       </c>
       <c r="AL102" s="15" t="n">
-        <v>-47671130.89804233</v>
+        <v>-48387318.14142857</v>
       </c>
     </row>
     <row r="103">
@@ -8906,22 +8936,22 @@
         <v>-1237435.248677249</v>
       </c>
       <c r="AG104" s="11" t="n">
-        <v>-17094600</v>
+        <v>-22046700</v>
       </c>
       <c r="AH104" s="11" t="n">
-        <v>-1005.564705882353</v>
+        <v>-1296.864705882353</v>
       </c>
       <c r="AI104" s="11" t="n">
-        <v>-90447.61904761905</v>
+        <v>-116649.2063492063</v>
       </c>
       <c r="AJ104" s="11" t="n">
-        <v>-250969862</v>
+        <v>-255921962</v>
       </c>
       <c r="AK104" s="11" t="n">
-        <v>-14762.93305882353</v>
+        <v>-15054.23305882353</v>
       </c>
       <c r="AL104" s="11" t="n">
-        <v>-1327882.867724868</v>
+        <v>-1354084.455026455</v>
       </c>
     </row>
     <row r="105">
@@ -9021,22 +9051,22 @@
         <v>-1864747.592592593</v>
       </c>
       <c r="AG105" s="13" t="n">
-        <v>-161522493</v>
+        <v>-170282139</v>
       </c>
       <c r="AH105" s="13" t="n">
-        <v>-9501.323117647058</v>
+        <v>-10016.59641176471</v>
       </c>
       <c r="AI105" s="13" t="n">
-        <v>-854616.3650793651</v>
+        <v>-900963.6984126985</v>
       </c>
       <c r="AJ105" s="13" t="n">
-        <v>-513959788</v>
+        <v>-522719434</v>
       </c>
       <c r="AK105" s="13" t="n">
-        <v>-30232.92870588235</v>
+        <v>-30748.202</v>
       </c>
       <c r="AL105" s="13" t="n">
-        <v>-2719363.957671958</v>
+        <v>-2765711.291005291</v>
       </c>
     </row>
     <row r="106">
@@ -9136,22 +9166,22 @@
         <v>-8926693.243386243</v>
       </c>
       <c r="AG106" s="11" t="n">
-        <v>-70776068</v>
+        <v>-136708815</v>
       </c>
       <c r="AH106" s="11" t="n">
-        <v>-4163.298117647058</v>
+        <v>-8041.695</v>
       </c>
       <c r="AI106" s="11" t="n">
-        <v>-374476.5502645503</v>
+        <v>-723327.0634920635</v>
       </c>
       <c r="AJ106" s="11" t="n">
-        <v>-1757921091</v>
+        <v>-1823853838</v>
       </c>
       <c r="AK106" s="11" t="n">
-        <v>-103407.123</v>
+        <v>-107285.5198823529</v>
       </c>
       <c r="AL106" s="11" t="n">
-        <v>-9301169.793650793</v>
+        <v>-9650020.306878306</v>
       </c>
     </row>
     <row r="107">
@@ -9245,22 +9275,22 @@
         <v>-1059205.370370371</v>
       </c>
       <c r="AG107" s="13" t="n">
-        <v>-34937225</v>
+        <v>-59088825</v>
       </c>
       <c r="AH107" s="13" t="n">
-        <v>-2055.130882352941</v>
+        <v>-3475.813235294117</v>
       </c>
       <c r="AI107" s="13" t="n">
-        <v>-184853.0423280423</v>
+        <v>-312639.2857142857</v>
       </c>
       <c r="AJ107" s="13" t="n">
-        <v>-235127040</v>
+        <v>-259278640</v>
       </c>
       <c r="AK107" s="13" t="n">
-        <v>-13831.00235294118</v>
+        <v>-15251.68470588235</v>
       </c>
       <c r="AL107" s="13" t="n">
-        <v>-1244058.412698413</v>
+        <v>-1371844.656084656</v>
       </c>
     </row>
     <row r="108">
@@ -9360,22 +9390,22 @@
         <v>-13088081.45502646</v>
       </c>
       <c r="AG108" s="15" t="n">
-        <v>-284330386</v>
+        <v>-388126479</v>
       </c>
       <c r="AH108" s="15" t="n">
-        <v>-16725.31682352941</v>
+        <v>-22830.96935294118</v>
       </c>
       <c r="AI108" s="15" t="n">
-        <v>-1504393.576719577</v>
+        <v>-2053579.253968254</v>
       </c>
       <c r="AJ108" s="15" t="n">
-        <v>-2757977781</v>
+        <v>-2861773874</v>
       </c>
       <c r="AK108" s="15" t="n">
-        <v>-162233.987117647</v>
+        <v>-168339.6396470588</v>
       </c>
       <c r="AL108" s="15" t="n">
-        <v>-14592475.03174603</v>
+        <v>-15141660.70899471</v>
       </c>
     </row>
     <row r="109">
@@ -9694,22 +9724,22 @@
         <v>-2487639.740740741</v>
       </c>
       <c r="AG112" s="11" t="n">
-        <v>-21587500</v>
+        <v>-22039000</v>
       </c>
       <c r="AH112" s="11" t="n">
-        <v>-1269.85294117647</v>
+        <v>-1296.411764705882</v>
       </c>
       <c r="AI112" s="11" t="n">
-        <v>-114219.5767195767</v>
+        <v>-116608.4656084656</v>
       </c>
       <c r="AJ112" s="11" t="n">
-        <v>-491751411</v>
+        <v>-492202911</v>
       </c>
       <c r="AK112" s="11" t="n">
-        <v>-28926.5535882353</v>
+        <v>-28953.11241176471</v>
       </c>
       <c r="AL112" s="11" t="n">
-        <v>-2601859.317460317</v>
+        <v>-2604248.206349206</v>
       </c>
     </row>
     <row r="113">
@@ -9809,22 +9839,22 @@
         <v>-3302494.767195768</v>
       </c>
       <c r="AG113" s="15" t="n">
-        <v>-21587500</v>
+        <v>-22039000</v>
       </c>
       <c r="AH113" s="15" t="n">
-        <v>-1269.85294117647</v>
+        <v>-1296.411764705882</v>
       </c>
       <c r="AI113" s="15" t="n">
-        <v>-114219.5767195767</v>
+        <v>-116608.4656084656</v>
       </c>
       <c r="AJ113" s="15" t="n">
-        <v>-645759011</v>
+        <v>-646210511</v>
       </c>
       <c r="AK113" s="15" t="n">
-        <v>-37985.82417647059</v>
+        <v>-38012.383</v>
       </c>
       <c r="AL113" s="15" t="n">
-        <v>-3416714.343915344</v>
+        <v>-3419103.232804233</v>
       </c>
     </row>
     <row r="114">
@@ -9961,22 +9991,22 @@
         <v>-2418823.142857143</v>
       </c>
       <c r="AG115" s="11" t="n">
-        <v>-37104000</v>
+        <v>-59994000</v>
       </c>
       <c r="AH115" s="11" t="n">
-        <v>-2182.588235294118</v>
+        <v>-3529.058823529412</v>
       </c>
       <c r="AI115" s="11" t="n">
-        <v>-196317.4603174603</v>
+        <v>-317428.5714285714</v>
       </c>
       <c r="AJ115" s="11" t="n">
-        <v>-494261574</v>
+        <v>-517151574</v>
       </c>
       <c r="AK115" s="11" t="n">
-        <v>-29074.21023529412</v>
+        <v>-30420.68082352942</v>
       </c>
       <c r="AL115" s="11" t="n">
-        <v>-2615140.603174603</v>
+        <v>-2736251.714285714</v>
       </c>
     </row>
     <row r="116">
@@ -10137,22 +10167,22 @@
         <v>-715199.5291005292</v>
       </c>
       <c r="AG117" s="11" t="n">
-        <v>-12740000</v>
+        <v>-15240000</v>
       </c>
       <c r="AH117" s="11" t="n">
-        <v>-749.4117647058823</v>
+        <v>-896.4705882352941</v>
       </c>
       <c r="AI117" s="11" t="n">
-        <v>-67407.4074074074</v>
+        <v>-80634.92063492064</v>
       </c>
       <c r="AJ117" s="11" t="n">
-        <v>-147912711</v>
+        <v>-150412711</v>
       </c>
       <c r="AK117" s="11" t="n">
-        <v>-8700.747705882353</v>
+        <v>-8847.806529411766</v>
       </c>
       <c r="AL117" s="11" t="n">
-        <v>-782606.9365079366</v>
+        <v>-795834.4497354497</v>
       </c>
     </row>
     <row r="118">
@@ -10252,22 +10282,22 @@
         <v>-2977326.375661375</v>
       </c>
       <c r="AG118" s="13" t="n">
-        <v>-14652000</v>
+        <v>-37873475</v>
       </c>
       <c r="AH118" s="13" t="n">
-        <v>-861.8823529411765</v>
+        <v>-2227.851470588235</v>
       </c>
       <c r="AI118" s="13" t="n">
-        <v>-77523.80952380953</v>
+        <v>-200388.7566137566</v>
       </c>
       <c r="AJ118" s="13" t="n">
-        <v>-577366685</v>
+        <v>-600588160</v>
       </c>
       <c r="AK118" s="13" t="n">
-        <v>-33962.74617647059</v>
+        <v>-35328.71529411765</v>
       </c>
       <c r="AL118" s="13" t="n">
-        <v>-3054850.185185185</v>
+        <v>-3177715.132275132</v>
       </c>
     </row>
     <row r="119">
@@ -10367,22 +10397,22 @@
         <v>-6180132.116402117</v>
       </c>
       <c r="AG119" s="15" t="n">
-        <v>-64496000</v>
+        <v>-113107475</v>
       </c>
       <c r="AH119" s="15" t="n">
-        <v>-3793.882352941177</v>
+        <v>-6653.380882352942</v>
       </c>
       <c r="AI119" s="15" t="n">
-        <v>-341248.6772486772</v>
+        <v>-598452.2486772487</v>
       </c>
       <c r="AJ119" s="15" t="n">
-        <v>-1232540970</v>
+        <v>-1281152445</v>
       </c>
       <c r="AK119" s="15" t="n">
-        <v>-72502.41</v>
+        <v>-75361.90852941177</v>
       </c>
       <c r="AL119" s="15" t="n">
-        <v>-6521380.793650794</v>
+        <v>-6778584.365079366</v>
       </c>
     </row>
     <row r="120">
@@ -10568,40 +10598,40 @@
         <v>-5643998.698412699</v>
       </c>
       <c r="AA122" s="13" t="n">
-        <v>-942329623</v>
+        <v>-942313623</v>
       </c>
       <c r="AB122" s="13" t="n">
-        <v>-55431.15429411764</v>
+        <v>-55430.21311764706</v>
       </c>
       <c r="AC122" s="13" t="n">
-        <v>-4985871.021164021</v>
+        <v>-4985786.365079365</v>
       </c>
       <c r="AD122" s="13" t="n">
-        <v>-6543389604</v>
+        <v>-6543373604</v>
       </c>
       <c r="AE122" s="13" t="n">
-        <v>-384905.2708235295</v>
+        <v>-384904.3296470589</v>
       </c>
       <c r="AF122" s="13" t="n">
-        <v>-34621109.01587301</v>
+        <v>-34621024.35978836</v>
       </c>
       <c r="AG122" s="13" t="n">
-        <v>-212354423</v>
+        <v>-386151687</v>
       </c>
       <c r="AH122" s="13" t="n">
-        <v>-12491.43664705882</v>
+        <v>-22714.80511764706</v>
       </c>
       <c r="AI122" s="13" t="n">
-        <v>-1123568.375661376</v>
+        <v>-2043130.619047619</v>
       </c>
       <c r="AJ122" s="13" t="n">
-        <v>-6755744027</v>
+        <v>-6929525291</v>
       </c>
       <c r="AK122" s="13" t="n">
-        <v>-397396.7074705883</v>
+        <v>-407619.1347647059</v>
       </c>
       <c r="AL122" s="13" t="n">
-        <v>-35744677.39153439</v>
+        <v>-36664154.97883598</v>
       </c>
     </row>
     <row r="123">
@@ -10683,40 +10713,40 @@
         <v>-5643998.698412699</v>
       </c>
       <c r="AA123" s="15" t="n">
-        <v>-1063308436</v>
+        <v>-1063292436</v>
       </c>
       <c r="AB123" s="15" t="n">
-        <v>-62547.55505882353</v>
+        <v>-62546.61388235294</v>
       </c>
       <c r="AC123" s="15" t="n">
-        <v>-5625970.560846561</v>
+        <v>-5625885.904761905</v>
       </c>
       <c r="AD123" s="15" t="n">
-        <v>-6664368417</v>
+        <v>-6664352417</v>
       </c>
       <c r="AE123" s="15" t="n">
-        <v>-392021.6715882354</v>
+        <v>-392020.7304117648</v>
       </c>
       <c r="AF123" s="15" t="n">
-        <v>-35261208.55555556</v>
+        <v>-35261123.8994709</v>
       </c>
       <c r="AG123" s="15" t="n">
-        <v>-212354423</v>
+        <v>-386151687</v>
       </c>
       <c r="AH123" s="15" t="n">
-        <v>-12491.43664705882</v>
+        <v>-22714.80511764706</v>
       </c>
       <c r="AI123" s="15" t="n">
-        <v>-1123568.375661376</v>
+        <v>-2043130.619047619</v>
       </c>
       <c r="AJ123" s="15" t="n">
-        <v>-6876722840</v>
+        <v>-7050504104</v>
       </c>
       <c r="AK123" s="15" t="n">
-        <v>-404513.1082352942</v>
+        <v>-414735.5355294118</v>
       </c>
       <c r="AL123" s="15" t="n">
-        <v>-36384776.93121693</v>
+        <v>-37304254.51851852</v>
       </c>
     </row>
     <row r="124">
@@ -11107,17 +11137,23 @@
       <c r="AF128" s="13" t="n">
         <v>-7042696.306878306</v>
       </c>
-      <c r="AG128" s="13" t="n"/>
-      <c r="AH128" s="13" t="n"/>
-      <c r="AI128" s="13" t="n"/>
+      <c r="AG128" s="13" t="n">
+        <v>-1842353</v>
+      </c>
+      <c r="AH128" s="13" t="n">
+        <v>-108.3737058823529</v>
+      </c>
+      <c r="AI128" s="13" t="n">
+        <v>-9747.899470899471</v>
+      </c>
       <c r="AJ128" s="13" t="n">
-        <v>-1331069602</v>
+        <v>-1332911955</v>
       </c>
       <c r="AK128" s="13" t="n">
-        <v>-78298.21188235295</v>
+        <v>-78406.58558823529</v>
       </c>
       <c r="AL128" s="13" t="n">
-        <v>-7042696.306878306</v>
+        <v>-7052444.206349205</v>
       </c>
     </row>
     <row r="129">
@@ -11422,17 +11458,23 @@
       <c r="AF131" s="11" t="n">
         <v>-6150777.666666665</v>
       </c>
-      <c r="AG131" s="11" t="n"/>
-      <c r="AH131" s="11" t="n"/>
-      <c r="AI131" s="11" t="n"/>
+      <c r="AG131" s="11" t="n">
+        <v>-67365078</v>
+      </c>
+      <c r="AH131" s="11" t="n">
+        <v>-3962.651647058824</v>
+      </c>
+      <c r="AI131" s="11" t="n">
+        <v>-356428.9841269841</v>
+      </c>
       <c r="AJ131" s="11" t="n">
-        <v>-1162496979</v>
+        <v>-1229862057</v>
       </c>
       <c r="AK131" s="11" t="n">
-        <v>-68382.17523529413</v>
+        <v>-72344.82688235295</v>
       </c>
       <c r="AL131" s="11" t="n">
-        <v>-6150777.666666665</v>
+        <v>-6507206.650793649</v>
       </c>
     </row>
     <row r="132">
@@ -11531,17 +11573,23 @@
       <c r="AF132" s="15" t="n">
         <v>-141497165.3492064</v>
       </c>
-      <c r="AG132" s="15" t="n"/>
-      <c r="AH132" s="15" t="n"/>
-      <c r="AI132" s="15" t="n"/>
+      <c r="AG132" s="15" t="n">
+        <v>-69207431</v>
+      </c>
+      <c r="AH132" s="15" t="n">
+        <v>-4071.025352941177</v>
+      </c>
+      <c r="AI132" s="15" t="n">
+        <v>-366176.8835978836</v>
+      </c>
       <c r="AJ132" s="15" t="n">
-        <v>-26742964251</v>
+        <v>-26812171682</v>
       </c>
       <c r="AK132" s="15" t="n">
-        <v>-1573115.54417647</v>
+        <v>-1577186.569529412</v>
       </c>
       <c r="AL132" s="15" t="n">
-        <v>-141497165.3492064</v>
+        <v>-141863342.2328042</v>
       </c>
     </row>
     <row r="133">
@@ -11672,22 +11720,22 @@
         <v>-197258.3068783069</v>
       </c>
       <c r="AG134" s="11" t="n">
-        <v>-2404000</v>
+        <v>-3141000</v>
       </c>
       <c r="AH134" s="11" t="n">
-        <v>-141.4117647058823</v>
+        <v>-184.7647058823529</v>
       </c>
       <c r="AI134" s="11" t="n">
-        <v>-12719.57671957672</v>
+        <v>-16619.04761904762</v>
       </c>
       <c r="AJ134" s="11" t="n">
-        <v>-39685820</v>
+        <v>-40422820</v>
       </c>
       <c r="AK134" s="11" t="n">
-        <v>-2334.46</v>
+        <v>-2377.81294117647</v>
       </c>
       <c r="AL134" s="11" t="n">
-        <v>-209977.8835978836</v>
+        <v>-213877.3544973545</v>
       </c>
     </row>
     <row r="135">
@@ -11775,22 +11823,22 @@
         <v>-2537128</v>
       </c>
       <c r="AG135" s="13" t="n">
-        <v>-59530720</v>
+        <v>-104729920</v>
       </c>
       <c r="AH135" s="13" t="n">
-        <v>-3501.80705882353</v>
+        <v>-6160.583529411765</v>
       </c>
       <c r="AI135" s="13" t="n">
-        <v>-314977.3544973545</v>
+        <v>-554126.5608465609</v>
       </c>
       <c r="AJ135" s="13" t="n">
-        <v>-539047912</v>
+        <v>-584247112</v>
       </c>
       <c r="AK135" s="13" t="n">
-        <v>-31708.70070588235</v>
+        <v>-34367.47717647059</v>
       </c>
       <c r="AL135" s="13" t="n">
-        <v>-2852105.354497354</v>
+        <v>-3091254.560846561</v>
       </c>
     </row>
     <row r="136">
@@ -11981,22 +12029,22 @@
         <v>-620735.5185185184</v>
       </c>
       <c r="AG137" s="13" t="n">
-        <v>-4216900</v>
+        <v>-4748900</v>
       </c>
       <c r="AH137" s="13" t="n">
-        <v>-248.0529411764706</v>
+        <v>-279.3470588235294</v>
       </c>
       <c r="AI137" s="13" t="n">
-        <v>-22311.64021164021</v>
+        <v>-25126.45502645503</v>
       </c>
       <c r="AJ137" s="13" t="n">
-        <v>-121535913</v>
+        <v>-122067913</v>
       </c>
       <c r="AK137" s="13" t="n">
-        <v>-7149.171352941176</v>
+        <v>-7180.465470588235</v>
       </c>
       <c r="AL137" s="13" t="n">
-        <v>-643047.1587301586</v>
+        <v>-645861.9735449734</v>
       </c>
     </row>
     <row r="138">
@@ -12169,22 +12217,22 @@
         <v>-9978.835978835979</v>
       </c>
       <c r="AG139" s="13" t="n">
-        <v>-144255</v>
+        <v>-253255</v>
       </c>
       <c r="AH139" s="13" t="n">
-        <v>-8.485588235294118</v>
+        <v>-14.89735294117647</v>
       </c>
       <c r="AI139" s="13" t="n">
-        <v>-763.2539682539683</v>
+        <v>-1339.973544973545</v>
       </c>
       <c r="AJ139" s="13" t="n">
-        <v>-2030255</v>
+        <v>-2139255</v>
       </c>
       <c r="AK139" s="13" t="n">
-        <v>-119.4267647058823</v>
+        <v>-125.8385294117647</v>
       </c>
       <c r="AL139" s="13" t="n">
-        <v>-10742.08994708995</v>
+        <v>-11318.80952380952</v>
       </c>
     </row>
     <row r="140">
@@ -12284,22 +12332,22 @@
         <v>-5569215.973544973</v>
       </c>
       <c r="AG140" s="15" t="n">
-        <v>-69008999</v>
+        <v>-115586199</v>
       </c>
       <c r="AH140" s="15" t="n">
-        <v>-4059.352882352941</v>
+        <v>-6799.188176470589</v>
       </c>
       <c r="AI140" s="15" t="n">
-        <v>-365126.9788359788</v>
+        <v>-611567.1904761905</v>
       </c>
       <c r="AJ140" s="15" t="n">
-        <v>-1121590818</v>
+        <v>-1168168018</v>
       </c>
       <c r="AK140" s="15" t="n">
-        <v>-65975.93047058824</v>
+        <v>-68715.76576470588</v>
       </c>
       <c r="AL140" s="15" t="n">
-        <v>-5934342.952380951</v>
+        <v>-6180783.164021163</v>
       </c>
     </row>
     <row r="141">
@@ -12381,40 +12429,40 @@
         <v>-17101325.59259259</v>
       </c>
       <c r="AA141" s="15" t="n">
-        <v>-4461884406.27</v>
+        <v>-4461868406.27</v>
       </c>
       <c r="AB141" s="15" t="n">
-        <v>-262463.7886041177</v>
+        <v>-262462.8474276471</v>
       </c>
       <c r="AC141" s="15" t="n">
-        <v>-23607854.00142857</v>
+        <v>-23607769.34534392</v>
       </c>
       <c r="AD141" s="15" t="n">
-        <v>-47956493559.17</v>
+        <v>-47956477559.17</v>
       </c>
       <c r="AE141" s="15" t="n">
-        <v>-2820970.209362941</v>
+        <v>-2820969.26818647</v>
       </c>
       <c r="AF141" s="15" t="n">
-        <v>-253738061.1596296</v>
+        <v>-253737976.503545</v>
       </c>
       <c r="AG141" s="15" t="n">
-        <v>-932127074</v>
+        <v>-1520790626</v>
       </c>
       <c r="AH141" s="15" t="n">
-        <v>-54831.00435294118</v>
+        <v>-89458.27211764707</v>
       </c>
       <c r="AI141" s="15" t="n">
-        <v>-4931889.280423281</v>
+        <v>-8046511.248677249</v>
       </c>
       <c r="AJ141" s="15" t="n">
-        <v>-48888620633.17</v>
+        <v>-49477268185.17</v>
       </c>
       <c r="AK141" s="15" t="n">
-        <v>-2875801.213715882</v>
+        <v>-2910427.540304117</v>
       </c>
       <c r="AL141" s="15" t="n">
-        <v>-258669950.4400529</v>
+        <v>-261784487.7522222</v>
       </c>
     </row>
     <row r="142">
@@ -12642,22 +12690,22 @@
         <v>-5281271.338624339</v>
       </c>
       <c r="AG144" s="13" t="n">
-        <v>-9500000</v>
+        <v>-60064418</v>
       </c>
       <c r="AH144" s="13" t="n">
-        <v>-558.8235294117648</v>
+        <v>-3533.201058823529</v>
       </c>
       <c r="AI144" s="13" t="n">
-        <v>-50264.55026455026</v>
+        <v>-317801.1534391535</v>
       </c>
       <c r="AJ144" s="13" t="n">
-        <v>-1007660283</v>
+        <v>-1058224701</v>
       </c>
       <c r="AK144" s="13" t="n">
-        <v>-59274.13429411764</v>
+        <v>-62248.51182352941</v>
       </c>
       <c r="AL144" s="13" t="n">
-        <v>-5331535.888888889</v>
+        <v>-5599072.492063493</v>
       </c>
     </row>
     <row r="145">
@@ -12879,22 +12927,22 @@
         <v>-14123139.06349206</v>
       </c>
       <c r="AG147" s="15" t="n">
-        <v>-9500000</v>
+        <v>-60064418</v>
       </c>
       <c r="AH147" s="15" t="n">
-        <v>-558.8235294117648</v>
+        <v>-3533.201058823529</v>
       </c>
       <c r="AI147" s="15" t="n">
-        <v>-50264.55026455026</v>
+        <v>-317801.1534391535</v>
       </c>
       <c r="AJ147" s="15" t="n">
-        <v>-2678773283</v>
+        <v>-2729337701</v>
       </c>
       <c r="AK147" s="15" t="n">
-        <v>-157574.899</v>
+        <v>-160549.2765294118</v>
       </c>
       <c r="AL147" s="15" t="n">
-        <v>-14173403.61375661</v>
+        <v>-14440940.21693122</v>
       </c>
     </row>
     <row r="148">
@@ -13019,40 +13067,40 @@
         <v>-12271.30158730159</v>
       </c>
       <c r="AA149" s="11" t="n">
-        <v>-1441290</v>
+        <v>-1457290</v>
       </c>
       <c r="AB149" s="11" t="n">
-        <v>-84.78176470588235</v>
+        <v>-85.72294117647058</v>
       </c>
       <c r="AC149" s="11" t="n">
-        <v>-7625.873015873016</v>
+        <v>-7710.5291005291</v>
       </c>
       <c r="AD149" s="11" t="n">
-        <v>-20237187.68</v>
+        <v>-20253187.68</v>
       </c>
       <c r="AE149" s="11" t="n">
-        <v>-1190.422804705882</v>
+        <v>-1191.363981176471</v>
       </c>
       <c r="AF149" s="11" t="n">
-        <v>-107075.0670899471</v>
+        <v>-107159.7231746032</v>
       </c>
       <c r="AG149" s="11" t="n">
-        <v>-600042</v>
+        <v>-1448262</v>
       </c>
       <c r="AH149" s="11" t="n">
-        <v>-35.29658823529412</v>
+        <v>-85.19188235294118</v>
       </c>
       <c r="AI149" s="11" t="n">
-        <v>-3174.825396825397</v>
+        <v>-7662.761904761905</v>
       </c>
       <c r="AJ149" s="11" t="n">
-        <v>-20837229.68</v>
+        <v>-21701449.68</v>
       </c>
       <c r="AK149" s="11" t="n">
-        <v>-1225.719392941176</v>
+        <v>-1276.555863529412</v>
       </c>
       <c r="AL149" s="11" t="n">
-        <v>-110249.8924867725</v>
+        <v>-114822.4850793651</v>
       </c>
     </row>
     <row r="150">
@@ -13662,40 +13710,40 @@
         <v>-1590824.077883598</v>
       </c>
       <c r="AA156" s="15" t="n">
-        <v>-283807215.53</v>
+        <v>-283823215.53</v>
       </c>
       <c r="AB156" s="15" t="n">
-        <v>-16694.54209</v>
+        <v>-16695.48326647059</v>
       </c>
       <c r="AC156" s="15" t="n">
-        <v>-1501625.478994709</v>
+        <v>-1501710.135079365</v>
       </c>
       <c r="AD156" s="15" t="n">
-        <v>-6253995472.77</v>
+        <v>-6254011472.77</v>
       </c>
       <c r="AE156" s="15" t="n">
-        <v>-367882.0866335295</v>
+        <v>-367883.0278100001</v>
       </c>
       <c r="AF156" s="15" t="n">
-        <v>-33089923.13634921</v>
+        <v>-33090007.79243387</v>
       </c>
       <c r="AG156" s="15" t="n">
-        <v>-176828318</v>
+        <v>-177676538</v>
       </c>
       <c r="AH156" s="15" t="n">
-        <v>-10401.66576470588</v>
+        <v>-10451.56105882353</v>
       </c>
       <c r="AI156" s="15" t="n">
-        <v>-935599.5661375661</v>
+        <v>-940087.5026455027</v>
       </c>
       <c r="AJ156" s="15" t="n">
-        <v>-6430823790.77</v>
+        <v>-6431688010.77</v>
       </c>
       <c r="AK156" s="15" t="n">
-        <v>-378283.7523982353</v>
+        <v>-378334.5888688236</v>
       </c>
       <c r="AL156" s="15" t="n">
-        <v>-34025522.70248678</v>
+        <v>-34030095.29507937</v>
       </c>
     </row>
     <row r="157">
@@ -13795,22 +13843,22 @@
         <v>-1609397741.344392</v>
       </c>
       <c r="AG157" s="19" t="n">
-        <v>-4672824291</v>
+        <v>-12498172521</v>
       </c>
       <c r="AH157" s="19" t="n">
-        <v>-274872.017117647</v>
+        <v>-735186.618882353</v>
       </c>
       <c r="AI157" s="19" t="n">
-        <v>-24723938.04761905</v>
+        <v>-66127896.93650793</v>
       </c>
       <c r="AJ157" s="19" t="n">
-        <v>-308848997405.09</v>
+        <v>-316674345635.09</v>
       </c>
       <c r="AK157" s="19" t="n">
-        <v>-18167588.08265235</v>
+        <v>-18627902.68441706</v>
       </c>
       <c r="AL157" s="19" t="n">
-        <v>-1634121679.392011</v>
+        <v>-1675525638.2809</v>
       </c>
     </row>
     <row r="158">
@@ -13910,22 +13958,22 @@
         <v>-277217918.5799472</v>
       </c>
       <c r="AG158" s="19" t="n">
-        <v>8853440492</v>
+        <v>1031929162</v>
       </c>
       <c r="AH158" s="19" t="n">
-        <v>520790.6171764706</v>
+        <v>60701.71541176471</v>
       </c>
       <c r="AI158" s="19" t="n">
-        <v>46843600.48677249</v>
+        <v>5459942.656084656</v>
       </c>
       <c r="AJ158" s="19" t="n">
-        <v>-43540746119.61</v>
+        <v>-51362257449.61</v>
       </c>
       <c r="AK158" s="19" t="n">
-        <v>-2561220.35997706</v>
+        <v>-3021309.261741766</v>
       </c>
       <c r="AL158" s="19" t="n">
-        <v>-230374318.0931748</v>
+        <v>-271757975.9238626</v>
       </c>
     </row>
     <row r="159">
@@ -14025,22 +14073,22 @@
         <v>79785577.85582009</v>
       </c>
       <c r="AG159" s="7" t="n">
-        <v>23932914706.75</v>
+        <v>16111403376.75</v>
       </c>
       <c r="AH159" s="7" t="n">
-        <v>1407818.512161765</v>
+        <v>947729.6103970588</v>
       </c>
       <c r="AI159" s="7" t="n">
-        <v>126629178.3425926</v>
+        <v>85245520.51190476</v>
       </c>
       <c r="AJ159" s="7" t="n">
-        <v>23932914706.75</v>
+        <v>16111403376.75</v>
       </c>
       <c r="AK159" s="7" t="n">
-        <v>1407818.512161765</v>
+        <v>947729.6103970588</v>
       </c>
       <c r="AL159" s="7" t="n">
-        <v>126629178.3425926</v>
+        <v>85245520.51190476</v>
       </c>
     </row>
   </sheetData>
@@ -14843,16 +14891,16 @@
         <v>14828882907</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>7548561035</v>
+        <v>128516414</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>22377443942</v>
+        <v>14957399321</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>1316320.231882353</v>
+        <v>879847.018882353</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>118399174.2962963</v>
+        <v>79139678.94708994</v>
       </c>
     </row>
     <row r="7">
@@ -14875,16 +14923,16 @@
         <v>18099375</v>
       </c>
       <c r="E7" s="13" t="n">
-        <v>23771724</v>
+        <v>23761724</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>41871099</v>
+        <v>41861099</v>
       </c>
       <c r="G7" s="24" t="n">
-        <v>2463.005823529412</v>
+        <v>2462.417588235294</v>
       </c>
       <c r="H7" s="24" t="n">
-        <v>221540.2063492064</v>
+        <v>221487.2962962963</v>
       </c>
     </row>
     <row r="8">
@@ -14939,16 +14987,16 @@
         <v>22400563.84000001</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>57810636</v>
+        <v>434113840</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>80211199.84</v>
+        <v>456514403.84</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>4718.305872941177</v>
+        <v>26853.78846117647</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>424397.8827513228</v>
+        <v>2415420.126137566</v>
       </c>
     </row>
     <row r="10">
@@ -15003,16 +15051,16 @@
         <v>175445396.6500001</v>
       </c>
       <c r="E11" s="13" t="n">
-        <v>-100832142</v>
+        <v>445512184</v>
       </c>
       <c r="F11" s="13" t="n">
-        <v>74613254.65000007</v>
+        <v>620957580.6500001</v>
       </c>
       <c r="G11" s="24" t="n">
-        <v>4389.014979411769</v>
+        <v>36526.91650882354</v>
       </c>
       <c r="H11" s="24" t="n">
-        <v>394779.1251322755</v>
+        <v>3285489.844708995</v>
       </c>
     </row>
     <row r="12">
@@ -15058,13 +15106,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>22608810469.75</v>
+        <v>16111403378.75</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>1329930.027632353</v>
+        <v>947729.6105147058</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>119623335.8187831</v>
+        <v>85245520.52248676</v>
       </c>
     </row>
   </sheetData>
@@ -15137,7 +15185,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 13 Oct 2026 09:33 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 15 Oct 2026 17:02 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -15219,14 +15267,14 @@
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 13 Oct 2026</t>
+          <t>MTD as of 15 Oct 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
       <c r="AI3" s="4" t="n"/>
       <c r="AJ3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 13 Oct 2026</t>
+          <t>YTD as of 15 Oct 2026</t>
         </is>
       </c>
       <c r="AK3" s="4" t="n"/>
@@ -16733,22 +16781,22 @@
         <v>2.521134965502646</v>
       </c>
       <c r="AG20" s="13" t="n">
-        <v>9.044499999999999</v>
+        <v>12.8814</v>
       </c>
       <c r="AH20" s="13" t="n">
-        <v>0.0005320294117647058</v>
+        <v>0.0007577294117647058</v>
       </c>
       <c r="AI20" s="13" t="n">
-        <v>0.04785449735449735</v>
+        <v>0.06815555555555555</v>
       </c>
       <c r="AJ20" s="13" t="n">
-        <v>485.53900848</v>
+        <v>489.37590848</v>
       </c>
       <c r="AK20" s="13" t="n">
-        <v>0.02856111814588235</v>
+        <v>0.02878681814588235</v>
       </c>
       <c r="AL20" s="13" t="n">
-        <v>2.568989462857143</v>
+        <v>2.589290521058202</v>
       </c>
     </row>
     <row r="21">
@@ -17006,22 +17054,22 @@
         <v>0.4919761904761905</v>
       </c>
       <c r="AG23" s="11" t="n">
-        <v>8.044499999999999</v>
+        <v>10.2495</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>0.0004732058823529411</v>
+        <v>0.0006029117647058823</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>0.04256349206349206</v>
+        <v>0.05423015873015873</v>
       </c>
       <c r="AJ23" s="11" t="n">
-        <v>101.028</v>
+        <v>103.233</v>
       </c>
       <c r="AK23" s="11" t="n">
-        <v>0.005942823529411766</v>
+        <v>0.006072529411764707</v>
       </c>
       <c r="AL23" s="11" t="n">
-        <v>0.5345396825396825</v>
+        <v>0.5462063492063491</v>
       </c>
     </row>
     <row r="24">
@@ -17358,17 +17406,23 @@
       <c r="AF28" s="13" t="n">
         <v>0.06546620105820106</v>
       </c>
-      <c r="AG28" s="13" t="n"/>
-      <c r="AH28" s="13" t="n"/>
-      <c r="AI28" s="13" t="n"/>
+      <c r="AG28" s="13" t="n">
+        <v>1.6319</v>
+      </c>
+      <c r="AH28" s="13" t="n">
+        <v>9.599411764705882e-05</v>
+      </c>
+      <c r="AI28" s="13" t="n">
+        <v>0.008634391534391534</v>
+      </c>
       <c r="AJ28" s="13" t="n">
-        <v>12.373112</v>
+        <v>14.005012</v>
       </c>
       <c r="AK28" s="13" t="n">
-        <v>0.0007278301176470588</v>
+        <v>0.0008238242352941177</v>
       </c>
       <c r="AL28" s="13" t="n">
-        <v>0.06546620105820106</v>
+        <v>0.07410059259259259</v>
       </c>
     </row>
     <row r="29">
@@ -18552,22 +18606,22 @@
         <v>1332.179822764444</v>
       </c>
       <c r="AG45" s="15" t="n">
-        <v>13526.264783</v>
+        <v>13530.101683</v>
       </c>
       <c r="AH45" s="15" t="n">
-        <v>0.7956626342941177</v>
+        <v>0.7958883342941176</v>
       </c>
       <c r="AI45" s="15" t="n">
-        <v>71.56753853439153</v>
+        <v>71.5878395925926</v>
       </c>
       <c r="AJ45" s="15" t="n">
-        <v>265308.25128548</v>
+        <v>265312.08818548</v>
       </c>
       <c r="AK45" s="15" t="n">
-        <v>15.60636772267529</v>
+        <v>15.60659342267529</v>
       </c>
       <c r="AL45" s="15" t="n">
-        <v>1403.747361298836</v>
+        <v>1403.767662357037</v>
       </c>
     </row>
     <row r="46">
@@ -18892,17 +18946,23 @@
       <c r="AF50" s="11" t="n">
         <v>-4.462156708994709</v>
       </c>
-      <c r="AG50" s="11" t="n"/>
-      <c r="AH50" s="11" t="n"/>
-      <c r="AI50" s="11" t="n"/>
+      <c r="AG50" s="11" t="n">
+        <v>-398.598156</v>
+      </c>
+      <c r="AH50" s="11" t="n">
+        <v>-0.02344695035294118</v>
+      </c>
+      <c r="AI50" s="11" t="n">
+        <v>-2.108984952380952</v>
+      </c>
       <c r="AJ50" s="11" t="n">
-        <v>-843.3476179999999</v>
+        <v>-1241.945774</v>
       </c>
       <c r="AK50" s="11" t="n">
-        <v>-0.04960868341176471</v>
+        <v>-0.07305563376470589</v>
       </c>
       <c r="AL50" s="11" t="n">
-        <v>-4.462156708994709</v>
+        <v>-6.571141661375661</v>
       </c>
     </row>
     <row r="51">
@@ -19075,22 +19135,22 @@
         <v>-0.9861469047619047</v>
       </c>
       <c r="AG52" s="11" t="n">
-        <v>-46.95078</v>
+        <v>-47.90427</v>
       </c>
       <c r="AH52" s="11" t="n">
-        <v>-0.002761810588235294</v>
+        <v>-0.002817898235294118</v>
       </c>
       <c r="AI52" s="11" t="n">
-        <v>-0.2484168253968254</v>
+        <v>-0.253461746031746</v>
       </c>
       <c r="AJ52" s="11" t="n">
-        <v>-233.332545</v>
+        <v>-234.286035</v>
       </c>
       <c r="AK52" s="11" t="n">
-        <v>-0.01372544382352941</v>
+        <v>-0.01378153147058823</v>
       </c>
       <c r="AL52" s="11" t="n">
-        <v>-1.23456373015873</v>
+        <v>-1.239608650793651</v>
       </c>
     </row>
     <row r="53">
@@ -19306,22 +19366,22 @@
         <v>-10.23762965079365</v>
       </c>
       <c r="AG55" s="13" t="n">
-        <v>-492.54</v>
+        <v>-517.41625</v>
       </c>
       <c r="AH55" s="13" t="n">
-        <v>-0.02897294117647059</v>
+        <v>-0.03043625</v>
       </c>
       <c r="AI55" s="13" t="n">
-        <v>-2.606031746031746</v>
+        <v>-2.737652116402116</v>
       </c>
       <c r="AJ55" s="13" t="n">
-        <v>-2427.452004</v>
+        <v>-2452.328254</v>
       </c>
       <c r="AK55" s="13" t="n">
-        <v>-0.1427912943529412</v>
+        <v>-0.1442546031764706</v>
       </c>
       <c r="AL55" s="13" t="n">
-        <v>-12.8436613968254</v>
+        <v>-12.97528176719577</v>
       </c>
     </row>
     <row r="56">
@@ -20034,22 +20094,22 @@
         <v>-95.0060828141799</v>
       </c>
       <c r="AG63" s="15" t="n">
-        <v>-891.781311</v>
+        <v>-1316.209207</v>
       </c>
       <c r="AH63" s="15" t="n">
-        <v>-0.05245772417647059</v>
+        <v>-0.07742407100000001</v>
       </c>
       <c r="AI63" s="15" t="n">
-        <v>-4.718419634920635</v>
+        <v>-6.964069878306879</v>
       </c>
       <c r="AJ63" s="15" t="n">
-        <v>-18847.93096288</v>
+        <v>-19272.35885888</v>
       </c>
       <c r="AK63" s="15" t="n">
-        <v>-1.108701821345882</v>
+        <v>-1.133668168169412</v>
       </c>
       <c r="AL63" s="15" t="n">
-        <v>-99.72450244910054</v>
+        <v>-101.9701526924868</v>
       </c>
     </row>
     <row r="64">
@@ -21162,22 +21222,22 @@
         <v>-53.01535581481481</v>
       </c>
       <c r="AG81" s="11" t="n">
-        <v>-903.478933</v>
+        <v>-4492.646413</v>
       </c>
       <c r="AH81" s="11" t="n">
-        <v>-0.05314581958823529</v>
+        <v>-0.2642733184117647</v>
       </c>
       <c r="AI81" s="11" t="n">
-        <v>-4.780311814814815</v>
+        <v>-23.77061594179894</v>
       </c>
       <c r="AJ81" s="11" t="n">
-        <v>-10923.381182</v>
+        <v>-14512.548662</v>
       </c>
       <c r="AK81" s="11" t="n">
-        <v>-0.6425518342352942</v>
+        <v>-0.8536793330588236</v>
       </c>
       <c r="AL81" s="11" t="n">
-        <v>-57.79566762962963</v>
+        <v>-76.78597175661375</v>
       </c>
     </row>
     <row r="82">
@@ -21277,22 +21337,22 @@
         <v>-58.93422933476191</v>
       </c>
       <c r="AG82" s="13" t="n">
-        <v>-1752.972535</v>
+        <v>-2507.660085</v>
       </c>
       <c r="AH82" s="13" t="n">
-        <v>-0.1031160314705882</v>
+        <v>-0.1475094167647059</v>
       </c>
       <c r="AI82" s="13" t="n">
-        <v>-9.274986957671958</v>
+        <v>-13.26804277777778</v>
       </c>
       <c r="AJ82" s="13" t="n">
-        <v>-12891.54187927</v>
+        <v>-13646.22942927</v>
       </c>
       <c r="AK82" s="13" t="n">
-        <v>-0.7583259928982352</v>
+        <v>-0.8027193781923528</v>
       </c>
       <c r="AL82" s="13" t="n">
-        <v>-68.20921629243387</v>
+        <v>-72.20227211253969</v>
       </c>
     </row>
     <row r="83">
@@ -21391,17 +21451,23 @@
       <c r="AF83" s="11" t="n">
         <v>-56.09650002645503</v>
       </c>
-      <c r="AG83" s="11" t="n"/>
-      <c r="AH83" s="11" t="n"/>
-      <c r="AI83" s="11" t="n"/>
+      <c r="AG83" s="11" t="n">
+        <v>-2411.754594</v>
+      </c>
+      <c r="AH83" s="11" t="n">
+        <v>-0.1418679172941177</v>
+      </c>
+      <c r="AI83" s="11" t="n">
+        <v>-12.76060631746032</v>
+      </c>
       <c r="AJ83" s="11" t="n">
-        <v>-10602.238505</v>
+        <v>-13013.993099</v>
       </c>
       <c r="AK83" s="11" t="n">
-        <v>-0.6236610885294117</v>
+        <v>-0.7655290058235293</v>
       </c>
       <c r="AL83" s="11" t="n">
-        <v>-56.09650002645503</v>
+        <v>-68.85710634391535</v>
       </c>
     </row>
     <row r="84">
@@ -21501,22 +21567,22 @@
         <v>-2.427178873015873</v>
       </c>
       <c r="AG84" s="13" t="n">
-        <v>-6.13612</v>
+        <v>-11.37064</v>
       </c>
       <c r="AH84" s="13" t="n">
-        <v>-0.0003609482352941177</v>
+        <v>-0.0006688611764705882</v>
       </c>
       <c r="AI84" s="13" t="n">
-        <v>-0.03246624338624338</v>
+        <v>-0.0601621164021164</v>
       </c>
       <c r="AJ84" s="13" t="n">
-        <v>-464.8729270000001</v>
+        <v>-470.107447</v>
       </c>
       <c r="AK84" s="13" t="n">
-        <v>-0.02734546629411765</v>
+        <v>-0.02765337923529412</v>
       </c>
       <c r="AL84" s="13" t="n">
-        <v>-2.459645116402116</v>
+        <v>-2.487340989417989</v>
       </c>
     </row>
     <row r="85">
@@ -21616,22 +21682,22 @@
         <v>-170.4732640490476</v>
       </c>
       <c r="AG85" s="15" t="n">
-        <v>-2662.587588</v>
+        <v>-9423.431731999999</v>
       </c>
       <c r="AH85" s="15" t="n">
-        <v>-0.1566227992941176</v>
+        <v>-0.5543195136470588</v>
       </c>
       <c r="AI85" s="15" t="n">
-        <v>-14.08776501587302</v>
+        <v>-49.85942715343915</v>
       </c>
       <c r="AJ85" s="15" t="n">
-        <v>-34882.03449327</v>
+        <v>-41642.87863727</v>
       </c>
       <c r="AK85" s="15" t="n">
-        <v>-2.051884381957059</v>
+        <v>-2.44958109631</v>
       </c>
       <c r="AL85" s="15" t="n">
-        <v>-184.5610290649206</v>
+        <v>-220.3326912024868</v>
       </c>
     </row>
     <row r="86">
@@ -21817,22 +21883,22 @@
         <v>-0.778818253968254</v>
       </c>
       <c r="AG88" s="11" t="n">
-        <v>-0.874372</v>
+        <v>-10.466372</v>
       </c>
       <c r="AH88" s="11" t="n">
-        <v>-5.143364705882353e-05</v>
+        <v>-0.0006156689411764706</v>
       </c>
       <c r="AI88" s="11" t="n">
-        <v>-0.004626306878306879</v>
+        <v>-0.05537762962962963</v>
       </c>
       <c r="AJ88" s="11" t="n">
-        <v>-148.071022</v>
+        <v>-157.663022</v>
       </c>
       <c r="AK88" s="11" t="n">
-        <v>-0.008710060117647057</v>
+        <v>-0.009274295411764704</v>
       </c>
       <c r="AL88" s="11" t="n">
-        <v>-0.7834445608465609</v>
+        <v>-0.8341958835978837</v>
       </c>
     </row>
     <row r="89">
@@ -21974,17 +22040,23 @@
       <c r="AF90" s="11" t="n">
         <v>-1.035486037037037</v>
       </c>
-      <c r="AG90" s="11" t="n"/>
-      <c r="AH90" s="11" t="n"/>
-      <c r="AI90" s="11" t="n"/>
+      <c r="AG90" s="11" t="n">
+        <v>-0.5047</v>
+      </c>
+      <c r="AH90" s="11" t="n">
+        <v>-2.968823529411765e-05</v>
+      </c>
+      <c r="AI90" s="11" t="n">
+        <v>-0.002670370370370371</v>
+      </c>
       <c r="AJ90" s="11" t="n">
-        <v>-195.706861</v>
+        <v>-196.211561</v>
       </c>
       <c r="AK90" s="11" t="n">
-        <v>-0.01151216829411765</v>
+        <v>-0.01154185652941176</v>
       </c>
       <c r="AL90" s="11" t="n">
-        <v>-1.035486037037037</v>
+        <v>-1.038156407407407</v>
       </c>
     </row>
     <row r="91">
@@ -22053,17 +22125,23 @@
       <c r="AF91" s="13" t="n">
         <v>-0.008838981164021162</v>
       </c>
-      <c r="AG91" s="13" t="n"/>
-      <c r="AH91" s="13" t="n"/>
-      <c r="AI91" s="13" t="n"/>
+      <c r="AG91" s="13" t="n">
+        <v>-0.7025</v>
+      </c>
+      <c r="AH91" s="13" t="n">
+        <v>-4.132352941176471e-05</v>
+      </c>
+      <c r="AI91" s="13" t="n">
+        <v>-0.003716931216931217</v>
+      </c>
       <c r="AJ91" s="13" t="n">
-        <v>-1.67056744</v>
+        <v>-2.37306744</v>
       </c>
       <c r="AK91" s="13" t="n">
-        <v>-9.826867294117647e-05</v>
+        <v>-0.0001395922023529412</v>
       </c>
       <c r="AL91" s="13" t="n">
-        <v>-0.008838981164021162</v>
+        <v>-0.01255591238095238</v>
       </c>
     </row>
     <row r="92">
@@ -22266,22 +22344,22 @@
         <v>-0.01277881481481482</v>
       </c>
       <c r="AG93" s="13" t="n">
-        <v>-0.2336</v>
+        <v>-0.2976</v>
       </c>
       <c r="AH93" s="13" t="n">
-        <v>-1.374117647058823e-05</v>
+        <v>-1.750588235294118e-05</v>
       </c>
       <c r="AI93" s="13" t="n">
-        <v>-0.001235978835978836</v>
+        <v>-0.001574603174603175</v>
       </c>
       <c r="AJ93" s="13" t="n">
-        <v>-2.648796</v>
+        <v>-2.712796</v>
       </c>
       <c r="AK93" s="13" t="n">
-        <v>-0.0001558115294117647</v>
+        <v>-0.0001595762352941177</v>
       </c>
       <c r="AL93" s="13" t="n">
-        <v>-0.01401479365079365</v>
+        <v>-0.01435341798941799</v>
       </c>
     </row>
     <row r="94">
@@ -22381,22 +22459,22 @@
         <v>-2.636230425608466</v>
       </c>
       <c r="AG94" s="15" t="n">
-        <v>-2.973672</v>
+        <v>-13.836872</v>
       </c>
       <c r="AH94" s="15" t="n">
-        <v>-0.0001749218823529412</v>
+        <v>-0.0008139336470588235</v>
       </c>
       <c r="AI94" s="15" t="n">
-        <v>-0.01573371428571428</v>
+        <v>-0.07321096296296296</v>
       </c>
       <c r="AJ94" s="15" t="n">
-        <v>-501.2212224400001</v>
+        <v>-512.08442244</v>
       </c>
       <c r="AK94" s="15" t="n">
-        <v>-0.02948360132</v>
+        <v>-0.03012261308470588</v>
       </c>
       <c r="AL94" s="15" t="n">
-        <v>-2.65196413989418</v>
+        <v>-2.709441388571429</v>
       </c>
     </row>
     <row r="95">
@@ -22576,22 +22654,22 @@
         <v>-0.4714513227513227</v>
       </c>
       <c r="AG97" s="13" t="n">
-        <v>-0.531541</v>
+        <v>-76.331541</v>
       </c>
       <c r="AH97" s="13" t="n">
-        <v>-3.126711764705883e-05</v>
+        <v>-0.004490090647058824</v>
       </c>
       <c r="AI97" s="13" t="n">
-        <v>-0.002812386243386244</v>
+        <v>-0.4038705873015873</v>
       </c>
       <c r="AJ97" s="13" t="n">
-        <v>-89.63584100000001</v>
+        <v>-165.435841</v>
       </c>
       <c r="AK97" s="13" t="n">
-        <v>-0.005272696529411766</v>
+        <v>-0.00973152005882353</v>
       </c>
       <c r="AL97" s="13" t="n">
-        <v>-0.474263708994709</v>
+        <v>-0.87532191005291</v>
       </c>
     </row>
     <row r="98">
@@ -22691,22 +22769,22 @@
         <v>-1.418156079365079</v>
       </c>
       <c r="AG98" s="11" t="n">
-        <v>-112.897</v>
+        <v>-128.353307</v>
       </c>
       <c r="AH98" s="11" t="n">
-        <v>-0.006641</v>
+        <v>-0.007550194529411765</v>
       </c>
       <c r="AI98" s="11" t="n">
-        <v>-0.5973386243386244</v>
+        <v>-0.6791180264550265</v>
       </c>
       <c r="AJ98" s="11" t="n">
-        <v>-380.928499</v>
+        <v>-396.384806</v>
       </c>
       <c r="AK98" s="11" t="n">
-        <v>-0.02240755876470588</v>
+        <v>-0.02331675329411765</v>
       </c>
       <c r="AL98" s="11" t="n">
-        <v>-2.015494703703704</v>
+        <v>-2.097274105820106</v>
       </c>
     </row>
     <row r="99">
@@ -22921,22 +22999,22 @@
         <v>-1.318975026455027</v>
       </c>
       <c r="AG100" s="11" t="n">
-        <v>-7.999429</v>
+        <v>-51.709011</v>
       </c>
       <c r="AH100" s="11" t="n">
-        <v>-0.0004705546470588235</v>
+        <v>-0.003041706529411764</v>
       </c>
       <c r="AI100" s="11" t="n">
-        <v>-0.04232502116402116</v>
+        <v>-0.2735926507936507</v>
       </c>
       <c r="AJ100" s="11" t="n">
-        <v>-257.285709</v>
+        <v>-300.995291</v>
       </c>
       <c r="AK100" s="11" t="n">
-        <v>-0.01513445347058823</v>
+        <v>-0.01770560535294118</v>
       </c>
       <c r="AL100" s="11" t="n">
-        <v>-1.361300047619048</v>
+        <v>-1.592567677248677</v>
       </c>
     </row>
     <row r="101">
@@ -23036,22 +23114,22 @@
         <v>-1.928168555555555</v>
       </c>
       <c r="AG101" s="13" t="n">
-        <v>-4.33215</v>
+        <v>-4.72565</v>
       </c>
       <c r="AH101" s="13" t="n">
-        <v>-0.0002548323529411765</v>
+        <v>-0.0002779794117647059</v>
       </c>
       <c r="AI101" s="13" t="n">
-        <v>-0.02292142857142857</v>
+        <v>-0.02500343915343915</v>
       </c>
       <c r="AJ101" s="13" t="n">
-        <v>-368.756007</v>
+        <v>-369.149507</v>
       </c>
       <c r="AK101" s="13" t="n">
-        <v>-0.02169152982352941</v>
+        <v>-0.02171467688235294</v>
       </c>
       <c r="AL101" s="13" t="n">
-        <v>-1.951089984126984</v>
+        <v>-1.953171994708994</v>
       </c>
     </row>
     <row r="102">
@@ -23151,22 +23229,22 @@
         <v>-46.20353251708994</v>
       </c>
       <c r="AG102" s="15" t="n">
-        <v>-277.376094</v>
+        <v>-412.735483</v>
       </c>
       <c r="AH102" s="15" t="n">
-        <v>-0.01631624082352941</v>
+        <v>-0.02427855782352941</v>
       </c>
       <c r="AI102" s="15" t="n">
-        <v>-1.467598380952381</v>
+        <v>-2.183785624338624</v>
       </c>
       <c r="AJ102" s="15" t="n">
-        <v>-9009.84373973</v>
+        <v>-9145.203128730001</v>
       </c>
       <c r="AK102" s="15" t="n">
-        <v>-0.5299908082194118</v>
+        <v>-0.5379531252194117</v>
       </c>
       <c r="AL102" s="15" t="n">
-        <v>-47.67113089804232</v>
+        <v>-48.38731814142857</v>
       </c>
     </row>
     <row r="103">
@@ -23309,22 +23387,22 @@
         <v>-1.237435248677249</v>
       </c>
       <c r="AG104" s="11" t="n">
-        <v>-17.0946</v>
+        <v>-22.0467</v>
       </c>
       <c r="AH104" s="11" t="n">
-        <v>-0.001005564705882353</v>
+        <v>-0.001296864705882353</v>
       </c>
       <c r="AI104" s="11" t="n">
-        <v>-0.09044761904761904</v>
+        <v>-0.1166492063492063</v>
       </c>
       <c r="AJ104" s="11" t="n">
-        <v>-250.969862</v>
+        <v>-255.921962</v>
       </c>
       <c r="AK104" s="11" t="n">
-        <v>-0.01476293305882353</v>
+        <v>-0.01505423305882353</v>
       </c>
       <c r="AL104" s="11" t="n">
-        <v>-1.327882867724868</v>
+        <v>-1.354084455026455</v>
       </c>
     </row>
     <row r="105">
@@ -23424,22 +23502,22 @@
         <v>-1.864747592592592</v>
       </c>
       <c r="AG105" s="13" t="n">
-        <v>-161.522493</v>
+        <v>-170.282139</v>
       </c>
       <c r="AH105" s="13" t="n">
-        <v>-0.00950132311764706</v>
+        <v>-0.01001659641176471</v>
       </c>
       <c r="AI105" s="13" t="n">
-        <v>-0.8546163650793651</v>
+        <v>-0.9009636984126984</v>
       </c>
       <c r="AJ105" s="13" t="n">
-        <v>-513.959788</v>
+        <v>-522.719434</v>
       </c>
       <c r="AK105" s="13" t="n">
-        <v>-0.03023292870588235</v>
+        <v>-0.030748202</v>
       </c>
       <c r="AL105" s="13" t="n">
-        <v>-2.719363957671958</v>
+        <v>-2.765711291005291</v>
       </c>
     </row>
     <row r="106">
@@ -23539,22 +23617,22 @@
         <v>-8.926693243386243</v>
       </c>
       <c r="AG106" s="11" t="n">
-        <v>-70.776068</v>
+        <v>-136.708815</v>
       </c>
       <c r="AH106" s="11" t="n">
-        <v>-0.004163298117647059</v>
+        <v>-0.008041695</v>
       </c>
       <c r="AI106" s="11" t="n">
-        <v>-0.3744765502645502</v>
+        <v>-0.7233270634920634</v>
       </c>
       <c r="AJ106" s="11" t="n">
-        <v>-1757.921091</v>
+        <v>-1823.853838</v>
       </c>
       <c r="AK106" s="11" t="n">
-        <v>-0.103407123</v>
+        <v>-0.1072855198823529</v>
       </c>
       <c r="AL106" s="11" t="n">
-        <v>-9.301169793650793</v>
+        <v>-9.650020306878307</v>
       </c>
     </row>
     <row r="107">
@@ -23648,22 +23726,22 @@
         <v>-1.059205370370371</v>
       </c>
       <c r="AG107" s="13" t="n">
-        <v>-34.937225</v>
+        <v>-59.088825</v>
       </c>
       <c r="AH107" s="13" t="n">
-        <v>-0.002055130882352941</v>
+        <v>-0.003475813235294117</v>
       </c>
       <c r="AI107" s="13" t="n">
-        <v>-0.1848530423280423</v>
+        <v>-0.3126392857142857</v>
       </c>
       <c r="AJ107" s="13" t="n">
-        <v>-235.12704</v>
+        <v>-259.27864</v>
       </c>
       <c r="AK107" s="13" t="n">
-        <v>-0.01383100235294118</v>
+        <v>-0.01525168470588235</v>
       </c>
       <c r="AL107" s="13" t="n">
-        <v>-1.244058412698413</v>
+        <v>-1.371844656084656</v>
       </c>
     </row>
     <row r="108">
@@ -23763,22 +23841,22 @@
         <v>-13.08808145502645</v>
       </c>
       <c r="AG108" s="15" t="n">
-        <v>-284.330386</v>
+        <v>-388.126479</v>
       </c>
       <c r="AH108" s="15" t="n">
-        <v>-0.01672531682352941</v>
+        <v>-0.02283096935294118</v>
       </c>
       <c r="AI108" s="15" t="n">
-        <v>-1.504393576719577</v>
+        <v>-2.053579253968254</v>
       </c>
       <c r="AJ108" s="15" t="n">
-        <v>-2757.977781</v>
+        <v>-2861.773874</v>
       </c>
       <c r="AK108" s="15" t="n">
-        <v>-0.162233987117647</v>
+        <v>-0.1683396396470588</v>
       </c>
       <c r="AL108" s="15" t="n">
-        <v>-14.59247503174603</v>
+        <v>-15.14166070899471</v>
       </c>
     </row>
     <row r="109">
@@ -24097,22 +24175,22 @@
         <v>-2.48763974074074</v>
       </c>
       <c r="AG112" s="11" t="n">
-        <v>-21.5875</v>
+        <v>-22.039</v>
       </c>
       <c r="AH112" s="11" t="n">
-        <v>-0.00126985294117647</v>
+        <v>-0.001296411764705883</v>
       </c>
       <c r="AI112" s="11" t="n">
-        <v>-0.1142195767195767</v>
+        <v>-0.1166084656084656</v>
       </c>
       <c r="AJ112" s="11" t="n">
-        <v>-491.751411</v>
+        <v>-492.202911</v>
       </c>
       <c r="AK112" s="11" t="n">
-        <v>-0.02892655358823529</v>
+        <v>-0.02895311241176471</v>
       </c>
       <c r="AL112" s="11" t="n">
-        <v>-2.601859317460317</v>
+        <v>-2.604248206349206</v>
       </c>
     </row>
     <row r="113">
@@ -24212,22 +24290,22 @@
         <v>-3.302494767195767</v>
       </c>
       <c r="AG113" s="15" t="n">
-        <v>-21.5875</v>
+        <v>-22.039</v>
       </c>
       <c r="AH113" s="15" t="n">
-        <v>-0.00126985294117647</v>
+        <v>-0.001296411764705883</v>
       </c>
       <c r="AI113" s="15" t="n">
-        <v>-0.1142195767195767</v>
+        <v>-0.1166084656084656</v>
       </c>
       <c r="AJ113" s="15" t="n">
-        <v>-645.7590109999999</v>
+        <v>-646.2105109999999</v>
       </c>
       <c r="AK113" s="15" t="n">
-        <v>-0.03798582417647058</v>
+        <v>-0.03801238299999999</v>
       </c>
       <c r="AL113" s="15" t="n">
-        <v>-3.416714343915344</v>
+        <v>-3.419103232804233</v>
       </c>
     </row>
     <row r="114">
@@ -24364,22 +24442,22 @@
         <v>-2.418823142857143</v>
       </c>
       <c r="AG115" s="11" t="n">
-        <v>-37.104</v>
+        <v>-59.994</v>
       </c>
       <c r="AH115" s="11" t="n">
-        <v>-0.002182588235294118</v>
+        <v>-0.003529058823529412</v>
       </c>
       <c r="AI115" s="11" t="n">
-        <v>-0.1963174603174603</v>
+        <v>-0.3174285714285714</v>
       </c>
       <c r="AJ115" s="11" t="n">
-        <v>-494.2615740000001</v>
+        <v>-517.1515740000001</v>
       </c>
       <c r="AK115" s="11" t="n">
-        <v>-0.02907421023529412</v>
+        <v>-0.03042068082352941</v>
       </c>
       <c r="AL115" s="11" t="n">
-        <v>-2.615140603174603</v>
+        <v>-2.736251714285714</v>
       </c>
     </row>
     <row r="116">
@@ -24540,22 +24618,22 @@
         <v>-0.7151995291005291</v>
       </c>
       <c r="AG117" s="11" t="n">
-        <v>-12.74</v>
+        <v>-15.24</v>
       </c>
       <c r="AH117" s="11" t="n">
-        <v>-0.0007494117647058823</v>
+        <v>-0.0008964705882352941</v>
       </c>
       <c r="AI117" s="11" t="n">
-        <v>-0.0674074074074074</v>
+        <v>-0.08063492063492064</v>
       </c>
       <c r="AJ117" s="11" t="n">
-        <v>-147.912711</v>
+        <v>-150.412711</v>
       </c>
       <c r="AK117" s="11" t="n">
-        <v>-0.008700747705882353</v>
+        <v>-0.008847806529411764</v>
       </c>
       <c r="AL117" s="11" t="n">
-        <v>-0.7826069365079364</v>
+        <v>-0.7958344497354497</v>
       </c>
     </row>
     <row r="118">
@@ -24655,22 +24733,22 @@
         <v>-2.977326375661375</v>
       </c>
       <c r="AG118" s="13" t="n">
-        <v>-14.652</v>
+        <v>-37.873475</v>
       </c>
       <c r="AH118" s="13" t="n">
-        <v>-0.0008618823529411764</v>
+        <v>-0.002227851470588235</v>
       </c>
       <c r="AI118" s="13" t="n">
-        <v>-0.07752380952380952</v>
+        <v>-0.2003887566137566</v>
       </c>
       <c r="AJ118" s="13" t="n">
-        <v>-577.3666850000001</v>
+        <v>-600.58816</v>
       </c>
       <c r="AK118" s="13" t="n">
-        <v>-0.03396274617647059</v>
+        <v>-0.03532871529411765</v>
       </c>
       <c r="AL118" s="13" t="n">
-        <v>-3.054850185185185</v>
+        <v>-3.177715132275132</v>
       </c>
     </row>
     <row r="119">
@@ -24770,22 +24848,22 @@
         <v>-6.180132116402117</v>
       </c>
       <c r="AG119" s="15" t="n">
-        <v>-64.496</v>
+        <v>-113.107475</v>
       </c>
       <c r="AH119" s="15" t="n">
-        <v>-0.003793882352941176</v>
+        <v>-0.006653380882352941</v>
       </c>
       <c r="AI119" s="15" t="n">
-        <v>-0.3412486772486772</v>
+        <v>-0.5984522486772487</v>
       </c>
       <c r="AJ119" s="15" t="n">
-        <v>-1232.54097</v>
+        <v>-1281.152445</v>
       </c>
       <c r="AK119" s="15" t="n">
-        <v>-0.07250241</v>
+        <v>-0.07536190852941177</v>
       </c>
       <c r="AL119" s="15" t="n">
-        <v>-6.521380793650794</v>
+        <v>-6.778584365079365</v>
       </c>
     </row>
     <row r="120">
@@ -24971,40 +25049,40 @@
         <v>-5.643998698412699</v>
       </c>
       <c r="AA122" s="13" t="n">
-        <v>-942.329623</v>
+        <v>-942.313623</v>
       </c>
       <c r="AB122" s="13" t="n">
-        <v>-0.05543115429411764</v>
+        <v>-0.05543021311764706</v>
       </c>
       <c r="AC122" s="13" t="n">
-        <v>-4.985871021164021</v>
+        <v>-4.985786365079365</v>
       </c>
       <c r="AD122" s="13" t="n">
-        <v>-6543.389603999999</v>
+        <v>-6543.373603999999</v>
       </c>
       <c r="AE122" s="13" t="n">
-        <v>-0.3849052708235294</v>
+        <v>-0.3849043296470588</v>
       </c>
       <c r="AF122" s="13" t="n">
-        <v>-34.62110901587301</v>
+        <v>-34.62102435978836</v>
       </c>
       <c r="AG122" s="13" t="n">
-        <v>-212.354423</v>
+        <v>-386.151687</v>
       </c>
       <c r="AH122" s="13" t="n">
-        <v>-0.01249143664705882</v>
+        <v>-0.02271480511764706</v>
       </c>
       <c r="AI122" s="13" t="n">
-        <v>-1.123568375661376</v>
+        <v>-2.043130619047619</v>
       </c>
       <c r="AJ122" s="13" t="n">
-        <v>-6755.744026999999</v>
+        <v>-6929.525290999999</v>
       </c>
       <c r="AK122" s="13" t="n">
-        <v>-0.3973967074705882</v>
+        <v>-0.4076191347647058</v>
       </c>
       <c r="AL122" s="13" t="n">
-        <v>-35.74467739153439</v>
+        <v>-36.66415497883597</v>
       </c>
     </row>
     <row r="123">
@@ -25086,40 +25164,40 @@
         <v>-5.643998698412699</v>
       </c>
       <c r="AA123" s="15" t="n">
-        <v>-1063.308436</v>
+        <v>-1063.292436</v>
       </c>
       <c r="AB123" s="15" t="n">
-        <v>-0.06254755505882353</v>
+        <v>-0.06254661388235294</v>
       </c>
       <c r="AC123" s="15" t="n">
-        <v>-5.625970560846561</v>
+        <v>-5.625885904761905</v>
       </c>
       <c r="AD123" s="15" t="n">
-        <v>-6664.368417</v>
+        <v>-6664.352416999999</v>
       </c>
       <c r="AE123" s="15" t="n">
-        <v>-0.3920216715882353</v>
+        <v>-0.3920207304117647</v>
       </c>
       <c r="AF123" s="15" t="n">
-        <v>-35.26120855555556</v>
+        <v>-35.2611238994709</v>
       </c>
       <c r="AG123" s="15" t="n">
-        <v>-212.354423</v>
+        <v>-386.151687</v>
       </c>
       <c r="AH123" s="15" t="n">
-        <v>-0.01249143664705882</v>
+        <v>-0.02271480511764706</v>
       </c>
       <c r="AI123" s="15" t="n">
-        <v>-1.123568375661376</v>
+        <v>-2.043130619047619</v>
       </c>
       <c r="AJ123" s="15" t="n">
-        <v>-6876.722839999999</v>
+        <v>-7050.504103999999</v>
       </c>
       <c r="AK123" s="15" t="n">
-        <v>-0.4045131082352941</v>
+        <v>-0.4147355355294117</v>
       </c>
       <c r="AL123" s="15" t="n">
-        <v>-36.38477693121693</v>
+        <v>-37.30425451851851</v>
       </c>
     </row>
     <row r="124">
@@ -25510,17 +25588,23 @@
       <c r="AF128" s="13" t="n">
         <v>-7.042696306878308</v>
       </c>
-      <c r="AG128" s="13" t="n"/>
-      <c r="AH128" s="13" t="n"/>
-      <c r="AI128" s="13" t="n"/>
+      <c r="AG128" s="13" t="n">
+        <v>-1.842353</v>
+      </c>
+      <c r="AH128" s="13" t="n">
+        <v>-0.0001083737058823529</v>
+      </c>
+      <c r="AI128" s="13" t="n">
+        <v>-0.00974789947089947</v>
+      </c>
       <c r="AJ128" s="13" t="n">
-        <v>-1331.069602</v>
+        <v>-1332.911955</v>
       </c>
       <c r="AK128" s="13" t="n">
-        <v>-0.07829821188235295</v>
+        <v>-0.07840658558823529</v>
       </c>
       <c r="AL128" s="13" t="n">
-        <v>-7.042696306878308</v>
+        <v>-7.052444206349207</v>
       </c>
     </row>
     <row r="129">
@@ -25825,17 +25909,23 @@
       <c r="AF131" s="11" t="n">
         <v>-6.150777666666667</v>
       </c>
-      <c r="AG131" s="11" t="n"/>
-      <c r="AH131" s="11" t="n"/>
-      <c r="AI131" s="11" t="n"/>
+      <c r="AG131" s="11" t="n">
+        <v>-67.365078</v>
+      </c>
+      <c r="AH131" s="11" t="n">
+        <v>-0.003962651647058823</v>
+      </c>
+      <c r="AI131" s="11" t="n">
+        <v>-0.3564289841269841</v>
+      </c>
       <c r="AJ131" s="11" t="n">
-        <v>-1162.496979</v>
+        <v>-1229.862057</v>
       </c>
       <c r="AK131" s="11" t="n">
-        <v>-0.06838217523529412</v>
+        <v>-0.07234482688235294</v>
       </c>
       <c r="AL131" s="11" t="n">
-        <v>-6.150777666666667</v>
+        <v>-6.507206650793652</v>
       </c>
     </row>
     <row r="132">
@@ -25934,17 +26024,23 @@
       <c r="AF132" s="15" t="n">
         <v>-141.4971653492063</v>
       </c>
-      <c r="AG132" s="15" t="n"/>
-      <c r="AH132" s="15" t="n"/>
-      <c r="AI132" s="15" t="n"/>
+      <c r="AG132" s="15" t="n">
+        <v>-69.207431</v>
+      </c>
+      <c r="AH132" s="15" t="n">
+        <v>-0.004071025352941176</v>
+      </c>
+      <c r="AI132" s="15" t="n">
+        <v>-0.3661768835978836</v>
+      </c>
       <c r="AJ132" s="15" t="n">
-        <v>-26742.964251</v>
+        <v>-26812.171682</v>
       </c>
       <c r="AK132" s="15" t="n">
-        <v>-1.573115544176471</v>
+        <v>-1.577186569529412</v>
       </c>
       <c r="AL132" s="15" t="n">
-        <v>-141.4971653492063</v>
+        <v>-141.8633422328042</v>
       </c>
     </row>
     <row r="133">
@@ -26075,22 +26171,22 @@
         <v>-0.1972583068783069</v>
       </c>
       <c r="AG134" s="11" t="n">
-        <v>-2.404</v>
+        <v>-3.141</v>
       </c>
       <c r="AH134" s="11" t="n">
-        <v>-0.0001414117647058823</v>
+        <v>-0.0001847647058823529</v>
       </c>
       <c r="AI134" s="11" t="n">
-        <v>-0.01271957671957672</v>
+        <v>-0.01661904761904762</v>
       </c>
       <c r="AJ134" s="11" t="n">
-        <v>-39.68582000000001</v>
+        <v>-40.42282</v>
       </c>
       <c r="AK134" s="11" t="n">
-        <v>-0.00233446</v>
+        <v>-0.002377812941176471</v>
       </c>
       <c r="AL134" s="11" t="n">
-        <v>-0.2099778835978836</v>
+        <v>-0.2138773544973545</v>
       </c>
     </row>
     <row r="135">
@@ -26178,22 +26274,22 @@
         <v>-2.537128</v>
       </c>
       <c r="AG135" s="13" t="n">
-        <v>-59.53072</v>
+        <v>-104.72992</v>
       </c>
       <c r="AH135" s="13" t="n">
-        <v>-0.003501807058823529</v>
+        <v>-0.006160583529411765</v>
       </c>
       <c r="AI135" s="13" t="n">
-        <v>-0.3149773544973545</v>
+        <v>-0.5541265608465609</v>
       </c>
       <c r="AJ135" s="13" t="n">
-        <v>-539.047912</v>
+        <v>-584.247112</v>
       </c>
       <c r="AK135" s="13" t="n">
-        <v>-0.03170870070588236</v>
+        <v>-0.0343674771764706</v>
       </c>
       <c r="AL135" s="13" t="n">
-        <v>-2.852105354497354</v>
+        <v>-3.091254560846561</v>
       </c>
     </row>
     <row r="136">
@@ -26384,22 +26480,22 @@
         <v>-0.6207355185185186</v>
       </c>
       <c r="AG137" s="13" t="n">
-        <v>-4.2169</v>
+        <v>-4.7489</v>
       </c>
       <c r="AH137" s="13" t="n">
-        <v>-0.0002480529411764706</v>
+        <v>-0.0002793470588235294</v>
       </c>
       <c r="AI137" s="13" t="n">
-        <v>-0.02231164021164021</v>
+        <v>-0.02512645502645502</v>
       </c>
       <c r="AJ137" s="13" t="n">
-        <v>-121.535913</v>
+        <v>-122.067913</v>
       </c>
       <c r="AK137" s="13" t="n">
-        <v>-0.007149171352941176</v>
+        <v>-0.007180465470588236</v>
       </c>
       <c r="AL137" s="13" t="n">
-        <v>-0.6430471587301588</v>
+        <v>-0.6458619735449737</v>
       </c>
     </row>
     <row r="138">
@@ -26572,22 +26668,22 @@
         <v>-0.009978835978835979</v>
       </c>
       <c r="AG139" s="13" t="n">
-        <v>-0.144255</v>
+        <v>-0.253255</v>
       </c>
       <c r="AH139" s="13" t="n">
-        <v>-8.485588235294117e-06</v>
+        <v>-1.489735294117647e-05</v>
       </c>
       <c r="AI139" s="13" t="n">
-        <v>-0.0007632539682539682</v>
+        <v>-0.001339973544973545</v>
       </c>
       <c r="AJ139" s="13" t="n">
-        <v>-2.030255</v>
+        <v>-2.139255</v>
       </c>
       <c r="AK139" s="13" t="n">
-        <v>-0.0001194267647058824</v>
+        <v>-0.0001258385294117647</v>
       </c>
       <c r="AL139" s="13" t="n">
-        <v>-0.01074208994708995</v>
+        <v>-0.01131880952380952</v>
       </c>
     </row>
     <row r="140">
@@ -26687,22 +26783,22 @@
         <v>-5.569215973544973</v>
       </c>
       <c r="AG140" s="15" t="n">
-        <v>-69.008999</v>
+        <v>-115.586199</v>
       </c>
       <c r="AH140" s="15" t="n">
-        <v>-0.004059352882352941</v>
+        <v>-0.006799188176470588</v>
       </c>
       <c r="AI140" s="15" t="n">
-        <v>-0.3651269788359788</v>
+        <v>-0.6115671904761905</v>
       </c>
       <c r="AJ140" s="15" t="n">
-        <v>-1121.590818</v>
+        <v>-1168.168018</v>
       </c>
       <c r="AK140" s="15" t="n">
-        <v>-0.06597593047058824</v>
+        <v>-0.06871576576470588</v>
       </c>
       <c r="AL140" s="15" t="n">
-        <v>-5.934342952380952</v>
+        <v>-6.180783164021164</v>
       </c>
     </row>
     <row r="141">
@@ -26784,40 +26880,40 @@
         <v>-17.10132559259259</v>
       </c>
       <c r="AA141" s="15" t="n">
-        <v>-4461.884406270001</v>
+        <v>-4461.86840627</v>
       </c>
       <c r="AB141" s="15" t="n">
-        <v>-0.2624637886041177</v>
+        <v>-0.2624628474276471</v>
       </c>
       <c r="AC141" s="15" t="n">
-        <v>-23.60785400142858</v>
+        <v>-23.60776934534392</v>
       </c>
       <c r="AD141" s="15" t="n">
-        <v>-47956.49355917001</v>
+        <v>-47956.47755917</v>
       </c>
       <c r="AE141" s="15" t="n">
-        <v>-2.820970209362941</v>
+        <v>-2.82096926818647</v>
       </c>
       <c r="AF141" s="15" t="n">
-        <v>-253.7380611596296</v>
+        <v>-253.7379765035449</v>
       </c>
       <c r="AG141" s="15" t="n">
-        <v>-932.127074</v>
+        <v>-1520.790626</v>
       </c>
       <c r="AH141" s="15" t="n">
-        <v>-0.05483100435294118</v>
+        <v>-0.08945827211764706</v>
       </c>
       <c r="AI141" s="15" t="n">
-        <v>-4.93188928042328</v>
+        <v>-8.046511248677248</v>
       </c>
       <c r="AJ141" s="15" t="n">
-        <v>-48888.62063317001</v>
+        <v>-49477.26818517</v>
       </c>
       <c r="AK141" s="15" t="n">
-        <v>-2.875801213715882</v>
+        <v>-2.910427540304117</v>
       </c>
       <c r="AL141" s="15" t="n">
-        <v>-258.6699504400528</v>
+        <v>-261.7844877522222</v>
       </c>
     </row>
     <row r="142">
@@ -27045,22 +27141,22 @@
         <v>-5.281271338624339</v>
       </c>
       <c r="AG144" s="13" t="n">
-        <v>-9.5</v>
+        <v>-60.064418</v>
       </c>
       <c r="AH144" s="13" t="n">
-        <v>-0.0005588235294117647</v>
+        <v>-0.00353320105882353</v>
       </c>
       <c r="AI144" s="13" t="n">
-        <v>-0.05026455026455026</v>
+        <v>-0.3178011534391534</v>
       </c>
       <c r="AJ144" s="13" t="n">
-        <v>-1007.660283</v>
+        <v>-1058.224701</v>
       </c>
       <c r="AK144" s="13" t="n">
-        <v>-0.05927413429411766</v>
+        <v>-0.06224851182352942</v>
       </c>
       <c r="AL144" s="13" t="n">
-        <v>-5.331535888888889</v>
+        <v>-5.599072492063492</v>
       </c>
     </row>
     <row r="145">
@@ -27282,22 +27378,22 @@
         <v>-14.12313906349206</v>
       </c>
       <c r="AG147" s="15" t="n">
-        <v>-9.5</v>
+        <v>-60.064418</v>
       </c>
       <c r="AH147" s="15" t="n">
-        <v>-0.0005588235294117647</v>
+        <v>-0.00353320105882353</v>
       </c>
       <c r="AI147" s="15" t="n">
-        <v>-0.05026455026455026</v>
+        <v>-0.3178011534391534</v>
       </c>
       <c r="AJ147" s="15" t="n">
-        <v>-2678.773283</v>
+        <v>-2729.337701</v>
       </c>
       <c r="AK147" s="15" t="n">
-        <v>-0.157574899</v>
+        <v>-0.1605492765294118</v>
       </c>
       <c r="AL147" s="15" t="n">
-        <v>-14.17340361375661</v>
+        <v>-14.44094021693122</v>
       </c>
     </row>
     <row r="148">
@@ -27422,40 +27518,40 @@
         <v>-0.01227130158730159</v>
       </c>
       <c r="AA149" s="11" t="n">
-        <v>-1.44129</v>
+        <v>-1.45729</v>
       </c>
       <c r="AB149" s="11" t="n">
-        <v>-8.478176470588236e-05</v>
+        <v>-8.572294117647058e-05</v>
       </c>
       <c r="AC149" s="11" t="n">
-        <v>-0.007625873015873016</v>
+        <v>-0.0077105291005291</v>
       </c>
       <c r="AD149" s="11" t="n">
-        <v>-20.23718768</v>
+        <v>-20.25318768</v>
       </c>
       <c r="AE149" s="11" t="n">
-        <v>-0.001190422804705882</v>
+        <v>-0.001191363981176471</v>
       </c>
       <c r="AF149" s="11" t="n">
-        <v>-0.1070750670899471</v>
+        <v>-0.1071597231746032</v>
       </c>
       <c r="AG149" s="11" t="n">
-        <v>-0.600042</v>
+        <v>-1.448262</v>
       </c>
       <c r="AH149" s="11" t="n">
-        <v>-3.529658823529412e-05</v>
+        <v>-8.519188235294118e-05</v>
       </c>
       <c r="AI149" s="11" t="n">
-        <v>-0.003174825396825397</v>
+        <v>-0.007662761904761905</v>
       </c>
       <c r="AJ149" s="11" t="n">
-        <v>-20.83722968</v>
+        <v>-21.70144968</v>
       </c>
       <c r="AK149" s="11" t="n">
-        <v>-0.001225719392941177</v>
+        <v>-0.001276555863529412</v>
       </c>
       <c r="AL149" s="11" t="n">
-        <v>-0.1102498924867725</v>
+        <v>-0.1148224850793651</v>
       </c>
     </row>
     <row r="150">
@@ -28065,40 +28161,40 @@
         <v>-1.590824077883598</v>
       </c>
       <c r="AA156" s="15" t="n">
-        <v>-283.80721553</v>
+        <v>-283.82321553</v>
       </c>
       <c r="AB156" s="15" t="n">
-        <v>-0.01669454209</v>
+        <v>-0.01669548326647059</v>
       </c>
       <c r="AC156" s="15" t="n">
-        <v>-1.501625478994709</v>
+        <v>-1.501710135079365</v>
       </c>
       <c r="AD156" s="15" t="n">
-        <v>-6253.99547277</v>
+        <v>-6254.01147277</v>
       </c>
       <c r="AE156" s="15" t="n">
-        <v>-0.3678820866335294</v>
+        <v>-0.36788302781</v>
       </c>
       <c r="AF156" s="15" t="n">
-        <v>-33.08992313634921</v>
+        <v>-33.09000779243386</v>
       </c>
       <c r="AG156" s="15" t="n">
-        <v>-176.828318</v>
+        <v>-177.676538</v>
       </c>
       <c r="AH156" s="15" t="n">
-        <v>-0.01040166576470588</v>
+        <v>-0.01045156105882353</v>
       </c>
       <c r="AI156" s="15" t="n">
-        <v>-0.9355995661375661</v>
+        <v>-0.9400875026455026</v>
       </c>
       <c r="AJ156" s="15" t="n">
-        <v>-6430.82379077</v>
+        <v>-6431.68801077</v>
       </c>
       <c r="AK156" s="15" t="n">
-        <v>-0.3782837523982353</v>
+        <v>-0.3783345888688235</v>
       </c>
       <c r="AL156" s="15" t="n">
-        <v>-34.02552270248678</v>
+        <v>-34.03009529507936</v>
       </c>
     </row>
     <row r="157">
@@ -28198,22 +28294,22 @@
         <v>-1609.397741344392</v>
       </c>
       <c r="AG157" s="19" t="n">
-        <v>-4672.824291</v>
+        <v>-12498.172521</v>
       </c>
       <c r="AH157" s="19" t="n">
-        <v>-0.274872017117647</v>
+        <v>-0.7351866188823529</v>
       </c>
       <c r="AI157" s="19" t="n">
-        <v>-24.72393804761905</v>
+        <v>-66.12789693650794</v>
       </c>
       <c r="AJ157" s="19" t="n">
-        <v>-308848.99740509</v>
+        <v>-316674.3456350899</v>
       </c>
       <c r="AK157" s="19" t="n">
-        <v>-18.16758808265235</v>
+        <v>-18.62790268441706</v>
       </c>
       <c r="AL157" s="19" t="n">
-        <v>-1634.12167939201</v>
+        <v>-1675.5256382809</v>
       </c>
     </row>
     <row r="158">
@@ -28313,22 +28409,22 @@
         <v>-277.2179185799473</v>
       </c>
       <c r="AG158" s="19" t="n">
-        <v>8853.440492</v>
+        <v>1031.929162</v>
       </c>
       <c r="AH158" s="19" t="n">
-        <v>0.5207906171764706</v>
+        <v>0.0607017154117647</v>
       </c>
       <c r="AI158" s="19" t="n">
-        <v>46.84360048677249</v>
+        <v>5.459942656084656</v>
       </c>
       <c r="AJ158" s="19" t="n">
-        <v>-43540.74611961</v>
+        <v>-51362.25744961</v>
       </c>
       <c r="AK158" s="19" t="n">
-        <v>-2.56122035997706</v>
+        <v>-3.021309261741766</v>
       </c>
       <c r="AL158" s="19" t="n">
-        <v>-230.3743180931748</v>
+        <v>-271.7579759238626</v>
       </c>
     </row>
     <row r="159">
@@ -28428,22 +28524,22 @@
         <v>79.78557785582009</v>
       </c>
       <c r="AG159" s="7" t="n">
-        <v>23932.91470675</v>
+        <v>16111.40337675</v>
       </c>
       <c r="AH159" s="7" t="n">
-        <v>1.407818512161765</v>
+        <v>0.9477296103970588</v>
       </c>
       <c r="AI159" s="7" t="n">
-        <v>126.6291783425926</v>
+        <v>85.24552051190476</v>
       </c>
       <c r="AJ159" s="7" t="n">
-        <v>23932.91470675</v>
+        <v>16111.40337675</v>
       </c>
       <c r="AK159" s="7" t="n">
-        <v>1.407818512161765</v>
+        <v>0.9477296103970588</v>
       </c>
       <c r="AL159" s="7" t="n">
-        <v>126.6291783425926</v>
+        <v>85.24552051190476</v>
       </c>
     </row>
   </sheetData>

</xml_diff>